<commit_message>
Master system update 2026-09-15 00:20
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1804 +568,1629 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>142.16</v>
+        <v>150.61</v>
       </c>
       <c r="C2" t="n">
-        <v>154.13</v>
+        <v>156.92</v>
       </c>
       <c r="D2" t="n">
-        <v>141.84</v>
+        <v>148.9</v>
       </c>
       <c r="E2" t="n">
-        <v>145.36</v>
+        <v>151.53</v>
       </c>
       <c r="F2" t="n">
-        <v>75.04000000000001</v>
+        <v>77.38</v>
       </c>
       <c r="G2" t="n">
-        <v>77.77</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>74.70999999999999</v>
+        <v>76.20999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>77.15000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>41.01</v>
+        <v>38.65</v>
       </c>
       <c r="K2" t="n">
-        <v>41.14</v>
+        <v>39.09</v>
       </c>
       <c r="L2" t="n">
-        <v>37.56</v>
+        <v>36.89</v>
       </c>
       <c r="M2" t="n">
-        <v>40.12</v>
+        <v>38.36</v>
       </c>
       <c r="N2" t="n">
-        <v>37.11</v>
+        <v>35.98</v>
       </c>
       <c r="O2" t="n">
-        <v>37.28</v>
+        <v>36.51</v>
       </c>
       <c r="P2" t="n">
-        <v>35.74</v>
+        <v>35.72</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.04</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>143.79</v>
+        <v>134.2</v>
       </c>
       <c r="C3" t="n">
-        <v>146.65</v>
+        <v>137.6</v>
       </c>
       <c r="D3" t="n">
-        <v>138.9</v>
+        <v>122.4</v>
       </c>
       <c r="E3" t="n">
-        <v>144.95</v>
+        <v>129.1</v>
       </c>
       <c r="F3" t="n">
-        <v>77.56999999999999</v>
+        <v>73.36</v>
       </c>
       <c r="G3" t="n">
-        <v>77.84999999999999</v>
+        <v>73.95999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>75.94</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>76.79000000000001</v>
+        <v>72.53</v>
       </c>
       <c r="J3" t="n">
-        <v>40.61</v>
+        <v>42.89</v>
       </c>
       <c r="K3" t="n">
-        <v>41.92</v>
+        <v>45.83</v>
       </c>
       <c r="L3" t="n">
-        <v>39.73</v>
+        <v>41.94</v>
       </c>
       <c r="M3" t="n">
-        <v>40.28</v>
+        <v>44.19</v>
       </c>
       <c r="N3" t="n">
-        <v>35.88</v>
+        <v>37.87</v>
       </c>
       <c r="O3" t="n">
-        <v>36.64</v>
+        <v>38.53</v>
       </c>
       <c r="P3" t="n">
-        <v>35.74</v>
+        <v>37.59</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.24</v>
+        <v>38.28</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.2821</v>
+        <v>-14.8023</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.4666</v>
+        <v>-5.0654</v>
       </c>
       <c r="X3" t="n">
-        <v>0.3988</v>
+        <v>15.1981</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.5548999999999999</v>
+        <v>5.1071</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>150.61</v>
+        <v>132.63</v>
       </c>
       <c r="C4" t="n">
-        <v>156.92</v>
+        <v>133.74</v>
       </c>
       <c r="D4" t="n">
-        <v>148.9</v>
+        <v>116.84</v>
       </c>
       <c r="E4" t="n">
-        <v>151.53</v>
+        <v>120.74</v>
       </c>
       <c r="F4" t="n">
-        <v>77.38</v>
+        <v>73.37</v>
       </c>
       <c r="G4" t="n">
-        <v>77.90000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="H4" t="n">
-        <v>76.20999999999999</v>
+        <v>71</v>
       </c>
       <c r="I4" t="n">
-        <v>76.40000000000001</v>
+        <v>72.06</v>
       </c>
       <c r="J4" t="n">
-        <v>38.65</v>
+        <v>42.83</v>
       </c>
       <c r="K4" t="n">
-        <v>39.09</v>
+        <v>48.34</v>
       </c>
       <c r="L4" t="n">
-        <v>36.89</v>
+        <v>42.48</v>
       </c>
       <c r="M4" t="n">
-        <v>38.36</v>
+        <v>47.05</v>
       </c>
       <c r="N4" t="n">
-        <v>35.98</v>
+        <v>37.83</v>
       </c>
       <c r="O4" t="n">
-        <v>36.51</v>
+        <v>39.08</v>
       </c>
       <c r="P4" t="n">
-        <v>35.72</v>
+        <v>37.66</v>
       </c>
       <c r="Q4" t="n">
-        <v>36.42</v>
+        <v>38.53</v>
       </c>
       <c r="R4" t="n">
-        <v>4.5395</v>
+        <v>-6.4756</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.5079</v>
+        <v>-0.648</v>
       </c>
       <c r="X4" t="n">
-        <v>-4.7666</v>
+        <v>6.4721</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.4967</v>
+        <v>0.6531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>134.2</v>
+        <v>119.99</v>
       </c>
       <c r="C5" t="n">
-        <v>137.6</v>
+        <v>124.56</v>
       </c>
       <c r="D5" t="n">
-        <v>122.4</v>
+        <v>117.42</v>
       </c>
       <c r="E5" t="n">
-        <v>129.1</v>
+        <v>122.21</v>
       </c>
       <c r="F5" t="n">
-        <v>73.36</v>
+        <v>70.83</v>
       </c>
       <c r="G5" t="n">
-        <v>73.95999999999999</v>
+        <v>71.69</v>
       </c>
       <c r="H5" t="n">
-        <v>72.01000000000001</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>72.53</v>
+        <v>70.48</v>
       </c>
       <c r="J5" t="n">
-        <v>42.89</v>
+        <v>47.33</v>
       </c>
       <c r="K5" t="n">
-        <v>45.83</v>
+        <v>48.29</v>
       </c>
       <c r="L5" t="n">
-        <v>41.94</v>
+        <v>45.47</v>
       </c>
       <c r="M5" t="n">
-        <v>44.19</v>
+        <v>46.25</v>
       </c>
       <c r="N5" t="n">
-        <v>37.87</v>
+        <v>39.18</v>
       </c>
       <c r="O5" t="n">
-        <v>38.53</v>
+        <v>39.77</v>
       </c>
       <c r="P5" t="n">
-        <v>37.59</v>
+        <v>38.74</v>
       </c>
       <c r="Q5" t="n">
-        <v>38.28</v>
+        <v>39.37</v>
       </c>
       <c r="R5" t="n">
-        <v>-14.8023</v>
+        <v>1.2175</v>
       </c>
       <c r="S5" t="n">
-        <v>-11.186</v>
+        <v>-19.3493</v>
       </c>
       <c r="U5" t="n">
-        <v>-5.0654</v>
+        <v>-2.1926</v>
       </c>
       <c r="V5" t="n">
-        <v>-5.9883</v>
+        <v>-7.7487</v>
       </c>
       <c r="X5" t="n">
-        <v>15.1981</v>
+        <v>-1.7003</v>
       </c>
       <c r="Y5" t="n">
-        <v>10.1446</v>
+        <v>20.5683</v>
       </c>
       <c r="AA5" t="n">
-        <v>5.1071</v>
+        <v>2.1801</v>
       </c>
       <c r="AB5" t="n">
-        <v>6.2153</v>
+        <v>8.0999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>132.63</v>
+        <v>126.59</v>
       </c>
       <c r="C6" t="n">
-        <v>133.74</v>
+        <v>126.79</v>
       </c>
       <c r="D6" t="n">
-        <v>116.84</v>
+        <v>116.71</v>
       </c>
       <c r="E6" t="n">
-        <v>120.74</v>
+        <v>120.6</v>
       </c>
       <c r="F6" t="n">
-        <v>73.37</v>
+        <v>71.7</v>
       </c>
       <c r="G6" t="n">
-        <v>73.7</v>
+        <v>71.83</v>
       </c>
       <c r="H6" t="n">
-        <v>71</v>
+        <v>69.91</v>
       </c>
       <c r="I6" t="n">
-        <v>72.06</v>
+        <v>71.17</v>
       </c>
       <c r="J6" t="n">
-        <v>42.83</v>
+        <v>44.67</v>
       </c>
       <c r="K6" t="n">
-        <v>48.34</v>
+        <v>48.46</v>
       </c>
       <c r="L6" t="n">
-        <v>42.48</v>
+        <v>44.65</v>
       </c>
       <c r="M6" t="n">
-        <v>47.05</v>
+        <v>47.03</v>
       </c>
       <c r="N6" t="n">
-        <v>37.83</v>
+        <v>38.71</v>
       </c>
       <c r="O6" t="n">
-        <v>39.08</v>
+        <v>39.72</v>
       </c>
       <c r="P6" t="n">
-        <v>37.66</v>
+        <v>38.64</v>
       </c>
       <c r="Q6" t="n">
-        <v>38.53</v>
+        <v>39.02</v>
       </c>
       <c r="R6" t="n">
-        <v>-6.4756</v>
+        <v>-1.3174</v>
       </c>
       <c r="S6" t="n">
-        <v>-16.7023</v>
+        <v>-6.584</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.648</v>
+        <v>0.979</v>
       </c>
       <c r="V6" t="n">
-        <v>-6.1597</v>
+        <v>-1.8751</v>
       </c>
       <c r="X6" t="n">
-        <v>6.4721</v>
+        <v>1.6865</v>
       </c>
       <c r="Y6" t="n">
-        <v>16.8073</v>
+        <v>6.4268</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.6531</v>
+        <v>-0.889</v>
       </c>
       <c r="AB6" t="n">
-        <v>6.319</v>
+        <v>1.9331</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>119.99</v>
+        <v>115.07</v>
       </c>
       <c r="C7" t="n">
-        <v>124.56</v>
+        <v>115.07</v>
       </c>
       <c r="D7" t="n">
-        <v>117.42</v>
+        <v>106</v>
       </c>
       <c r="E7" t="n">
-        <v>122.21</v>
+        <v>111.16</v>
       </c>
       <c r="F7" t="n">
-        <v>70.83</v>
+        <v>70</v>
       </c>
       <c r="G7" t="n">
-        <v>71.69</v>
+        <v>70.05</v>
       </c>
       <c r="H7" t="n">
-        <v>69.76000000000001</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>70.48</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>47.33</v>
+        <v>49.14</v>
       </c>
       <c r="K7" t="n">
-        <v>48.29</v>
+        <v>52.81</v>
       </c>
       <c r="L7" t="n">
-        <v>45.47</v>
+        <v>49.13</v>
       </c>
       <c r="M7" t="n">
-        <v>46.25</v>
+        <v>50.75</v>
       </c>
       <c r="N7" t="n">
-        <v>39.18</v>
+        <v>39.65</v>
       </c>
       <c r="O7" t="n">
-        <v>39.77</v>
+        <v>40.79</v>
       </c>
       <c r="P7" t="n">
-        <v>38.74</v>
+        <v>39.64</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.37</v>
+        <v>40.19</v>
       </c>
       <c r="R7" t="n">
-        <v>1.2175</v>
+        <v>-7.8275</v>
       </c>
       <c r="S7" t="n">
-        <v>-19.3493</v>
+        <v>-7.9344</v>
       </c>
       <c r="T7" t="n">
-        <v>-15.926</v>
+        <v>-26.6416</v>
       </c>
       <c r="U7" t="n">
-        <v>-2.1926</v>
+        <v>-3.035</v>
       </c>
       <c r="V7" t="n">
-        <v>-7.7487</v>
+        <v>-4.2326</v>
       </c>
       <c r="W7" t="n">
-        <v>-8.6455</v>
+        <v>-9.672800000000001</v>
       </c>
       <c r="X7" t="n">
-        <v>-1.7003</v>
+        <v>7.9098</v>
       </c>
       <c r="Y7" t="n">
-        <v>20.5683</v>
+        <v>7.864</v>
       </c>
       <c r="Z7" t="n">
-        <v>15.2792</v>
+        <v>32.2993</v>
       </c>
       <c r="AA7" t="n">
-        <v>2.1801</v>
+        <v>2.9985</v>
       </c>
       <c r="AB7" t="n">
-        <v>8.0999</v>
+        <v>4.3083</v>
       </c>
       <c r="AC7" t="n">
-        <v>9.239699999999999</v>
+        <v>10.3515</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>126.59</v>
+        <v>117.37</v>
       </c>
       <c r="C8" t="n">
-        <v>126.79</v>
+        <v>119.88</v>
       </c>
       <c r="D8" t="n">
-        <v>116.71</v>
+        <v>113.13</v>
       </c>
       <c r="E8" t="n">
-        <v>120.6</v>
+        <v>115.67</v>
       </c>
       <c r="F8" t="n">
-        <v>71.7</v>
+        <v>70.42</v>
       </c>
       <c r="G8" t="n">
-        <v>71.83</v>
+        <v>71.27</v>
       </c>
       <c r="H8" t="n">
-        <v>69.91</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>71.17</v>
+        <v>70.27</v>
       </c>
       <c r="J8" t="n">
-        <v>44.67</v>
+        <v>47.82</v>
       </c>
       <c r="K8" t="n">
-        <v>48.46</v>
+        <v>49.83</v>
       </c>
       <c r="L8" t="n">
-        <v>44.65</v>
+        <v>46.66</v>
       </c>
       <c r="M8" t="n">
-        <v>47.03</v>
+        <v>48.42</v>
       </c>
       <c r="N8" t="n">
-        <v>38.71</v>
+        <v>39.38</v>
       </c>
       <c r="O8" t="n">
-        <v>39.72</v>
+        <v>40.02</v>
       </c>
       <c r="P8" t="n">
-        <v>38.64</v>
+        <v>38.89</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.02</v>
+        <v>39.46</v>
       </c>
       <c r="R8" t="n">
-        <v>-1.3174</v>
+        <v>4.0572</v>
       </c>
       <c r="S8" t="n">
-        <v>-6.584</v>
+        <v>-5.3514</v>
       </c>
       <c r="T8" t="n">
-        <v>-16.7989</v>
+        <v>-10.4028</v>
       </c>
       <c r="U8" t="n">
-        <v>0.979</v>
+        <v>1.8258</v>
       </c>
       <c r="V8" t="n">
-        <v>-1.8751</v>
+        <v>-0.298</v>
       </c>
       <c r="W8" t="n">
-        <v>-7.3187</v>
+        <v>-3.116</v>
       </c>
       <c r="X8" t="n">
-        <v>1.6865</v>
+        <v>-4.5911</v>
       </c>
       <c r="Y8" t="n">
-        <v>6.4268</v>
+        <v>4.6919</v>
       </c>
       <c r="Z8" t="n">
-        <v>16.7577</v>
+        <v>9.5723</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.889</v>
+        <v>-1.8164</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.9331</v>
+        <v>0.2286</v>
       </c>
       <c r="AC8" t="n">
-        <v>7.6711</v>
+        <v>3.0825</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>115.07</v>
+        <v>114.7</v>
       </c>
       <c r="C9" t="n">
-        <v>115.07</v>
+        <v>117.39</v>
       </c>
       <c r="D9" t="n">
-        <v>106</v>
+        <v>112.53</v>
       </c>
       <c r="E9" t="n">
-        <v>111.16</v>
+        <v>116.6</v>
       </c>
       <c r="F9" t="n">
-        <v>70</v>
+        <v>69.56</v>
       </c>
       <c r="G9" t="n">
-        <v>70.05</v>
+        <v>70.94</v>
       </c>
       <c r="H9" t="n">
-        <v>67.93000000000001</v>
+        <v>69.44</v>
       </c>
       <c r="I9" t="n">
-        <v>69.01000000000001</v>
+        <v>70.47</v>
       </c>
       <c r="J9" t="n">
-        <v>49.14</v>
+        <v>49.01</v>
       </c>
       <c r="K9" t="n">
-        <v>52.81</v>
+        <v>49.89</v>
       </c>
       <c r="L9" t="n">
-        <v>49.13</v>
+        <v>47.87</v>
       </c>
       <c r="M9" t="n">
-        <v>50.75</v>
+        <v>48.09</v>
       </c>
       <c r="N9" t="n">
-        <v>39.65</v>
+        <v>39.86</v>
       </c>
       <c r="O9" t="n">
-        <v>40.79</v>
+        <v>39.93</v>
       </c>
       <c r="P9" t="n">
-        <v>39.64</v>
+        <v>39.09</v>
       </c>
       <c r="Q9" t="n">
-        <v>40.19</v>
+        <v>39.38</v>
       </c>
       <c r="R9" t="n">
-        <v>-7.8275</v>
+        <v>0.804</v>
       </c>
       <c r="S9" t="n">
-        <v>-7.9344</v>
+        <v>-3.3167</v>
       </c>
       <c r="T9" t="n">
-        <v>-26.6416</v>
+        <v>-3.4289</v>
       </c>
       <c r="U9" t="n">
-        <v>-3.035</v>
+        <v>0.2846</v>
       </c>
       <c r="V9" t="n">
-        <v>-4.2326</v>
+        <v>-0.9836</v>
       </c>
       <c r="W9" t="n">
-        <v>-9.672800000000001</v>
+        <v>-2.2065</v>
       </c>
       <c r="X9" t="n">
-        <v>7.9098</v>
+        <v>-0.6815</v>
       </c>
       <c r="Y9" t="n">
-        <v>7.864</v>
+        <v>2.2539</v>
       </c>
       <c r="Z9" t="n">
-        <v>32.2993</v>
+        <v>2.2104</v>
       </c>
       <c r="AA9" t="n">
-        <v>2.9985</v>
+        <v>-0.2027</v>
       </c>
       <c r="AB9" t="n">
-        <v>4.3083</v>
+        <v>0.9226</v>
       </c>
       <c r="AC9" t="n">
-        <v>10.3515</v>
+        <v>2.2061</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>117.37</v>
+        <v>123.4</v>
       </c>
       <c r="C10" t="n">
-        <v>119.88</v>
+        <v>124.88</v>
       </c>
       <c r="D10" t="n">
-        <v>113.13</v>
+        <v>117.69</v>
       </c>
       <c r="E10" t="n">
-        <v>115.67</v>
+        <v>123.05</v>
       </c>
       <c r="F10" t="n">
-        <v>70.42</v>
+        <v>72.09</v>
       </c>
       <c r="G10" t="n">
-        <v>71.27</v>
+        <v>73.38</v>
       </c>
       <c r="H10" t="n">
-        <v>69.34999999999999</v>
+        <v>71.38</v>
       </c>
       <c r="I10" t="n">
-        <v>70.27</v>
+        <v>73.3</v>
       </c>
       <c r="J10" t="n">
-        <v>47.82</v>
+        <v>45.42</v>
       </c>
       <c r="K10" t="n">
-        <v>49.83</v>
+        <v>47.71</v>
       </c>
       <c r="L10" t="n">
-        <v>46.66</v>
+        <v>44.71</v>
       </c>
       <c r="M10" t="n">
-        <v>48.42</v>
+        <v>45.35</v>
       </c>
       <c r="N10" t="n">
-        <v>39.38</v>
+        <v>38.46</v>
       </c>
       <c r="O10" t="n">
-        <v>40.02</v>
+        <v>38.86</v>
       </c>
       <c r="P10" t="n">
-        <v>38.89</v>
+        <v>37.73</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.46</v>
+        <v>37.78</v>
       </c>
       <c r="R10" t="n">
-        <v>4.0572</v>
+        <v>5.5317</v>
       </c>
       <c r="S10" t="n">
-        <v>-5.3514</v>
+        <v>10.6963</v>
       </c>
       <c r="T10" t="n">
-        <v>-10.4028</v>
+        <v>0.6873</v>
       </c>
       <c r="U10" t="n">
-        <v>1.8258</v>
+        <v>4.0159</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.298</v>
+        <v>6.2165</v>
       </c>
       <c r="W10" t="n">
-        <v>-3.116</v>
+        <v>4.0011</v>
       </c>
       <c r="X10" t="n">
-        <v>-4.5911</v>
+        <v>-5.6977</v>
       </c>
       <c r="Y10" t="n">
-        <v>4.6919</v>
+        <v>-10.6404</v>
       </c>
       <c r="Z10" t="n">
-        <v>9.5723</v>
+        <v>-1.9459</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.8164</v>
+        <v>-4.063</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.2286</v>
+        <v>-5.9965</v>
       </c>
       <c r="AC10" t="n">
-        <v>3.0825</v>
+        <v>-4.0386</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>114.7</v>
+        <v>119.92</v>
       </c>
       <c r="C11" t="n">
-        <v>117.39</v>
+        <v>121.2</v>
       </c>
       <c r="D11" t="n">
-        <v>112.53</v>
+        <v>110.21</v>
       </c>
       <c r="E11" t="n">
-        <v>116.6</v>
+        <v>111.34</v>
       </c>
       <c r="F11" t="n">
-        <v>69.56</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>70.94</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>69.44</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>70.47</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>49.01</v>
+        <v>46.61</v>
       </c>
       <c r="K11" t="n">
-        <v>49.89</v>
+        <v>50.23</v>
       </c>
       <c r="L11" t="n">
-        <v>47.87</v>
+        <v>46.15</v>
       </c>
       <c r="M11" t="n">
-        <v>48.09</v>
+        <v>49.82</v>
       </c>
       <c r="N11" t="n">
-        <v>39.86</v>
+        <v>38.02</v>
       </c>
       <c r="O11" t="n">
-        <v>39.93</v>
+        <v>38.76</v>
       </c>
       <c r="P11" t="n">
-        <v>39.09</v>
+        <v>37.33</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.38</v>
+        <v>38.54</v>
       </c>
       <c r="R11" t="n">
-        <v>0.804</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="S11" t="n">
-        <v>-3.3167</v>
+        <v>-3.7434</v>
       </c>
       <c r="T11" t="n">
-        <v>-3.4289</v>
+        <v>-7.6783</v>
       </c>
       <c r="U11" t="n">
-        <v>0.2846</v>
+        <v>-1.9782</v>
       </c>
       <c r="V11" t="n">
-        <v>-0.9836</v>
+        <v>2.2485</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.2065</v>
+        <v>0.9555</v>
       </c>
       <c r="X11" t="n">
-        <v>-0.6815</v>
+        <v>9.8567</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.2539</v>
+        <v>2.8914</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.2104</v>
+        <v>5.9324</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.2027</v>
+        <v>2.0116</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.9226</v>
+        <v>-2.3315</v>
       </c>
       <c r="AC11" t="n">
-        <v>2.2061</v>
+        <v>-1.2301</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>123.4</v>
+        <v>112.41</v>
       </c>
       <c r="C12" t="n">
-        <v>124.88</v>
+        <v>115.05</v>
       </c>
       <c r="D12" t="n">
-        <v>117.69</v>
+        <v>110.33</v>
       </c>
       <c r="E12" t="n">
-        <v>123.05</v>
+        <v>112.79</v>
       </c>
       <c r="F12" t="n">
-        <v>72.09</v>
+        <v>71.44</v>
       </c>
       <c r="G12" t="n">
-        <v>73.38</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>71.38</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>73.3</v>
+        <v>71.92</v>
       </c>
       <c r="J12" t="n">
-        <v>45.42</v>
+        <v>49.27</v>
       </c>
       <c r="K12" t="n">
-        <v>47.71</v>
+        <v>50.24</v>
       </c>
       <c r="L12" t="n">
-        <v>44.71</v>
+        <v>48.09</v>
       </c>
       <c r="M12" t="n">
-        <v>45.35</v>
+        <v>49.02</v>
       </c>
       <c r="N12" t="n">
-        <v>38.46</v>
+        <v>38.77</v>
       </c>
       <c r="O12" t="n">
-        <v>38.86</v>
+        <v>39.09</v>
       </c>
       <c r="P12" t="n">
-        <v>37.73</v>
+        <v>38.37</v>
       </c>
       <c r="Q12" t="n">
-        <v>37.78</v>
+        <v>38.51</v>
       </c>
       <c r="R12" t="n">
-        <v>5.5317</v>
+        <v>1.3023</v>
       </c>
       <c r="S12" t="n">
-        <v>10.6963</v>
+        <v>-3.2676</v>
       </c>
       <c r="T12" t="n">
-        <v>0.6873</v>
+        <v>1.4664</v>
       </c>
       <c r="U12" t="n">
-        <v>4.0159</v>
+        <v>0.0974</v>
       </c>
       <c r="V12" t="n">
-        <v>6.2165</v>
+        <v>2.0576</v>
       </c>
       <c r="W12" t="n">
-        <v>4.0011</v>
+        <v>4.2168</v>
       </c>
       <c r="X12" t="n">
-        <v>-5.6977</v>
+        <v>-1.6058</v>
       </c>
       <c r="Y12" t="n">
-        <v>-10.6404</v>
+        <v>1.9339</v>
       </c>
       <c r="Z12" t="n">
-        <v>-1.9459</v>
+        <v>-3.4089</v>
       </c>
       <c r="AA12" t="n">
-        <v>-4.063</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="AB12" t="n">
-        <v>-5.9965</v>
+        <v>-2.2092</v>
       </c>
       <c r="AC12" t="n">
-        <v>-4.0386</v>
+        <v>-4.1801</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>119.92</v>
+        <v>106.36</v>
       </c>
       <c r="C13" t="n">
-        <v>121.2</v>
+        <v>108.64</v>
       </c>
       <c r="D13" t="n">
-        <v>110.21</v>
+        <v>102.31</v>
       </c>
       <c r="E13" t="n">
-        <v>111.34</v>
+        <v>105.91</v>
       </c>
       <c r="F13" t="n">
-        <v>72.84999999999999</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>74.18000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="H13" t="n">
-        <v>71.43000000000001</v>
+        <v>68.25</v>
       </c>
       <c r="I13" t="n">
-        <v>71.84999999999999</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>46.61</v>
+        <v>51.88</v>
       </c>
       <c r="K13" t="n">
-        <v>50.23</v>
+        <v>53.69</v>
       </c>
       <c r="L13" t="n">
-        <v>46.15</v>
+        <v>50.9</v>
       </c>
       <c r="M13" t="n">
-        <v>49.82</v>
+        <v>52.22</v>
       </c>
       <c r="N13" t="n">
-        <v>38.02</v>
+        <v>40.03</v>
       </c>
       <c r="O13" t="n">
-        <v>38.76</v>
+        <v>40.47</v>
       </c>
       <c r="P13" t="n">
-        <v>37.33</v>
+        <v>39.23</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.54</v>
+        <v>39.97</v>
       </c>
       <c r="R13" t="n">
-        <v>-9.516500000000001</v>
+        <v>-6.0998</v>
       </c>
       <c r="S13" t="n">
-        <v>-3.7434</v>
+        <v>-13.9293</v>
       </c>
       <c r="T13" t="n">
-        <v>-7.6783</v>
+        <v>-8.437799999999999</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.9782</v>
+        <v>-3.8515</v>
       </c>
       <c r="V13" t="n">
-        <v>2.2485</v>
+        <v>-5.6617</v>
       </c>
       <c r="W13" t="n">
-        <v>0.9555</v>
+        <v>-1.5939</v>
       </c>
       <c r="X13" t="n">
-        <v>9.8567</v>
+        <v>6.5279</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.8914</v>
+        <v>15.1488</v>
       </c>
       <c r="Z13" t="n">
-        <v>5.9324</v>
+        <v>7.848</v>
       </c>
       <c r="AA13" t="n">
-        <v>2.0116</v>
+        <v>3.7912</v>
       </c>
       <c r="AB13" t="n">
-        <v>-2.3315</v>
+        <v>5.7967</v>
       </c>
       <c r="AC13" t="n">
-        <v>-1.2301</v>
+        <v>1.2924</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>112.41</v>
+        <v>104.5</v>
       </c>
       <c r="C14" t="n">
-        <v>115.05</v>
+        <v>108.07</v>
       </c>
       <c r="D14" t="n">
-        <v>110.33</v>
+        <v>101.34</v>
       </c>
       <c r="E14" t="n">
-        <v>112.79</v>
+        <v>106.35</v>
       </c>
       <c r="F14" t="n">
-        <v>71.44</v>
+        <v>68.97</v>
       </c>
       <c r="G14" t="n">
-        <v>72.15000000000001</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>70.81999999999999</v>
+        <v>68.39</v>
       </c>
       <c r="I14" t="n">
-        <v>71.92</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>49.27</v>
+        <v>52.8</v>
       </c>
       <c r="K14" t="n">
-        <v>50.24</v>
+        <v>54.39</v>
       </c>
       <c r="L14" t="n">
-        <v>48.09</v>
+        <v>51.05</v>
       </c>
       <c r="M14" t="n">
-        <v>49.02</v>
+        <v>51.83</v>
       </c>
       <c r="N14" t="n">
-        <v>38.77</v>
+        <v>40.09</v>
       </c>
       <c r="O14" t="n">
-        <v>39.09</v>
+        <v>40.43</v>
       </c>
       <c r="P14" t="n">
-        <v>38.37</v>
+        <v>39.63</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.51</v>
+        <v>39.71</v>
       </c>
       <c r="R14" t="n">
-        <v>1.3023</v>
+        <v>0.4154</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.2676</v>
+        <v>-4.4818</v>
       </c>
       <c r="T14" t="n">
-        <v>1.4664</v>
+        <v>-8.790699999999999</v>
       </c>
       <c r="U14" t="n">
-        <v>0.0974</v>
+        <v>0.6508</v>
       </c>
       <c r="V14" t="n">
-        <v>2.0576</v>
+        <v>-3.1315</v>
       </c>
       <c r="W14" t="n">
-        <v>4.2168</v>
+        <v>-1.2346</v>
       </c>
       <c r="X14" t="n">
-        <v>-1.6058</v>
+        <v>-0.7468</v>
       </c>
       <c r="Y14" t="n">
-        <v>1.9339</v>
+        <v>4.0345</v>
       </c>
       <c r="Z14" t="n">
-        <v>-3.4089</v>
+        <v>7.7771</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.07779999999999999</v>
+        <v>-0.6505</v>
       </c>
       <c r="AB14" t="n">
-        <v>-2.2092</v>
+        <v>3.0358</v>
       </c>
       <c r="AC14" t="n">
-        <v>-4.1801</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>106.36</v>
+        <v>103</v>
       </c>
       <c r="C15" t="n">
-        <v>108.64</v>
+        <v>107.49</v>
       </c>
       <c r="D15" t="n">
-        <v>102.31</v>
+        <v>98.62</v>
       </c>
       <c r="E15" t="n">
-        <v>105.91</v>
+        <v>106.74</v>
       </c>
       <c r="F15" t="n">
-        <v>69.06999999999999</v>
+        <v>70.06</v>
       </c>
       <c r="G15" t="n">
-        <v>70.55</v>
+        <v>72.42</v>
       </c>
       <c r="H15" t="n">
-        <v>68.25</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>69.15000000000001</v>
+        <v>72.03</v>
       </c>
       <c r="J15" t="n">
-        <v>51.88</v>
+        <v>53.5</v>
       </c>
       <c r="K15" t="n">
-        <v>53.69</v>
+        <v>55.69</v>
       </c>
       <c r="L15" t="n">
-        <v>50.9</v>
+        <v>51.28</v>
       </c>
       <c r="M15" t="n">
-        <v>52.22</v>
+        <v>51.6</v>
       </c>
       <c r="N15" t="n">
-        <v>40.03</v>
+        <v>39.49</v>
       </c>
       <c r="O15" t="n">
-        <v>40.47</v>
+        <v>39.68</v>
       </c>
       <c r="P15" t="n">
-        <v>39.23</v>
+        <v>38.12</v>
       </c>
       <c r="Q15" t="n">
-        <v>39.97</v>
+        <v>38.34</v>
       </c>
       <c r="R15" t="n">
-        <v>-6.0998</v>
+        <v>0.3667</v>
       </c>
       <c r="S15" t="n">
-        <v>-13.9293</v>
+        <v>-5.364</v>
       </c>
       <c r="T15" t="n">
-        <v>-8.437799999999999</v>
+        <v>-13.2548</v>
       </c>
       <c r="U15" t="n">
-        <v>-3.8515</v>
+        <v>3.4914</v>
       </c>
       <c r="V15" t="n">
-        <v>-5.6617</v>
+        <v>0.1529</v>
       </c>
       <c r="W15" t="n">
-        <v>-1.5939</v>
+        <v>-1.7326</v>
       </c>
       <c r="X15" t="n">
-        <v>6.5279</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y15" t="n">
-        <v>15.1488</v>
+        <v>5.2632</v>
       </c>
       <c r="Z15" t="n">
-        <v>7.848</v>
+        <v>13.7817</v>
       </c>
       <c r="AA15" t="n">
-        <v>3.7912</v>
+        <v>-3.45</v>
       </c>
       <c r="AB15" t="n">
-        <v>5.7967</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.2924</v>
+        <v>1.4823</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>104.5</v>
+        <v>111.22</v>
       </c>
       <c r="C16" t="n">
-        <v>108.07</v>
+        <v>118.18</v>
       </c>
       <c r="D16" t="n">
-        <v>101.34</v>
+        <v>109.73</v>
       </c>
       <c r="E16" t="n">
-        <v>106.35</v>
+        <v>117.28</v>
       </c>
       <c r="F16" t="n">
-        <v>68.97</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>69.76000000000001</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>68.39</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>69.59999999999999</v>
+        <v>72.37</v>
       </c>
       <c r="J16" t="n">
-        <v>52.8</v>
+        <v>49.56</v>
       </c>
       <c r="K16" t="n">
-        <v>54.39</v>
+        <v>50.21</v>
       </c>
       <c r="L16" t="n">
-        <v>51.05</v>
+        <v>46.1</v>
       </c>
       <c r="M16" t="n">
-        <v>51.83</v>
+        <v>46.34</v>
       </c>
       <c r="N16" t="n">
-        <v>40.09</v>
+        <v>38.12</v>
       </c>
       <c r="O16" t="n">
-        <v>40.43</v>
+        <v>38.58</v>
       </c>
       <c r="P16" t="n">
-        <v>39.63</v>
+        <v>37.72</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.71</v>
+        <v>38.18</v>
       </c>
       <c r="R16" t="n">
-        <v>0.4154</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S16" t="n">
-        <v>-4.4818</v>
+        <v>10.7355</v>
       </c>
       <c r="T16" t="n">
-        <v>-8.790699999999999</v>
+        <v>5.335</v>
       </c>
       <c r="U16" t="n">
-        <v>0.6508</v>
+        <v>0.472</v>
       </c>
       <c r="V16" t="n">
-        <v>-3.1315</v>
+        <v>4.6565</v>
       </c>
       <c r="W16" t="n">
-        <v>-1.2346</v>
+        <v>0.7237</v>
       </c>
       <c r="X16" t="n">
-        <v>-0.7468</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y16" t="n">
-        <v>4.0345</v>
+        <v>-11.2601</v>
       </c>
       <c r="Z16" t="n">
-        <v>7.7771</v>
+        <v>-6.9851</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.6505</v>
+        <v>-0.4173</v>
       </c>
       <c r="AB16" t="n">
-        <v>3.0358</v>
+        <v>-4.4784</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.838</v>
+        <v>-0.9341</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>103</v>
+        <v>125.12</v>
       </c>
       <c r="C17" t="n">
-        <v>107.49</v>
+        <v>127.54</v>
       </c>
       <c r="D17" t="n">
-        <v>98.62</v>
+        <v>121.6</v>
       </c>
       <c r="E17" t="n">
-        <v>106.74</v>
+        <v>123.27</v>
       </c>
       <c r="F17" t="n">
-        <v>70.06</v>
+        <v>72.95</v>
       </c>
       <c r="G17" t="n">
-        <v>72.42</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>69.70999999999999</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>72.03</v>
+        <v>72.16</v>
       </c>
       <c r="J17" t="n">
-        <v>53.5</v>
+        <v>43.55</v>
       </c>
       <c r="K17" t="n">
-        <v>55.69</v>
+        <v>44.83</v>
       </c>
       <c r="L17" t="n">
-        <v>51.28</v>
+        <v>42.51</v>
       </c>
       <c r="M17" t="n">
-        <v>51.6</v>
+        <v>44.08</v>
       </c>
       <c r="N17" t="n">
-        <v>39.49</v>
+        <v>37.89</v>
       </c>
       <c r="O17" t="n">
-        <v>39.68</v>
+        <v>38.74</v>
       </c>
       <c r="P17" t="n">
-        <v>38.12</v>
+        <v>37.75</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.34</v>
+        <v>38.31</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3667</v>
+        <v>5.1074</v>
       </c>
       <c r="S17" t="n">
-        <v>-5.364</v>
+        <v>15.9097</v>
       </c>
       <c r="T17" t="n">
-        <v>-13.2548</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U17" t="n">
-        <v>3.4914</v>
+        <v>-0.2902</v>
       </c>
       <c r="V17" t="n">
-        <v>0.1529</v>
+        <v>3.6782</v>
       </c>
       <c r="W17" t="n">
-        <v>-1.7326</v>
+        <v>0.3337</v>
       </c>
       <c r="X17" t="n">
-        <v>-0.4438</v>
+        <v>-4.877</v>
       </c>
       <c r="Y17" t="n">
-        <v>5.2632</v>
+        <v>-14.9527</v>
       </c>
       <c r="Z17" t="n">
-        <v>13.7817</v>
+        <v>-10.0775</v>
       </c>
       <c r="AA17" t="n">
-        <v>-3.45</v>
+        <v>0.3405</v>
       </c>
       <c r="AB17" t="n">
-        <v>-0.4414</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.4823</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>111.22</v>
+        <v>121.24</v>
       </c>
       <c r="C18" t="n">
-        <v>118.18</v>
+        <v>128.48</v>
       </c>
       <c r="D18" t="n">
-        <v>109.73</v>
+        <v>121.24</v>
       </c>
       <c r="E18" t="n">
-        <v>117.28</v>
+        <v>125.87</v>
       </c>
       <c r="F18" t="n">
-        <v>72.48999999999999</v>
+        <v>71.55</v>
       </c>
       <c r="G18" t="n">
-        <v>73.23999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="H18" t="n">
-        <v>71.65000000000001</v>
+        <v>70.84</v>
       </c>
       <c r="I18" t="n">
-        <v>72.37</v>
+        <v>71.55</v>
       </c>
       <c r="J18" t="n">
-        <v>49.56</v>
+        <v>44.8</v>
       </c>
       <c r="K18" t="n">
-        <v>50.21</v>
+        <v>44.82</v>
       </c>
       <c r="L18" t="n">
-        <v>46.1</v>
+        <v>42.32</v>
       </c>
       <c r="M18" t="n">
-        <v>46.34</v>
+        <v>43.24</v>
       </c>
       <c r="N18" t="n">
-        <v>38.12</v>
+        <v>38.63</v>
       </c>
       <c r="O18" t="n">
-        <v>38.58</v>
+        <v>39.01</v>
       </c>
       <c r="P18" t="n">
-        <v>37.72</v>
+        <v>38.1</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.18</v>
+        <v>38.64</v>
       </c>
       <c r="R18" t="n">
-        <v>9.874499999999999</v>
+        <v>2.1092</v>
       </c>
       <c r="S18" t="n">
-        <v>10.7355</v>
+        <v>17.9221</v>
       </c>
       <c r="T18" t="n">
-        <v>5.335</v>
+        <v>18.8462</v>
       </c>
       <c r="U18" t="n">
-        <v>0.472</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V18" t="n">
-        <v>4.6565</v>
+        <v>-0.6664</v>
       </c>
       <c r="W18" t="n">
-        <v>0.7237</v>
+        <v>3.4707</v>
       </c>
       <c r="X18" t="n">
-        <v>-10.1938</v>
+        <v>-1.9056</v>
       </c>
       <c r="Y18" t="n">
-        <v>-11.2601</v>
+        <v>-16.2016</v>
       </c>
       <c r="Z18" t="n">
-        <v>-6.9851</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA18" t="n">
-        <v>-0.4173</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AB18" t="n">
-        <v>-4.4784</v>
+        <v>0.7825</v>
       </c>
       <c r="AC18" t="n">
-        <v>-0.9341</v>
+        <v>-3.3275</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>125.12</v>
+        <v>116.35</v>
       </c>
       <c r="C19" t="n">
-        <v>127.54</v>
+        <v>119.32</v>
       </c>
       <c r="D19" t="n">
-        <v>121.6</v>
+        <v>113.55</v>
       </c>
       <c r="E19" t="n">
-        <v>123.27</v>
+        <v>115.76</v>
       </c>
       <c r="F19" t="n">
-        <v>72.95</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>73.20999999999999</v>
+        <v>70.23</v>
       </c>
       <c r="H19" t="n">
-        <v>71.31999999999999</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>72.16</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>43.55</v>
+        <v>46.52</v>
       </c>
       <c r="K19" t="n">
-        <v>44.83</v>
+        <v>47.49</v>
       </c>
       <c r="L19" t="n">
-        <v>42.51</v>
+        <v>45.5</v>
       </c>
       <c r="M19" t="n">
-        <v>44.08</v>
+        <v>46.74</v>
       </c>
       <c r="N19" t="n">
-        <v>37.89</v>
+        <v>40.08</v>
       </c>
       <c r="O19" t="n">
-        <v>38.74</v>
+        <v>40.19</v>
       </c>
       <c r="P19" t="n">
-        <v>37.75</v>
+        <v>39.35</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.31</v>
+        <v>39.9</v>
       </c>
       <c r="R19" t="n">
-        <v>5.1074</v>
+        <v>-8.0321</v>
       </c>
       <c r="S19" t="n">
-        <v>15.9097</v>
+        <v>-1.296</v>
       </c>
       <c r="T19" t="n">
-        <v>9.291600000000001</v>
+        <v>8.848100000000001</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.2902</v>
+        <v>-3.2704</v>
       </c>
       <c r="V19" t="n">
-        <v>3.6782</v>
+        <v>-4.3665</v>
       </c>
       <c r="W19" t="n">
-        <v>0.3337</v>
+        <v>-0.5603</v>
       </c>
       <c r="X19" t="n">
-        <v>-4.877</v>
+        <v>8.0944</v>
       </c>
       <c r="Y19" t="n">
-        <v>-14.9527</v>
+        <v>0.8632</v>
       </c>
       <c r="Z19" t="n">
-        <v>-10.0775</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.3405</v>
+        <v>3.2609</v>
       </c>
       <c r="AB19" t="n">
-        <v>-3.5256</v>
+        <v>4.505</v>
       </c>
       <c r="AC19" t="n">
-        <v>-0.5193</v>
+        <v>0.4785</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>121.24</v>
+        <v>120.71</v>
       </c>
       <c r="C20" t="n">
-        <v>128.48</v>
+        <v>124.5</v>
       </c>
       <c r="D20" t="n">
-        <v>121.24</v>
+        <v>117.87</v>
       </c>
       <c r="E20" t="n">
-        <v>125.87</v>
+        <v>121.82</v>
       </c>
       <c r="F20" t="n">
-        <v>71.55</v>
+        <v>71.19</v>
       </c>
       <c r="G20" t="n">
-        <v>72.55</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>70.84</v>
+        <v>70.61</v>
       </c>
       <c r="I20" t="n">
-        <v>71.55</v>
+        <v>70.98</v>
       </c>
       <c r="J20" t="n">
-        <v>44.8</v>
+        <v>44.69</v>
       </c>
       <c r="K20" t="n">
-        <v>44.82</v>
+        <v>45.82</v>
       </c>
       <c r="L20" t="n">
-        <v>42.32</v>
+        <v>43.12</v>
       </c>
       <c r="M20" t="n">
-        <v>43.24</v>
+        <v>44.14</v>
       </c>
       <c r="N20" t="n">
-        <v>38.63</v>
+        <v>38.77</v>
       </c>
       <c r="O20" t="n">
-        <v>39.01</v>
+        <v>39.1</v>
       </c>
       <c r="P20" t="n">
-        <v>38.1</v>
+        <v>38.42</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.64</v>
+        <v>38.87</v>
       </c>
       <c r="R20" t="n">
-        <v>2.1092</v>
+        <v>5.235</v>
       </c>
       <c r="S20" t="n">
-        <v>17.9221</v>
+        <v>-1.1763</v>
       </c>
       <c r="T20" t="n">
-        <v>18.8462</v>
+        <v>14.1278</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.8453000000000001</v>
+        <v>2.5574</v>
       </c>
       <c r="V20" t="n">
-        <v>-0.6664</v>
+        <v>-1.6353</v>
       </c>
       <c r="W20" t="n">
-        <v>3.4707</v>
+        <v>-1.4577</v>
       </c>
       <c r="X20" t="n">
-        <v>-1.9056</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y20" t="n">
-        <v>-16.2016</v>
+        <v>0.1361</v>
       </c>
       <c r="Z20" t="n">
-        <v>-17.1965</v>
+        <v>-14.4574</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.8614000000000001</v>
+        <v>-2.5815</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.7825</v>
+        <v>1.4618</v>
       </c>
       <c r="AC20" t="n">
-        <v>-3.3275</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>116.35</v>
-      </c>
-      <c r="C21" t="n">
-        <v>119.32</v>
-      </c>
-      <c r="D21" t="n">
-        <v>113.55</v>
-      </c>
-      <c r="E21" t="n">
-        <v>115.76</v>
-      </c>
-      <c r="F21" t="n">
-        <v>68.90000000000001</v>
-      </c>
-      <c r="G21" t="n">
-        <v>70.23</v>
-      </c>
-      <c r="H21" t="n">
-        <v>68.68000000000001</v>
-      </c>
-      <c r="I21" t="n">
-        <v>69.20999999999999</v>
-      </c>
-      <c r="J21" t="n">
-        <v>46.52</v>
-      </c>
-      <c r="K21" t="n">
-        <v>47.49</v>
-      </c>
-      <c r="L21" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="M21" t="n">
-        <v>46.74</v>
-      </c>
-      <c r="N21" t="n">
-        <v>40.08</v>
-      </c>
-      <c r="O21" t="n">
-        <v>40.19</v>
-      </c>
-      <c r="P21" t="n">
-        <v>39.35</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="R21" t="n">
-        <v>-8.0321</v>
-      </c>
-      <c r="S21" t="n">
-        <v>-1.296</v>
-      </c>
-      <c r="T21" t="n">
-        <v>8.848100000000001</v>
-      </c>
-      <c r="U21" t="n">
-        <v>-3.2704</v>
-      </c>
-      <c r="V21" t="n">
-        <v>-4.3665</v>
-      </c>
-      <c r="W21" t="n">
-        <v>-0.5603</v>
-      </c>
-      <c r="X21" t="n">
-        <v>8.0944</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>0.8632</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>-9.820600000000001</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>3.2609</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>4.505</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>0.4785</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>120.71</v>
-      </c>
-      <c r="C22" t="n">
-        <v>124.5</v>
-      </c>
-      <c r="D22" t="n">
-        <v>117.8656</v>
-      </c>
-      <c r="E22" t="n">
-        <v>121.82</v>
-      </c>
-      <c r="F22" t="n">
-        <v>71.18899999999999</v>
-      </c>
-      <c r="G22" t="n">
-        <v>71.76000000000001</v>
-      </c>
-      <c r="H22" t="n">
-        <v>70.6112</v>
-      </c>
-      <c r="I22" t="n">
-        <v>70.98</v>
-      </c>
-      <c r="J22" t="n">
-        <v>44.69</v>
-      </c>
-      <c r="K22" t="n">
-        <v>45.82</v>
-      </c>
-      <c r="L22" t="n">
-        <v>43.1205</v>
-      </c>
-      <c r="M22" t="n">
-        <v>44.14</v>
-      </c>
-      <c r="N22" t="n">
-        <v>38.79</v>
-      </c>
-      <c r="O22" t="n">
-        <v>39.1</v>
-      </c>
-      <c r="P22" t="n">
-        <v>38.42</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>38.87</v>
-      </c>
-      <c r="R22" t="n">
-        <v>5.235</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-1.1763</v>
-      </c>
-      <c r="T22" t="n">
-        <v>14.1278</v>
-      </c>
-      <c r="U22" t="n">
-        <v>2.5574</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-1.6353</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-1.4577</v>
-      </c>
-      <c r="X22" t="n">
-        <v>-5.5627</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>0.1361</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>-14.4574</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-2.5815</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>1.4618</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>1.3824</v>
+          <t>2026-09-14</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2237,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-15 23:59
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2191,6 +2191,181 @@
         <is>
           <t>2026-09-14</t>
         </is>
+      </c>
+      <c r="B21" t="n">
+        <v>101.53</v>
+      </c>
+      <c r="C21" t="n">
+        <v>105.39</v>
+      </c>
+      <c r="D21" t="n">
+        <v>99.87</v>
+      </c>
+      <c r="E21" t="n">
+        <v>101.13</v>
+      </c>
+      <c r="F21" t="n">
+        <v>67.53</v>
+      </c>
+      <c r="G21" t="n">
+        <v>70.39</v>
+      </c>
+      <c r="H21" t="n">
+        <v>67.34</v>
+      </c>
+      <c r="I21" t="n">
+        <v>69.27</v>
+      </c>
+      <c r="J21" t="n">
+        <v>51.61</v>
+      </c>
+      <c r="K21" t="n">
+        <v>52.22</v>
+      </c>
+      <c r="L21" t="n">
+        <v>50.21</v>
+      </c>
+      <c r="M21" t="n">
+        <v>51.73</v>
+      </c>
+      <c r="N21" t="n">
+        <v>40.78</v>
+      </c>
+      <c r="O21" t="n">
+        <v>40.88</v>
+      </c>
+      <c r="P21" t="n">
+        <v>39.21</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>39.83</v>
+      </c>
+      <c r="R21" t="n">
+        <v>-16.9841</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-19.6552</v>
+      </c>
+      <c r="T21" t="n">
+        <v>-13.7705</v>
+      </c>
+      <c r="U21" t="n">
+        <v>-2.4091</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-3.1866</v>
+      </c>
+      <c r="W21" t="n">
+        <v>-4.2835</v>
+      </c>
+      <c r="X21" t="n">
+        <v>17.1953</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>19.6346</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>11.6314</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>2.4698</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>3.0797</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>4.3216</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>104.55</v>
+      </c>
+      <c r="C22" t="n">
+        <v>105.94</v>
+      </c>
+      <c r="D22" t="n">
+        <v>100.9618</v>
+      </c>
+      <c r="E22" t="n">
+        <v>102.32</v>
+      </c>
+      <c r="F22" t="n">
+        <v>69.125</v>
+      </c>
+      <c r="G22" t="n">
+        <v>69.33</v>
+      </c>
+      <c r="H22" t="n">
+        <v>67.61</v>
+      </c>
+      <c r="I22" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="K22" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="L22" t="n">
+        <v>49.26</v>
+      </c>
+      <c r="M22" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="N22" t="n">
+        <v>39.92</v>
+      </c>
+      <c r="O22" t="n">
+        <v>40.7799</v>
+      </c>
+      <c r="P22" t="n">
+        <v>39.79</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>40.62</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1.1767</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-11.6102</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-16.9952</v>
+      </c>
+      <c r="U22" t="n">
+        <v>-1.9778</v>
+      </c>
+      <c r="V22" t="n">
+        <v>-1.8928</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-5.9035</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-1.2179</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>9.328200000000001</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>15.9256</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>1.9834</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>1.8045</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>6.0298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master system update 2026-09-17 00:09
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1720 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150.61</v>
+        <v>134.2</v>
       </c>
       <c r="C2" t="n">
-        <v>156.92</v>
+        <v>137.6</v>
       </c>
       <c r="D2" t="n">
-        <v>148.9</v>
+        <v>122.4</v>
       </c>
       <c r="E2" t="n">
-        <v>151.53</v>
+        <v>129.1</v>
       </c>
       <c r="F2" t="n">
-        <v>77.38</v>
+        <v>73.36</v>
       </c>
       <c r="G2" t="n">
-        <v>77.90000000000001</v>
+        <v>73.95999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>76.20999999999999</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>76.40000000000001</v>
+        <v>72.53</v>
       </c>
       <c r="J2" t="n">
-        <v>38.65</v>
+        <v>42.89</v>
       </c>
       <c r="K2" t="n">
-        <v>39.09</v>
+        <v>45.83</v>
       </c>
       <c r="L2" t="n">
-        <v>36.89</v>
+        <v>41.94</v>
       </c>
       <c r="M2" t="n">
-        <v>38.36</v>
+        <v>44.19</v>
       </c>
       <c r="N2" t="n">
-        <v>35.98</v>
+        <v>37.87</v>
       </c>
       <c r="O2" t="n">
-        <v>36.51</v>
+        <v>38.53</v>
       </c>
       <c r="P2" t="n">
-        <v>35.72</v>
+        <v>37.59</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.42</v>
+        <v>38.28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>134.2</v>
+        <v>132.63</v>
       </c>
       <c r="C3" t="n">
-        <v>137.6</v>
+        <v>133.74</v>
       </c>
       <c r="D3" t="n">
-        <v>122.4</v>
+        <v>116.84</v>
       </c>
       <c r="E3" t="n">
-        <v>129.1</v>
+        <v>120.74</v>
       </c>
       <c r="F3" t="n">
-        <v>73.36</v>
+        <v>73.37</v>
       </c>
       <c r="G3" t="n">
-        <v>73.95999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="H3" t="n">
-        <v>72.01000000000001</v>
+        <v>71</v>
       </c>
       <c r="I3" t="n">
-        <v>72.53</v>
+        <v>72.06</v>
       </c>
       <c r="J3" t="n">
-        <v>42.89</v>
+        <v>42.83</v>
       </c>
       <c r="K3" t="n">
-        <v>45.83</v>
+        <v>48.34</v>
       </c>
       <c r="L3" t="n">
-        <v>41.94</v>
+        <v>42.48</v>
       </c>
       <c r="M3" t="n">
-        <v>44.19</v>
+        <v>47.05</v>
       </c>
       <c r="N3" t="n">
-        <v>37.87</v>
+        <v>37.83</v>
       </c>
       <c r="O3" t="n">
+        <v>39.08</v>
+      </c>
+      <c r="P3" t="n">
+        <v>37.66</v>
+      </c>
+      <c r="Q3" t="n">
         <v>38.53</v>
       </c>
-      <c r="P3" t="n">
-        <v>37.59</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>38.28</v>
-      </c>
       <c r="R3" t="n">
-        <v>-14.8023</v>
+        <v>-6.4756</v>
       </c>
       <c r="U3" t="n">
-        <v>-5.0654</v>
+        <v>-0.648</v>
       </c>
       <c r="X3" t="n">
-        <v>15.1981</v>
+        <v>6.4721</v>
       </c>
       <c r="AA3" t="n">
-        <v>5.1071</v>
+        <v>0.6531</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>132.63</v>
+        <v>119.99</v>
       </c>
       <c r="C4" t="n">
-        <v>133.74</v>
+        <v>124.56</v>
       </c>
       <c r="D4" t="n">
-        <v>116.84</v>
+        <v>117.42</v>
       </c>
       <c r="E4" t="n">
-        <v>120.74</v>
+        <v>122.21</v>
       </c>
       <c r="F4" t="n">
-        <v>73.37</v>
+        <v>70.83</v>
       </c>
       <c r="G4" t="n">
-        <v>73.7</v>
+        <v>71.69</v>
       </c>
       <c r="H4" t="n">
-        <v>71</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>72.06</v>
+        <v>70.48</v>
       </c>
       <c r="J4" t="n">
-        <v>42.83</v>
+        <v>47.33</v>
       </c>
       <c r="K4" t="n">
-        <v>48.34</v>
+        <v>48.29</v>
       </c>
       <c r="L4" t="n">
-        <v>42.48</v>
+        <v>45.47</v>
       </c>
       <c r="M4" t="n">
-        <v>47.05</v>
+        <v>46.25</v>
       </c>
       <c r="N4" t="n">
-        <v>37.83</v>
+        <v>39.18</v>
       </c>
       <c r="O4" t="n">
-        <v>39.08</v>
+        <v>39.77</v>
       </c>
       <c r="P4" t="n">
-        <v>37.66</v>
+        <v>38.74</v>
       </c>
       <c r="Q4" t="n">
-        <v>38.53</v>
+        <v>39.37</v>
       </c>
       <c r="R4" t="n">
-        <v>-6.4756</v>
+        <v>1.2175</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.648</v>
+        <v>-2.1926</v>
       </c>
       <c r="X4" t="n">
-        <v>6.4721</v>
+        <v>-1.7003</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.6531</v>
+        <v>2.1801</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>119.99</v>
+        <v>126.59</v>
       </c>
       <c r="C5" t="n">
-        <v>124.56</v>
+        <v>126.79</v>
       </c>
       <c r="D5" t="n">
-        <v>117.42</v>
+        <v>116.71</v>
       </c>
       <c r="E5" t="n">
-        <v>122.21</v>
+        <v>120.6</v>
       </c>
       <c r="F5" t="n">
-        <v>70.83</v>
+        <v>71.7</v>
       </c>
       <c r="G5" t="n">
-        <v>71.69</v>
+        <v>71.83</v>
       </c>
       <c r="H5" t="n">
-        <v>69.76000000000001</v>
+        <v>69.91</v>
       </c>
       <c r="I5" t="n">
-        <v>70.48</v>
+        <v>71.17</v>
       </c>
       <c r="J5" t="n">
-        <v>47.33</v>
+        <v>44.67</v>
       </c>
       <c r="K5" t="n">
-        <v>48.29</v>
+        <v>48.46</v>
       </c>
       <c r="L5" t="n">
-        <v>45.47</v>
+        <v>44.65</v>
       </c>
       <c r="M5" t="n">
-        <v>46.25</v>
+        <v>47.03</v>
       </c>
       <c r="N5" t="n">
-        <v>39.18</v>
+        <v>38.71</v>
       </c>
       <c r="O5" t="n">
-        <v>39.77</v>
+        <v>39.72</v>
       </c>
       <c r="P5" t="n">
-        <v>38.74</v>
+        <v>38.64</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.37</v>
+        <v>39.02</v>
       </c>
       <c r="R5" t="n">
-        <v>1.2175</v>
+        <v>-1.3174</v>
       </c>
       <c r="S5" t="n">
-        <v>-19.3493</v>
+        <v>-6.584</v>
       </c>
       <c r="U5" t="n">
-        <v>-2.1926</v>
+        <v>0.979</v>
       </c>
       <c r="V5" t="n">
-        <v>-7.7487</v>
+        <v>-1.8751</v>
       </c>
       <c r="X5" t="n">
-        <v>-1.7003</v>
+        <v>1.6865</v>
       </c>
       <c r="Y5" t="n">
-        <v>20.5683</v>
+        <v>6.4268</v>
       </c>
       <c r="AA5" t="n">
-        <v>2.1801</v>
+        <v>-0.889</v>
       </c>
       <c r="AB5" t="n">
-        <v>8.0999</v>
+        <v>1.9331</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>126.59</v>
+        <v>115.07</v>
       </c>
       <c r="C6" t="n">
-        <v>126.79</v>
+        <v>115.07</v>
       </c>
       <c r="D6" t="n">
-        <v>116.71</v>
+        <v>106</v>
       </c>
       <c r="E6" t="n">
-        <v>120.6</v>
+        <v>111.16</v>
       </c>
       <c r="F6" t="n">
-        <v>71.7</v>
+        <v>70</v>
       </c>
       <c r="G6" t="n">
-        <v>71.83</v>
+        <v>70.05</v>
       </c>
       <c r="H6" t="n">
-        <v>69.91</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>71.17</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>44.67</v>
+        <v>49.14</v>
       </c>
       <c r="K6" t="n">
-        <v>48.46</v>
+        <v>52.81</v>
       </c>
       <c r="L6" t="n">
-        <v>44.65</v>
+        <v>49.13</v>
       </c>
       <c r="M6" t="n">
-        <v>47.03</v>
+        <v>50.75</v>
       </c>
       <c r="N6" t="n">
-        <v>38.71</v>
+        <v>39.65</v>
       </c>
       <c r="O6" t="n">
-        <v>39.72</v>
+        <v>40.79</v>
       </c>
       <c r="P6" t="n">
-        <v>38.64</v>
+        <v>39.64</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.02</v>
+        <v>40.19</v>
       </c>
       <c r="R6" t="n">
-        <v>-1.3174</v>
+        <v>-7.8275</v>
       </c>
       <c r="S6" t="n">
-        <v>-6.584</v>
+        <v>-7.9344</v>
       </c>
       <c r="U6" t="n">
-        <v>0.979</v>
+        <v>-3.035</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.8751</v>
+        <v>-4.2326</v>
       </c>
       <c r="X6" t="n">
-        <v>1.6865</v>
+        <v>7.9098</v>
       </c>
       <c r="Y6" t="n">
-        <v>6.4268</v>
+        <v>7.864</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.889</v>
+        <v>2.9985</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.9331</v>
+        <v>4.3083</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>115.07</v>
+        <v>117.37</v>
       </c>
       <c r="C7" t="n">
-        <v>115.07</v>
+        <v>119.88</v>
       </c>
       <c r="D7" t="n">
-        <v>106</v>
+        <v>113.13</v>
       </c>
       <c r="E7" t="n">
-        <v>111.16</v>
+        <v>115.67</v>
       </c>
       <c r="F7" t="n">
-        <v>70</v>
+        <v>70.42</v>
       </c>
       <c r="G7" t="n">
-        <v>70.05</v>
+        <v>71.27</v>
       </c>
       <c r="H7" t="n">
-        <v>67.93000000000001</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>69.01000000000001</v>
+        <v>70.27</v>
       </c>
       <c r="J7" t="n">
-        <v>49.14</v>
+        <v>47.82</v>
       </c>
       <c r="K7" t="n">
-        <v>52.81</v>
+        <v>49.83</v>
       </c>
       <c r="L7" t="n">
-        <v>49.13</v>
+        <v>46.66</v>
       </c>
       <c r="M7" t="n">
-        <v>50.75</v>
+        <v>48.42</v>
       </c>
       <c r="N7" t="n">
-        <v>39.65</v>
+        <v>39.38</v>
       </c>
       <c r="O7" t="n">
-        <v>40.79</v>
+        <v>40.02</v>
       </c>
       <c r="P7" t="n">
-        <v>39.64</v>
+        <v>38.89</v>
       </c>
       <c r="Q7" t="n">
-        <v>40.19</v>
+        <v>39.46</v>
       </c>
       <c r="R7" t="n">
-        <v>-7.8275</v>
+        <v>4.0572</v>
       </c>
       <c r="S7" t="n">
-        <v>-7.9344</v>
+        <v>-5.3514</v>
       </c>
       <c r="T7" t="n">
-        <v>-26.6416</v>
+        <v>-10.4028</v>
       </c>
       <c r="U7" t="n">
-        <v>-3.035</v>
+        <v>1.8258</v>
       </c>
       <c r="V7" t="n">
-        <v>-4.2326</v>
+        <v>-0.298</v>
       </c>
       <c r="W7" t="n">
-        <v>-9.672800000000001</v>
+        <v>-3.116</v>
       </c>
       <c r="X7" t="n">
-        <v>7.9098</v>
+        <v>-4.5911</v>
       </c>
       <c r="Y7" t="n">
-        <v>7.864</v>
+        <v>4.6919</v>
       </c>
       <c r="Z7" t="n">
-        <v>32.2993</v>
+        <v>9.5723</v>
       </c>
       <c r="AA7" t="n">
-        <v>2.9985</v>
+        <v>-1.8164</v>
       </c>
       <c r="AB7" t="n">
-        <v>4.3083</v>
+        <v>0.2286</v>
       </c>
       <c r="AC7" t="n">
-        <v>10.3515</v>
+        <v>3.0825</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>117.37</v>
+        <v>114.7</v>
       </c>
       <c r="C8" t="n">
-        <v>119.88</v>
+        <v>117.39</v>
       </c>
       <c r="D8" t="n">
-        <v>113.13</v>
+        <v>112.53</v>
       </c>
       <c r="E8" t="n">
-        <v>115.67</v>
+        <v>116.6</v>
       </c>
       <c r="F8" t="n">
-        <v>70.42</v>
+        <v>69.56</v>
       </c>
       <c r="G8" t="n">
-        <v>71.27</v>
+        <v>70.94</v>
       </c>
       <c r="H8" t="n">
-        <v>69.34999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="I8" t="n">
-        <v>70.27</v>
+        <v>70.47</v>
       </c>
       <c r="J8" t="n">
-        <v>47.82</v>
+        <v>49.01</v>
       </c>
       <c r="K8" t="n">
-        <v>49.83</v>
+        <v>49.89</v>
       </c>
       <c r="L8" t="n">
-        <v>46.66</v>
+        <v>47.87</v>
       </c>
       <c r="M8" t="n">
-        <v>48.42</v>
+        <v>48.09</v>
       </c>
       <c r="N8" t="n">
+        <v>39.86</v>
+      </c>
+      <c r="O8" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="P8" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="Q8" t="n">
         <v>39.38</v>
       </c>
-      <c r="O8" t="n">
-        <v>40.02</v>
-      </c>
-      <c r="P8" t="n">
-        <v>38.89</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>39.46</v>
-      </c>
       <c r="R8" t="n">
-        <v>4.0572</v>
+        <v>0.804</v>
       </c>
       <c r="S8" t="n">
-        <v>-5.3514</v>
+        <v>-3.3167</v>
       </c>
       <c r="T8" t="n">
-        <v>-10.4028</v>
+        <v>-3.4289</v>
       </c>
       <c r="U8" t="n">
-        <v>1.8258</v>
+        <v>0.2846</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.298</v>
+        <v>-0.9836</v>
       </c>
       <c r="W8" t="n">
-        <v>-3.116</v>
+        <v>-2.2065</v>
       </c>
       <c r="X8" t="n">
-        <v>-4.5911</v>
+        <v>-0.6815</v>
       </c>
       <c r="Y8" t="n">
-        <v>4.6919</v>
+        <v>2.2539</v>
       </c>
       <c r="Z8" t="n">
-        <v>9.5723</v>
+        <v>2.2104</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.8164</v>
+        <v>-0.2027</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.2286</v>
+        <v>0.9226</v>
       </c>
       <c r="AC8" t="n">
-        <v>3.0825</v>
+        <v>2.2061</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>114.7</v>
+        <v>123.4</v>
       </c>
       <c r="C9" t="n">
-        <v>117.39</v>
+        <v>124.88</v>
       </c>
       <c r="D9" t="n">
-        <v>112.53</v>
+        <v>117.69</v>
       </c>
       <c r="E9" t="n">
-        <v>116.6</v>
+        <v>123.05</v>
       </c>
       <c r="F9" t="n">
-        <v>69.56</v>
+        <v>72.09</v>
       </c>
       <c r="G9" t="n">
-        <v>70.94</v>
+        <v>73.38</v>
       </c>
       <c r="H9" t="n">
-        <v>69.44</v>
+        <v>71.38</v>
       </c>
       <c r="I9" t="n">
-        <v>70.47</v>
+        <v>73.3</v>
       </c>
       <c r="J9" t="n">
-        <v>49.01</v>
+        <v>45.42</v>
       </c>
       <c r="K9" t="n">
-        <v>49.89</v>
+        <v>47.71</v>
       </c>
       <c r="L9" t="n">
-        <v>47.87</v>
+        <v>44.71</v>
       </c>
       <c r="M9" t="n">
-        <v>48.09</v>
+        <v>45.35</v>
       </c>
       <c r="N9" t="n">
-        <v>39.86</v>
+        <v>38.46</v>
       </c>
       <c r="O9" t="n">
-        <v>39.93</v>
+        <v>38.86</v>
       </c>
       <c r="P9" t="n">
-        <v>39.09</v>
+        <v>37.73</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.38</v>
+        <v>37.78</v>
       </c>
       <c r="R9" t="n">
-        <v>0.804</v>
+        <v>5.5317</v>
       </c>
       <c r="S9" t="n">
-        <v>-3.3167</v>
+        <v>10.6963</v>
       </c>
       <c r="T9" t="n">
-        <v>-3.4289</v>
+        <v>0.6873</v>
       </c>
       <c r="U9" t="n">
-        <v>0.2846</v>
+        <v>4.0159</v>
       </c>
       <c r="V9" t="n">
-        <v>-0.9836</v>
+        <v>6.2165</v>
       </c>
       <c r="W9" t="n">
-        <v>-2.2065</v>
+        <v>4.0011</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.6815</v>
+        <v>-5.6977</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.2539</v>
+        <v>-10.6404</v>
       </c>
       <c r="Z9" t="n">
-        <v>2.2104</v>
+        <v>-1.9459</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.2027</v>
+        <v>-4.063</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.9226</v>
+        <v>-5.9965</v>
       </c>
       <c r="AC9" t="n">
-        <v>2.2061</v>
+        <v>-4.0386</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>123.4</v>
+        <v>119.92</v>
       </c>
       <c r="C10" t="n">
-        <v>124.88</v>
+        <v>121.2</v>
       </c>
       <c r="D10" t="n">
-        <v>117.69</v>
+        <v>110.21</v>
       </c>
       <c r="E10" t="n">
-        <v>123.05</v>
+        <v>111.34</v>
       </c>
       <c r="F10" t="n">
-        <v>72.09</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>73.38</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>71.38</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>73.3</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>45.42</v>
+        <v>46.61</v>
       </c>
       <c r="K10" t="n">
-        <v>47.71</v>
+        <v>50.23</v>
       </c>
       <c r="L10" t="n">
-        <v>44.71</v>
+        <v>46.15</v>
       </c>
       <c r="M10" t="n">
-        <v>45.35</v>
+        <v>49.82</v>
       </c>
       <c r="N10" t="n">
-        <v>38.46</v>
+        <v>38.02</v>
       </c>
       <c r="O10" t="n">
-        <v>38.86</v>
+        <v>38.76</v>
       </c>
       <c r="P10" t="n">
-        <v>37.73</v>
+        <v>37.33</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.78</v>
+        <v>38.54</v>
       </c>
       <c r="R10" t="n">
-        <v>5.5317</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="S10" t="n">
-        <v>10.6963</v>
+        <v>-3.7434</v>
       </c>
       <c r="T10" t="n">
-        <v>0.6873</v>
+        <v>-7.6783</v>
       </c>
       <c r="U10" t="n">
-        <v>4.0159</v>
+        <v>-1.9782</v>
       </c>
       <c r="V10" t="n">
-        <v>6.2165</v>
+        <v>2.2485</v>
       </c>
       <c r="W10" t="n">
-        <v>4.0011</v>
+        <v>0.9555</v>
       </c>
       <c r="X10" t="n">
-        <v>-5.6977</v>
+        <v>9.8567</v>
       </c>
       <c r="Y10" t="n">
-        <v>-10.6404</v>
+        <v>2.8914</v>
       </c>
       <c r="Z10" t="n">
-        <v>-1.9459</v>
+        <v>5.9324</v>
       </c>
       <c r="AA10" t="n">
-        <v>-4.063</v>
+        <v>2.0116</v>
       </c>
       <c r="AB10" t="n">
-        <v>-5.9965</v>
+        <v>-2.3315</v>
       </c>
       <c r="AC10" t="n">
-        <v>-4.0386</v>
+        <v>-1.2301</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>119.92</v>
+        <v>112.41</v>
       </c>
       <c r="C11" t="n">
-        <v>121.2</v>
+        <v>115.05</v>
       </c>
       <c r="D11" t="n">
-        <v>110.21</v>
+        <v>110.33</v>
       </c>
       <c r="E11" t="n">
-        <v>111.34</v>
+        <v>112.79</v>
       </c>
       <c r="F11" t="n">
-        <v>72.84999999999999</v>
+        <v>71.44</v>
       </c>
       <c r="G11" t="n">
-        <v>74.18000000000001</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>71.43000000000001</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>71.84999999999999</v>
+        <v>71.92</v>
       </c>
       <c r="J11" t="n">
-        <v>46.61</v>
+        <v>49.27</v>
       </c>
       <c r="K11" t="n">
-        <v>50.23</v>
+        <v>50.24</v>
       </c>
       <c r="L11" t="n">
-        <v>46.15</v>
+        <v>48.09</v>
       </c>
       <c r="M11" t="n">
-        <v>49.82</v>
+        <v>49.02</v>
       </c>
       <c r="N11" t="n">
-        <v>38.02</v>
+        <v>38.77</v>
       </c>
       <c r="O11" t="n">
-        <v>38.76</v>
+        <v>39.09</v>
       </c>
       <c r="P11" t="n">
-        <v>37.33</v>
+        <v>38.37</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.54</v>
+        <v>38.51</v>
       </c>
       <c r="R11" t="n">
-        <v>-9.516500000000001</v>
+        <v>1.3023</v>
       </c>
       <c r="S11" t="n">
-        <v>-3.7434</v>
+        <v>-3.2676</v>
       </c>
       <c r="T11" t="n">
-        <v>-7.6783</v>
+        <v>1.4664</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.9782</v>
+        <v>0.0974</v>
       </c>
       <c r="V11" t="n">
-        <v>2.2485</v>
+        <v>2.0576</v>
       </c>
       <c r="W11" t="n">
-        <v>0.9555</v>
+        <v>4.2168</v>
       </c>
       <c r="X11" t="n">
-        <v>9.8567</v>
+        <v>-1.6058</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.8914</v>
+        <v>1.9339</v>
       </c>
       <c r="Z11" t="n">
-        <v>5.9324</v>
+        <v>-3.4089</v>
       </c>
       <c r="AA11" t="n">
-        <v>2.0116</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="AB11" t="n">
-        <v>-2.3315</v>
+        <v>-2.2092</v>
       </c>
       <c r="AC11" t="n">
-        <v>-1.2301</v>
+        <v>-4.1801</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>112.41</v>
+        <v>106.36</v>
       </c>
       <c r="C12" t="n">
-        <v>115.05</v>
+        <v>108.64</v>
       </c>
       <c r="D12" t="n">
-        <v>110.33</v>
+        <v>102.31</v>
       </c>
       <c r="E12" t="n">
-        <v>112.79</v>
+        <v>105.91</v>
       </c>
       <c r="F12" t="n">
-        <v>71.44</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>72.15000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="H12" t="n">
-        <v>70.81999999999999</v>
+        <v>68.25</v>
       </c>
       <c r="I12" t="n">
-        <v>71.92</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>49.27</v>
+        <v>51.88</v>
       </c>
       <c r="K12" t="n">
-        <v>50.24</v>
+        <v>53.69</v>
       </c>
       <c r="L12" t="n">
-        <v>48.09</v>
+        <v>50.9</v>
       </c>
       <c r="M12" t="n">
-        <v>49.02</v>
+        <v>52.22</v>
       </c>
       <c r="N12" t="n">
-        <v>38.77</v>
+        <v>40.03</v>
       </c>
       <c r="O12" t="n">
-        <v>39.09</v>
+        <v>40.47</v>
       </c>
       <c r="P12" t="n">
-        <v>38.37</v>
+        <v>39.23</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.51</v>
+        <v>39.97</v>
       </c>
       <c r="R12" t="n">
-        <v>1.3023</v>
+        <v>-6.0998</v>
       </c>
       <c r="S12" t="n">
-        <v>-3.2676</v>
+        <v>-13.9293</v>
       </c>
       <c r="T12" t="n">
-        <v>1.4664</v>
+        <v>-8.437799999999999</v>
       </c>
       <c r="U12" t="n">
-        <v>0.0974</v>
+        <v>-3.8515</v>
       </c>
       <c r="V12" t="n">
-        <v>2.0576</v>
+        <v>-5.6617</v>
       </c>
       <c r="W12" t="n">
-        <v>4.2168</v>
+        <v>-1.5939</v>
       </c>
       <c r="X12" t="n">
-        <v>-1.6058</v>
+        <v>6.5279</v>
       </c>
       <c r="Y12" t="n">
-        <v>1.9339</v>
+        <v>15.1488</v>
       </c>
       <c r="Z12" t="n">
-        <v>-3.4089</v>
+        <v>7.848</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.07779999999999999</v>
+        <v>3.7912</v>
       </c>
       <c r="AB12" t="n">
-        <v>-2.2092</v>
+        <v>5.7967</v>
       </c>
       <c r="AC12" t="n">
-        <v>-4.1801</v>
+        <v>1.2924</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>106.36</v>
+        <v>104.5</v>
       </c>
       <c r="C13" t="n">
-        <v>108.64</v>
+        <v>108.07</v>
       </c>
       <c r="D13" t="n">
-        <v>102.31</v>
+        <v>101.34</v>
       </c>
       <c r="E13" t="n">
-        <v>105.91</v>
+        <v>106.35</v>
       </c>
       <c r="F13" t="n">
-        <v>69.06999999999999</v>
+        <v>68.97</v>
       </c>
       <c r="G13" t="n">
-        <v>70.55</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>68.25</v>
+        <v>68.39</v>
       </c>
       <c r="I13" t="n">
-        <v>69.15000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>51.88</v>
+        <v>52.8</v>
       </c>
       <c r="K13" t="n">
-        <v>53.69</v>
+        <v>54.39</v>
       </c>
       <c r="L13" t="n">
-        <v>50.9</v>
+        <v>51.05</v>
       </c>
       <c r="M13" t="n">
-        <v>52.22</v>
+        <v>51.83</v>
       </c>
       <c r="N13" t="n">
-        <v>40.03</v>
+        <v>40.09</v>
       </c>
       <c r="O13" t="n">
-        <v>40.47</v>
+        <v>40.43</v>
       </c>
       <c r="P13" t="n">
-        <v>39.23</v>
+        <v>39.63</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.97</v>
+        <v>39.71</v>
       </c>
       <c r="R13" t="n">
-        <v>-6.0998</v>
+        <v>0.4154</v>
       </c>
       <c r="S13" t="n">
-        <v>-13.9293</v>
+        <v>-4.4818</v>
       </c>
       <c r="T13" t="n">
-        <v>-8.437799999999999</v>
+        <v>-8.790699999999999</v>
       </c>
       <c r="U13" t="n">
-        <v>-3.8515</v>
+        <v>0.6508</v>
       </c>
       <c r="V13" t="n">
-        <v>-5.6617</v>
+        <v>-3.1315</v>
       </c>
       <c r="W13" t="n">
-        <v>-1.5939</v>
+        <v>-1.2346</v>
       </c>
       <c r="X13" t="n">
-        <v>6.5279</v>
+        <v>-0.7468</v>
       </c>
       <c r="Y13" t="n">
-        <v>15.1488</v>
+        <v>4.0345</v>
       </c>
       <c r="Z13" t="n">
-        <v>7.848</v>
+        <v>7.7771</v>
       </c>
       <c r="AA13" t="n">
-        <v>3.7912</v>
+        <v>-0.6505</v>
       </c>
       <c r="AB13" t="n">
-        <v>5.7967</v>
+        <v>3.0358</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.2924</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>104.5</v>
+        <v>103</v>
       </c>
       <c r="C14" t="n">
-        <v>108.07</v>
+        <v>107.49</v>
       </c>
       <c r="D14" t="n">
-        <v>101.34</v>
+        <v>98.62</v>
       </c>
       <c r="E14" t="n">
-        <v>106.35</v>
+        <v>106.74</v>
       </c>
       <c r="F14" t="n">
-        <v>68.97</v>
+        <v>70.06</v>
       </c>
       <c r="G14" t="n">
-        <v>69.76000000000001</v>
+        <v>72.42</v>
       </c>
       <c r="H14" t="n">
-        <v>68.39</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>69.59999999999999</v>
+        <v>72.03</v>
       </c>
       <c r="J14" t="n">
-        <v>52.8</v>
+        <v>53.5</v>
       </c>
       <c r="K14" t="n">
-        <v>54.39</v>
+        <v>55.69</v>
       </c>
       <c r="L14" t="n">
-        <v>51.05</v>
+        <v>51.28</v>
       </c>
       <c r="M14" t="n">
-        <v>51.83</v>
+        <v>51.6</v>
       </c>
       <c r="N14" t="n">
-        <v>40.09</v>
+        <v>39.49</v>
       </c>
       <c r="O14" t="n">
-        <v>40.43</v>
+        <v>39.68</v>
       </c>
       <c r="P14" t="n">
-        <v>39.63</v>
+        <v>38.12</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.71</v>
+        <v>38.34</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4154</v>
+        <v>0.3667</v>
       </c>
       <c r="S14" t="n">
-        <v>-4.4818</v>
+        <v>-5.364</v>
       </c>
       <c r="T14" t="n">
-        <v>-8.790699999999999</v>
+        <v>-13.2548</v>
       </c>
       <c r="U14" t="n">
-        <v>0.6508</v>
+        <v>3.4914</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.1315</v>
+        <v>0.1529</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.2346</v>
+        <v>-1.7326</v>
       </c>
       <c r="X14" t="n">
-        <v>-0.7468</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y14" t="n">
-        <v>4.0345</v>
+        <v>5.2632</v>
       </c>
       <c r="Z14" t="n">
-        <v>7.7771</v>
+        <v>13.7817</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.6505</v>
+        <v>-3.45</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.0358</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.838</v>
+        <v>1.4823</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>103</v>
+        <v>111.22</v>
       </c>
       <c r="C15" t="n">
-        <v>107.49</v>
+        <v>118.18</v>
       </c>
       <c r="D15" t="n">
-        <v>98.62</v>
+        <v>109.73</v>
       </c>
       <c r="E15" t="n">
-        <v>106.74</v>
+        <v>117.28</v>
       </c>
       <c r="F15" t="n">
-        <v>70.06</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>72.42</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>69.70999999999999</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>72.03</v>
+        <v>72.37</v>
       </c>
       <c r="J15" t="n">
-        <v>53.5</v>
+        <v>49.56</v>
       </c>
       <c r="K15" t="n">
-        <v>55.69</v>
+        <v>50.21</v>
       </c>
       <c r="L15" t="n">
-        <v>51.28</v>
+        <v>46.1</v>
       </c>
       <c r="M15" t="n">
-        <v>51.6</v>
+        <v>46.34</v>
       </c>
       <c r="N15" t="n">
-        <v>39.49</v>
+        <v>38.12</v>
       </c>
       <c r="O15" t="n">
-        <v>39.68</v>
+        <v>38.58</v>
       </c>
       <c r="P15" t="n">
-        <v>38.12</v>
+        <v>37.72</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.34</v>
+        <v>38.18</v>
       </c>
       <c r="R15" t="n">
-        <v>0.3667</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S15" t="n">
-        <v>-5.364</v>
+        <v>10.7355</v>
       </c>
       <c r="T15" t="n">
-        <v>-13.2548</v>
+        <v>5.335</v>
       </c>
       <c r="U15" t="n">
-        <v>3.4914</v>
+        <v>0.472</v>
       </c>
       <c r="V15" t="n">
-        <v>0.1529</v>
+        <v>4.6565</v>
       </c>
       <c r="W15" t="n">
-        <v>-1.7326</v>
+        <v>0.7237</v>
       </c>
       <c r="X15" t="n">
-        <v>-0.4438</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y15" t="n">
-        <v>5.2632</v>
+        <v>-11.2601</v>
       </c>
       <c r="Z15" t="n">
-        <v>13.7817</v>
+        <v>-6.9851</v>
       </c>
       <c r="AA15" t="n">
-        <v>-3.45</v>
+        <v>-0.4173</v>
       </c>
       <c r="AB15" t="n">
-        <v>-0.4414</v>
+        <v>-4.4784</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.4823</v>
+        <v>-0.9341</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>111.22</v>
+        <v>125.12</v>
       </c>
       <c r="C16" t="n">
-        <v>118.18</v>
+        <v>127.54</v>
       </c>
       <c r="D16" t="n">
-        <v>109.73</v>
+        <v>121.6</v>
       </c>
       <c r="E16" t="n">
-        <v>117.28</v>
+        <v>123.27</v>
       </c>
       <c r="F16" t="n">
-        <v>72.48999999999999</v>
+        <v>72.95</v>
       </c>
       <c r="G16" t="n">
-        <v>73.23999999999999</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>71.65000000000001</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>72.37</v>
+        <v>72.16</v>
       </c>
       <c r="J16" t="n">
-        <v>49.56</v>
+        <v>43.55</v>
       </c>
       <c r="K16" t="n">
-        <v>50.21</v>
+        <v>44.83</v>
       </c>
       <c r="L16" t="n">
-        <v>46.1</v>
+        <v>42.51</v>
       </c>
       <c r="M16" t="n">
-        <v>46.34</v>
+        <v>44.08</v>
       </c>
       <c r="N16" t="n">
-        <v>38.12</v>
+        <v>37.89</v>
       </c>
       <c r="O16" t="n">
-        <v>38.58</v>
+        <v>38.74</v>
       </c>
       <c r="P16" t="n">
-        <v>37.72</v>
+        <v>37.75</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.18</v>
+        <v>38.31</v>
       </c>
       <c r="R16" t="n">
-        <v>9.874499999999999</v>
+        <v>5.1074</v>
       </c>
       <c r="S16" t="n">
-        <v>10.7355</v>
+        <v>15.9097</v>
       </c>
       <c r="T16" t="n">
-        <v>5.335</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U16" t="n">
-        <v>0.472</v>
+        <v>-0.2902</v>
       </c>
       <c r="V16" t="n">
-        <v>4.6565</v>
+        <v>3.6782</v>
       </c>
       <c r="W16" t="n">
-        <v>0.7237</v>
+        <v>0.3337</v>
       </c>
       <c r="X16" t="n">
-        <v>-10.1938</v>
+        <v>-4.877</v>
       </c>
       <c r="Y16" t="n">
-        <v>-11.2601</v>
+        <v>-14.9527</v>
       </c>
       <c r="Z16" t="n">
-        <v>-6.9851</v>
+        <v>-10.0775</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.4173</v>
+        <v>0.3405</v>
       </c>
       <c r="AB16" t="n">
-        <v>-4.4784</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC16" t="n">
-        <v>-0.9341</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>125.12</v>
+        <v>121.24</v>
       </c>
       <c r="C17" t="n">
-        <v>127.54</v>
+        <v>128.48</v>
       </c>
       <c r="D17" t="n">
-        <v>121.6</v>
+        <v>121.24</v>
       </c>
       <c r="E17" t="n">
-        <v>123.27</v>
+        <v>125.87</v>
       </c>
       <c r="F17" t="n">
-        <v>72.95</v>
+        <v>71.55</v>
       </c>
       <c r="G17" t="n">
-        <v>73.20999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="H17" t="n">
-        <v>71.31999999999999</v>
+        <v>70.84</v>
       </c>
       <c r="I17" t="n">
-        <v>72.16</v>
+        <v>71.55</v>
       </c>
       <c r="J17" t="n">
-        <v>43.55</v>
+        <v>44.8</v>
       </c>
       <c r="K17" t="n">
-        <v>44.83</v>
+        <v>44.82</v>
       </c>
       <c r="L17" t="n">
-        <v>42.51</v>
+        <v>42.32</v>
       </c>
       <c r="M17" t="n">
-        <v>44.08</v>
+        <v>43.24</v>
       </c>
       <c r="N17" t="n">
-        <v>37.89</v>
+        <v>38.63</v>
       </c>
       <c r="O17" t="n">
-        <v>38.74</v>
+        <v>39.01</v>
       </c>
       <c r="P17" t="n">
-        <v>37.75</v>
+        <v>38.1</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.31</v>
+        <v>38.64</v>
       </c>
       <c r="R17" t="n">
-        <v>5.1074</v>
+        <v>2.1092</v>
       </c>
       <c r="S17" t="n">
-        <v>15.9097</v>
+        <v>17.9221</v>
       </c>
       <c r="T17" t="n">
-        <v>9.291600000000001</v>
+        <v>18.8462</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.2902</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V17" t="n">
-        <v>3.6782</v>
+        <v>-0.6664</v>
       </c>
       <c r="W17" t="n">
-        <v>0.3337</v>
+        <v>3.4707</v>
       </c>
       <c r="X17" t="n">
-        <v>-4.877</v>
+        <v>-1.9056</v>
       </c>
       <c r="Y17" t="n">
-        <v>-14.9527</v>
+        <v>-16.2016</v>
       </c>
       <c r="Z17" t="n">
-        <v>-10.0775</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.3405</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AB17" t="n">
-        <v>-3.5256</v>
+        <v>0.7825</v>
       </c>
       <c r="AC17" t="n">
-        <v>-0.5193</v>
+        <v>-3.3275</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>121.24</v>
+        <v>116.35</v>
       </c>
       <c r="C18" t="n">
-        <v>128.48</v>
+        <v>119.32</v>
       </c>
       <c r="D18" t="n">
-        <v>121.24</v>
+        <v>113.55</v>
       </c>
       <c r="E18" t="n">
-        <v>125.87</v>
+        <v>115.76</v>
       </c>
       <c r="F18" t="n">
-        <v>71.55</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>72.55</v>
+        <v>70.23</v>
       </c>
       <c r="H18" t="n">
-        <v>70.84</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>71.55</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>44.8</v>
+        <v>46.52</v>
       </c>
       <c r="K18" t="n">
-        <v>44.82</v>
+        <v>47.49</v>
       </c>
       <c r="L18" t="n">
-        <v>42.32</v>
+        <v>45.5</v>
       </c>
       <c r="M18" t="n">
-        <v>43.24</v>
+        <v>46.74</v>
       </c>
       <c r="N18" t="n">
-        <v>38.63</v>
+        <v>40.08</v>
       </c>
       <c r="O18" t="n">
-        <v>39.01</v>
+        <v>40.19</v>
       </c>
       <c r="P18" t="n">
-        <v>38.1</v>
+        <v>39.35</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.64</v>
+        <v>39.9</v>
       </c>
       <c r="R18" t="n">
-        <v>2.1092</v>
+        <v>-8.0321</v>
       </c>
       <c r="S18" t="n">
-        <v>17.9221</v>
+        <v>-1.296</v>
       </c>
       <c r="T18" t="n">
-        <v>18.8462</v>
+        <v>8.848100000000001</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2704</v>
       </c>
       <c r="V18" t="n">
-        <v>-0.6664</v>
+        <v>-4.3665</v>
       </c>
       <c r="W18" t="n">
-        <v>3.4707</v>
+        <v>-0.5603</v>
       </c>
       <c r="X18" t="n">
-        <v>-1.9056</v>
+        <v>8.0944</v>
       </c>
       <c r="Y18" t="n">
-        <v>-16.2016</v>
+        <v>0.8632</v>
       </c>
       <c r="Z18" t="n">
-        <v>-17.1965</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.8614000000000001</v>
+        <v>3.2609</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.7825</v>
+        <v>4.505</v>
       </c>
       <c r="AC18" t="n">
-        <v>-3.3275</v>
+        <v>0.4785</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>116.35</v>
+        <v>120.71</v>
       </c>
       <c r="C19" t="n">
-        <v>119.32</v>
+        <v>124.5</v>
       </c>
       <c r="D19" t="n">
-        <v>113.55</v>
+        <v>117.87</v>
       </c>
       <c r="E19" t="n">
-        <v>115.76</v>
+        <v>121.82</v>
       </c>
       <c r="F19" t="n">
-        <v>68.90000000000001</v>
+        <v>71.19</v>
       </c>
       <c r="G19" t="n">
-        <v>70.23</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>68.68000000000001</v>
+        <v>70.61</v>
       </c>
       <c r="I19" t="n">
-        <v>69.20999999999999</v>
+        <v>70.98</v>
       </c>
       <c r="J19" t="n">
-        <v>46.52</v>
+        <v>44.69</v>
       </c>
       <c r="K19" t="n">
-        <v>47.49</v>
+        <v>45.82</v>
       </c>
       <c r="L19" t="n">
-        <v>45.5</v>
+        <v>43.12</v>
       </c>
       <c r="M19" t="n">
-        <v>46.74</v>
+        <v>44.14</v>
       </c>
       <c r="N19" t="n">
-        <v>40.08</v>
+        <v>38.77</v>
       </c>
       <c r="O19" t="n">
-        <v>40.19</v>
+        <v>39.1</v>
       </c>
       <c r="P19" t="n">
-        <v>39.35</v>
+        <v>38.42</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.9</v>
+        <v>38.87</v>
       </c>
       <c r="R19" t="n">
-        <v>-8.0321</v>
+        <v>5.235</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.296</v>
+        <v>-1.1763</v>
       </c>
       <c r="T19" t="n">
-        <v>8.848100000000001</v>
+        <v>14.1278</v>
       </c>
       <c r="U19" t="n">
-        <v>-3.2704</v>
+        <v>2.5574</v>
       </c>
       <c r="V19" t="n">
-        <v>-4.3665</v>
+        <v>-1.6353</v>
       </c>
       <c r="W19" t="n">
-        <v>-0.5603</v>
+        <v>-1.4577</v>
       </c>
       <c r="X19" t="n">
-        <v>8.0944</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.8632</v>
+        <v>0.1361</v>
       </c>
       <c r="Z19" t="n">
-        <v>-9.820600000000001</v>
+        <v>-14.4574</v>
       </c>
       <c r="AA19" t="n">
-        <v>3.2609</v>
+        <v>-2.5815</v>
       </c>
       <c r="AB19" t="n">
-        <v>4.505</v>
+        <v>1.4618</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.4785</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>120.71</v>
+        <v>101.53</v>
       </c>
       <c r="C20" t="n">
-        <v>124.5</v>
+        <v>105.39</v>
       </c>
       <c r="D20" t="n">
-        <v>117.87</v>
+        <v>99.87</v>
       </c>
       <c r="E20" t="n">
-        <v>121.82</v>
+        <v>101.13</v>
       </c>
       <c r="F20" t="n">
-        <v>71.19</v>
+        <v>67.53</v>
       </c>
       <c r="G20" t="n">
-        <v>71.76000000000001</v>
+        <v>70.39</v>
       </c>
       <c r="H20" t="n">
-        <v>70.61</v>
+        <v>67.34</v>
       </c>
       <c r="I20" t="n">
-        <v>70.98</v>
+        <v>69.27</v>
       </c>
       <c r="J20" t="n">
-        <v>44.69</v>
+        <v>51.61</v>
       </c>
       <c r="K20" t="n">
-        <v>45.82</v>
+        <v>52.22</v>
       </c>
       <c r="L20" t="n">
-        <v>43.12</v>
+        <v>50.21</v>
       </c>
       <c r="M20" t="n">
-        <v>44.14</v>
+        <v>51.73</v>
       </c>
       <c r="N20" t="n">
-        <v>38.77</v>
+        <v>40.78</v>
       </c>
       <c r="O20" t="n">
-        <v>39.1</v>
+        <v>40.88</v>
       </c>
       <c r="P20" t="n">
-        <v>38.42</v>
+        <v>39.21</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.87</v>
+        <v>39.83</v>
       </c>
       <c r="R20" t="n">
-        <v>5.235</v>
+        <v>-16.9841</v>
       </c>
       <c r="S20" t="n">
-        <v>-1.1763</v>
+        <v>-19.6552</v>
       </c>
       <c r="T20" t="n">
-        <v>14.1278</v>
+        <v>-13.7705</v>
       </c>
       <c r="U20" t="n">
-        <v>2.5574</v>
+        <v>-2.4091</v>
       </c>
       <c r="V20" t="n">
-        <v>-1.6353</v>
+        <v>-3.1866</v>
       </c>
       <c r="W20" t="n">
-        <v>-1.4577</v>
+        <v>-4.2835</v>
       </c>
       <c r="X20" t="n">
-        <v>-5.5627</v>
+        <v>17.1953</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.1361</v>
+        <v>19.6346</v>
       </c>
       <c r="Z20" t="n">
-        <v>-14.4574</v>
+        <v>11.6314</v>
       </c>
       <c r="AA20" t="n">
-        <v>-2.5815</v>
+        <v>2.4698</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.4618</v>
+        <v>3.0797</v>
       </c>
       <c r="AC20" t="n">
-        <v>1.3824</v>
+        <v>4.3216</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>101.53</v>
+        <v>104.55</v>
       </c>
       <c r="C21" t="n">
-        <v>105.39</v>
+        <v>105.94</v>
       </c>
       <c r="D21" t="n">
-        <v>99.87</v>
+        <v>100.96</v>
       </c>
       <c r="E21" t="n">
-        <v>101.13</v>
+        <v>102.32</v>
       </c>
       <c r="F21" t="n">
-        <v>67.53</v>
+        <v>69.13</v>
       </c>
       <c r="G21" t="n">
-        <v>70.39</v>
+        <v>69.33</v>
       </c>
       <c r="H21" t="n">
-        <v>67.34</v>
+        <v>67.61</v>
       </c>
       <c r="I21" t="n">
-        <v>69.27</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>51.61</v>
+        <v>49.87</v>
       </c>
       <c r="K21" t="n">
-        <v>52.22</v>
+        <v>51.8</v>
       </c>
       <c r="L21" t="n">
-        <v>50.21</v>
+        <v>49.26</v>
       </c>
       <c r="M21" t="n">
-        <v>51.73</v>
+        <v>51.1</v>
       </c>
       <c r="N21" t="n">
+        <v>39.91</v>
+      </c>
+      <c r="O21" t="n">
         <v>40.78</v>
       </c>
-      <c r="O21" t="n">
-        <v>40.88</v>
-      </c>
       <c r="P21" t="n">
-        <v>39.21</v>
+        <v>39.79</v>
       </c>
       <c r="Q21" t="n">
-        <v>39.83</v>
+        <v>40.62</v>
       </c>
       <c r="R21" t="n">
-        <v>-16.9841</v>
+        <v>1.1767</v>
       </c>
       <c r="S21" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="T21" t="n">
-        <v>-13.7705</v>
+        <v>-16.9952</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.4091</v>
+        <v>-1.9778</v>
       </c>
       <c r="V21" t="n">
-        <v>-3.1866</v>
+        <v>-1.8928</v>
       </c>
       <c r="W21" t="n">
-        <v>-4.2835</v>
+        <v>-5.9035</v>
       </c>
       <c r="X21" t="n">
-        <v>17.1953</v>
+        <v>-1.2179</v>
       </c>
       <c r="Y21" t="n">
-        <v>19.6346</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z21" t="n">
-        <v>11.6314</v>
+        <v>15.9256</v>
       </c>
       <c r="AA21" t="n">
-        <v>2.4698</v>
+        <v>1.9834</v>
       </c>
       <c r="AB21" t="n">
-        <v>3.0797</v>
+        <v>1.8045</v>
       </c>
       <c r="AC21" t="n">
-        <v>4.3216</v>
+        <v>6.0298</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>104.55</v>
-      </c>
-      <c r="C22" t="n">
-        <v>105.94</v>
-      </c>
-      <c r="D22" t="n">
-        <v>100.9618</v>
-      </c>
-      <c r="E22" t="n">
-        <v>102.32</v>
-      </c>
-      <c r="F22" t="n">
-        <v>69.125</v>
-      </c>
-      <c r="G22" t="n">
-        <v>69.33</v>
-      </c>
-      <c r="H22" t="n">
-        <v>67.61</v>
-      </c>
-      <c r="I22" t="n">
-        <v>67.90000000000001</v>
-      </c>
-      <c r="J22" t="n">
-        <v>49.87</v>
-      </c>
-      <c r="K22" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="L22" t="n">
-        <v>49.26</v>
-      </c>
-      <c r="M22" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="N22" t="n">
-        <v>39.92</v>
-      </c>
-      <c r="O22" t="n">
-        <v>40.7799</v>
-      </c>
-      <c r="P22" t="n">
-        <v>39.79</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>40.62</v>
-      </c>
-      <c r="R22" t="n">
-        <v>1.1767</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-11.6102</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-16.9952</v>
-      </c>
-      <c r="U22" t="n">
-        <v>-1.9778</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-1.8928</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-5.9035</v>
-      </c>
-      <c r="X22" t="n">
-        <v>-1.2179</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>9.328200000000001</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>15.9256</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>1.9834</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>1.8045</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>6.0298</v>
+          <t>2026-09-16</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-17 23:56
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1720 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>134.2</v>
+        <v>132.63</v>
       </c>
       <c r="C2" t="n">
-        <v>137.6</v>
+        <v>133.74</v>
       </c>
       <c r="D2" t="n">
-        <v>122.4</v>
+        <v>116.84</v>
       </c>
       <c r="E2" t="n">
-        <v>129.1</v>
+        <v>120.74</v>
       </c>
       <c r="F2" t="n">
-        <v>73.36</v>
+        <v>73.37</v>
       </c>
       <c r="G2" t="n">
-        <v>73.95999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="H2" t="n">
-        <v>72.01000000000001</v>
+        <v>71</v>
       </c>
       <c r="I2" t="n">
-        <v>72.53</v>
+        <v>72.06</v>
       </c>
       <c r="J2" t="n">
-        <v>42.89</v>
+        <v>42.83</v>
       </c>
       <c r="K2" t="n">
-        <v>45.83</v>
+        <v>48.34</v>
       </c>
       <c r="L2" t="n">
-        <v>41.94</v>
+        <v>42.48</v>
       </c>
       <c r="M2" t="n">
-        <v>44.19</v>
+        <v>47.05</v>
       </c>
       <c r="N2" t="n">
-        <v>37.87</v>
+        <v>37.83</v>
       </c>
       <c r="O2" t="n">
+        <v>39.08</v>
+      </c>
+      <c r="P2" t="n">
+        <v>37.66</v>
+      </c>
+      <c r="Q2" t="n">
         <v>38.53</v>
-      </c>
-      <c r="P2" t="n">
-        <v>37.59</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>38.28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>132.63</v>
+        <v>119.99</v>
       </c>
       <c r="C3" t="n">
-        <v>133.74</v>
+        <v>124.56</v>
       </c>
       <c r="D3" t="n">
-        <v>116.84</v>
+        <v>117.42</v>
       </c>
       <c r="E3" t="n">
-        <v>120.74</v>
+        <v>122.21</v>
       </c>
       <c r="F3" t="n">
-        <v>73.37</v>
+        <v>70.83</v>
       </c>
       <c r="G3" t="n">
-        <v>73.7</v>
+        <v>71.69</v>
       </c>
       <c r="H3" t="n">
-        <v>71</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>72.06</v>
+        <v>70.48</v>
       </c>
       <c r="J3" t="n">
-        <v>42.83</v>
+        <v>47.33</v>
       </c>
       <c r="K3" t="n">
-        <v>48.34</v>
+        <v>48.29</v>
       </c>
       <c r="L3" t="n">
-        <v>42.48</v>
+        <v>45.47</v>
       </c>
       <c r="M3" t="n">
-        <v>47.05</v>
+        <v>46.25</v>
       </c>
       <c r="N3" t="n">
-        <v>37.83</v>
+        <v>39.18</v>
       </c>
       <c r="O3" t="n">
-        <v>39.08</v>
+        <v>39.77</v>
       </c>
       <c r="P3" t="n">
-        <v>37.66</v>
+        <v>38.74</v>
       </c>
       <c r="Q3" t="n">
-        <v>38.53</v>
+        <v>39.37</v>
       </c>
       <c r="R3" t="n">
-        <v>-6.4756</v>
+        <v>1.2175</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.648</v>
+        <v>-2.1926</v>
       </c>
       <c r="X3" t="n">
-        <v>6.4721</v>
+        <v>-1.7003</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.6531</v>
+        <v>2.1801</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>119.99</v>
+        <v>126.59</v>
       </c>
       <c r="C4" t="n">
-        <v>124.56</v>
+        <v>126.79</v>
       </c>
       <c r="D4" t="n">
-        <v>117.42</v>
+        <v>116.71</v>
       </c>
       <c r="E4" t="n">
-        <v>122.21</v>
+        <v>120.6</v>
       </c>
       <c r="F4" t="n">
-        <v>70.83</v>
+        <v>71.7</v>
       </c>
       <c r="G4" t="n">
-        <v>71.69</v>
+        <v>71.83</v>
       </c>
       <c r="H4" t="n">
-        <v>69.76000000000001</v>
+        <v>69.91</v>
       </c>
       <c r="I4" t="n">
-        <v>70.48</v>
+        <v>71.17</v>
       </c>
       <c r="J4" t="n">
-        <v>47.33</v>
+        <v>44.67</v>
       </c>
       <c r="K4" t="n">
-        <v>48.29</v>
+        <v>48.46</v>
       </c>
       <c r="L4" t="n">
-        <v>45.47</v>
+        <v>44.65</v>
       </c>
       <c r="M4" t="n">
-        <v>46.25</v>
+        <v>47.03</v>
       </c>
       <c r="N4" t="n">
-        <v>39.18</v>
+        <v>38.71</v>
       </c>
       <c r="O4" t="n">
-        <v>39.77</v>
+        <v>39.72</v>
       </c>
       <c r="P4" t="n">
-        <v>38.74</v>
+        <v>38.64</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.37</v>
+        <v>39.02</v>
       </c>
       <c r="R4" t="n">
-        <v>1.2175</v>
+        <v>-1.3174</v>
       </c>
       <c r="U4" t="n">
-        <v>-2.1926</v>
+        <v>0.979</v>
       </c>
       <c r="X4" t="n">
-        <v>-1.7003</v>
+        <v>1.6865</v>
       </c>
       <c r="AA4" t="n">
-        <v>2.1801</v>
+        <v>-0.889</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>126.59</v>
+        <v>115.07</v>
       </c>
       <c r="C5" t="n">
-        <v>126.79</v>
+        <v>115.07</v>
       </c>
       <c r="D5" t="n">
-        <v>116.71</v>
+        <v>106</v>
       </c>
       <c r="E5" t="n">
-        <v>120.6</v>
+        <v>111.16</v>
       </c>
       <c r="F5" t="n">
-        <v>71.7</v>
+        <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>71.83</v>
+        <v>70.05</v>
       </c>
       <c r="H5" t="n">
-        <v>69.91</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>71.17</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>44.67</v>
+        <v>49.14</v>
       </c>
       <c r="K5" t="n">
-        <v>48.46</v>
+        <v>52.81</v>
       </c>
       <c r="L5" t="n">
-        <v>44.65</v>
+        <v>49.13</v>
       </c>
       <c r="M5" t="n">
-        <v>47.03</v>
+        <v>50.75</v>
       </c>
       <c r="N5" t="n">
-        <v>38.71</v>
+        <v>39.65</v>
       </c>
       <c r="O5" t="n">
-        <v>39.72</v>
+        <v>40.79</v>
       </c>
       <c r="P5" t="n">
-        <v>38.64</v>
+        <v>39.64</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.02</v>
+        <v>40.19</v>
       </c>
       <c r="R5" t="n">
-        <v>-1.3174</v>
+        <v>-7.8275</v>
       </c>
       <c r="S5" t="n">
-        <v>-6.584</v>
+        <v>-7.9344</v>
       </c>
       <c r="U5" t="n">
-        <v>0.979</v>
+        <v>-3.035</v>
       </c>
       <c r="V5" t="n">
-        <v>-1.8751</v>
+        <v>-4.2326</v>
       </c>
       <c r="X5" t="n">
-        <v>1.6865</v>
+        <v>7.9098</v>
       </c>
       <c r="Y5" t="n">
-        <v>6.4268</v>
+        <v>7.864</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.889</v>
+        <v>2.9985</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.9331</v>
+        <v>4.3083</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>115.07</v>
+        <v>117.37</v>
       </c>
       <c r="C6" t="n">
-        <v>115.07</v>
+        <v>119.88</v>
       </c>
       <c r="D6" t="n">
-        <v>106</v>
+        <v>113.13</v>
       </c>
       <c r="E6" t="n">
-        <v>111.16</v>
+        <v>115.67</v>
       </c>
       <c r="F6" t="n">
-        <v>70</v>
+        <v>70.42</v>
       </c>
       <c r="G6" t="n">
-        <v>70.05</v>
+        <v>71.27</v>
       </c>
       <c r="H6" t="n">
-        <v>67.93000000000001</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>69.01000000000001</v>
+        <v>70.27</v>
       </c>
       <c r="J6" t="n">
-        <v>49.14</v>
+        <v>47.82</v>
       </c>
       <c r="K6" t="n">
-        <v>52.81</v>
+        <v>49.83</v>
       </c>
       <c r="L6" t="n">
-        <v>49.13</v>
+        <v>46.66</v>
       </c>
       <c r="M6" t="n">
-        <v>50.75</v>
+        <v>48.42</v>
       </c>
       <c r="N6" t="n">
-        <v>39.65</v>
+        <v>39.38</v>
       </c>
       <c r="O6" t="n">
-        <v>40.79</v>
+        <v>40.02</v>
       </c>
       <c r="P6" t="n">
-        <v>39.64</v>
+        <v>38.89</v>
       </c>
       <c r="Q6" t="n">
-        <v>40.19</v>
+        <v>39.46</v>
       </c>
       <c r="R6" t="n">
-        <v>-7.8275</v>
+        <v>4.0572</v>
       </c>
       <c r="S6" t="n">
-        <v>-7.9344</v>
+        <v>-5.3514</v>
       </c>
       <c r="U6" t="n">
-        <v>-3.035</v>
+        <v>1.8258</v>
       </c>
       <c r="V6" t="n">
-        <v>-4.2326</v>
+        <v>-0.298</v>
       </c>
       <c r="X6" t="n">
-        <v>7.9098</v>
+        <v>-4.5911</v>
       </c>
       <c r="Y6" t="n">
-        <v>7.864</v>
+        <v>4.6919</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.9985</v>
+        <v>-1.8164</v>
       </c>
       <c r="AB6" t="n">
-        <v>4.3083</v>
+        <v>0.2286</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>117.37</v>
+        <v>114.7</v>
       </c>
       <c r="C7" t="n">
-        <v>119.88</v>
+        <v>117.39</v>
       </c>
       <c r="D7" t="n">
-        <v>113.13</v>
+        <v>112.53</v>
       </c>
       <c r="E7" t="n">
-        <v>115.67</v>
+        <v>116.6</v>
       </c>
       <c r="F7" t="n">
-        <v>70.42</v>
+        <v>69.56</v>
       </c>
       <c r="G7" t="n">
-        <v>71.27</v>
+        <v>70.94</v>
       </c>
       <c r="H7" t="n">
-        <v>69.34999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="I7" t="n">
-        <v>70.27</v>
+        <v>70.47</v>
       </c>
       <c r="J7" t="n">
-        <v>47.82</v>
+        <v>49.01</v>
       </c>
       <c r="K7" t="n">
-        <v>49.83</v>
+        <v>49.89</v>
       </c>
       <c r="L7" t="n">
-        <v>46.66</v>
+        <v>47.87</v>
       </c>
       <c r="M7" t="n">
-        <v>48.42</v>
+        <v>48.09</v>
       </c>
       <c r="N7" t="n">
+        <v>39.86</v>
+      </c>
+      <c r="O7" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="P7" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="Q7" t="n">
         <v>39.38</v>
       </c>
-      <c r="O7" t="n">
-        <v>40.02</v>
-      </c>
-      <c r="P7" t="n">
-        <v>38.89</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>39.46</v>
-      </c>
       <c r="R7" t="n">
-        <v>4.0572</v>
+        <v>0.804</v>
       </c>
       <c r="S7" t="n">
-        <v>-5.3514</v>
+        <v>-3.3167</v>
       </c>
       <c r="T7" t="n">
-        <v>-10.4028</v>
+        <v>-3.4289</v>
       </c>
       <c r="U7" t="n">
-        <v>1.8258</v>
+        <v>0.2846</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.298</v>
+        <v>-0.9836</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.116</v>
+        <v>-2.2065</v>
       </c>
       <c r="X7" t="n">
-        <v>-4.5911</v>
+        <v>-0.6815</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.6919</v>
+        <v>2.2539</v>
       </c>
       <c r="Z7" t="n">
-        <v>9.5723</v>
+        <v>2.2104</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.8164</v>
+        <v>-0.2027</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.2286</v>
+        <v>0.9226</v>
       </c>
       <c r="AC7" t="n">
-        <v>3.0825</v>
+        <v>2.2061</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>114.7</v>
+        <v>123.4</v>
       </c>
       <c r="C8" t="n">
-        <v>117.39</v>
+        <v>124.88</v>
       </c>
       <c r="D8" t="n">
-        <v>112.53</v>
+        <v>117.69</v>
       </c>
       <c r="E8" t="n">
-        <v>116.6</v>
+        <v>123.05</v>
       </c>
       <c r="F8" t="n">
-        <v>69.56</v>
+        <v>72.09</v>
       </c>
       <c r="G8" t="n">
-        <v>70.94</v>
+        <v>73.38</v>
       </c>
       <c r="H8" t="n">
-        <v>69.44</v>
+        <v>71.38</v>
       </c>
       <c r="I8" t="n">
-        <v>70.47</v>
+        <v>73.3</v>
       </c>
       <c r="J8" t="n">
-        <v>49.01</v>
+        <v>45.42</v>
       </c>
       <c r="K8" t="n">
-        <v>49.89</v>
+        <v>47.71</v>
       </c>
       <c r="L8" t="n">
-        <v>47.87</v>
+        <v>44.71</v>
       </c>
       <c r="M8" t="n">
-        <v>48.09</v>
+        <v>45.35</v>
       </c>
       <c r="N8" t="n">
-        <v>39.86</v>
+        <v>38.46</v>
       </c>
       <c r="O8" t="n">
-        <v>39.93</v>
+        <v>38.86</v>
       </c>
       <c r="P8" t="n">
-        <v>39.09</v>
+        <v>37.73</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.38</v>
+        <v>37.78</v>
       </c>
       <c r="R8" t="n">
-        <v>0.804</v>
+        <v>5.5317</v>
       </c>
       <c r="S8" t="n">
-        <v>-3.3167</v>
+        <v>10.6963</v>
       </c>
       <c r="T8" t="n">
-        <v>-3.4289</v>
+        <v>0.6873</v>
       </c>
       <c r="U8" t="n">
-        <v>0.2846</v>
+        <v>4.0159</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.9836</v>
+        <v>6.2165</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.2065</v>
+        <v>4.0011</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.6815</v>
+        <v>-5.6977</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.2539</v>
+        <v>-10.6404</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.2104</v>
+        <v>-1.9459</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.2027</v>
+        <v>-4.063</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.9226</v>
+        <v>-5.9965</v>
       </c>
       <c r="AC8" t="n">
-        <v>2.2061</v>
+        <v>-4.0386</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>123.4</v>
+        <v>119.92</v>
       </c>
       <c r="C9" t="n">
-        <v>124.88</v>
+        <v>121.2</v>
       </c>
       <c r="D9" t="n">
-        <v>117.69</v>
+        <v>110.21</v>
       </c>
       <c r="E9" t="n">
-        <v>123.05</v>
+        <v>111.34</v>
       </c>
       <c r="F9" t="n">
-        <v>72.09</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>73.38</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>71.38</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>73.3</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>45.42</v>
+        <v>46.61</v>
       </c>
       <c r="K9" t="n">
-        <v>47.71</v>
+        <v>50.23</v>
       </c>
       <c r="L9" t="n">
-        <v>44.71</v>
+        <v>46.15</v>
       </c>
       <c r="M9" t="n">
-        <v>45.35</v>
+        <v>49.82</v>
       </c>
       <c r="N9" t="n">
-        <v>38.46</v>
+        <v>38.02</v>
       </c>
       <c r="O9" t="n">
-        <v>38.86</v>
+        <v>38.76</v>
       </c>
       <c r="P9" t="n">
-        <v>37.73</v>
+        <v>37.33</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.78</v>
+        <v>38.54</v>
       </c>
       <c r="R9" t="n">
-        <v>5.5317</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="S9" t="n">
-        <v>10.6963</v>
+        <v>-3.7434</v>
       </c>
       <c r="T9" t="n">
-        <v>0.6873</v>
+        <v>-7.6783</v>
       </c>
       <c r="U9" t="n">
-        <v>4.0159</v>
+        <v>-1.9782</v>
       </c>
       <c r="V9" t="n">
-        <v>6.2165</v>
+        <v>2.2485</v>
       </c>
       <c r="W9" t="n">
-        <v>4.0011</v>
+        <v>0.9555</v>
       </c>
       <c r="X9" t="n">
-        <v>-5.6977</v>
+        <v>9.8567</v>
       </c>
       <c r="Y9" t="n">
-        <v>-10.6404</v>
+        <v>2.8914</v>
       </c>
       <c r="Z9" t="n">
-        <v>-1.9459</v>
+        <v>5.9324</v>
       </c>
       <c r="AA9" t="n">
-        <v>-4.063</v>
+        <v>2.0116</v>
       </c>
       <c r="AB9" t="n">
-        <v>-5.9965</v>
+        <v>-2.3315</v>
       </c>
       <c r="AC9" t="n">
-        <v>-4.0386</v>
+        <v>-1.2301</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>119.92</v>
+        <v>112.41</v>
       </c>
       <c r="C10" t="n">
-        <v>121.2</v>
+        <v>115.05</v>
       </c>
       <c r="D10" t="n">
-        <v>110.21</v>
+        <v>110.33</v>
       </c>
       <c r="E10" t="n">
-        <v>111.34</v>
+        <v>112.79</v>
       </c>
       <c r="F10" t="n">
-        <v>72.84999999999999</v>
+        <v>71.44</v>
       </c>
       <c r="G10" t="n">
-        <v>74.18000000000001</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>71.43000000000001</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>71.84999999999999</v>
+        <v>71.92</v>
       </c>
       <c r="J10" t="n">
-        <v>46.61</v>
+        <v>49.27</v>
       </c>
       <c r="K10" t="n">
-        <v>50.23</v>
+        <v>50.24</v>
       </c>
       <c r="L10" t="n">
-        <v>46.15</v>
+        <v>48.09</v>
       </c>
       <c r="M10" t="n">
-        <v>49.82</v>
+        <v>49.02</v>
       </c>
       <c r="N10" t="n">
-        <v>38.02</v>
+        <v>38.77</v>
       </c>
       <c r="O10" t="n">
-        <v>38.76</v>
+        <v>39.09</v>
       </c>
       <c r="P10" t="n">
-        <v>37.33</v>
+        <v>38.37</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.54</v>
+        <v>38.51</v>
       </c>
       <c r="R10" t="n">
-        <v>-9.516500000000001</v>
+        <v>1.3023</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.7434</v>
+        <v>-3.2676</v>
       </c>
       <c r="T10" t="n">
-        <v>-7.6783</v>
+        <v>1.4664</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.9782</v>
+        <v>0.0974</v>
       </c>
       <c r="V10" t="n">
-        <v>2.2485</v>
+        <v>2.0576</v>
       </c>
       <c r="W10" t="n">
-        <v>0.9555</v>
+        <v>4.2168</v>
       </c>
       <c r="X10" t="n">
-        <v>9.8567</v>
+        <v>-1.6058</v>
       </c>
       <c r="Y10" t="n">
-        <v>2.8914</v>
+        <v>1.9339</v>
       </c>
       <c r="Z10" t="n">
-        <v>5.9324</v>
+        <v>-3.4089</v>
       </c>
       <c r="AA10" t="n">
-        <v>2.0116</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2.3315</v>
+        <v>-2.2092</v>
       </c>
       <c r="AC10" t="n">
-        <v>-1.2301</v>
+        <v>-4.1801</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>112.41</v>
+        <v>106.36</v>
       </c>
       <c r="C11" t="n">
-        <v>115.05</v>
+        <v>108.64</v>
       </c>
       <c r="D11" t="n">
-        <v>110.33</v>
+        <v>102.31</v>
       </c>
       <c r="E11" t="n">
-        <v>112.79</v>
+        <v>105.91</v>
       </c>
       <c r="F11" t="n">
-        <v>71.44</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>72.15000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="H11" t="n">
-        <v>70.81999999999999</v>
+        <v>68.25</v>
       </c>
       <c r="I11" t="n">
-        <v>71.92</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>49.27</v>
+        <v>51.88</v>
       </c>
       <c r="K11" t="n">
-        <v>50.24</v>
+        <v>53.69</v>
       </c>
       <c r="L11" t="n">
-        <v>48.09</v>
+        <v>50.9</v>
       </c>
       <c r="M11" t="n">
-        <v>49.02</v>
+        <v>52.22</v>
       </c>
       <c r="N11" t="n">
-        <v>38.77</v>
+        <v>40.03</v>
       </c>
       <c r="O11" t="n">
-        <v>39.09</v>
+        <v>40.47</v>
       </c>
       <c r="P11" t="n">
-        <v>38.37</v>
+        <v>39.23</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.51</v>
+        <v>39.97</v>
       </c>
       <c r="R11" t="n">
-        <v>1.3023</v>
+        <v>-6.0998</v>
       </c>
       <c r="S11" t="n">
-        <v>-3.2676</v>
+        <v>-13.9293</v>
       </c>
       <c r="T11" t="n">
-        <v>1.4664</v>
+        <v>-8.437799999999999</v>
       </c>
       <c r="U11" t="n">
-        <v>0.0974</v>
+        <v>-3.8515</v>
       </c>
       <c r="V11" t="n">
-        <v>2.0576</v>
+        <v>-5.6617</v>
       </c>
       <c r="W11" t="n">
-        <v>4.2168</v>
+        <v>-1.5939</v>
       </c>
       <c r="X11" t="n">
-        <v>-1.6058</v>
+        <v>6.5279</v>
       </c>
       <c r="Y11" t="n">
-        <v>1.9339</v>
+        <v>15.1488</v>
       </c>
       <c r="Z11" t="n">
-        <v>-3.4089</v>
+        <v>7.848</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.07779999999999999</v>
+        <v>3.7912</v>
       </c>
       <c r="AB11" t="n">
-        <v>-2.2092</v>
+        <v>5.7967</v>
       </c>
       <c r="AC11" t="n">
-        <v>-4.1801</v>
+        <v>1.2924</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>106.36</v>
+        <v>104.5</v>
       </c>
       <c r="C12" t="n">
-        <v>108.64</v>
+        <v>108.07</v>
       </c>
       <c r="D12" t="n">
-        <v>102.31</v>
+        <v>101.34</v>
       </c>
       <c r="E12" t="n">
-        <v>105.91</v>
+        <v>106.35</v>
       </c>
       <c r="F12" t="n">
-        <v>69.06999999999999</v>
+        <v>68.97</v>
       </c>
       <c r="G12" t="n">
-        <v>70.55</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>68.25</v>
+        <v>68.39</v>
       </c>
       <c r="I12" t="n">
-        <v>69.15000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>51.88</v>
+        <v>52.8</v>
       </c>
       <c r="K12" t="n">
-        <v>53.69</v>
+        <v>54.39</v>
       </c>
       <c r="L12" t="n">
-        <v>50.9</v>
+        <v>51.05</v>
       </c>
       <c r="M12" t="n">
-        <v>52.22</v>
+        <v>51.83</v>
       </c>
       <c r="N12" t="n">
-        <v>40.03</v>
+        <v>40.09</v>
       </c>
       <c r="O12" t="n">
-        <v>40.47</v>
+        <v>40.43</v>
       </c>
       <c r="P12" t="n">
-        <v>39.23</v>
+        <v>39.63</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.97</v>
+        <v>39.71</v>
       </c>
       <c r="R12" t="n">
-        <v>-6.0998</v>
+        <v>0.4154</v>
       </c>
       <c r="S12" t="n">
-        <v>-13.9293</v>
+        <v>-4.4818</v>
       </c>
       <c r="T12" t="n">
-        <v>-8.437799999999999</v>
+        <v>-8.790699999999999</v>
       </c>
       <c r="U12" t="n">
-        <v>-3.8515</v>
+        <v>0.6508</v>
       </c>
       <c r="V12" t="n">
-        <v>-5.6617</v>
+        <v>-3.1315</v>
       </c>
       <c r="W12" t="n">
-        <v>-1.5939</v>
+        <v>-1.2346</v>
       </c>
       <c r="X12" t="n">
-        <v>6.5279</v>
+        <v>-0.7468</v>
       </c>
       <c r="Y12" t="n">
-        <v>15.1488</v>
+        <v>4.0345</v>
       </c>
       <c r="Z12" t="n">
-        <v>7.848</v>
+        <v>7.7771</v>
       </c>
       <c r="AA12" t="n">
-        <v>3.7912</v>
+        <v>-0.6505</v>
       </c>
       <c r="AB12" t="n">
-        <v>5.7967</v>
+        <v>3.0358</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.2924</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>104.5</v>
+        <v>103</v>
       </c>
       <c r="C13" t="n">
-        <v>108.07</v>
+        <v>107.49</v>
       </c>
       <c r="D13" t="n">
-        <v>101.34</v>
+        <v>98.62</v>
       </c>
       <c r="E13" t="n">
-        <v>106.35</v>
+        <v>106.74</v>
       </c>
       <c r="F13" t="n">
-        <v>68.97</v>
+        <v>70.06</v>
       </c>
       <c r="G13" t="n">
-        <v>69.76000000000001</v>
+        <v>72.42</v>
       </c>
       <c r="H13" t="n">
-        <v>68.39</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>69.59999999999999</v>
+        <v>72.03</v>
       </c>
       <c r="J13" t="n">
-        <v>52.8</v>
+        <v>53.5</v>
       </c>
       <c r="K13" t="n">
-        <v>54.39</v>
+        <v>55.69</v>
       </c>
       <c r="L13" t="n">
-        <v>51.05</v>
+        <v>51.28</v>
       </c>
       <c r="M13" t="n">
-        <v>51.83</v>
+        <v>51.6</v>
       </c>
       <c r="N13" t="n">
-        <v>40.09</v>
+        <v>39.49</v>
       </c>
       <c r="O13" t="n">
-        <v>40.43</v>
+        <v>39.68</v>
       </c>
       <c r="P13" t="n">
-        <v>39.63</v>
+        <v>38.12</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.71</v>
+        <v>38.34</v>
       </c>
       <c r="R13" t="n">
-        <v>0.4154</v>
+        <v>0.3667</v>
       </c>
       <c r="S13" t="n">
-        <v>-4.4818</v>
+        <v>-5.364</v>
       </c>
       <c r="T13" t="n">
-        <v>-8.790699999999999</v>
+        <v>-13.2548</v>
       </c>
       <c r="U13" t="n">
-        <v>0.6508</v>
+        <v>3.4914</v>
       </c>
       <c r="V13" t="n">
-        <v>-3.1315</v>
+        <v>0.1529</v>
       </c>
       <c r="W13" t="n">
-        <v>-1.2346</v>
+        <v>-1.7326</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.7468</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y13" t="n">
-        <v>4.0345</v>
+        <v>5.2632</v>
       </c>
       <c r="Z13" t="n">
-        <v>7.7771</v>
+        <v>13.7817</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.6505</v>
+        <v>-3.45</v>
       </c>
       <c r="AB13" t="n">
-        <v>3.0358</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.838</v>
+        <v>1.4823</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>103</v>
+        <v>111.22</v>
       </c>
       <c r="C14" t="n">
-        <v>107.49</v>
+        <v>118.18</v>
       </c>
       <c r="D14" t="n">
-        <v>98.62</v>
+        <v>109.73</v>
       </c>
       <c r="E14" t="n">
-        <v>106.74</v>
+        <v>117.28</v>
       </c>
       <c r="F14" t="n">
-        <v>70.06</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>72.42</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>69.70999999999999</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>72.03</v>
+        <v>72.37</v>
       </c>
       <c r="J14" t="n">
-        <v>53.5</v>
+        <v>49.56</v>
       </c>
       <c r="K14" t="n">
-        <v>55.69</v>
+        <v>50.21</v>
       </c>
       <c r="L14" t="n">
-        <v>51.28</v>
+        <v>46.1</v>
       </c>
       <c r="M14" t="n">
-        <v>51.6</v>
+        <v>46.34</v>
       </c>
       <c r="N14" t="n">
-        <v>39.49</v>
+        <v>38.12</v>
       </c>
       <c r="O14" t="n">
-        <v>39.68</v>
+        <v>38.58</v>
       </c>
       <c r="P14" t="n">
-        <v>38.12</v>
+        <v>37.72</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.34</v>
+        <v>38.18</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3667</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S14" t="n">
-        <v>-5.364</v>
+        <v>10.7355</v>
       </c>
       <c r="T14" t="n">
-        <v>-13.2548</v>
+        <v>5.335</v>
       </c>
       <c r="U14" t="n">
-        <v>3.4914</v>
+        <v>0.472</v>
       </c>
       <c r="V14" t="n">
-        <v>0.1529</v>
+        <v>4.6565</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.7326</v>
+        <v>0.7237</v>
       </c>
       <c r="X14" t="n">
-        <v>-0.4438</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y14" t="n">
-        <v>5.2632</v>
+        <v>-11.2601</v>
       </c>
       <c r="Z14" t="n">
-        <v>13.7817</v>
+        <v>-6.9851</v>
       </c>
       <c r="AA14" t="n">
-        <v>-3.45</v>
+        <v>-0.4173</v>
       </c>
       <c r="AB14" t="n">
-        <v>-0.4414</v>
+        <v>-4.4784</v>
       </c>
       <c r="AC14" t="n">
-        <v>1.4823</v>
+        <v>-0.9341</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>111.22</v>
+        <v>125.12</v>
       </c>
       <c r="C15" t="n">
-        <v>118.18</v>
+        <v>127.54</v>
       </c>
       <c r="D15" t="n">
-        <v>109.73</v>
+        <v>121.6</v>
       </c>
       <c r="E15" t="n">
-        <v>117.28</v>
+        <v>123.27</v>
       </c>
       <c r="F15" t="n">
-        <v>72.48999999999999</v>
+        <v>72.95</v>
       </c>
       <c r="G15" t="n">
-        <v>73.23999999999999</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>71.65000000000001</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>72.37</v>
+        <v>72.16</v>
       </c>
       <c r="J15" t="n">
-        <v>49.56</v>
+        <v>43.55</v>
       </c>
       <c r="K15" t="n">
-        <v>50.21</v>
+        <v>44.83</v>
       </c>
       <c r="L15" t="n">
-        <v>46.1</v>
+        <v>42.51</v>
       </c>
       <c r="M15" t="n">
-        <v>46.34</v>
+        <v>44.08</v>
       </c>
       <c r="N15" t="n">
-        <v>38.12</v>
+        <v>37.89</v>
       </c>
       <c r="O15" t="n">
-        <v>38.58</v>
+        <v>38.74</v>
       </c>
       <c r="P15" t="n">
-        <v>37.72</v>
+        <v>37.75</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.18</v>
+        <v>38.31</v>
       </c>
       <c r="R15" t="n">
-        <v>9.874499999999999</v>
+        <v>5.1074</v>
       </c>
       <c r="S15" t="n">
-        <v>10.7355</v>
+        <v>15.9097</v>
       </c>
       <c r="T15" t="n">
-        <v>5.335</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U15" t="n">
-        <v>0.472</v>
+        <v>-0.2902</v>
       </c>
       <c r="V15" t="n">
-        <v>4.6565</v>
+        <v>3.6782</v>
       </c>
       <c r="W15" t="n">
-        <v>0.7237</v>
+        <v>0.3337</v>
       </c>
       <c r="X15" t="n">
-        <v>-10.1938</v>
+        <v>-4.877</v>
       </c>
       <c r="Y15" t="n">
-        <v>-11.2601</v>
+        <v>-14.9527</v>
       </c>
       <c r="Z15" t="n">
-        <v>-6.9851</v>
+        <v>-10.0775</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.4173</v>
+        <v>0.3405</v>
       </c>
       <c r="AB15" t="n">
-        <v>-4.4784</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC15" t="n">
-        <v>-0.9341</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>125.12</v>
+        <v>121.24</v>
       </c>
       <c r="C16" t="n">
-        <v>127.54</v>
+        <v>128.48</v>
       </c>
       <c r="D16" t="n">
-        <v>121.6</v>
+        <v>121.24</v>
       </c>
       <c r="E16" t="n">
-        <v>123.27</v>
+        <v>125.87</v>
       </c>
       <c r="F16" t="n">
-        <v>72.95</v>
+        <v>71.55</v>
       </c>
       <c r="G16" t="n">
-        <v>73.20999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="H16" t="n">
-        <v>71.31999999999999</v>
+        <v>70.84</v>
       </c>
       <c r="I16" t="n">
-        <v>72.16</v>
+        <v>71.55</v>
       </c>
       <c r="J16" t="n">
-        <v>43.55</v>
+        <v>44.8</v>
       </c>
       <c r="K16" t="n">
-        <v>44.83</v>
+        <v>44.82</v>
       </c>
       <c r="L16" t="n">
-        <v>42.51</v>
+        <v>42.32</v>
       </c>
       <c r="M16" t="n">
-        <v>44.08</v>
+        <v>43.24</v>
       </c>
       <c r="N16" t="n">
-        <v>37.89</v>
+        <v>38.63</v>
       </c>
       <c r="O16" t="n">
-        <v>38.74</v>
+        <v>39.01</v>
       </c>
       <c r="P16" t="n">
-        <v>37.75</v>
+        <v>38.1</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.31</v>
+        <v>38.64</v>
       </c>
       <c r="R16" t="n">
-        <v>5.1074</v>
+        <v>2.1092</v>
       </c>
       <c r="S16" t="n">
-        <v>15.9097</v>
+        <v>17.9221</v>
       </c>
       <c r="T16" t="n">
-        <v>9.291600000000001</v>
+        <v>18.8462</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.2902</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V16" t="n">
-        <v>3.6782</v>
+        <v>-0.6664</v>
       </c>
       <c r="W16" t="n">
-        <v>0.3337</v>
+        <v>3.4707</v>
       </c>
       <c r="X16" t="n">
-        <v>-4.877</v>
+        <v>-1.9056</v>
       </c>
       <c r="Y16" t="n">
-        <v>-14.9527</v>
+        <v>-16.2016</v>
       </c>
       <c r="Z16" t="n">
-        <v>-10.0775</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.3405</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AB16" t="n">
-        <v>-3.5256</v>
+        <v>0.7825</v>
       </c>
       <c r="AC16" t="n">
-        <v>-0.5193</v>
+        <v>-3.3275</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>121.24</v>
+        <v>116.35</v>
       </c>
       <c r="C17" t="n">
-        <v>128.48</v>
+        <v>119.32</v>
       </c>
       <c r="D17" t="n">
-        <v>121.24</v>
+        <v>113.55</v>
       </c>
       <c r="E17" t="n">
-        <v>125.87</v>
+        <v>115.76</v>
       </c>
       <c r="F17" t="n">
-        <v>71.55</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>72.55</v>
+        <v>70.23</v>
       </c>
       <c r="H17" t="n">
-        <v>70.84</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>71.55</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>44.8</v>
+        <v>46.52</v>
       </c>
       <c r="K17" t="n">
-        <v>44.82</v>
+        <v>47.49</v>
       </c>
       <c r="L17" t="n">
-        <v>42.32</v>
+        <v>45.5</v>
       </c>
       <c r="M17" t="n">
-        <v>43.24</v>
+        <v>46.74</v>
       </c>
       <c r="N17" t="n">
-        <v>38.63</v>
+        <v>40.08</v>
       </c>
       <c r="O17" t="n">
-        <v>39.01</v>
+        <v>40.19</v>
       </c>
       <c r="P17" t="n">
-        <v>38.1</v>
+        <v>39.35</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.64</v>
+        <v>39.9</v>
       </c>
       <c r="R17" t="n">
-        <v>2.1092</v>
+        <v>-8.0321</v>
       </c>
       <c r="S17" t="n">
-        <v>17.9221</v>
+        <v>-1.296</v>
       </c>
       <c r="T17" t="n">
-        <v>18.8462</v>
+        <v>8.848100000000001</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2704</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.6664</v>
+        <v>-4.3665</v>
       </c>
       <c r="W17" t="n">
-        <v>3.4707</v>
+        <v>-0.5603</v>
       </c>
       <c r="X17" t="n">
-        <v>-1.9056</v>
+        <v>8.0944</v>
       </c>
       <c r="Y17" t="n">
-        <v>-16.2016</v>
+        <v>0.8632</v>
       </c>
       <c r="Z17" t="n">
-        <v>-17.1965</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.8614000000000001</v>
+        <v>3.2609</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.7825</v>
+        <v>4.505</v>
       </c>
       <c r="AC17" t="n">
-        <v>-3.3275</v>
+        <v>0.4785</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>116.35</v>
+        <v>120.71</v>
       </c>
       <c r="C18" t="n">
-        <v>119.32</v>
+        <v>124.5</v>
       </c>
       <c r="D18" t="n">
-        <v>113.55</v>
+        <v>117.87</v>
       </c>
       <c r="E18" t="n">
-        <v>115.76</v>
+        <v>121.82</v>
       </c>
       <c r="F18" t="n">
-        <v>68.90000000000001</v>
+        <v>71.19</v>
       </c>
       <c r="G18" t="n">
-        <v>70.23</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>68.68000000000001</v>
+        <v>70.61</v>
       </c>
       <c r="I18" t="n">
-        <v>69.20999999999999</v>
+        <v>70.98</v>
       </c>
       <c r="J18" t="n">
-        <v>46.52</v>
+        <v>44.69</v>
       </c>
       <c r="K18" t="n">
-        <v>47.49</v>
+        <v>45.82</v>
       </c>
       <c r="L18" t="n">
-        <v>45.5</v>
+        <v>43.12</v>
       </c>
       <c r="M18" t="n">
-        <v>46.74</v>
+        <v>44.14</v>
       </c>
       <c r="N18" t="n">
-        <v>40.08</v>
+        <v>38.77</v>
       </c>
       <c r="O18" t="n">
-        <v>40.19</v>
+        <v>39.1</v>
       </c>
       <c r="P18" t="n">
-        <v>39.35</v>
+        <v>38.42</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.9</v>
+        <v>38.87</v>
       </c>
       <c r="R18" t="n">
-        <v>-8.0321</v>
+        <v>5.235</v>
       </c>
       <c r="S18" t="n">
-        <v>-1.296</v>
+        <v>-1.1763</v>
       </c>
       <c r="T18" t="n">
-        <v>8.848100000000001</v>
+        <v>14.1278</v>
       </c>
       <c r="U18" t="n">
-        <v>-3.2704</v>
+        <v>2.5574</v>
       </c>
       <c r="V18" t="n">
-        <v>-4.3665</v>
+        <v>-1.6353</v>
       </c>
       <c r="W18" t="n">
-        <v>-0.5603</v>
+        <v>-1.4577</v>
       </c>
       <c r="X18" t="n">
-        <v>8.0944</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.8632</v>
+        <v>0.1361</v>
       </c>
       <c r="Z18" t="n">
-        <v>-9.820600000000001</v>
+        <v>-14.4574</v>
       </c>
       <c r="AA18" t="n">
-        <v>3.2609</v>
+        <v>-2.5815</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.505</v>
+        <v>1.4618</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.4785</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>120.71</v>
+        <v>101.53</v>
       </c>
       <c r="C19" t="n">
-        <v>124.5</v>
+        <v>105.39</v>
       </c>
       <c r="D19" t="n">
-        <v>117.87</v>
+        <v>99.87</v>
       </c>
       <c r="E19" t="n">
-        <v>121.82</v>
+        <v>101.13</v>
       </c>
       <c r="F19" t="n">
-        <v>71.19</v>
+        <v>67.53</v>
       </c>
       <c r="G19" t="n">
-        <v>71.76000000000001</v>
+        <v>70.39</v>
       </c>
       <c r="H19" t="n">
-        <v>70.61</v>
+        <v>67.34</v>
       </c>
       <c r="I19" t="n">
-        <v>70.98</v>
+        <v>69.27</v>
       </c>
       <c r="J19" t="n">
-        <v>44.69</v>
+        <v>51.61</v>
       </c>
       <c r="K19" t="n">
-        <v>45.82</v>
+        <v>52.22</v>
       </c>
       <c r="L19" t="n">
-        <v>43.12</v>
+        <v>50.21</v>
       </c>
       <c r="M19" t="n">
-        <v>44.14</v>
+        <v>51.73</v>
       </c>
       <c r="N19" t="n">
-        <v>38.77</v>
+        <v>40.78</v>
       </c>
       <c r="O19" t="n">
-        <v>39.1</v>
+        <v>40.88</v>
       </c>
       <c r="P19" t="n">
-        <v>38.42</v>
+        <v>39.21</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.87</v>
+        <v>39.83</v>
       </c>
       <c r="R19" t="n">
-        <v>5.235</v>
+        <v>-16.9841</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.1763</v>
+        <v>-19.6552</v>
       </c>
       <c r="T19" t="n">
-        <v>14.1278</v>
+        <v>-13.7705</v>
       </c>
       <c r="U19" t="n">
-        <v>2.5574</v>
+        <v>-2.4091</v>
       </c>
       <c r="V19" t="n">
-        <v>-1.6353</v>
+        <v>-3.1866</v>
       </c>
       <c r="W19" t="n">
-        <v>-1.4577</v>
+        <v>-4.2835</v>
       </c>
       <c r="X19" t="n">
-        <v>-5.5627</v>
+        <v>17.1953</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.1361</v>
+        <v>19.6346</v>
       </c>
       <c r="Z19" t="n">
-        <v>-14.4574</v>
+        <v>11.6314</v>
       </c>
       <c r="AA19" t="n">
-        <v>-2.5815</v>
+        <v>2.4698</v>
       </c>
       <c r="AB19" t="n">
-        <v>1.4618</v>
+        <v>3.0797</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.3824</v>
+        <v>4.3216</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>101.53</v>
+        <v>104.55</v>
       </c>
       <c r="C20" t="n">
-        <v>105.39</v>
+        <v>105.94</v>
       </c>
       <c r="D20" t="n">
-        <v>99.87</v>
+        <v>100.96</v>
       </c>
       <c r="E20" t="n">
-        <v>101.13</v>
+        <v>102.32</v>
       </c>
       <c r="F20" t="n">
-        <v>67.53</v>
+        <v>69.13</v>
       </c>
       <c r="G20" t="n">
-        <v>70.39</v>
+        <v>69.33</v>
       </c>
       <c r="H20" t="n">
-        <v>67.34</v>
+        <v>67.61</v>
       </c>
       <c r="I20" t="n">
-        <v>69.27</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>51.61</v>
+        <v>49.87</v>
       </c>
       <c r="K20" t="n">
-        <v>52.22</v>
+        <v>51.8</v>
       </c>
       <c r="L20" t="n">
-        <v>50.21</v>
+        <v>49.26</v>
       </c>
       <c r="M20" t="n">
-        <v>51.73</v>
+        <v>51.1</v>
       </c>
       <c r="N20" t="n">
+        <v>39.91</v>
+      </c>
+      <c r="O20" t="n">
         <v>40.78</v>
       </c>
-      <c r="O20" t="n">
-        <v>40.88</v>
-      </c>
       <c r="P20" t="n">
-        <v>39.21</v>
+        <v>39.79</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.83</v>
+        <v>40.62</v>
       </c>
       <c r="R20" t="n">
-        <v>-16.9841</v>
+        <v>1.1767</v>
       </c>
       <c r="S20" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="T20" t="n">
-        <v>-13.7705</v>
+        <v>-16.9952</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.4091</v>
+        <v>-1.9778</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.1866</v>
+        <v>-1.8928</v>
       </c>
       <c r="W20" t="n">
-        <v>-4.2835</v>
+        <v>-5.9035</v>
       </c>
       <c r="X20" t="n">
-        <v>17.1953</v>
+        <v>-1.2179</v>
       </c>
       <c r="Y20" t="n">
-        <v>19.6346</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z20" t="n">
-        <v>11.6314</v>
+        <v>15.9256</v>
       </c>
       <c r="AA20" t="n">
-        <v>2.4698</v>
+        <v>1.9834</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.0797</v>
+        <v>1.8045</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.3216</v>
+        <v>6.0298</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>104.55</v>
+        <v>107.44</v>
       </c>
       <c r="C21" t="n">
-        <v>105.94</v>
+        <v>109.32</v>
       </c>
       <c r="D21" t="n">
-        <v>100.96</v>
+        <v>101.06</v>
       </c>
       <c r="E21" t="n">
-        <v>102.32</v>
+        <v>103.97</v>
       </c>
       <c r="F21" t="n">
-        <v>69.13</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>69.33</v>
+        <v>69.97</v>
       </c>
       <c r="H21" t="n">
-        <v>67.61</v>
+        <v>66.55</v>
       </c>
       <c r="I21" t="n">
-        <v>67.90000000000001</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>49.87</v>
+        <v>48.55</v>
       </c>
       <c r="K21" t="n">
-        <v>51.8</v>
+        <v>51.74</v>
       </c>
       <c r="L21" t="n">
-        <v>49.26</v>
+        <v>47.57</v>
       </c>
       <c r="M21" t="n">
-        <v>51.1</v>
+        <v>50.11</v>
       </c>
       <c r="N21" t="n">
-        <v>39.91</v>
+        <v>40.06</v>
       </c>
       <c r="O21" t="n">
-        <v>40.78</v>
+        <v>41.44</v>
       </c>
       <c r="P21" t="n">
-        <v>39.79</v>
+        <v>39.37</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.62</v>
+        <v>40.61</v>
       </c>
       <c r="R21" t="n">
-        <v>1.1767</v>
+        <v>1.6126</v>
       </c>
       <c r="S21" t="n">
-        <v>-11.6102</v>
+        <v>-14.6528</v>
       </c>
       <c r="T21" t="n">
-        <v>-16.9952</v>
+        <v>-17.3989</v>
       </c>
       <c r="U21" t="n">
-        <v>-1.9778</v>
+        <v>0.0442</v>
       </c>
       <c r="V21" t="n">
-        <v>-1.8928</v>
+        <v>-4.297</v>
       </c>
       <c r="W21" t="n">
-        <v>-5.9035</v>
+        <v>-5.0594</v>
       </c>
       <c r="X21" t="n">
-        <v>-1.2179</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y21" t="n">
-        <v>9.328200000000001</v>
+        <v>13.5251</v>
       </c>
       <c r="Z21" t="n">
-        <v>15.9256</v>
+        <v>15.8881</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.9834</v>
+        <v>-0.0246</v>
       </c>
       <c r="AB21" t="n">
-        <v>1.8045</v>
+        <v>4.4765</v>
       </c>
       <c r="AC21" t="n">
-        <v>6.0298</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
-        </is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>113.33</v>
+      </c>
+      <c r="C22" t="n">
+        <v>115.48</v>
+      </c>
+      <c r="D22" t="n">
+        <v>112.0101</v>
+      </c>
+      <c r="E22" t="n">
+        <v>114.82</v>
+      </c>
+      <c r="F22" t="n">
+        <v>71.13</v>
+      </c>
+      <c r="G22" t="n">
+        <v>71.72</v>
+      </c>
+      <c r="H22" t="n">
+        <v>70.37</v>
+      </c>
+      <c r="I22" t="n">
+        <v>71.38</v>
+      </c>
+      <c r="J22" t="n">
+        <v>45.715</v>
+      </c>
+      <c r="K22" t="n">
+        <v>46.34</v>
+      </c>
+      <c r="L22" t="n">
+        <v>44.67</v>
+      </c>
+      <c r="M22" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="N22" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="O22" t="n">
+        <v>39.14</v>
+      </c>
+      <c r="P22" t="n">
+        <v>38.33</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>38.53</v>
+      </c>
+      <c r="R22" t="n">
+        <v>10.4357</v>
+      </c>
+      <c r="S22" t="n">
+        <v>13.537</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-0.8120000000000001</v>
+      </c>
+      <c r="U22" t="n">
+        <v>5.0788</v>
+      </c>
+      <c r="V22" t="n">
+        <v>3.0461</v>
+      </c>
+      <c r="W22" t="n">
+        <v>3.1354</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-10.2175</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-13.0292</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-3.7441</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-5.1219</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-3.2639</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>-3.4336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master system update 2026-09-18 23:54
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>132.63</v>
+        <v>119.99</v>
       </c>
       <c r="C2" t="n">
-        <v>133.74</v>
+        <v>124.56</v>
       </c>
       <c r="D2" t="n">
-        <v>116.84</v>
+        <v>117.42</v>
       </c>
       <c r="E2" t="n">
-        <v>120.74</v>
+        <v>122.21</v>
       </c>
       <c r="F2" t="n">
-        <v>73.37</v>
+        <v>70.83</v>
       </c>
       <c r="G2" t="n">
-        <v>73.7</v>
+        <v>71.69</v>
       </c>
       <c r="H2" t="n">
-        <v>71</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>72.06</v>
+        <v>70.48</v>
       </c>
       <c r="J2" t="n">
-        <v>42.83</v>
+        <v>47.33</v>
       </c>
       <c r="K2" t="n">
-        <v>48.34</v>
+        <v>48.29</v>
       </c>
       <c r="L2" t="n">
-        <v>42.48</v>
+        <v>45.47</v>
       </c>
       <c r="M2" t="n">
-        <v>47.05</v>
+        <v>46.25</v>
       </c>
       <c r="N2" t="n">
-        <v>37.83</v>
+        <v>39.18</v>
       </c>
       <c r="O2" t="n">
-        <v>39.08</v>
+        <v>39.77</v>
       </c>
       <c r="P2" t="n">
-        <v>37.66</v>
+        <v>38.74</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.53</v>
+        <v>39.37</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>119.99</v>
+        <v>126.59</v>
       </c>
       <c r="C3" t="n">
-        <v>124.56</v>
+        <v>126.79</v>
       </c>
       <c r="D3" t="n">
-        <v>117.42</v>
+        <v>116.71</v>
       </c>
       <c r="E3" t="n">
-        <v>122.21</v>
+        <v>120.6</v>
       </c>
       <c r="F3" t="n">
-        <v>70.83</v>
+        <v>71.7</v>
       </c>
       <c r="G3" t="n">
-        <v>71.69</v>
+        <v>71.83</v>
       </c>
       <c r="H3" t="n">
-        <v>69.76000000000001</v>
+        <v>69.91</v>
       </c>
       <c r="I3" t="n">
-        <v>70.48</v>
+        <v>71.17</v>
       </c>
       <c r="J3" t="n">
-        <v>47.33</v>
+        <v>44.67</v>
       </c>
       <c r="K3" t="n">
-        <v>48.29</v>
+        <v>48.46</v>
       </c>
       <c r="L3" t="n">
-        <v>45.47</v>
+        <v>44.65</v>
       </c>
       <c r="M3" t="n">
-        <v>46.25</v>
+        <v>47.03</v>
       </c>
       <c r="N3" t="n">
-        <v>39.18</v>
+        <v>38.71</v>
       </c>
       <c r="O3" t="n">
-        <v>39.77</v>
+        <v>39.72</v>
       </c>
       <c r="P3" t="n">
-        <v>38.74</v>
+        <v>38.64</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.37</v>
+        <v>39.02</v>
       </c>
       <c r="R3" t="n">
-        <v>1.2175</v>
+        <v>-1.3174</v>
       </c>
       <c r="U3" t="n">
-        <v>-2.1926</v>
+        <v>0.979</v>
       </c>
       <c r="X3" t="n">
-        <v>-1.7003</v>
+        <v>1.6865</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.1801</v>
+        <v>-0.889</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>126.59</v>
+        <v>115.07</v>
       </c>
       <c r="C4" t="n">
-        <v>126.79</v>
+        <v>115.07</v>
       </c>
       <c r="D4" t="n">
-        <v>116.71</v>
+        <v>106</v>
       </c>
       <c r="E4" t="n">
-        <v>120.6</v>
+        <v>111.16</v>
       </c>
       <c r="F4" t="n">
-        <v>71.7</v>
+        <v>70</v>
       </c>
       <c r="G4" t="n">
-        <v>71.83</v>
+        <v>70.05</v>
       </c>
       <c r="H4" t="n">
-        <v>69.91</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>71.17</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>44.67</v>
+        <v>49.14</v>
       </c>
       <c r="K4" t="n">
-        <v>48.46</v>
+        <v>52.81</v>
       </c>
       <c r="L4" t="n">
-        <v>44.65</v>
+        <v>49.13</v>
       </c>
       <c r="M4" t="n">
-        <v>47.03</v>
+        <v>50.75</v>
       </c>
       <c r="N4" t="n">
-        <v>38.71</v>
+        <v>39.65</v>
       </c>
       <c r="O4" t="n">
-        <v>39.72</v>
+        <v>40.79</v>
       </c>
       <c r="P4" t="n">
-        <v>38.64</v>
+        <v>39.64</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.02</v>
+        <v>40.19</v>
       </c>
       <c r="R4" t="n">
-        <v>-1.3174</v>
+        <v>-7.8275</v>
       </c>
       <c r="U4" t="n">
-        <v>0.979</v>
+        <v>-3.035</v>
       </c>
       <c r="X4" t="n">
-        <v>1.6865</v>
+        <v>7.9098</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.889</v>
+        <v>2.9985</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>115.07</v>
+        <v>117.37</v>
       </c>
       <c r="C5" t="n">
-        <v>115.07</v>
+        <v>119.88</v>
       </c>
       <c r="D5" t="n">
-        <v>106</v>
+        <v>113.13</v>
       </c>
       <c r="E5" t="n">
-        <v>111.16</v>
+        <v>115.67</v>
       </c>
       <c r="F5" t="n">
-        <v>70</v>
+        <v>70.42</v>
       </c>
       <c r="G5" t="n">
-        <v>70.05</v>
+        <v>71.27</v>
       </c>
       <c r="H5" t="n">
-        <v>67.93000000000001</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>69.01000000000001</v>
+        <v>70.27</v>
       </c>
       <c r="J5" t="n">
-        <v>49.14</v>
+        <v>47.82</v>
       </c>
       <c r="K5" t="n">
-        <v>52.81</v>
+        <v>49.83</v>
       </c>
       <c r="L5" t="n">
-        <v>49.13</v>
+        <v>46.66</v>
       </c>
       <c r="M5" t="n">
-        <v>50.75</v>
+        <v>48.42</v>
       </c>
       <c r="N5" t="n">
-        <v>39.65</v>
+        <v>39.38</v>
       </c>
       <c r="O5" t="n">
-        <v>40.79</v>
+        <v>40.02</v>
       </c>
       <c r="P5" t="n">
-        <v>39.64</v>
+        <v>38.89</v>
       </c>
       <c r="Q5" t="n">
-        <v>40.19</v>
+        <v>39.46</v>
       </c>
       <c r="R5" t="n">
-        <v>-7.8275</v>
+        <v>4.0572</v>
       </c>
       <c r="S5" t="n">
-        <v>-7.9344</v>
+        <v>-5.3514</v>
       </c>
       <c r="U5" t="n">
-        <v>-3.035</v>
+        <v>1.8258</v>
       </c>
       <c r="V5" t="n">
-        <v>-4.2326</v>
+        <v>-0.298</v>
       </c>
       <c r="X5" t="n">
-        <v>7.9098</v>
+        <v>-4.5911</v>
       </c>
       <c r="Y5" t="n">
-        <v>7.864</v>
+        <v>4.6919</v>
       </c>
       <c r="AA5" t="n">
-        <v>2.9985</v>
+        <v>-1.8164</v>
       </c>
       <c r="AB5" t="n">
-        <v>4.3083</v>
+        <v>0.2286</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>117.37</v>
+        <v>114.7</v>
       </c>
       <c r="C6" t="n">
-        <v>119.88</v>
+        <v>117.39</v>
       </c>
       <c r="D6" t="n">
-        <v>113.13</v>
+        <v>112.53</v>
       </c>
       <c r="E6" t="n">
-        <v>115.67</v>
+        <v>116.6</v>
       </c>
       <c r="F6" t="n">
-        <v>70.42</v>
+        <v>69.56</v>
       </c>
       <c r="G6" t="n">
-        <v>71.27</v>
+        <v>70.94</v>
       </c>
       <c r="H6" t="n">
-        <v>69.34999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="I6" t="n">
-        <v>70.27</v>
+        <v>70.47</v>
       </c>
       <c r="J6" t="n">
-        <v>47.82</v>
+        <v>49.01</v>
       </c>
       <c r="K6" t="n">
-        <v>49.83</v>
+        <v>49.89</v>
       </c>
       <c r="L6" t="n">
-        <v>46.66</v>
+        <v>47.87</v>
       </c>
       <c r="M6" t="n">
-        <v>48.42</v>
+        <v>48.09</v>
       </c>
       <c r="N6" t="n">
+        <v>39.86</v>
+      </c>
+      <c r="O6" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="P6" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="Q6" t="n">
         <v>39.38</v>
       </c>
-      <c r="O6" t="n">
-        <v>40.02</v>
-      </c>
-      <c r="P6" t="n">
-        <v>38.89</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>39.46</v>
-      </c>
       <c r="R6" t="n">
-        <v>4.0572</v>
+        <v>0.804</v>
       </c>
       <c r="S6" t="n">
-        <v>-5.3514</v>
+        <v>-3.3167</v>
       </c>
       <c r="U6" t="n">
-        <v>1.8258</v>
+        <v>0.2846</v>
       </c>
       <c r="V6" t="n">
-        <v>-0.298</v>
+        <v>-0.9836</v>
       </c>
       <c r="X6" t="n">
-        <v>-4.5911</v>
+        <v>-0.6815</v>
       </c>
       <c r="Y6" t="n">
-        <v>4.6919</v>
+        <v>2.2539</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.8164</v>
+        <v>-0.2027</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.2286</v>
+        <v>0.9226</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>114.7</v>
+        <v>123.4</v>
       </c>
       <c r="C7" t="n">
-        <v>117.39</v>
+        <v>124.88</v>
       </c>
       <c r="D7" t="n">
-        <v>112.53</v>
+        <v>117.69</v>
       </c>
       <c r="E7" t="n">
-        <v>116.6</v>
+        <v>123.05</v>
       </c>
       <c r="F7" t="n">
-        <v>69.56</v>
+        <v>72.09</v>
       </c>
       <c r="G7" t="n">
-        <v>70.94</v>
+        <v>73.38</v>
       </c>
       <c r="H7" t="n">
-        <v>69.44</v>
+        <v>71.38</v>
       </c>
       <c r="I7" t="n">
-        <v>70.47</v>
+        <v>73.3</v>
       </c>
       <c r="J7" t="n">
-        <v>49.01</v>
+        <v>45.42</v>
       </c>
       <c r="K7" t="n">
-        <v>49.89</v>
+        <v>47.71</v>
       </c>
       <c r="L7" t="n">
-        <v>47.87</v>
+        <v>44.71</v>
       </c>
       <c r="M7" t="n">
-        <v>48.09</v>
+        <v>45.35</v>
       </c>
       <c r="N7" t="n">
-        <v>39.86</v>
+        <v>38.46</v>
       </c>
       <c r="O7" t="n">
-        <v>39.93</v>
+        <v>38.86</v>
       </c>
       <c r="P7" t="n">
-        <v>39.09</v>
+        <v>37.73</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.38</v>
+        <v>37.78</v>
       </c>
       <c r="R7" t="n">
-        <v>0.804</v>
+        <v>5.5317</v>
       </c>
       <c r="S7" t="n">
-        <v>-3.3167</v>
+        <v>10.6963</v>
       </c>
       <c r="T7" t="n">
-        <v>-3.4289</v>
+        <v>0.6873</v>
       </c>
       <c r="U7" t="n">
-        <v>0.2846</v>
+        <v>4.0159</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.9836</v>
+        <v>6.2165</v>
       </c>
       <c r="W7" t="n">
-        <v>-2.2065</v>
+        <v>4.0011</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.6815</v>
+        <v>-5.6977</v>
       </c>
       <c r="Y7" t="n">
-        <v>2.2539</v>
+        <v>-10.6404</v>
       </c>
       <c r="Z7" t="n">
-        <v>2.2104</v>
+        <v>-1.9459</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.2027</v>
+        <v>-4.063</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.9226</v>
+        <v>-5.9965</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.2061</v>
+        <v>-4.0386</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>123.4</v>
+        <v>119.92</v>
       </c>
       <c r="C8" t="n">
-        <v>124.88</v>
+        <v>121.2</v>
       </c>
       <c r="D8" t="n">
-        <v>117.69</v>
+        <v>110.21</v>
       </c>
       <c r="E8" t="n">
-        <v>123.05</v>
+        <v>111.34</v>
       </c>
       <c r="F8" t="n">
-        <v>72.09</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>73.38</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>71.38</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>73.3</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>45.42</v>
+        <v>46.61</v>
       </c>
       <c r="K8" t="n">
-        <v>47.71</v>
+        <v>50.23</v>
       </c>
       <c r="L8" t="n">
-        <v>44.71</v>
+        <v>46.15</v>
       </c>
       <c r="M8" t="n">
-        <v>45.35</v>
+        <v>49.82</v>
       </c>
       <c r="N8" t="n">
-        <v>38.46</v>
+        <v>38.02</v>
       </c>
       <c r="O8" t="n">
-        <v>38.86</v>
+        <v>38.76</v>
       </c>
       <c r="P8" t="n">
-        <v>37.73</v>
+        <v>37.33</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.78</v>
+        <v>38.54</v>
       </c>
       <c r="R8" t="n">
-        <v>5.5317</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>10.6963</v>
+        <v>-3.7434</v>
       </c>
       <c r="T8" t="n">
-        <v>0.6873</v>
+        <v>-7.6783</v>
       </c>
       <c r="U8" t="n">
-        <v>4.0159</v>
+        <v>-1.9782</v>
       </c>
       <c r="V8" t="n">
-        <v>6.2165</v>
+        <v>2.2485</v>
       </c>
       <c r="W8" t="n">
-        <v>4.0011</v>
+        <v>0.9555</v>
       </c>
       <c r="X8" t="n">
-        <v>-5.6977</v>
+        <v>9.8567</v>
       </c>
       <c r="Y8" t="n">
-        <v>-10.6404</v>
+        <v>2.8914</v>
       </c>
       <c r="Z8" t="n">
-        <v>-1.9459</v>
+        <v>5.9324</v>
       </c>
       <c r="AA8" t="n">
-        <v>-4.063</v>
+        <v>2.0116</v>
       </c>
       <c r="AB8" t="n">
-        <v>-5.9965</v>
+        <v>-2.3315</v>
       </c>
       <c r="AC8" t="n">
-        <v>-4.0386</v>
+        <v>-1.2301</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>119.92</v>
+        <v>112.41</v>
       </c>
       <c r="C9" t="n">
-        <v>121.2</v>
+        <v>115.05</v>
       </c>
       <c r="D9" t="n">
-        <v>110.21</v>
+        <v>110.33</v>
       </c>
       <c r="E9" t="n">
-        <v>111.34</v>
+        <v>112.79</v>
       </c>
       <c r="F9" t="n">
-        <v>72.84999999999999</v>
+        <v>71.44</v>
       </c>
       <c r="G9" t="n">
-        <v>74.18000000000001</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>71.43000000000001</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>71.84999999999999</v>
+        <v>71.92</v>
       </c>
       <c r="J9" t="n">
-        <v>46.61</v>
+        <v>49.27</v>
       </c>
       <c r="K9" t="n">
-        <v>50.23</v>
+        <v>50.24</v>
       </c>
       <c r="L9" t="n">
-        <v>46.15</v>
+        <v>48.09</v>
       </c>
       <c r="M9" t="n">
-        <v>49.82</v>
+        <v>49.02</v>
       </c>
       <c r="N9" t="n">
-        <v>38.02</v>
+        <v>38.77</v>
       </c>
       <c r="O9" t="n">
-        <v>38.76</v>
+        <v>39.09</v>
       </c>
       <c r="P9" t="n">
-        <v>37.33</v>
+        <v>38.37</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.54</v>
+        <v>38.51</v>
       </c>
       <c r="R9" t="n">
-        <v>-9.516500000000001</v>
+        <v>1.3023</v>
       </c>
       <c r="S9" t="n">
-        <v>-3.7434</v>
+        <v>-3.2676</v>
       </c>
       <c r="T9" t="n">
-        <v>-7.6783</v>
+        <v>1.4664</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.9782</v>
+        <v>0.0974</v>
       </c>
       <c r="V9" t="n">
-        <v>2.2485</v>
+        <v>2.0576</v>
       </c>
       <c r="W9" t="n">
-        <v>0.9555</v>
+        <v>4.2168</v>
       </c>
       <c r="X9" t="n">
-        <v>9.8567</v>
+        <v>-1.6058</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.8914</v>
+        <v>1.9339</v>
       </c>
       <c r="Z9" t="n">
-        <v>5.9324</v>
+        <v>-3.4089</v>
       </c>
       <c r="AA9" t="n">
-        <v>2.0116</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="AB9" t="n">
-        <v>-2.3315</v>
+        <v>-2.2092</v>
       </c>
       <c r="AC9" t="n">
-        <v>-1.2301</v>
+        <v>-4.1801</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>112.41</v>
+        <v>106.36</v>
       </c>
       <c r="C10" t="n">
-        <v>115.05</v>
+        <v>108.64</v>
       </c>
       <c r="D10" t="n">
-        <v>110.33</v>
+        <v>102.31</v>
       </c>
       <c r="E10" t="n">
-        <v>112.79</v>
+        <v>105.91</v>
       </c>
       <c r="F10" t="n">
-        <v>71.44</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>72.15000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="H10" t="n">
-        <v>70.81999999999999</v>
+        <v>68.25</v>
       </c>
       <c r="I10" t="n">
-        <v>71.92</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>49.27</v>
+        <v>51.88</v>
       </c>
       <c r="K10" t="n">
-        <v>50.24</v>
+        <v>53.69</v>
       </c>
       <c r="L10" t="n">
-        <v>48.09</v>
+        <v>50.9</v>
       </c>
       <c r="M10" t="n">
-        <v>49.02</v>
+        <v>52.22</v>
       </c>
       <c r="N10" t="n">
-        <v>38.77</v>
+        <v>40.03</v>
       </c>
       <c r="O10" t="n">
-        <v>39.09</v>
+        <v>40.47</v>
       </c>
       <c r="P10" t="n">
-        <v>38.37</v>
+        <v>39.23</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.51</v>
+        <v>39.97</v>
       </c>
       <c r="R10" t="n">
-        <v>1.3023</v>
+        <v>-6.0998</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.2676</v>
+        <v>-13.9293</v>
       </c>
       <c r="T10" t="n">
-        <v>1.4664</v>
+        <v>-8.437799999999999</v>
       </c>
       <c r="U10" t="n">
-        <v>0.0974</v>
+        <v>-3.8515</v>
       </c>
       <c r="V10" t="n">
-        <v>2.0576</v>
+        <v>-5.6617</v>
       </c>
       <c r="W10" t="n">
-        <v>4.2168</v>
+        <v>-1.5939</v>
       </c>
       <c r="X10" t="n">
-        <v>-1.6058</v>
+        <v>6.5279</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.9339</v>
+        <v>15.1488</v>
       </c>
       <c r="Z10" t="n">
-        <v>-3.4089</v>
+        <v>7.848</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.07779999999999999</v>
+        <v>3.7912</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2.2092</v>
+        <v>5.7967</v>
       </c>
       <c r="AC10" t="n">
-        <v>-4.1801</v>
+        <v>1.2924</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>106.36</v>
+        <v>104.5</v>
       </c>
       <c r="C11" t="n">
-        <v>108.64</v>
+        <v>108.07</v>
       </c>
       <c r="D11" t="n">
-        <v>102.31</v>
+        <v>101.34</v>
       </c>
       <c r="E11" t="n">
-        <v>105.91</v>
+        <v>106.35</v>
       </c>
       <c r="F11" t="n">
-        <v>69.06999999999999</v>
+        <v>68.97</v>
       </c>
       <c r="G11" t="n">
-        <v>70.55</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>68.25</v>
+        <v>68.39</v>
       </c>
       <c r="I11" t="n">
-        <v>69.15000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>51.88</v>
+        <v>52.8</v>
       </c>
       <c r="K11" t="n">
-        <v>53.69</v>
+        <v>54.39</v>
       </c>
       <c r="L11" t="n">
-        <v>50.9</v>
+        <v>51.05</v>
       </c>
       <c r="M11" t="n">
-        <v>52.22</v>
+        <v>51.83</v>
       </c>
       <c r="N11" t="n">
-        <v>40.03</v>
+        <v>40.09</v>
       </c>
       <c r="O11" t="n">
-        <v>40.47</v>
+        <v>40.43</v>
       </c>
       <c r="P11" t="n">
-        <v>39.23</v>
+        <v>39.63</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.97</v>
+        <v>39.71</v>
       </c>
       <c r="R11" t="n">
-        <v>-6.0998</v>
+        <v>0.4154</v>
       </c>
       <c r="S11" t="n">
-        <v>-13.9293</v>
+        <v>-4.4818</v>
       </c>
       <c r="T11" t="n">
-        <v>-8.437799999999999</v>
+        <v>-8.790699999999999</v>
       </c>
       <c r="U11" t="n">
-        <v>-3.8515</v>
+        <v>0.6508</v>
       </c>
       <c r="V11" t="n">
-        <v>-5.6617</v>
+        <v>-3.1315</v>
       </c>
       <c r="W11" t="n">
-        <v>-1.5939</v>
+        <v>-1.2346</v>
       </c>
       <c r="X11" t="n">
-        <v>6.5279</v>
+        <v>-0.7468</v>
       </c>
       <c r="Y11" t="n">
-        <v>15.1488</v>
+        <v>4.0345</v>
       </c>
       <c r="Z11" t="n">
-        <v>7.848</v>
+        <v>7.7771</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.7912</v>
+        <v>-0.6505</v>
       </c>
       <c r="AB11" t="n">
-        <v>5.7967</v>
+        <v>3.0358</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.2924</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>104.5</v>
+        <v>103</v>
       </c>
       <c r="C12" t="n">
-        <v>108.07</v>
+        <v>107.49</v>
       </c>
       <c r="D12" t="n">
-        <v>101.34</v>
+        <v>98.62</v>
       </c>
       <c r="E12" t="n">
-        <v>106.35</v>
+        <v>106.74</v>
       </c>
       <c r="F12" t="n">
-        <v>68.97</v>
+        <v>70.06</v>
       </c>
       <c r="G12" t="n">
-        <v>69.76000000000001</v>
+        <v>72.42</v>
       </c>
       <c r="H12" t="n">
-        <v>68.39</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>69.59999999999999</v>
+        <v>72.03</v>
       </c>
       <c r="J12" t="n">
-        <v>52.8</v>
+        <v>53.5</v>
       </c>
       <c r="K12" t="n">
-        <v>54.39</v>
+        <v>55.69</v>
       </c>
       <c r="L12" t="n">
-        <v>51.05</v>
+        <v>51.28</v>
       </c>
       <c r="M12" t="n">
-        <v>51.83</v>
+        <v>51.6</v>
       </c>
       <c r="N12" t="n">
-        <v>40.09</v>
+        <v>39.49</v>
       </c>
       <c r="O12" t="n">
-        <v>40.43</v>
+        <v>39.68</v>
       </c>
       <c r="P12" t="n">
-        <v>39.63</v>
+        <v>38.12</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.71</v>
+        <v>38.34</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4154</v>
+        <v>0.3667</v>
       </c>
       <c r="S12" t="n">
-        <v>-4.4818</v>
+        <v>-5.364</v>
       </c>
       <c r="T12" t="n">
-        <v>-8.790699999999999</v>
+        <v>-13.2548</v>
       </c>
       <c r="U12" t="n">
-        <v>0.6508</v>
+        <v>3.4914</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.1315</v>
+        <v>0.1529</v>
       </c>
       <c r="W12" t="n">
-        <v>-1.2346</v>
+        <v>-1.7326</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.7468</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y12" t="n">
-        <v>4.0345</v>
+        <v>5.2632</v>
       </c>
       <c r="Z12" t="n">
-        <v>7.7771</v>
+        <v>13.7817</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.6505</v>
+        <v>-3.45</v>
       </c>
       <c r="AB12" t="n">
-        <v>3.0358</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.838</v>
+        <v>1.4823</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>103</v>
+        <v>111.22</v>
       </c>
       <c r="C13" t="n">
-        <v>107.49</v>
+        <v>118.18</v>
       </c>
       <c r="D13" t="n">
-        <v>98.62</v>
+        <v>109.73</v>
       </c>
       <c r="E13" t="n">
-        <v>106.74</v>
+        <v>117.28</v>
       </c>
       <c r="F13" t="n">
-        <v>70.06</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>72.42</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>69.70999999999999</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>72.03</v>
+        <v>72.37</v>
       </c>
       <c r="J13" t="n">
-        <v>53.5</v>
+        <v>49.56</v>
       </c>
       <c r="K13" t="n">
-        <v>55.69</v>
+        <v>50.21</v>
       </c>
       <c r="L13" t="n">
-        <v>51.28</v>
+        <v>46.1</v>
       </c>
       <c r="M13" t="n">
-        <v>51.6</v>
+        <v>46.34</v>
       </c>
       <c r="N13" t="n">
-        <v>39.49</v>
+        <v>38.12</v>
       </c>
       <c r="O13" t="n">
-        <v>39.68</v>
+        <v>38.58</v>
       </c>
       <c r="P13" t="n">
-        <v>38.12</v>
+        <v>37.72</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.34</v>
+        <v>38.18</v>
       </c>
       <c r="R13" t="n">
-        <v>0.3667</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S13" t="n">
-        <v>-5.364</v>
+        <v>10.7355</v>
       </c>
       <c r="T13" t="n">
-        <v>-13.2548</v>
+        <v>5.335</v>
       </c>
       <c r="U13" t="n">
-        <v>3.4914</v>
+        <v>0.472</v>
       </c>
       <c r="V13" t="n">
-        <v>0.1529</v>
+        <v>4.6565</v>
       </c>
       <c r="W13" t="n">
-        <v>-1.7326</v>
+        <v>0.7237</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.4438</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y13" t="n">
-        <v>5.2632</v>
+        <v>-11.2601</v>
       </c>
       <c r="Z13" t="n">
-        <v>13.7817</v>
+        <v>-6.9851</v>
       </c>
       <c r="AA13" t="n">
-        <v>-3.45</v>
+        <v>-0.4173</v>
       </c>
       <c r="AB13" t="n">
-        <v>-0.4414</v>
+        <v>-4.4784</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.4823</v>
+        <v>-0.9341</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>111.22</v>
+        <v>125.12</v>
       </c>
       <c r="C14" t="n">
-        <v>118.18</v>
+        <v>127.54</v>
       </c>
       <c r="D14" t="n">
-        <v>109.73</v>
+        <v>121.6</v>
       </c>
       <c r="E14" t="n">
-        <v>117.28</v>
+        <v>123.27</v>
       </c>
       <c r="F14" t="n">
-        <v>72.48999999999999</v>
+        <v>72.95</v>
       </c>
       <c r="G14" t="n">
-        <v>73.23999999999999</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>71.65000000000001</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>72.37</v>
+        <v>72.16</v>
       </c>
       <c r="J14" t="n">
-        <v>49.56</v>
+        <v>43.55</v>
       </c>
       <c r="K14" t="n">
-        <v>50.21</v>
+        <v>44.83</v>
       </c>
       <c r="L14" t="n">
-        <v>46.1</v>
+        <v>42.51</v>
       </c>
       <c r="M14" t="n">
-        <v>46.34</v>
+        <v>44.08</v>
       </c>
       <c r="N14" t="n">
-        <v>38.12</v>
+        <v>37.89</v>
       </c>
       <c r="O14" t="n">
-        <v>38.58</v>
+        <v>38.74</v>
       </c>
       <c r="P14" t="n">
-        <v>37.72</v>
+        <v>37.75</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.18</v>
+        <v>38.31</v>
       </c>
       <c r="R14" t="n">
-        <v>9.874499999999999</v>
+        <v>5.1074</v>
       </c>
       <c r="S14" t="n">
-        <v>10.7355</v>
+        <v>15.9097</v>
       </c>
       <c r="T14" t="n">
-        <v>5.335</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U14" t="n">
-        <v>0.472</v>
+        <v>-0.2902</v>
       </c>
       <c r="V14" t="n">
-        <v>4.6565</v>
+        <v>3.6782</v>
       </c>
       <c r="W14" t="n">
-        <v>0.7237</v>
+        <v>0.3337</v>
       </c>
       <c r="X14" t="n">
-        <v>-10.1938</v>
+        <v>-4.877</v>
       </c>
       <c r="Y14" t="n">
-        <v>-11.2601</v>
+        <v>-14.9527</v>
       </c>
       <c r="Z14" t="n">
-        <v>-6.9851</v>
+        <v>-10.0775</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.4173</v>
+        <v>0.3405</v>
       </c>
       <c r="AB14" t="n">
-        <v>-4.4784</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC14" t="n">
-        <v>-0.9341</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>125.12</v>
+        <v>121.24</v>
       </c>
       <c r="C15" t="n">
-        <v>127.54</v>
+        <v>128.48</v>
       </c>
       <c r="D15" t="n">
-        <v>121.6</v>
+        <v>121.24</v>
       </c>
       <c r="E15" t="n">
-        <v>123.27</v>
+        <v>125.87</v>
       </c>
       <c r="F15" t="n">
-        <v>72.95</v>
+        <v>71.55</v>
       </c>
       <c r="G15" t="n">
-        <v>73.20999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="H15" t="n">
-        <v>71.31999999999999</v>
+        <v>70.84</v>
       </c>
       <c r="I15" t="n">
-        <v>72.16</v>
+        <v>71.55</v>
       </c>
       <c r="J15" t="n">
-        <v>43.55</v>
+        <v>44.8</v>
       </c>
       <c r="K15" t="n">
-        <v>44.83</v>
+        <v>44.82</v>
       </c>
       <c r="L15" t="n">
-        <v>42.51</v>
+        <v>42.32</v>
       </c>
       <c r="M15" t="n">
-        <v>44.08</v>
+        <v>43.24</v>
       </c>
       <c r="N15" t="n">
-        <v>37.89</v>
+        <v>38.63</v>
       </c>
       <c r="O15" t="n">
-        <v>38.74</v>
+        <v>39.01</v>
       </c>
       <c r="P15" t="n">
-        <v>37.75</v>
+        <v>38.1</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.31</v>
+        <v>38.64</v>
       </c>
       <c r="R15" t="n">
-        <v>5.1074</v>
+        <v>2.1092</v>
       </c>
       <c r="S15" t="n">
-        <v>15.9097</v>
+        <v>17.9221</v>
       </c>
       <c r="T15" t="n">
-        <v>9.291600000000001</v>
+        <v>18.8462</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.2902</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>3.6782</v>
+        <v>-0.6664</v>
       </c>
       <c r="W15" t="n">
-        <v>0.3337</v>
+        <v>3.4707</v>
       </c>
       <c r="X15" t="n">
-        <v>-4.877</v>
+        <v>-1.9056</v>
       </c>
       <c r="Y15" t="n">
-        <v>-14.9527</v>
+        <v>-16.2016</v>
       </c>
       <c r="Z15" t="n">
-        <v>-10.0775</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.3405</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AB15" t="n">
-        <v>-3.5256</v>
+        <v>0.7825</v>
       </c>
       <c r="AC15" t="n">
-        <v>-0.5193</v>
+        <v>-3.3275</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>121.24</v>
+        <v>116.35</v>
       </c>
       <c r="C16" t="n">
-        <v>128.48</v>
+        <v>119.32</v>
       </c>
       <c r="D16" t="n">
-        <v>121.24</v>
+        <v>113.55</v>
       </c>
       <c r="E16" t="n">
-        <v>125.87</v>
+        <v>115.76</v>
       </c>
       <c r="F16" t="n">
-        <v>71.55</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>72.55</v>
+        <v>70.23</v>
       </c>
       <c r="H16" t="n">
-        <v>70.84</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>71.55</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>44.8</v>
+        <v>46.52</v>
       </c>
       <c r="K16" t="n">
-        <v>44.82</v>
+        <v>47.49</v>
       </c>
       <c r="L16" t="n">
-        <v>42.32</v>
+        <v>45.5</v>
       </c>
       <c r="M16" t="n">
-        <v>43.24</v>
+        <v>46.74</v>
       </c>
       <c r="N16" t="n">
-        <v>38.63</v>
+        <v>40.08</v>
       </c>
       <c r="O16" t="n">
-        <v>39.01</v>
+        <v>40.19</v>
       </c>
       <c r="P16" t="n">
-        <v>38.1</v>
+        <v>39.35</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.64</v>
+        <v>39.9</v>
       </c>
       <c r="R16" t="n">
-        <v>2.1092</v>
+        <v>-8.0321</v>
       </c>
       <c r="S16" t="n">
-        <v>17.9221</v>
+        <v>-1.296</v>
       </c>
       <c r="T16" t="n">
-        <v>18.8462</v>
+        <v>8.848100000000001</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2704</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.6664</v>
+        <v>-4.3665</v>
       </c>
       <c r="W16" t="n">
-        <v>3.4707</v>
+        <v>-0.5603</v>
       </c>
       <c r="X16" t="n">
-        <v>-1.9056</v>
+        <v>8.0944</v>
       </c>
       <c r="Y16" t="n">
-        <v>-16.2016</v>
+        <v>0.8632</v>
       </c>
       <c r="Z16" t="n">
-        <v>-17.1965</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.8614000000000001</v>
+        <v>3.2609</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.7825</v>
+        <v>4.505</v>
       </c>
       <c r="AC16" t="n">
-        <v>-3.3275</v>
+        <v>0.4785</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>116.35</v>
+        <v>120.71</v>
       </c>
       <c r="C17" t="n">
-        <v>119.32</v>
+        <v>124.5</v>
       </c>
       <c r="D17" t="n">
-        <v>113.55</v>
+        <v>117.87</v>
       </c>
       <c r="E17" t="n">
-        <v>115.76</v>
+        <v>121.82</v>
       </c>
       <c r="F17" t="n">
-        <v>68.90000000000001</v>
+        <v>71.19</v>
       </c>
       <c r="G17" t="n">
-        <v>70.23</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>68.68000000000001</v>
+        <v>70.61</v>
       </c>
       <c r="I17" t="n">
-        <v>69.20999999999999</v>
+        <v>70.98</v>
       </c>
       <c r="J17" t="n">
-        <v>46.52</v>
+        <v>44.69</v>
       </c>
       <c r="K17" t="n">
-        <v>47.49</v>
+        <v>45.82</v>
       </c>
       <c r="L17" t="n">
-        <v>45.5</v>
+        <v>43.12</v>
       </c>
       <c r="M17" t="n">
-        <v>46.74</v>
+        <v>44.14</v>
       </c>
       <c r="N17" t="n">
-        <v>40.08</v>
+        <v>38.77</v>
       </c>
       <c r="O17" t="n">
-        <v>40.19</v>
+        <v>39.1</v>
       </c>
       <c r="P17" t="n">
-        <v>39.35</v>
+        <v>38.42</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.9</v>
+        <v>38.87</v>
       </c>
       <c r="R17" t="n">
-        <v>-8.0321</v>
+        <v>5.235</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.296</v>
+        <v>-1.1763</v>
       </c>
       <c r="T17" t="n">
-        <v>8.848100000000001</v>
+        <v>14.1278</v>
       </c>
       <c r="U17" t="n">
-        <v>-3.2704</v>
+        <v>2.5574</v>
       </c>
       <c r="V17" t="n">
-        <v>-4.3665</v>
+        <v>-1.6353</v>
       </c>
       <c r="W17" t="n">
-        <v>-0.5603</v>
+        <v>-1.4577</v>
       </c>
       <c r="X17" t="n">
-        <v>8.0944</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.8632</v>
+        <v>0.1361</v>
       </c>
       <c r="Z17" t="n">
-        <v>-9.820600000000001</v>
+        <v>-14.4574</v>
       </c>
       <c r="AA17" t="n">
-        <v>3.2609</v>
+        <v>-2.5815</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.505</v>
+        <v>1.4618</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.4785</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>120.71</v>
+        <v>101.53</v>
       </c>
       <c r="C18" t="n">
-        <v>124.5</v>
+        <v>105.39</v>
       </c>
       <c r="D18" t="n">
-        <v>117.87</v>
+        <v>99.87</v>
       </c>
       <c r="E18" t="n">
-        <v>121.82</v>
+        <v>101.13</v>
       </c>
       <c r="F18" t="n">
-        <v>71.19</v>
+        <v>67.53</v>
       </c>
       <c r="G18" t="n">
-        <v>71.76000000000001</v>
+        <v>70.39</v>
       </c>
       <c r="H18" t="n">
-        <v>70.61</v>
+        <v>67.34</v>
       </c>
       <c r="I18" t="n">
-        <v>70.98</v>
+        <v>69.27</v>
       </c>
       <c r="J18" t="n">
-        <v>44.69</v>
+        <v>51.61</v>
       </c>
       <c r="K18" t="n">
-        <v>45.82</v>
+        <v>52.22</v>
       </c>
       <c r="L18" t="n">
-        <v>43.12</v>
+        <v>50.21</v>
       </c>
       <c r="M18" t="n">
-        <v>44.14</v>
+        <v>51.73</v>
       </c>
       <c r="N18" t="n">
-        <v>38.77</v>
+        <v>40.78</v>
       </c>
       <c r="O18" t="n">
-        <v>39.1</v>
+        <v>40.88</v>
       </c>
       <c r="P18" t="n">
-        <v>38.42</v>
+        <v>39.21</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.87</v>
+        <v>39.83</v>
       </c>
       <c r="R18" t="n">
-        <v>5.235</v>
+        <v>-16.9841</v>
       </c>
       <c r="S18" t="n">
-        <v>-1.1763</v>
+        <v>-19.6552</v>
       </c>
       <c r="T18" t="n">
-        <v>14.1278</v>
+        <v>-13.7705</v>
       </c>
       <c r="U18" t="n">
-        <v>2.5574</v>
+        <v>-2.4091</v>
       </c>
       <c r="V18" t="n">
-        <v>-1.6353</v>
+        <v>-3.1866</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.4577</v>
+        <v>-4.2835</v>
       </c>
       <c r="X18" t="n">
-        <v>-5.5627</v>
+        <v>17.1953</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.1361</v>
+        <v>19.6346</v>
       </c>
       <c r="Z18" t="n">
-        <v>-14.4574</v>
+        <v>11.6314</v>
       </c>
       <c r="AA18" t="n">
-        <v>-2.5815</v>
+        <v>2.4698</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.4618</v>
+        <v>3.0797</v>
       </c>
       <c r="AC18" t="n">
-        <v>1.3824</v>
+        <v>4.3216</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>101.53</v>
+        <v>104.55</v>
       </c>
       <c r="C19" t="n">
-        <v>105.39</v>
+        <v>105.94</v>
       </c>
       <c r="D19" t="n">
-        <v>99.87</v>
+        <v>100.96</v>
       </c>
       <c r="E19" t="n">
-        <v>101.13</v>
+        <v>102.32</v>
       </c>
       <c r="F19" t="n">
-        <v>67.53</v>
+        <v>69.13</v>
       </c>
       <c r="G19" t="n">
-        <v>70.39</v>
+        <v>69.33</v>
       </c>
       <c r="H19" t="n">
-        <v>67.34</v>
+        <v>67.61</v>
       </c>
       <c r="I19" t="n">
-        <v>69.27</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>51.61</v>
+        <v>49.87</v>
       </c>
       <c r="K19" t="n">
-        <v>52.22</v>
+        <v>51.8</v>
       </c>
       <c r="L19" t="n">
-        <v>50.21</v>
+        <v>49.26</v>
       </c>
       <c r="M19" t="n">
-        <v>51.73</v>
+        <v>51.1</v>
       </c>
       <c r="N19" t="n">
+        <v>39.91</v>
+      </c>
+      <c r="O19" t="n">
         <v>40.78</v>
       </c>
-      <c r="O19" t="n">
-        <v>40.88</v>
-      </c>
       <c r="P19" t="n">
-        <v>39.21</v>
+        <v>39.79</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.83</v>
+        <v>40.62</v>
       </c>
       <c r="R19" t="n">
-        <v>-16.9841</v>
+        <v>1.1767</v>
       </c>
       <c r="S19" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="T19" t="n">
-        <v>-13.7705</v>
+        <v>-16.9952</v>
       </c>
       <c r="U19" t="n">
-        <v>-2.4091</v>
+        <v>-1.9778</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.1866</v>
+        <v>-1.8928</v>
       </c>
       <c r="W19" t="n">
-        <v>-4.2835</v>
+        <v>-5.9035</v>
       </c>
       <c r="X19" t="n">
-        <v>17.1953</v>
+        <v>-1.2179</v>
       </c>
       <c r="Y19" t="n">
-        <v>19.6346</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z19" t="n">
-        <v>11.6314</v>
+        <v>15.9256</v>
       </c>
       <c r="AA19" t="n">
-        <v>2.4698</v>
+        <v>1.9834</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.0797</v>
+        <v>1.8045</v>
       </c>
       <c r="AC19" t="n">
-        <v>4.3216</v>
+        <v>6.0298</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>104.55</v>
+        <v>107.44</v>
       </c>
       <c r="C20" t="n">
-        <v>105.94</v>
+        <v>109.32</v>
       </c>
       <c r="D20" t="n">
-        <v>100.96</v>
+        <v>101.06</v>
       </c>
       <c r="E20" t="n">
-        <v>102.32</v>
+        <v>103.97</v>
       </c>
       <c r="F20" t="n">
-        <v>69.13</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>69.33</v>
+        <v>69.97</v>
       </c>
       <c r="H20" t="n">
-        <v>67.61</v>
+        <v>66.55</v>
       </c>
       <c r="I20" t="n">
-        <v>67.90000000000001</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>49.87</v>
+        <v>48.55</v>
       </c>
       <c r="K20" t="n">
-        <v>51.8</v>
+        <v>51.74</v>
       </c>
       <c r="L20" t="n">
-        <v>49.26</v>
+        <v>47.57</v>
       </c>
       <c r="M20" t="n">
-        <v>51.1</v>
+        <v>50.11</v>
       </c>
       <c r="N20" t="n">
-        <v>39.91</v>
+        <v>40.06</v>
       </c>
       <c r="O20" t="n">
-        <v>40.78</v>
+        <v>41.44</v>
       </c>
       <c r="P20" t="n">
-        <v>39.79</v>
+        <v>39.37</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.62</v>
+        <v>40.61</v>
       </c>
       <c r="R20" t="n">
-        <v>1.1767</v>
+        <v>1.6126</v>
       </c>
       <c r="S20" t="n">
-        <v>-11.6102</v>
+        <v>-14.6528</v>
       </c>
       <c r="T20" t="n">
-        <v>-16.9952</v>
+        <v>-17.3989</v>
       </c>
       <c r="U20" t="n">
-        <v>-1.9778</v>
+        <v>0.0442</v>
       </c>
       <c r="V20" t="n">
-        <v>-1.8928</v>
+        <v>-4.297</v>
       </c>
       <c r="W20" t="n">
-        <v>-5.9035</v>
+        <v>-5.0594</v>
       </c>
       <c r="X20" t="n">
-        <v>-1.2179</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y20" t="n">
-        <v>9.328200000000001</v>
+        <v>13.5251</v>
       </c>
       <c r="Z20" t="n">
-        <v>15.9256</v>
+        <v>15.8881</v>
       </c>
       <c r="AA20" t="n">
-        <v>1.9834</v>
+        <v>-0.0246</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.8045</v>
+        <v>4.4765</v>
       </c>
       <c r="AC20" t="n">
-        <v>6.0298</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>107.44</v>
+        <v>113.33</v>
       </c>
       <c r="C21" t="n">
-        <v>109.32</v>
+        <v>115.48</v>
       </c>
       <c r="D21" t="n">
-        <v>101.06</v>
+        <v>112.01</v>
       </c>
       <c r="E21" t="n">
-        <v>103.97</v>
+        <v>114.82</v>
       </c>
       <c r="F21" t="n">
-        <v>68.84999999999999</v>
+        <v>71.13</v>
       </c>
       <c r="G21" t="n">
-        <v>69.97</v>
+        <v>71.72</v>
       </c>
       <c r="H21" t="n">
-        <v>66.55</v>
+        <v>70.37</v>
       </c>
       <c r="I21" t="n">
-        <v>67.93000000000001</v>
+        <v>71.38</v>
       </c>
       <c r="J21" t="n">
-        <v>48.55</v>
+        <v>45.72</v>
       </c>
       <c r="K21" t="n">
-        <v>51.74</v>
+        <v>46.34</v>
       </c>
       <c r="L21" t="n">
-        <v>47.57</v>
+        <v>44.67</v>
       </c>
       <c r="M21" t="n">
-        <v>50.11</v>
+        <v>44.99</v>
       </c>
       <c r="N21" t="n">
-        <v>40.06</v>
+        <v>38.69</v>
       </c>
       <c r="O21" t="n">
-        <v>41.44</v>
+        <v>39.14</v>
       </c>
       <c r="P21" t="n">
-        <v>39.37</v>
+        <v>38.33</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.61</v>
+        <v>38.53</v>
       </c>
       <c r="R21" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="S21" t="n">
-        <v>-14.6528</v>
+        <v>13.537</v>
       </c>
       <c r="T21" t="n">
-        <v>-17.3989</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U21" t="n">
-        <v>0.0442</v>
+        <v>5.0788</v>
       </c>
       <c r="V21" t="n">
-        <v>-4.297</v>
+        <v>3.0461</v>
       </c>
       <c r="W21" t="n">
-        <v>-5.0594</v>
+        <v>3.1354</v>
       </c>
       <c r="X21" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y21" t="n">
-        <v>13.5251</v>
+        <v>-13.0292</v>
       </c>
       <c r="Z21" t="n">
-        <v>15.8881</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA21" t="n">
-        <v>-0.0246</v>
+        <v>-5.1219</v>
       </c>
       <c r="AB21" t="n">
-        <v>4.4765</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC21" t="n">
-        <v>5.0983</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>113.33</v>
+        <v>117.03</v>
       </c>
       <c r="C22" t="n">
-        <v>115.48</v>
+        <v>123.86</v>
       </c>
       <c r="D22" t="n">
-        <v>112.0101</v>
+        <v>116.68</v>
       </c>
       <c r="E22" t="n">
-        <v>114.82</v>
+        <v>123.67</v>
       </c>
       <c r="F22" t="n">
-        <v>71.13</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>71.72</v>
+        <v>72.7777</v>
       </c>
       <c r="H22" t="n">
-        <v>70.37</v>
+        <v>70.8094</v>
       </c>
       <c r="I22" t="n">
-        <v>71.38</v>
+        <v>72.64</v>
       </c>
       <c r="J22" t="n">
-        <v>45.715</v>
+        <v>44.11</v>
       </c>
       <c r="K22" t="n">
-        <v>46.34</v>
+        <v>44.26</v>
       </c>
       <c r="L22" t="n">
-        <v>44.67</v>
+        <v>41.465</v>
       </c>
       <c r="M22" t="n">
-        <v>44.99</v>
+        <v>41.49</v>
       </c>
       <c r="N22" t="n">
-        <v>38.68</v>
+        <v>38.25</v>
       </c>
       <c r="O22" t="n">
-        <v>39.14</v>
+        <v>38.8675</v>
       </c>
       <c r="P22" t="n">
-        <v>38.33</v>
+        <v>37.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>38.53</v>
+        <v>37.87</v>
       </c>
       <c r="R22" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="S22" t="n">
-        <v>13.537</v>
+        <v>20.8659</v>
       </c>
       <c r="T22" t="n">
-        <v>-0.8120000000000001</v>
+        <v>1.5186</v>
       </c>
       <c r="U22" t="n">
-        <v>5.0788</v>
+        <v>1.7652</v>
       </c>
       <c r="V22" t="n">
-        <v>3.0461</v>
+        <v>6.9809</v>
       </c>
       <c r="W22" t="n">
-        <v>3.1354</v>
+        <v>2.3387</v>
       </c>
       <c r="X22" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y22" t="n">
-        <v>-13.0292</v>
+        <v>-18.8063</v>
       </c>
       <c r="Z22" t="n">
-        <v>-3.7441</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA22" t="n">
-        <v>-5.1219</v>
+        <v>-1.713</v>
       </c>
       <c r="AB22" t="n">
-        <v>-3.2639</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC22" t="n">
-        <v>-3.4336</v>
+        <v>-2.5727</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-22 00:36
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1804 +568,1629 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>119.99</v>
+        <v>115.07</v>
       </c>
       <c r="C2" t="n">
-        <v>124.56</v>
+        <v>115.07</v>
       </c>
       <c r="D2" t="n">
-        <v>117.42</v>
+        <v>106</v>
       </c>
       <c r="E2" t="n">
-        <v>122.21</v>
+        <v>111.16</v>
       </c>
       <c r="F2" t="n">
-        <v>70.83</v>
+        <v>70</v>
       </c>
       <c r="G2" t="n">
-        <v>71.69</v>
+        <v>70.05</v>
       </c>
       <c r="H2" t="n">
-        <v>69.76000000000001</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>70.48</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>47.33</v>
+        <v>49.14</v>
       </c>
       <c r="K2" t="n">
-        <v>48.29</v>
+        <v>52.81</v>
       </c>
       <c r="L2" t="n">
-        <v>45.47</v>
+        <v>49.13</v>
       </c>
       <c r="M2" t="n">
-        <v>46.25</v>
+        <v>50.75</v>
       </c>
       <c r="N2" t="n">
-        <v>39.18</v>
+        <v>39.65</v>
       </c>
       <c r="O2" t="n">
-        <v>39.77</v>
+        <v>40.79</v>
       </c>
       <c r="P2" t="n">
-        <v>38.74</v>
+        <v>39.64</v>
       </c>
       <c r="Q2" t="n">
-        <v>39.37</v>
+        <v>40.19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>126.59</v>
+        <v>117.37</v>
       </c>
       <c r="C3" t="n">
-        <v>126.79</v>
+        <v>119.88</v>
       </c>
       <c r="D3" t="n">
-        <v>116.71</v>
+        <v>113.13</v>
       </c>
       <c r="E3" t="n">
-        <v>120.6</v>
+        <v>115.67</v>
       </c>
       <c r="F3" t="n">
-        <v>71.7</v>
+        <v>70.42</v>
       </c>
       <c r="G3" t="n">
-        <v>71.83</v>
+        <v>71.27</v>
       </c>
       <c r="H3" t="n">
-        <v>69.91</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>71.17</v>
+        <v>70.27</v>
       </c>
       <c r="J3" t="n">
-        <v>44.67</v>
+        <v>47.82</v>
       </c>
       <c r="K3" t="n">
-        <v>48.46</v>
+        <v>49.83</v>
       </c>
       <c r="L3" t="n">
-        <v>44.65</v>
+        <v>46.66</v>
       </c>
       <c r="M3" t="n">
-        <v>47.03</v>
+        <v>48.42</v>
       </c>
       <c r="N3" t="n">
-        <v>38.71</v>
+        <v>39.38</v>
       </c>
       <c r="O3" t="n">
-        <v>39.72</v>
+        <v>40.02</v>
       </c>
       <c r="P3" t="n">
-        <v>38.64</v>
+        <v>38.89</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.02</v>
+        <v>39.46</v>
       </c>
       <c r="R3" t="n">
-        <v>-1.3174</v>
+        <v>4.0572</v>
       </c>
       <c r="U3" t="n">
-        <v>0.979</v>
+        <v>1.8258</v>
       </c>
       <c r="X3" t="n">
-        <v>1.6865</v>
+        <v>-4.5911</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.889</v>
+        <v>-1.8164</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>115.07</v>
+        <v>114.7</v>
       </c>
       <c r="C4" t="n">
-        <v>115.07</v>
+        <v>117.39</v>
       </c>
       <c r="D4" t="n">
-        <v>106</v>
+        <v>112.53</v>
       </c>
       <c r="E4" t="n">
-        <v>111.16</v>
+        <v>116.6</v>
       </c>
       <c r="F4" t="n">
-        <v>70</v>
+        <v>69.56</v>
       </c>
       <c r="G4" t="n">
-        <v>70.05</v>
+        <v>70.94</v>
       </c>
       <c r="H4" t="n">
-        <v>67.93000000000001</v>
+        <v>69.44</v>
       </c>
       <c r="I4" t="n">
-        <v>69.01000000000001</v>
+        <v>70.47</v>
       </c>
       <c r="J4" t="n">
-        <v>49.14</v>
+        <v>49.01</v>
       </c>
       <c r="K4" t="n">
-        <v>52.81</v>
+        <v>49.89</v>
       </c>
       <c r="L4" t="n">
-        <v>49.13</v>
+        <v>47.87</v>
       </c>
       <c r="M4" t="n">
-        <v>50.75</v>
+        <v>48.09</v>
       </c>
       <c r="N4" t="n">
-        <v>39.65</v>
+        <v>39.86</v>
       </c>
       <c r="O4" t="n">
-        <v>40.79</v>
+        <v>39.93</v>
       </c>
       <c r="P4" t="n">
-        <v>39.64</v>
+        <v>39.09</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.19</v>
+        <v>39.38</v>
       </c>
       <c r="R4" t="n">
-        <v>-7.8275</v>
+        <v>0.804</v>
       </c>
       <c r="U4" t="n">
-        <v>-3.035</v>
+        <v>0.2846</v>
       </c>
       <c r="X4" t="n">
-        <v>7.9098</v>
+        <v>-0.6815</v>
       </c>
       <c r="AA4" t="n">
-        <v>2.9985</v>
+        <v>-0.2027</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>117.37</v>
+        <v>123.4</v>
       </c>
       <c r="C5" t="n">
-        <v>119.88</v>
+        <v>124.88</v>
       </c>
       <c r="D5" t="n">
-        <v>113.13</v>
+        <v>117.69</v>
       </c>
       <c r="E5" t="n">
-        <v>115.67</v>
+        <v>123.05</v>
       </c>
       <c r="F5" t="n">
-        <v>70.42</v>
+        <v>72.09</v>
       </c>
       <c r="G5" t="n">
-        <v>71.27</v>
+        <v>73.38</v>
       </c>
       <c r="H5" t="n">
-        <v>69.34999999999999</v>
+        <v>71.38</v>
       </c>
       <c r="I5" t="n">
-        <v>70.27</v>
+        <v>73.3</v>
       </c>
       <c r="J5" t="n">
-        <v>47.82</v>
+        <v>45.42</v>
       </c>
       <c r="K5" t="n">
-        <v>49.83</v>
+        <v>47.71</v>
       </c>
       <c r="L5" t="n">
-        <v>46.66</v>
+        <v>44.71</v>
       </c>
       <c r="M5" t="n">
-        <v>48.42</v>
+        <v>45.35</v>
       </c>
       <c r="N5" t="n">
-        <v>39.38</v>
+        <v>38.46</v>
       </c>
       <c r="O5" t="n">
-        <v>40.02</v>
+        <v>38.86</v>
       </c>
       <c r="P5" t="n">
-        <v>38.89</v>
+        <v>37.73</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.46</v>
+        <v>37.78</v>
       </c>
       <c r="R5" t="n">
-        <v>4.0572</v>
+        <v>5.5317</v>
       </c>
       <c r="S5" t="n">
-        <v>-5.3514</v>
+        <v>10.6963</v>
       </c>
       <c r="U5" t="n">
-        <v>1.8258</v>
+        <v>4.0159</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.298</v>
+        <v>6.2165</v>
       </c>
       <c r="X5" t="n">
-        <v>-4.5911</v>
+        <v>-5.6977</v>
       </c>
       <c r="Y5" t="n">
-        <v>4.6919</v>
+        <v>-10.6404</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.8164</v>
+        <v>-4.063</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.2286</v>
+        <v>-5.9965</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>114.7</v>
+        <v>119.92</v>
       </c>
       <c r="C6" t="n">
-        <v>117.39</v>
+        <v>121.2</v>
       </c>
       <c r="D6" t="n">
-        <v>112.53</v>
+        <v>110.21</v>
       </c>
       <c r="E6" t="n">
-        <v>116.6</v>
+        <v>111.34</v>
       </c>
       <c r="F6" t="n">
-        <v>69.56</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>70.94</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>69.44</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>70.47</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>49.01</v>
+        <v>46.61</v>
       </c>
       <c r="K6" t="n">
-        <v>49.89</v>
+        <v>50.23</v>
       </c>
       <c r="L6" t="n">
-        <v>47.87</v>
+        <v>46.15</v>
       </c>
       <c r="M6" t="n">
-        <v>48.09</v>
+        <v>49.82</v>
       </c>
       <c r="N6" t="n">
-        <v>39.86</v>
+        <v>38.02</v>
       </c>
       <c r="O6" t="n">
-        <v>39.93</v>
+        <v>38.76</v>
       </c>
       <c r="P6" t="n">
-        <v>39.09</v>
+        <v>37.33</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.38</v>
+        <v>38.54</v>
       </c>
       <c r="R6" t="n">
-        <v>0.804</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="S6" t="n">
-        <v>-3.3167</v>
+        <v>-3.7434</v>
       </c>
       <c r="U6" t="n">
-        <v>0.2846</v>
+        <v>-1.9782</v>
       </c>
       <c r="V6" t="n">
-        <v>-0.9836</v>
+        <v>2.2485</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.6815</v>
+        <v>9.8567</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.2539</v>
+        <v>2.8914</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.2027</v>
+        <v>2.0116</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.9226</v>
+        <v>-2.3315</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>123.4</v>
+        <v>112.41</v>
       </c>
       <c r="C7" t="n">
-        <v>124.88</v>
+        <v>115.05</v>
       </c>
       <c r="D7" t="n">
-        <v>117.69</v>
+        <v>110.33</v>
       </c>
       <c r="E7" t="n">
-        <v>123.05</v>
+        <v>112.79</v>
       </c>
       <c r="F7" t="n">
-        <v>72.09</v>
+        <v>71.44</v>
       </c>
       <c r="G7" t="n">
-        <v>73.38</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>71.38</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>73.3</v>
+        <v>71.92</v>
       </c>
       <c r="J7" t="n">
-        <v>45.42</v>
+        <v>49.27</v>
       </c>
       <c r="K7" t="n">
-        <v>47.71</v>
+        <v>50.24</v>
       </c>
       <c r="L7" t="n">
-        <v>44.71</v>
+        <v>48.09</v>
       </c>
       <c r="M7" t="n">
-        <v>45.35</v>
+        <v>49.02</v>
       </c>
       <c r="N7" t="n">
-        <v>38.46</v>
+        <v>38.77</v>
       </c>
       <c r="O7" t="n">
-        <v>38.86</v>
+        <v>39.09</v>
       </c>
       <c r="P7" t="n">
-        <v>37.73</v>
+        <v>38.37</v>
       </c>
       <c r="Q7" t="n">
-        <v>37.78</v>
+        <v>38.51</v>
       </c>
       <c r="R7" t="n">
-        <v>5.5317</v>
+        <v>1.3023</v>
       </c>
       <c r="S7" t="n">
-        <v>10.6963</v>
+        <v>-3.2676</v>
       </c>
       <c r="T7" t="n">
-        <v>0.6873</v>
+        <v>1.4664</v>
       </c>
       <c r="U7" t="n">
-        <v>4.0159</v>
+        <v>0.0974</v>
       </c>
       <c r="V7" t="n">
-        <v>6.2165</v>
+        <v>2.0576</v>
       </c>
       <c r="W7" t="n">
-        <v>4.0011</v>
+        <v>4.2168</v>
       </c>
       <c r="X7" t="n">
-        <v>-5.6977</v>
+        <v>-1.6058</v>
       </c>
       <c r="Y7" t="n">
-        <v>-10.6404</v>
+        <v>1.9339</v>
       </c>
       <c r="Z7" t="n">
-        <v>-1.9459</v>
+        <v>-3.4089</v>
       </c>
       <c r="AA7" t="n">
-        <v>-4.063</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="AB7" t="n">
-        <v>-5.9965</v>
+        <v>-2.2092</v>
       </c>
       <c r="AC7" t="n">
-        <v>-4.0386</v>
+        <v>-4.1801</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>119.92</v>
+        <v>106.36</v>
       </c>
       <c r="C8" t="n">
-        <v>121.2</v>
+        <v>108.64</v>
       </c>
       <c r="D8" t="n">
-        <v>110.21</v>
+        <v>102.31</v>
       </c>
       <c r="E8" t="n">
-        <v>111.34</v>
+        <v>105.91</v>
       </c>
       <c r="F8" t="n">
-        <v>72.84999999999999</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>74.18000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="H8" t="n">
-        <v>71.43000000000001</v>
+        <v>68.25</v>
       </c>
       <c r="I8" t="n">
-        <v>71.84999999999999</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>46.61</v>
+        <v>51.88</v>
       </c>
       <c r="K8" t="n">
-        <v>50.23</v>
+        <v>53.69</v>
       </c>
       <c r="L8" t="n">
-        <v>46.15</v>
+        <v>50.9</v>
       </c>
       <c r="M8" t="n">
-        <v>49.82</v>
+        <v>52.22</v>
       </c>
       <c r="N8" t="n">
-        <v>38.02</v>
+        <v>40.03</v>
       </c>
       <c r="O8" t="n">
-        <v>38.76</v>
+        <v>40.47</v>
       </c>
       <c r="P8" t="n">
-        <v>37.33</v>
+        <v>39.23</v>
       </c>
       <c r="Q8" t="n">
-        <v>38.54</v>
+        <v>39.97</v>
       </c>
       <c r="R8" t="n">
-        <v>-9.516500000000001</v>
+        <v>-6.0998</v>
       </c>
       <c r="S8" t="n">
-        <v>-3.7434</v>
+        <v>-13.9293</v>
       </c>
       <c r="T8" t="n">
-        <v>-7.6783</v>
+        <v>-8.437799999999999</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.9782</v>
+        <v>-3.8515</v>
       </c>
       <c r="V8" t="n">
-        <v>2.2485</v>
+        <v>-5.6617</v>
       </c>
       <c r="W8" t="n">
-        <v>0.9555</v>
+        <v>-1.5939</v>
       </c>
       <c r="X8" t="n">
-        <v>9.8567</v>
+        <v>6.5279</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.8914</v>
+        <v>15.1488</v>
       </c>
       <c r="Z8" t="n">
-        <v>5.9324</v>
+        <v>7.848</v>
       </c>
       <c r="AA8" t="n">
-        <v>2.0116</v>
+        <v>3.7912</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.3315</v>
+        <v>5.7967</v>
       </c>
       <c r="AC8" t="n">
-        <v>-1.2301</v>
+        <v>1.2924</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>112.41</v>
+        <v>104.5</v>
       </c>
       <c r="C9" t="n">
-        <v>115.05</v>
+        <v>108.07</v>
       </c>
       <c r="D9" t="n">
-        <v>110.33</v>
+        <v>101.34</v>
       </c>
       <c r="E9" t="n">
-        <v>112.79</v>
+        <v>106.35</v>
       </c>
       <c r="F9" t="n">
-        <v>71.44</v>
+        <v>68.97</v>
       </c>
       <c r="G9" t="n">
-        <v>72.15000000000001</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>70.81999999999999</v>
+        <v>68.39</v>
       </c>
       <c r="I9" t="n">
-        <v>71.92</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>49.27</v>
+        <v>52.8</v>
       </c>
       <c r="K9" t="n">
-        <v>50.24</v>
+        <v>54.39</v>
       </c>
       <c r="L9" t="n">
-        <v>48.09</v>
+        <v>51.05</v>
       </c>
       <c r="M9" t="n">
-        <v>49.02</v>
+        <v>51.83</v>
       </c>
       <c r="N9" t="n">
-        <v>38.77</v>
+        <v>40.09</v>
       </c>
       <c r="O9" t="n">
-        <v>39.09</v>
+        <v>40.43</v>
       </c>
       <c r="P9" t="n">
-        <v>38.37</v>
+        <v>39.63</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.51</v>
+        <v>39.71</v>
       </c>
       <c r="R9" t="n">
-        <v>1.3023</v>
+        <v>0.4154</v>
       </c>
       <c r="S9" t="n">
-        <v>-3.2676</v>
+        <v>-4.4818</v>
       </c>
       <c r="T9" t="n">
-        <v>1.4664</v>
+        <v>-8.790699999999999</v>
       </c>
       <c r="U9" t="n">
-        <v>0.0974</v>
+        <v>0.6508</v>
       </c>
       <c r="V9" t="n">
-        <v>2.0576</v>
+        <v>-3.1315</v>
       </c>
       <c r="W9" t="n">
-        <v>4.2168</v>
+        <v>-1.2346</v>
       </c>
       <c r="X9" t="n">
-        <v>-1.6058</v>
+        <v>-0.7468</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.9339</v>
+        <v>4.0345</v>
       </c>
       <c r="Z9" t="n">
-        <v>-3.4089</v>
+        <v>7.7771</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.07779999999999999</v>
+        <v>-0.6505</v>
       </c>
       <c r="AB9" t="n">
-        <v>-2.2092</v>
+        <v>3.0358</v>
       </c>
       <c r="AC9" t="n">
-        <v>-4.1801</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>106.36</v>
+        <v>103</v>
       </c>
       <c r="C10" t="n">
-        <v>108.64</v>
+        <v>107.49</v>
       </c>
       <c r="D10" t="n">
-        <v>102.31</v>
+        <v>98.62</v>
       </c>
       <c r="E10" t="n">
-        <v>105.91</v>
+        <v>106.74</v>
       </c>
       <c r="F10" t="n">
-        <v>69.06999999999999</v>
+        <v>70.06</v>
       </c>
       <c r="G10" t="n">
-        <v>70.55</v>
+        <v>72.42</v>
       </c>
       <c r="H10" t="n">
-        <v>68.25</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>69.15000000000001</v>
+        <v>72.03</v>
       </c>
       <c r="J10" t="n">
-        <v>51.88</v>
+        <v>53.5</v>
       </c>
       <c r="K10" t="n">
-        <v>53.69</v>
+        <v>55.69</v>
       </c>
       <c r="L10" t="n">
-        <v>50.9</v>
+        <v>51.28</v>
       </c>
       <c r="M10" t="n">
-        <v>52.22</v>
+        <v>51.6</v>
       </c>
       <c r="N10" t="n">
-        <v>40.03</v>
+        <v>39.49</v>
       </c>
       <c r="O10" t="n">
-        <v>40.47</v>
+        <v>39.68</v>
       </c>
       <c r="P10" t="n">
-        <v>39.23</v>
+        <v>38.12</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.97</v>
+        <v>38.34</v>
       </c>
       <c r="R10" t="n">
-        <v>-6.0998</v>
+        <v>0.3667</v>
       </c>
       <c r="S10" t="n">
-        <v>-13.9293</v>
+        <v>-5.364</v>
       </c>
       <c r="T10" t="n">
-        <v>-8.437799999999999</v>
+        <v>-13.2548</v>
       </c>
       <c r="U10" t="n">
-        <v>-3.8515</v>
+        <v>3.4914</v>
       </c>
       <c r="V10" t="n">
-        <v>-5.6617</v>
+        <v>0.1529</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.5939</v>
+        <v>-1.7326</v>
       </c>
       <c r="X10" t="n">
-        <v>6.5279</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y10" t="n">
-        <v>15.1488</v>
+        <v>5.2632</v>
       </c>
       <c r="Z10" t="n">
-        <v>7.848</v>
+        <v>13.7817</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.7912</v>
+        <v>-3.45</v>
       </c>
       <c r="AB10" t="n">
-        <v>5.7967</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.2924</v>
+        <v>1.4823</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>104.5</v>
+        <v>111.22</v>
       </c>
       <c r="C11" t="n">
-        <v>108.07</v>
+        <v>118.18</v>
       </c>
       <c r="D11" t="n">
-        <v>101.34</v>
+        <v>109.73</v>
       </c>
       <c r="E11" t="n">
-        <v>106.35</v>
+        <v>117.28</v>
       </c>
       <c r="F11" t="n">
-        <v>68.97</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>69.76000000000001</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>68.39</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>69.59999999999999</v>
+        <v>72.37</v>
       </c>
       <c r="J11" t="n">
-        <v>52.8</v>
+        <v>49.56</v>
       </c>
       <c r="K11" t="n">
-        <v>54.39</v>
+        <v>50.21</v>
       </c>
       <c r="L11" t="n">
-        <v>51.05</v>
+        <v>46.1</v>
       </c>
       <c r="M11" t="n">
-        <v>51.83</v>
+        <v>46.34</v>
       </c>
       <c r="N11" t="n">
-        <v>40.09</v>
+        <v>38.12</v>
       </c>
       <c r="O11" t="n">
-        <v>40.43</v>
+        <v>38.58</v>
       </c>
       <c r="P11" t="n">
-        <v>39.63</v>
+        <v>37.72</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.71</v>
+        <v>38.18</v>
       </c>
       <c r="R11" t="n">
-        <v>0.4154</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S11" t="n">
-        <v>-4.4818</v>
+        <v>10.7355</v>
       </c>
       <c r="T11" t="n">
-        <v>-8.790699999999999</v>
+        <v>5.335</v>
       </c>
       <c r="U11" t="n">
-        <v>0.6508</v>
+        <v>0.472</v>
       </c>
       <c r="V11" t="n">
-        <v>-3.1315</v>
+        <v>4.6565</v>
       </c>
       <c r="W11" t="n">
-        <v>-1.2346</v>
+        <v>0.7237</v>
       </c>
       <c r="X11" t="n">
-        <v>-0.7468</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y11" t="n">
-        <v>4.0345</v>
+        <v>-11.2601</v>
       </c>
       <c r="Z11" t="n">
-        <v>7.7771</v>
+        <v>-6.9851</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.6505</v>
+        <v>-0.4173</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.0358</v>
+        <v>-4.4784</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.838</v>
+        <v>-0.9341</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>103</v>
+        <v>125.12</v>
       </c>
       <c r="C12" t="n">
-        <v>107.49</v>
+        <v>127.54</v>
       </c>
       <c r="D12" t="n">
-        <v>98.62</v>
+        <v>121.6</v>
       </c>
       <c r="E12" t="n">
-        <v>106.74</v>
+        <v>123.27</v>
       </c>
       <c r="F12" t="n">
-        <v>70.06</v>
+        <v>72.95</v>
       </c>
       <c r="G12" t="n">
-        <v>72.42</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>69.70999999999999</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>72.03</v>
+        <v>72.16</v>
       </c>
       <c r="J12" t="n">
-        <v>53.5</v>
+        <v>43.55</v>
       </c>
       <c r="K12" t="n">
-        <v>55.69</v>
+        <v>44.83</v>
       </c>
       <c r="L12" t="n">
-        <v>51.28</v>
+        <v>42.51</v>
       </c>
       <c r="M12" t="n">
-        <v>51.6</v>
+        <v>44.08</v>
       </c>
       <c r="N12" t="n">
-        <v>39.49</v>
+        <v>37.89</v>
       </c>
       <c r="O12" t="n">
-        <v>39.68</v>
+        <v>38.74</v>
       </c>
       <c r="P12" t="n">
-        <v>38.12</v>
+        <v>37.75</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.34</v>
+        <v>38.31</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3667</v>
+        <v>5.1074</v>
       </c>
       <c r="S12" t="n">
-        <v>-5.364</v>
+        <v>15.9097</v>
       </c>
       <c r="T12" t="n">
-        <v>-13.2548</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U12" t="n">
-        <v>3.4914</v>
+        <v>-0.2902</v>
       </c>
       <c r="V12" t="n">
-        <v>0.1529</v>
+        <v>3.6782</v>
       </c>
       <c r="W12" t="n">
-        <v>-1.7326</v>
+        <v>0.3337</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.4438</v>
+        <v>-4.877</v>
       </c>
       <c r="Y12" t="n">
-        <v>5.2632</v>
+        <v>-14.9527</v>
       </c>
       <c r="Z12" t="n">
-        <v>13.7817</v>
+        <v>-10.0775</v>
       </c>
       <c r="AA12" t="n">
-        <v>-3.45</v>
+        <v>0.3405</v>
       </c>
       <c r="AB12" t="n">
-        <v>-0.4414</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.4823</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>111.22</v>
+        <v>121.24</v>
       </c>
       <c r="C13" t="n">
-        <v>118.18</v>
+        <v>128.48</v>
       </c>
       <c r="D13" t="n">
-        <v>109.73</v>
+        <v>121.24</v>
       </c>
       <c r="E13" t="n">
-        <v>117.28</v>
+        <v>125.87</v>
       </c>
       <c r="F13" t="n">
-        <v>72.48999999999999</v>
+        <v>71.55</v>
       </c>
       <c r="G13" t="n">
-        <v>73.23999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="H13" t="n">
-        <v>71.65000000000001</v>
+        <v>70.84</v>
       </c>
       <c r="I13" t="n">
-        <v>72.37</v>
+        <v>71.55</v>
       </c>
       <c r="J13" t="n">
-        <v>49.56</v>
+        <v>44.8</v>
       </c>
       <c r="K13" t="n">
-        <v>50.21</v>
+        <v>44.82</v>
       </c>
       <c r="L13" t="n">
-        <v>46.1</v>
+        <v>42.32</v>
       </c>
       <c r="M13" t="n">
-        <v>46.34</v>
+        <v>43.24</v>
       </c>
       <c r="N13" t="n">
-        <v>38.12</v>
+        <v>38.63</v>
       </c>
       <c r="O13" t="n">
-        <v>38.58</v>
+        <v>39.01</v>
       </c>
       <c r="P13" t="n">
-        <v>37.72</v>
+        <v>38.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.18</v>
+        <v>38.64</v>
       </c>
       <c r="R13" t="n">
-        <v>9.874499999999999</v>
+        <v>2.1092</v>
       </c>
       <c r="S13" t="n">
-        <v>10.7355</v>
+        <v>17.9221</v>
       </c>
       <c r="T13" t="n">
-        <v>5.335</v>
+        <v>18.8462</v>
       </c>
       <c r="U13" t="n">
-        <v>0.472</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V13" t="n">
-        <v>4.6565</v>
+        <v>-0.6664</v>
       </c>
       <c r="W13" t="n">
-        <v>0.7237</v>
+        <v>3.4707</v>
       </c>
       <c r="X13" t="n">
-        <v>-10.1938</v>
+        <v>-1.9056</v>
       </c>
       <c r="Y13" t="n">
-        <v>-11.2601</v>
+        <v>-16.2016</v>
       </c>
       <c r="Z13" t="n">
-        <v>-6.9851</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.4173</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AB13" t="n">
-        <v>-4.4784</v>
+        <v>0.7825</v>
       </c>
       <c r="AC13" t="n">
-        <v>-0.9341</v>
+        <v>-3.3275</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>125.12</v>
+        <v>116.35</v>
       </c>
       <c r="C14" t="n">
-        <v>127.54</v>
+        <v>119.32</v>
       </c>
       <c r="D14" t="n">
-        <v>121.6</v>
+        <v>113.55</v>
       </c>
       <c r="E14" t="n">
-        <v>123.27</v>
+        <v>115.76</v>
       </c>
       <c r="F14" t="n">
-        <v>72.95</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>73.20999999999999</v>
+        <v>70.23</v>
       </c>
       <c r="H14" t="n">
-        <v>71.31999999999999</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>72.16</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>43.55</v>
+        <v>46.52</v>
       </c>
       <c r="K14" t="n">
-        <v>44.83</v>
+        <v>47.49</v>
       </c>
       <c r="L14" t="n">
-        <v>42.51</v>
+        <v>45.5</v>
       </c>
       <c r="M14" t="n">
-        <v>44.08</v>
+        <v>46.74</v>
       </c>
       <c r="N14" t="n">
-        <v>37.89</v>
+        <v>40.08</v>
       </c>
       <c r="O14" t="n">
-        <v>38.74</v>
+        <v>40.19</v>
       </c>
       <c r="P14" t="n">
-        <v>37.75</v>
+        <v>39.35</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.31</v>
+        <v>39.9</v>
       </c>
       <c r="R14" t="n">
-        <v>5.1074</v>
+        <v>-8.0321</v>
       </c>
       <c r="S14" t="n">
-        <v>15.9097</v>
+        <v>-1.296</v>
       </c>
       <c r="T14" t="n">
-        <v>9.291600000000001</v>
+        <v>8.848100000000001</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.2902</v>
+        <v>-3.2704</v>
       </c>
       <c r="V14" t="n">
-        <v>3.6782</v>
+        <v>-4.3665</v>
       </c>
       <c r="W14" t="n">
-        <v>0.3337</v>
+        <v>-0.5603</v>
       </c>
       <c r="X14" t="n">
-        <v>-4.877</v>
+        <v>8.0944</v>
       </c>
       <c r="Y14" t="n">
-        <v>-14.9527</v>
+        <v>0.8632</v>
       </c>
       <c r="Z14" t="n">
-        <v>-10.0775</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.3405</v>
+        <v>3.2609</v>
       </c>
       <c r="AB14" t="n">
-        <v>-3.5256</v>
+        <v>4.505</v>
       </c>
       <c r="AC14" t="n">
-        <v>-0.5193</v>
+        <v>0.4785</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>121.24</v>
+        <v>120.71</v>
       </c>
       <c r="C15" t="n">
-        <v>128.48</v>
+        <v>124.5</v>
       </c>
       <c r="D15" t="n">
-        <v>121.24</v>
+        <v>117.87</v>
       </c>
       <c r="E15" t="n">
-        <v>125.87</v>
+        <v>121.82</v>
       </c>
       <c r="F15" t="n">
-        <v>71.55</v>
+        <v>71.19</v>
       </c>
       <c r="G15" t="n">
-        <v>72.55</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>70.84</v>
+        <v>70.61</v>
       </c>
       <c r="I15" t="n">
-        <v>71.55</v>
+        <v>70.98</v>
       </c>
       <c r="J15" t="n">
-        <v>44.8</v>
+        <v>44.69</v>
       </c>
       <c r="K15" t="n">
-        <v>44.82</v>
+        <v>45.82</v>
       </c>
       <c r="L15" t="n">
-        <v>42.32</v>
+        <v>43.12</v>
       </c>
       <c r="M15" t="n">
-        <v>43.24</v>
+        <v>44.14</v>
       </c>
       <c r="N15" t="n">
-        <v>38.63</v>
+        <v>38.77</v>
       </c>
       <c r="O15" t="n">
-        <v>39.01</v>
+        <v>39.1</v>
       </c>
       <c r="P15" t="n">
-        <v>38.1</v>
+        <v>38.42</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.64</v>
+        <v>38.87</v>
       </c>
       <c r="R15" t="n">
-        <v>2.1092</v>
+        <v>5.235</v>
       </c>
       <c r="S15" t="n">
-        <v>17.9221</v>
+        <v>-1.1763</v>
       </c>
       <c r="T15" t="n">
-        <v>18.8462</v>
+        <v>14.1278</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.8453000000000001</v>
+        <v>2.5574</v>
       </c>
       <c r="V15" t="n">
-        <v>-0.6664</v>
+        <v>-1.6353</v>
       </c>
       <c r="W15" t="n">
-        <v>3.4707</v>
+        <v>-1.4577</v>
       </c>
       <c r="X15" t="n">
-        <v>-1.9056</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y15" t="n">
-        <v>-16.2016</v>
+        <v>0.1361</v>
       </c>
       <c r="Z15" t="n">
-        <v>-17.1965</v>
+        <v>-14.4574</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.8614000000000001</v>
+        <v>-2.5815</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.7825</v>
+        <v>1.4618</v>
       </c>
       <c r="AC15" t="n">
-        <v>-3.3275</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>116.35</v>
+        <v>101.53</v>
       </c>
       <c r="C16" t="n">
-        <v>119.32</v>
+        <v>105.39</v>
       </c>
       <c r="D16" t="n">
-        <v>113.55</v>
+        <v>99.87</v>
       </c>
       <c r="E16" t="n">
-        <v>115.76</v>
+        <v>101.13</v>
       </c>
       <c r="F16" t="n">
-        <v>68.90000000000001</v>
+        <v>67.53</v>
       </c>
       <c r="G16" t="n">
-        <v>70.23</v>
+        <v>70.39</v>
       </c>
       <c r="H16" t="n">
-        <v>68.68000000000001</v>
+        <v>67.34</v>
       </c>
       <c r="I16" t="n">
-        <v>69.20999999999999</v>
+        <v>69.27</v>
       </c>
       <c r="J16" t="n">
-        <v>46.52</v>
+        <v>51.61</v>
       </c>
       <c r="K16" t="n">
-        <v>47.49</v>
+        <v>52.22</v>
       </c>
       <c r="L16" t="n">
-        <v>45.5</v>
+        <v>50.21</v>
       </c>
       <c r="M16" t="n">
-        <v>46.74</v>
+        <v>51.73</v>
       </c>
       <c r="N16" t="n">
-        <v>40.08</v>
+        <v>40.78</v>
       </c>
       <c r="O16" t="n">
-        <v>40.19</v>
+        <v>40.88</v>
       </c>
       <c r="P16" t="n">
-        <v>39.35</v>
+        <v>39.21</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.9</v>
+        <v>39.83</v>
       </c>
       <c r="R16" t="n">
-        <v>-8.0321</v>
+        <v>-16.9841</v>
       </c>
       <c r="S16" t="n">
-        <v>-1.296</v>
+        <v>-19.6552</v>
       </c>
       <c r="T16" t="n">
-        <v>8.848100000000001</v>
+        <v>-13.7705</v>
       </c>
       <c r="U16" t="n">
-        <v>-3.2704</v>
+        <v>-2.4091</v>
       </c>
       <c r="V16" t="n">
-        <v>-4.3665</v>
+        <v>-3.1866</v>
       </c>
       <c r="W16" t="n">
-        <v>-0.5603</v>
+        <v>-4.2835</v>
       </c>
       <c r="X16" t="n">
-        <v>8.0944</v>
+        <v>17.1953</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.8632</v>
+        <v>19.6346</v>
       </c>
       <c r="Z16" t="n">
-        <v>-9.820600000000001</v>
+        <v>11.6314</v>
       </c>
       <c r="AA16" t="n">
-        <v>3.2609</v>
+        <v>2.4698</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.505</v>
+        <v>3.0797</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.4785</v>
+        <v>4.3216</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>120.71</v>
+        <v>104.55</v>
       </c>
       <c r="C17" t="n">
-        <v>124.5</v>
+        <v>105.94</v>
       </c>
       <c r="D17" t="n">
-        <v>117.87</v>
+        <v>100.96</v>
       </c>
       <c r="E17" t="n">
-        <v>121.82</v>
+        <v>102.32</v>
       </c>
       <c r="F17" t="n">
-        <v>71.19</v>
+        <v>69.13</v>
       </c>
       <c r="G17" t="n">
-        <v>71.76000000000001</v>
+        <v>69.33</v>
       </c>
       <c r="H17" t="n">
-        <v>70.61</v>
+        <v>67.61</v>
       </c>
       <c r="I17" t="n">
-        <v>70.98</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>44.69</v>
+        <v>49.87</v>
       </c>
       <c r="K17" t="n">
-        <v>45.82</v>
+        <v>51.8</v>
       </c>
       <c r="L17" t="n">
-        <v>43.12</v>
+        <v>49.26</v>
       </c>
       <c r="M17" t="n">
-        <v>44.14</v>
+        <v>51.1</v>
       </c>
       <c r="N17" t="n">
-        <v>38.77</v>
+        <v>39.91</v>
       </c>
       <c r="O17" t="n">
-        <v>39.1</v>
+        <v>40.78</v>
       </c>
       <c r="P17" t="n">
-        <v>38.42</v>
+        <v>39.79</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.87</v>
+        <v>40.62</v>
       </c>
       <c r="R17" t="n">
-        <v>5.235</v>
+        <v>1.1767</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.1763</v>
+        <v>-11.6102</v>
       </c>
       <c r="T17" t="n">
-        <v>14.1278</v>
+        <v>-16.9952</v>
       </c>
       <c r="U17" t="n">
-        <v>2.5574</v>
+        <v>-1.9778</v>
       </c>
       <c r="V17" t="n">
-        <v>-1.6353</v>
+        <v>-1.8928</v>
       </c>
       <c r="W17" t="n">
-        <v>-1.4577</v>
+        <v>-5.9035</v>
       </c>
       <c r="X17" t="n">
-        <v>-5.5627</v>
+        <v>-1.2179</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.1361</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z17" t="n">
-        <v>-14.4574</v>
+        <v>15.9256</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.5815</v>
+        <v>1.9834</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.4618</v>
+        <v>1.8045</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.3824</v>
+        <v>6.0298</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>101.53</v>
+        <v>107.44</v>
       </c>
       <c r="C18" t="n">
-        <v>105.39</v>
+        <v>109.32</v>
       </c>
       <c r="D18" t="n">
-        <v>99.87</v>
+        <v>101.06</v>
       </c>
       <c r="E18" t="n">
-        <v>101.13</v>
+        <v>103.97</v>
       </c>
       <c r="F18" t="n">
-        <v>67.53</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>70.39</v>
+        <v>69.97</v>
       </c>
       <c r="H18" t="n">
-        <v>67.34</v>
+        <v>66.55</v>
       </c>
       <c r="I18" t="n">
-        <v>69.27</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>51.61</v>
+        <v>48.55</v>
       </c>
       <c r="K18" t="n">
-        <v>52.22</v>
+        <v>51.74</v>
       </c>
       <c r="L18" t="n">
-        <v>50.21</v>
+        <v>47.57</v>
       </c>
       <c r="M18" t="n">
-        <v>51.73</v>
+        <v>50.11</v>
       </c>
       <c r="N18" t="n">
-        <v>40.78</v>
+        <v>40.06</v>
       </c>
       <c r="O18" t="n">
-        <v>40.88</v>
+        <v>41.44</v>
       </c>
       <c r="P18" t="n">
-        <v>39.21</v>
+        <v>39.37</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.83</v>
+        <v>40.61</v>
       </c>
       <c r="R18" t="n">
-        <v>-16.9841</v>
+        <v>1.6126</v>
       </c>
       <c r="S18" t="n">
-        <v>-19.6552</v>
+        <v>-14.6528</v>
       </c>
       <c r="T18" t="n">
-        <v>-13.7705</v>
+        <v>-17.3989</v>
       </c>
       <c r="U18" t="n">
-        <v>-2.4091</v>
+        <v>0.0442</v>
       </c>
       <c r="V18" t="n">
-        <v>-3.1866</v>
+        <v>-4.297</v>
       </c>
       <c r="W18" t="n">
-        <v>-4.2835</v>
+        <v>-5.0594</v>
       </c>
       <c r="X18" t="n">
-        <v>17.1953</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y18" t="n">
-        <v>19.6346</v>
+        <v>13.5251</v>
       </c>
       <c r="Z18" t="n">
-        <v>11.6314</v>
+        <v>15.8881</v>
       </c>
       <c r="AA18" t="n">
-        <v>2.4698</v>
+        <v>-0.0246</v>
       </c>
       <c r="AB18" t="n">
-        <v>3.0797</v>
+        <v>4.4765</v>
       </c>
       <c r="AC18" t="n">
-        <v>4.3216</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>104.55</v>
+        <v>113.33</v>
       </c>
       <c r="C19" t="n">
-        <v>105.94</v>
+        <v>115.48</v>
       </c>
       <c r="D19" t="n">
-        <v>100.96</v>
+        <v>112.01</v>
       </c>
       <c r="E19" t="n">
-        <v>102.32</v>
+        <v>114.82</v>
       </c>
       <c r="F19" t="n">
-        <v>69.13</v>
+        <v>71.13</v>
       </c>
       <c r="G19" t="n">
-        <v>69.33</v>
+        <v>71.72</v>
       </c>
       <c r="H19" t="n">
-        <v>67.61</v>
+        <v>70.37</v>
       </c>
       <c r="I19" t="n">
-        <v>67.90000000000001</v>
+        <v>71.38</v>
       </c>
       <c r="J19" t="n">
-        <v>49.87</v>
+        <v>45.72</v>
       </c>
       <c r="K19" t="n">
-        <v>51.8</v>
+        <v>46.34</v>
       </c>
       <c r="L19" t="n">
-        <v>49.26</v>
+        <v>44.67</v>
       </c>
       <c r="M19" t="n">
-        <v>51.1</v>
+        <v>44.99</v>
       </c>
       <c r="N19" t="n">
-        <v>39.91</v>
+        <v>38.69</v>
       </c>
       <c r="O19" t="n">
-        <v>40.78</v>
+        <v>39.14</v>
       </c>
       <c r="P19" t="n">
-        <v>39.79</v>
+        <v>38.33</v>
       </c>
       <c r="Q19" t="n">
-        <v>40.62</v>
+        <v>38.53</v>
       </c>
       <c r="R19" t="n">
-        <v>1.1767</v>
+        <v>10.4357</v>
       </c>
       <c r="S19" t="n">
-        <v>-11.6102</v>
+        <v>13.537</v>
       </c>
       <c r="T19" t="n">
-        <v>-16.9952</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U19" t="n">
-        <v>-1.9778</v>
+        <v>5.0788</v>
       </c>
       <c r="V19" t="n">
-        <v>-1.8928</v>
+        <v>3.0461</v>
       </c>
       <c r="W19" t="n">
-        <v>-5.9035</v>
+        <v>3.1354</v>
       </c>
       <c r="X19" t="n">
-        <v>-1.2179</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y19" t="n">
-        <v>9.328200000000001</v>
+        <v>-13.0292</v>
       </c>
       <c r="Z19" t="n">
-        <v>15.9256</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA19" t="n">
-        <v>1.9834</v>
+        <v>-5.1219</v>
       </c>
       <c r="AB19" t="n">
-        <v>1.8045</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC19" t="n">
-        <v>6.0298</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>107.44</v>
+        <v>117.03</v>
       </c>
       <c r="C20" t="n">
-        <v>109.32</v>
+        <v>123.9</v>
       </c>
       <c r="D20" t="n">
-        <v>101.06</v>
+        <v>116.68</v>
       </c>
       <c r="E20" t="n">
-        <v>103.97</v>
+        <v>123.67</v>
       </c>
       <c r="F20" t="n">
-        <v>68.84999999999999</v>
+        <v>71.92</v>
       </c>
       <c r="G20" t="n">
-        <v>69.97</v>
+        <v>72.78</v>
       </c>
       <c r="H20" t="n">
-        <v>66.55</v>
+        <v>70.81</v>
       </c>
       <c r="I20" t="n">
-        <v>67.93000000000001</v>
+        <v>72.64</v>
       </c>
       <c r="J20" t="n">
-        <v>48.55</v>
+        <v>44.11</v>
       </c>
       <c r="K20" t="n">
-        <v>51.74</v>
+        <v>44.26</v>
       </c>
       <c r="L20" t="n">
-        <v>47.57</v>
+        <v>41.47</v>
       </c>
       <c r="M20" t="n">
-        <v>50.11</v>
+        <v>41.49</v>
       </c>
       <c r="N20" t="n">
-        <v>40.06</v>
+        <v>38.26</v>
       </c>
       <c r="O20" t="n">
-        <v>41.44</v>
+        <v>38.87</v>
       </c>
       <c r="P20" t="n">
-        <v>39.37</v>
+        <v>37.8</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.61</v>
+        <v>37.87</v>
       </c>
       <c r="R20" t="n">
-        <v>1.6126</v>
+        <v>7.7077</v>
       </c>
       <c r="S20" t="n">
-        <v>-14.6528</v>
+        <v>20.8659</v>
       </c>
       <c r="T20" t="n">
-        <v>-17.3989</v>
+        <v>1.5186</v>
       </c>
       <c r="U20" t="n">
-        <v>0.0442</v>
+        <v>1.7652</v>
       </c>
       <c r="V20" t="n">
-        <v>-4.297</v>
+        <v>6.9809</v>
       </c>
       <c r="W20" t="n">
-        <v>-5.0594</v>
+        <v>2.3387</v>
       </c>
       <c r="X20" t="n">
-        <v>-1.9374</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y20" t="n">
-        <v>13.5251</v>
+        <v>-18.8063</v>
       </c>
       <c r="Z20" t="n">
-        <v>15.8881</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA20" t="n">
-        <v>-0.0246</v>
+        <v>-1.713</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.4765</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC20" t="n">
-        <v>5.0983</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>113.33</v>
-      </c>
-      <c r="C21" t="n">
-        <v>115.48</v>
-      </c>
-      <c r="D21" t="n">
-        <v>112.01</v>
-      </c>
-      <c r="E21" t="n">
-        <v>114.82</v>
-      </c>
-      <c r="F21" t="n">
-        <v>71.13</v>
-      </c>
-      <c r="G21" t="n">
-        <v>71.72</v>
-      </c>
-      <c r="H21" t="n">
-        <v>70.37</v>
-      </c>
-      <c r="I21" t="n">
-        <v>71.38</v>
-      </c>
-      <c r="J21" t="n">
-        <v>45.72</v>
-      </c>
-      <c r="K21" t="n">
-        <v>46.34</v>
-      </c>
-      <c r="L21" t="n">
-        <v>44.67</v>
-      </c>
-      <c r="M21" t="n">
-        <v>44.99</v>
-      </c>
-      <c r="N21" t="n">
-        <v>38.69</v>
-      </c>
-      <c r="O21" t="n">
-        <v>39.14</v>
-      </c>
-      <c r="P21" t="n">
-        <v>38.33</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>38.53</v>
-      </c>
-      <c r="R21" t="n">
-        <v>10.4357</v>
-      </c>
-      <c r="S21" t="n">
-        <v>13.537</v>
-      </c>
-      <c r="T21" t="n">
-        <v>-0.8120000000000001</v>
-      </c>
-      <c r="U21" t="n">
-        <v>5.0788</v>
-      </c>
-      <c r="V21" t="n">
-        <v>3.0461</v>
-      </c>
-      <c r="W21" t="n">
-        <v>3.1354</v>
-      </c>
-      <c r="X21" t="n">
-        <v>-10.2175</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>-13.0292</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>-3.7441</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>-5.1219</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>-3.2639</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>-3.4336</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>117.03</v>
-      </c>
-      <c r="C22" t="n">
-        <v>123.86</v>
-      </c>
-      <c r="D22" t="n">
-        <v>116.68</v>
-      </c>
-      <c r="E22" t="n">
-        <v>123.67</v>
-      </c>
-      <c r="F22" t="n">
-        <v>71.93000000000001</v>
-      </c>
-      <c r="G22" t="n">
-        <v>72.7777</v>
-      </c>
-      <c r="H22" t="n">
-        <v>70.8094</v>
-      </c>
-      <c r="I22" t="n">
-        <v>72.64</v>
-      </c>
-      <c r="J22" t="n">
-        <v>44.11</v>
-      </c>
-      <c r="K22" t="n">
-        <v>44.26</v>
-      </c>
-      <c r="L22" t="n">
-        <v>41.465</v>
-      </c>
-      <c r="M22" t="n">
-        <v>41.49</v>
-      </c>
-      <c r="N22" t="n">
-        <v>38.25</v>
-      </c>
-      <c r="O22" t="n">
-        <v>38.8675</v>
-      </c>
-      <c r="P22" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>37.87</v>
-      </c>
-      <c r="R22" t="n">
-        <v>7.7077</v>
-      </c>
-      <c r="S22" t="n">
-        <v>20.8659</v>
-      </c>
-      <c r="T22" t="n">
-        <v>1.5186</v>
-      </c>
-      <c r="U22" t="n">
-        <v>1.7652</v>
-      </c>
-      <c r="V22" t="n">
-        <v>6.9809</v>
-      </c>
-      <c r="W22" t="n">
-        <v>2.3387</v>
-      </c>
-      <c r="X22" t="n">
-        <v>-7.7795</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>-18.8063</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>-6.0036</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-1.713</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>-6.7701</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>-2.5727</v>
+          <t>2026-09-21</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2237,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-23 00:02
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2190,6 +2190,97 @@
       <c r="A21" t="inlineStr">
         <is>
           <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>132.07</v>
+      </c>
+      <c r="C21" t="n">
+        <v>144</v>
+      </c>
+      <c r="D21" t="n">
+        <v>129.62</v>
+      </c>
+      <c r="E21" t="n">
+        <v>141.93</v>
+      </c>
+      <c r="F21" t="n">
+        <v>74.83</v>
+      </c>
+      <c r="G21" t="n">
+        <v>79.48999999999999</v>
+      </c>
+      <c r="H21" t="n">
+        <v>74.83</v>
+      </c>
+      <c r="I21" t="n">
+        <v>78.91</v>
+      </c>
+      <c r="J21" t="n">
+        <v>38.75</v>
+      </c>
+      <c r="K21" t="n">
+        <v>39.51</v>
+      </c>
+      <c r="L21" t="n">
+        <v>34.68</v>
+      </c>
+      <c r="M21" t="n">
+        <v>35.33</v>
+      </c>
+      <c r="N21" t="n">
+        <v>36.73</v>
+      </c>
+      <c r="O21" t="n">
+        <v>36.74</v>
+      </c>
+      <c r="P21" t="n">
+        <v>34.31</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="R21" t="n">
+        <v>14.7651</v>
+      </c>
+      <c r="S21" t="n">
+        <v>36.5105</v>
+      </c>
+      <c r="T21" t="n">
+        <v>40.3441</v>
+      </c>
+      <c r="U21" t="n">
+        <v>8.631600000000001</v>
+      </c>
+      <c r="V21" t="n">
+        <v>16.1637</v>
+      </c>
+      <c r="W21" t="n">
+        <v>13.9166</v>
+      </c>
+      <c r="X21" t="n">
+        <v>-14.847</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>-29.4951</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>-31.7031</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>-8.6348</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>-14.7993</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>-13.1308</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-24 00:15
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1719 +568,1719 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>115.07</v>
+        <v>117.2931</v>
       </c>
       <c r="C2" t="n">
-        <v>115.07</v>
+        <v>119.8014</v>
       </c>
       <c r="D2" t="n">
-        <v>106</v>
+        <v>113.0559</v>
       </c>
       <c r="E2" t="n">
-        <v>111.16</v>
+        <v>115.5942</v>
       </c>
       <c r="F2" t="n">
-        <v>70</v>
+        <v>70.42</v>
       </c>
       <c r="G2" t="n">
-        <v>70.05</v>
+        <v>71.27</v>
       </c>
       <c r="H2" t="n">
-        <v>67.93000000000001</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>69.01000000000001</v>
+        <v>70.27</v>
       </c>
       <c r="J2" t="n">
-        <v>49.14</v>
+        <v>47.2299</v>
       </c>
       <c r="K2" t="n">
-        <v>52.81</v>
+        <v>49.2151</v>
       </c>
       <c r="L2" t="n">
-        <v>49.13</v>
+        <v>46.0842</v>
       </c>
       <c r="M2" t="n">
-        <v>50.75</v>
+        <v>47.8225</v>
       </c>
       <c r="N2" t="n">
-        <v>39.65</v>
+        <v>39.38</v>
       </c>
       <c r="O2" t="n">
-        <v>40.79</v>
+        <v>40.02</v>
       </c>
       <c r="P2" t="n">
-        <v>39.64</v>
+        <v>38.89</v>
       </c>
       <c r="Q2" t="n">
-        <v>40.19</v>
+        <v>39.46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>117.37</v>
+        <v>114.6248</v>
       </c>
       <c r="C3" t="n">
-        <v>119.88</v>
+        <v>117.3131</v>
       </c>
       <c r="D3" t="n">
-        <v>113.13</v>
+        <v>112.4563</v>
       </c>
       <c r="E3" t="n">
-        <v>115.67</v>
+        <v>116.5236</v>
       </c>
       <c r="F3" t="n">
-        <v>70.42</v>
+        <v>69.56</v>
       </c>
       <c r="G3" t="n">
-        <v>71.27</v>
+        <v>70.94</v>
       </c>
       <c r="H3" t="n">
-        <v>69.34999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="I3" t="n">
-        <v>70.27</v>
+        <v>70.47</v>
       </c>
       <c r="J3" t="n">
-        <v>47.82</v>
+        <v>48.4052</v>
       </c>
       <c r="K3" t="n">
-        <v>49.83</v>
+        <v>49.2743</v>
       </c>
       <c r="L3" t="n">
-        <v>46.66</v>
+        <v>47.2792</v>
       </c>
       <c r="M3" t="n">
-        <v>48.42</v>
+        <v>47.4965</v>
       </c>
       <c r="N3" t="n">
+        <v>39.86</v>
+      </c>
+      <c r="O3" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="P3" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="Q3" t="n">
         <v>39.38</v>
       </c>
-      <c r="O3" t="n">
-        <v>40.02</v>
-      </c>
-      <c r="P3" t="n">
-        <v>38.89</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>39.46</v>
-      </c>
       <c r="R3" t="n">
-        <v>4.0572</v>
+        <v>0.804</v>
       </c>
       <c r="U3" t="n">
-        <v>1.8258</v>
+        <v>0.2846</v>
       </c>
       <c r="X3" t="n">
-        <v>-4.5911</v>
+        <v>-0.6817</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.8164</v>
+        <v>-0.2027</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>114.7</v>
+        <v>123.3191</v>
       </c>
       <c r="C4" t="n">
-        <v>117.39</v>
+        <v>124.7982</v>
       </c>
       <c r="D4" t="n">
-        <v>112.53</v>
+        <v>117.6129</v>
       </c>
       <c r="E4" t="n">
-        <v>116.6</v>
+        <v>122.9694</v>
       </c>
       <c r="F4" t="n">
-        <v>69.56</v>
+        <v>72.09</v>
       </c>
       <c r="G4" t="n">
-        <v>70.94</v>
+        <v>73.38</v>
       </c>
       <c r="H4" t="n">
-        <v>69.44</v>
+        <v>71.38</v>
       </c>
       <c r="I4" t="n">
-        <v>70.47</v>
+        <v>73.3</v>
       </c>
       <c r="J4" t="n">
-        <v>49.01</v>
+        <v>44.8595</v>
       </c>
       <c r="K4" t="n">
-        <v>49.89</v>
+        <v>47.1212</v>
       </c>
       <c r="L4" t="n">
-        <v>47.87</v>
+        <v>44.1582</v>
       </c>
       <c r="M4" t="n">
-        <v>48.09</v>
+        <v>44.7903</v>
       </c>
       <c r="N4" t="n">
-        <v>39.86</v>
+        <v>38.46</v>
       </c>
       <c r="O4" t="n">
-        <v>39.93</v>
+        <v>38.86</v>
       </c>
       <c r="P4" t="n">
-        <v>39.09</v>
+        <v>37.73</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.38</v>
+        <v>37.78</v>
       </c>
       <c r="R4" t="n">
-        <v>0.804</v>
+        <v>5.5318</v>
       </c>
       <c r="U4" t="n">
-        <v>0.2846</v>
+        <v>4.0159</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.6815</v>
+        <v>-5.6977</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.2027</v>
+        <v>-4.063</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>123.4</v>
+        <v>119.8414</v>
       </c>
       <c r="C5" t="n">
-        <v>124.88</v>
+        <v>121.1206</v>
       </c>
       <c r="D5" t="n">
-        <v>117.69</v>
+        <v>110.1378</v>
       </c>
       <c r="E5" t="n">
-        <v>123.05</v>
+        <v>111.267</v>
       </c>
       <c r="F5" t="n">
-        <v>72.09</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>73.38</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>71.38</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>73.3</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>45.42</v>
+        <v>46.0348</v>
       </c>
       <c r="K5" t="n">
-        <v>47.71</v>
+        <v>49.6101</v>
       </c>
       <c r="L5" t="n">
-        <v>44.71</v>
+        <v>45.5805</v>
       </c>
       <c r="M5" t="n">
-        <v>45.35</v>
+        <v>49.2052</v>
       </c>
       <c r="N5" t="n">
-        <v>38.46</v>
+        <v>38.02</v>
       </c>
       <c r="O5" t="n">
-        <v>38.86</v>
+        <v>38.76</v>
       </c>
       <c r="P5" t="n">
-        <v>37.73</v>
+        <v>37.33</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.78</v>
+        <v>38.54</v>
       </c>
       <c r="R5" t="n">
-        <v>5.5317</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="S5" t="n">
-        <v>10.6963</v>
+        <v>-3.7434</v>
       </c>
       <c r="U5" t="n">
-        <v>4.0159</v>
+        <v>-1.9782</v>
       </c>
       <c r="V5" t="n">
-        <v>6.2165</v>
+        <v>2.2485</v>
       </c>
       <c r="X5" t="n">
-        <v>-5.6977</v>
+        <v>9.8568</v>
       </c>
       <c r="Y5" t="n">
-        <v>-10.6404</v>
+        <v>2.8913</v>
       </c>
       <c r="AA5" t="n">
-        <v>-4.063</v>
+        <v>2.0116</v>
       </c>
       <c r="AB5" t="n">
-        <v>-5.9965</v>
+        <v>-2.3315</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>119.92</v>
+        <v>112.3363</v>
       </c>
       <c r="C6" t="n">
-        <v>121.2</v>
+        <v>114.9746</v>
       </c>
       <c r="D6" t="n">
-        <v>110.21</v>
+        <v>110.2577</v>
       </c>
       <c r="E6" t="n">
-        <v>111.34</v>
+        <v>112.7161</v>
       </c>
       <c r="F6" t="n">
-        <v>72.84999999999999</v>
+        <v>71.44</v>
       </c>
       <c r="G6" t="n">
-        <v>74.18000000000001</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>71.43000000000001</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>71.84999999999999</v>
+        <v>71.92</v>
       </c>
       <c r="J6" t="n">
-        <v>46.61</v>
+        <v>48.662</v>
       </c>
       <c r="K6" t="n">
-        <v>50.23</v>
+        <v>49.62</v>
       </c>
       <c r="L6" t="n">
-        <v>46.15</v>
+        <v>47.4965</v>
       </c>
       <c r="M6" t="n">
-        <v>49.82</v>
+        <v>48.4151</v>
       </c>
       <c r="N6" t="n">
-        <v>38.02</v>
+        <v>38.77</v>
       </c>
       <c r="O6" t="n">
-        <v>38.76</v>
+        <v>39.09</v>
       </c>
       <c r="P6" t="n">
-        <v>37.33</v>
+        <v>38.37</v>
       </c>
       <c r="Q6" t="n">
-        <v>38.54</v>
+        <v>38.51</v>
       </c>
       <c r="R6" t="n">
-        <v>-9.516500000000001</v>
+        <v>1.3024</v>
       </c>
       <c r="S6" t="n">
-        <v>-3.7434</v>
+        <v>-3.2676</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.9782</v>
+        <v>0.0974</v>
       </c>
       <c r="V6" t="n">
-        <v>2.2485</v>
+        <v>2.0576</v>
       </c>
       <c r="X6" t="n">
-        <v>9.8567</v>
+        <v>-1.6057</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.8914</v>
+        <v>1.934</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.0116</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="AB6" t="n">
-        <v>-2.3315</v>
+        <v>-2.2092</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>112.41</v>
+        <v>106.2903</v>
       </c>
       <c r="C7" t="n">
-        <v>115.05</v>
+        <v>108.5688</v>
       </c>
       <c r="D7" t="n">
-        <v>110.33</v>
+        <v>102.243</v>
       </c>
       <c r="E7" t="n">
-        <v>112.79</v>
+        <v>105.8406</v>
       </c>
       <c r="F7" t="n">
-        <v>71.44</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>72.15000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="H7" t="n">
-        <v>70.81999999999999</v>
+        <v>68.25</v>
       </c>
       <c r="I7" t="n">
-        <v>71.92</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>49.27</v>
+        <v>51.2398</v>
       </c>
       <c r="K7" t="n">
-        <v>50.24</v>
+        <v>53.0274</v>
       </c>
       <c r="L7" t="n">
-        <v>48.09</v>
+        <v>50.2719</v>
       </c>
       <c r="M7" t="n">
-        <v>49.02</v>
+        <v>51.5756</v>
       </c>
       <c r="N7" t="n">
-        <v>38.77</v>
+        <v>40.03</v>
       </c>
       <c r="O7" t="n">
-        <v>39.09</v>
+        <v>40.47</v>
       </c>
       <c r="P7" t="n">
-        <v>38.37</v>
+        <v>39.23</v>
       </c>
       <c r="Q7" t="n">
-        <v>38.51</v>
+        <v>39.97</v>
       </c>
       <c r="R7" t="n">
-        <v>1.3023</v>
+        <v>-6.0998</v>
       </c>
       <c r="S7" t="n">
-        <v>-3.2676</v>
+        <v>-13.9293</v>
       </c>
       <c r="T7" t="n">
-        <v>1.4664</v>
+        <v>-8.437799999999999</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0974</v>
+        <v>-3.8515</v>
       </c>
       <c r="V7" t="n">
-        <v>2.0576</v>
+        <v>-5.6617</v>
       </c>
       <c r="W7" t="n">
-        <v>4.2168</v>
+        <v>-1.5939</v>
       </c>
       <c r="X7" t="n">
-        <v>-1.6058</v>
+        <v>6.5279</v>
       </c>
       <c r="Y7" t="n">
-        <v>1.9339</v>
+        <v>15.149</v>
       </c>
       <c r="Z7" t="n">
-        <v>-3.4089</v>
+        <v>7.848</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.07779999999999999</v>
+        <v>3.7912</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.2092</v>
+        <v>5.7967</v>
       </c>
       <c r="AC7" t="n">
-        <v>-4.1801</v>
+        <v>1.2924</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>106.36</v>
+        <v>104.4315</v>
       </c>
       <c r="C8" t="n">
-        <v>108.64</v>
+        <v>107.9992</v>
       </c>
       <c r="D8" t="n">
-        <v>102.31</v>
+        <v>101.2736</v>
       </c>
       <c r="E8" t="n">
-        <v>105.91</v>
+        <v>106.2803</v>
       </c>
       <c r="F8" t="n">
-        <v>69.06999999999999</v>
+        <v>68.97</v>
       </c>
       <c r="G8" t="n">
-        <v>70.55</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>68.25</v>
+        <v>68.39</v>
       </c>
       <c r="I8" t="n">
-        <v>69.15000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>51.88</v>
+        <v>52.1484</v>
       </c>
       <c r="K8" t="n">
-        <v>53.69</v>
+        <v>53.7188</v>
       </c>
       <c r="L8" t="n">
-        <v>50.9</v>
+        <v>50.42</v>
       </c>
       <c r="M8" t="n">
-        <v>52.22</v>
+        <v>51.1904</v>
       </c>
       <c r="N8" t="n">
-        <v>40.03</v>
+        <v>40.09</v>
       </c>
       <c r="O8" t="n">
-        <v>40.47</v>
+        <v>40.43</v>
       </c>
       <c r="P8" t="n">
-        <v>39.23</v>
+        <v>39.63</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.97</v>
+        <v>39.71</v>
       </c>
       <c r="R8" t="n">
-        <v>-6.0998</v>
+        <v>0.4154</v>
       </c>
       <c r="S8" t="n">
-        <v>-13.9293</v>
+        <v>-4.4817</v>
       </c>
       <c r="T8" t="n">
-        <v>-8.437799999999999</v>
+        <v>-8.790800000000001</v>
       </c>
       <c r="U8" t="n">
-        <v>-3.8515</v>
+        <v>0.6508</v>
       </c>
       <c r="V8" t="n">
-        <v>-5.6617</v>
+        <v>-3.1315</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.5939</v>
+        <v>-1.2346</v>
       </c>
       <c r="X8" t="n">
-        <v>6.5279</v>
+        <v>-0.7469</v>
       </c>
       <c r="Y8" t="n">
-        <v>15.1488</v>
+        <v>4.0345</v>
       </c>
       <c r="Z8" t="n">
-        <v>7.848</v>
+        <v>7.7772</v>
       </c>
       <c r="AA8" t="n">
-        <v>3.7912</v>
+        <v>-0.6505</v>
       </c>
       <c r="AB8" t="n">
-        <v>5.7967</v>
+        <v>3.0358</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.2924</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>104.5</v>
+        <v>102.9325</v>
       </c>
       <c r="C9" t="n">
-        <v>108.07</v>
+        <v>107.4196</v>
       </c>
       <c r="D9" t="n">
-        <v>101.34</v>
+        <v>98.55540000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>106.35</v>
+        <v>106.6701</v>
       </c>
       <c r="F9" t="n">
-        <v>68.97</v>
+        <v>70.06</v>
       </c>
       <c r="G9" t="n">
-        <v>69.76000000000001</v>
+        <v>72.42</v>
       </c>
       <c r="H9" t="n">
-        <v>68.39</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>69.59999999999999</v>
+        <v>72.03</v>
       </c>
       <c r="J9" t="n">
-        <v>52.8</v>
+        <v>52.8398</v>
       </c>
       <c r="K9" t="n">
-        <v>54.39</v>
+        <v>55.0027</v>
       </c>
       <c r="L9" t="n">
-        <v>51.05</v>
+        <v>50.6472</v>
       </c>
       <c r="M9" t="n">
-        <v>51.83</v>
+        <v>50.9632</v>
       </c>
       <c r="N9" t="n">
-        <v>40.09</v>
+        <v>39.49</v>
       </c>
       <c r="O9" t="n">
-        <v>40.43</v>
+        <v>39.68</v>
       </c>
       <c r="P9" t="n">
-        <v>39.63</v>
+        <v>38.12</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.71</v>
+        <v>38.34</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4154</v>
+        <v>0.3668</v>
       </c>
       <c r="S9" t="n">
-        <v>-4.4818</v>
+        <v>-5.3639</v>
       </c>
       <c r="T9" t="n">
-        <v>-8.790699999999999</v>
+        <v>-13.2548</v>
       </c>
       <c r="U9" t="n">
-        <v>0.6508</v>
+        <v>3.4914</v>
       </c>
       <c r="V9" t="n">
-        <v>-3.1315</v>
+        <v>0.1529</v>
       </c>
       <c r="W9" t="n">
-        <v>-1.2346</v>
+        <v>-1.7326</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.7468</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y9" t="n">
-        <v>4.0345</v>
+        <v>5.263</v>
       </c>
       <c r="Z9" t="n">
-        <v>7.7771</v>
+        <v>13.7818</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.6505</v>
+        <v>-3.45</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.0358</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.838</v>
+        <v>1.4823</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>103</v>
+        <v>111.1471</v>
       </c>
       <c r="C10" t="n">
-        <v>107.49</v>
+        <v>118.1026</v>
       </c>
       <c r="D10" t="n">
-        <v>98.62</v>
+        <v>109.6581</v>
       </c>
       <c r="E10" t="n">
-        <v>106.74</v>
+        <v>117.2032</v>
       </c>
       <c r="F10" t="n">
-        <v>70.06</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>72.42</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>69.70999999999999</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>72.03</v>
+        <v>72.37</v>
       </c>
       <c r="J10" t="n">
-        <v>53.5</v>
+        <v>48.9484</v>
       </c>
       <c r="K10" t="n">
-        <v>55.69</v>
+        <v>49.5904</v>
       </c>
       <c r="L10" t="n">
-        <v>51.28</v>
+        <v>45.5311</v>
       </c>
       <c r="M10" t="n">
-        <v>51.6</v>
+        <v>45.7681</v>
       </c>
       <c r="N10" t="n">
-        <v>39.49</v>
+        <v>38.12</v>
       </c>
       <c r="O10" t="n">
-        <v>39.68</v>
+        <v>38.58</v>
       </c>
       <c r="P10" t="n">
-        <v>38.12</v>
+        <v>37.72</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.34</v>
+        <v>38.18</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3667</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S10" t="n">
-        <v>-5.364</v>
+        <v>10.7356</v>
       </c>
       <c r="T10" t="n">
-        <v>-13.2548</v>
+        <v>5.3351</v>
       </c>
       <c r="U10" t="n">
-        <v>3.4914</v>
+        <v>0.472</v>
       </c>
       <c r="V10" t="n">
-        <v>0.1529</v>
+        <v>4.6565</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.7326</v>
+        <v>0.7237</v>
       </c>
       <c r="X10" t="n">
-        <v>-0.4438</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y10" t="n">
-        <v>5.2632</v>
+        <v>-11.2602</v>
       </c>
       <c r="Z10" t="n">
-        <v>13.7817</v>
+        <v>-6.9852</v>
       </c>
       <c r="AA10" t="n">
-        <v>-3.45</v>
+        <v>-0.4173</v>
       </c>
       <c r="AB10" t="n">
-        <v>-0.4414</v>
+        <v>-4.4784</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.4823</v>
+        <v>-0.9341</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>111.22</v>
+        <v>125.038</v>
       </c>
       <c r="C11" t="n">
-        <v>118.18</v>
+        <v>127.4564</v>
       </c>
       <c r="D11" t="n">
-        <v>109.73</v>
+        <v>121.5203</v>
       </c>
       <c r="E11" t="n">
-        <v>117.28</v>
+        <v>123.1892</v>
       </c>
       <c r="F11" t="n">
-        <v>72.48999999999999</v>
+        <v>72.95</v>
       </c>
       <c r="G11" t="n">
-        <v>73.23999999999999</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>71.65000000000001</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>72.37</v>
+        <v>72.16</v>
       </c>
       <c r="J11" t="n">
-        <v>49.56</v>
+        <v>43.0126</v>
       </c>
       <c r="K11" t="n">
-        <v>50.21</v>
+        <v>44.2768</v>
       </c>
       <c r="L11" t="n">
-        <v>46.1</v>
+        <v>41.9854</v>
       </c>
       <c r="M11" t="n">
-        <v>46.34</v>
+        <v>43.536</v>
       </c>
       <c r="N11" t="n">
-        <v>38.12</v>
+        <v>37.89</v>
       </c>
       <c r="O11" t="n">
-        <v>38.58</v>
+        <v>38.74</v>
       </c>
       <c r="P11" t="n">
-        <v>37.72</v>
+        <v>37.75</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.18</v>
+        <v>38.31</v>
       </c>
       <c r="R11" t="n">
-        <v>9.874499999999999</v>
+        <v>5.1074</v>
       </c>
       <c r="S11" t="n">
-        <v>10.7355</v>
+        <v>15.9097</v>
       </c>
       <c r="T11" t="n">
-        <v>5.335</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U11" t="n">
-        <v>0.472</v>
+        <v>-0.2902</v>
       </c>
       <c r="V11" t="n">
-        <v>4.6565</v>
+        <v>3.6782</v>
       </c>
       <c r="W11" t="n">
-        <v>0.7237</v>
+        <v>0.3337</v>
       </c>
       <c r="X11" t="n">
-        <v>-10.1938</v>
+        <v>-4.877</v>
       </c>
       <c r="Y11" t="n">
-        <v>-11.2601</v>
+        <v>-14.9528</v>
       </c>
       <c r="Z11" t="n">
-        <v>-6.9851</v>
+        <v>-10.0776</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.4173</v>
+        <v>0.3405</v>
       </c>
       <c r="AB11" t="n">
-        <v>-4.4784</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC11" t="n">
-        <v>-0.9341</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>125.12</v>
+        <v>121.1606</v>
       </c>
       <c r="C12" t="n">
-        <v>127.54</v>
+        <v>128.3958</v>
       </c>
       <c r="D12" t="n">
-        <v>121.6</v>
+        <v>121.1606</v>
       </c>
       <c r="E12" t="n">
-        <v>123.27</v>
+        <v>125.7875</v>
       </c>
       <c r="F12" t="n">
-        <v>72.95</v>
+        <v>71.55</v>
       </c>
       <c r="G12" t="n">
-        <v>73.20999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="H12" t="n">
-        <v>71.31999999999999</v>
+        <v>70.84</v>
       </c>
       <c r="I12" t="n">
-        <v>72.16</v>
+        <v>71.55</v>
       </c>
       <c r="J12" t="n">
-        <v>43.55</v>
+        <v>44.2471</v>
       </c>
       <c r="K12" t="n">
-        <v>44.83</v>
+        <v>44.2669</v>
       </c>
       <c r="L12" t="n">
-        <v>42.51</v>
+        <v>41.7977</v>
       </c>
       <c r="M12" t="n">
-        <v>44.08</v>
+        <v>42.7064</v>
       </c>
       <c r="N12" t="n">
-        <v>37.89</v>
+        <v>38.63</v>
       </c>
       <c r="O12" t="n">
-        <v>38.74</v>
+        <v>39.01</v>
       </c>
       <c r="P12" t="n">
-        <v>37.75</v>
+        <v>38.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.31</v>
+        <v>38.64</v>
       </c>
       <c r="R12" t="n">
-        <v>5.1074</v>
+        <v>2.1092</v>
       </c>
       <c r="S12" t="n">
-        <v>15.9097</v>
+        <v>17.922</v>
       </c>
       <c r="T12" t="n">
-        <v>9.291600000000001</v>
+        <v>18.8462</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.2902</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V12" t="n">
-        <v>3.6782</v>
+        <v>-0.6664</v>
       </c>
       <c r="W12" t="n">
-        <v>0.3337</v>
+        <v>3.4707</v>
       </c>
       <c r="X12" t="n">
-        <v>-4.877</v>
+        <v>-1.9055</v>
       </c>
       <c r="Y12" t="n">
-        <v>-14.9527</v>
+        <v>-16.2015</v>
       </c>
       <c r="Z12" t="n">
-        <v>-10.0775</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.3405</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AB12" t="n">
-        <v>-3.5256</v>
+        <v>0.7825</v>
       </c>
       <c r="AC12" t="n">
-        <v>-0.5193</v>
+        <v>-3.3275</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>121.24</v>
+        <v>116.2738</v>
       </c>
       <c r="C13" t="n">
-        <v>128.48</v>
+        <v>119.2418</v>
       </c>
       <c r="D13" t="n">
-        <v>121.24</v>
+        <v>113.4756</v>
       </c>
       <c r="E13" t="n">
-        <v>125.87</v>
+        <v>115.6842</v>
       </c>
       <c r="F13" t="n">
-        <v>71.55</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>72.55</v>
+        <v>70.23</v>
       </c>
       <c r="H13" t="n">
-        <v>70.84</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>71.55</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>44.8</v>
+        <v>45.9459</v>
       </c>
       <c r="K13" t="n">
-        <v>44.82</v>
+        <v>46.9039</v>
       </c>
       <c r="L13" t="n">
-        <v>42.32</v>
+        <v>44.9385</v>
       </c>
       <c r="M13" t="n">
-        <v>43.24</v>
+        <v>46.1632</v>
       </c>
       <c r="N13" t="n">
-        <v>38.63</v>
+        <v>40.08</v>
       </c>
       <c r="O13" t="n">
-        <v>39.01</v>
+        <v>40.19</v>
       </c>
       <c r="P13" t="n">
-        <v>38.1</v>
+        <v>39.35</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.64</v>
+        <v>39.9</v>
       </c>
       <c r="R13" t="n">
-        <v>2.1092</v>
+        <v>-8.032</v>
       </c>
       <c r="S13" t="n">
-        <v>17.9221</v>
+        <v>-1.296</v>
       </c>
       <c r="T13" t="n">
-        <v>18.8462</v>
+        <v>8.8482</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2704</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.6664</v>
+        <v>-4.3665</v>
       </c>
       <c r="W13" t="n">
-        <v>3.4707</v>
+        <v>-0.5603</v>
       </c>
       <c r="X13" t="n">
-        <v>-1.9056</v>
+        <v>8.0943</v>
       </c>
       <c r="Y13" t="n">
-        <v>-16.2016</v>
+        <v>0.8633</v>
       </c>
       <c r="Z13" t="n">
-        <v>-17.1965</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.8614000000000001</v>
+        <v>3.2609</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.7825</v>
+        <v>4.505</v>
       </c>
       <c r="AC13" t="n">
-        <v>-3.3275</v>
+        <v>0.4785</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>116.35</v>
+        <v>120.6309</v>
       </c>
       <c r="C14" t="n">
-        <v>119.32</v>
+        <v>124.4184</v>
       </c>
       <c r="D14" t="n">
-        <v>113.55</v>
+        <v>117.7928</v>
       </c>
       <c r="E14" t="n">
-        <v>115.76</v>
+        <v>121.7402</v>
       </c>
       <c r="F14" t="n">
-        <v>68.90000000000001</v>
+        <v>71.19</v>
       </c>
       <c r="G14" t="n">
-        <v>70.23</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>68.68000000000001</v>
+        <v>70.61</v>
       </c>
       <c r="I14" t="n">
-        <v>69.20999999999999</v>
+        <v>70.98</v>
       </c>
       <c r="J14" t="n">
-        <v>46.52</v>
+        <v>44.1385</v>
       </c>
       <c r="K14" t="n">
-        <v>47.49</v>
+        <v>45.2545</v>
       </c>
       <c r="L14" t="n">
-        <v>45.5</v>
+        <v>42.5879</v>
       </c>
       <c r="M14" t="n">
-        <v>46.74</v>
+        <v>43.5953</v>
       </c>
       <c r="N14" t="n">
-        <v>40.08</v>
+        <v>38.77</v>
       </c>
       <c r="O14" t="n">
-        <v>40.19</v>
+        <v>39.1</v>
       </c>
       <c r="P14" t="n">
-        <v>39.35</v>
+        <v>38.42</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.9</v>
+        <v>38.87</v>
       </c>
       <c r="R14" t="n">
-        <v>-8.0321</v>
+        <v>5.2349</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.296</v>
+        <v>-1.1762</v>
       </c>
       <c r="T14" t="n">
-        <v>8.848100000000001</v>
+        <v>14.1278</v>
       </c>
       <c r="U14" t="n">
-        <v>-3.2704</v>
+        <v>2.5574</v>
       </c>
       <c r="V14" t="n">
-        <v>-4.3665</v>
+        <v>-1.6353</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.5603</v>
+        <v>-1.4577</v>
       </c>
       <c r="X14" t="n">
-        <v>8.0944</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.8632</v>
+        <v>0.1362</v>
       </c>
       <c r="Z14" t="n">
-        <v>-9.820600000000001</v>
+        <v>-14.4573</v>
       </c>
       <c r="AA14" t="n">
-        <v>3.2609</v>
+        <v>-2.5815</v>
       </c>
       <c r="AB14" t="n">
-        <v>4.505</v>
+        <v>1.4618</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.4785</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>120.71</v>
+        <v>101.4635</v>
       </c>
       <c r="C15" t="n">
-        <v>124.5</v>
+        <v>105.3209</v>
       </c>
       <c r="D15" t="n">
-        <v>117.87</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>121.82</v>
+        <v>101.0637</v>
       </c>
       <c r="F15" t="n">
-        <v>71.19</v>
+        <v>67.53</v>
       </c>
       <c r="G15" t="n">
-        <v>71.76000000000001</v>
+        <v>70.39</v>
       </c>
       <c r="H15" t="n">
-        <v>70.61</v>
+        <v>67.34</v>
       </c>
       <c r="I15" t="n">
-        <v>70.98</v>
+        <v>69.27</v>
       </c>
       <c r="J15" t="n">
-        <v>44.69</v>
+        <v>50.9731</v>
       </c>
       <c r="K15" t="n">
-        <v>45.82</v>
+        <v>51.5756</v>
       </c>
       <c r="L15" t="n">
-        <v>43.12</v>
+        <v>49.5904</v>
       </c>
       <c r="M15" t="n">
-        <v>44.14</v>
+        <v>51.0916</v>
       </c>
       <c r="N15" t="n">
-        <v>38.77</v>
+        <v>40.78</v>
       </c>
       <c r="O15" t="n">
-        <v>39.1</v>
+        <v>40.88</v>
       </c>
       <c r="P15" t="n">
-        <v>38.42</v>
+        <v>39.21</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.87</v>
+        <v>39.83</v>
       </c>
       <c r="R15" t="n">
-        <v>5.235</v>
+        <v>-16.9841</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.1763</v>
+        <v>-19.6552</v>
       </c>
       <c r="T15" t="n">
-        <v>14.1278</v>
+        <v>-13.7705</v>
       </c>
       <c r="U15" t="n">
-        <v>2.5574</v>
+        <v>-2.4091</v>
       </c>
       <c r="V15" t="n">
-        <v>-1.6353</v>
+        <v>-3.1866</v>
       </c>
       <c r="W15" t="n">
-        <v>-1.4577</v>
+        <v>-4.2835</v>
       </c>
       <c r="X15" t="n">
-        <v>-5.5627</v>
+        <v>17.1952</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.1361</v>
+        <v>19.6345</v>
       </c>
       <c r="Z15" t="n">
-        <v>-14.4574</v>
+        <v>11.6315</v>
       </c>
       <c r="AA15" t="n">
-        <v>-2.5815</v>
+        <v>2.4698</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.4618</v>
+        <v>3.0797</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.3824</v>
+        <v>4.3216</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>101.53</v>
+        <v>104.4815</v>
       </c>
       <c r="C16" t="n">
-        <v>105.39</v>
+        <v>105.8706</v>
       </c>
       <c r="D16" t="n">
-        <v>99.87</v>
+        <v>100.8938</v>
       </c>
       <c r="E16" t="n">
-        <v>101.13</v>
+        <v>102.253</v>
       </c>
       <c r="F16" t="n">
-        <v>67.53</v>
+        <v>69.13</v>
       </c>
       <c r="G16" t="n">
-        <v>70.39</v>
+        <v>69.33</v>
       </c>
       <c r="H16" t="n">
-        <v>67.34</v>
+        <v>67.61</v>
       </c>
       <c r="I16" t="n">
-        <v>69.27</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>51.61</v>
+        <v>49.2546</v>
       </c>
       <c r="K16" t="n">
-        <v>52.22</v>
+        <v>51.1607</v>
       </c>
       <c r="L16" t="n">
-        <v>50.21</v>
+        <v>48.6521</v>
       </c>
       <c r="M16" t="n">
-        <v>51.73</v>
+        <v>50.4694</v>
       </c>
       <c r="N16" t="n">
+        <v>39.91</v>
+      </c>
+      <c r="O16" t="n">
         <v>40.78</v>
       </c>
-      <c r="O16" t="n">
-        <v>40.88</v>
-      </c>
       <c r="P16" t="n">
-        <v>39.21</v>
+        <v>39.79</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.83</v>
+        <v>40.62</v>
       </c>
       <c r="R16" t="n">
-        <v>-16.9841</v>
+        <v>1.1768</v>
       </c>
       <c r="S16" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="T16" t="n">
-        <v>-13.7705</v>
+        <v>-16.9952</v>
       </c>
       <c r="U16" t="n">
-        <v>-2.4091</v>
+        <v>-1.9778</v>
       </c>
       <c r="V16" t="n">
-        <v>-3.1866</v>
+        <v>-1.8928</v>
       </c>
       <c r="W16" t="n">
-        <v>-4.2835</v>
+        <v>-5.9035</v>
       </c>
       <c r="X16" t="n">
-        <v>17.1953</v>
+        <v>-1.2178</v>
       </c>
       <c r="Y16" t="n">
-        <v>19.6346</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z16" t="n">
-        <v>11.6314</v>
+        <v>15.9257</v>
       </c>
       <c r="AA16" t="n">
-        <v>2.4698</v>
+        <v>1.9834</v>
       </c>
       <c r="AB16" t="n">
-        <v>3.0797</v>
+        <v>1.8045</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.3216</v>
+        <v>6.0298</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>104.55</v>
+        <v>107.3696</v>
       </c>
       <c r="C17" t="n">
-        <v>105.94</v>
+        <v>109.2484</v>
       </c>
       <c r="D17" t="n">
-        <v>100.96</v>
+        <v>100.9938</v>
       </c>
       <c r="E17" t="n">
-        <v>102.32</v>
+        <v>103.9019</v>
       </c>
       <c r="F17" t="n">
-        <v>69.13</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>69.33</v>
+        <v>69.97</v>
       </c>
       <c r="H17" t="n">
-        <v>67.61</v>
+        <v>66.55</v>
       </c>
       <c r="I17" t="n">
-        <v>67.90000000000001</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>49.87</v>
+        <v>47.9509</v>
       </c>
       <c r="K17" t="n">
-        <v>51.8</v>
+        <v>51.1015</v>
       </c>
       <c r="L17" t="n">
-        <v>49.26</v>
+        <v>46.9829</v>
       </c>
       <c r="M17" t="n">
-        <v>51.1</v>
+        <v>49.4916</v>
       </c>
       <c r="N17" t="n">
-        <v>39.91</v>
+        <v>40.06</v>
       </c>
       <c r="O17" t="n">
-        <v>40.78</v>
+        <v>41.44</v>
       </c>
       <c r="P17" t="n">
-        <v>39.79</v>
+        <v>39.37</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.62</v>
+        <v>40.61</v>
       </c>
       <c r="R17" t="n">
-        <v>1.1767</v>
+        <v>1.6126</v>
       </c>
       <c r="S17" t="n">
-        <v>-11.6102</v>
+        <v>-14.6528</v>
       </c>
       <c r="T17" t="n">
-        <v>-16.9952</v>
+        <v>-17.3989</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.9778</v>
+        <v>0.0442</v>
       </c>
       <c r="V17" t="n">
-        <v>-1.8928</v>
+        <v>-4.297</v>
       </c>
       <c r="W17" t="n">
-        <v>-5.9035</v>
+        <v>-5.0594</v>
       </c>
       <c r="X17" t="n">
-        <v>-1.2179</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y17" t="n">
-        <v>9.328200000000001</v>
+        <v>13.5251</v>
       </c>
       <c r="Z17" t="n">
-        <v>15.9256</v>
+        <v>15.888</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.9834</v>
+        <v>-0.0246</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.8045</v>
+        <v>4.4765</v>
       </c>
       <c r="AC17" t="n">
-        <v>6.0298</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>107.44</v>
+        <v>113.2557</v>
       </c>
       <c r="C18" t="n">
-        <v>109.32</v>
+        <v>115.4043</v>
       </c>
       <c r="D18" t="n">
-        <v>101.06</v>
+        <v>111.9366</v>
       </c>
       <c r="E18" t="n">
-        <v>103.97</v>
+        <v>114.7448</v>
       </c>
       <c r="F18" t="n">
-        <v>68.84999999999999</v>
+        <v>71.13</v>
       </c>
       <c r="G18" t="n">
-        <v>69.97</v>
+        <v>71.72</v>
       </c>
       <c r="H18" t="n">
-        <v>66.55</v>
+        <v>70.37</v>
       </c>
       <c r="I18" t="n">
-        <v>67.93000000000001</v>
+        <v>71.38</v>
       </c>
       <c r="J18" t="n">
-        <v>48.55</v>
+        <v>45.1558</v>
       </c>
       <c r="K18" t="n">
-        <v>51.74</v>
+        <v>45.7681</v>
       </c>
       <c r="L18" t="n">
-        <v>47.57</v>
+        <v>44.1187</v>
       </c>
       <c r="M18" t="n">
-        <v>50.11</v>
+        <v>44.4348</v>
       </c>
       <c r="N18" t="n">
-        <v>40.06</v>
+        <v>38.69</v>
       </c>
       <c r="O18" t="n">
-        <v>41.44</v>
+        <v>39.14</v>
       </c>
       <c r="P18" t="n">
-        <v>39.37</v>
+        <v>38.33</v>
       </c>
       <c r="Q18" t="n">
-        <v>40.61</v>
+        <v>38.53</v>
       </c>
       <c r="R18" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="S18" t="n">
-        <v>-14.6528</v>
+        <v>13.5371</v>
       </c>
       <c r="T18" t="n">
-        <v>-17.3989</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U18" t="n">
-        <v>0.0442</v>
+        <v>5.0788</v>
       </c>
       <c r="V18" t="n">
-        <v>-4.297</v>
+        <v>3.0461</v>
       </c>
       <c r="W18" t="n">
-        <v>-5.0594</v>
+        <v>3.1354</v>
       </c>
       <c r="X18" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y18" t="n">
-        <v>13.5251</v>
+        <v>-13.0291</v>
       </c>
       <c r="Z18" t="n">
-        <v>15.8881</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA18" t="n">
-        <v>-0.0246</v>
+        <v>-5.1219</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.4765</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC18" t="n">
-        <v>5.0983</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>113.33</v>
+        <v>116.9533</v>
       </c>
       <c r="C19" t="n">
-        <v>115.48</v>
+        <v>123.8188</v>
       </c>
       <c r="D19" t="n">
-        <v>112.01</v>
+        <v>116.6035</v>
       </c>
       <c r="E19" t="n">
-        <v>114.82</v>
+        <v>123.589</v>
       </c>
       <c r="F19" t="n">
-        <v>71.13</v>
+        <v>71.92</v>
       </c>
       <c r="G19" t="n">
-        <v>71.72</v>
+        <v>72.78</v>
       </c>
       <c r="H19" t="n">
-        <v>70.37</v>
+        <v>70.81</v>
       </c>
       <c r="I19" t="n">
-        <v>71.38</v>
+        <v>72.64</v>
       </c>
       <c r="J19" t="n">
-        <v>45.72</v>
+        <v>43.5656</v>
       </c>
       <c r="K19" t="n">
-        <v>46.34</v>
+        <v>43.7138</v>
       </c>
       <c r="L19" t="n">
-        <v>44.67</v>
+        <v>40.9582</v>
       </c>
       <c r="M19" t="n">
-        <v>44.99</v>
+        <v>40.978</v>
       </c>
       <c r="N19" t="n">
-        <v>38.69</v>
+        <v>38.26</v>
       </c>
       <c r="O19" t="n">
-        <v>39.14</v>
+        <v>38.87</v>
       </c>
       <c r="P19" t="n">
-        <v>38.33</v>
+        <v>37.8</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.53</v>
+        <v>37.87</v>
       </c>
       <c r="R19" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="S19" t="n">
-        <v>13.537</v>
+        <v>20.8659</v>
       </c>
       <c r="T19" t="n">
-        <v>-0.8120000000000001</v>
+        <v>1.5186</v>
       </c>
       <c r="U19" t="n">
-        <v>5.0788</v>
+        <v>1.7652</v>
       </c>
       <c r="V19" t="n">
-        <v>3.0461</v>
+        <v>6.9809</v>
       </c>
       <c r="W19" t="n">
-        <v>3.1354</v>
+        <v>2.3387</v>
       </c>
       <c r="X19" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y19" t="n">
-        <v>-13.0292</v>
+        <v>-18.8062</v>
       </c>
       <c r="Z19" t="n">
-        <v>-3.7441</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA19" t="n">
-        <v>-5.1219</v>
+        <v>-1.713</v>
       </c>
       <c r="AB19" t="n">
-        <v>-3.2639</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC19" t="n">
-        <v>-3.4336</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>117.03</v>
+        <v>131.9835</v>
       </c>
       <c r="C20" t="n">
-        <v>123.9</v>
+        <v>143.9056</v>
       </c>
       <c r="D20" t="n">
-        <v>116.68</v>
+        <v>129.5351</v>
       </c>
       <c r="E20" t="n">
-        <v>123.67</v>
+        <v>141.837</v>
       </c>
       <c r="F20" t="n">
-        <v>71.92</v>
+        <v>74.83</v>
       </c>
       <c r="G20" t="n">
-        <v>72.78</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>70.81</v>
+        <v>74.83</v>
       </c>
       <c r="I20" t="n">
-        <v>72.64</v>
+        <v>78.91</v>
       </c>
       <c r="J20" t="n">
-        <v>44.11</v>
+        <v>38.2718</v>
       </c>
       <c r="K20" t="n">
-        <v>44.26</v>
+        <v>39.0224</v>
       </c>
       <c r="L20" t="n">
-        <v>41.47</v>
+        <v>34.252</v>
       </c>
       <c r="M20" t="n">
-        <v>41.49</v>
+        <v>34.894</v>
       </c>
       <c r="N20" t="n">
-        <v>38.26</v>
+        <v>36.73</v>
       </c>
       <c r="O20" t="n">
-        <v>38.87</v>
+        <v>36.74</v>
       </c>
       <c r="P20" t="n">
-        <v>37.8</v>
+        <v>34.31</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.87</v>
+        <v>34.6</v>
       </c>
       <c r="R20" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="S20" t="n">
-        <v>20.8659</v>
+        <v>36.5105</v>
       </c>
       <c r="T20" t="n">
-        <v>1.5186</v>
+        <v>40.3442</v>
       </c>
       <c r="U20" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V20" t="n">
-        <v>6.9809</v>
+        <v>16.1637</v>
       </c>
       <c r="W20" t="n">
-        <v>2.3387</v>
+        <v>13.9166</v>
       </c>
       <c r="X20" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="Y20" t="n">
-        <v>-18.8063</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z20" t="n">
-        <v>-6.0036</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.713</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.7701</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC20" t="n">
-        <v>-2.5727</v>
+        <v>-13.1308</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>132.07</v>
+        <v>137.67</v>
       </c>
       <c r="C21" t="n">
-        <v>144</v>
+        <v>152.64</v>
       </c>
       <c r="D21" t="n">
-        <v>129.62</v>
+        <v>137.46</v>
       </c>
       <c r="E21" t="n">
-        <v>141.93</v>
+        <v>151.95</v>
       </c>
       <c r="F21" t="n">
-        <v>74.83</v>
+        <v>78.77</v>
       </c>
       <c r="G21" t="n">
-        <v>79.48999999999999</v>
+        <v>81.12</v>
       </c>
       <c r="H21" t="n">
-        <v>74.83</v>
+        <v>78.77</v>
       </c>
       <c r="I21" t="n">
-        <v>78.91</v>
+        <v>80.83</v>
       </c>
       <c r="J21" t="n">
-        <v>38.75</v>
+        <v>35.98</v>
       </c>
       <c r="K21" t="n">
-        <v>39.51</v>
+        <v>36.01</v>
       </c>
       <c r="L21" t="n">
-        <v>34.68</v>
+        <v>32.25</v>
       </c>
       <c r="M21" t="n">
-        <v>35.33</v>
+        <v>32.42</v>
       </c>
       <c r="N21" t="n">
-        <v>36.73</v>
+        <v>34.66</v>
       </c>
       <c r="O21" t="n">
-        <v>36.74</v>
+        <v>34.66</v>
       </c>
       <c r="P21" t="n">
-        <v>34.31</v>
+        <v>33.64</v>
       </c>
       <c r="Q21" t="n">
-        <v>34.6</v>
+        <v>33.77</v>
       </c>
       <c r="R21" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S21" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="T21" t="n">
-        <v>40.3441</v>
+        <v>48.602</v>
       </c>
       <c r="U21" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V21" t="n">
-        <v>16.1637</v>
+        <v>13.239</v>
       </c>
       <c r="W21" t="n">
-        <v>13.9166</v>
+        <v>19.0427</v>
       </c>
       <c r="X21" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y21" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z21" t="n">
-        <v>-31.7031</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA21" t="n">
-        <v>-8.6348</v>
+        <v>-2.3988</v>
       </c>
       <c r="AB21" t="n">
-        <v>-14.7993</v>
+        <v>-12.354</v>
       </c>
       <c r="AC21" t="n">
-        <v>-13.1308</v>
+        <v>-16.8636</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-25 00:18
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1719 +568,1719 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>117.2931</v>
+        <v>114.6248</v>
       </c>
       <c r="C2" t="n">
-        <v>119.8014</v>
+        <v>117.3131</v>
       </c>
       <c r="D2" t="n">
-        <v>113.0559</v>
+        <v>112.4563</v>
       </c>
       <c r="E2" t="n">
-        <v>115.5942</v>
+        <v>116.5236</v>
       </c>
       <c r="F2" t="n">
-        <v>70.42</v>
+        <v>69.42570000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>71.27</v>
+        <v>70.8031</v>
       </c>
       <c r="H2" t="n">
-        <v>69.34999999999999</v>
+        <v>69.306</v>
       </c>
       <c r="I2" t="n">
-        <v>70.27</v>
+        <v>70.334</v>
       </c>
       <c r="J2" t="n">
-        <v>47.2299</v>
+        <v>48.4052</v>
       </c>
       <c r="K2" t="n">
-        <v>49.2151</v>
+        <v>49.2743</v>
       </c>
       <c r="L2" t="n">
-        <v>46.0842</v>
+        <v>47.2792</v>
       </c>
       <c r="M2" t="n">
-        <v>47.8225</v>
+        <v>47.4965</v>
       </c>
       <c r="N2" t="n">
-        <v>39.38</v>
+        <v>39.3017</v>
       </c>
       <c r="O2" t="n">
-        <v>40.02</v>
+        <v>39.3707</v>
       </c>
       <c r="P2" t="n">
-        <v>38.89</v>
+        <v>38.5425</v>
       </c>
       <c r="Q2" t="n">
-        <v>39.46</v>
+        <v>38.8284</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114.6248</v>
+        <v>123.3191</v>
       </c>
       <c r="C3" t="n">
-        <v>117.3131</v>
+        <v>124.7982</v>
       </c>
       <c r="D3" t="n">
-        <v>112.4563</v>
+        <v>117.6129</v>
       </c>
       <c r="E3" t="n">
-        <v>116.5236</v>
+        <v>122.9694</v>
       </c>
       <c r="F3" t="n">
-        <v>69.56</v>
+        <v>71.9509</v>
       </c>
       <c r="G3" t="n">
-        <v>70.94</v>
+        <v>73.2384</v>
       </c>
       <c r="H3" t="n">
-        <v>69.44</v>
+        <v>71.2422</v>
       </c>
       <c r="I3" t="n">
-        <v>70.47</v>
+        <v>73.1585</v>
       </c>
       <c r="J3" t="n">
-        <v>48.4052</v>
+        <v>44.8595</v>
       </c>
       <c r="K3" t="n">
-        <v>49.2743</v>
+        <v>47.1212</v>
       </c>
       <c r="L3" t="n">
-        <v>47.2792</v>
+        <v>44.1582</v>
       </c>
       <c r="M3" t="n">
-        <v>47.4965</v>
+        <v>44.7903</v>
       </c>
       <c r="N3" t="n">
-        <v>39.86</v>
+        <v>37.9213</v>
       </c>
       <c r="O3" t="n">
-        <v>39.93</v>
+        <v>38.3157</v>
       </c>
       <c r="P3" t="n">
-        <v>39.09</v>
+        <v>37.2015</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.38</v>
+        <v>37.2508</v>
       </c>
       <c r="R3" t="n">
-        <v>0.804</v>
+        <v>5.5318</v>
       </c>
       <c r="U3" t="n">
-        <v>0.2846</v>
+        <v>4.0158</v>
       </c>
       <c r="X3" t="n">
-        <v>-0.6817</v>
+        <v>-5.6977</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.2027</v>
+        <v>-4.063</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>123.3191</v>
+        <v>119.8414</v>
       </c>
       <c r="C4" t="n">
-        <v>124.7982</v>
+        <v>121.1206</v>
       </c>
       <c r="D4" t="n">
-        <v>117.6129</v>
+        <v>110.1378</v>
       </c>
       <c r="E4" t="n">
-        <v>122.9694</v>
+        <v>111.267</v>
       </c>
       <c r="F4" t="n">
-        <v>72.09</v>
+        <v>72.7094</v>
       </c>
       <c r="G4" t="n">
-        <v>73.38</v>
+        <v>74.0368</v>
       </c>
       <c r="H4" t="n">
-        <v>71.38</v>
+        <v>71.2921</v>
       </c>
       <c r="I4" t="n">
-        <v>73.3</v>
+        <v>71.71129999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>44.8595</v>
+        <v>46.0348</v>
       </c>
       <c r="K4" t="n">
-        <v>47.1212</v>
+        <v>49.6101</v>
       </c>
       <c r="L4" t="n">
-        <v>44.1582</v>
+        <v>45.5805</v>
       </c>
       <c r="M4" t="n">
-        <v>44.7903</v>
+        <v>49.2052</v>
       </c>
       <c r="N4" t="n">
-        <v>38.46</v>
+        <v>37.4875</v>
       </c>
       <c r="O4" t="n">
-        <v>38.86</v>
+        <v>38.2171</v>
       </c>
       <c r="P4" t="n">
-        <v>37.73</v>
+        <v>36.8071</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.78</v>
+        <v>38.0002</v>
       </c>
       <c r="R4" t="n">
-        <v>5.5318</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>4.0159</v>
+        <v>-1.9782</v>
       </c>
       <c r="X4" t="n">
-        <v>-5.6977</v>
+        <v>9.8568</v>
       </c>
       <c r="AA4" t="n">
-        <v>-4.063</v>
+        <v>2.0118</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>119.8414</v>
+        <v>112.3363</v>
       </c>
       <c r="C5" t="n">
-        <v>121.1206</v>
+        <v>114.9746</v>
       </c>
       <c r="D5" t="n">
-        <v>110.1378</v>
+        <v>110.2577</v>
       </c>
       <c r="E5" t="n">
-        <v>111.267</v>
+        <v>112.7161</v>
       </c>
       <c r="F5" t="n">
-        <v>72.84999999999999</v>
+        <v>71.3021</v>
       </c>
       <c r="G5" t="n">
-        <v>74.18000000000001</v>
+        <v>72.0107</v>
       </c>
       <c r="H5" t="n">
-        <v>71.43000000000001</v>
+        <v>70.6833</v>
       </c>
       <c r="I5" t="n">
-        <v>71.84999999999999</v>
+        <v>71.7812</v>
       </c>
       <c r="J5" t="n">
-        <v>46.0348</v>
+        <v>48.662</v>
       </c>
       <c r="K5" t="n">
-        <v>49.6101</v>
+        <v>49.62</v>
       </c>
       <c r="L5" t="n">
-        <v>45.5805</v>
+        <v>47.4965</v>
       </c>
       <c r="M5" t="n">
-        <v>49.2052</v>
+        <v>48.4151</v>
       </c>
       <c r="N5" t="n">
-        <v>38.02</v>
+        <v>38.227</v>
       </c>
       <c r="O5" t="n">
-        <v>38.76</v>
+        <v>38.5425</v>
       </c>
       <c r="P5" t="n">
-        <v>37.33</v>
+        <v>37.8326</v>
       </c>
       <c r="Q5" t="n">
-        <v>38.54</v>
+        <v>37.9706</v>
       </c>
       <c r="R5" t="n">
-        <v>-9.516500000000001</v>
+        <v>1.3024</v>
       </c>
       <c r="S5" t="n">
-        <v>-3.7434</v>
+        <v>-3.2676</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.9782</v>
+        <v>0.0975</v>
       </c>
       <c r="V5" t="n">
-        <v>2.2485</v>
+        <v>2.0576</v>
       </c>
       <c r="X5" t="n">
-        <v>9.8568</v>
+        <v>-1.6057</v>
       </c>
       <c r="Y5" t="n">
-        <v>2.8913</v>
+        <v>1.934</v>
       </c>
       <c r="AA5" t="n">
-        <v>2.0116</v>
+        <v>-0.0779</v>
       </c>
       <c r="AB5" t="n">
-        <v>-2.3315</v>
+        <v>-2.2092</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>112.3363</v>
+        <v>106.2903</v>
       </c>
       <c r="C6" t="n">
-        <v>114.9746</v>
+        <v>108.5688</v>
       </c>
       <c r="D6" t="n">
-        <v>110.2577</v>
+        <v>102.243</v>
       </c>
       <c r="E6" t="n">
-        <v>112.7161</v>
+        <v>105.8406</v>
       </c>
       <c r="F6" t="n">
-        <v>71.44</v>
+        <v>68.9367</v>
       </c>
       <c r="G6" t="n">
-        <v>72.15000000000001</v>
+        <v>70.41379999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>70.81999999999999</v>
+        <v>68.1183</v>
       </c>
       <c r="I6" t="n">
-        <v>71.92</v>
+        <v>69.01649999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>48.662</v>
+        <v>51.2398</v>
       </c>
       <c r="K6" t="n">
-        <v>49.62</v>
+        <v>53.0274</v>
       </c>
       <c r="L6" t="n">
-        <v>47.4965</v>
+        <v>50.2719</v>
       </c>
       <c r="M6" t="n">
-        <v>48.4151</v>
+        <v>51.5756</v>
       </c>
       <c r="N6" t="n">
-        <v>38.77</v>
+        <v>39.4693</v>
       </c>
       <c r="O6" t="n">
-        <v>39.09</v>
+        <v>39.9032</v>
       </c>
       <c r="P6" t="n">
-        <v>38.37</v>
+        <v>38.6805</v>
       </c>
       <c r="Q6" t="n">
-        <v>38.51</v>
+        <v>39.4102</v>
       </c>
       <c r="R6" t="n">
-        <v>1.3024</v>
+        <v>-6.0998</v>
       </c>
       <c r="S6" t="n">
-        <v>-3.2676</v>
+        <v>-13.9293</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0974</v>
+        <v>-3.8516</v>
       </c>
       <c r="V6" t="n">
-        <v>2.0576</v>
+        <v>-5.6617</v>
       </c>
       <c r="X6" t="n">
-        <v>-1.6057</v>
+        <v>6.5279</v>
       </c>
       <c r="Y6" t="n">
-        <v>1.934</v>
+        <v>15.149</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.07779999999999999</v>
+        <v>3.7914</v>
       </c>
       <c r="AB6" t="n">
-        <v>-2.2092</v>
+        <v>5.7969</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>106.2903</v>
+        <v>104.4315</v>
       </c>
       <c r="C7" t="n">
-        <v>108.5688</v>
+        <v>107.9992</v>
       </c>
       <c r="D7" t="n">
-        <v>102.243</v>
+        <v>101.2736</v>
       </c>
       <c r="E7" t="n">
-        <v>105.8406</v>
+        <v>106.2803</v>
       </c>
       <c r="F7" t="n">
-        <v>69.06999999999999</v>
+        <v>68.8369</v>
       </c>
       <c r="G7" t="n">
-        <v>70.55</v>
+        <v>69.6254</v>
       </c>
       <c r="H7" t="n">
-        <v>68.25</v>
+        <v>68.258</v>
       </c>
       <c r="I7" t="n">
-        <v>69.15000000000001</v>
+        <v>69.4657</v>
       </c>
       <c r="J7" t="n">
-        <v>51.2398</v>
+        <v>52.1484</v>
       </c>
       <c r="K7" t="n">
-        <v>53.0274</v>
+        <v>53.7188</v>
       </c>
       <c r="L7" t="n">
-        <v>50.2719</v>
+        <v>50.42</v>
       </c>
       <c r="M7" t="n">
-        <v>51.5756</v>
+        <v>51.1904</v>
       </c>
       <c r="N7" t="n">
-        <v>40.03</v>
+        <v>39.5285</v>
       </c>
       <c r="O7" t="n">
-        <v>40.47</v>
+        <v>39.8637</v>
       </c>
       <c r="P7" t="n">
-        <v>39.23</v>
+        <v>39.0749</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.97</v>
+        <v>39.1538</v>
       </c>
       <c r="R7" t="n">
-        <v>-6.0998</v>
+        <v>0.4154</v>
       </c>
       <c r="S7" t="n">
-        <v>-13.9293</v>
+        <v>-4.4817</v>
       </c>
       <c r="T7" t="n">
-        <v>-8.437799999999999</v>
+        <v>-8.790800000000001</v>
       </c>
       <c r="U7" t="n">
-        <v>-3.8515</v>
+        <v>0.6509</v>
       </c>
       <c r="V7" t="n">
-        <v>-5.6617</v>
+        <v>-3.1314</v>
       </c>
       <c r="W7" t="n">
-        <v>-1.5939</v>
+        <v>-1.2345</v>
       </c>
       <c r="X7" t="n">
-        <v>6.5279</v>
+        <v>-0.7469</v>
       </c>
       <c r="Y7" t="n">
-        <v>15.149</v>
+        <v>4.0345</v>
       </c>
       <c r="Z7" t="n">
-        <v>7.848</v>
+        <v>7.7772</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.7912</v>
+        <v>-0.6506</v>
       </c>
       <c r="AB7" t="n">
-        <v>5.7967</v>
+        <v>3.0358</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.2924</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>104.4315</v>
+        <v>102.9325</v>
       </c>
       <c r="C8" t="n">
-        <v>107.9992</v>
+        <v>107.4196</v>
       </c>
       <c r="D8" t="n">
-        <v>101.2736</v>
+        <v>98.55540000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>106.2803</v>
+        <v>106.6701</v>
       </c>
       <c r="F8" t="n">
-        <v>68.97</v>
+        <v>69.9248</v>
       </c>
       <c r="G8" t="n">
-        <v>69.76000000000001</v>
+        <v>72.28019999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>68.39</v>
+        <v>69.57550000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>69.59999999999999</v>
+        <v>71.89100000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>52.1484</v>
+        <v>52.8398</v>
       </c>
       <c r="K8" t="n">
-        <v>53.7188</v>
+        <v>55.0027</v>
       </c>
       <c r="L8" t="n">
-        <v>50.42</v>
+        <v>50.6472</v>
       </c>
       <c r="M8" t="n">
-        <v>51.1904</v>
+        <v>50.9632</v>
       </c>
       <c r="N8" t="n">
-        <v>40.09</v>
+        <v>38.9369</v>
       </c>
       <c r="O8" t="n">
-        <v>40.43</v>
+        <v>39.1242</v>
       </c>
       <c r="P8" t="n">
-        <v>39.63</v>
+        <v>37.5861</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.71</v>
+        <v>37.803</v>
       </c>
       <c r="R8" t="n">
-        <v>0.4154</v>
+        <v>0.3668</v>
       </c>
       <c r="S8" t="n">
-        <v>-4.4817</v>
+        <v>-5.3639</v>
       </c>
       <c r="T8" t="n">
-        <v>-8.790800000000001</v>
+        <v>-13.2548</v>
       </c>
       <c r="U8" t="n">
-        <v>0.6508</v>
+        <v>3.4914</v>
       </c>
       <c r="V8" t="n">
-        <v>-3.1315</v>
+        <v>0.153</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.2346</v>
+        <v>-1.7325</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.7469</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y8" t="n">
-        <v>4.0345</v>
+        <v>5.263</v>
       </c>
       <c r="Z8" t="n">
-        <v>7.7772</v>
+        <v>13.7818</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.6505</v>
+        <v>-3.45</v>
       </c>
       <c r="AB8" t="n">
-        <v>3.0358</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.838</v>
+        <v>1.4824</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>102.9325</v>
+        <v>111.1471</v>
       </c>
       <c r="C9" t="n">
-        <v>107.4196</v>
+        <v>118.1026</v>
       </c>
       <c r="D9" t="n">
-        <v>98.55540000000001</v>
+        <v>109.6581</v>
       </c>
       <c r="E9" t="n">
-        <v>106.6701</v>
+        <v>117.2032</v>
       </c>
       <c r="F9" t="n">
-        <v>70.06</v>
+        <v>72.3501</v>
       </c>
       <c r="G9" t="n">
-        <v>72.42</v>
+        <v>73.0986</v>
       </c>
       <c r="H9" t="n">
-        <v>69.70999999999999</v>
+        <v>71.5117</v>
       </c>
       <c r="I9" t="n">
-        <v>72.03</v>
+        <v>72.2303</v>
       </c>
       <c r="J9" t="n">
-        <v>52.8398</v>
+        <v>48.9484</v>
       </c>
       <c r="K9" t="n">
-        <v>55.0027</v>
+        <v>49.5904</v>
       </c>
       <c r="L9" t="n">
-        <v>50.6472</v>
+        <v>45.5311</v>
       </c>
       <c r="M9" t="n">
-        <v>50.9632</v>
+        <v>45.7681</v>
       </c>
       <c r="N9" t="n">
-        <v>39.49</v>
+        <v>37.5861</v>
       </c>
       <c r="O9" t="n">
-        <v>39.68</v>
+        <v>38.0396</v>
       </c>
       <c r="P9" t="n">
-        <v>38.12</v>
+        <v>37.1917</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.34</v>
+        <v>37.6452</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3668</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S9" t="n">
-        <v>-5.3639</v>
+        <v>10.7356</v>
       </c>
       <c r="T9" t="n">
-        <v>-13.2548</v>
+        <v>5.3351</v>
       </c>
       <c r="U9" t="n">
-        <v>3.4914</v>
+        <v>0.472</v>
       </c>
       <c r="V9" t="n">
-        <v>0.1529</v>
+        <v>4.6566</v>
       </c>
       <c r="W9" t="n">
-        <v>-1.7326</v>
+        <v>0.7237</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.4438</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y9" t="n">
-        <v>5.263</v>
+        <v>-11.2602</v>
       </c>
       <c r="Z9" t="n">
-        <v>13.7818</v>
+        <v>-6.9852</v>
       </c>
       <c r="AA9" t="n">
-        <v>-3.45</v>
+        <v>-0.4174</v>
       </c>
       <c r="AB9" t="n">
-        <v>-0.4414</v>
+        <v>-4.4785</v>
       </c>
       <c r="AC9" t="n">
-        <v>1.4823</v>
+        <v>-0.9342</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>111.1471</v>
+        <v>125.038</v>
       </c>
       <c r="C10" t="n">
-        <v>118.1026</v>
+        <v>127.4564</v>
       </c>
       <c r="D10" t="n">
-        <v>109.6581</v>
+        <v>121.5203</v>
       </c>
       <c r="E10" t="n">
-        <v>117.2032</v>
+        <v>123.1892</v>
       </c>
       <c r="F10" t="n">
-        <v>72.48999999999999</v>
+        <v>72.8092</v>
       </c>
       <c r="G10" t="n">
-        <v>73.23999999999999</v>
+        <v>73.06870000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>71.65000000000001</v>
+        <v>71.1824</v>
       </c>
       <c r="I10" t="n">
-        <v>72.37</v>
+        <v>72.02070000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>48.9484</v>
+        <v>43.0126</v>
       </c>
       <c r="K10" t="n">
-        <v>49.5904</v>
+        <v>44.2768</v>
       </c>
       <c r="L10" t="n">
-        <v>45.5311</v>
+        <v>41.9854</v>
       </c>
       <c r="M10" t="n">
-        <v>45.7681</v>
+        <v>43.536</v>
       </c>
       <c r="N10" t="n">
-        <v>38.12</v>
+        <v>37.3593</v>
       </c>
       <c r="O10" t="n">
-        <v>38.58</v>
+        <v>38.1974</v>
       </c>
       <c r="P10" t="n">
-        <v>37.72</v>
+        <v>37.2213</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.18</v>
+        <v>37.7734</v>
       </c>
       <c r="R10" t="n">
-        <v>9.874499999999999</v>
+        <v>5.1074</v>
       </c>
       <c r="S10" t="n">
-        <v>10.7356</v>
+        <v>15.9097</v>
       </c>
       <c r="T10" t="n">
-        <v>5.3351</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U10" t="n">
-        <v>0.472</v>
+        <v>-0.2902</v>
       </c>
       <c r="V10" t="n">
-        <v>4.6565</v>
+        <v>3.6781</v>
       </c>
       <c r="W10" t="n">
-        <v>0.7237</v>
+        <v>0.3337</v>
       </c>
       <c r="X10" t="n">
-        <v>-10.1938</v>
+        <v>-4.877</v>
       </c>
       <c r="Y10" t="n">
-        <v>-11.2602</v>
+        <v>-14.9528</v>
       </c>
       <c r="Z10" t="n">
-        <v>-6.9852</v>
+        <v>-10.0776</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.4173</v>
+        <v>0.3405</v>
       </c>
       <c r="AB10" t="n">
-        <v>-4.4784</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC10" t="n">
-        <v>-0.9341</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>125.038</v>
+        <v>121.1606</v>
       </c>
       <c r="C11" t="n">
-        <v>127.4564</v>
+        <v>128.3958</v>
       </c>
       <c r="D11" t="n">
-        <v>121.5203</v>
+        <v>121.1606</v>
       </c>
       <c r="E11" t="n">
-        <v>123.1892</v>
+        <v>125.7875</v>
       </c>
       <c r="F11" t="n">
-        <v>72.95</v>
+        <v>71.4119</v>
       </c>
       <c r="G11" t="n">
-        <v>73.20999999999999</v>
+        <v>72.41</v>
       </c>
       <c r="H11" t="n">
-        <v>71.31999999999999</v>
+        <v>70.7033</v>
       </c>
       <c r="I11" t="n">
-        <v>72.16</v>
+        <v>71.4119</v>
       </c>
       <c r="J11" t="n">
-        <v>43.0126</v>
+        <v>44.2471</v>
       </c>
       <c r="K11" t="n">
-        <v>44.2768</v>
+        <v>44.2669</v>
       </c>
       <c r="L11" t="n">
-        <v>41.9854</v>
+        <v>41.7977</v>
       </c>
       <c r="M11" t="n">
-        <v>43.536</v>
+        <v>42.7064</v>
       </c>
       <c r="N11" t="n">
-        <v>37.89</v>
+        <v>38.0889</v>
       </c>
       <c r="O11" t="n">
-        <v>38.74</v>
+        <v>38.4636</v>
       </c>
       <c r="P11" t="n">
-        <v>37.75</v>
+        <v>37.5664</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.31</v>
+        <v>38.0988</v>
       </c>
       <c r="R11" t="n">
-        <v>5.1074</v>
+        <v>2.1092</v>
       </c>
       <c r="S11" t="n">
-        <v>15.9097</v>
+        <v>17.922</v>
       </c>
       <c r="T11" t="n">
-        <v>9.291600000000001</v>
+        <v>18.8462</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.2902</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>3.6782</v>
+        <v>-0.6664</v>
       </c>
       <c r="W11" t="n">
-        <v>0.3337</v>
+        <v>3.4708</v>
       </c>
       <c r="X11" t="n">
-        <v>-4.877</v>
+        <v>-1.9055</v>
       </c>
       <c r="Y11" t="n">
-        <v>-14.9528</v>
+        <v>-16.2015</v>
       </c>
       <c r="Z11" t="n">
-        <v>-10.0776</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.3405</v>
+        <v>0.8615</v>
       </c>
       <c r="AB11" t="n">
-        <v>-3.5256</v>
+        <v>0.7825</v>
       </c>
       <c r="AC11" t="n">
-        <v>-0.5193</v>
+        <v>-3.3276</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>121.1606</v>
+        <v>116.2738</v>
       </c>
       <c r="C12" t="n">
-        <v>128.3958</v>
+        <v>119.2418</v>
       </c>
       <c r="D12" t="n">
-        <v>121.1606</v>
+        <v>113.4756</v>
       </c>
       <c r="E12" t="n">
-        <v>125.7875</v>
+        <v>115.6842</v>
       </c>
       <c r="F12" t="n">
-        <v>71.55</v>
+        <v>68.767</v>
       </c>
       <c r="G12" t="n">
-        <v>72.55</v>
+        <v>70.0945</v>
       </c>
       <c r="H12" t="n">
-        <v>70.84</v>
+        <v>68.5474</v>
       </c>
       <c r="I12" t="n">
-        <v>71.55</v>
+        <v>69.07640000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>44.2471</v>
+        <v>45.9459</v>
       </c>
       <c r="K12" t="n">
-        <v>44.2669</v>
+        <v>46.9039</v>
       </c>
       <c r="L12" t="n">
-        <v>41.7977</v>
+        <v>44.9385</v>
       </c>
       <c r="M12" t="n">
-        <v>42.7064</v>
+        <v>46.1632</v>
       </c>
       <c r="N12" t="n">
-        <v>38.63</v>
+        <v>39.5186</v>
       </c>
       <c r="O12" t="n">
-        <v>39.01</v>
+        <v>39.6271</v>
       </c>
       <c r="P12" t="n">
-        <v>38.1</v>
+        <v>38.7988</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.64</v>
+        <v>39.3411</v>
       </c>
       <c r="R12" t="n">
-        <v>2.1092</v>
+        <v>-8.032</v>
       </c>
       <c r="S12" t="n">
-        <v>17.922</v>
+        <v>-1.296</v>
       </c>
       <c r="T12" t="n">
-        <v>18.8462</v>
+        <v>8.8482</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2705</v>
       </c>
       <c r="V12" t="n">
-        <v>-0.6664</v>
+        <v>-4.3665</v>
       </c>
       <c r="W12" t="n">
-        <v>3.4707</v>
+        <v>-0.5604</v>
       </c>
       <c r="X12" t="n">
-        <v>-1.9055</v>
+        <v>8.0943</v>
       </c>
       <c r="Y12" t="n">
-        <v>-16.2015</v>
+        <v>0.8633</v>
       </c>
       <c r="Z12" t="n">
-        <v>-17.1965</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.8614000000000001</v>
+        <v>3.2607</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.7825</v>
+        <v>4.505</v>
       </c>
       <c r="AC12" t="n">
-        <v>-3.3275</v>
+        <v>0.4784</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>116.2738</v>
+        <v>120.6309</v>
       </c>
       <c r="C13" t="n">
-        <v>119.2418</v>
+        <v>124.4184</v>
       </c>
       <c r="D13" t="n">
-        <v>113.4756</v>
+        <v>117.7928</v>
       </c>
       <c r="E13" t="n">
-        <v>115.6842</v>
+        <v>121.7402</v>
       </c>
       <c r="F13" t="n">
-        <v>68.90000000000001</v>
+        <v>71.0526</v>
       </c>
       <c r="G13" t="n">
-        <v>70.23</v>
+        <v>71.6215</v>
       </c>
       <c r="H13" t="n">
-        <v>68.68000000000001</v>
+        <v>70.47369999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>69.20999999999999</v>
+        <v>70.843</v>
       </c>
       <c r="J13" t="n">
-        <v>45.9459</v>
+        <v>44.1385</v>
       </c>
       <c r="K13" t="n">
-        <v>46.9039</v>
+        <v>45.2545</v>
       </c>
       <c r="L13" t="n">
-        <v>44.9385</v>
+        <v>42.5879</v>
       </c>
       <c r="M13" t="n">
-        <v>46.1632</v>
+        <v>43.5953</v>
       </c>
       <c r="N13" t="n">
-        <v>40.08</v>
+        <v>38.227</v>
       </c>
       <c r="O13" t="n">
-        <v>40.19</v>
+        <v>38.5523</v>
       </c>
       <c r="P13" t="n">
-        <v>39.35</v>
+        <v>37.8819</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.9</v>
+        <v>38.3256</v>
       </c>
       <c r="R13" t="n">
-        <v>-8.032</v>
+        <v>5.2349</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.296</v>
+        <v>-1.1762</v>
       </c>
       <c r="T13" t="n">
-        <v>8.8482</v>
+        <v>14.1278</v>
       </c>
       <c r="U13" t="n">
-        <v>-3.2704</v>
+        <v>2.5575</v>
       </c>
       <c r="V13" t="n">
-        <v>-4.3665</v>
+        <v>-1.6352</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.5603</v>
+        <v>-1.4578</v>
       </c>
       <c r="X13" t="n">
-        <v>8.0943</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.8633</v>
+        <v>0.1362</v>
       </c>
       <c r="Z13" t="n">
-        <v>-9.820600000000001</v>
+        <v>-14.4573</v>
       </c>
       <c r="AA13" t="n">
-        <v>3.2609</v>
+        <v>-2.5813</v>
       </c>
       <c r="AB13" t="n">
-        <v>4.505</v>
+        <v>1.4619</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.4785</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>120.6309</v>
+        <v>101.4635</v>
       </c>
       <c r="C14" t="n">
-        <v>124.4184</v>
+        <v>105.3209</v>
       </c>
       <c r="D14" t="n">
-        <v>117.7928</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>121.7402</v>
+        <v>101.0637</v>
       </c>
       <c r="F14" t="n">
-        <v>71.19</v>
+        <v>67.3997</v>
       </c>
       <c r="G14" t="n">
-        <v>71.76000000000001</v>
+        <v>70.25409999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>70.61</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>70.98</v>
+        <v>69.13630000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>44.1385</v>
+        <v>50.9731</v>
       </c>
       <c r="K14" t="n">
-        <v>45.2545</v>
+        <v>51.5756</v>
       </c>
       <c r="L14" t="n">
-        <v>42.5879</v>
+        <v>49.5904</v>
       </c>
       <c r="M14" t="n">
-        <v>43.5953</v>
+        <v>51.0916</v>
       </c>
       <c r="N14" t="n">
-        <v>38.77</v>
+        <v>40.2088</v>
       </c>
       <c r="O14" t="n">
-        <v>39.1</v>
+        <v>40.3074</v>
       </c>
       <c r="P14" t="n">
-        <v>38.42</v>
+        <v>38.6608</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.87</v>
+        <v>39.2721</v>
       </c>
       <c r="R14" t="n">
-        <v>5.2349</v>
+        <v>-16.9841</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.1762</v>
+        <v>-19.6552</v>
       </c>
       <c r="T14" t="n">
-        <v>14.1278</v>
+        <v>-13.7705</v>
       </c>
       <c r="U14" t="n">
-        <v>2.5574</v>
+        <v>-2.4091</v>
       </c>
       <c r="V14" t="n">
-        <v>-1.6353</v>
+        <v>-3.1866</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.4577</v>
+        <v>-4.2835</v>
       </c>
       <c r="X14" t="n">
-        <v>-5.5627</v>
+        <v>17.1952</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.1362</v>
+        <v>19.6345</v>
       </c>
       <c r="Z14" t="n">
-        <v>-14.4573</v>
+        <v>11.6315</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.5815</v>
+        <v>2.4696</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.4618</v>
+        <v>3.0796</v>
       </c>
       <c r="AC14" t="n">
-        <v>1.3824</v>
+        <v>4.3217</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>101.4635</v>
+        <v>104.4815</v>
       </c>
       <c r="C15" t="n">
-        <v>105.3209</v>
+        <v>105.8706</v>
       </c>
       <c r="D15" t="n">
-        <v>99.80459999999999</v>
+        <v>100.8938</v>
       </c>
       <c r="E15" t="n">
-        <v>101.0637</v>
+        <v>102.253</v>
       </c>
       <c r="F15" t="n">
-        <v>67.53</v>
+        <v>68.9966</v>
       </c>
       <c r="G15" t="n">
-        <v>70.39</v>
+        <v>69.1962</v>
       </c>
       <c r="H15" t="n">
-        <v>67.34</v>
+        <v>67.4795</v>
       </c>
       <c r="I15" t="n">
-        <v>69.27</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>50.9731</v>
+        <v>49.2546</v>
       </c>
       <c r="K15" t="n">
-        <v>51.5756</v>
+        <v>51.1607</v>
       </c>
       <c r="L15" t="n">
-        <v>49.5904</v>
+        <v>48.6521</v>
       </c>
       <c r="M15" t="n">
-        <v>51.0916</v>
+        <v>50.4694</v>
       </c>
       <c r="N15" t="n">
-        <v>40.78</v>
+        <v>39.351</v>
       </c>
       <c r="O15" t="n">
-        <v>40.88</v>
+        <v>40.2088</v>
       </c>
       <c r="P15" t="n">
-        <v>39.21</v>
+        <v>39.2327</v>
       </c>
       <c r="Q15" t="n">
-        <v>39.83</v>
+        <v>40.0511</v>
       </c>
       <c r="R15" t="n">
-        <v>-16.9841</v>
+        <v>1.1768</v>
       </c>
       <c r="S15" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="T15" t="n">
-        <v>-13.7705</v>
+        <v>-16.9952</v>
       </c>
       <c r="U15" t="n">
-        <v>-2.4091</v>
+        <v>-1.9777</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.1866</v>
+        <v>-1.8927</v>
       </c>
       <c r="W15" t="n">
-        <v>-4.2835</v>
+        <v>-5.9034</v>
       </c>
       <c r="X15" t="n">
-        <v>17.1952</v>
+        <v>-1.2178</v>
       </c>
       <c r="Y15" t="n">
-        <v>19.6345</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z15" t="n">
-        <v>11.6315</v>
+        <v>15.9257</v>
       </c>
       <c r="AA15" t="n">
-        <v>2.4698</v>
+        <v>1.9836</v>
       </c>
       <c r="AB15" t="n">
-        <v>3.0797</v>
+        <v>1.8047</v>
       </c>
       <c r="AC15" t="n">
-        <v>4.3216</v>
+        <v>6.0299</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>104.4815</v>
+        <v>107.3696</v>
       </c>
       <c r="C16" t="n">
-        <v>105.8706</v>
+        <v>109.2484</v>
       </c>
       <c r="D16" t="n">
-        <v>100.8938</v>
+        <v>100.9938</v>
       </c>
       <c r="E16" t="n">
-        <v>102.253</v>
+        <v>103.9019</v>
       </c>
       <c r="F16" t="n">
-        <v>69.13</v>
+        <v>68.7171</v>
       </c>
       <c r="G16" t="n">
-        <v>69.33</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>67.61</v>
+        <v>66.4216</v>
       </c>
       <c r="I16" t="n">
-        <v>67.90000000000001</v>
+        <v>67.7989</v>
       </c>
       <c r="J16" t="n">
-        <v>49.2546</v>
+        <v>47.9509</v>
       </c>
       <c r="K16" t="n">
-        <v>51.1607</v>
+        <v>51.1015</v>
       </c>
       <c r="L16" t="n">
-        <v>48.6521</v>
+        <v>46.9829</v>
       </c>
       <c r="M16" t="n">
-        <v>50.4694</v>
+        <v>49.4916</v>
       </c>
       <c r="N16" t="n">
-        <v>39.91</v>
+        <v>39.4989</v>
       </c>
       <c r="O16" t="n">
-        <v>40.78</v>
+        <v>40.8596</v>
       </c>
       <c r="P16" t="n">
-        <v>39.79</v>
+        <v>38.8186</v>
       </c>
       <c r="Q16" t="n">
-        <v>40.62</v>
+        <v>40.0412</v>
       </c>
       <c r="R16" t="n">
-        <v>1.1768</v>
+        <v>1.6126</v>
       </c>
       <c r="S16" t="n">
-        <v>-11.6102</v>
+        <v>-14.6528</v>
       </c>
       <c r="T16" t="n">
-        <v>-16.9952</v>
+        <v>-17.3989</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.9778</v>
+        <v>0.0441</v>
       </c>
       <c r="V16" t="n">
-        <v>-1.8928</v>
+        <v>-4.297</v>
       </c>
       <c r="W16" t="n">
-        <v>-5.9035</v>
+        <v>-5.0594</v>
       </c>
       <c r="X16" t="n">
-        <v>-1.2178</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y16" t="n">
-        <v>9.328200000000001</v>
+        <v>13.5251</v>
       </c>
       <c r="Z16" t="n">
-        <v>15.9257</v>
+        <v>15.888</v>
       </c>
       <c r="AA16" t="n">
-        <v>1.9834</v>
+        <v>-0.0247</v>
       </c>
       <c r="AB16" t="n">
-        <v>1.8045</v>
+        <v>4.4764</v>
       </c>
       <c r="AC16" t="n">
-        <v>6.0298</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>107.3696</v>
+        <v>113.2557</v>
       </c>
       <c r="C17" t="n">
-        <v>109.2484</v>
+        <v>115.4043</v>
       </c>
       <c r="D17" t="n">
-        <v>100.9938</v>
+        <v>111.9366</v>
       </c>
       <c r="E17" t="n">
-        <v>103.9019</v>
+        <v>114.7448</v>
       </c>
       <c r="F17" t="n">
-        <v>68.84999999999999</v>
+        <v>70.9927</v>
       </c>
       <c r="G17" t="n">
-        <v>69.97</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>66.55</v>
+        <v>70.2342</v>
       </c>
       <c r="I17" t="n">
-        <v>67.93000000000001</v>
+        <v>71.2422</v>
       </c>
       <c r="J17" t="n">
-        <v>47.9509</v>
+        <v>45.1558</v>
       </c>
       <c r="K17" t="n">
-        <v>51.1015</v>
+        <v>45.7681</v>
       </c>
       <c r="L17" t="n">
-        <v>46.9829</v>
+        <v>44.1187</v>
       </c>
       <c r="M17" t="n">
-        <v>49.4916</v>
+        <v>44.4348</v>
       </c>
       <c r="N17" t="n">
-        <v>40.06</v>
+        <v>38.1481</v>
       </c>
       <c r="O17" t="n">
-        <v>41.44</v>
+        <v>38.5918</v>
       </c>
       <c r="P17" t="n">
-        <v>39.37</v>
+        <v>37.7931</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.61</v>
+        <v>37.9903</v>
       </c>
       <c r="R17" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="S17" t="n">
-        <v>-14.6528</v>
+        <v>13.5371</v>
       </c>
       <c r="T17" t="n">
-        <v>-17.3989</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U17" t="n">
-        <v>0.0442</v>
+        <v>5.0787</v>
       </c>
       <c r="V17" t="n">
-        <v>-4.297</v>
+        <v>3.046</v>
       </c>
       <c r="W17" t="n">
-        <v>-5.0594</v>
+        <v>3.1354</v>
       </c>
       <c r="X17" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y17" t="n">
-        <v>13.5251</v>
+        <v>-13.0291</v>
       </c>
       <c r="Z17" t="n">
-        <v>15.888</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.0246</v>
+        <v>-5.122</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.4765</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC17" t="n">
-        <v>5.0983</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>113.2557</v>
+        <v>116.9533</v>
       </c>
       <c r="C18" t="n">
-        <v>115.4043</v>
+        <v>123.8188</v>
       </c>
       <c r="D18" t="n">
-        <v>111.9366</v>
+        <v>116.6035</v>
       </c>
       <c r="E18" t="n">
-        <v>114.7448</v>
+        <v>123.589</v>
       </c>
       <c r="F18" t="n">
-        <v>71.13</v>
+        <v>71.7812</v>
       </c>
       <c r="G18" t="n">
-        <v>71.72</v>
+        <v>72.6395</v>
       </c>
       <c r="H18" t="n">
-        <v>70.37</v>
+        <v>70.6733</v>
       </c>
       <c r="I18" t="n">
-        <v>71.38</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>45.1558</v>
+        <v>43.5656</v>
       </c>
       <c r="K18" t="n">
-        <v>45.7681</v>
+        <v>43.7138</v>
       </c>
       <c r="L18" t="n">
-        <v>44.1187</v>
+        <v>40.9582</v>
       </c>
       <c r="M18" t="n">
-        <v>44.4348</v>
+        <v>40.978</v>
       </c>
       <c r="N18" t="n">
-        <v>38.69</v>
+        <v>37.7241</v>
       </c>
       <c r="O18" t="n">
-        <v>39.14</v>
+        <v>38.3256</v>
       </c>
       <c r="P18" t="n">
-        <v>38.33</v>
+        <v>37.2706</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.53</v>
+        <v>37.3396</v>
       </c>
       <c r="R18" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="S18" t="n">
-        <v>13.5371</v>
+        <v>20.8659</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.8120000000000001</v>
+        <v>1.5186</v>
       </c>
       <c r="U18" t="n">
-        <v>5.0788</v>
+        <v>1.7652</v>
       </c>
       <c r="V18" t="n">
-        <v>3.0461</v>
+        <v>6.9808</v>
       </c>
       <c r="W18" t="n">
-        <v>3.1354</v>
+        <v>2.3387</v>
       </c>
       <c r="X18" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y18" t="n">
-        <v>-13.0291</v>
+        <v>-18.8062</v>
       </c>
       <c r="Z18" t="n">
-        <v>-3.7441</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA18" t="n">
-        <v>-5.1219</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB18" t="n">
-        <v>-3.2639</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC18" t="n">
-        <v>-3.4336</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>116.9533</v>
+        <v>131.9835</v>
       </c>
       <c r="C19" t="n">
-        <v>123.8188</v>
+        <v>143.9056</v>
       </c>
       <c r="D19" t="n">
-        <v>116.6035</v>
+        <v>129.5351</v>
       </c>
       <c r="E19" t="n">
-        <v>123.589</v>
+        <v>141.837</v>
       </c>
       <c r="F19" t="n">
-        <v>71.92</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>72.78</v>
+        <v>79.3366</v>
       </c>
       <c r="H19" t="n">
-        <v>70.81</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>72.64</v>
+        <v>78.7577</v>
       </c>
       <c r="J19" t="n">
-        <v>43.5656</v>
+        <v>38.2718</v>
       </c>
       <c r="K19" t="n">
-        <v>43.7138</v>
+        <v>39.0224</v>
       </c>
       <c r="L19" t="n">
-        <v>40.9582</v>
+        <v>34.252</v>
       </c>
       <c r="M19" t="n">
-        <v>40.978</v>
+        <v>34.894</v>
       </c>
       <c r="N19" t="n">
-        <v>38.26</v>
+        <v>36.2155</v>
       </c>
       <c r="O19" t="n">
-        <v>38.87</v>
+        <v>36.2254</v>
       </c>
       <c r="P19" t="n">
-        <v>37.8</v>
+        <v>33.8294</v>
       </c>
       <c r="Q19" t="n">
-        <v>37.87</v>
+        <v>34.1154</v>
       </c>
       <c r="R19" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="S19" t="n">
-        <v>20.8659</v>
+        <v>36.5105</v>
       </c>
       <c r="T19" t="n">
-        <v>1.5186</v>
+        <v>40.3442</v>
       </c>
       <c r="U19" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V19" t="n">
-        <v>6.9809</v>
+        <v>16.1637</v>
       </c>
       <c r="W19" t="n">
-        <v>2.3387</v>
+        <v>13.9166</v>
       </c>
       <c r="X19" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="Y19" t="n">
-        <v>-18.8062</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z19" t="n">
-        <v>-6.0036</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.713</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.7701</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC19" t="n">
-        <v>-2.5727</v>
+        <v>-13.1307</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C20" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D20" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E20" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F20" t="n">
-        <v>74.83</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>79.48999999999999</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>74.83</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>78.91</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K20" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L20" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M20" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N20" t="n">
-        <v>36.73</v>
+        <v>34.1745</v>
       </c>
       <c r="O20" t="n">
-        <v>36.74</v>
+        <v>34.1745</v>
       </c>
       <c r="P20" t="n">
-        <v>34.31</v>
+        <v>33.1688</v>
       </c>
       <c r="Q20" t="n">
-        <v>34.6</v>
+        <v>33.297</v>
       </c>
       <c r="R20" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S20" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="T20" t="n">
-        <v>40.3442</v>
+        <v>48.602</v>
       </c>
       <c r="U20" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V20" t="n">
-        <v>16.1637</v>
+        <v>13.2391</v>
       </c>
       <c r="W20" t="n">
-        <v>13.9166</v>
+        <v>19.0426</v>
       </c>
       <c r="X20" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y20" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z20" t="n">
-        <v>-31.7031</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA20" t="n">
-        <v>-8.6348</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB20" t="n">
-        <v>-14.7993</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC20" t="n">
-        <v>-13.1308</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C21" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D21" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E21" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F21" t="n">
-        <v>78.77</v>
+        <v>80.53</v>
       </c>
       <c r="G21" t="n">
-        <v>81.12</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>78.77</v>
+        <v>77.69</v>
       </c>
       <c r="I21" t="n">
-        <v>80.83</v>
+        <v>78.66</v>
       </c>
       <c r="J21" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K21" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L21" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M21" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N21" t="n">
-        <v>34.66</v>
+        <v>33.37</v>
       </c>
       <c r="O21" t="n">
-        <v>34.66</v>
+        <v>34.54</v>
       </c>
       <c r="P21" t="n">
-        <v>33.64</v>
+        <v>33.35</v>
       </c>
       <c r="Q21" t="n">
-        <v>33.77</v>
+        <v>34.14</v>
       </c>
       <c r="R21" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="S21" t="n">
-        <v>32.4243</v>
+        <v>18.3358</v>
       </c>
       <c r="T21" t="n">
-        <v>48.602</v>
+        <v>40.7578</v>
       </c>
       <c r="U21" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="V21" t="n">
-        <v>13.239</v>
+        <v>8.4969</v>
       </c>
       <c r="W21" t="n">
-        <v>19.0427</v>
+        <v>16.0196</v>
       </c>
       <c r="X21" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="Y21" t="n">
-        <v>-27.0392</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z21" t="n">
-        <v>-35.7631</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA21" t="n">
-        <v>-2.3988</v>
+        <v>2.5318</v>
       </c>
       <c r="AB21" t="n">
-        <v>-12.354</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC21" t="n">
-        <v>-16.8636</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-26 00:24
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1719 +568,1719 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>114.6248</v>
+        <v>123.3191</v>
       </c>
       <c r="C2" t="n">
-        <v>117.3131</v>
+        <v>124.7982</v>
       </c>
       <c r="D2" t="n">
-        <v>112.4563</v>
+        <v>117.6129</v>
       </c>
       <c r="E2" t="n">
-        <v>116.5236</v>
+        <v>122.9694</v>
       </c>
       <c r="F2" t="n">
-        <v>69.42570000000001</v>
+        <v>71.9509</v>
       </c>
       <c r="G2" t="n">
-        <v>70.8031</v>
+        <v>73.2384</v>
       </c>
       <c r="H2" t="n">
-        <v>69.306</v>
+        <v>71.2422</v>
       </c>
       <c r="I2" t="n">
-        <v>70.334</v>
+        <v>73.1585</v>
       </c>
       <c r="J2" t="n">
-        <v>48.4052</v>
+        <v>44.8595</v>
       </c>
       <c r="K2" t="n">
-        <v>49.2743</v>
+        <v>47.1212</v>
       </c>
       <c r="L2" t="n">
-        <v>47.2792</v>
+        <v>44.1582</v>
       </c>
       <c r="M2" t="n">
-        <v>47.4965</v>
+        <v>44.7903</v>
       </c>
       <c r="N2" t="n">
-        <v>39.3017</v>
+        <v>37.9213</v>
       </c>
       <c r="O2" t="n">
-        <v>39.3707</v>
+        <v>38.3157</v>
       </c>
       <c r="P2" t="n">
-        <v>38.5425</v>
+        <v>37.2015</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.8284</v>
+        <v>37.2508</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>123.3191</v>
+        <v>119.8414</v>
       </c>
       <c r="C3" t="n">
-        <v>124.7982</v>
+        <v>121.1206</v>
       </c>
       <c r="D3" t="n">
-        <v>117.6129</v>
+        <v>110.1378</v>
       </c>
       <c r="E3" t="n">
-        <v>122.9694</v>
+        <v>111.267</v>
       </c>
       <c r="F3" t="n">
-        <v>71.9509</v>
+        <v>72.7094</v>
       </c>
       <c r="G3" t="n">
-        <v>73.2384</v>
+        <v>74.0368</v>
       </c>
       <c r="H3" t="n">
-        <v>71.2422</v>
+        <v>71.2921</v>
       </c>
       <c r="I3" t="n">
-        <v>73.1585</v>
+        <v>71.71129999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>44.8595</v>
+        <v>46.0348</v>
       </c>
       <c r="K3" t="n">
-        <v>47.1212</v>
+        <v>49.6101</v>
       </c>
       <c r="L3" t="n">
-        <v>44.1582</v>
+        <v>45.5805</v>
       </c>
       <c r="M3" t="n">
-        <v>44.7903</v>
+        <v>49.2052</v>
       </c>
       <c r="N3" t="n">
-        <v>37.9213</v>
+        <v>37.4875</v>
       </c>
       <c r="O3" t="n">
-        <v>38.3157</v>
+        <v>38.2171</v>
       </c>
       <c r="P3" t="n">
-        <v>37.2015</v>
+        <v>36.8071</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.2508</v>
+        <v>38.0002</v>
       </c>
       <c r="R3" t="n">
-        <v>5.5318</v>
+        <v>-9.516500000000001</v>
       </c>
       <c r="U3" t="n">
-        <v>4.0158</v>
+        <v>-1.9782</v>
       </c>
       <c r="X3" t="n">
-        <v>-5.6977</v>
+        <v>9.8568</v>
       </c>
       <c r="AA3" t="n">
-        <v>-4.063</v>
+        <v>2.0118</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>119.8414</v>
+        <v>112.3363</v>
       </c>
       <c r="C4" t="n">
-        <v>121.1206</v>
+        <v>114.9746</v>
       </c>
       <c r="D4" t="n">
-        <v>110.1378</v>
+        <v>110.2577</v>
       </c>
       <c r="E4" t="n">
-        <v>111.267</v>
+        <v>112.7161</v>
       </c>
       <c r="F4" t="n">
-        <v>72.7094</v>
+        <v>71.3021</v>
       </c>
       <c r="G4" t="n">
-        <v>74.0368</v>
+        <v>72.0107</v>
       </c>
       <c r="H4" t="n">
-        <v>71.2921</v>
+        <v>70.6833</v>
       </c>
       <c r="I4" t="n">
-        <v>71.71129999999999</v>
+        <v>71.7812</v>
       </c>
       <c r="J4" t="n">
-        <v>46.0348</v>
+        <v>48.662</v>
       </c>
       <c r="K4" t="n">
-        <v>49.6101</v>
+        <v>49.62</v>
       </c>
       <c r="L4" t="n">
-        <v>45.5805</v>
+        <v>47.4965</v>
       </c>
       <c r="M4" t="n">
-        <v>49.2052</v>
+        <v>48.4151</v>
       </c>
       <c r="N4" t="n">
-        <v>37.4875</v>
+        <v>38.227</v>
       </c>
       <c r="O4" t="n">
-        <v>38.2171</v>
+        <v>38.5425</v>
       </c>
       <c r="P4" t="n">
-        <v>36.8071</v>
+        <v>37.8326</v>
       </c>
       <c r="Q4" t="n">
-        <v>38.0002</v>
+        <v>37.9706</v>
       </c>
       <c r="R4" t="n">
-        <v>-9.516500000000001</v>
+        <v>1.3024</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.9782</v>
+        <v>0.0975</v>
       </c>
       <c r="X4" t="n">
-        <v>9.8568</v>
+        <v>-1.6057</v>
       </c>
       <c r="AA4" t="n">
-        <v>2.0118</v>
+        <v>-0.0779</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>112.3363</v>
+        <v>106.2903</v>
       </c>
       <c r="C5" t="n">
-        <v>114.9746</v>
+        <v>108.5688</v>
       </c>
       <c r="D5" t="n">
-        <v>110.2577</v>
+        <v>102.243</v>
       </c>
       <c r="E5" t="n">
-        <v>112.7161</v>
+        <v>105.8406</v>
       </c>
       <c r="F5" t="n">
-        <v>71.3021</v>
+        <v>68.9367</v>
       </c>
       <c r="G5" t="n">
-        <v>72.0107</v>
+        <v>70.41379999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>70.6833</v>
+        <v>68.1183</v>
       </c>
       <c r="I5" t="n">
-        <v>71.7812</v>
+        <v>69.01649999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>48.662</v>
+        <v>51.2398</v>
       </c>
       <c r="K5" t="n">
-        <v>49.62</v>
+        <v>53.0274</v>
       </c>
       <c r="L5" t="n">
-        <v>47.4965</v>
+        <v>50.2719</v>
       </c>
       <c r="M5" t="n">
-        <v>48.4151</v>
+        <v>51.5756</v>
       </c>
       <c r="N5" t="n">
-        <v>38.227</v>
+        <v>39.4693</v>
       </c>
       <c r="O5" t="n">
-        <v>38.5425</v>
+        <v>39.9032</v>
       </c>
       <c r="P5" t="n">
-        <v>37.8326</v>
+        <v>38.6805</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.9706</v>
+        <v>39.4102</v>
       </c>
       <c r="R5" t="n">
-        <v>1.3024</v>
+        <v>-6.0998</v>
       </c>
       <c r="S5" t="n">
-        <v>-3.2676</v>
+        <v>-13.9293</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0975</v>
+        <v>-3.8516</v>
       </c>
       <c r="V5" t="n">
-        <v>2.0576</v>
+        <v>-5.6617</v>
       </c>
       <c r="X5" t="n">
-        <v>-1.6057</v>
+        <v>6.5279</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.934</v>
+        <v>15.149</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.0779</v>
+        <v>3.7914</v>
       </c>
       <c r="AB5" t="n">
-        <v>-2.2092</v>
+        <v>5.7969</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>106.2903</v>
+        <v>104.4315</v>
       </c>
       <c r="C6" t="n">
-        <v>108.5688</v>
+        <v>107.9992</v>
       </c>
       <c r="D6" t="n">
-        <v>102.243</v>
+        <v>101.2736</v>
       </c>
       <c r="E6" t="n">
-        <v>105.8406</v>
+        <v>106.2803</v>
       </c>
       <c r="F6" t="n">
-        <v>68.9367</v>
+        <v>68.8369</v>
       </c>
       <c r="G6" t="n">
-        <v>70.41379999999999</v>
+        <v>69.6254</v>
       </c>
       <c r="H6" t="n">
-        <v>68.1183</v>
+        <v>68.258</v>
       </c>
       <c r="I6" t="n">
-        <v>69.01649999999999</v>
+        <v>69.4657</v>
       </c>
       <c r="J6" t="n">
-        <v>51.2398</v>
+        <v>52.1484</v>
       </c>
       <c r="K6" t="n">
-        <v>53.0274</v>
+        <v>53.7188</v>
       </c>
       <c r="L6" t="n">
-        <v>50.2719</v>
+        <v>50.42</v>
       </c>
       <c r="M6" t="n">
-        <v>51.5756</v>
+        <v>51.1904</v>
       </c>
       <c r="N6" t="n">
-        <v>39.4693</v>
+        <v>39.5285</v>
       </c>
       <c r="O6" t="n">
-        <v>39.9032</v>
+        <v>39.8637</v>
       </c>
       <c r="P6" t="n">
-        <v>38.6805</v>
+        <v>39.0749</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.4102</v>
+        <v>39.1538</v>
       </c>
       <c r="R6" t="n">
-        <v>-6.0998</v>
+        <v>0.4154</v>
       </c>
       <c r="S6" t="n">
-        <v>-13.9293</v>
+        <v>-4.4817</v>
       </c>
       <c r="U6" t="n">
-        <v>-3.8516</v>
+        <v>0.6509</v>
       </c>
       <c r="V6" t="n">
-        <v>-5.6617</v>
+        <v>-3.1314</v>
       </c>
       <c r="X6" t="n">
-        <v>6.5279</v>
+        <v>-0.7469</v>
       </c>
       <c r="Y6" t="n">
-        <v>15.149</v>
+        <v>4.0345</v>
       </c>
       <c r="AA6" t="n">
-        <v>3.7914</v>
+        <v>-0.6506</v>
       </c>
       <c r="AB6" t="n">
-        <v>5.7969</v>
+        <v>3.0358</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>104.4315</v>
+        <v>102.9325</v>
       </c>
       <c r="C7" t="n">
-        <v>107.9992</v>
+        <v>107.4196</v>
       </c>
       <c r="D7" t="n">
-        <v>101.2736</v>
+        <v>98.55540000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>106.2803</v>
+        <v>106.6701</v>
       </c>
       <c r="F7" t="n">
-        <v>68.8369</v>
+        <v>69.9248</v>
       </c>
       <c r="G7" t="n">
-        <v>69.6254</v>
+        <v>72.28019999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>68.258</v>
+        <v>69.57550000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>69.4657</v>
+        <v>71.89100000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>52.1484</v>
+        <v>52.8398</v>
       </c>
       <c r="K7" t="n">
-        <v>53.7188</v>
+        <v>55.0027</v>
       </c>
       <c r="L7" t="n">
-        <v>50.42</v>
+        <v>50.6472</v>
       </c>
       <c r="M7" t="n">
-        <v>51.1904</v>
+        <v>50.9632</v>
       </c>
       <c r="N7" t="n">
-        <v>39.5285</v>
+        <v>38.9369</v>
       </c>
       <c r="O7" t="n">
-        <v>39.8637</v>
+        <v>39.1242</v>
       </c>
       <c r="P7" t="n">
-        <v>39.0749</v>
+        <v>37.5861</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.1538</v>
+        <v>37.803</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4154</v>
+        <v>0.3668</v>
       </c>
       <c r="S7" t="n">
-        <v>-4.4817</v>
+        <v>-5.3639</v>
       </c>
       <c r="T7" t="n">
-        <v>-8.790800000000001</v>
+        <v>-13.2548</v>
       </c>
       <c r="U7" t="n">
-        <v>0.6509</v>
+        <v>3.4914</v>
       </c>
       <c r="V7" t="n">
-        <v>-3.1314</v>
+        <v>0.153</v>
       </c>
       <c r="W7" t="n">
-        <v>-1.2345</v>
+        <v>-1.7325</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.7469</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.0345</v>
+        <v>5.263</v>
       </c>
       <c r="Z7" t="n">
-        <v>7.7772</v>
+        <v>13.7818</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.6506</v>
+        <v>-3.45</v>
       </c>
       <c r="AB7" t="n">
-        <v>3.0358</v>
+        <v>-0.4414</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.838</v>
+        <v>1.4824</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>102.9325</v>
+        <v>111.1471</v>
       </c>
       <c r="C8" t="n">
-        <v>107.4196</v>
+        <v>118.1026</v>
       </c>
       <c r="D8" t="n">
-        <v>98.55540000000001</v>
+        <v>109.6581</v>
       </c>
       <c r="E8" t="n">
-        <v>106.6701</v>
+        <v>117.2032</v>
       </c>
       <c r="F8" t="n">
-        <v>69.9248</v>
+        <v>72.3501</v>
       </c>
       <c r="G8" t="n">
-        <v>72.28019999999999</v>
+        <v>73.0986</v>
       </c>
       <c r="H8" t="n">
-        <v>69.57550000000001</v>
+        <v>71.5117</v>
       </c>
       <c r="I8" t="n">
-        <v>71.89100000000001</v>
+        <v>72.2303</v>
       </c>
       <c r="J8" t="n">
-        <v>52.8398</v>
+        <v>48.9484</v>
       </c>
       <c r="K8" t="n">
-        <v>55.0027</v>
+        <v>49.5904</v>
       </c>
       <c r="L8" t="n">
-        <v>50.6472</v>
+        <v>45.5311</v>
       </c>
       <c r="M8" t="n">
-        <v>50.9632</v>
+        <v>45.7681</v>
       </c>
       <c r="N8" t="n">
-        <v>38.9369</v>
+        <v>37.5861</v>
       </c>
       <c r="O8" t="n">
-        <v>39.1242</v>
+        <v>38.0396</v>
       </c>
       <c r="P8" t="n">
-        <v>37.5861</v>
+        <v>37.1917</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.803</v>
+        <v>37.6452</v>
       </c>
       <c r="R8" t="n">
-        <v>0.3668</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S8" t="n">
-        <v>-5.3639</v>
+        <v>10.7356</v>
       </c>
       <c r="T8" t="n">
-        <v>-13.2548</v>
+        <v>5.3351</v>
       </c>
       <c r="U8" t="n">
-        <v>3.4914</v>
+        <v>0.472</v>
       </c>
       <c r="V8" t="n">
-        <v>0.153</v>
+        <v>4.6566</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.7325</v>
+        <v>0.7237</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.4438</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y8" t="n">
-        <v>5.263</v>
+        <v>-11.2602</v>
       </c>
       <c r="Z8" t="n">
-        <v>13.7818</v>
+        <v>-6.9852</v>
       </c>
       <c r="AA8" t="n">
-        <v>-3.45</v>
+        <v>-0.4174</v>
       </c>
       <c r="AB8" t="n">
-        <v>-0.4414</v>
+        <v>-4.4785</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.4824</v>
+        <v>-0.9342</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>111.1471</v>
+        <v>125.038</v>
       </c>
       <c r="C9" t="n">
-        <v>118.1026</v>
+        <v>127.4564</v>
       </c>
       <c r="D9" t="n">
-        <v>109.6581</v>
+        <v>121.5203</v>
       </c>
       <c r="E9" t="n">
-        <v>117.2032</v>
+        <v>123.1892</v>
       </c>
       <c r="F9" t="n">
-        <v>72.3501</v>
+        <v>72.8092</v>
       </c>
       <c r="G9" t="n">
-        <v>73.0986</v>
+        <v>73.06870000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>71.5117</v>
+        <v>71.1824</v>
       </c>
       <c r="I9" t="n">
-        <v>72.2303</v>
+        <v>72.02070000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>48.9484</v>
+        <v>43.0126</v>
       </c>
       <c r="K9" t="n">
-        <v>49.5904</v>
+        <v>44.2768</v>
       </c>
       <c r="L9" t="n">
-        <v>45.5311</v>
+        <v>41.9854</v>
       </c>
       <c r="M9" t="n">
-        <v>45.7681</v>
+        <v>43.536</v>
       </c>
       <c r="N9" t="n">
-        <v>37.5861</v>
+        <v>37.3593</v>
       </c>
       <c r="O9" t="n">
-        <v>38.0396</v>
+        <v>38.1974</v>
       </c>
       <c r="P9" t="n">
-        <v>37.1917</v>
+        <v>37.2213</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.6452</v>
+        <v>37.7734</v>
       </c>
       <c r="R9" t="n">
-        <v>9.874499999999999</v>
+        <v>5.1074</v>
       </c>
       <c r="S9" t="n">
-        <v>10.7356</v>
+        <v>15.9097</v>
       </c>
       <c r="T9" t="n">
-        <v>5.3351</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U9" t="n">
-        <v>0.472</v>
+        <v>-0.2902</v>
       </c>
       <c r="V9" t="n">
-        <v>4.6566</v>
+        <v>3.6781</v>
       </c>
       <c r="W9" t="n">
-        <v>0.7237</v>
+        <v>0.3337</v>
       </c>
       <c r="X9" t="n">
-        <v>-10.1938</v>
+        <v>-4.877</v>
       </c>
       <c r="Y9" t="n">
-        <v>-11.2602</v>
+        <v>-14.9528</v>
       </c>
       <c r="Z9" t="n">
-        <v>-6.9852</v>
+        <v>-10.0776</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.4174</v>
+        <v>0.3405</v>
       </c>
       <c r="AB9" t="n">
-        <v>-4.4785</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC9" t="n">
-        <v>-0.9342</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>125.038</v>
+        <v>121.1606</v>
       </c>
       <c r="C10" t="n">
-        <v>127.4564</v>
+        <v>128.3958</v>
       </c>
       <c r="D10" t="n">
-        <v>121.5203</v>
+        <v>121.1606</v>
       </c>
       <c r="E10" t="n">
-        <v>123.1892</v>
+        <v>125.7875</v>
       </c>
       <c r="F10" t="n">
-        <v>72.8092</v>
+        <v>71.4119</v>
       </c>
       <c r="G10" t="n">
-        <v>73.06870000000001</v>
+        <v>72.41</v>
       </c>
       <c r="H10" t="n">
-        <v>71.1824</v>
+        <v>70.7033</v>
       </c>
       <c r="I10" t="n">
-        <v>72.02070000000001</v>
+        <v>71.4119</v>
       </c>
       <c r="J10" t="n">
-        <v>43.0126</v>
+        <v>44.2471</v>
       </c>
       <c r="K10" t="n">
-        <v>44.2768</v>
+        <v>44.2669</v>
       </c>
       <c r="L10" t="n">
-        <v>41.9854</v>
+        <v>41.7977</v>
       </c>
       <c r="M10" t="n">
-        <v>43.536</v>
+        <v>42.7064</v>
       </c>
       <c r="N10" t="n">
-        <v>37.3593</v>
+        <v>38.0889</v>
       </c>
       <c r="O10" t="n">
-        <v>38.1974</v>
+        <v>38.4636</v>
       </c>
       <c r="P10" t="n">
-        <v>37.2213</v>
+        <v>37.5664</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.7734</v>
+        <v>38.0988</v>
       </c>
       <c r="R10" t="n">
-        <v>5.1074</v>
+        <v>2.1092</v>
       </c>
       <c r="S10" t="n">
-        <v>15.9097</v>
+        <v>17.922</v>
       </c>
       <c r="T10" t="n">
-        <v>9.291600000000001</v>
+        <v>18.8462</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.2902</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>3.6781</v>
+        <v>-0.6664</v>
       </c>
       <c r="W10" t="n">
-        <v>0.3337</v>
+        <v>3.4708</v>
       </c>
       <c r="X10" t="n">
-        <v>-4.877</v>
+        <v>-1.9055</v>
       </c>
       <c r="Y10" t="n">
-        <v>-14.9528</v>
+        <v>-16.2015</v>
       </c>
       <c r="Z10" t="n">
-        <v>-10.0776</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.3405</v>
+        <v>0.8615</v>
       </c>
       <c r="AB10" t="n">
-        <v>-3.5256</v>
+        <v>0.7825</v>
       </c>
       <c r="AC10" t="n">
-        <v>-0.5193</v>
+        <v>-3.3276</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>121.1606</v>
+        <v>116.2738</v>
       </c>
       <c r="C11" t="n">
-        <v>128.3958</v>
+        <v>119.2418</v>
       </c>
       <c r="D11" t="n">
-        <v>121.1606</v>
+        <v>113.4756</v>
       </c>
       <c r="E11" t="n">
-        <v>125.7875</v>
+        <v>115.6842</v>
       </c>
       <c r="F11" t="n">
-        <v>71.4119</v>
+        <v>68.767</v>
       </c>
       <c r="G11" t="n">
-        <v>72.41</v>
+        <v>70.0945</v>
       </c>
       <c r="H11" t="n">
-        <v>70.7033</v>
+        <v>68.5474</v>
       </c>
       <c r="I11" t="n">
-        <v>71.4119</v>
+        <v>69.07640000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>44.2471</v>
+        <v>45.9459</v>
       </c>
       <c r="K11" t="n">
-        <v>44.2669</v>
+        <v>46.9039</v>
       </c>
       <c r="L11" t="n">
-        <v>41.7977</v>
+        <v>44.9385</v>
       </c>
       <c r="M11" t="n">
-        <v>42.7064</v>
+        <v>46.1632</v>
       </c>
       <c r="N11" t="n">
-        <v>38.0889</v>
+        <v>39.5186</v>
       </c>
       <c r="O11" t="n">
-        <v>38.4636</v>
+        <v>39.6271</v>
       </c>
       <c r="P11" t="n">
-        <v>37.5664</v>
+        <v>38.7988</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.0988</v>
+        <v>39.3411</v>
       </c>
       <c r="R11" t="n">
-        <v>2.1092</v>
+        <v>-8.032</v>
       </c>
       <c r="S11" t="n">
-        <v>17.922</v>
+        <v>-1.296</v>
       </c>
       <c r="T11" t="n">
-        <v>18.8462</v>
+        <v>8.8482</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2705</v>
       </c>
       <c r="V11" t="n">
-        <v>-0.6664</v>
+        <v>-4.3665</v>
       </c>
       <c r="W11" t="n">
-        <v>3.4708</v>
+        <v>-0.5604</v>
       </c>
       <c r="X11" t="n">
-        <v>-1.9055</v>
+        <v>8.0943</v>
       </c>
       <c r="Y11" t="n">
-        <v>-16.2015</v>
+        <v>0.8633</v>
       </c>
       <c r="Z11" t="n">
-        <v>-17.1965</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.8615</v>
+        <v>3.2607</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.7825</v>
+        <v>4.505</v>
       </c>
       <c r="AC11" t="n">
-        <v>-3.3276</v>
+        <v>0.4784</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>116.2738</v>
+        <v>120.6309</v>
       </c>
       <c r="C12" t="n">
-        <v>119.2418</v>
+        <v>124.4184</v>
       </c>
       <c r="D12" t="n">
-        <v>113.4756</v>
+        <v>117.7928</v>
       </c>
       <c r="E12" t="n">
-        <v>115.6842</v>
+        <v>121.7402</v>
       </c>
       <c r="F12" t="n">
-        <v>68.767</v>
+        <v>71.0526</v>
       </c>
       <c r="G12" t="n">
-        <v>70.0945</v>
+        <v>71.6215</v>
       </c>
       <c r="H12" t="n">
-        <v>68.5474</v>
+        <v>70.47369999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>69.07640000000001</v>
+        <v>70.843</v>
       </c>
       <c r="J12" t="n">
-        <v>45.9459</v>
+        <v>44.1385</v>
       </c>
       <c r="K12" t="n">
-        <v>46.9039</v>
+        <v>45.2545</v>
       </c>
       <c r="L12" t="n">
-        <v>44.9385</v>
+        <v>42.5879</v>
       </c>
       <c r="M12" t="n">
-        <v>46.1632</v>
+        <v>43.5953</v>
       </c>
       <c r="N12" t="n">
-        <v>39.5186</v>
+        <v>38.227</v>
       </c>
       <c r="O12" t="n">
-        <v>39.6271</v>
+        <v>38.5523</v>
       </c>
       <c r="P12" t="n">
-        <v>38.7988</v>
+        <v>37.8819</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.3411</v>
+        <v>38.3256</v>
       </c>
       <c r="R12" t="n">
-        <v>-8.032</v>
+        <v>5.2349</v>
       </c>
       <c r="S12" t="n">
-        <v>-1.296</v>
+        <v>-1.1762</v>
       </c>
       <c r="T12" t="n">
-        <v>8.8482</v>
+        <v>14.1278</v>
       </c>
       <c r="U12" t="n">
-        <v>-3.2705</v>
+        <v>2.5575</v>
       </c>
       <c r="V12" t="n">
-        <v>-4.3665</v>
+        <v>-1.6352</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.5604</v>
+        <v>-1.4578</v>
       </c>
       <c r="X12" t="n">
-        <v>8.0943</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.8633</v>
+        <v>0.1362</v>
       </c>
       <c r="Z12" t="n">
-        <v>-9.820600000000001</v>
+        <v>-14.4573</v>
       </c>
       <c r="AA12" t="n">
-        <v>3.2607</v>
+        <v>-2.5813</v>
       </c>
       <c r="AB12" t="n">
-        <v>4.505</v>
+        <v>1.4619</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.4784</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>120.6309</v>
+        <v>101.4635</v>
       </c>
       <c r="C13" t="n">
-        <v>124.4184</v>
+        <v>105.3209</v>
       </c>
       <c r="D13" t="n">
-        <v>117.7928</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>121.7402</v>
+        <v>101.0637</v>
       </c>
       <c r="F13" t="n">
-        <v>71.0526</v>
+        <v>67.3997</v>
       </c>
       <c r="G13" t="n">
-        <v>71.6215</v>
+        <v>70.25409999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>70.47369999999999</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>70.843</v>
+        <v>69.13630000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>44.1385</v>
+        <v>50.9731</v>
       </c>
       <c r="K13" t="n">
-        <v>45.2545</v>
+        <v>51.5756</v>
       </c>
       <c r="L13" t="n">
-        <v>42.5879</v>
+        <v>49.5904</v>
       </c>
       <c r="M13" t="n">
-        <v>43.5953</v>
+        <v>51.0916</v>
       </c>
       <c r="N13" t="n">
-        <v>38.227</v>
+        <v>40.2088</v>
       </c>
       <c r="O13" t="n">
-        <v>38.5523</v>
+        <v>40.3074</v>
       </c>
       <c r="P13" t="n">
-        <v>37.8819</v>
+        <v>38.6608</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.3256</v>
+        <v>39.2721</v>
       </c>
       <c r="R13" t="n">
-        <v>5.2349</v>
+        <v>-16.9841</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.1762</v>
+        <v>-19.6552</v>
       </c>
       <c r="T13" t="n">
-        <v>14.1278</v>
+        <v>-13.7705</v>
       </c>
       <c r="U13" t="n">
-        <v>2.5575</v>
+        <v>-2.4091</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.6352</v>
+        <v>-3.1866</v>
       </c>
       <c r="W13" t="n">
-        <v>-1.4578</v>
+        <v>-4.2835</v>
       </c>
       <c r="X13" t="n">
-        <v>-5.5627</v>
+        <v>17.1952</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.1362</v>
+        <v>19.6345</v>
       </c>
       <c r="Z13" t="n">
-        <v>-14.4573</v>
+        <v>11.6315</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.5813</v>
+        <v>2.4696</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.4619</v>
+        <v>3.0796</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.3824</v>
+        <v>4.3217</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>101.4635</v>
+        <v>104.4815</v>
       </c>
       <c r="C14" t="n">
-        <v>105.3209</v>
+        <v>105.8706</v>
       </c>
       <c r="D14" t="n">
-        <v>99.80459999999999</v>
+        <v>100.8938</v>
       </c>
       <c r="E14" t="n">
-        <v>101.0637</v>
+        <v>102.253</v>
       </c>
       <c r="F14" t="n">
-        <v>67.3997</v>
+        <v>68.9966</v>
       </c>
       <c r="G14" t="n">
-        <v>70.25409999999999</v>
+        <v>69.1962</v>
       </c>
       <c r="H14" t="n">
-        <v>67.20999999999999</v>
+        <v>67.4795</v>
       </c>
       <c r="I14" t="n">
-        <v>69.13630000000001</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>50.9731</v>
+        <v>49.2546</v>
       </c>
       <c r="K14" t="n">
-        <v>51.5756</v>
+        <v>51.1607</v>
       </c>
       <c r="L14" t="n">
-        <v>49.5904</v>
+        <v>48.6521</v>
       </c>
       <c r="M14" t="n">
-        <v>51.0916</v>
+        <v>50.4694</v>
       </c>
       <c r="N14" t="n">
+        <v>39.351</v>
+      </c>
+      <c r="O14" t="n">
         <v>40.2088</v>
       </c>
-      <c r="O14" t="n">
-        <v>40.3074</v>
-      </c>
       <c r="P14" t="n">
-        <v>38.6608</v>
+        <v>39.2327</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.2721</v>
+        <v>40.0511</v>
       </c>
       <c r="R14" t="n">
-        <v>-16.9841</v>
+        <v>1.1768</v>
       </c>
       <c r="S14" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="T14" t="n">
-        <v>-13.7705</v>
+        <v>-16.9952</v>
       </c>
       <c r="U14" t="n">
-        <v>-2.4091</v>
+        <v>-1.9777</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.1866</v>
+        <v>-1.8927</v>
       </c>
       <c r="W14" t="n">
-        <v>-4.2835</v>
+        <v>-5.9034</v>
       </c>
       <c r="X14" t="n">
-        <v>17.1952</v>
+        <v>-1.2178</v>
       </c>
       <c r="Y14" t="n">
-        <v>19.6345</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z14" t="n">
-        <v>11.6315</v>
+        <v>15.9257</v>
       </c>
       <c r="AA14" t="n">
-        <v>2.4696</v>
+        <v>1.9836</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.0796</v>
+        <v>1.8047</v>
       </c>
       <c r="AC14" t="n">
-        <v>4.3217</v>
+        <v>6.0299</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>104.4815</v>
+        <v>107.3696</v>
       </c>
       <c r="C15" t="n">
-        <v>105.8706</v>
+        <v>109.2484</v>
       </c>
       <c r="D15" t="n">
-        <v>100.8938</v>
+        <v>100.9938</v>
       </c>
       <c r="E15" t="n">
-        <v>102.253</v>
+        <v>103.9019</v>
       </c>
       <c r="F15" t="n">
-        <v>68.9966</v>
+        <v>68.7171</v>
       </c>
       <c r="G15" t="n">
-        <v>69.1962</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>67.4795</v>
+        <v>66.4216</v>
       </c>
       <c r="I15" t="n">
-        <v>67.76900000000001</v>
+        <v>67.7989</v>
       </c>
       <c r="J15" t="n">
-        <v>49.2546</v>
+        <v>47.9509</v>
       </c>
       <c r="K15" t="n">
-        <v>51.1607</v>
+        <v>51.1015</v>
       </c>
       <c r="L15" t="n">
-        <v>48.6521</v>
+        <v>46.9829</v>
       </c>
       <c r="M15" t="n">
-        <v>50.4694</v>
+        <v>49.4916</v>
       </c>
       <c r="N15" t="n">
-        <v>39.351</v>
+        <v>39.4989</v>
       </c>
       <c r="O15" t="n">
-        <v>40.2088</v>
+        <v>40.8596</v>
       </c>
       <c r="P15" t="n">
-        <v>39.2327</v>
+        <v>38.8186</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.0511</v>
+        <v>40.0412</v>
       </c>
       <c r="R15" t="n">
-        <v>1.1768</v>
+        <v>1.6126</v>
       </c>
       <c r="S15" t="n">
-        <v>-11.6102</v>
+        <v>-14.6528</v>
       </c>
       <c r="T15" t="n">
-        <v>-16.9952</v>
+        <v>-17.3989</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.9777</v>
+        <v>0.0441</v>
       </c>
       <c r="V15" t="n">
-        <v>-1.8927</v>
+        <v>-4.297</v>
       </c>
       <c r="W15" t="n">
-        <v>-5.9034</v>
+        <v>-5.0594</v>
       </c>
       <c r="X15" t="n">
-        <v>-1.2178</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y15" t="n">
-        <v>9.328200000000001</v>
+        <v>13.5251</v>
       </c>
       <c r="Z15" t="n">
-        <v>15.9257</v>
+        <v>15.888</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.9836</v>
+        <v>-0.0247</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.8047</v>
+        <v>4.4764</v>
       </c>
       <c r="AC15" t="n">
-        <v>6.0299</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>107.3696</v>
+        <v>113.2557</v>
       </c>
       <c r="C16" t="n">
-        <v>109.2484</v>
+        <v>115.4043</v>
       </c>
       <c r="D16" t="n">
-        <v>100.9938</v>
+        <v>111.9366</v>
       </c>
       <c r="E16" t="n">
-        <v>103.9019</v>
+        <v>114.7448</v>
       </c>
       <c r="F16" t="n">
-        <v>68.7171</v>
+        <v>70.9927</v>
       </c>
       <c r="G16" t="n">
-        <v>69.83499999999999</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>66.4216</v>
+        <v>70.2342</v>
       </c>
       <c r="I16" t="n">
-        <v>67.7989</v>
+        <v>71.2422</v>
       </c>
       <c r="J16" t="n">
-        <v>47.9509</v>
+        <v>45.1558</v>
       </c>
       <c r="K16" t="n">
-        <v>51.1015</v>
+        <v>45.7681</v>
       </c>
       <c r="L16" t="n">
-        <v>46.9829</v>
+        <v>44.1187</v>
       </c>
       <c r="M16" t="n">
-        <v>49.4916</v>
+        <v>44.4348</v>
       </c>
       <c r="N16" t="n">
-        <v>39.4989</v>
+        <v>38.1481</v>
       </c>
       <c r="O16" t="n">
-        <v>40.8596</v>
+        <v>38.5918</v>
       </c>
       <c r="P16" t="n">
-        <v>38.8186</v>
+        <v>37.7931</v>
       </c>
       <c r="Q16" t="n">
-        <v>40.0412</v>
+        <v>37.9903</v>
       </c>
       <c r="R16" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="S16" t="n">
-        <v>-14.6528</v>
+        <v>13.5371</v>
       </c>
       <c r="T16" t="n">
-        <v>-17.3989</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U16" t="n">
-        <v>0.0441</v>
+        <v>5.0787</v>
       </c>
       <c r="V16" t="n">
-        <v>-4.297</v>
+        <v>3.046</v>
       </c>
       <c r="W16" t="n">
-        <v>-5.0594</v>
+        <v>3.1354</v>
       </c>
       <c r="X16" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y16" t="n">
-        <v>13.5251</v>
+        <v>-13.0291</v>
       </c>
       <c r="Z16" t="n">
-        <v>15.888</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.0247</v>
+        <v>-5.122</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.4764</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC16" t="n">
-        <v>5.0983</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>113.2557</v>
+        <v>116.9533</v>
       </c>
       <c r="C17" t="n">
-        <v>115.4043</v>
+        <v>123.8188</v>
       </c>
       <c r="D17" t="n">
-        <v>111.9366</v>
+        <v>116.6035</v>
       </c>
       <c r="E17" t="n">
-        <v>114.7448</v>
+        <v>123.589</v>
       </c>
       <c r="F17" t="n">
-        <v>70.9927</v>
+        <v>71.7812</v>
       </c>
       <c r="G17" t="n">
-        <v>71.58159999999999</v>
+        <v>72.6395</v>
       </c>
       <c r="H17" t="n">
-        <v>70.2342</v>
+        <v>70.6733</v>
       </c>
       <c r="I17" t="n">
-        <v>71.2422</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>45.1558</v>
+        <v>43.5656</v>
       </c>
       <c r="K17" t="n">
-        <v>45.7681</v>
+        <v>43.7138</v>
       </c>
       <c r="L17" t="n">
-        <v>44.1187</v>
+        <v>40.9582</v>
       </c>
       <c r="M17" t="n">
-        <v>44.4348</v>
+        <v>40.978</v>
       </c>
       <c r="N17" t="n">
-        <v>38.1481</v>
+        <v>37.7241</v>
       </c>
       <c r="O17" t="n">
-        <v>38.5918</v>
+        <v>38.3256</v>
       </c>
       <c r="P17" t="n">
-        <v>37.7931</v>
+        <v>37.2706</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.9903</v>
+        <v>37.3396</v>
       </c>
       <c r="R17" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="S17" t="n">
-        <v>13.5371</v>
+        <v>20.8659</v>
       </c>
       <c r="T17" t="n">
-        <v>-0.8120000000000001</v>
+        <v>1.5186</v>
       </c>
       <c r="U17" t="n">
-        <v>5.0787</v>
+        <v>1.7652</v>
       </c>
       <c r="V17" t="n">
-        <v>3.046</v>
+        <v>6.9808</v>
       </c>
       <c r="W17" t="n">
-        <v>3.1354</v>
+        <v>2.3387</v>
       </c>
       <c r="X17" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y17" t="n">
-        <v>-13.0291</v>
+        <v>-18.8062</v>
       </c>
       <c r="Z17" t="n">
-        <v>-3.7441</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA17" t="n">
-        <v>-5.122</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB17" t="n">
-        <v>-3.2639</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC17" t="n">
-        <v>-3.4336</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>116.9533</v>
+        <v>131.9835</v>
       </c>
       <c r="C18" t="n">
-        <v>123.8188</v>
+        <v>143.9056</v>
       </c>
       <c r="D18" t="n">
-        <v>116.6035</v>
+        <v>129.5351</v>
       </c>
       <c r="E18" t="n">
-        <v>123.589</v>
+        <v>141.837</v>
       </c>
       <c r="F18" t="n">
-        <v>71.7812</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>72.6395</v>
+        <v>79.3366</v>
       </c>
       <c r="H18" t="n">
-        <v>70.6733</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>72.49979999999999</v>
+        <v>78.7577</v>
       </c>
       <c r="J18" t="n">
-        <v>43.5656</v>
+        <v>38.2718</v>
       </c>
       <c r="K18" t="n">
-        <v>43.7138</v>
+        <v>39.0224</v>
       </c>
       <c r="L18" t="n">
-        <v>40.9582</v>
+        <v>34.252</v>
       </c>
       <c r="M18" t="n">
-        <v>40.978</v>
+        <v>34.894</v>
       </c>
       <c r="N18" t="n">
-        <v>37.7241</v>
+        <v>36.2155</v>
       </c>
       <c r="O18" t="n">
-        <v>38.3256</v>
+        <v>36.2254</v>
       </c>
       <c r="P18" t="n">
-        <v>37.2706</v>
+        <v>33.8294</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.3396</v>
+        <v>34.1154</v>
       </c>
       <c r="R18" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="S18" t="n">
-        <v>20.8659</v>
+        <v>36.5105</v>
       </c>
       <c r="T18" t="n">
-        <v>1.5186</v>
+        <v>40.3442</v>
       </c>
       <c r="U18" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V18" t="n">
-        <v>6.9808</v>
+        <v>16.1637</v>
       </c>
       <c r="W18" t="n">
-        <v>2.3387</v>
+        <v>13.9166</v>
       </c>
       <c r="X18" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="Y18" t="n">
-        <v>-18.8062</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z18" t="n">
-        <v>-6.0036</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.7128</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.7701</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC18" t="n">
-        <v>-2.5727</v>
+        <v>-13.1307</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C19" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D19" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E19" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F19" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>79.3366</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>78.7577</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K19" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L19" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M19" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N19" t="n">
-        <v>36.2155</v>
+        <v>34.1745</v>
       </c>
       <c r="O19" t="n">
-        <v>36.2254</v>
+        <v>34.1745</v>
       </c>
       <c r="P19" t="n">
-        <v>33.8294</v>
+        <v>33.1688</v>
       </c>
       <c r="Q19" t="n">
-        <v>34.1154</v>
+        <v>33.297</v>
       </c>
       <c r="R19" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S19" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="T19" t="n">
-        <v>40.3442</v>
+        <v>48.602</v>
       </c>
       <c r="U19" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V19" t="n">
-        <v>16.1637</v>
+        <v>13.2391</v>
       </c>
       <c r="W19" t="n">
-        <v>13.9166</v>
+        <v>19.0426</v>
       </c>
       <c r="X19" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y19" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z19" t="n">
-        <v>-31.7031</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA19" t="n">
-        <v>-8.6348</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB19" t="n">
-        <v>-14.7993</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC19" t="n">
-        <v>-13.1307</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C20" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D20" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E20" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F20" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G20" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I20" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J20" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K20" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L20" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M20" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N20" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O20" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P20" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q20" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
       <c r="R20" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="S20" t="n">
-        <v>32.4243</v>
+        <v>18.3358</v>
       </c>
       <c r="T20" t="n">
-        <v>48.602</v>
+        <v>40.7578</v>
       </c>
       <c r="U20" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="V20" t="n">
-        <v>13.2391</v>
+        <v>8.4969</v>
       </c>
       <c r="W20" t="n">
-        <v>19.0426</v>
+        <v>16.0196</v>
       </c>
       <c r="X20" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="Y20" t="n">
-        <v>-27.0392</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z20" t="n">
-        <v>-35.7631</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA20" t="n">
-        <v>-2.3989</v>
+        <v>2.5318</v>
       </c>
       <c r="AB20" t="n">
-        <v>-12.3539</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC20" t="n">
-        <v>-16.8637</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C21" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D21" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E21" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F21" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G21" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I21" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J21" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K21" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L21" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M21" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N21" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O21" t="n">
         <v>35.06</v>
       </c>
-      <c r="L21" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M21" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N21" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O21" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P21" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q21" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R21" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="S21" t="n">
-        <v>18.3358</v>
+        <v>3.1677</v>
       </c>
       <c r="T21" t="n">
-        <v>40.7578</v>
+        <v>27.5265</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="V21" t="n">
-        <v>8.4969</v>
+        <v>-0.2256</v>
       </c>
       <c r="W21" t="n">
-        <v>16.0196</v>
+        <v>10.2998</v>
       </c>
       <c r="X21" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y21" t="n">
-        <v>-17.8584</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z21" t="n">
-        <v>-31.9885</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA21" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
       <c r="AB21" t="n">
-        <v>-8.568899999999999</v>
+        <v>0.1894</v>
       </c>
       <c r="AC21" t="n">
-        <v>-14.7378</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-09-29 01:30
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1720 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>123.3191</v>
+        <v>112.3363</v>
       </c>
       <c r="C2" t="n">
-        <v>124.7982</v>
+        <v>114.9746</v>
       </c>
       <c r="D2" t="n">
-        <v>117.6129</v>
+        <v>110.2577</v>
       </c>
       <c r="E2" t="n">
-        <v>122.9694</v>
+        <v>112.7161</v>
       </c>
       <c r="F2" t="n">
-        <v>71.9509</v>
+        <v>71.3021</v>
       </c>
       <c r="G2" t="n">
-        <v>73.2384</v>
+        <v>72.0107</v>
       </c>
       <c r="H2" t="n">
-        <v>71.2422</v>
+        <v>70.6833</v>
       </c>
       <c r="I2" t="n">
-        <v>73.1585</v>
+        <v>71.7812</v>
       </c>
       <c r="J2" t="n">
-        <v>44.8595</v>
+        <v>48.662</v>
       </c>
       <c r="K2" t="n">
-        <v>47.1212</v>
+        <v>49.62</v>
       </c>
       <c r="L2" t="n">
-        <v>44.1582</v>
+        <v>47.4965</v>
       </c>
       <c r="M2" t="n">
-        <v>44.7903</v>
+        <v>48.4151</v>
       </c>
       <c r="N2" t="n">
-        <v>37.9213</v>
+        <v>38.227</v>
       </c>
       <c r="O2" t="n">
-        <v>38.3157</v>
+        <v>38.5425</v>
       </c>
       <c r="P2" t="n">
-        <v>37.2015</v>
+        <v>37.8326</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.2508</v>
+        <v>37.9706</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>119.8414</v>
+        <v>106.2903</v>
       </c>
       <c r="C3" t="n">
-        <v>121.1206</v>
+        <v>108.5688</v>
       </c>
       <c r="D3" t="n">
-        <v>110.1378</v>
+        <v>102.243</v>
       </c>
       <c r="E3" t="n">
-        <v>111.267</v>
+        <v>105.8406</v>
       </c>
       <c r="F3" t="n">
-        <v>72.7094</v>
+        <v>68.9367</v>
       </c>
       <c r="G3" t="n">
-        <v>74.0368</v>
+        <v>70.41379999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>71.2921</v>
+        <v>68.1183</v>
       </c>
       <c r="I3" t="n">
-        <v>71.71129999999999</v>
+        <v>69.01649999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>46.0348</v>
+        <v>51.2398</v>
       </c>
       <c r="K3" t="n">
-        <v>49.6101</v>
+        <v>53.0274</v>
       </c>
       <c r="L3" t="n">
-        <v>45.5805</v>
+        <v>50.2719</v>
       </c>
       <c r="M3" t="n">
-        <v>49.2052</v>
+        <v>51.5756</v>
       </c>
       <c r="N3" t="n">
-        <v>37.4875</v>
+        <v>39.4693</v>
       </c>
       <c r="O3" t="n">
-        <v>38.2171</v>
+        <v>39.9032</v>
       </c>
       <c r="P3" t="n">
-        <v>36.8071</v>
+        <v>38.6805</v>
       </c>
       <c r="Q3" t="n">
-        <v>38.0002</v>
+        <v>39.4102</v>
       </c>
       <c r="R3" t="n">
-        <v>-9.516500000000001</v>
+        <v>-6.0998</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.9782</v>
+        <v>-3.8516</v>
       </c>
       <c r="X3" t="n">
-        <v>9.8568</v>
+        <v>6.5279</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.0118</v>
+        <v>3.7914</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>112.3363</v>
+        <v>104.4315</v>
       </c>
       <c r="C4" t="n">
-        <v>114.9746</v>
+        <v>107.9992</v>
       </c>
       <c r="D4" t="n">
-        <v>110.2577</v>
+        <v>101.2736</v>
       </c>
       <c r="E4" t="n">
-        <v>112.7161</v>
+        <v>106.2803</v>
       </c>
       <c r="F4" t="n">
-        <v>71.3021</v>
+        <v>68.8369</v>
       </c>
       <c r="G4" t="n">
-        <v>72.0107</v>
+        <v>69.6254</v>
       </c>
       <c r="H4" t="n">
-        <v>70.6833</v>
+        <v>68.258</v>
       </c>
       <c r="I4" t="n">
-        <v>71.7812</v>
+        <v>69.4657</v>
       </c>
       <c r="J4" t="n">
-        <v>48.662</v>
+        <v>52.1484</v>
       </c>
       <c r="K4" t="n">
-        <v>49.62</v>
+        <v>53.7188</v>
       </c>
       <c r="L4" t="n">
-        <v>47.4965</v>
+        <v>50.42</v>
       </c>
       <c r="M4" t="n">
-        <v>48.4151</v>
+        <v>51.1904</v>
       </c>
       <c r="N4" t="n">
-        <v>38.227</v>
+        <v>39.5285</v>
       </c>
       <c r="O4" t="n">
-        <v>38.5425</v>
+        <v>39.8637</v>
       </c>
       <c r="P4" t="n">
-        <v>37.8326</v>
+        <v>39.0749</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.9706</v>
+        <v>39.1538</v>
       </c>
       <c r="R4" t="n">
-        <v>1.3024</v>
+        <v>0.4154</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0975</v>
+        <v>0.6509</v>
       </c>
       <c r="X4" t="n">
-        <v>-1.6057</v>
+        <v>-0.7469</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.0779</v>
+        <v>-0.6506</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>106.2903</v>
+        <v>102.9325</v>
       </c>
       <c r="C5" t="n">
-        <v>108.5688</v>
+        <v>107.4196</v>
       </c>
       <c r="D5" t="n">
-        <v>102.243</v>
+        <v>98.55540000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>105.8406</v>
+        <v>106.6701</v>
       </c>
       <c r="F5" t="n">
-        <v>68.9367</v>
+        <v>69.9248</v>
       </c>
       <c r="G5" t="n">
-        <v>70.41379999999999</v>
+        <v>72.28019999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>68.1183</v>
+        <v>69.57550000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>69.01649999999999</v>
+        <v>71.89100000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>51.2398</v>
+        <v>52.8398</v>
       </c>
       <c r="K5" t="n">
-        <v>53.0274</v>
+        <v>55.0027</v>
       </c>
       <c r="L5" t="n">
-        <v>50.2719</v>
+        <v>50.6472</v>
       </c>
       <c r="M5" t="n">
-        <v>51.5756</v>
+        <v>50.9632</v>
       </c>
       <c r="N5" t="n">
-        <v>39.4693</v>
+        <v>38.9369</v>
       </c>
       <c r="O5" t="n">
-        <v>39.9032</v>
+        <v>39.1242</v>
       </c>
       <c r="P5" t="n">
-        <v>38.6805</v>
+        <v>37.5861</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.4102</v>
+        <v>37.803</v>
       </c>
       <c r="R5" t="n">
-        <v>-6.0998</v>
+        <v>0.3668</v>
       </c>
       <c r="S5" t="n">
-        <v>-13.9293</v>
+        <v>-5.3639</v>
       </c>
       <c r="U5" t="n">
-        <v>-3.8516</v>
+        <v>3.4914</v>
       </c>
       <c r="V5" t="n">
-        <v>-5.6617</v>
+        <v>0.153</v>
       </c>
       <c r="X5" t="n">
-        <v>6.5279</v>
+        <v>-0.4438</v>
       </c>
       <c r="Y5" t="n">
-        <v>15.149</v>
+        <v>5.263</v>
       </c>
       <c r="AA5" t="n">
-        <v>3.7914</v>
+        <v>-3.45</v>
       </c>
       <c r="AB5" t="n">
-        <v>5.7969</v>
+        <v>-0.4414</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>104.4315</v>
+        <v>111.1471</v>
       </c>
       <c r="C6" t="n">
-        <v>107.9992</v>
+        <v>118.1026</v>
       </c>
       <c r="D6" t="n">
-        <v>101.2736</v>
+        <v>109.6581</v>
       </c>
       <c r="E6" t="n">
-        <v>106.2803</v>
+        <v>117.2032</v>
       </c>
       <c r="F6" t="n">
-        <v>68.8369</v>
+        <v>72.3501</v>
       </c>
       <c r="G6" t="n">
-        <v>69.6254</v>
+        <v>73.0986</v>
       </c>
       <c r="H6" t="n">
-        <v>68.258</v>
+        <v>71.5117</v>
       </c>
       <c r="I6" t="n">
-        <v>69.4657</v>
+        <v>72.2303</v>
       </c>
       <c r="J6" t="n">
-        <v>52.1484</v>
+        <v>48.9484</v>
       </c>
       <c r="K6" t="n">
-        <v>53.7188</v>
+        <v>49.5904</v>
       </c>
       <c r="L6" t="n">
-        <v>50.42</v>
+        <v>45.5311</v>
       </c>
       <c r="M6" t="n">
-        <v>51.1904</v>
+        <v>45.7681</v>
       </c>
       <c r="N6" t="n">
-        <v>39.5285</v>
+        <v>37.5861</v>
       </c>
       <c r="O6" t="n">
-        <v>39.8637</v>
+        <v>38.0396</v>
       </c>
       <c r="P6" t="n">
-        <v>39.0749</v>
+        <v>37.1917</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.1538</v>
+        <v>37.6452</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4154</v>
+        <v>9.874499999999999</v>
       </c>
       <c r="S6" t="n">
-        <v>-4.4817</v>
+        <v>10.7356</v>
       </c>
       <c r="U6" t="n">
-        <v>0.6509</v>
+        <v>0.472</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.1314</v>
+        <v>4.6566</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.7469</v>
+        <v>-10.1938</v>
       </c>
       <c r="Y6" t="n">
-        <v>4.0345</v>
+        <v>-11.2602</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.6506</v>
+        <v>-0.4174</v>
       </c>
       <c r="AB6" t="n">
-        <v>3.0358</v>
+        <v>-4.4785</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>102.9325</v>
+        <v>125.038</v>
       </c>
       <c r="C7" t="n">
-        <v>107.4196</v>
+        <v>127.4564</v>
       </c>
       <c r="D7" t="n">
-        <v>98.55540000000001</v>
+        <v>121.5203</v>
       </c>
       <c r="E7" t="n">
-        <v>106.6701</v>
+        <v>123.1892</v>
       </c>
       <c r="F7" t="n">
-        <v>69.9248</v>
+        <v>72.8092</v>
       </c>
       <c r="G7" t="n">
-        <v>72.28019999999999</v>
+        <v>73.06870000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>69.57550000000001</v>
+        <v>71.1824</v>
       </c>
       <c r="I7" t="n">
-        <v>71.89100000000001</v>
+        <v>72.02070000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>52.8398</v>
+        <v>43.0126</v>
       </c>
       <c r="K7" t="n">
-        <v>55.0027</v>
+        <v>44.2768</v>
       </c>
       <c r="L7" t="n">
-        <v>50.6472</v>
+        <v>41.9854</v>
       </c>
       <c r="M7" t="n">
-        <v>50.9632</v>
+        <v>43.536</v>
       </c>
       <c r="N7" t="n">
-        <v>38.9369</v>
+        <v>37.3593</v>
       </c>
       <c r="O7" t="n">
-        <v>39.1242</v>
+        <v>38.1974</v>
       </c>
       <c r="P7" t="n">
-        <v>37.5861</v>
+        <v>37.2213</v>
       </c>
       <c r="Q7" t="n">
-        <v>37.803</v>
+        <v>37.7734</v>
       </c>
       <c r="R7" t="n">
-        <v>0.3668</v>
+        <v>5.1074</v>
       </c>
       <c r="S7" t="n">
-        <v>-5.3639</v>
+        <v>15.9097</v>
       </c>
       <c r="T7" t="n">
-        <v>-13.2548</v>
+        <v>9.291600000000001</v>
       </c>
       <c r="U7" t="n">
-        <v>3.4914</v>
+        <v>-0.2902</v>
       </c>
       <c r="V7" t="n">
-        <v>0.153</v>
+        <v>3.6781</v>
       </c>
       <c r="W7" t="n">
-        <v>-1.7325</v>
+        <v>0.3337</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.4438</v>
+        <v>-4.877</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.263</v>
+        <v>-14.9528</v>
       </c>
       <c r="Z7" t="n">
-        <v>13.7818</v>
+        <v>-10.0776</v>
       </c>
       <c r="AA7" t="n">
-        <v>-3.45</v>
+        <v>0.3405</v>
       </c>
       <c r="AB7" t="n">
-        <v>-0.4414</v>
+        <v>-3.5256</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.4824</v>
+        <v>-0.5193</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>111.1471</v>
+        <v>121.1606</v>
       </c>
       <c r="C8" t="n">
-        <v>118.1026</v>
+        <v>128.3958</v>
       </c>
       <c r="D8" t="n">
-        <v>109.6581</v>
+        <v>121.1606</v>
       </c>
       <c r="E8" t="n">
-        <v>117.2032</v>
+        <v>125.7875</v>
       </c>
       <c r="F8" t="n">
-        <v>72.3501</v>
+        <v>71.4119</v>
       </c>
       <c r="G8" t="n">
-        <v>73.0986</v>
+        <v>72.41</v>
       </c>
       <c r="H8" t="n">
-        <v>71.5117</v>
+        <v>70.7033</v>
       </c>
       <c r="I8" t="n">
-        <v>72.2303</v>
+        <v>71.4119</v>
       </c>
       <c r="J8" t="n">
-        <v>48.9484</v>
+        <v>44.2471</v>
       </c>
       <c r="K8" t="n">
-        <v>49.5904</v>
+        <v>44.2669</v>
       </c>
       <c r="L8" t="n">
-        <v>45.5311</v>
+        <v>41.7977</v>
       </c>
       <c r="M8" t="n">
-        <v>45.7681</v>
+        <v>42.7064</v>
       </c>
       <c r="N8" t="n">
-        <v>37.5861</v>
+        <v>38.0889</v>
       </c>
       <c r="O8" t="n">
-        <v>38.0396</v>
+        <v>38.4636</v>
       </c>
       <c r="P8" t="n">
-        <v>37.1917</v>
+        <v>37.5664</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.6452</v>
+        <v>38.0988</v>
       </c>
       <c r="R8" t="n">
-        <v>9.874499999999999</v>
+        <v>2.1092</v>
       </c>
       <c r="S8" t="n">
-        <v>10.7356</v>
+        <v>17.922</v>
       </c>
       <c r="T8" t="n">
-        <v>5.3351</v>
+        <v>18.8462</v>
       </c>
       <c r="U8" t="n">
-        <v>0.472</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="V8" t="n">
-        <v>4.6566</v>
+        <v>-0.6664</v>
       </c>
       <c r="W8" t="n">
-        <v>0.7237</v>
+        <v>3.4708</v>
       </c>
       <c r="X8" t="n">
-        <v>-10.1938</v>
+        <v>-1.9055</v>
       </c>
       <c r="Y8" t="n">
-        <v>-11.2602</v>
+        <v>-16.2015</v>
       </c>
       <c r="Z8" t="n">
-        <v>-6.9852</v>
+        <v>-17.1965</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.4174</v>
+        <v>0.8615</v>
       </c>
       <c r="AB8" t="n">
-        <v>-4.4785</v>
+        <v>0.7825</v>
       </c>
       <c r="AC8" t="n">
-        <v>-0.9342</v>
+        <v>-3.3276</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>125.038</v>
+        <v>116.2738</v>
       </c>
       <c r="C9" t="n">
-        <v>127.4564</v>
+        <v>119.2418</v>
       </c>
       <c r="D9" t="n">
-        <v>121.5203</v>
+        <v>113.4756</v>
       </c>
       <c r="E9" t="n">
-        <v>123.1892</v>
+        <v>115.6842</v>
       </c>
       <c r="F9" t="n">
-        <v>72.8092</v>
+        <v>68.767</v>
       </c>
       <c r="G9" t="n">
-        <v>73.06870000000001</v>
+        <v>70.0945</v>
       </c>
       <c r="H9" t="n">
-        <v>71.1824</v>
+        <v>68.5474</v>
       </c>
       <c r="I9" t="n">
-        <v>72.02070000000001</v>
+        <v>69.07640000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>43.0126</v>
+        <v>45.9459</v>
       </c>
       <c r="K9" t="n">
-        <v>44.2768</v>
+        <v>46.9039</v>
       </c>
       <c r="L9" t="n">
-        <v>41.9854</v>
+        <v>44.9385</v>
       </c>
       <c r="M9" t="n">
-        <v>43.536</v>
+        <v>46.1632</v>
       </c>
       <c r="N9" t="n">
-        <v>37.3593</v>
+        <v>39.5186</v>
       </c>
       <c r="O9" t="n">
-        <v>38.1974</v>
+        <v>39.6271</v>
       </c>
       <c r="P9" t="n">
-        <v>37.2213</v>
+        <v>38.7988</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.7734</v>
+        <v>39.3411</v>
       </c>
       <c r="R9" t="n">
-        <v>5.1074</v>
+        <v>-8.032</v>
       </c>
       <c r="S9" t="n">
-        <v>15.9097</v>
+        <v>-1.296</v>
       </c>
       <c r="T9" t="n">
-        <v>9.291600000000001</v>
+        <v>8.8482</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.2902</v>
+        <v>-3.2705</v>
       </c>
       <c r="V9" t="n">
-        <v>3.6781</v>
+        <v>-4.3665</v>
       </c>
       <c r="W9" t="n">
-        <v>0.3337</v>
+        <v>-0.5604</v>
       </c>
       <c r="X9" t="n">
-        <v>-4.877</v>
+        <v>8.0943</v>
       </c>
       <c r="Y9" t="n">
-        <v>-14.9528</v>
+        <v>0.8633</v>
       </c>
       <c r="Z9" t="n">
-        <v>-10.0776</v>
+        <v>-9.820600000000001</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.3405</v>
+        <v>3.2607</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3.5256</v>
+        <v>4.505</v>
       </c>
       <c r="AC9" t="n">
-        <v>-0.5193</v>
+        <v>0.4784</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>121.1606</v>
+        <v>120.6309</v>
       </c>
       <c r="C10" t="n">
-        <v>128.3958</v>
+        <v>124.4184</v>
       </c>
       <c r="D10" t="n">
-        <v>121.1606</v>
+        <v>117.7928</v>
       </c>
       <c r="E10" t="n">
-        <v>125.7875</v>
+        <v>121.7402</v>
       </c>
       <c r="F10" t="n">
-        <v>71.4119</v>
+        <v>71.0526</v>
       </c>
       <c r="G10" t="n">
-        <v>72.41</v>
+        <v>71.6215</v>
       </c>
       <c r="H10" t="n">
-        <v>70.7033</v>
+        <v>70.47369999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>71.4119</v>
+        <v>70.843</v>
       </c>
       <c r="J10" t="n">
-        <v>44.2471</v>
+        <v>44.1385</v>
       </c>
       <c r="K10" t="n">
-        <v>44.2669</v>
+        <v>45.2545</v>
       </c>
       <c r="L10" t="n">
-        <v>41.7977</v>
+        <v>42.5879</v>
       </c>
       <c r="M10" t="n">
-        <v>42.7064</v>
+        <v>43.5953</v>
       </c>
       <c r="N10" t="n">
-        <v>38.0889</v>
+        <v>38.227</v>
       </c>
       <c r="O10" t="n">
-        <v>38.4636</v>
+        <v>38.5523</v>
       </c>
       <c r="P10" t="n">
-        <v>37.5664</v>
+        <v>37.8819</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.0988</v>
+        <v>38.3256</v>
       </c>
       <c r="R10" t="n">
-        <v>2.1092</v>
+        <v>5.2349</v>
       </c>
       <c r="S10" t="n">
-        <v>17.922</v>
+        <v>-1.1762</v>
       </c>
       <c r="T10" t="n">
-        <v>18.8462</v>
+        <v>14.1278</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.8453000000000001</v>
+        <v>2.5575</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.6664</v>
+        <v>-1.6352</v>
       </c>
       <c r="W10" t="n">
-        <v>3.4708</v>
+        <v>-1.4578</v>
       </c>
       <c r="X10" t="n">
-        <v>-1.9055</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y10" t="n">
-        <v>-16.2015</v>
+        <v>0.1362</v>
       </c>
       <c r="Z10" t="n">
-        <v>-17.1965</v>
+        <v>-14.4573</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.8615</v>
+        <v>-2.5813</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.7825</v>
+        <v>1.4619</v>
       </c>
       <c r="AC10" t="n">
-        <v>-3.3276</v>
+        <v>1.3824</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>116.2738</v>
+        <v>101.4635</v>
       </c>
       <c r="C11" t="n">
-        <v>119.2418</v>
+        <v>105.3209</v>
       </c>
       <c r="D11" t="n">
-        <v>113.4756</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>115.6842</v>
+        <v>101.0637</v>
       </c>
       <c r="F11" t="n">
-        <v>68.767</v>
+        <v>67.3997</v>
       </c>
       <c r="G11" t="n">
-        <v>70.0945</v>
+        <v>70.25409999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>68.5474</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>69.07640000000001</v>
+        <v>69.13630000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>45.9459</v>
+        <v>50.9731</v>
       </c>
       <c r="K11" t="n">
-        <v>46.9039</v>
+        <v>51.5756</v>
       </c>
       <c r="L11" t="n">
-        <v>44.9385</v>
+        <v>49.5904</v>
       </c>
       <c r="M11" t="n">
-        <v>46.1632</v>
+        <v>51.0916</v>
       </c>
       <c r="N11" t="n">
-        <v>39.5186</v>
+        <v>40.2088</v>
       </c>
       <c r="O11" t="n">
-        <v>39.6271</v>
+        <v>40.3074</v>
       </c>
       <c r="P11" t="n">
-        <v>38.7988</v>
+        <v>38.6608</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.3411</v>
+        <v>39.2721</v>
       </c>
       <c r="R11" t="n">
-        <v>-8.032</v>
+        <v>-16.9841</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.296</v>
+        <v>-19.6552</v>
       </c>
       <c r="T11" t="n">
-        <v>8.8482</v>
+        <v>-13.7705</v>
       </c>
       <c r="U11" t="n">
-        <v>-3.2705</v>
+        <v>-2.4091</v>
       </c>
       <c r="V11" t="n">
-        <v>-4.3665</v>
+        <v>-3.1866</v>
       </c>
       <c r="W11" t="n">
-        <v>-0.5604</v>
+        <v>-4.2835</v>
       </c>
       <c r="X11" t="n">
-        <v>8.0943</v>
+        <v>17.1952</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.8633</v>
+        <v>19.6345</v>
       </c>
       <c r="Z11" t="n">
-        <v>-9.820600000000001</v>
+        <v>11.6315</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.2607</v>
+        <v>2.4696</v>
       </c>
       <c r="AB11" t="n">
-        <v>4.505</v>
+        <v>3.0796</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.4784</v>
+        <v>4.3217</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>120.6309</v>
+        <v>104.4815</v>
       </c>
       <c r="C12" t="n">
-        <v>124.4184</v>
+        <v>105.8706</v>
       </c>
       <c r="D12" t="n">
-        <v>117.7928</v>
+        <v>100.8938</v>
       </c>
       <c r="E12" t="n">
-        <v>121.7402</v>
+        <v>102.253</v>
       </c>
       <c r="F12" t="n">
-        <v>71.0526</v>
+        <v>68.9966</v>
       </c>
       <c r="G12" t="n">
-        <v>71.6215</v>
+        <v>69.1962</v>
       </c>
       <c r="H12" t="n">
-        <v>70.47369999999999</v>
+        <v>67.4795</v>
       </c>
       <c r="I12" t="n">
-        <v>70.843</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>44.1385</v>
+        <v>49.2546</v>
       </c>
       <c r="K12" t="n">
-        <v>45.2545</v>
+        <v>51.1607</v>
       </c>
       <c r="L12" t="n">
-        <v>42.5879</v>
+        <v>48.6521</v>
       </c>
       <c r="M12" t="n">
-        <v>43.5953</v>
+        <v>50.4694</v>
       </c>
       <c r="N12" t="n">
-        <v>38.227</v>
+        <v>39.351</v>
       </c>
       <c r="O12" t="n">
-        <v>38.5523</v>
+        <v>40.2088</v>
       </c>
       <c r="P12" t="n">
-        <v>37.8819</v>
+        <v>39.2327</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.3256</v>
+        <v>40.0511</v>
       </c>
       <c r="R12" t="n">
-        <v>5.2349</v>
+        <v>1.1768</v>
       </c>
       <c r="S12" t="n">
-        <v>-1.1762</v>
+        <v>-11.6102</v>
       </c>
       <c r="T12" t="n">
-        <v>14.1278</v>
+        <v>-16.9952</v>
       </c>
       <c r="U12" t="n">
-        <v>2.5575</v>
+        <v>-1.9777</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.6352</v>
+        <v>-1.8927</v>
       </c>
       <c r="W12" t="n">
-        <v>-1.4578</v>
+        <v>-5.9034</v>
       </c>
       <c r="X12" t="n">
-        <v>-5.5627</v>
+        <v>-1.2178</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.1362</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z12" t="n">
-        <v>-14.4573</v>
+        <v>15.9257</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.5813</v>
+        <v>1.9836</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.4619</v>
+        <v>1.8047</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.3824</v>
+        <v>6.0299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>101.4635</v>
+        <v>107.3696</v>
       </c>
       <c r="C13" t="n">
-        <v>105.3209</v>
+        <v>109.2484</v>
       </c>
       <c r="D13" t="n">
-        <v>99.80459999999999</v>
+        <v>100.9938</v>
       </c>
       <c r="E13" t="n">
-        <v>101.0637</v>
+        <v>103.9019</v>
       </c>
       <c r="F13" t="n">
-        <v>67.3997</v>
+        <v>68.7171</v>
       </c>
       <c r="G13" t="n">
-        <v>70.25409999999999</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>67.20999999999999</v>
+        <v>66.4216</v>
       </c>
       <c r="I13" t="n">
-        <v>69.13630000000001</v>
+        <v>67.7989</v>
       </c>
       <c r="J13" t="n">
-        <v>50.9731</v>
+        <v>47.9509</v>
       </c>
       <c r="K13" t="n">
-        <v>51.5756</v>
+        <v>51.1015</v>
       </c>
       <c r="L13" t="n">
-        <v>49.5904</v>
+        <v>46.9829</v>
       </c>
       <c r="M13" t="n">
-        <v>51.0916</v>
+        <v>49.4916</v>
       </c>
       <c r="N13" t="n">
-        <v>40.2088</v>
+        <v>39.4989</v>
       </c>
       <c r="O13" t="n">
-        <v>40.3074</v>
+        <v>40.8596</v>
       </c>
       <c r="P13" t="n">
-        <v>38.6608</v>
+        <v>38.8186</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.2721</v>
+        <v>40.0412</v>
       </c>
       <c r="R13" t="n">
-        <v>-16.9841</v>
+        <v>1.6126</v>
       </c>
       <c r="S13" t="n">
-        <v>-19.6552</v>
+        <v>-14.6528</v>
       </c>
       <c r="T13" t="n">
-        <v>-13.7705</v>
+        <v>-17.3989</v>
       </c>
       <c r="U13" t="n">
-        <v>-2.4091</v>
+        <v>0.0441</v>
       </c>
       <c r="V13" t="n">
-        <v>-3.1866</v>
+        <v>-4.297</v>
       </c>
       <c r="W13" t="n">
-        <v>-4.2835</v>
+        <v>-5.0594</v>
       </c>
       <c r="X13" t="n">
-        <v>17.1952</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y13" t="n">
-        <v>19.6345</v>
+        <v>13.5251</v>
       </c>
       <c r="Z13" t="n">
-        <v>11.6315</v>
+        <v>15.888</v>
       </c>
       <c r="AA13" t="n">
-        <v>2.4696</v>
+        <v>-0.0247</v>
       </c>
       <c r="AB13" t="n">
-        <v>3.0796</v>
+        <v>4.4764</v>
       </c>
       <c r="AC13" t="n">
-        <v>4.3217</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>104.4815</v>
+        <v>113.2557</v>
       </c>
       <c r="C14" t="n">
-        <v>105.8706</v>
+        <v>115.4043</v>
       </c>
       <c r="D14" t="n">
-        <v>100.8938</v>
+        <v>111.9366</v>
       </c>
       <c r="E14" t="n">
-        <v>102.253</v>
+        <v>114.7448</v>
       </c>
       <c r="F14" t="n">
-        <v>68.9966</v>
+        <v>70.9927</v>
       </c>
       <c r="G14" t="n">
-        <v>69.1962</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>67.4795</v>
+        <v>70.2342</v>
       </c>
       <c r="I14" t="n">
-        <v>67.76900000000001</v>
+        <v>71.2422</v>
       </c>
       <c r="J14" t="n">
-        <v>49.2546</v>
+        <v>45.1558</v>
       </c>
       <c r="K14" t="n">
-        <v>51.1607</v>
+        <v>45.7681</v>
       </c>
       <c r="L14" t="n">
-        <v>48.6521</v>
+        <v>44.1187</v>
       </c>
       <c r="M14" t="n">
-        <v>50.4694</v>
+        <v>44.4348</v>
       </c>
       <c r="N14" t="n">
-        <v>39.351</v>
+        <v>38.1481</v>
       </c>
       <c r="O14" t="n">
-        <v>40.2088</v>
+        <v>38.5918</v>
       </c>
       <c r="P14" t="n">
-        <v>39.2327</v>
+        <v>37.7931</v>
       </c>
       <c r="Q14" t="n">
-        <v>40.0511</v>
+        <v>37.9903</v>
       </c>
       <c r="R14" t="n">
-        <v>1.1768</v>
+        <v>10.4357</v>
       </c>
       <c r="S14" t="n">
-        <v>-11.6102</v>
+        <v>13.5371</v>
       </c>
       <c r="T14" t="n">
-        <v>-16.9952</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U14" t="n">
-        <v>-1.9777</v>
+        <v>5.0787</v>
       </c>
       <c r="V14" t="n">
-        <v>-1.8927</v>
+        <v>3.046</v>
       </c>
       <c r="W14" t="n">
-        <v>-5.9034</v>
+        <v>3.1354</v>
       </c>
       <c r="X14" t="n">
-        <v>-1.2178</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y14" t="n">
-        <v>9.328200000000001</v>
+        <v>-13.0291</v>
       </c>
       <c r="Z14" t="n">
-        <v>15.9257</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA14" t="n">
-        <v>1.9836</v>
+        <v>-5.122</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.8047</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC14" t="n">
-        <v>6.0299</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>107.3696</v>
+        <v>116.9533</v>
       </c>
       <c r="C15" t="n">
-        <v>109.2484</v>
+        <v>123.8188</v>
       </c>
       <c r="D15" t="n">
-        <v>100.9938</v>
+        <v>116.6035</v>
       </c>
       <c r="E15" t="n">
-        <v>103.9019</v>
+        <v>123.589</v>
       </c>
       <c r="F15" t="n">
-        <v>68.7171</v>
+        <v>71.7812</v>
       </c>
       <c r="G15" t="n">
-        <v>69.83499999999999</v>
+        <v>72.6395</v>
       </c>
       <c r="H15" t="n">
-        <v>66.4216</v>
+        <v>70.6733</v>
       </c>
       <c r="I15" t="n">
-        <v>67.7989</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>47.9509</v>
+        <v>43.5656</v>
       </c>
       <c r="K15" t="n">
-        <v>51.1015</v>
+        <v>43.7138</v>
       </c>
       <c r="L15" t="n">
-        <v>46.9829</v>
+        <v>40.9582</v>
       </c>
       <c r="M15" t="n">
-        <v>49.4916</v>
+        <v>40.978</v>
       </c>
       <c r="N15" t="n">
-        <v>39.4989</v>
+        <v>37.7241</v>
       </c>
       <c r="O15" t="n">
-        <v>40.8596</v>
+        <v>38.3256</v>
       </c>
       <c r="P15" t="n">
-        <v>38.8186</v>
+        <v>37.2706</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.0412</v>
+        <v>37.3396</v>
       </c>
       <c r="R15" t="n">
-        <v>1.6126</v>
+        <v>7.7077</v>
       </c>
       <c r="S15" t="n">
-        <v>-14.6528</v>
+        <v>20.8659</v>
       </c>
       <c r="T15" t="n">
-        <v>-17.3989</v>
+        <v>1.5186</v>
       </c>
       <c r="U15" t="n">
-        <v>0.0441</v>
+        <v>1.7652</v>
       </c>
       <c r="V15" t="n">
-        <v>-4.297</v>
+        <v>6.9808</v>
       </c>
       <c r="W15" t="n">
-        <v>-5.0594</v>
+        <v>2.3387</v>
       </c>
       <c r="X15" t="n">
-        <v>-1.9374</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y15" t="n">
-        <v>13.5251</v>
+        <v>-18.8062</v>
       </c>
       <c r="Z15" t="n">
-        <v>15.888</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.0247</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB15" t="n">
-        <v>4.4764</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC15" t="n">
-        <v>5.0983</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>113.2557</v>
+        <v>131.9835</v>
       </c>
       <c r="C16" t="n">
-        <v>115.4043</v>
+        <v>143.9056</v>
       </c>
       <c r="D16" t="n">
-        <v>111.9366</v>
+        <v>129.5351</v>
       </c>
       <c r="E16" t="n">
-        <v>114.7448</v>
+        <v>141.837</v>
       </c>
       <c r="F16" t="n">
-        <v>70.9927</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>71.58159999999999</v>
+        <v>79.3366</v>
       </c>
       <c r="H16" t="n">
-        <v>70.2342</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>71.2422</v>
+        <v>78.7577</v>
       </c>
       <c r="J16" t="n">
-        <v>45.1558</v>
+        <v>38.2718</v>
       </c>
       <c r="K16" t="n">
-        <v>45.7681</v>
+        <v>39.0224</v>
       </c>
       <c r="L16" t="n">
-        <v>44.1187</v>
+        <v>34.252</v>
       </c>
       <c r="M16" t="n">
-        <v>44.4348</v>
+        <v>34.894</v>
       </c>
       <c r="N16" t="n">
-        <v>38.1481</v>
+        <v>36.2155</v>
       </c>
       <c r="O16" t="n">
-        <v>38.5918</v>
+        <v>36.2254</v>
       </c>
       <c r="P16" t="n">
-        <v>37.7931</v>
+        <v>33.8294</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.9903</v>
+        <v>34.1154</v>
       </c>
       <c r="R16" t="n">
-        <v>10.4357</v>
+        <v>14.7651</v>
       </c>
       <c r="S16" t="n">
-        <v>13.5371</v>
+        <v>36.5105</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.8120000000000001</v>
+        <v>40.3442</v>
       </c>
       <c r="U16" t="n">
-        <v>5.0787</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V16" t="n">
-        <v>3.046</v>
+        <v>16.1637</v>
       </c>
       <c r="W16" t="n">
-        <v>3.1354</v>
+        <v>13.9166</v>
       </c>
       <c r="X16" t="n">
-        <v>-10.2175</v>
+        <v>-14.847</v>
       </c>
       <c r="Y16" t="n">
-        <v>-13.0291</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z16" t="n">
-        <v>-3.7441</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA16" t="n">
-        <v>-5.122</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB16" t="n">
-        <v>-3.2639</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC16" t="n">
-        <v>-3.4336</v>
+        <v>-13.1307</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>116.9533</v>
+        <v>137.67</v>
       </c>
       <c r="C17" t="n">
-        <v>123.8188</v>
+        <v>152.64</v>
       </c>
       <c r="D17" t="n">
-        <v>116.6035</v>
+        <v>137.46</v>
       </c>
       <c r="E17" t="n">
-        <v>123.589</v>
+        <v>151.95</v>
       </c>
       <c r="F17" t="n">
-        <v>71.7812</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>72.6395</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>70.6733</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>72.49979999999999</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>43.5656</v>
+        <v>35.98</v>
       </c>
       <c r="K17" t="n">
-        <v>43.7138</v>
+        <v>36.01</v>
       </c>
       <c r="L17" t="n">
-        <v>40.9582</v>
+        <v>32.25</v>
       </c>
       <c r="M17" t="n">
-        <v>40.978</v>
+        <v>32.42</v>
       </c>
       <c r="N17" t="n">
-        <v>37.7241</v>
+        <v>34.1745</v>
       </c>
       <c r="O17" t="n">
-        <v>38.3256</v>
+        <v>34.1745</v>
       </c>
       <c r="P17" t="n">
-        <v>37.2706</v>
+        <v>33.1688</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.3396</v>
+        <v>33.297</v>
       </c>
       <c r="R17" t="n">
-        <v>7.7077</v>
+        <v>7.13</v>
       </c>
       <c r="S17" t="n">
-        <v>20.8659</v>
+        <v>32.4243</v>
       </c>
       <c r="T17" t="n">
-        <v>1.5186</v>
+        <v>48.602</v>
       </c>
       <c r="U17" t="n">
-        <v>1.7652</v>
+        <v>2.4332</v>
       </c>
       <c r="V17" t="n">
-        <v>6.9808</v>
+        <v>13.2391</v>
       </c>
       <c r="W17" t="n">
-        <v>2.3387</v>
+        <v>19.0426</v>
       </c>
       <c r="X17" t="n">
-        <v>-7.7795</v>
+        <v>-7.09</v>
       </c>
       <c r="Y17" t="n">
-        <v>-18.8062</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z17" t="n">
-        <v>-6.0036</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA17" t="n">
-        <v>-1.7128</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.7701</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC17" t="n">
-        <v>-2.5727</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>131.9835</v>
+        <v>149.89</v>
       </c>
       <c r="C18" t="n">
-        <v>143.9056</v>
+        <v>151</v>
       </c>
       <c r="D18" t="n">
-        <v>129.5351</v>
+        <v>139.58</v>
       </c>
       <c r="E18" t="n">
-        <v>141.837</v>
+        <v>146.25</v>
       </c>
       <c r="F18" t="n">
-        <v>74.68559999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G18" t="n">
-        <v>79.3366</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>74.68559999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I18" t="n">
-        <v>78.7577</v>
+        <v>78.66</v>
       </c>
       <c r="J18" t="n">
-        <v>38.2718</v>
+        <v>32.87</v>
       </c>
       <c r="K18" t="n">
-        <v>39.0224</v>
+        <v>35.06</v>
       </c>
       <c r="L18" t="n">
-        <v>34.252</v>
+        <v>32.63</v>
       </c>
       <c r="M18" t="n">
-        <v>34.894</v>
+        <v>33.66</v>
       </c>
       <c r="N18" t="n">
-        <v>36.2155</v>
+        <v>33.37</v>
       </c>
       <c r="O18" t="n">
-        <v>36.2254</v>
+        <v>34.54</v>
       </c>
       <c r="P18" t="n">
-        <v>33.8294</v>
+        <v>33.35</v>
       </c>
       <c r="Q18" t="n">
-        <v>34.1154</v>
+        <v>34.14</v>
       </c>
       <c r="R18" t="n">
-        <v>14.7651</v>
+        <v>-3.7512</v>
       </c>
       <c r="S18" t="n">
-        <v>36.5105</v>
+        <v>18.3358</v>
       </c>
       <c r="T18" t="n">
-        <v>40.3442</v>
+        <v>40.7578</v>
       </c>
       <c r="U18" t="n">
-        <v>8.631600000000001</v>
+        <v>-2.4965</v>
       </c>
       <c r="V18" t="n">
-        <v>16.1637</v>
+        <v>8.4969</v>
       </c>
       <c r="W18" t="n">
-        <v>13.9166</v>
+        <v>16.0196</v>
       </c>
       <c r="X18" t="n">
-        <v>-14.847</v>
+        <v>3.8248</v>
       </c>
       <c r="Y18" t="n">
-        <v>-29.4951</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z18" t="n">
-        <v>-31.7031</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA18" t="n">
-        <v>-8.6348</v>
+        <v>2.5318</v>
       </c>
       <c r="AB18" t="n">
-        <v>-14.7993</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC18" t="n">
-        <v>-13.1307</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>137.67</v>
+        <v>138.47</v>
       </c>
       <c r="C19" t="n">
-        <v>152.64</v>
+        <v>147.2</v>
       </c>
       <c r="D19" t="n">
-        <v>137.46</v>
+        <v>136.9</v>
       </c>
       <c r="E19" t="n">
-        <v>151.95</v>
+        <v>146.33</v>
       </c>
       <c r="F19" t="n">
-        <v>78.61799999999999</v>
+        <v>76.75</v>
       </c>
       <c r="G19" t="n">
-        <v>80.96339999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>78.61799999999999</v>
+        <v>76.55</v>
       </c>
       <c r="I19" t="n">
-        <v>80.67400000000001</v>
+        <v>78.58</v>
       </c>
       <c r="J19" t="n">
-        <v>35.98</v>
+        <v>35.45</v>
       </c>
       <c r="K19" t="n">
-        <v>36.01</v>
+        <v>35.85</v>
       </c>
       <c r="L19" t="n">
-        <v>32.25</v>
+        <v>33.43</v>
       </c>
       <c r="M19" t="n">
-        <v>32.42</v>
+        <v>33.63</v>
       </c>
       <c r="N19" t="n">
-        <v>34.1745</v>
+        <v>34.98</v>
       </c>
       <c r="O19" t="n">
-        <v>34.1745</v>
+        <v>35.06</v>
       </c>
       <c r="P19" t="n">
-        <v>33.1688</v>
+        <v>33.95</v>
       </c>
       <c r="Q19" t="n">
-        <v>33.297</v>
+        <v>34.18</v>
       </c>
       <c r="R19" t="n">
-        <v>7.13</v>
+        <v>0.0547</v>
       </c>
       <c r="S19" t="n">
-        <v>32.4243</v>
+        <v>3.1677</v>
       </c>
       <c r="T19" t="n">
-        <v>48.602</v>
+        <v>27.5265</v>
       </c>
       <c r="U19" t="n">
-        <v>2.4332</v>
+        <v>-0.1017</v>
       </c>
       <c r="V19" t="n">
-        <v>13.2391</v>
+        <v>-0.2256</v>
       </c>
       <c r="W19" t="n">
-        <v>19.0426</v>
+        <v>10.2998</v>
       </c>
       <c r="X19" t="n">
-        <v>-7.09</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y19" t="n">
-        <v>-27.0392</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z19" t="n">
-        <v>-35.7631</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA19" t="n">
-        <v>-2.3989</v>
+        <v>0.1172</v>
       </c>
       <c r="AB19" t="n">
-        <v>-12.3539</v>
+        <v>0.1894</v>
       </c>
       <c r="AC19" t="n">
-        <v>-16.8637</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>149.89</v>
+        <v>149.24</v>
       </c>
       <c r="C20" t="n">
-        <v>151</v>
+        <v>153.9</v>
       </c>
       <c r="D20" t="n">
-        <v>139.58</v>
+        <v>147.39</v>
       </c>
       <c r="E20" t="n">
-        <v>146.25</v>
+        <v>151.45</v>
       </c>
       <c r="F20" t="n">
-        <v>80.53</v>
+        <v>79.09</v>
       </c>
       <c r="G20" t="n">
-        <v>80.56999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H20" t="n">
-        <v>77.69</v>
+        <v>78.06</v>
       </c>
       <c r="I20" t="n">
-        <v>78.66</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>32.87</v>
+        <v>32.97</v>
       </c>
       <c r="K20" t="n">
-        <v>35.06</v>
+        <v>33.39</v>
       </c>
       <c r="L20" t="n">
-        <v>32.63</v>
+        <v>31.9</v>
       </c>
       <c r="M20" t="n">
-        <v>33.66</v>
+        <v>32.43</v>
       </c>
       <c r="N20" t="n">
-        <v>33.37</v>
+        <v>33.97</v>
       </c>
       <c r="O20" t="n">
-        <v>34.54</v>
+        <v>34.41</v>
       </c>
       <c r="P20" t="n">
-        <v>33.35</v>
+        <v>33.54</v>
       </c>
       <c r="Q20" t="n">
-        <v>34.14</v>
+        <v>33.75</v>
       </c>
       <c r="R20" t="n">
-        <v>-3.7512</v>
+        <v>3.4989</v>
       </c>
       <c r="S20" t="n">
-        <v>18.3358</v>
+        <v>-0.3291</v>
       </c>
       <c r="T20" t="n">
-        <v>40.7578</v>
+        <v>22.5433</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.4965</v>
+        <v>1.298</v>
       </c>
       <c r="V20" t="n">
-        <v>8.4969</v>
+        <v>-1.3313</v>
       </c>
       <c r="W20" t="n">
-        <v>16.0196</v>
+        <v>9.7934</v>
       </c>
       <c r="X20" t="n">
-        <v>3.8248</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y20" t="n">
-        <v>-17.8584</v>
+        <v>0.0308</v>
       </c>
       <c r="Z20" t="n">
-        <v>-31.9885</v>
+        <v>-20.86</v>
       </c>
       <c r="AA20" t="n">
-        <v>2.5318</v>
+        <v>-1.258</v>
       </c>
       <c r="AB20" t="n">
-        <v>-8.568899999999999</v>
+        <v>1.3605</v>
       </c>
       <c r="AC20" t="n">
-        <v>-14.7378</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>138.47</v>
+        <v>148.14</v>
       </c>
       <c r="C21" t="n">
-        <v>147.2</v>
+        <v>149.99</v>
       </c>
       <c r="D21" t="n">
-        <v>136.9</v>
+        <v>135.21</v>
       </c>
       <c r="E21" t="n">
-        <v>146.33</v>
+        <v>142.29</v>
       </c>
       <c r="F21" t="n">
-        <v>76.75</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>79.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>76.55</v>
+        <v>75.47</v>
       </c>
       <c r="I21" t="n">
-        <v>78.58</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>35.45</v>
+        <v>33.17</v>
       </c>
       <c r="K21" t="n">
-        <v>35.85</v>
+        <v>35.95</v>
       </c>
       <c r="L21" t="n">
-        <v>33.43</v>
+        <v>32.77</v>
       </c>
       <c r="M21" t="n">
-        <v>33.63</v>
+        <v>34.43</v>
       </c>
       <c r="N21" t="n">
-        <v>34.98</v>
+        <v>34.31</v>
       </c>
       <c r="O21" t="n">
-        <v>35.06</v>
+        <v>35.53</v>
       </c>
       <c r="P21" t="n">
-        <v>33.95</v>
+        <v>34.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>34.18</v>
+        <v>34.83</v>
       </c>
       <c r="R21" t="n">
-        <v>0.0547</v>
+        <v>-6.0482</v>
       </c>
       <c r="S21" t="n">
-        <v>3.1677</v>
+        <v>-2.7077</v>
       </c>
       <c r="T21" t="n">
-        <v>27.5265</v>
+        <v>0.3194</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.1017</v>
+        <v>-3.2161</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.2256</v>
+        <v>-2.0595</v>
       </c>
       <c r="W21" t="n">
-        <v>10.2998</v>
+        <v>-2.181</v>
       </c>
       <c r="X21" t="n">
-        <v>-0.0891</v>
+        <v>6.1671</v>
       </c>
       <c r="Y21" t="n">
-        <v>-3.6224</v>
+        <v>2.2876</v>
       </c>
       <c r="Z21" t="n">
-        <v>-24.3161</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.1172</v>
+        <v>3.2</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.1894</v>
+        <v>2.0211</v>
       </c>
       <c r="AC21" t="n">
-        <v>-10.0297</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
+        <v>2.0947</v>
       </c>
     </row>
   </sheetData>
@@ -2328,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-06 02:04
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112.3363</v>
+        <v>125.038</v>
       </c>
       <c r="C2" t="n">
-        <v>114.9746</v>
+        <v>127.4564</v>
       </c>
       <c r="D2" t="n">
-        <v>110.2577</v>
+        <v>121.5203</v>
       </c>
       <c r="E2" t="n">
-        <v>112.7161</v>
+        <v>123.1892</v>
       </c>
       <c r="F2" t="n">
-        <v>71.3021</v>
+        <v>72.8092</v>
       </c>
       <c r="G2" t="n">
-        <v>72.0107</v>
+        <v>73.06870000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>70.6833</v>
+        <v>71.1824</v>
       </c>
       <c r="I2" t="n">
-        <v>71.7812</v>
+        <v>72.02070000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>48.662</v>
+        <v>43.0126</v>
       </c>
       <c r="K2" t="n">
-        <v>49.62</v>
+        <v>44.2768</v>
       </c>
       <c r="L2" t="n">
-        <v>47.4965</v>
+        <v>41.9854</v>
       </c>
       <c r="M2" t="n">
-        <v>48.4151</v>
+        <v>43.536</v>
       </c>
       <c r="N2" t="n">
-        <v>38.227</v>
+        <v>37.3593</v>
       </c>
       <c r="O2" t="n">
-        <v>38.5425</v>
+        <v>38.1974</v>
       </c>
       <c r="P2" t="n">
-        <v>37.8326</v>
+        <v>37.2213</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.9706</v>
+        <v>37.7734</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>106.2903</v>
+        <v>121.1606</v>
       </c>
       <c r="C3" t="n">
-        <v>108.5688</v>
+        <v>128.3958</v>
       </c>
       <c r="D3" t="n">
-        <v>102.243</v>
+        <v>121.1606</v>
       </c>
       <c r="E3" t="n">
-        <v>105.8406</v>
+        <v>125.7875</v>
       </c>
       <c r="F3" t="n">
-        <v>68.9367</v>
+        <v>71.4119</v>
       </c>
       <c r="G3" t="n">
-        <v>70.41379999999999</v>
+        <v>72.41</v>
       </c>
       <c r="H3" t="n">
-        <v>68.1183</v>
+        <v>70.7033</v>
       </c>
       <c r="I3" t="n">
-        <v>69.01649999999999</v>
+        <v>71.4119</v>
       </c>
       <c r="J3" t="n">
-        <v>51.2398</v>
+        <v>44.2471</v>
       </c>
       <c r="K3" t="n">
-        <v>53.0274</v>
+        <v>44.2669</v>
       </c>
       <c r="L3" t="n">
-        <v>50.2719</v>
+        <v>41.7977</v>
       </c>
       <c r="M3" t="n">
-        <v>51.5756</v>
+        <v>42.7064</v>
       </c>
       <c r="N3" t="n">
-        <v>39.4693</v>
+        <v>38.0889</v>
       </c>
       <c r="O3" t="n">
-        <v>39.9032</v>
+        <v>38.4636</v>
       </c>
       <c r="P3" t="n">
-        <v>38.6805</v>
+        <v>37.5664</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.4102</v>
+        <v>38.0988</v>
       </c>
       <c r="R3" t="n">
-        <v>-6.0998</v>
+        <v>2.1092</v>
       </c>
       <c r="U3" t="n">
-        <v>-3.8516</v>
+        <v>-0.8453000000000001</v>
       </c>
       <c r="X3" t="n">
-        <v>6.5279</v>
+        <v>-1.9055</v>
       </c>
       <c r="AA3" t="n">
-        <v>3.7914</v>
+        <v>0.8615</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>104.4315</v>
+        <v>116.2738</v>
       </c>
       <c r="C4" t="n">
-        <v>107.9992</v>
+        <v>119.2418</v>
       </c>
       <c r="D4" t="n">
-        <v>101.2736</v>
+        <v>113.4756</v>
       </c>
       <c r="E4" t="n">
-        <v>106.2803</v>
+        <v>115.6842</v>
       </c>
       <c r="F4" t="n">
-        <v>68.8369</v>
+        <v>68.767</v>
       </c>
       <c r="G4" t="n">
-        <v>69.6254</v>
+        <v>70.0945</v>
       </c>
       <c r="H4" t="n">
-        <v>68.258</v>
+        <v>68.5474</v>
       </c>
       <c r="I4" t="n">
-        <v>69.4657</v>
+        <v>69.07640000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>52.1484</v>
+        <v>45.9459</v>
       </c>
       <c r="K4" t="n">
-        <v>53.7188</v>
+        <v>46.9039</v>
       </c>
       <c r="L4" t="n">
-        <v>50.42</v>
+        <v>44.9385</v>
       </c>
       <c r="M4" t="n">
-        <v>51.1904</v>
+        <v>46.1632</v>
       </c>
       <c r="N4" t="n">
-        <v>39.5285</v>
+        <v>39.5186</v>
       </c>
       <c r="O4" t="n">
-        <v>39.8637</v>
+        <v>39.6271</v>
       </c>
       <c r="P4" t="n">
-        <v>39.0749</v>
+        <v>38.7988</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.1538</v>
+        <v>39.3411</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4154</v>
+        <v>-8.032</v>
       </c>
       <c r="U4" t="n">
-        <v>0.6509</v>
+        <v>-3.2705</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.7469</v>
+        <v>8.0943</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.6506</v>
+        <v>3.2607</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>102.9325</v>
+        <v>120.6309</v>
       </c>
       <c r="C5" t="n">
-        <v>107.4196</v>
+        <v>124.4184</v>
       </c>
       <c r="D5" t="n">
-        <v>98.55540000000001</v>
+        <v>117.7928</v>
       </c>
       <c r="E5" t="n">
-        <v>106.6701</v>
+        <v>121.7402</v>
       </c>
       <c r="F5" t="n">
-        <v>69.9248</v>
+        <v>71.0526</v>
       </c>
       <c r="G5" t="n">
-        <v>72.28019999999999</v>
+        <v>71.6215</v>
       </c>
       <c r="H5" t="n">
-        <v>69.57550000000001</v>
+        <v>70.47369999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>71.89100000000001</v>
+        <v>70.843</v>
       </c>
       <c r="J5" t="n">
-        <v>52.8398</v>
+        <v>44.1385</v>
       </c>
       <c r="K5" t="n">
-        <v>55.0027</v>
+        <v>45.2545</v>
       </c>
       <c r="L5" t="n">
-        <v>50.6472</v>
+        <v>42.5879</v>
       </c>
       <c r="M5" t="n">
-        <v>50.9632</v>
+        <v>43.5953</v>
       </c>
       <c r="N5" t="n">
-        <v>38.9369</v>
+        <v>38.227</v>
       </c>
       <c r="O5" t="n">
-        <v>39.1242</v>
+        <v>38.5523</v>
       </c>
       <c r="P5" t="n">
-        <v>37.5861</v>
+        <v>37.8819</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.803</v>
+        <v>38.3256</v>
       </c>
       <c r="R5" t="n">
-        <v>0.3668</v>
+        <v>5.2349</v>
       </c>
       <c r="S5" t="n">
-        <v>-5.3639</v>
+        <v>-1.1762</v>
       </c>
       <c r="U5" t="n">
-        <v>3.4914</v>
+        <v>2.5575</v>
       </c>
       <c r="V5" t="n">
-        <v>0.153</v>
+        <v>-1.6352</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.4438</v>
+        <v>-5.5627</v>
       </c>
       <c r="Y5" t="n">
-        <v>5.263</v>
+        <v>0.1362</v>
       </c>
       <c r="AA5" t="n">
-        <v>-3.45</v>
+        <v>-2.5813</v>
       </c>
       <c r="AB5" t="n">
-        <v>-0.4414</v>
+        <v>1.4619</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>111.1471</v>
+        <v>101.4635</v>
       </c>
       <c r="C6" t="n">
-        <v>118.1026</v>
+        <v>105.3209</v>
       </c>
       <c r="D6" t="n">
-        <v>109.6581</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>117.2032</v>
+        <v>101.0637</v>
       </c>
       <c r="F6" t="n">
-        <v>72.3501</v>
+        <v>67.3997</v>
       </c>
       <c r="G6" t="n">
-        <v>73.0986</v>
+        <v>70.25409999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>71.5117</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>72.2303</v>
+        <v>69.13630000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>48.9484</v>
+        <v>50.9731</v>
       </c>
       <c r="K6" t="n">
+        <v>51.5756</v>
+      </c>
+      <c r="L6" t="n">
         <v>49.5904</v>
       </c>
-      <c r="L6" t="n">
-        <v>45.5311</v>
-      </c>
       <c r="M6" t="n">
-        <v>45.7681</v>
+        <v>51.0916</v>
       </c>
       <c r="N6" t="n">
-        <v>37.5861</v>
+        <v>40.2088</v>
       </c>
       <c r="O6" t="n">
-        <v>38.0396</v>
+        <v>40.3074</v>
       </c>
       <c r="P6" t="n">
-        <v>37.1917</v>
+        <v>38.6608</v>
       </c>
       <c r="Q6" t="n">
-        <v>37.6452</v>
+        <v>39.2721</v>
       </c>
       <c r="R6" t="n">
-        <v>9.874499999999999</v>
+        <v>-16.9841</v>
       </c>
       <c r="S6" t="n">
-        <v>10.7356</v>
+        <v>-19.6552</v>
       </c>
       <c r="U6" t="n">
-        <v>0.472</v>
+        <v>-2.4091</v>
       </c>
       <c r="V6" t="n">
-        <v>4.6566</v>
+        <v>-3.1866</v>
       </c>
       <c r="X6" t="n">
-        <v>-10.1938</v>
+        <v>17.1952</v>
       </c>
       <c r="Y6" t="n">
-        <v>-11.2602</v>
+        <v>19.6345</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.4174</v>
+        <v>2.4696</v>
       </c>
       <c r="AB6" t="n">
-        <v>-4.4785</v>
+        <v>3.0796</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>125.038</v>
+        <v>104.4815</v>
       </c>
       <c r="C7" t="n">
-        <v>127.4564</v>
+        <v>105.8706</v>
       </c>
       <c r="D7" t="n">
-        <v>121.5203</v>
+        <v>100.8938</v>
       </c>
       <c r="E7" t="n">
-        <v>123.1892</v>
+        <v>102.253</v>
       </c>
       <c r="F7" t="n">
-        <v>72.8092</v>
+        <v>68.9966</v>
       </c>
       <c r="G7" t="n">
-        <v>73.06870000000001</v>
+        <v>69.1962</v>
       </c>
       <c r="H7" t="n">
-        <v>71.1824</v>
+        <v>67.4795</v>
       </c>
       <c r="I7" t="n">
-        <v>72.02070000000001</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>43.0126</v>
+        <v>49.2546</v>
       </c>
       <c r="K7" t="n">
-        <v>44.2768</v>
+        <v>51.1607</v>
       </c>
       <c r="L7" t="n">
-        <v>41.9854</v>
+        <v>48.6521</v>
       </c>
       <c r="M7" t="n">
-        <v>43.536</v>
+        <v>50.4694</v>
       </c>
       <c r="N7" t="n">
-        <v>37.3593</v>
+        <v>39.351</v>
       </c>
       <c r="O7" t="n">
-        <v>38.1974</v>
+        <v>40.2088</v>
       </c>
       <c r="P7" t="n">
-        <v>37.2213</v>
+        <v>39.2327</v>
       </c>
       <c r="Q7" t="n">
-        <v>37.7734</v>
+        <v>40.0511</v>
       </c>
       <c r="R7" t="n">
-        <v>5.1074</v>
+        <v>1.1768</v>
       </c>
       <c r="S7" t="n">
-        <v>15.9097</v>
+        <v>-11.6102</v>
       </c>
       <c r="T7" t="n">
-        <v>9.291600000000001</v>
+        <v>-16.9952</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.2902</v>
+        <v>-1.9777</v>
       </c>
       <c r="V7" t="n">
-        <v>3.6781</v>
+        <v>-1.8927</v>
       </c>
       <c r="W7" t="n">
-        <v>0.3337</v>
+        <v>-5.9034</v>
       </c>
       <c r="X7" t="n">
-        <v>-4.877</v>
+        <v>-1.2178</v>
       </c>
       <c r="Y7" t="n">
-        <v>-14.9528</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="Z7" t="n">
-        <v>-10.0776</v>
+        <v>15.9257</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.3405</v>
+        <v>1.9836</v>
       </c>
       <c r="AB7" t="n">
-        <v>-3.5256</v>
+        <v>1.8047</v>
       </c>
       <c r="AC7" t="n">
-        <v>-0.5193</v>
+        <v>6.0299</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>121.1606</v>
+        <v>107.3696</v>
       </c>
       <c r="C8" t="n">
-        <v>128.3958</v>
+        <v>109.2484</v>
       </c>
       <c r="D8" t="n">
-        <v>121.1606</v>
+        <v>100.9938</v>
       </c>
       <c r="E8" t="n">
-        <v>125.7875</v>
+        <v>103.9019</v>
       </c>
       <c r="F8" t="n">
-        <v>71.4119</v>
+        <v>68.7171</v>
       </c>
       <c r="G8" t="n">
-        <v>72.41</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>70.7033</v>
+        <v>66.4216</v>
       </c>
       <c r="I8" t="n">
-        <v>71.4119</v>
+        <v>67.7989</v>
       </c>
       <c r="J8" t="n">
-        <v>44.2471</v>
+        <v>47.9509</v>
       </c>
       <c r="K8" t="n">
-        <v>44.2669</v>
+        <v>51.1015</v>
       </c>
       <c r="L8" t="n">
-        <v>41.7977</v>
+        <v>46.9829</v>
       </c>
       <c r="M8" t="n">
-        <v>42.7064</v>
+        <v>49.4916</v>
       </c>
       <c r="N8" t="n">
-        <v>38.0889</v>
+        <v>39.4989</v>
       </c>
       <c r="O8" t="n">
-        <v>38.4636</v>
+        <v>40.8596</v>
       </c>
       <c r="P8" t="n">
-        <v>37.5664</v>
+        <v>38.8186</v>
       </c>
       <c r="Q8" t="n">
-        <v>38.0988</v>
+        <v>40.0412</v>
       </c>
       <c r="R8" t="n">
-        <v>2.1092</v>
+        <v>1.6126</v>
       </c>
       <c r="S8" t="n">
-        <v>17.922</v>
+        <v>-14.6528</v>
       </c>
       <c r="T8" t="n">
-        <v>18.8462</v>
+        <v>-17.3989</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.8453000000000001</v>
+        <v>0.0441</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.6664</v>
+        <v>-4.297</v>
       </c>
       <c r="W8" t="n">
-        <v>3.4708</v>
+        <v>-5.0594</v>
       </c>
       <c r="X8" t="n">
-        <v>-1.9055</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y8" t="n">
-        <v>-16.2015</v>
+        <v>13.5251</v>
       </c>
       <c r="Z8" t="n">
-        <v>-17.1965</v>
+        <v>15.888</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.8615</v>
+        <v>-0.0247</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.7825</v>
+        <v>4.4764</v>
       </c>
       <c r="AC8" t="n">
-        <v>-3.3276</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>116.2738</v>
+        <v>113.2557</v>
       </c>
       <c r="C9" t="n">
-        <v>119.2418</v>
+        <v>115.4043</v>
       </c>
       <c r="D9" t="n">
-        <v>113.4756</v>
+        <v>111.9366</v>
       </c>
       <c r="E9" t="n">
-        <v>115.6842</v>
+        <v>114.7448</v>
       </c>
       <c r="F9" t="n">
-        <v>68.767</v>
+        <v>70.9927</v>
       </c>
       <c r="G9" t="n">
-        <v>70.0945</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>68.5474</v>
+        <v>70.2342</v>
       </c>
       <c r="I9" t="n">
-        <v>69.07640000000001</v>
+        <v>71.2422</v>
       </c>
       <c r="J9" t="n">
-        <v>45.9459</v>
+        <v>45.1558</v>
       </c>
       <c r="K9" t="n">
-        <v>46.9039</v>
+        <v>45.7681</v>
       </c>
       <c r="L9" t="n">
-        <v>44.9385</v>
+        <v>44.1187</v>
       </c>
       <c r="M9" t="n">
-        <v>46.1632</v>
+        <v>44.4348</v>
       </c>
       <c r="N9" t="n">
-        <v>39.5186</v>
+        <v>38.1481</v>
       </c>
       <c r="O9" t="n">
-        <v>39.6271</v>
+        <v>38.5918</v>
       </c>
       <c r="P9" t="n">
-        <v>38.7988</v>
+        <v>37.7931</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.3411</v>
+        <v>37.9903</v>
       </c>
       <c r="R9" t="n">
-        <v>-8.032</v>
+        <v>10.4357</v>
       </c>
       <c r="S9" t="n">
-        <v>-1.296</v>
+        <v>13.5371</v>
       </c>
       <c r="T9" t="n">
-        <v>8.8482</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U9" t="n">
-        <v>-3.2705</v>
+        <v>5.0787</v>
       </c>
       <c r="V9" t="n">
-        <v>-4.3665</v>
+        <v>3.046</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.5604</v>
+        <v>3.1354</v>
       </c>
       <c r="X9" t="n">
-        <v>8.0943</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.8633</v>
+        <v>-13.0291</v>
       </c>
       <c r="Z9" t="n">
-        <v>-9.820600000000001</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA9" t="n">
-        <v>3.2607</v>
+        <v>-5.122</v>
       </c>
       <c r="AB9" t="n">
-        <v>4.505</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.4784</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>120.6309</v>
+        <v>116.9533</v>
       </c>
       <c r="C10" t="n">
-        <v>124.4184</v>
+        <v>123.8188</v>
       </c>
       <c r="D10" t="n">
-        <v>117.7928</v>
+        <v>116.6035</v>
       </c>
       <c r="E10" t="n">
-        <v>121.7402</v>
+        <v>123.589</v>
       </c>
       <c r="F10" t="n">
-        <v>71.0526</v>
+        <v>71.7812</v>
       </c>
       <c r="G10" t="n">
-        <v>71.6215</v>
+        <v>72.6395</v>
       </c>
       <c r="H10" t="n">
-        <v>70.47369999999999</v>
+        <v>70.6733</v>
       </c>
       <c r="I10" t="n">
-        <v>70.843</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>44.1385</v>
+        <v>43.5656</v>
       </c>
       <c r="K10" t="n">
-        <v>45.2545</v>
+        <v>43.7138</v>
       </c>
       <c r="L10" t="n">
-        <v>42.5879</v>
+        <v>40.9582</v>
       </c>
       <c r="M10" t="n">
-        <v>43.5953</v>
+        <v>40.978</v>
       </c>
       <c r="N10" t="n">
-        <v>38.227</v>
+        <v>37.7241</v>
       </c>
       <c r="O10" t="n">
-        <v>38.5523</v>
+        <v>38.3256</v>
       </c>
       <c r="P10" t="n">
-        <v>37.8819</v>
+        <v>37.2706</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.3256</v>
+        <v>37.3396</v>
       </c>
       <c r="R10" t="n">
-        <v>5.2349</v>
+        <v>7.7077</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.1762</v>
+        <v>20.8659</v>
       </c>
       <c r="T10" t="n">
-        <v>14.1278</v>
+        <v>1.5186</v>
       </c>
       <c r="U10" t="n">
-        <v>2.5575</v>
+        <v>1.7652</v>
       </c>
       <c r="V10" t="n">
-        <v>-1.6352</v>
+        <v>6.9808</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.4578</v>
+        <v>2.3387</v>
       </c>
       <c r="X10" t="n">
-        <v>-5.5627</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.1362</v>
+        <v>-18.8062</v>
       </c>
       <c r="Z10" t="n">
-        <v>-14.4573</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA10" t="n">
-        <v>-2.5813</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.4619</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.3824</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>101.4635</v>
+        <v>131.9835</v>
       </c>
       <c r="C11" t="n">
-        <v>105.3209</v>
+        <v>143.9056</v>
       </c>
       <c r="D11" t="n">
-        <v>99.80459999999999</v>
+        <v>129.5351</v>
       </c>
       <c r="E11" t="n">
-        <v>101.0637</v>
+        <v>141.837</v>
       </c>
       <c r="F11" t="n">
-        <v>67.3997</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>70.25409999999999</v>
+        <v>79.3366</v>
       </c>
       <c r="H11" t="n">
-        <v>67.20999999999999</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>69.13630000000001</v>
+        <v>78.7577</v>
       </c>
       <c r="J11" t="n">
-        <v>50.9731</v>
+        <v>38.2718</v>
       </c>
       <c r="K11" t="n">
-        <v>51.5756</v>
+        <v>39.0224</v>
       </c>
       <c r="L11" t="n">
-        <v>49.5904</v>
+        <v>34.252</v>
       </c>
       <c r="M11" t="n">
-        <v>51.0916</v>
+        <v>34.894</v>
       </c>
       <c r="N11" t="n">
-        <v>40.2088</v>
+        <v>36.2155</v>
       </c>
       <c r="O11" t="n">
-        <v>40.3074</v>
+        <v>36.2254</v>
       </c>
       <c r="P11" t="n">
-        <v>38.6608</v>
+        <v>33.8294</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.2721</v>
+        <v>34.1154</v>
       </c>
       <c r="R11" t="n">
-        <v>-16.9841</v>
+        <v>14.7651</v>
       </c>
       <c r="S11" t="n">
-        <v>-19.6552</v>
+        <v>36.5105</v>
       </c>
       <c r="T11" t="n">
-        <v>-13.7705</v>
+        <v>40.3442</v>
       </c>
       <c r="U11" t="n">
-        <v>-2.4091</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>-3.1866</v>
+        <v>16.1637</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.2835</v>
+        <v>13.9166</v>
       </c>
       <c r="X11" t="n">
-        <v>17.1952</v>
+        <v>-14.847</v>
       </c>
       <c r="Y11" t="n">
-        <v>19.6345</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z11" t="n">
-        <v>11.6315</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA11" t="n">
-        <v>2.4696</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.0796</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC11" t="n">
-        <v>4.3217</v>
+        <v>-13.1307</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>104.4815</v>
+        <v>137.67</v>
       </c>
       <c r="C12" t="n">
-        <v>105.8706</v>
+        <v>152.64</v>
       </c>
       <c r="D12" t="n">
-        <v>100.8938</v>
+        <v>137.46</v>
       </c>
       <c r="E12" t="n">
-        <v>102.253</v>
+        <v>151.95</v>
       </c>
       <c r="F12" t="n">
-        <v>68.9966</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>69.1962</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>67.4795</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>67.76900000000001</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>49.2546</v>
+        <v>35.98</v>
       </c>
       <c r="K12" t="n">
-        <v>51.1607</v>
+        <v>36.01</v>
       </c>
       <c r="L12" t="n">
-        <v>48.6521</v>
+        <v>32.25</v>
       </c>
       <c r="M12" t="n">
-        <v>50.4694</v>
+        <v>32.42</v>
       </c>
       <c r="N12" t="n">
-        <v>39.351</v>
+        <v>34.1745</v>
       </c>
       <c r="O12" t="n">
-        <v>40.2088</v>
+        <v>34.1745</v>
       </c>
       <c r="P12" t="n">
-        <v>39.2327</v>
+        <v>33.1688</v>
       </c>
       <c r="Q12" t="n">
-        <v>40.0511</v>
+        <v>33.297</v>
       </c>
       <c r="R12" t="n">
-        <v>1.1768</v>
+        <v>7.13</v>
       </c>
       <c r="S12" t="n">
-        <v>-11.6102</v>
+        <v>32.4243</v>
       </c>
       <c r="T12" t="n">
-        <v>-16.9952</v>
+        <v>48.602</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.9777</v>
+        <v>2.4332</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.8927</v>
+        <v>13.2391</v>
       </c>
       <c r="W12" t="n">
-        <v>-5.9034</v>
+        <v>19.0426</v>
       </c>
       <c r="X12" t="n">
-        <v>-1.2178</v>
+        <v>-7.09</v>
       </c>
       <c r="Y12" t="n">
-        <v>9.328200000000001</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z12" t="n">
-        <v>15.9257</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.9836</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.8047</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC12" t="n">
-        <v>6.0299</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>107.3696</v>
+        <v>149.89</v>
       </c>
       <c r="C13" t="n">
-        <v>109.2484</v>
+        <v>151</v>
       </c>
       <c r="D13" t="n">
-        <v>100.9938</v>
+        <v>139.58</v>
       </c>
       <c r="E13" t="n">
-        <v>103.9019</v>
+        <v>146.25</v>
       </c>
       <c r="F13" t="n">
-        <v>68.7171</v>
+        <v>80.53</v>
       </c>
       <c r="G13" t="n">
-        <v>69.83499999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>66.4216</v>
+        <v>77.69</v>
       </c>
       <c r="I13" t="n">
-        <v>67.7989</v>
+        <v>78.66</v>
       </c>
       <c r="J13" t="n">
-        <v>47.9509</v>
+        <v>32.87</v>
       </c>
       <c r="K13" t="n">
-        <v>51.1015</v>
+        <v>35.06</v>
       </c>
       <c r="L13" t="n">
-        <v>46.9829</v>
+        <v>32.63</v>
       </c>
       <c r="M13" t="n">
-        <v>49.4916</v>
+        <v>33.66</v>
       </c>
       <c r="N13" t="n">
-        <v>39.4989</v>
+        <v>33.37</v>
       </c>
       <c r="O13" t="n">
-        <v>40.8596</v>
+        <v>34.54</v>
       </c>
       <c r="P13" t="n">
-        <v>38.8186</v>
+        <v>33.35</v>
       </c>
       <c r="Q13" t="n">
-        <v>40.0412</v>
+        <v>34.14</v>
       </c>
       <c r="R13" t="n">
-        <v>1.6126</v>
+        <v>-3.7512</v>
       </c>
       <c r="S13" t="n">
-        <v>-14.6528</v>
+        <v>18.3358</v>
       </c>
       <c r="T13" t="n">
-        <v>-17.3989</v>
+        <v>40.7578</v>
       </c>
       <c r="U13" t="n">
-        <v>0.0441</v>
+        <v>-2.4965</v>
       </c>
       <c r="V13" t="n">
-        <v>-4.297</v>
+        <v>8.4969</v>
       </c>
       <c r="W13" t="n">
-        <v>-5.0594</v>
+        <v>16.0196</v>
       </c>
       <c r="X13" t="n">
-        <v>-1.9374</v>
+        <v>3.8248</v>
       </c>
       <c r="Y13" t="n">
-        <v>13.5251</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z13" t="n">
-        <v>15.888</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.0247</v>
+        <v>2.5318</v>
       </c>
       <c r="AB13" t="n">
-        <v>4.4764</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC13" t="n">
-        <v>5.0983</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>113.2557</v>
+        <v>138.47</v>
       </c>
       <c r="C14" t="n">
-        <v>115.4043</v>
+        <v>147.2</v>
       </c>
       <c r="D14" t="n">
-        <v>111.9366</v>
+        <v>136.9</v>
       </c>
       <c r="E14" t="n">
-        <v>114.7448</v>
+        <v>146.33</v>
       </c>
       <c r="F14" t="n">
-        <v>70.9927</v>
+        <v>76.75</v>
       </c>
       <c r="G14" t="n">
-        <v>71.58159999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>70.2342</v>
+        <v>76.55</v>
       </c>
       <c r="I14" t="n">
-        <v>71.2422</v>
+        <v>78.58</v>
       </c>
       <c r="J14" t="n">
-        <v>45.1558</v>
+        <v>35.45</v>
       </c>
       <c r="K14" t="n">
-        <v>45.7681</v>
+        <v>35.85</v>
       </c>
       <c r="L14" t="n">
-        <v>44.1187</v>
+        <v>33.43</v>
       </c>
       <c r="M14" t="n">
-        <v>44.4348</v>
+        <v>33.63</v>
       </c>
       <c r="N14" t="n">
-        <v>38.1481</v>
+        <v>34.98</v>
       </c>
       <c r="O14" t="n">
-        <v>38.5918</v>
+        <v>35.06</v>
       </c>
       <c r="P14" t="n">
-        <v>37.7931</v>
+        <v>33.95</v>
       </c>
       <c r="Q14" t="n">
-        <v>37.9903</v>
+        <v>34.18</v>
       </c>
       <c r="R14" t="n">
-        <v>10.4357</v>
+        <v>0.0547</v>
       </c>
       <c r="S14" t="n">
-        <v>13.5371</v>
+        <v>3.1677</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.8120000000000001</v>
+        <v>27.5265</v>
       </c>
       <c r="U14" t="n">
-        <v>5.0787</v>
+        <v>-0.1017</v>
       </c>
       <c r="V14" t="n">
-        <v>3.046</v>
+        <v>-0.2256</v>
       </c>
       <c r="W14" t="n">
-        <v>3.1354</v>
+        <v>10.2998</v>
       </c>
       <c r="X14" t="n">
-        <v>-10.2175</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y14" t="n">
-        <v>-13.0291</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z14" t="n">
-        <v>-3.7441</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA14" t="n">
-        <v>-5.122</v>
+        <v>0.1172</v>
       </c>
       <c r="AB14" t="n">
-        <v>-3.2639</v>
+        <v>0.1894</v>
       </c>
       <c r="AC14" t="n">
-        <v>-3.4336</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>116.9533</v>
+        <v>149.24</v>
       </c>
       <c r="C15" t="n">
-        <v>123.8188</v>
+        <v>153.9</v>
       </c>
       <c r="D15" t="n">
-        <v>116.6035</v>
+        <v>147.39</v>
       </c>
       <c r="E15" t="n">
-        <v>123.589</v>
+        <v>151.45</v>
       </c>
       <c r="F15" t="n">
-        <v>71.7812</v>
+        <v>79.09</v>
       </c>
       <c r="G15" t="n">
-        <v>72.6395</v>
+        <v>80.06</v>
       </c>
       <c r="H15" t="n">
-        <v>70.6733</v>
+        <v>78.06</v>
       </c>
       <c r="I15" t="n">
-        <v>72.49979999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>43.5656</v>
+        <v>32.97</v>
       </c>
       <c r="K15" t="n">
-        <v>43.7138</v>
+        <v>33.39</v>
       </c>
       <c r="L15" t="n">
-        <v>40.9582</v>
+        <v>31.9</v>
       </c>
       <c r="M15" t="n">
-        <v>40.978</v>
+        <v>32.43</v>
       </c>
       <c r="N15" t="n">
-        <v>37.7241</v>
+        <v>33.97</v>
       </c>
       <c r="O15" t="n">
-        <v>38.3256</v>
+        <v>34.41</v>
       </c>
       <c r="P15" t="n">
-        <v>37.2706</v>
+        <v>33.54</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.3396</v>
+        <v>33.75</v>
       </c>
       <c r="R15" t="n">
-        <v>7.7077</v>
+        <v>3.4989</v>
       </c>
       <c r="S15" t="n">
-        <v>20.8659</v>
+        <v>-0.3291</v>
       </c>
       <c r="T15" t="n">
-        <v>1.5186</v>
+        <v>22.5433</v>
       </c>
       <c r="U15" t="n">
-        <v>1.7652</v>
+        <v>1.298</v>
       </c>
       <c r="V15" t="n">
-        <v>6.9808</v>
+        <v>-1.3313</v>
       </c>
       <c r="W15" t="n">
-        <v>2.3387</v>
+        <v>9.7934</v>
       </c>
       <c r="X15" t="n">
-        <v>-7.7795</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y15" t="n">
-        <v>-18.8062</v>
+        <v>0.0308</v>
       </c>
       <c r="Z15" t="n">
-        <v>-6.0036</v>
+        <v>-20.86</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.7128</v>
+        <v>-1.258</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.7701</v>
+        <v>1.3605</v>
       </c>
       <c r="AC15" t="n">
-        <v>-2.5727</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>131.9835</v>
+        <v>148.14</v>
       </c>
       <c r="C16" t="n">
-        <v>143.9056</v>
+        <v>149.99</v>
       </c>
       <c r="D16" t="n">
-        <v>129.5351</v>
+        <v>135.21</v>
       </c>
       <c r="E16" t="n">
-        <v>141.837</v>
+        <v>142.29</v>
       </c>
       <c r="F16" t="n">
-        <v>74.68559999999999</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>79.3366</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>74.68559999999999</v>
+        <v>75.47</v>
       </c>
       <c r="I16" t="n">
-        <v>78.7577</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>38.2718</v>
+        <v>33.17</v>
       </c>
       <c r="K16" t="n">
-        <v>39.0224</v>
+        <v>35.95</v>
       </c>
       <c r="L16" t="n">
-        <v>34.252</v>
+        <v>32.77</v>
       </c>
       <c r="M16" t="n">
-        <v>34.894</v>
+        <v>34.43</v>
       </c>
       <c r="N16" t="n">
-        <v>36.2155</v>
+        <v>34.31</v>
       </c>
       <c r="O16" t="n">
-        <v>36.2254</v>
+        <v>35.53</v>
       </c>
       <c r="P16" t="n">
-        <v>33.8294</v>
+        <v>34.17</v>
       </c>
       <c r="Q16" t="n">
-        <v>34.1154</v>
+        <v>34.83</v>
       </c>
       <c r="R16" t="n">
-        <v>14.7651</v>
+        <v>-6.0482</v>
       </c>
       <c r="S16" t="n">
-        <v>36.5105</v>
+        <v>-2.7077</v>
       </c>
       <c r="T16" t="n">
-        <v>40.3442</v>
+        <v>0.3194</v>
       </c>
       <c r="U16" t="n">
-        <v>8.631600000000001</v>
+        <v>-3.2161</v>
       </c>
       <c r="V16" t="n">
-        <v>16.1637</v>
+        <v>-2.0595</v>
       </c>
       <c r="W16" t="n">
-        <v>13.9166</v>
+        <v>-2.181</v>
       </c>
       <c r="X16" t="n">
-        <v>-14.847</v>
+        <v>6.1671</v>
       </c>
       <c r="Y16" t="n">
-        <v>-29.4951</v>
+        <v>2.2876</v>
       </c>
       <c r="Z16" t="n">
-        <v>-31.7031</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA16" t="n">
-        <v>-8.6348</v>
+        <v>3.2</v>
       </c>
       <c r="AB16" t="n">
-        <v>-14.7993</v>
+        <v>2.0211</v>
       </c>
       <c r="AC16" t="n">
-        <v>-13.1307</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>137.67</v>
+        <v>148.94</v>
       </c>
       <c r="C17" t="n">
-        <v>152.64</v>
+        <v>152.37</v>
       </c>
       <c r="D17" t="n">
-        <v>137.46</v>
+        <v>145.49</v>
       </c>
       <c r="E17" t="n">
-        <v>151.95</v>
+        <v>147</v>
       </c>
       <c r="F17" t="n">
-        <v>78.61799999999999</v>
+        <v>78.13</v>
       </c>
       <c r="G17" t="n">
-        <v>80.96339999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>78.61799999999999</v>
+        <v>76.62</v>
       </c>
       <c r="I17" t="n">
-        <v>80.67400000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>35.98</v>
+        <v>32.82</v>
       </c>
       <c r="K17" t="n">
-        <v>36.01</v>
+        <v>33.64</v>
       </c>
       <c r="L17" t="n">
-        <v>32.25</v>
+        <v>31.96</v>
       </c>
       <c r="M17" t="n">
-        <v>32.42</v>
+        <v>33.26</v>
       </c>
       <c r="N17" t="n">
-        <v>34.1745</v>
+        <v>34.34</v>
       </c>
       <c r="O17" t="n">
-        <v>34.1745</v>
+        <v>35.02</v>
       </c>
       <c r="P17" t="n">
-        <v>33.1688</v>
+        <v>34.28</v>
       </c>
       <c r="Q17" t="n">
-        <v>33.297</v>
+        <v>34.66</v>
       </c>
       <c r="R17" t="n">
-        <v>7.13</v>
+        <v>3.3101</v>
       </c>
       <c r="S17" t="n">
-        <v>32.4243</v>
+        <v>0.4579</v>
       </c>
       <c r="T17" t="n">
-        <v>48.602</v>
+        <v>-3.2577</v>
       </c>
       <c r="U17" t="n">
-        <v>2.4332</v>
+        <v>0.5452</v>
       </c>
       <c r="V17" t="n">
-        <v>13.2391</v>
+        <v>-1.4253</v>
       </c>
       <c r="W17" t="n">
-        <v>19.0426</v>
+        <v>-3.9839</v>
       </c>
       <c r="X17" t="n">
-        <v>-7.09</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y17" t="n">
-        <v>-27.0392</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z17" t="n">
-        <v>-35.7631</v>
+        <v>2.591</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.3989</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB17" t="n">
-        <v>-12.3539</v>
+        <v>1.4043</v>
       </c>
       <c r="AC17" t="n">
-        <v>-16.8637</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>149.89</v>
+        <v>147.95</v>
       </c>
       <c r="C18" t="n">
-        <v>151</v>
+        <v>150.77</v>
       </c>
       <c r="D18" t="n">
-        <v>139.58</v>
+        <v>144.41</v>
       </c>
       <c r="E18" t="n">
-        <v>146.25</v>
+        <v>147.86</v>
       </c>
       <c r="F18" t="n">
-        <v>80.53</v>
+        <v>78.13</v>
       </c>
       <c r="G18" t="n">
-        <v>80.56999999999999</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>77.69</v>
+        <v>77.94</v>
       </c>
       <c r="I18" t="n">
-        <v>78.66</v>
+        <v>78.03</v>
       </c>
       <c r="J18" t="n">
-        <v>32.87</v>
+        <v>33.07</v>
       </c>
       <c r="K18" t="n">
-        <v>35.06</v>
+        <v>33.86</v>
       </c>
       <c r="L18" t="n">
-        <v>32.63</v>
+        <v>32.42</v>
       </c>
       <c r="M18" t="n">
+        <v>33.08</v>
+      </c>
+      <c r="N18" t="n">
+        <v>34.36</v>
+      </c>
+      <c r="O18" t="n">
+        <v>34.44</v>
+      </c>
+      <c r="P18" t="n">
         <v>33.66</v>
       </c>
-      <c r="N18" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O18" t="n">
-        <v>34.54</v>
-      </c>
-      <c r="P18" t="n">
-        <v>33.35</v>
-      </c>
       <c r="Q18" t="n">
-        <v>34.14</v>
+        <v>34.41</v>
       </c>
       <c r="R18" t="n">
-        <v>-3.7512</v>
+        <v>0.585</v>
       </c>
       <c r="S18" t="n">
-        <v>18.3358</v>
+        <v>-2.3704</v>
       </c>
       <c r="T18" t="n">
-        <v>40.7578</v>
+        <v>1.1009</v>
       </c>
       <c r="U18" t="n">
-        <v>-2.4965</v>
+        <v>0.7359</v>
       </c>
       <c r="V18" t="n">
-        <v>8.4969</v>
+        <v>-1.9724</v>
       </c>
       <c r="W18" t="n">
-        <v>16.0196</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X18" t="n">
-        <v>3.8248</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y18" t="n">
-        <v>-17.8584</v>
+        <v>2.0043</v>
       </c>
       <c r="Z18" t="n">
-        <v>-31.9885</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA18" t="n">
-        <v>2.5318</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB18" t="n">
-        <v>-8.568899999999999</v>
+        <v>1.9556</v>
       </c>
       <c r="AC18" t="n">
-        <v>-14.7378</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>138.47</v>
+        <v>148.56</v>
       </c>
       <c r="C19" t="n">
-        <v>147.2</v>
+        <v>156.71</v>
       </c>
       <c r="D19" t="n">
-        <v>136.9</v>
+        <v>144.31</v>
       </c>
       <c r="E19" t="n">
-        <v>146.33</v>
+        <v>153.69</v>
       </c>
       <c r="F19" t="n">
-        <v>76.75</v>
+        <v>78.88</v>
       </c>
       <c r="G19" t="n">
-        <v>79.09999999999999</v>
+        <v>79.53</v>
       </c>
       <c r="H19" t="n">
-        <v>76.55</v>
+        <v>76.87</v>
       </c>
       <c r="I19" t="n">
-        <v>78.58</v>
+        <v>78.73</v>
       </c>
       <c r="J19" t="n">
-        <v>35.45</v>
+        <v>32.95</v>
       </c>
       <c r="K19" t="n">
-        <v>35.85</v>
+        <v>33.89</v>
       </c>
       <c r="L19" t="n">
-        <v>33.43</v>
+        <v>31.1</v>
       </c>
       <c r="M19" t="n">
-        <v>33.63</v>
+        <v>31.76</v>
       </c>
       <c r="N19" t="n">
-        <v>34.98</v>
+        <v>34.04</v>
       </c>
       <c r="O19" t="n">
-        <v>35.06</v>
+        <v>34.92</v>
       </c>
       <c r="P19" t="n">
-        <v>33.95</v>
+        <v>33.74</v>
       </c>
       <c r="Q19" t="n">
-        <v>34.18</v>
+        <v>34.11</v>
       </c>
       <c r="R19" t="n">
-        <v>0.0547</v>
+        <v>3.9429</v>
       </c>
       <c r="S19" t="n">
-        <v>3.1677</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T19" t="n">
-        <v>27.5265</v>
+        <v>5.0297</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.1017</v>
+        <v>0.8971</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.2256</v>
+        <v>2.1937</v>
       </c>
       <c r="W19" t="n">
-        <v>10.2998</v>
+        <v>0.1909</v>
       </c>
       <c r="X19" t="n">
-        <v>-0.0891</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y19" t="n">
-        <v>-3.6224</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z19" t="n">
-        <v>-24.3161</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.1172</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.1894</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC19" t="n">
-        <v>-10.0297</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>149.24</v>
+        <v>165.39</v>
       </c>
       <c r="C20" t="n">
-        <v>153.9</v>
+        <v>169.75</v>
       </c>
       <c r="D20" t="n">
-        <v>147.39</v>
+        <v>162.4</v>
       </c>
       <c r="E20" t="n">
-        <v>151.45</v>
+        <v>163.71</v>
       </c>
       <c r="F20" t="n">
-        <v>79.09</v>
+        <v>81.59</v>
       </c>
       <c r="G20" t="n">
-        <v>80.06</v>
+        <v>82.61</v>
       </c>
       <c r="H20" t="n">
-        <v>78.06</v>
+        <v>80.37</v>
       </c>
       <c r="I20" t="n">
-        <v>79.59999999999999</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>32.97</v>
+        <v>29.39</v>
       </c>
       <c r="K20" t="n">
-        <v>33.39</v>
+        <v>29.98</v>
       </c>
       <c r="L20" t="n">
-        <v>31.9</v>
+        <v>28.46</v>
       </c>
       <c r="M20" t="n">
-        <v>32.43</v>
+        <v>29.71</v>
       </c>
       <c r="N20" t="n">
-        <v>33.97</v>
+        <v>32.87</v>
       </c>
       <c r="O20" t="n">
-        <v>34.41</v>
+        <v>33.41</v>
       </c>
       <c r="P20" t="n">
-        <v>33.54</v>
+        <v>32.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>33.75</v>
+        <v>33.12</v>
       </c>
       <c r="R20" t="n">
-        <v>3.4989</v>
+        <v>6.5196</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.3291</v>
+        <v>11.3673</v>
       </c>
       <c r="T20" t="n">
-        <v>22.5433</v>
+        <v>8.0951</v>
       </c>
       <c r="U20" t="n">
-        <v>1.298</v>
+        <v>2.896</v>
       </c>
       <c r="V20" t="n">
-        <v>-1.3313</v>
+        <v>4.583</v>
       </c>
       <c r="W20" t="n">
-        <v>9.7934</v>
+        <v>1.7714</v>
       </c>
       <c r="X20" t="n">
-        <v>-3.5682</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.0308</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z20" t="n">
-        <v>-20.86</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.258</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.3605</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC20" t="n">
-        <v>-9.6134</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>148.14</v>
+        <v>161.66</v>
       </c>
       <c r="C21" t="n">
-        <v>149.99</v>
+        <v>164.38</v>
       </c>
       <c r="D21" t="n">
-        <v>135.21</v>
+        <v>158.08</v>
       </c>
       <c r="E21" t="n">
-        <v>142.29</v>
+        <v>164.27</v>
       </c>
       <c r="F21" t="n">
-        <v>78.29000000000001</v>
+        <v>80.95</v>
       </c>
       <c r="G21" t="n">
-        <v>78.59999999999999</v>
+        <v>83.38</v>
       </c>
       <c r="H21" t="n">
-        <v>75.47</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>77.04000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J21" t="n">
+        <v>30.09</v>
+      </c>
+      <c r="K21" t="n">
+        <v>30.75</v>
+      </c>
+      <c r="L21" t="n">
+        <v>29.62</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29.62</v>
+      </c>
+      <c r="N21" t="n">
         <v>33.17</v>
       </c>
-      <c r="K21" t="n">
-        <v>35.95</v>
-      </c>
-      <c r="L21" t="n">
-        <v>32.77</v>
-      </c>
-      <c r="M21" t="n">
-        <v>34.43</v>
-      </c>
-      <c r="N21" t="n">
-        <v>34.31</v>
-      </c>
       <c r="O21" t="n">
-        <v>35.53</v>
+        <v>33.2</v>
       </c>
       <c r="P21" t="n">
-        <v>34.17</v>
+        <v>32.16</v>
       </c>
       <c r="Q21" t="n">
-        <v>34.83</v>
+        <v>32.25</v>
       </c>
       <c r="R21" t="n">
-        <v>-6.0482</v>
+        <v>0.3421</v>
       </c>
       <c r="S21" t="n">
-        <v>-2.7077</v>
+        <v>11.0983</v>
       </c>
       <c r="T21" t="n">
-        <v>0.3194</v>
+        <v>15.4473</v>
       </c>
       <c r="U21" t="n">
-        <v>-3.2161</v>
+        <v>2.6046</v>
       </c>
       <c r="V21" t="n">
-        <v>-2.0595</v>
+        <v>6.5231</v>
       </c>
       <c r="W21" t="n">
-        <v>-2.181</v>
+        <v>7.892</v>
       </c>
       <c r="X21" t="n">
-        <v>6.1671</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y21" t="n">
-        <v>2.2876</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z21" t="n">
-        <v>-1.3297</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA21" t="n">
-        <v>3.2</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB21" t="n">
-        <v>2.0211</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC21" t="n">
-        <v>2.0947</v>
+        <v>-7.4074</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-07 01:13
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>-7.4074</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>167.34</v>
+      </c>
+      <c r="C22" t="n">
+        <v>169.83</v>
+      </c>
+      <c r="D22" t="n">
+        <v>163.42</v>
+      </c>
+      <c r="E22" t="n">
+        <v>164.26</v>
+      </c>
+      <c r="F22" t="n">
+        <v>84.54000000000001</v>
+      </c>
+      <c r="G22" t="n">
+        <v>85.31999999999999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>84.09</v>
+      </c>
+      <c r="I22" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="J22" t="n">
+        <v>29.06</v>
+      </c>
+      <c r="K22" t="n">
+        <v>29.77</v>
+      </c>
+      <c r="L22" t="n">
+        <v>28.62</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29.63</v>
+      </c>
+      <c r="N22" t="n">
+        <v>31.72</v>
+      </c>
+      <c r="O22" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="P22" t="n">
+        <v>31.42</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>31.83</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-0.0061</v>
+      </c>
+      <c r="S22" t="n">
+        <v>6.8775</v>
+      </c>
+      <c r="T22" t="n">
+        <v>11.7415</v>
+      </c>
+      <c r="U22" t="n">
+        <v>1.3595</v>
+      </c>
+      <c r="V22" t="n">
+        <v>7.0113</v>
+      </c>
+      <c r="W22" t="n">
+        <v>8.7658</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0.0338</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-6.7065</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-10.914</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-1.3023</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-6.6843</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>-8.164999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-08 01:35
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2366,6 +2366,97 @@
       </c>
       <c r="AC22" t="n">
         <v>-8.164999999999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>153.7</v>
+      </c>
+      <c r="C23" t="n">
+        <v>159.49</v>
+      </c>
+      <c r="D23" t="n">
+        <v>151.42</v>
+      </c>
+      <c r="E23" t="n">
+        <v>158.91</v>
+      </c>
+      <c r="F23" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="G23" t="n">
+        <v>83.75</v>
+      </c>
+      <c r="H23" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="I23" t="n">
+        <v>83.62</v>
+      </c>
+      <c r="J23" t="n">
+        <v>31.55</v>
+      </c>
+      <c r="K23" t="n">
+        <v>31.97</v>
+      </c>
+      <c r="L23" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="M23" t="n">
+        <v>30.65</v>
+      </c>
+      <c r="N23" t="n">
+        <v>32.58</v>
+      </c>
+      <c r="O23" t="n">
+        <v>32.84</v>
+      </c>
+      <c r="P23" t="n">
+        <v>32.02</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>32.07</v>
+      </c>
+      <c r="R23" t="n">
+        <v>-3.257</v>
+      </c>
+      <c r="S23" t="n">
+        <v>-2.932</v>
+      </c>
+      <c r="T23" t="n">
+        <v>7.4733</v>
+      </c>
+      <c r="U23" t="n">
+        <v>-0.7478</v>
+      </c>
+      <c r="V23" t="n">
+        <v>3.2218</v>
+      </c>
+      <c r="W23" t="n">
+        <v>7.1639</v>
+      </c>
+      <c r="X23" t="n">
+        <v>3.4425</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>3.1639</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>-7.3458</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>-3.1703</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>-6.8003</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-09 01:45
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>125.038</v>
+        <v>121.1606</v>
       </c>
       <c r="C2" t="n">
-        <v>127.4564</v>
+        <v>128.3958</v>
       </c>
       <c r="D2" t="n">
-        <v>121.5203</v>
+        <v>121.1606</v>
       </c>
       <c r="E2" t="n">
-        <v>123.1892</v>
+        <v>125.7875</v>
       </c>
       <c r="F2" t="n">
-        <v>72.8092</v>
+        <v>71.4119</v>
       </c>
       <c r="G2" t="n">
-        <v>73.06870000000001</v>
+        <v>72.41</v>
       </c>
       <c r="H2" t="n">
-        <v>71.1824</v>
+        <v>70.7033</v>
       </c>
       <c r="I2" t="n">
-        <v>72.02070000000001</v>
+        <v>71.4119</v>
       </c>
       <c r="J2" t="n">
-        <v>43.0126</v>
+        <v>44.2471</v>
       </c>
       <c r="K2" t="n">
-        <v>44.2768</v>
+        <v>44.2669</v>
       </c>
       <c r="L2" t="n">
-        <v>41.9854</v>
+        <v>41.7977</v>
       </c>
       <c r="M2" t="n">
-        <v>43.536</v>
+        <v>42.7064</v>
       </c>
       <c r="N2" t="n">
-        <v>37.3593</v>
+        <v>38.0889</v>
       </c>
       <c r="O2" t="n">
-        <v>38.1974</v>
+        <v>38.4636</v>
       </c>
       <c r="P2" t="n">
-        <v>37.2213</v>
+        <v>37.5664</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.7734</v>
+        <v>38.0988</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>121.1606</v>
+        <v>116.2738</v>
       </c>
       <c r="C3" t="n">
-        <v>128.3958</v>
+        <v>119.2418</v>
       </c>
       <c r="D3" t="n">
-        <v>121.1606</v>
+        <v>113.4756</v>
       </c>
       <c r="E3" t="n">
-        <v>125.7875</v>
+        <v>115.6842</v>
       </c>
       <c r="F3" t="n">
-        <v>71.4119</v>
+        <v>68.767</v>
       </c>
       <c r="G3" t="n">
-        <v>72.41</v>
+        <v>70.0945</v>
       </c>
       <c r="H3" t="n">
-        <v>70.7033</v>
+        <v>68.5474</v>
       </c>
       <c r="I3" t="n">
-        <v>71.4119</v>
+        <v>69.07640000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>44.2471</v>
+        <v>45.9459</v>
       </c>
       <c r="K3" t="n">
-        <v>44.2669</v>
+        <v>46.9039</v>
       </c>
       <c r="L3" t="n">
-        <v>41.7977</v>
+        <v>44.9385</v>
       </c>
       <c r="M3" t="n">
-        <v>42.7064</v>
+        <v>46.1632</v>
       </c>
       <c r="N3" t="n">
-        <v>38.0889</v>
+        <v>39.5186</v>
       </c>
       <c r="O3" t="n">
-        <v>38.4636</v>
+        <v>39.6271</v>
       </c>
       <c r="P3" t="n">
-        <v>37.5664</v>
+        <v>38.7988</v>
       </c>
       <c r="Q3" t="n">
-        <v>38.0988</v>
+        <v>39.3411</v>
       </c>
       <c r="R3" t="n">
-        <v>2.1092</v>
+        <v>-8.032</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.8453000000000001</v>
+        <v>-3.2705</v>
       </c>
       <c r="X3" t="n">
-        <v>-1.9055</v>
+        <v>8.0943</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.8615</v>
+        <v>3.2607</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>116.2738</v>
+        <v>120.6309</v>
       </c>
       <c r="C4" t="n">
-        <v>119.2418</v>
+        <v>124.4184</v>
       </c>
       <c r="D4" t="n">
-        <v>113.4756</v>
+        <v>117.7928</v>
       </c>
       <c r="E4" t="n">
-        <v>115.6842</v>
+        <v>121.7402</v>
       </c>
       <c r="F4" t="n">
-        <v>68.767</v>
+        <v>71.0526</v>
       </c>
       <c r="G4" t="n">
-        <v>70.0945</v>
+        <v>71.6215</v>
       </c>
       <c r="H4" t="n">
-        <v>68.5474</v>
+        <v>70.47369999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>69.07640000000001</v>
+        <v>70.843</v>
       </c>
       <c r="J4" t="n">
-        <v>45.9459</v>
+        <v>44.1385</v>
       </c>
       <c r="K4" t="n">
-        <v>46.9039</v>
+        <v>45.2545</v>
       </c>
       <c r="L4" t="n">
-        <v>44.9385</v>
+        <v>42.5879</v>
       </c>
       <c r="M4" t="n">
-        <v>46.1632</v>
+        <v>43.5953</v>
       </c>
       <c r="N4" t="n">
-        <v>39.5186</v>
+        <v>38.227</v>
       </c>
       <c r="O4" t="n">
-        <v>39.6271</v>
+        <v>38.5523</v>
       </c>
       <c r="P4" t="n">
-        <v>38.7988</v>
+        <v>37.8819</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.3411</v>
+        <v>38.3256</v>
       </c>
       <c r="R4" t="n">
-        <v>-8.032</v>
+        <v>5.2349</v>
       </c>
       <c r="U4" t="n">
-        <v>-3.2705</v>
+        <v>2.5575</v>
       </c>
       <c r="X4" t="n">
-        <v>8.0943</v>
+        <v>-5.5627</v>
       </c>
       <c r="AA4" t="n">
-        <v>3.2607</v>
+        <v>-2.5813</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120.6309</v>
+        <v>101.4635</v>
       </c>
       <c r="C5" t="n">
-        <v>124.4184</v>
+        <v>105.3209</v>
       </c>
       <c r="D5" t="n">
-        <v>117.7928</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>121.7402</v>
+        <v>101.0637</v>
       </c>
       <c r="F5" t="n">
-        <v>71.0526</v>
+        <v>67.3997</v>
       </c>
       <c r="G5" t="n">
-        <v>71.6215</v>
+        <v>70.25409999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>70.47369999999999</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>70.843</v>
+        <v>69.13630000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>44.1385</v>
+        <v>50.9731</v>
       </c>
       <c r="K5" t="n">
-        <v>45.2545</v>
+        <v>51.5756</v>
       </c>
       <c r="L5" t="n">
-        <v>42.5879</v>
+        <v>49.5904</v>
       </c>
       <c r="M5" t="n">
-        <v>43.5953</v>
+        <v>51.0916</v>
       </c>
       <c r="N5" t="n">
-        <v>38.227</v>
+        <v>40.2088</v>
       </c>
       <c r="O5" t="n">
-        <v>38.5523</v>
+        <v>40.3074</v>
       </c>
       <c r="P5" t="n">
-        <v>37.8819</v>
+        <v>38.6608</v>
       </c>
       <c r="Q5" t="n">
-        <v>38.3256</v>
+        <v>39.2721</v>
       </c>
       <c r="R5" t="n">
-        <v>5.2349</v>
+        <v>-16.9841</v>
       </c>
       <c r="S5" t="n">
-        <v>-1.1762</v>
+        <v>-19.6552</v>
       </c>
       <c r="U5" t="n">
-        <v>2.5575</v>
+        <v>-2.4091</v>
       </c>
       <c r="V5" t="n">
-        <v>-1.6352</v>
+        <v>-3.1866</v>
       </c>
       <c r="X5" t="n">
-        <v>-5.5627</v>
+        <v>17.1952</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.1362</v>
+        <v>19.6345</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.5813</v>
+        <v>2.4696</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.4619</v>
+        <v>3.0796</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>101.4635</v>
+        <v>104.4815</v>
       </c>
       <c r="C6" t="n">
-        <v>105.3209</v>
+        <v>105.8706</v>
       </c>
       <c r="D6" t="n">
-        <v>99.80459999999999</v>
+        <v>100.8938</v>
       </c>
       <c r="E6" t="n">
-        <v>101.0637</v>
+        <v>102.253</v>
       </c>
       <c r="F6" t="n">
-        <v>67.3997</v>
+        <v>68.9966</v>
       </c>
       <c r="G6" t="n">
-        <v>70.25409999999999</v>
+        <v>69.1962</v>
       </c>
       <c r="H6" t="n">
-        <v>67.20999999999999</v>
+        <v>67.4795</v>
       </c>
       <c r="I6" t="n">
-        <v>69.13630000000001</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>50.9731</v>
+        <v>49.2546</v>
       </c>
       <c r="K6" t="n">
-        <v>51.5756</v>
+        <v>51.1607</v>
       </c>
       <c r="L6" t="n">
-        <v>49.5904</v>
+        <v>48.6521</v>
       </c>
       <c r="M6" t="n">
-        <v>51.0916</v>
+        <v>50.4694</v>
       </c>
       <c r="N6" t="n">
+        <v>39.351</v>
+      </c>
+      <c r="O6" t="n">
         <v>40.2088</v>
       </c>
-      <c r="O6" t="n">
-        <v>40.3074</v>
-      </c>
       <c r="P6" t="n">
-        <v>38.6608</v>
+        <v>39.2327</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.2721</v>
+        <v>40.0511</v>
       </c>
       <c r="R6" t="n">
-        <v>-16.9841</v>
+        <v>1.1768</v>
       </c>
       <c r="S6" t="n">
-        <v>-19.6552</v>
+        <v>-11.6102</v>
       </c>
       <c r="U6" t="n">
-        <v>-2.4091</v>
+        <v>-1.9777</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.1866</v>
+        <v>-1.8927</v>
       </c>
       <c r="X6" t="n">
-        <v>17.1952</v>
+        <v>-1.2178</v>
       </c>
       <c r="Y6" t="n">
-        <v>19.6345</v>
+        <v>9.328200000000001</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.4696</v>
+        <v>1.9836</v>
       </c>
       <c r="AB6" t="n">
-        <v>3.0796</v>
+        <v>1.8047</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>104.4815</v>
+        <v>107.3696</v>
       </c>
       <c r="C7" t="n">
-        <v>105.8706</v>
+        <v>109.2484</v>
       </c>
       <c r="D7" t="n">
-        <v>100.8938</v>
+        <v>100.9938</v>
       </c>
       <c r="E7" t="n">
-        <v>102.253</v>
+        <v>103.9019</v>
       </c>
       <c r="F7" t="n">
-        <v>68.9966</v>
+        <v>68.7171</v>
       </c>
       <c r="G7" t="n">
-        <v>69.1962</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>67.4795</v>
+        <v>66.4216</v>
       </c>
       <c r="I7" t="n">
-        <v>67.76900000000001</v>
+        <v>67.7989</v>
       </c>
       <c r="J7" t="n">
-        <v>49.2546</v>
+        <v>47.9509</v>
       </c>
       <c r="K7" t="n">
-        <v>51.1607</v>
+        <v>51.1015</v>
       </c>
       <c r="L7" t="n">
-        <v>48.6521</v>
+        <v>46.9829</v>
       </c>
       <c r="M7" t="n">
-        <v>50.4694</v>
+        <v>49.4916</v>
       </c>
       <c r="N7" t="n">
-        <v>39.351</v>
+        <v>39.4989</v>
       </c>
       <c r="O7" t="n">
-        <v>40.2088</v>
+        <v>40.8596</v>
       </c>
       <c r="P7" t="n">
-        <v>39.2327</v>
+        <v>38.8186</v>
       </c>
       <c r="Q7" t="n">
-        <v>40.0511</v>
+        <v>40.0412</v>
       </c>
       <c r="R7" t="n">
-        <v>1.1768</v>
+        <v>1.6126</v>
       </c>
       <c r="S7" t="n">
-        <v>-11.6102</v>
+        <v>-14.6528</v>
       </c>
       <c r="T7" t="n">
-        <v>-16.9952</v>
+        <v>-17.3989</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.9777</v>
+        <v>0.0441</v>
       </c>
       <c r="V7" t="n">
-        <v>-1.8927</v>
+        <v>-4.297</v>
       </c>
       <c r="W7" t="n">
-        <v>-5.9034</v>
+        <v>-5.0594</v>
       </c>
       <c r="X7" t="n">
-        <v>-1.2178</v>
+        <v>-1.9374</v>
       </c>
       <c r="Y7" t="n">
-        <v>9.328200000000001</v>
+        <v>13.5251</v>
       </c>
       <c r="Z7" t="n">
-        <v>15.9257</v>
+        <v>15.888</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.9836</v>
+        <v>-0.0247</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.8047</v>
+        <v>4.4764</v>
       </c>
       <c r="AC7" t="n">
-        <v>6.0299</v>
+        <v>5.0983</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>107.3696</v>
+        <v>113.2557</v>
       </c>
       <c r="C8" t="n">
-        <v>109.2484</v>
+        <v>115.4043</v>
       </c>
       <c r="D8" t="n">
-        <v>100.9938</v>
+        <v>111.9366</v>
       </c>
       <c r="E8" t="n">
-        <v>103.9019</v>
+        <v>114.7448</v>
       </c>
       <c r="F8" t="n">
-        <v>68.7171</v>
+        <v>70.9927</v>
       </c>
       <c r="G8" t="n">
-        <v>69.83499999999999</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>66.4216</v>
+        <v>70.2342</v>
       </c>
       <c r="I8" t="n">
-        <v>67.7989</v>
+        <v>71.2422</v>
       </c>
       <c r="J8" t="n">
-        <v>47.9509</v>
+        <v>45.1558</v>
       </c>
       <c r="K8" t="n">
-        <v>51.1015</v>
+        <v>45.7681</v>
       </c>
       <c r="L8" t="n">
-        <v>46.9829</v>
+        <v>44.1187</v>
       </c>
       <c r="M8" t="n">
-        <v>49.4916</v>
+        <v>44.4348</v>
       </c>
       <c r="N8" t="n">
-        <v>39.4989</v>
+        <v>38.1481</v>
       </c>
       <c r="O8" t="n">
-        <v>40.8596</v>
+        <v>38.5918</v>
       </c>
       <c r="P8" t="n">
-        <v>38.8186</v>
+        <v>37.7931</v>
       </c>
       <c r="Q8" t="n">
-        <v>40.0412</v>
+        <v>37.9903</v>
       </c>
       <c r="R8" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="S8" t="n">
-        <v>-14.6528</v>
+        <v>13.5371</v>
       </c>
       <c r="T8" t="n">
-        <v>-17.3989</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0441</v>
+        <v>5.0787</v>
       </c>
       <c r="V8" t="n">
-        <v>-4.297</v>
+        <v>3.046</v>
       </c>
       <c r="W8" t="n">
-        <v>-5.0594</v>
+        <v>3.1354</v>
       </c>
       <c r="X8" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y8" t="n">
-        <v>13.5251</v>
+        <v>-13.0291</v>
       </c>
       <c r="Z8" t="n">
-        <v>15.888</v>
+        <v>-3.7441</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.0247</v>
+        <v>-5.122</v>
       </c>
       <c r="AB8" t="n">
-        <v>4.4764</v>
+        <v>-3.2639</v>
       </c>
       <c r="AC8" t="n">
-        <v>5.0983</v>
+        <v>-3.4336</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>113.2557</v>
+        <v>116.9533</v>
       </c>
       <c r="C9" t="n">
-        <v>115.4043</v>
+        <v>123.8188</v>
       </c>
       <c r="D9" t="n">
-        <v>111.9366</v>
+        <v>116.6035</v>
       </c>
       <c r="E9" t="n">
-        <v>114.7448</v>
+        <v>123.589</v>
       </c>
       <c r="F9" t="n">
-        <v>70.9927</v>
+        <v>71.7812</v>
       </c>
       <c r="G9" t="n">
-        <v>71.58159999999999</v>
+        <v>72.6395</v>
       </c>
       <c r="H9" t="n">
-        <v>70.2342</v>
+        <v>70.6733</v>
       </c>
       <c r="I9" t="n">
-        <v>71.2422</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>45.1558</v>
+        <v>43.5656</v>
       </c>
       <c r="K9" t="n">
-        <v>45.7681</v>
+        <v>43.7138</v>
       </c>
       <c r="L9" t="n">
-        <v>44.1187</v>
+        <v>40.9582</v>
       </c>
       <c r="M9" t="n">
-        <v>44.4348</v>
+        <v>40.978</v>
       </c>
       <c r="N9" t="n">
-        <v>38.1481</v>
+        <v>37.7241</v>
       </c>
       <c r="O9" t="n">
-        <v>38.5918</v>
+        <v>38.3256</v>
       </c>
       <c r="P9" t="n">
-        <v>37.7931</v>
+        <v>37.2706</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.9903</v>
+        <v>37.3396</v>
       </c>
       <c r="R9" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="S9" t="n">
-        <v>13.5371</v>
+        <v>20.8659</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.8120000000000001</v>
+        <v>1.5186</v>
       </c>
       <c r="U9" t="n">
-        <v>5.0787</v>
+        <v>1.7652</v>
       </c>
       <c r="V9" t="n">
-        <v>3.046</v>
+        <v>6.9808</v>
       </c>
       <c r="W9" t="n">
-        <v>3.1354</v>
+        <v>2.3387</v>
       </c>
       <c r="X9" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y9" t="n">
-        <v>-13.0291</v>
+        <v>-18.8062</v>
       </c>
       <c r="Z9" t="n">
-        <v>-3.7441</v>
+        <v>-6.0036</v>
       </c>
       <c r="AA9" t="n">
-        <v>-5.122</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3.2639</v>
+        <v>-6.7701</v>
       </c>
       <c r="AC9" t="n">
-        <v>-3.4336</v>
+        <v>-2.5727</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>116.9533</v>
+        <v>131.9835</v>
       </c>
       <c r="C10" t="n">
-        <v>123.8188</v>
+        <v>143.9056</v>
       </c>
       <c r="D10" t="n">
-        <v>116.6035</v>
+        <v>129.5351</v>
       </c>
       <c r="E10" t="n">
-        <v>123.589</v>
+        <v>141.837</v>
       </c>
       <c r="F10" t="n">
-        <v>71.7812</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>72.6395</v>
+        <v>79.3366</v>
       </c>
       <c r="H10" t="n">
-        <v>70.6733</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>72.49979999999999</v>
+        <v>78.7577</v>
       </c>
       <c r="J10" t="n">
-        <v>43.5656</v>
+        <v>38.2718</v>
       </c>
       <c r="K10" t="n">
-        <v>43.7138</v>
+        <v>39.0224</v>
       </c>
       <c r="L10" t="n">
-        <v>40.9582</v>
+        <v>34.252</v>
       </c>
       <c r="M10" t="n">
-        <v>40.978</v>
+        <v>34.894</v>
       </c>
       <c r="N10" t="n">
-        <v>37.7241</v>
+        <v>36.2155</v>
       </c>
       <c r="O10" t="n">
-        <v>38.3256</v>
+        <v>36.2254</v>
       </c>
       <c r="P10" t="n">
-        <v>37.2706</v>
+        <v>33.8294</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.3396</v>
+        <v>34.1154</v>
       </c>
       <c r="R10" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="S10" t="n">
-        <v>20.8659</v>
+        <v>36.5105</v>
       </c>
       <c r="T10" t="n">
-        <v>1.5186</v>
+        <v>40.3442</v>
       </c>
       <c r="U10" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>6.9808</v>
+        <v>16.1637</v>
       </c>
       <c r="W10" t="n">
-        <v>2.3387</v>
+        <v>13.9166</v>
       </c>
       <c r="X10" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="Y10" t="n">
-        <v>-18.8062</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z10" t="n">
-        <v>-6.0036</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.7128</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.7701</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC10" t="n">
-        <v>-2.5727</v>
+        <v>-13.1307</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C11" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D11" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E11" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F11" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>79.3366</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>78.7577</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K11" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L11" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M11" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N11" t="n">
-        <v>36.2155</v>
+        <v>34.1745</v>
       </c>
       <c r="O11" t="n">
-        <v>36.2254</v>
+        <v>34.1745</v>
       </c>
       <c r="P11" t="n">
-        <v>33.8294</v>
+        <v>33.1688</v>
       </c>
       <c r="Q11" t="n">
-        <v>34.1154</v>
+        <v>33.297</v>
       </c>
       <c r="R11" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S11" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="T11" t="n">
-        <v>40.3442</v>
+        <v>48.602</v>
       </c>
       <c r="U11" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V11" t="n">
-        <v>16.1637</v>
+        <v>13.2391</v>
       </c>
       <c r="W11" t="n">
-        <v>13.9166</v>
+        <v>19.0426</v>
       </c>
       <c r="X11" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y11" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z11" t="n">
-        <v>-31.7031</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA11" t="n">
-        <v>-8.6348</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB11" t="n">
-        <v>-14.7993</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC11" t="n">
-        <v>-13.1307</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C12" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D12" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E12" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F12" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G12" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I12" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J12" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K12" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L12" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M12" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N12" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O12" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P12" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q12" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
       <c r="R12" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="S12" t="n">
-        <v>32.4243</v>
+        <v>18.3358</v>
       </c>
       <c r="T12" t="n">
-        <v>48.602</v>
+        <v>40.7578</v>
       </c>
       <c r="U12" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="V12" t="n">
-        <v>13.2391</v>
+        <v>8.4969</v>
       </c>
       <c r="W12" t="n">
-        <v>19.0426</v>
+        <v>16.0196</v>
       </c>
       <c r="X12" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="Y12" t="n">
-        <v>-27.0392</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z12" t="n">
-        <v>-35.7631</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.3989</v>
+        <v>2.5318</v>
       </c>
       <c r="AB12" t="n">
-        <v>-12.3539</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC12" t="n">
-        <v>-16.8637</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C13" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D13" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E13" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F13" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G13" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I13" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J13" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K13" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L13" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M13" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N13" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O13" t="n">
         <v>35.06</v>
       </c>
-      <c r="L13" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M13" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N13" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O13" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P13" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q13" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R13" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="S13" t="n">
-        <v>18.3358</v>
+        <v>3.1677</v>
       </c>
       <c r="T13" t="n">
-        <v>40.7578</v>
+        <v>27.5265</v>
       </c>
       <c r="U13" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="V13" t="n">
-        <v>8.4969</v>
+        <v>-0.2256</v>
       </c>
       <c r="W13" t="n">
-        <v>16.0196</v>
+        <v>10.2998</v>
       </c>
       <c r="X13" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y13" t="n">
-        <v>-17.8584</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z13" t="n">
-        <v>-31.9885</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA13" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
       <c r="AB13" t="n">
-        <v>-8.568899999999999</v>
+        <v>0.1894</v>
       </c>
       <c r="AC13" t="n">
-        <v>-14.7378</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C14" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D14" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E14" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F14" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G14" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H14" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I14" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K14" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L14" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M14" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N14" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O14" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P14" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q14" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R14" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="S14" t="n">
-        <v>3.1677</v>
+        <v>-0.3291</v>
       </c>
       <c r="T14" t="n">
-        <v>27.5265</v>
+        <v>22.5433</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.2256</v>
+        <v>-1.3313</v>
       </c>
       <c r="W14" t="n">
-        <v>10.2998</v>
+        <v>9.7934</v>
       </c>
       <c r="X14" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y14" t="n">
-        <v>-3.6224</v>
+        <v>0.0308</v>
       </c>
       <c r="Z14" t="n">
-        <v>-24.3161</v>
+        <v>-20.86</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.1894</v>
+        <v>1.3605</v>
       </c>
       <c r="AC14" t="n">
-        <v>-10.0297</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C15" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D15" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E15" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F15" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I15" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K15" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L15" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M15" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N15" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O15" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P15" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q15" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R15" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.3291</v>
+        <v>-2.7077</v>
       </c>
       <c r="T15" t="n">
-        <v>22.5433</v>
+        <v>0.3194</v>
       </c>
       <c r="U15" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="V15" t="n">
-        <v>-1.3313</v>
+        <v>-2.0595</v>
       </c>
       <c r="W15" t="n">
-        <v>9.7934</v>
+        <v>-2.181</v>
       </c>
       <c r="X15" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.0308</v>
+        <v>2.2876</v>
       </c>
       <c r="Z15" t="n">
-        <v>-20.86</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.3605</v>
+        <v>2.0211</v>
       </c>
       <c r="AC15" t="n">
-        <v>-9.6134</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C16" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D16" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E16" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F16" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G16" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I16" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K16" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L16" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M16" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N16" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O16" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P16" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q16" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R16" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S16" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="T16" t="n">
-        <v>0.3194</v>
+        <v>-3.2577</v>
       </c>
       <c r="U16" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V16" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="W16" t="n">
-        <v>-2.181</v>
+        <v>-3.9839</v>
       </c>
       <c r="X16" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y16" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z16" t="n">
-        <v>-1.3297</v>
+        <v>2.591</v>
       </c>
       <c r="AA16" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB16" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
       <c r="AC16" t="n">
-        <v>2.0947</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C17" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D17" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E17" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F17" t="n">
         <v>78.13</v>
       </c>
       <c r="G17" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I17" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J17" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K17" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L17" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M17" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N17" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O17" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P17" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q17" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R17" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S17" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="T17" t="n">
-        <v>-3.2577</v>
+        <v>1.1009</v>
       </c>
       <c r="U17" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V17" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="W17" t="n">
-        <v>-3.9839</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X17" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y17" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="Z17" t="n">
-        <v>2.591</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
       <c r="AC17" t="n">
-        <v>4.0935</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C18" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D18" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E18" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F18" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G18" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H18" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I18" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J18" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K18" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L18" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M18" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N18" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O18" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P18" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q18" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R18" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S18" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T18" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U18" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V18" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W18" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X18" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y18" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z18" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA18" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C19" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D19" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E19" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F19" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G19" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H19" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I19" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K19" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L19" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M19" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N19" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O19" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P19" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q19" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R19" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S19" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T19" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U19" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V19" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W19" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X19" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y19" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z19" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA19" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB19" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC19" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C20" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D20" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E20" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F20" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G20" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H20" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J20" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K20" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L20" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M20" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N20" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O20" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P20" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q20" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R20" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S20" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T20" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U20" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V20" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W20" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X20" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y20" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z20" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA20" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB20" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC20" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C21" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D21" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E21" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F21" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I21" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J21" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K21" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L21" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M21" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N21" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O21" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P21" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q21" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R21" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S21" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T21" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U21" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V21" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W21" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X21" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y21" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z21" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA21" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC21" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C22" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D22" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E22" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F22" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H22" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J22" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K22" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L22" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M22" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N22" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O22" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P22" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q22" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R22" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S22" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T22" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U22" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V22" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W22" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X22" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y22" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z22" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA22" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB22" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC22" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C23" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D23" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E23" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F23" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G23" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I23" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J23" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K23" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L23" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M23" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N23" t="n">
         <v>32.58</v>
       </c>
       <c r="O23" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P23" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q23" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R23" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S23" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T23" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U23" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V23" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W23" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X23" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y23" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z23" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA23" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB23" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC23" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-13 02:51
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1895 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>121.1606</v>
+        <v>101.4635</v>
       </c>
       <c r="C2" t="n">
-        <v>128.3958</v>
+        <v>105.3209</v>
       </c>
       <c r="D2" t="n">
-        <v>121.1606</v>
+        <v>99.80459999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>125.7875</v>
+        <v>101.0637</v>
       </c>
       <c r="F2" t="n">
-        <v>71.4119</v>
+        <v>67.3997</v>
       </c>
       <c r="G2" t="n">
-        <v>72.41</v>
+        <v>70.25409999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>70.7033</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>71.4119</v>
+        <v>69.13630000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>44.2471</v>
+        <v>50.9731</v>
       </c>
       <c r="K2" t="n">
-        <v>44.2669</v>
+        <v>51.5756</v>
       </c>
       <c r="L2" t="n">
-        <v>41.7977</v>
+        <v>49.5904</v>
       </c>
       <c r="M2" t="n">
-        <v>42.7064</v>
+        <v>51.0916</v>
       </c>
       <c r="N2" t="n">
-        <v>38.0889</v>
+        <v>40.2088</v>
       </c>
       <c r="O2" t="n">
-        <v>38.4636</v>
+        <v>40.3074</v>
       </c>
       <c r="P2" t="n">
-        <v>37.5664</v>
+        <v>38.6608</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.0988</v>
+        <v>39.2721</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>116.2738</v>
+        <v>104.4815</v>
       </c>
       <c r="C3" t="n">
-        <v>119.2418</v>
+        <v>105.8706</v>
       </c>
       <c r="D3" t="n">
-        <v>113.4756</v>
+        <v>100.8938</v>
       </c>
       <c r="E3" t="n">
-        <v>115.6842</v>
+        <v>102.253</v>
       </c>
       <c r="F3" t="n">
-        <v>68.767</v>
+        <v>68.9966</v>
       </c>
       <c r="G3" t="n">
-        <v>70.0945</v>
+        <v>69.1962</v>
       </c>
       <c r="H3" t="n">
-        <v>68.5474</v>
+        <v>67.4795</v>
       </c>
       <c r="I3" t="n">
-        <v>69.07640000000001</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>45.9459</v>
+        <v>49.2546</v>
       </c>
       <c r="K3" t="n">
-        <v>46.9039</v>
+        <v>51.1607</v>
       </c>
       <c r="L3" t="n">
-        <v>44.9385</v>
+        <v>48.6521</v>
       </c>
       <c r="M3" t="n">
-        <v>46.1632</v>
+        <v>50.4694</v>
       </c>
       <c r="N3" t="n">
-        <v>39.5186</v>
+        <v>39.351</v>
       </c>
       <c r="O3" t="n">
-        <v>39.6271</v>
+        <v>40.2088</v>
       </c>
       <c r="P3" t="n">
-        <v>38.7988</v>
+        <v>39.2327</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.3411</v>
+        <v>40.0511</v>
       </c>
       <c r="R3" t="n">
-        <v>-8.032</v>
+        <v>1.1768</v>
       </c>
       <c r="U3" t="n">
-        <v>-3.2705</v>
+        <v>-1.9777</v>
       </c>
       <c r="X3" t="n">
-        <v>8.0943</v>
+        <v>-1.2178</v>
       </c>
       <c r="AA3" t="n">
-        <v>3.2607</v>
+        <v>1.9836</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>120.6309</v>
+        <v>107.3696</v>
       </c>
       <c r="C4" t="n">
-        <v>124.4184</v>
+        <v>109.2484</v>
       </c>
       <c r="D4" t="n">
-        <v>117.7928</v>
+        <v>100.9938</v>
       </c>
       <c r="E4" t="n">
-        <v>121.7402</v>
+        <v>103.9019</v>
       </c>
       <c r="F4" t="n">
-        <v>71.0526</v>
+        <v>68.7171</v>
       </c>
       <c r="G4" t="n">
-        <v>71.6215</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>70.47369999999999</v>
+        <v>66.4216</v>
       </c>
       <c r="I4" t="n">
-        <v>70.843</v>
+        <v>67.7989</v>
       </c>
       <c r="J4" t="n">
-        <v>44.1385</v>
+        <v>47.9509</v>
       </c>
       <c r="K4" t="n">
-        <v>45.2545</v>
+        <v>51.1015</v>
       </c>
       <c r="L4" t="n">
-        <v>42.5879</v>
+        <v>46.9829</v>
       </c>
       <c r="M4" t="n">
-        <v>43.5953</v>
+        <v>49.4916</v>
       </c>
       <c r="N4" t="n">
-        <v>38.227</v>
+        <v>39.4989</v>
       </c>
       <c r="O4" t="n">
-        <v>38.5523</v>
+        <v>40.8596</v>
       </c>
       <c r="P4" t="n">
-        <v>37.8819</v>
+        <v>38.8186</v>
       </c>
       <c r="Q4" t="n">
-        <v>38.3256</v>
+        <v>40.0412</v>
       </c>
       <c r="R4" t="n">
-        <v>5.2349</v>
+        <v>1.6126</v>
       </c>
       <c r="U4" t="n">
-        <v>2.5575</v>
+        <v>0.0441</v>
       </c>
       <c r="X4" t="n">
-        <v>-5.5627</v>
+        <v>-1.9374</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.5813</v>
+        <v>-0.0247</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>101.4635</v>
+        <v>113.2557</v>
       </c>
       <c r="C5" t="n">
-        <v>105.3209</v>
+        <v>115.4043</v>
       </c>
       <c r="D5" t="n">
-        <v>99.80459999999999</v>
+        <v>111.9366</v>
       </c>
       <c r="E5" t="n">
-        <v>101.0637</v>
+        <v>114.7448</v>
       </c>
       <c r="F5" t="n">
-        <v>67.3997</v>
+        <v>70.9927</v>
       </c>
       <c r="G5" t="n">
-        <v>70.25409999999999</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>67.20999999999999</v>
+        <v>70.2342</v>
       </c>
       <c r="I5" t="n">
-        <v>69.13630000000001</v>
+        <v>71.2422</v>
       </c>
       <c r="J5" t="n">
-        <v>50.9731</v>
+        <v>45.1558</v>
       </c>
       <c r="K5" t="n">
-        <v>51.5756</v>
+        <v>45.7681</v>
       </c>
       <c r="L5" t="n">
-        <v>49.5904</v>
+        <v>44.1187</v>
       </c>
       <c r="M5" t="n">
-        <v>51.0916</v>
+        <v>44.4348</v>
       </c>
       <c r="N5" t="n">
-        <v>40.2088</v>
+        <v>38.1481</v>
       </c>
       <c r="O5" t="n">
-        <v>40.3074</v>
+        <v>38.5918</v>
       </c>
       <c r="P5" t="n">
-        <v>38.6608</v>
+        <v>37.7931</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.2721</v>
+        <v>37.9903</v>
       </c>
       <c r="R5" t="n">
-        <v>-16.9841</v>
+        <v>10.4357</v>
       </c>
       <c r="S5" t="n">
-        <v>-19.6552</v>
+        <v>13.5371</v>
       </c>
       <c r="U5" t="n">
-        <v>-2.4091</v>
+        <v>5.0787</v>
       </c>
       <c r="V5" t="n">
-        <v>-3.1866</v>
+        <v>3.046</v>
       </c>
       <c r="X5" t="n">
-        <v>17.1952</v>
+        <v>-10.2175</v>
       </c>
       <c r="Y5" t="n">
-        <v>19.6345</v>
+        <v>-13.0291</v>
       </c>
       <c r="AA5" t="n">
-        <v>2.4696</v>
+        <v>-5.122</v>
       </c>
       <c r="AB5" t="n">
-        <v>3.0796</v>
+        <v>-3.2639</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>104.4815</v>
+        <v>116.9533</v>
       </c>
       <c r="C6" t="n">
-        <v>105.8706</v>
+        <v>123.8188</v>
       </c>
       <c r="D6" t="n">
-        <v>100.8938</v>
+        <v>116.6035</v>
       </c>
       <c r="E6" t="n">
-        <v>102.253</v>
+        <v>123.589</v>
       </c>
       <c r="F6" t="n">
-        <v>68.9966</v>
+        <v>71.7812</v>
       </c>
       <c r="G6" t="n">
-        <v>69.1962</v>
+        <v>72.6395</v>
       </c>
       <c r="H6" t="n">
-        <v>67.4795</v>
+        <v>70.6733</v>
       </c>
       <c r="I6" t="n">
-        <v>67.76900000000001</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>49.2546</v>
+        <v>43.5656</v>
       </c>
       <c r="K6" t="n">
-        <v>51.1607</v>
+        <v>43.7138</v>
       </c>
       <c r="L6" t="n">
-        <v>48.6521</v>
+        <v>40.9582</v>
       </c>
       <c r="M6" t="n">
-        <v>50.4694</v>
+        <v>40.978</v>
       </c>
       <c r="N6" t="n">
-        <v>39.351</v>
+        <v>37.7241</v>
       </c>
       <c r="O6" t="n">
-        <v>40.2088</v>
+        <v>38.3256</v>
       </c>
       <c r="P6" t="n">
-        <v>39.2327</v>
+        <v>37.2706</v>
       </c>
       <c r="Q6" t="n">
-        <v>40.0511</v>
+        <v>37.3396</v>
       </c>
       <c r="R6" t="n">
-        <v>1.1768</v>
+        <v>7.7077</v>
       </c>
       <c r="S6" t="n">
-        <v>-11.6102</v>
+        <v>20.8659</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.9777</v>
+        <v>1.7652</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.8927</v>
+        <v>6.9808</v>
       </c>
       <c r="X6" t="n">
-        <v>-1.2178</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y6" t="n">
-        <v>9.328200000000001</v>
+        <v>-18.8062</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.9836</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.8047</v>
+        <v>-6.7701</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>107.3696</v>
+        <v>131.9835</v>
       </c>
       <c r="C7" t="n">
-        <v>109.2484</v>
+        <v>143.9056</v>
       </c>
       <c r="D7" t="n">
-        <v>100.9938</v>
+        <v>129.5351</v>
       </c>
       <c r="E7" t="n">
-        <v>103.9019</v>
+        <v>141.837</v>
       </c>
       <c r="F7" t="n">
-        <v>68.7171</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>69.83499999999999</v>
+        <v>79.3366</v>
       </c>
       <c r="H7" t="n">
-        <v>66.4216</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>67.7989</v>
+        <v>78.7577</v>
       </c>
       <c r="J7" t="n">
-        <v>47.9509</v>
+        <v>38.2718</v>
       </c>
       <c r="K7" t="n">
-        <v>51.1015</v>
+        <v>39.0224</v>
       </c>
       <c r="L7" t="n">
-        <v>46.9829</v>
+        <v>34.252</v>
       </c>
       <c r="M7" t="n">
-        <v>49.4916</v>
+        <v>34.894</v>
       </c>
       <c r="N7" t="n">
-        <v>39.4989</v>
+        <v>36.2155</v>
       </c>
       <c r="O7" t="n">
-        <v>40.8596</v>
+        <v>36.2254</v>
       </c>
       <c r="P7" t="n">
-        <v>38.8186</v>
+        <v>33.8294</v>
       </c>
       <c r="Q7" t="n">
-        <v>40.0412</v>
+        <v>34.1154</v>
       </c>
       <c r="R7" t="n">
-        <v>1.6126</v>
+        <v>14.7651</v>
       </c>
       <c r="S7" t="n">
-        <v>-14.6528</v>
+        <v>36.5105</v>
       </c>
       <c r="T7" t="n">
-        <v>-17.3989</v>
+        <v>40.3442</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0441</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V7" t="n">
-        <v>-4.297</v>
+        <v>16.1637</v>
       </c>
       <c r="W7" t="n">
-        <v>-5.0594</v>
+        <v>13.9166</v>
       </c>
       <c r="X7" t="n">
-        <v>-1.9374</v>
+        <v>-14.847</v>
       </c>
       <c r="Y7" t="n">
-        <v>13.5251</v>
+        <v>-29.4951</v>
       </c>
       <c r="Z7" t="n">
-        <v>15.888</v>
+        <v>-31.7031</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.0247</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB7" t="n">
-        <v>4.4764</v>
+        <v>-14.7993</v>
       </c>
       <c r="AC7" t="n">
-        <v>5.0983</v>
+        <v>-13.1307</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>113.2557</v>
+        <v>137.67</v>
       </c>
       <c r="C8" t="n">
-        <v>115.4043</v>
+        <v>152.64</v>
       </c>
       <c r="D8" t="n">
-        <v>111.9366</v>
+        <v>137.46</v>
       </c>
       <c r="E8" t="n">
-        <v>114.7448</v>
+        <v>151.95</v>
       </c>
       <c r="F8" t="n">
-        <v>70.9927</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>71.58159999999999</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>70.2342</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>71.2422</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>45.1558</v>
+        <v>35.98</v>
       </c>
       <c r="K8" t="n">
-        <v>45.7681</v>
+        <v>36.01</v>
       </c>
       <c r="L8" t="n">
-        <v>44.1187</v>
+        <v>32.25</v>
       </c>
       <c r="M8" t="n">
-        <v>44.4348</v>
+        <v>32.42</v>
       </c>
       <c r="N8" t="n">
-        <v>38.1481</v>
+        <v>34.1745</v>
       </c>
       <c r="O8" t="n">
-        <v>38.5918</v>
+        <v>34.1745</v>
       </c>
       <c r="P8" t="n">
-        <v>37.7931</v>
+        <v>33.1688</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.9903</v>
+        <v>33.297</v>
       </c>
       <c r="R8" t="n">
-        <v>10.4357</v>
+        <v>7.13</v>
       </c>
       <c r="S8" t="n">
-        <v>13.5371</v>
+        <v>32.4243</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.8120000000000001</v>
+        <v>48.602</v>
       </c>
       <c r="U8" t="n">
-        <v>5.0787</v>
+        <v>2.4332</v>
       </c>
       <c r="V8" t="n">
-        <v>3.046</v>
+        <v>13.2391</v>
       </c>
       <c r="W8" t="n">
-        <v>3.1354</v>
+        <v>19.0426</v>
       </c>
       <c r="X8" t="n">
-        <v>-10.2175</v>
+        <v>-7.09</v>
       </c>
       <c r="Y8" t="n">
-        <v>-13.0291</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z8" t="n">
-        <v>-3.7441</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA8" t="n">
-        <v>-5.122</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB8" t="n">
-        <v>-3.2639</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC8" t="n">
-        <v>-3.4336</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>116.9533</v>
+        <v>149.89</v>
       </c>
       <c r="C9" t="n">
-        <v>123.8188</v>
+        <v>151</v>
       </c>
       <c r="D9" t="n">
-        <v>116.6035</v>
+        <v>139.58</v>
       </c>
       <c r="E9" t="n">
-        <v>123.589</v>
+        <v>146.25</v>
       </c>
       <c r="F9" t="n">
-        <v>71.7812</v>
+        <v>80.53</v>
       </c>
       <c r="G9" t="n">
-        <v>72.6395</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>70.6733</v>
+        <v>77.69</v>
       </c>
       <c r="I9" t="n">
-        <v>72.49979999999999</v>
+        <v>78.66</v>
       </c>
       <c r="J9" t="n">
-        <v>43.5656</v>
+        <v>32.87</v>
       </c>
       <c r="K9" t="n">
-        <v>43.7138</v>
+        <v>35.06</v>
       </c>
       <c r="L9" t="n">
-        <v>40.9582</v>
+        <v>32.63</v>
       </c>
       <c r="M9" t="n">
-        <v>40.978</v>
+        <v>33.66</v>
       </c>
       <c r="N9" t="n">
-        <v>37.7241</v>
+        <v>33.37</v>
       </c>
       <c r="O9" t="n">
-        <v>38.3256</v>
+        <v>34.54</v>
       </c>
       <c r="P9" t="n">
-        <v>37.2706</v>
+        <v>33.35</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.3396</v>
+        <v>34.14</v>
       </c>
       <c r="R9" t="n">
-        <v>7.7077</v>
+        <v>-3.7512</v>
       </c>
       <c r="S9" t="n">
-        <v>20.8659</v>
+        <v>18.3358</v>
       </c>
       <c r="T9" t="n">
-        <v>1.5186</v>
+        <v>40.7578</v>
       </c>
       <c r="U9" t="n">
-        <v>1.7652</v>
+        <v>-2.4965</v>
       </c>
       <c r="V9" t="n">
-        <v>6.9808</v>
+        <v>8.4969</v>
       </c>
       <c r="W9" t="n">
-        <v>2.3387</v>
+        <v>16.0196</v>
       </c>
       <c r="X9" t="n">
-        <v>-7.7795</v>
+        <v>3.8248</v>
       </c>
       <c r="Y9" t="n">
-        <v>-18.8062</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z9" t="n">
-        <v>-6.0036</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.7128</v>
+        <v>2.5318</v>
       </c>
       <c r="AB9" t="n">
-        <v>-6.7701</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC9" t="n">
-        <v>-2.5727</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>131.9835</v>
+        <v>138.47</v>
       </c>
       <c r="C10" t="n">
-        <v>143.9056</v>
+        <v>147.2</v>
       </c>
       <c r="D10" t="n">
-        <v>129.5351</v>
+        <v>136.9</v>
       </c>
       <c r="E10" t="n">
-        <v>141.837</v>
+        <v>146.33</v>
       </c>
       <c r="F10" t="n">
-        <v>74.68559999999999</v>
+        <v>76.75</v>
       </c>
       <c r="G10" t="n">
-        <v>79.3366</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>74.68559999999999</v>
+        <v>76.55</v>
       </c>
       <c r="I10" t="n">
-        <v>78.7577</v>
+        <v>78.58</v>
       </c>
       <c r="J10" t="n">
-        <v>38.2718</v>
+        <v>35.45</v>
       </c>
       <c r="K10" t="n">
-        <v>39.0224</v>
+        <v>35.85</v>
       </c>
       <c r="L10" t="n">
-        <v>34.252</v>
+        <v>33.43</v>
       </c>
       <c r="M10" t="n">
-        <v>34.894</v>
+        <v>33.63</v>
       </c>
       <c r="N10" t="n">
-        <v>36.2155</v>
+        <v>34.98</v>
       </c>
       <c r="O10" t="n">
-        <v>36.2254</v>
+        <v>35.06</v>
       </c>
       <c r="P10" t="n">
-        <v>33.8294</v>
+        <v>33.95</v>
       </c>
       <c r="Q10" t="n">
-        <v>34.1154</v>
+        <v>34.18</v>
       </c>
       <c r="R10" t="n">
-        <v>14.7651</v>
+        <v>0.0547</v>
       </c>
       <c r="S10" t="n">
-        <v>36.5105</v>
+        <v>3.1677</v>
       </c>
       <c r="T10" t="n">
-        <v>40.3442</v>
+        <v>27.5265</v>
       </c>
       <c r="U10" t="n">
-        <v>8.631600000000001</v>
+        <v>-0.1017</v>
       </c>
       <c r="V10" t="n">
-        <v>16.1637</v>
+        <v>-0.2256</v>
       </c>
       <c r="W10" t="n">
-        <v>13.9166</v>
+        <v>10.2998</v>
       </c>
       <c r="X10" t="n">
-        <v>-14.847</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y10" t="n">
-        <v>-29.4951</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z10" t="n">
-        <v>-31.7031</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA10" t="n">
-        <v>-8.6348</v>
+        <v>0.1172</v>
       </c>
       <c r="AB10" t="n">
-        <v>-14.7993</v>
+        <v>0.1894</v>
       </c>
       <c r="AC10" t="n">
-        <v>-13.1307</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>137.67</v>
+        <v>149.24</v>
       </c>
       <c r="C11" t="n">
-        <v>152.64</v>
+        <v>153.9</v>
       </c>
       <c r="D11" t="n">
-        <v>137.46</v>
+        <v>147.39</v>
       </c>
       <c r="E11" t="n">
-        <v>151.95</v>
+        <v>151.45</v>
       </c>
       <c r="F11" t="n">
-        <v>78.61799999999999</v>
+        <v>79.09</v>
       </c>
       <c r="G11" t="n">
-        <v>80.96339999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H11" t="n">
-        <v>78.61799999999999</v>
+        <v>78.06</v>
       </c>
       <c r="I11" t="n">
-        <v>80.67400000000001</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>35.98</v>
+        <v>32.97</v>
       </c>
       <c r="K11" t="n">
-        <v>36.01</v>
+        <v>33.39</v>
       </c>
       <c r="L11" t="n">
-        <v>32.25</v>
+        <v>31.9</v>
       </c>
       <c r="M11" t="n">
-        <v>32.42</v>
+        <v>32.43</v>
       </c>
       <c r="N11" t="n">
-        <v>34.1745</v>
+        <v>33.97</v>
       </c>
       <c r="O11" t="n">
-        <v>34.1745</v>
+        <v>34.41</v>
       </c>
       <c r="P11" t="n">
-        <v>33.1688</v>
+        <v>33.54</v>
       </c>
       <c r="Q11" t="n">
-        <v>33.297</v>
+        <v>33.75</v>
       </c>
       <c r="R11" t="n">
-        <v>7.13</v>
+        <v>3.4989</v>
       </c>
       <c r="S11" t="n">
-        <v>32.4243</v>
+        <v>-0.3291</v>
       </c>
       <c r="T11" t="n">
-        <v>48.602</v>
+        <v>22.5433</v>
       </c>
       <c r="U11" t="n">
-        <v>2.4332</v>
+        <v>1.298</v>
       </c>
       <c r="V11" t="n">
-        <v>13.2391</v>
+        <v>-1.3313</v>
       </c>
       <c r="W11" t="n">
-        <v>19.0426</v>
+        <v>9.7934</v>
       </c>
       <c r="X11" t="n">
-        <v>-7.09</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y11" t="n">
-        <v>-27.0392</v>
+        <v>0.0308</v>
       </c>
       <c r="Z11" t="n">
-        <v>-35.7631</v>
+        <v>-20.86</v>
       </c>
       <c r="AA11" t="n">
-        <v>-2.3989</v>
+        <v>-1.258</v>
       </c>
       <c r="AB11" t="n">
-        <v>-12.3539</v>
+        <v>1.3605</v>
       </c>
       <c r="AC11" t="n">
-        <v>-16.8637</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>149.89</v>
+        <v>148.14</v>
       </c>
       <c r="C12" t="n">
-        <v>151</v>
+        <v>149.99</v>
       </c>
       <c r="D12" t="n">
-        <v>139.58</v>
+        <v>135.21</v>
       </c>
       <c r="E12" t="n">
-        <v>146.25</v>
+        <v>142.29</v>
       </c>
       <c r="F12" t="n">
-        <v>80.53</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>80.56999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>77.69</v>
+        <v>75.47</v>
       </c>
       <c r="I12" t="n">
-        <v>78.66</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="K12" t="n">
-        <v>35.06</v>
+        <v>35.95</v>
       </c>
       <c r="L12" t="n">
-        <v>32.63</v>
+        <v>32.77</v>
       </c>
       <c r="M12" t="n">
-        <v>33.66</v>
+        <v>34.43</v>
       </c>
       <c r="N12" t="n">
-        <v>33.37</v>
+        <v>34.31</v>
       </c>
       <c r="O12" t="n">
-        <v>34.54</v>
+        <v>35.53</v>
       </c>
       <c r="P12" t="n">
-        <v>33.35</v>
+        <v>34.17</v>
       </c>
       <c r="Q12" t="n">
-        <v>34.14</v>
+        <v>34.83</v>
       </c>
       <c r="R12" t="n">
-        <v>-3.7512</v>
+        <v>-6.0482</v>
       </c>
       <c r="S12" t="n">
-        <v>18.3358</v>
+        <v>-2.7077</v>
       </c>
       <c r="T12" t="n">
-        <v>40.7578</v>
+        <v>0.3194</v>
       </c>
       <c r="U12" t="n">
-        <v>-2.4965</v>
+        <v>-3.2161</v>
       </c>
       <c r="V12" t="n">
-        <v>8.4969</v>
+        <v>-2.0595</v>
       </c>
       <c r="W12" t="n">
-        <v>16.0196</v>
+        <v>-2.181</v>
       </c>
       <c r="X12" t="n">
-        <v>3.8248</v>
+        <v>6.1671</v>
       </c>
       <c r="Y12" t="n">
-        <v>-17.8584</v>
+        <v>2.2876</v>
       </c>
       <c r="Z12" t="n">
-        <v>-31.9885</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA12" t="n">
-        <v>2.5318</v>
+        <v>3.2</v>
       </c>
       <c r="AB12" t="n">
-        <v>-8.568899999999999</v>
+        <v>2.0211</v>
       </c>
       <c r="AC12" t="n">
-        <v>-14.7378</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>138.47</v>
+        <v>148.94</v>
       </c>
       <c r="C13" t="n">
-        <v>147.2</v>
+        <v>152.37</v>
       </c>
       <c r="D13" t="n">
-        <v>136.9</v>
+        <v>145.49</v>
       </c>
       <c r="E13" t="n">
-        <v>146.33</v>
+        <v>147</v>
       </c>
       <c r="F13" t="n">
-        <v>76.75</v>
+        <v>78.13</v>
       </c>
       <c r="G13" t="n">
-        <v>79.09999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>76.55</v>
+        <v>76.62</v>
       </c>
       <c r="I13" t="n">
-        <v>78.58</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>35.45</v>
+        <v>32.82</v>
       </c>
       <c r="K13" t="n">
-        <v>35.85</v>
+        <v>33.64</v>
       </c>
       <c r="L13" t="n">
-        <v>33.43</v>
+        <v>31.96</v>
       </c>
       <c r="M13" t="n">
-        <v>33.63</v>
+        <v>33.26</v>
       </c>
       <c r="N13" t="n">
-        <v>34.98</v>
+        <v>34.34</v>
       </c>
       <c r="O13" t="n">
-        <v>35.06</v>
+        <v>35.02</v>
       </c>
       <c r="P13" t="n">
-        <v>33.95</v>
+        <v>34.28</v>
       </c>
       <c r="Q13" t="n">
-        <v>34.18</v>
+        <v>34.66</v>
       </c>
       <c r="R13" t="n">
-        <v>0.0547</v>
+        <v>3.3101</v>
       </c>
       <c r="S13" t="n">
-        <v>3.1677</v>
+        <v>0.4579</v>
       </c>
       <c r="T13" t="n">
-        <v>27.5265</v>
+        <v>-3.2577</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.1017</v>
+        <v>0.5452</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.2256</v>
+        <v>-1.4253</v>
       </c>
       <c r="W13" t="n">
-        <v>10.2998</v>
+        <v>-3.9839</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.0891</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y13" t="n">
-        <v>-3.6224</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z13" t="n">
-        <v>-24.3161</v>
+        <v>2.591</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.1172</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.1894</v>
+        <v>1.4043</v>
       </c>
       <c r="AC13" t="n">
-        <v>-10.0297</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>149.24</v>
+        <v>147.95</v>
       </c>
       <c r="C14" t="n">
-        <v>153.9</v>
+        <v>150.77</v>
       </c>
       <c r="D14" t="n">
-        <v>147.39</v>
+        <v>144.41</v>
       </c>
       <c r="E14" t="n">
-        <v>151.45</v>
+        <v>147.86</v>
       </c>
       <c r="F14" t="n">
-        <v>79.09</v>
+        <v>78.13</v>
       </c>
       <c r="G14" t="n">
-        <v>80.06</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>78.06</v>
+        <v>77.94</v>
       </c>
       <c r="I14" t="n">
-        <v>79.59999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J14" t="n">
-        <v>32.97</v>
+        <v>33.07</v>
       </c>
       <c r="K14" t="n">
-        <v>33.39</v>
+        <v>33.86</v>
       </c>
       <c r="L14" t="n">
-        <v>31.9</v>
+        <v>32.42</v>
       </c>
       <c r="M14" t="n">
-        <v>32.43</v>
+        <v>33.08</v>
       </c>
       <c r="N14" t="n">
-        <v>33.97</v>
+        <v>34.36</v>
       </c>
       <c r="O14" t="n">
+        <v>34.44</v>
+      </c>
+      <c r="P14" t="n">
+        <v>33.66</v>
+      </c>
+      <c r="Q14" t="n">
         <v>34.41</v>
       </c>
-      <c r="P14" t="n">
-        <v>33.54</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>33.75</v>
-      </c>
       <c r="R14" t="n">
-        <v>3.4989</v>
+        <v>0.585</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.3291</v>
+        <v>-2.3704</v>
       </c>
       <c r="T14" t="n">
-        <v>22.5433</v>
+        <v>1.1009</v>
       </c>
       <c r="U14" t="n">
-        <v>1.298</v>
+        <v>0.7359</v>
       </c>
       <c r="V14" t="n">
-        <v>-1.3313</v>
+        <v>-1.9724</v>
       </c>
       <c r="W14" t="n">
-        <v>9.7934</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X14" t="n">
-        <v>-3.5682</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.0308</v>
+        <v>2.0043</v>
       </c>
       <c r="Z14" t="n">
-        <v>-20.86</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.258</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.3605</v>
+        <v>1.9556</v>
       </c>
       <c r="AC14" t="n">
-        <v>-9.6134</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>148.14</v>
+        <v>148.56</v>
       </c>
       <c r="C15" t="n">
-        <v>149.99</v>
+        <v>156.71</v>
       </c>
       <c r="D15" t="n">
-        <v>135.21</v>
+        <v>144.31</v>
       </c>
       <c r="E15" t="n">
-        <v>142.29</v>
+        <v>153.69</v>
       </c>
       <c r="F15" t="n">
-        <v>78.29000000000001</v>
+        <v>78.88</v>
       </c>
       <c r="G15" t="n">
-        <v>78.59999999999999</v>
+        <v>79.53</v>
       </c>
       <c r="H15" t="n">
-        <v>75.47</v>
+        <v>76.87</v>
       </c>
       <c r="I15" t="n">
-        <v>77.04000000000001</v>
+        <v>78.73</v>
       </c>
       <c r="J15" t="n">
-        <v>33.17</v>
+        <v>32.95</v>
       </c>
       <c r="K15" t="n">
-        <v>35.95</v>
+        <v>33.89</v>
       </c>
       <c r="L15" t="n">
-        <v>32.77</v>
+        <v>31.1</v>
       </c>
       <c r="M15" t="n">
-        <v>34.43</v>
+        <v>31.76</v>
       </c>
       <c r="N15" t="n">
-        <v>34.31</v>
+        <v>34.04</v>
       </c>
       <c r="O15" t="n">
-        <v>35.53</v>
+        <v>34.92</v>
       </c>
       <c r="P15" t="n">
-        <v>34.17</v>
+        <v>33.74</v>
       </c>
       <c r="Q15" t="n">
-        <v>34.83</v>
+        <v>34.11</v>
       </c>
       <c r="R15" t="n">
-        <v>-6.0482</v>
+        <v>3.9429</v>
       </c>
       <c r="S15" t="n">
-        <v>-2.7077</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T15" t="n">
-        <v>0.3194</v>
+        <v>5.0297</v>
       </c>
       <c r="U15" t="n">
-        <v>-3.2161</v>
+        <v>0.8971</v>
       </c>
       <c r="V15" t="n">
-        <v>-2.0595</v>
+        <v>2.1937</v>
       </c>
       <c r="W15" t="n">
-        <v>-2.181</v>
+        <v>0.1909</v>
       </c>
       <c r="X15" t="n">
-        <v>6.1671</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y15" t="n">
-        <v>2.2876</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z15" t="n">
-        <v>-1.3297</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA15" t="n">
-        <v>3.2</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB15" t="n">
-        <v>2.0211</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC15" t="n">
-        <v>2.0947</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>148.94</v>
+        <v>165.39</v>
       </c>
       <c r="C16" t="n">
-        <v>152.37</v>
+        <v>169.75</v>
       </c>
       <c r="D16" t="n">
-        <v>145.49</v>
+        <v>162.4</v>
       </c>
       <c r="E16" t="n">
-        <v>147</v>
+        <v>163.71</v>
       </c>
       <c r="F16" t="n">
-        <v>78.13</v>
+        <v>81.59</v>
       </c>
       <c r="G16" t="n">
-        <v>78.26000000000001</v>
+        <v>82.61</v>
       </c>
       <c r="H16" t="n">
-        <v>76.62</v>
+        <v>80.37</v>
       </c>
       <c r="I16" t="n">
-        <v>77.45999999999999</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>32.82</v>
+        <v>29.39</v>
       </c>
       <c r="K16" t="n">
-        <v>33.64</v>
+        <v>29.98</v>
       </c>
       <c r="L16" t="n">
-        <v>31.96</v>
+        <v>28.46</v>
       </c>
       <c r="M16" t="n">
-        <v>33.26</v>
+        <v>29.71</v>
       </c>
       <c r="N16" t="n">
-        <v>34.34</v>
+        <v>32.87</v>
       </c>
       <c r="O16" t="n">
-        <v>35.02</v>
+        <v>33.41</v>
       </c>
       <c r="P16" t="n">
-        <v>34.28</v>
+        <v>32.44</v>
       </c>
       <c r="Q16" t="n">
-        <v>34.66</v>
+        <v>33.12</v>
       </c>
       <c r="R16" t="n">
-        <v>3.3101</v>
+        <v>6.5196</v>
       </c>
       <c r="S16" t="n">
-        <v>0.4579</v>
+        <v>11.3673</v>
       </c>
       <c r="T16" t="n">
-        <v>-3.2577</v>
+        <v>8.0951</v>
       </c>
       <c r="U16" t="n">
-        <v>0.5452</v>
+        <v>2.896</v>
       </c>
       <c r="V16" t="n">
-        <v>-1.4253</v>
+        <v>4.583</v>
       </c>
       <c r="W16" t="n">
-        <v>-3.9839</v>
+        <v>1.7714</v>
       </c>
       <c r="X16" t="n">
-        <v>-3.3982</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y16" t="n">
-        <v>-1.1002</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z16" t="n">
-        <v>2.591</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.4881</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB16" t="n">
-        <v>1.4043</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.0935</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>147.95</v>
+        <v>161.66</v>
       </c>
       <c r="C17" t="n">
-        <v>150.77</v>
+        <v>164.38</v>
       </c>
       <c r="D17" t="n">
-        <v>144.41</v>
+        <v>158.08</v>
       </c>
       <c r="E17" t="n">
-        <v>147.86</v>
+        <v>164.27</v>
       </c>
       <c r="F17" t="n">
-        <v>78.13</v>
+        <v>80.95</v>
       </c>
       <c r="G17" t="n">
-        <v>79.68000000000001</v>
+        <v>83.38</v>
       </c>
       <c r="H17" t="n">
-        <v>77.94</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>78.03</v>
+        <v>83.12</v>
       </c>
       <c r="J17" t="n">
-        <v>33.07</v>
+        <v>30.09</v>
       </c>
       <c r="K17" t="n">
-        <v>33.86</v>
+        <v>30.75</v>
       </c>
       <c r="L17" t="n">
-        <v>32.42</v>
+        <v>29.62</v>
       </c>
       <c r="M17" t="n">
-        <v>33.08</v>
+        <v>29.62</v>
       </c>
       <c r="N17" t="n">
-        <v>34.36</v>
+        <v>33.17</v>
       </c>
       <c r="O17" t="n">
-        <v>34.44</v>
+        <v>33.2</v>
       </c>
       <c r="P17" t="n">
-        <v>33.66</v>
+        <v>32.16</v>
       </c>
       <c r="Q17" t="n">
-        <v>34.41</v>
+        <v>32.25</v>
       </c>
       <c r="R17" t="n">
-        <v>0.585</v>
+        <v>0.3421</v>
       </c>
       <c r="S17" t="n">
-        <v>-2.3704</v>
+        <v>11.0983</v>
       </c>
       <c r="T17" t="n">
-        <v>1.1009</v>
+        <v>15.4473</v>
       </c>
       <c r="U17" t="n">
-        <v>0.7359</v>
+        <v>2.6046</v>
       </c>
       <c r="V17" t="n">
-        <v>-1.9724</v>
+        <v>6.5231</v>
       </c>
       <c r="W17" t="n">
-        <v>-0.8008999999999999</v>
+        <v>7.892</v>
       </c>
       <c r="X17" t="n">
-        <v>-0.5412</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y17" t="n">
-        <v>2.0043</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z17" t="n">
-        <v>-1.7231</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.9556</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.7909</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>148.56</v>
+        <v>167.34</v>
       </c>
       <c r="C18" t="n">
-        <v>156.71</v>
+        <v>169.83</v>
       </c>
       <c r="D18" t="n">
-        <v>144.31</v>
+        <v>163.42</v>
       </c>
       <c r="E18" t="n">
-        <v>153.69</v>
+        <v>164.26</v>
       </c>
       <c r="F18" t="n">
-        <v>78.88</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>79.53</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>76.87</v>
+        <v>84.09</v>
       </c>
       <c r="I18" t="n">
-        <v>78.73</v>
+        <v>84.25</v>
       </c>
       <c r="J18" t="n">
-        <v>32.95</v>
+        <v>29.06</v>
       </c>
       <c r="K18" t="n">
-        <v>33.89</v>
+        <v>29.77</v>
       </c>
       <c r="L18" t="n">
-        <v>31.1</v>
+        <v>28.62</v>
       </c>
       <c r="M18" t="n">
-        <v>31.76</v>
+        <v>29.63</v>
       </c>
       <c r="N18" t="n">
-        <v>34.04</v>
+        <v>31.72</v>
       </c>
       <c r="O18" t="n">
-        <v>34.92</v>
+        <v>31.9</v>
       </c>
       <c r="P18" t="n">
-        <v>33.74</v>
+        <v>31.42</v>
       </c>
       <c r="Q18" t="n">
-        <v>34.11</v>
+        <v>31.83</v>
       </c>
       <c r="R18" t="n">
-        <v>3.9429</v>
+        <v>-0.0061</v>
       </c>
       <c r="S18" t="n">
-        <v>8.011799999999999</v>
+        <v>6.8775</v>
       </c>
       <c r="T18" t="n">
-        <v>5.0297</v>
+        <v>11.7415</v>
       </c>
       <c r="U18" t="n">
-        <v>0.8971</v>
+        <v>1.3595</v>
       </c>
       <c r="V18" t="n">
-        <v>2.1937</v>
+        <v>7.0113</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1909</v>
+        <v>8.7658</v>
       </c>
       <c r="X18" t="n">
-        <v>-3.9903</v>
+        <v>0.0338</v>
       </c>
       <c r="Y18" t="n">
-        <v>-7.7549</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z18" t="n">
-        <v>-5.5605</v>
+        <v>-10.914</v>
       </c>
       <c r="AA18" t="n">
-        <v>-0.8718</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB18" t="n">
-        <v>-2.0672</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC18" t="n">
-        <v>-0.2048</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>165.39</v>
+        <v>153.7</v>
       </c>
       <c r="C19" t="n">
-        <v>169.75</v>
+        <v>159.49</v>
       </c>
       <c r="D19" t="n">
-        <v>162.4</v>
+        <v>151.42</v>
       </c>
       <c r="E19" t="n">
-        <v>163.71</v>
+        <v>158.91</v>
       </c>
       <c r="F19" t="n">
-        <v>81.59</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>82.61</v>
+        <v>83.75</v>
       </c>
       <c r="H19" t="n">
-        <v>80.37</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>81.01000000000001</v>
+        <v>83.62</v>
       </c>
       <c r="J19" t="n">
-        <v>29.39</v>
+        <v>31.55</v>
       </c>
       <c r="K19" t="n">
-        <v>29.98</v>
+        <v>31.97</v>
       </c>
       <c r="L19" t="n">
-        <v>28.46</v>
+        <v>30.5</v>
       </c>
       <c r="M19" t="n">
-        <v>29.71</v>
+        <v>30.65</v>
       </c>
       <c r="N19" t="n">
-        <v>32.87</v>
+        <v>32.58</v>
       </c>
       <c r="O19" t="n">
-        <v>33.41</v>
+        <v>32.84</v>
       </c>
       <c r="P19" t="n">
-        <v>32.44</v>
+        <v>32.02</v>
       </c>
       <c r="Q19" t="n">
-        <v>33.12</v>
+        <v>32.07</v>
       </c>
       <c r="R19" t="n">
-        <v>6.5196</v>
+        <v>-3.257</v>
       </c>
       <c r="S19" t="n">
-        <v>11.3673</v>
+        <v>-2.932</v>
       </c>
       <c r="T19" t="n">
-        <v>8.0951</v>
+        <v>7.4733</v>
       </c>
       <c r="U19" t="n">
-        <v>2.896</v>
+        <v>-0.7478</v>
       </c>
       <c r="V19" t="n">
-        <v>4.583</v>
+        <v>3.2218</v>
       </c>
       <c r="W19" t="n">
-        <v>1.7714</v>
+        <v>7.1639</v>
       </c>
       <c r="X19" t="n">
-        <v>-6.4547</v>
+        <v>3.4425</v>
       </c>
       <c r="Y19" t="n">
-        <v>-10.6735</v>
+        <v>3.1639</v>
       </c>
       <c r="Z19" t="n">
-        <v>-8.3873</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA19" t="n">
-        <v>-2.9024</v>
+        <v>0.754</v>
       </c>
       <c r="AB19" t="n">
-        <v>-4.4432</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC19" t="n">
-        <v>-1.8667</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>161.66</v>
+        <v>150.48</v>
       </c>
       <c r="C20" t="n">
-        <v>164.38</v>
+        <v>155.5</v>
       </c>
       <c r="D20" t="n">
-        <v>158.08</v>
+        <v>136.32</v>
       </c>
       <c r="E20" t="n">
-        <v>164.27</v>
+        <v>142.52</v>
       </c>
       <c r="F20" t="n">
-        <v>80.95</v>
+        <v>82.33</v>
       </c>
       <c r="G20" t="n">
-        <v>83.38</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>80.84999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I20" t="n">
-        <v>83.12</v>
+        <v>80.23</v>
       </c>
       <c r="J20" t="n">
-        <v>30.09</v>
+        <v>32.25</v>
       </c>
       <c r="K20" t="n">
-        <v>30.75</v>
+        <v>34.96</v>
       </c>
       <c r="L20" t="n">
-        <v>29.62</v>
+        <v>31.25</v>
       </c>
       <c r="M20" t="n">
-        <v>29.62</v>
+        <v>33.79</v>
       </c>
       <c r="N20" t="n">
-        <v>33.17</v>
+        <v>32.58</v>
       </c>
       <c r="O20" t="n">
-        <v>33.2</v>
+        <v>33.94</v>
       </c>
       <c r="P20" t="n">
         <v>32.16</v>
       </c>
       <c r="Q20" t="n">
-        <v>32.25</v>
+        <v>33.37</v>
       </c>
       <c r="R20" t="n">
-        <v>0.3421</v>
+        <v>-10.314</v>
       </c>
       <c r="S20" t="n">
-        <v>11.0983</v>
+        <v>-13.2404</v>
       </c>
       <c r="T20" t="n">
-        <v>15.4473</v>
+        <v>-7.2679</v>
       </c>
       <c r="U20" t="n">
-        <v>2.6046</v>
+        <v>-4.0541</v>
       </c>
       <c r="V20" t="n">
-        <v>6.5231</v>
+        <v>-3.4769</v>
       </c>
       <c r="W20" t="n">
-        <v>7.892</v>
+        <v>1.9052</v>
       </c>
       <c r="X20" t="n">
-        <v>-0.3029</v>
+        <v>10.2447</v>
       </c>
       <c r="Y20" t="n">
-        <v>-10.4595</v>
+        <v>14.0783</v>
       </c>
       <c r="Z20" t="n">
-        <v>-13.9704</v>
+        <v>6.3917</v>
       </c>
       <c r="AA20" t="n">
-        <v>-2.6268</v>
+        <v>4.0536</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.2772</v>
+        <v>3.4729</v>
       </c>
       <c r="AC20" t="n">
-        <v>-7.4074</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>167.34</v>
+        <v>148.18</v>
       </c>
       <c r="C21" t="n">
-        <v>169.83</v>
+        <v>148.18</v>
       </c>
       <c r="D21" t="n">
-        <v>163.42</v>
+        <v>137.71</v>
       </c>
       <c r="E21" t="n">
-        <v>164.26</v>
+        <v>139.76</v>
       </c>
       <c r="F21" t="n">
-        <v>84.54000000000001</v>
+        <v>81.72</v>
       </c>
       <c r="G21" t="n">
-        <v>85.31999999999999</v>
+        <v>81.81</v>
       </c>
       <c r="H21" t="n">
-        <v>84.09</v>
+        <v>80.37</v>
       </c>
       <c r="I21" t="n">
-        <v>84.25</v>
+        <v>81.28</v>
       </c>
       <c r="J21" t="n">
-        <v>29.06</v>
+        <v>32.4</v>
       </c>
       <c r="K21" t="n">
-        <v>29.77</v>
+        <v>34.91</v>
       </c>
       <c r="L21" t="n">
-        <v>28.62</v>
+        <v>32.39</v>
       </c>
       <c r="M21" t="n">
-        <v>29.63</v>
+        <v>34.39</v>
       </c>
       <c r="N21" t="n">
-        <v>31.72</v>
+        <v>32.78</v>
       </c>
       <c r="O21" t="n">
-        <v>31.9</v>
+        <v>33.34</v>
       </c>
       <c r="P21" t="n">
-        <v>31.42</v>
+        <v>32.73</v>
       </c>
       <c r="Q21" t="n">
-        <v>31.83</v>
+        <v>32.95</v>
       </c>
       <c r="R21" t="n">
-        <v>-0.0061</v>
+        <v>-1.9366</v>
       </c>
       <c r="S21" t="n">
-        <v>6.8775</v>
+        <v>-14.9154</v>
       </c>
       <c r="T21" t="n">
-        <v>11.7415</v>
+        <v>-14.6295</v>
       </c>
       <c r="U21" t="n">
-        <v>1.3595</v>
+        <v>1.3087</v>
       </c>
       <c r="V21" t="n">
-        <v>7.0113</v>
+        <v>-3.5252</v>
       </c>
       <c r="W21" t="n">
-        <v>8.7658</v>
+        <v>0.3333</v>
       </c>
       <c r="X21" t="n">
-        <v>0.0338</v>
+        <v>1.7757</v>
       </c>
       <c r="Y21" t="n">
-        <v>-6.7065</v>
+        <v>16.0648</v>
       </c>
       <c r="Z21" t="n">
-        <v>-10.914</v>
+        <v>15.7523</v>
       </c>
       <c r="AA21" t="n">
-        <v>-1.3023</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.6843</v>
+        <v>3.5187</v>
       </c>
       <c r="AC21" t="n">
-        <v>-8.164999999999999</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>153.7</v>
+        <v>134.43</v>
       </c>
       <c r="C22" t="n">
-        <v>159.49</v>
+        <v>134.54</v>
       </c>
       <c r="D22" t="n">
-        <v>151.42</v>
+        <v>127.27</v>
       </c>
       <c r="E22" t="n">
-        <v>158.91</v>
+        <v>128.4</v>
       </c>
       <c r="F22" t="n">
-        <v>82.31999999999999</v>
+        <v>80.78</v>
       </c>
       <c r="G22" t="n">
-        <v>83.75</v>
+        <v>80.81</v>
       </c>
       <c r="H22" t="n">
-        <v>81.59999999999999</v>
+        <v>79.22</v>
       </c>
       <c r="I22" t="n">
-        <v>83.62</v>
+        <v>79.61</v>
       </c>
       <c r="J22" t="n">
-        <v>31.55</v>
+        <v>35.75</v>
       </c>
       <c r="K22" t="n">
-        <v>31.97</v>
+        <v>37.5</v>
       </c>
       <c r="L22" t="n">
-        <v>30.5</v>
+        <v>35.68</v>
       </c>
       <c r="M22" t="n">
-        <v>30.65</v>
+        <v>37.19</v>
       </c>
       <c r="N22" t="n">
-        <v>32.58</v>
+        <v>33.17</v>
       </c>
       <c r="O22" t="n">
-        <v>32.84</v>
+        <v>33.8</v>
       </c>
       <c r="P22" t="n">
-        <v>32.02</v>
+        <v>33.17</v>
       </c>
       <c r="Q22" t="n">
-        <v>32.07</v>
+        <v>33.63</v>
       </c>
       <c r="R22" t="n">
-        <v>-3.257</v>
+        <v>-8.1282</v>
       </c>
       <c r="S22" t="n">
-        <v>-2.932</v>
+        <v>-19.1995</v>
       </c>
       <c r="T22" t="n">
-        <v>7.4733</v>
+        <v>-21.836</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.7478</v>
+        <v>-2.0546</v>
       </c>
       <c r="V22" t="n">
-        <v>3.2218</v>
+        <v>-4.7955</v>
       </c>
       <c r="W22" t="n">
-        <v>7.1639</v>
+        <v>-4.2228</v>
       </c>
       <c r="X22" t="n">
-        <v>3.4425</v>
+        <v>8.1419</v>
       </c>
       <c r="Y22" t="n">
-        <v>3.1639</v>
+        <v>21.3377</v>
       </c>
       <c r="Z22" t="n">
-        <v>-7.3458</v>
+        <v>25.5571</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.754</v>
+        <v>2.0637</v>
       </c>
       <c r="AB22" t="n">
-        <v>-3.1703</v>
+        <v>4.8644</v>
       </c>
       <c r="AC22" t="n">
-        <v>-6.8003</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>150.48</v>
-      </c>
-      <c r="C23" t="n">
-        <v>155.5</v>
-      </c>
-      <c r="D23" t="n">
-        <v>136.32</v>
-      </c>
-      <c r="E23" t="n">
-        <v>142.52</v>
-      </c>
-      <c r="F23" t="n">
-        <v>82.33</v>
-      </c>
-      <c r="G23" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="H23" t="n">
-        <v>78.78</v>
-      </c>
-      <c r="I23" t="n">
-        <v>80.23</v>
-      </c>
-      <c r="J23" t="n">
-        <v>32.25</v>
-      </c>
-      <c r="K23" t="n">
-        <v>34.96</v>
-      </c>
-      <c r="L23" t="n">
-        <v>31.25</v>
-      </c>
-      <c r="M23" t="n">
-        <v>33.79</v>
-      </c>
-      <c r="N23" t="n">
-        <v>32.58</v>
-      </c>
-      <c r="O23" t="n">
-        <v>33.94</v>
-      </c>
-      <c r="P23" t="n">
-        <v>32.16</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="R23" t="n">
-        <v>-10.314</v>
-      </c>
-      <c r="S23" t="n">
-        <v>-13.2404</v>
-      </c>
-      <c r="T23" t="n">
-        <v>-7.2679</v>
-      </c>
-      <c r="U23" t="n">
-        <v>-4.0541</v>
-      </c>
-      <c r="V23" t="n">
-        <v>-3.4769</v>
-      </c>
-      <c r="W23" t="n">
-        <v>1.9052</v>
-      </c>
-      <c r="X23" t="n">
-        <v>10.2447</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>14.0783</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>6.3917</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>4.0536</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>3.4729</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>-2.1695</v>
+        <v>4.2791</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-14 00:54
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2366,6 +2366,13 @@
       </c>
       <c r="AC22" t="n">
         <v>4.2791</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-15 00:18
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1810 +568,1810 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>101.4635</v>
+        <v>104.4815</v>
       </c>
       <c r="C2" t="n">
-        <v>105.3209</v>
+        <v>105.8706</v>
       </c>
       <c r="D2" t="n">
-        <v>99.80459999999999</v>
+        <v>100.8938</v>
       </c>
       <c r="E2" t="n">
-        <v>101.0637</v>
+        <v>102.253</v>
       </c>
       <c r="F2" t="n">
-        <v>67.3997</v>
+        <v>68.9966</v>
       </c>
       <c r="G2" t="n">
-        <v>70.25409999999999</v>
+        <v>69.1962</v>
       </c>
       <c r="H2" t="n">
-        <v>67.20999999999999</v>
+        <v>67.4795</v>
       </c>
       <c r="I2" t="n">
-        <v>69.13630000000001</v>
+        <v>67.76900000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>50.9731</v>
+        <v>49.2546</v>
       </c>
       <c r="K2" t="n">
-        <v>51.5756</v>
+        <v>51.1607</v>
       </c>
       <c r="L2" t="n">
-        <v>49.5904</v>
+        <v>48.6521</v>
       </c>
       <c r="M2" t="n">
-        <v>51.0916</v>
+        <v>50.4694</v>
       </c>
       <c r="N2" t="n">
+        <v>39.351</v>
+      </c>
+      <c r="O2" t="n">
         <v>40.2088</v>
       </c>
-      <c r="O2" t="n">
-        <v>40.3074</v>
-      </c>
       <c r="P2" t="n">
-        <v>38.6608</v>
+        <v>39.2327</v>
       </c>
       <c r="Q2" t="n">
-        <v>39.2721</v>
+        <v>40.0511</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104.4815</v>
+        <v>107.3696</v>
       </c>
       <c r="C3" t="n">
-        <v>105.8706</v>
+        <v>109.2484</v>
       </c>
       <c r="D3" t="n">
-        <v>100.8938</v>
+        <v>100.9938</v>
       </c>
       <c r="E3" t="n">
-        <v>102.253</v>
+        <v>103.9019</v>
       </c>
       <c r="F3" t="n">
-        <v>68.9966</v>
+        <v>68.7171</v>
       </c>
       <c r="G3" t="n">
-        <v>69.1962</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>67.4795</v>
+        <v>66.4216</v>
       </c>
       <c r="I3" t="n">
-        <v>67.76900000000001</v>
+        <v>67.7989</v>
       </c>
       <c r="J3" t="n">
-        <v>49.2546</v>
+        <v>47.9509</v>
       </c>
       <c r="K3" t="n">
-        <v>51.1607</v>
+        <v>51.1015</v>
       </c>
       <c r="L3" t="n">
-        <v>48.6521</v>
+        <v>46.9829</v>
       </c>
       <c r="M3" t="n">
-        <v>50.4694</v>
+        <v>49.4916</v>
       </c>
       <c r="N3" t="n">
-        <v>39.351</v>
+        <v>39.4989</v>
       </c>
       <c r="O3" t="n">
-        <v>40.2088</v>
+        <v>40.8596</v>
       </c>
       <c r="P3" t="n">
-        <v>39.2327</v>
+        <v>38.8186</v>
       </c>
       <c r="Q3" t="n">
-        <v>40.0511</v>
+        <v>40.0412</v>
       </c>
       <c r="R3" t="n">
-        <v>1.1768</v>
+        <v>1.6126</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.9777</v>
+        <v>0.0441</v>
       </c>
       <c r="X3" t="n">
-        <v>-1.2178</v>
+        <v>-1.9374</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.9836</v>
+        <v>-0.0247</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>107.3696</v>
+        <v>113.2557</v>
       </c>
       <c r="C4" t="n">
-        <v>109.2484</v>
+        <v>115.4043</v>
       </c>
       <c r="D4" t="n">
-        <v>100.9938</v>
+        <v>111.9366</v>
       </c>
       <c r="E4" t="n">
-        <v>103.9019</v>
+        <v>114.7448</v>
       </c>
       <c r="F4" t="n">
-        <v>68.7171</v>
+        <v>70.9927</v>
       </c>
       <c r="G4" t="n">
-        <v>69.83499999999999</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>66.4216</v>
+        <v>70.2342</v>
       </c>
       <c r="I4" t="n">
-        <v>67.7989</v>
+        <v>71.2422</v>
       </c>
       <c r="J4" t="n">
-        <v>47.9509</v>
+        <v>45.1558</v>
       </c>
       <c r="K4" t="n">
-        <v>51.1015</v>
+        <v>45.7681</v>
       </c>
       <c r="L4" t="n">
-        <v>46.9829</v>
+        <v>44.1187</v>
       </c>
       <c r="M4" t="n">
-        <v>49.4916</v>
+        <v>44.4348</v>
       </c>
       <c r="N4" t="n">
-        <v>39.4989</v>
+        <v>38.1481</v>
       </c>
       <c r="O4" t="n">
-        <v>40.8596</v>
+        <v>38.5918</v>
       </c>
       <c r="P4" t="n">
-        <v>38.8186</v>
+        <v>37.7931</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.0412</v>
+        <v>37.9903</v>
       </c>
       <c r="R4" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0441</v>
+        <v>5.0787</v>
       </c>
       <c r="X4" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.0247</v>
+        <v>-5.122</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>113.2557</v>
+        <v>116.9533</v>
       </c>
       <c r="C5" t="n">
-        <v>115.4043</v>
+        <v>123.8188</v>
       </c>
       <c r="D5" t="n">
-        <v>111.9366</v>
+        <v>116.6035</v>
       </c>
       <c r="E5" t="n">
-        <v>114.7448</v>
+        <v>123.589</v>
       </c>
       <c r="F5" t="n">
-        <v>70.9927</v>
+        <v>71.7812</v>
       </c>
       <c r="G5" t="n">
-        <v>71.58159999999999</v>
+        <v>72.6395</v>
       </c>
       <c r="H5" t="n">
-        <v>70.2342</v>
+        <v>70.6733</v>
       </c>
       <c r="I5" t="n">
-        <v>71.2422</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>45.1558</v>
+        <v>43.5656</v>
       </c>
       <c r="K5" t="n">
-        <v>45.7681</v>
+        <v>43.7138</v>
       </c>
       <c r="L5" t="n">
-        <v>44.1187</v>
+        <v>40.9582</v>
       </c>
       <c r="M5" t="n">
-        <v>44.4348</v>
+        <v>40.978</v>
       </c>
       <c r="N5" t="n">
-        <v>38.1481</v>
+        <v>37.7241</v>
       </c>
       <c r="O5" t="n">
-        <v>38.5918</v>
+        <v>38.3256</v>
       </c>
       <c r="P5" t="n">
-        <v>37.7931</v>
+        <v>37.2706</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.9903</v>
+        <v>37.3396</v>
       </c>
       <c r="R5" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="S5" t="n">
-        <v>13.5371</v>
+        <v>20.8659</v>
       </c>
       <c r="U5" t="n">
-        <v>5.0787</v>
+        <v>1.7652</v>
       </c>
       <c r="V5" t="n">
-        <v>3.046</v>
+        <v>6.9808</v>
       </c>
       <c r="X5" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="Y5" t="n">
-        <v>-13.0291</v>
+        <v>-18.8062</v>
       </c>
       <c r="AA5" t="n">
-        <v>-5.122</v>
+        <v>-1.7128</v>
       </c>
       <c r="AB5" t="n">
-        <v>-3.2639</v>
+        <v>-6.7701</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>116.9533</v>
+        <v>131.9835</v>
       </c>
       <c r="C6" t="n">
-        <v>123.8188</v>
+        <v>143.9056</v>
       </c>
       <c r="D6" t="n">
-        <v>116.6035</v>
+        <v>129.5351</v>
       </c>
       <c r="E6" t="n">
-        <v>123.589</v>
+        <v>141.837</v>
       </c>
       <c r="F6" t="n">
-        <v>71.7812</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>72.6395</v>
+        <v>79.3366</v>
       </c>
       <c r="H6" t="n">
-        <v>70.6733</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>72.49979999999999</v>
+        <v>78.7577</v>
       </c>
       <c r="J6" t="n">
-        <v>43.5656</v>
+        <v>38.2718</v>
       </c>
       <c r="K6" t="n">
-        <v>43.7138</v>
+        <v>39.0224</v>
       </c>
       <c r="L6" t="n">
-        <v>40.9582</v>
+        <v>34.252</v>
       </c>
       <c r="M6" t="n">
-        <v>40.978</v>
+        <v>34.894</v>
       </c>
       <c r="N6" t="n">
-        <v>37.7241</v>
+        <v>36.2155</v>
       </c>
       <c r="O6" t="n">
-        <v>38.3256</v>
+        <v>36.2254</v>
       </c>
       <c r="P6" t="n">
-        <v>37.2706</v>
+        <v>33.8294</v>
       </c>
       <c r="Q6" t="n">
-        <v>37.3396</v>
+        <v>34.1154</v>
       </c>
       <c r="R6" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="S6" t="n">
-        <v>20.8659</v>
+        <v>36.5105</v>
       </c>
       <c r="U6" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V6" t="n">
-        <v>6.9808</v>
+        <v>16.1637</v>
       </c>
       <c r="X6" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="Y6" t="n">
-        <v>-18.8062</v>
+        <v>-29.4951</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.7128</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.7701</v>
+        <v>-14.7993</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C7" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D7" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E7" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F7" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>79.3366</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>78.7577</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K7" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L7" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M7" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N7" t="n">
-        <v>36.2155</v>
+        <v>34.1745</v>
       </c>
       <c r="O7" t="n">
-        <v>36.2254</v>
+        <v>34.1745</v>
       </c>
       <c r="P7" t="n">
-        <v>33.8294</v>
+        <v>33.1688</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.1154</v>
+        <v>33.297</v>
       </c>
       <c r="R7" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S7" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="T7" t="n">
-        <v>40.3442</v>
+        <v>48.602</v>
       </c>
       <c r="U7" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V7" t="n">
-        <v>16.1637</v>
+        <v>13.2391</v>
       </c>
       <c r="W7" t="n">
-        <v>13.9166</v>
+        <v>19.0426</v>
       </c>
       <c r="X7" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y7" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="Z7" t="n">
-        <v>-31.7031</v>
+        <v>-35.7631</v>
       </c>
       <c r="AA7" t="n">
-        <v>-8.6348</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB7" t="n">
-        <v>-14.7993</v>
+        <v>-12.3539</v>
       </c>
       <c r="AC7" t="n">
-        <v>-13.1307</v>
+        <v>-16.8637</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C8" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D8" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E8" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F8" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G8" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I8" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J8" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K8" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L8" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M8" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N8" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O8" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P8" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q8" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
       <c r="R8" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="S8" t="n">
-        <v>32.4243</v>
+        <v>18.3358</v>
       </c>
       <c r="T8" t="n">
-        <v>48.602</v>
+        <v>40.7578</v>
       </c>
       <c r="U8" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="V8" t="n">
-        <v>13.2391</v>
+        <v>8.4969</v>
       </c>
       <c r="W8" t="n">
-        <v>19.0426</v>
+        <v>16.0196</v>
       </c>
       <c r="X8" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="Y8" t="n">
-        <v>-27.0392</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z8" t="n">
-        <v>-35.7631</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.3989</v>
+        <v>2.5318</v>
       </c>
       <c r="AB8" t="n">
-        <v>-12.3539</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC8" t="n">
-        <v>-16.8637</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C9" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D9" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E9" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F9" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G9" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I9" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J9" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K9" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L9" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M9" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N9" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O9" t="n">
         <v>35.06</v>
       </c>
-      <c r="L9" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M9" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N9" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O9" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P9" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q9" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R9" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="S9" t="n">
-        <v>18.3358</v>
+        <v>3.1677</v>
       </c>
       <c r="T9" t="n">
-        <v>40.7578</v>
+        <v>27.5265</v>
       </c>
       <c r="U9" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="V9" t="n">
-        <v>8.4969</v>
+        <v>-0.2256</v>
       </c>
       <c r="W9" t="n">
-        <v>16.0196</v>
+        <v>10.2998</v>
       </c>
       <c r="X9" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y9" t="n">
-        <v>-17.8584</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z9" t="n">
-        <v>-31.9885</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA9" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
       <c r="AB9" t="n">
-        <v>-8.568899999999999</v>
+        <v>0.1894</v>
       </c>
       <c r="AC9" t="n">
-        <v>-14.7378</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C10" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D10" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E10" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F10" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G10" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H10" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I10" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K10" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L10" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M10" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N10" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O10" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P10" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q10" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R10" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="S10" t="n">
-        <v>3.1677</v>
+        <v>-0.3291</v>
       </c>
       <c r="T10" t="n">
-        <v>27.5265</v>
+        <v>22.5433</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.2256</v>
+        <v>-1.3313</v>
       </c>
       <c r="W10" t="n">
-        <v>10.2998</v>
+        <v>9.7934</v>
       </c>
       <c r="X10" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y10" t="n">
-        <v>-3.6224</v>
+        <v>0.0308</v>
       </c>
       <c r="Z10" t="n">
-        <v>-24.3161</v>
+        <v>-20.86</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.1894</v>
+        <v>1.3605</v>
       </c>
       <c r="AC10" t="n">
-        <v>-10.0297</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C11" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D11" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E11" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F11" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I11" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K11" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L11" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M11" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N11" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O11" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P11" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q11" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R11" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.3291</v>
+        <v>-2.7077</v>
       </c>
       <c r="T11" t="n">
-        <v>22.5433</v>
+        <v>0.3194</v>
       </c>
       <c r="U11" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.3313</v>
+        <v>-2.0595</v>
       </c>
       <c r="W11" t="n">
-        <v>9.7934</v>
+        <v>-2.181</v>
       </c>
       <c r="X11" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.0308</v>
+        <v>2.2876</v>
       </c>
       <c r="Z11" t="n">
-        <v>-20.86</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
       <c r="AB11" t="n">
-        <v>1.3605</v>
+        <v>2.0211</v>
       </c>
       <c r="AC11" t="n">
-        <v>-9.6134</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C12" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D12" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E12" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F12" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G12" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I12" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K12" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L12" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M12" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N12" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O12" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P12" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q12" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R12" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S12" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="T12" t="n">
-        <v>0.3194</v>
+        <v>-3.2577</v>
       </c>
       <c r="U12" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V12" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="W12" t="n">
-        <v>-2.181</v>
+        <v>-3.9839</v>
       </c>
       <c r="X12" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y12" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z12" t="n">
-        <v>-1.3297</v>
+        <v>2.591</v>
       </c>
       <c r="AA12" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB12" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.0947</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C13" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D13" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E13" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F13" t="n">
         <v>78.13</v>
       </c>
       <c r="G13" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I13" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J13" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K13" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L13" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M13" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N13" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O13" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P13" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q13" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R13" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S13" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="T13" t="n">
-        <v>-3.2577</v>
+        <v>1.1009</v>
       </c>
       <c r="U13" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="W13" t="n">
-        <v>-3.9839</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X13" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y13" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="Z13" t="n">
-        <v>2.591</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
       <c r="AC13" t="n">
-        <v>4.0935</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C14" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D14" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E14" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F14" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G14" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H14" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I14" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J14" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K14" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L14" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M14" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N14" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O14" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P14" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q14" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R14" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T14" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U14" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V14" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X14" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y14" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z14" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C15" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D15" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E15" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F15" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G15" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H15" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I15" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K15" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L15" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M15" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N15" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O15" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P15" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q15" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R15" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S15" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T15" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U15" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V15" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X15" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y15" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z15" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB15" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC15" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C16" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D16" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E16" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F16" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G16" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H16" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J16" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K16" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L16" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M16" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N16" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O16" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P16" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q16" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R16" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S16" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T16" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U16" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V16" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W16" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X16" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y16" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z16" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA16" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB16" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC16" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C17" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D17" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E17" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F17" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I17" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J17" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K17" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L17" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M17" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N17" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O17" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P17" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q17" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S17" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T17" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U17" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V17" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W17" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X17" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y17" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z17" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC17" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C18" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D18" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E18" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F18" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H18" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J18" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K18" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L18" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M18" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N18" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O18" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P18" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q18" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S18" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T18" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U18" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V18" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W18" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X18" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y18" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z18" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC18" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C19" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D19" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E19" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F19" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G19" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I19" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J19" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K19" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L19" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M19" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N19" t="n">
         <v>32.58</v>
       </c>
       <c r="O19" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P19" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q19" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R19" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S19" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T19" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V19" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W19" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X19" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z19" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB19" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC19" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C20" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D20" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E20" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F20" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G20" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H20" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I20" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J20" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K20" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L20" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M20" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N20" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O20" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P20" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q20" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R20" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S20" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T20" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U20" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W20" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X20" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y20" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z20" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA20" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC20" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C21" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D21" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E21" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F21" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G21" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H21" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I21" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J21" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K21" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L21" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M21" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N21" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O21" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P21" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R21" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S21" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T21" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U21" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V21" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W21" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X21" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y21" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z21" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA21" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB21" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC21" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C22" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D22" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E22" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F22" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H22" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I22" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J22" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K22" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L22" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M22" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N22" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O22" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P22" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q22" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R22" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S22" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T22" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U22" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V22" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W22" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X22" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y22" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z22" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA22" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC22" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-16 00:06
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1810 +568,1810 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>104.4815</v>
+        <v>107.3696</v>
       </c>
       <c r="C2" t="n">
-        <v>105.8706</v>
+        <v>109.2484</v>
       </c>
       <c r="D2" t="n">
-        <v>100.8938</v>
+        <v>100.9938</v>
       </c>
       <c r="E2" t="n">
-        <v>102.253</v>
+        <v>103.9019</v>
       </c>
       <c r="F2" t="n">
-        <v>68.9966</v>
+        <v>68.7171</v>
       </c>
       <c r="G2" t="n">
-        <v>69.1962</v>
+        <v>69.83499999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>67.4795</v>
+        <v>66.4216</v>
       </c>
       <c r="I2" t="n">
-        <v>67.76900000000001</v>
+        <v>67.7989</v>
       </c>
       <c r="J2" t="n">
-        <v>49.2546</v>
+        <v>47.9509</v>
       </c>
       <c r="K2" t="n">
-        <v>51.1607</v>
+        <v>51.1015</v>
       </c>
       <c r="L2" t="n">
-        <v>48.6521</v>
+        <v>46.9829</v>
       </c>
       <c r="M2" t="n">
-        <v>50.4694</v>
+        <v>49.4916</v>
       </c>
       <c r="N2" t="n">
-        <v>39.351</v>
+        <v>39.4989</v>
       </c>
       <c r="O2" t="n">
-        <v>40.2088</v>
+        <v>40.8596</v>
       </c>
       <c r="P2" t="n">
-        <v>39.2327</v>
+        <v>38.8186</v>
       </c>
       <c r="Q2" t="n">
-        <v>40.0511</v>
+        <v>40.0412</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>107.3696</v>
+        <v>113.2557</v>
       </c>
       <c r="C3" t="n">
-        <v>109.2484</v>
+        <v>115.4043</v>
       </c>
       <c r="D3" t="n">
-        <v>100.9938</v>
+        <v>111.9366</v>
       </c>
       <c r="E3" t="n">
-        <v>103.9019</v>
+        <v>114.7448</v>
       </c>
       <c r="F3" t="n">
-        <v>68.7171</v>
+        <v>70.9927</v>
       </c>
       <c r="G3" t="n">
-        <v>69.83499999999999</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>66.4216</v>
+        <v>70.2342</v>
       </c>
       <c r="I3" t="n">
-        <v>67.7989</v>
+        <v>71.2422</v>
       </c>
       <c r="J3" t="n">
-        <v>47.9509</v>
+        <v>45.1558</v>
       </c>
       <c r="K3" t="n">
-        <v>51.1015</v>
+        <v>45.7681</v>
       </c>
       <c r="L3" t="n">
-        <v>46.9829</v>
+        <v>44.1187</v>
       </c>
       <c r="M3" t="n">
-        <v>49.4916</v>
+        <v>44.4348</v>
       </c>
       <c r="N3" t="n">
-        <v>39.4989</v>
+        <v>38.1481</v>
       </c>
       <c r="O3" t="n">
-        <v>40.8596</v>
+        <v>38.5918</v>
       </c>
       <c r="P3" t="n">
-        <v>38.8186</v>
+        <v>37.7931</v>
       </c>
       <c r="Q3" t="n">
-        <v>40.0412</v>
+        <v>37.9903</v>
       </c>
       <c r="R3" t="n">
-        <v>1.6126</v>
+        <v>10.4357</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0441</v>
+        <v>5.0787</v>
       </c>
       <c r="X3" t="n">
-        <v>-1.9374</v>
+        <v>-10.2175</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.0247</v>
+        <v>-5.122</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>113.2557</v>
+        <v>116.9533</v>
       </c>
       <c r="C4" t="n">
-        <v>115.4043</v>
+        <v>123.8188</v>
       </c>
       <c r="D4" t="n">
-        <v>111.9366</v>
+        <v>116.6035</v>
       </c>
       <c r="E4" t="n">
-        <v>114.7448</v>
+        <v>123.589</v>
       </c>
       <c r="F4" t="n">
-        <v>70.9927</v>
+        <v>71.7812</v>
       </c>
       <c r="G4" t="n">
-        <v>71.58159999999999</v>
+        <v>72.6395</v>
       </c>
       <c r="H4" t="n">
-        <v>70.2342</v>
+        <v>70.6733</v>
       </c>
       <c r="I4" t="n">
-        <v>71.2422</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>45.1558</v>
+        <v>43.5656</v>
       </c>
       <c r="K4" t="n">
-        <v>45.7681</v>
+        <v>43.7138</v>
       </c>
       <c r="L4" t="n">
-        <v>44.1187</v>
+        <v>40.9582</v>
       </c>
       <c r="M4" t="n">
-        <v>44.4348</v>
+        <v>40.978</v>
       </c>
       <c r="N4" t="n">
-        <v>38.1481</v>
+        <v>37.7241</v>
       </c>
       <c r="O4" t="n">
-        <v>38.5918</v>
+        <v>38.3256</v>
       </c>
       <c r="P4" t="n">
-        <v>37.7931</v>
+        <v>37.2706</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.9903</v>
+        <v>37.3396</v>
       </c>
       <c r="R4" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="U4" t="n">
-        <v>5.0787</v>
+        <v>1.7652</v>
       </c>
       <c r="X4" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="AA4" t="n">
-        <v>-5.122</v>
+        <v>-1.7128</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>116.9533</v>
+        <v>131.9835</v>
       </c>
       <c r="C5" t="n">
-        <v>123.8188</v>
+        <v>143.9056</v>
       </c>
       <c r="D5" t="n">
-        <v>116.6035</v>
+        <v>129.5351</v>
       </c>
       <c r="E5" t="n">
-        <v>123.589</v>
+        <v>141.837</v>
       </c>
       <c r="F5" t="n">
-        <v>71.7812</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>72.6395</v>
+        <v>79.3366</v>
       </c>
       <c r="H5" t="n">
-        <v>70.6733</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>72.49979999999999</v>
+        <v>78.7577</v>
       </c>
       <c r="J5" t="n">
-        <v>43.5656</v>
+        <v>38.2718</v>
       </c>
       <c r="K5" t="n">
-        <v>43.7138</v>
+        <v>39.0224</v>
       </c>
       <c r="L5" t="n">
-        <v>40.9582</v>
+        <v>34.252</v>
       </c>
       <c r="M5" t="n">
-        <v>40.978</v>
+        <v>34.894</v>
       </c>
       <c r="N5" t="n">
-        <v>37.7241</v>
+        <v>36.2155</v>
       </c>
       <c r="O5" t="n">
-        <v>38.3256</v>
+        <v>36.2254</v>
       </c>
       <c r="P5" t="n">
-        <v>37.2706</v>
+        <v>33.8294</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.3396</v>
+        <v>34.1154</v>
       </c>
       <c r="R5" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="S5" t="n">
-        <v>20.8659</v>
+        <v>36.5105</v>
       </c>
       <c r="U5" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="V5" t="n">
-        <v>6.9808</v>
+        <v>16.1637</v>
       </c>
       <c r="X5" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="Y5" t="n">
-        <v>-18.8062</v>
+        <v>-29.4951</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.7128</v>
+        <v>-8.6348</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.7701</v>
+        <v>-14.7993</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C6" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D6" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E6" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F6" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>79.3366</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>78.7577</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K6" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L6" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M6" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N6" t="n">
-        <v>36.2155</v>
+        <v>34.1745</v>
       </c>
       <c r="O6" t="n">
-        <v>36.2254</v>
+        <v>34.1745</v>
       </c>
       <c r="P6" t="n">
-        <v>33.8294</v>
+        <v>33.1688</v>
       </c>
       <c r="Q6" t="n">
-        <v>34.1154</v>
+        <v>33.297</v>
       </c>
       <c r="R6" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S6" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="U6" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V6" t="n">
-        <v>16.1637</v>
+        <v>13.2391</v>
       </c>
       <c r="X6" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y6" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="AA6" t="n">
-        <v>-8.6348</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB6" t="n">
-        <v>-14.7993</v>
+        <v>-12.3539</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C7" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D7" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E7" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F7" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G7" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I7" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J7" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K7" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L7" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M7" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N7" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O7" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P7" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q7" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
       <c r="R7" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="S7" t="n">
-        <v>32.4243</v>
+        <v>18.3358</v>
       </c>
       <c r="T7" t="n">
-        <v>48.602</v>
+        <v>40.7578</v>
       </c>
       <c r="U7" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="V7" t="n">
-        <v>13.2391</v>
+        <v>8.4969</v>
       </c>
       <c r="W7" t="n">
-        <v>19.0426</v>
+        <v>16.0196</v>
       </c>
       <c r="X7" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="Y7" t="n">
-        <v>-27.0392</v>
+        <v>-17.8584</v>
       </c>
       <c r="Z7" t="n">
-        <v>-35.7631</v>
+        <v>-31.9885</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.3989</v>
+        <v>2.5318</v>
       </c>
       <c r="AB7" t="n">
-        <v>-12.3539</v>
+        <v>-8.568899999999999</v>
       </c>
       <c r="AC7" t="n">
-        <v>-16.8637</v>
+        <v>-14.7378</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C8" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D8" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E8" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F8" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G8" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I8" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J8" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K8" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L8" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M8" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N8" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O8" t="n">
         <v>35.06</v>
       </c>
-      <c r="L8" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M8" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N8" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O8" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P8" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q8" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R8" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="S8" t="n">
-        <v>18.3358</v>
+        <v>3.1677</v>
       </c>
       <c r="T8" t="n">
-        <v>40.7578</v>
+        <v>27.5265</v>
       </c>
       <c r="U8" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="V8" t="n">
-        <v>8.4969</v>
+        <v>-0.2256</v>
       </c>
       <c r="W8" t="n">
-        <v>16.0196</v>
+        <v>10.2998</v>
       </c>
       <c r="X8" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y8" t="n">
-        <v>-17.8584</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z8" t="n">
-        <v>-31.9885</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA8" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
       <c r="AB8" t="n">
-        <v>-8.568899999999999</v>
+        <v>0.1894</v>
       </c>
       <c r="AC8" t="n">
-        <v>-14.7378</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C9" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D9" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E9" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F9" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G9" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H9" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I9" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K9" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L9" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M9" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N9" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O9" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P9" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q9" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R9" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="S9" t="n">
-        <v>3.1677</v>
+        <v>-0.3291</v>
       </c>
       <c r="T9" t="n">
-        <v>27.5265</v>
+        <v>22.5433</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="V9" t="n">
-        <v>-0.2256</v>
+        <v>-1.3313</v>
       </c>
       <c r="W9" t="n">
-        <v>10.2998</v>
+        <v>9.7934</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y9" t="n">
-        <v>-3.6224</v>
+        <v>0.0308</v>
       </c>
       <c r="Z9" t="n">
-        <v>-24.3161</v>
+        <v>-20.86</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.1894</v>
+        <v>1.3605</v>
       </c>
       <c r="AC9" t="n">
-        <v>-10.0297</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C10" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D10" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E10" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F10" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I10" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K10" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L10" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M10" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N10" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O10" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P10" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q10" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R10" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.3291</v>
+        <v>-2.7077</v>
       </c>
       <c r="T10" t="n">
-        <v>22.5433</v>
+        <v>0.3194</v>
       </c>
       <c r="U10" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="V10" t="n">
-        <v>-1.3313</v>
+        <v>-2.0595</v>
       </c>
       <c r="W10" t="n">
-        <v>9.7934</v>
+        <v>-2.181</v>
       </c>
       <c r="X10" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.0308</v>
+        <v>2.2876</v>
       </c>
       <c r="Z10" t="n">
-        <v>-20.86</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.3605</v>
+        <v>2.0211</v>
       </c>
       <c r="AC10" t="n">
-        <v>-9.6134</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C11" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D11" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E11" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F11" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G11" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I11" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K11" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L11" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M11" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N11" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O11" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P11" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q11" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R11" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S11" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="T11" t="n">
-        <v>0.3194</v>
+        <v>-3.2577</v>
       </c>
       <c r="U11" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V11" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.181</v>
+        <v>-3.9839</v>
       </c>
       <c r="X11" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z11" t="n">
-        <v>-1.3297</v>
+        <v>2.591</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB11" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
       <c r="AC11" t="n">
-        <v>2.0947</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C12" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D12" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E12" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F12" t="n">
         <v>78.13</v>
       </c>
       <c r="G12" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I12" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J12" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K12" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L12" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M12" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N12" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O12" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P12" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q12" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R12" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S12" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="T12" t="n">
-        <v>-3.2577</v>
+        <v>1.1009</v>
       </c>
       <c r="U12" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.9839</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X12" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y12" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="Z12" t="n">
-        <v>2.591</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
       <c r="AC12" t="n">
-        <v>4.0935</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C13" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D13" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E13" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F13" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G13" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H13" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I13" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J13" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K13" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L13" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M13" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N13" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O13" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P13" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q13" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R13" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S13" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T13" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U13" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z13" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C14" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D14" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E14" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F14" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G14" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H14" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I14" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K14" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L14" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M14" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N14" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O14" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P14" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q14" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R14" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S14" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T14" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U14" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V14" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X14" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y14" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z14" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB14" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC14" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C15" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D15" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E15" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F15" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G15" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H15" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J15" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K15" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L15" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M15" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N15" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O15" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P15" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q15" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R15" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S15" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T15" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U15" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V15" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W15" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X15" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y15" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z15" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA15" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB15" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC15" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C16" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D16" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E16" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F16" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I16" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J16" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K16" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L16" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M16" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N16" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O16" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P16" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q16" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R16" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S16" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T16" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U16" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V16" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W16" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X16" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y16" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z16" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA16" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC16" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C17" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D17" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E17" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F17" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H17" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J17" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K17" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L17" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M17" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N17" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O17" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P17" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q17" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S17" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T17" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U17" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V17" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W17" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X17" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y17" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z17" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA17" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC17" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C18" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D18" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E18" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F18" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G18" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I18" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J18" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K18" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L18" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M18" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N18" t="n">
         <v>32.58</v>
       </c>
       <c r="O18" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P18" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q18" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R18" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S18" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T18" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V18" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W18" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X18" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z18" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB18" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC18" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C19" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D19" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E19" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F19" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G19" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H19" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I19" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J19" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K19" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L19" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M19" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N19" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O19" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P19" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q19" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R19" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S19" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T19" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U19" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W19" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X19" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y19" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z19" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA19" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC19" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C20" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D20" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E20" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F20" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G20" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H20" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I20" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J20" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K20" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L20" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M20" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N20" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O20" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P20" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q20" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R20" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S20" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T20" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U20" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W20" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X20" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y20" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z20" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC20" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C21" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D21" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E21" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F21" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H21" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I21" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J21" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K21" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L21" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M21" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N21" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O21" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P21" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q21" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R21" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S21" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T21" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V21" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W21" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X21" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y21" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z21" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA21" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB21" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC21" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C22" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D22" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E22" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F22" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G22" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I22" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J22" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K22" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L22" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M22" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N22" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O22" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P22" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q22" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R22" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S22" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T22" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U22" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V22" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W22" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X22" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y22" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z22" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA22" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB22" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC22" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-17 00:10
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1810 +568,1810 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>107.3696</v>
+        <v>113.2557</v>
       </c>
       <c r="C2" t="n">
-        <v>109.2484</v>
+        <v>115.4043</v>
       </c>
       <c r="D2" t="n">
-        <v>100.9938</v>
+        <v>111.9366</v>
       </c>
       <c r="E2" t="n">
-        <v>103.9019</v>
+        <v>114.7448</v>
       </c>
       <c r="F2" t="n">
-        <v>68.7171</v>
+        <v>70.9927</v>
       </c>
       <c r="G2" t="n">
-        <v>69.83499999999999</v>
+        <v>71.58159999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>66.4216</v>
+        <v>70.2342</v>
       </c>
       <c r="I2" t="n">
-        <v>67.7989</v>
+        <v>71.2422</v>
       </c>
       <c r="J2" t="n">
-        <v>47.9509</v>
+        <v>45.1558</v>
       </c>
       <c r="K2" t="n">
-        <v>51.1015</v>
+        <v>45.7681</v>
       </c>
       <c r="L2" t="n">
-        <v>46.9829</v>
+        <v>44.1187</v>
       </c>
       <c r="M2" t="n">
-        <v>49.4916</v>
+        <v>44.4348</v>
       </c>
       <c r="N2" t="n">
-        <v>39.4989</v>
+        <v>38.1481</v>
       </c>
       <c r="O2" t="n">
-        <v>40.8596</v>
+        <v>38.5918</v>
       </c>
       <c r="P2" t="n">
-        <v>38.8186</v>
+        <v>37.7931</v>
       </c>
       <c r="Q2" t="n">
-        <v>40.0412</v>
+        <v>37.9903</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>113.2557</v>
+        <v>116.9533</v>
       </c>
       <c r="C3" t="n">
-        <v>115.4043</v>
+        <v>123.8188</v>
       </c>
       <c r="D3" t="n">
-        <v>111.9366</v>
+        <v>116.6035</v>
       </c>
       <c r="E3" t="n">
-        <v>114.7448</v>
+        <v>123.589</v>
       </c>
       <c r="F3" t="n">
-        <v>70.9927</v>
+        <v>71.7812</v>
       </c>
       <c r="G3" t="n">
-        <v>71.58159999999999</v>
+        <v>72.6395</v>
       </c>
       <c r="H3" t="n">
-        <v>70.2342</v>
+        <v>70.6733</v>
       </c>
       <c r="I3" t="n">
-        <v>71.2422</v>
+        <v>72.49979999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>45.1558</v>
+        <v>43.5656</v>
       </c>
       <c r="K3" t="n">
-        <v>45.7681</v>
+        <v>43.7138</v>
       </c>
       <c r="L3" t="n">
-        <v>44.1187</v>
+        <v>40.9582</v>
       </c>
       <c r="M3" t="n">
-        <v>44.4348</v>
+        <v>40.978</v>
       </c>
       <c r="N3" t="n">
-        <v>38.1481</v>
+        <v>37.7241</v>
       </c>
       <c r="O3" t="n">
-        <v>38.5918</v>
+        <v>38.3256</v>
       </c>
       <c r="P3" t="n">
-        <v>37.7931</v>
+        <v>37.2706</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.9903</v>
+        <v>37.3396</v>
       </c>
       <c r="R3" t="n">
-        <v>10.4357</v>
+        <v>7.7077</v>
       </c>
       <c r="U3" t="n">
-        <v>5.0787</v>
+        <v>1.7652</v>
       </c>
       <c r="X3" t="n">
-        <v>-10.2175</v>
+        <v>-7.7795</v>
       </c>
       <c r="AA3" t="n">
-        <v>-5.122</v>
+        <v>-1.7128</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>116.9533</v>
+        <v>131.9835</v>
       </c>
       <c r="C4" t="n">
-        <v>123.8188</v>
+        <v>143.9056</v>
       </c>
       <c r="D4" t="n">
-        <v>116.6035</v>
+        <v>129.5351</v>
       </c>
       <c r="E4" t="n">
-        <v>123.589</v>
+        <v>141.837</v>
       </c>
       <c r="F4" t="n">
-        <v>71.7812</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>72.6395</v>
+        <v>79.3366</v>
       </c>
       <c r="H4" t="n">
-        <v>70.6733</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>72.49979999999999</v>
+        <v>78.7577</v>
       </c>
       <c r="J4" t="n">
-        <v>43.5656</v>
+        <v>38.2718</v>
       </c>
       <c r="K4" t="n">
-        <v>43.7138</v>
+        <v>39.0224</v>
       </c>
       <c r="L4" t="n">
-        <v>40.9582</v>
+        <v>34.252</v>
       </c>
       <c r="M4" t="n">
-        <v>40.978</v>
+        <v>34.894</v>
       </c>
       <c r="N4" t="n">
-        <v>37.7241</v>
+        <v>36.2155</v>
       </c>
       <c r="O4" t="n">
-        <v>38.3256</v>
+        <v>36.2254</v>
       </c>
       <c r="P4" t="n">
-        <v>37.2706</v>
+        <v>33.8294</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.3396</v>
+        <v>34.1154</v>
       </c>
       <c r="R4" t="n">
-        <v>7.7077</v>
+        <v>14.7651</v>
       </c>
       <c r="U4" t="n">
-        <v>1.7652</v>
+        <v>8.631600000000001</v>
       </c>
       <c r="X4" t="n">
-        <v>-7.7795</v>
+        <v>-14.847</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.7128</v>
+        <v>-8.6348</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C5" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D5" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E5" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F5" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>79.3366</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>78.7577</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K5" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L5" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M5" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N5" t="n">
-        <v>36.2155</v>
+        <v>34.1745</v>
       </c>
       <c r="O5" t="n">
-        <v>36.2254</v>
+        <v>34.1745</v>
       </c>
       <c r="P5" t="n">
-        <v>33.8294</v>
+        <v>33.1688</v>
       </c>
       <c r="Q5" t="n">
-        <v>34.1154</v>
+        <v>33.297</v>
       </c>
       <c r="R5" t="n">
-        <v>14.7651</v>
+        <v>7.13</v>
       </c>
       <c r="S5" t="n">
-        <v>36.5105</v>
+        <v>32.4243</v>
       </c>
       <c r="U5" t="n">
-        <v>8.631600000000001</v>
+        <v>2.4332</v>
       </c>
       <c r="V5" t="n">
-        <v>16.1637</v>
+        <v>13.2391</v>
       </c>
       <c r="X5" t="n">
-        <v>-14.847</v>
+        <v>-7.09</v>
       </c>
       <c r="Y5" t="n">
-        <v>-29.4951</v>
+        <v>-27.0392</v>
       </c>
       <c r="AA5" t="n">
-        <v>-8.6348</v>
+        <v>-2.3989</v>
       </c>
       <c r="AB5" t="n">
-        <v>-14.7993</v>
+        <v>-12.3539</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C6" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D6" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E6" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F6" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G6" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I6" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J6" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K6" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L6" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M6" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N6" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O6" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P6" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q6" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
       <c r="R6" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="S6" t="n">
-        <v>32.4243</v>
+        <v>18.3358</v>
       </c>
       <c r="U6" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="V6" t="n">
-        <v>13.2391</v>
+        <v>8.4969</v>
       </c>
       <c r="X6" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="Y6" t="n">
-        <v>-27.0392</v>
+        <v>-17.8584</v>
       </c>
       <c r="AA6" t="n">
-        <v>-2.3989</v>
+        <v>2.5318</v>
       </c>
       <c r="AB6" t="n">
-        <v>-12.3539</v>
+        <v>-8.568899999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C7" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D7" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E7" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F7" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G7" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I7" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J7" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K7" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L7" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M7" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N7" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O7" t="n">
         <v>35.06</v>
       </c>
-      <c r="L7" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M7" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N7" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O7" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P7" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R7" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="S7" t="n">
-        <v>18.3358</v>
+        <v>3.1677</v>
       </c>
       <c r="T7" t="n">
-        <v>40.7578</v>
+        <v>27.5265</v>
       </c>
       <c r="U7" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="V7" t="n">
-        <v>8.4969</v>
+        <v>-0.2256</v>
       </c>
       <c r="W7" t="n">
-        <v>16.0196</v>
+        <v>10.2998</v>
       </c>
       <c r="X7" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y7" t="n">
-        <v>-17.8584</v>
+        <v>-3.6224</v>
       </c>
       <c r="Z7" t="n">
-        <v>-31.9885</v>
+        <v>-24.3161</v>
       </c>
       <c r="AA7" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
       <c r="AB7" t="n">
-        <v>-8.568899999999999</v>
+        <v>0.1894</v>
       </c>
       <c r="AC7" t="n">
-        <v>-14.7378</v>
+        <v>-10.0297</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C8" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D8" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E8" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F8" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G8" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H8" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I8" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K8" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L8" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M8" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N8" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O8" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P8" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q8" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R8" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="S8" t="n">
-        <v>3.1677</v>
+        <v>-0.3291</v>
       </c>
       <c r="T8" t="n">
-        <v>27.5265</v>
+        <v>22.5433</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.2256</v>
+        <v>-1.3313</v>
       </c>
       <c r="W8" t="n">
-        <v>10.2998</v>
+        <v>9.7934</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y8" t="n">
-        <v>-3.6224</v>
+        <v>0.0308</v>
       </c>
       <c r="Z8" t="n">
-        <v>-24.3161</v>
+        <v>-20.86</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.1894</v>
+        <v>1.3605</v>
       </c>
       <c r="AC8" t="n">
-        <v>-10.0297</v>
+        <v>-9.6134</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C9" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D9" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E9" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F9" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I9" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K9" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L9" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M9" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N9" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O9" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P9" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q9" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R9" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.3291</v>
+        <v>-2.7077</v>
       </c>
       <c r="T9" t="n">
-        <v>22.5433</v>
+        <v>0.3194</v>
       </c>
       <c r="U9" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="V9" t="n">
-        <v>-1.3313</v>
+        <v>-2.0595</v>
       </c>
       <c r="W9" t="n">
-        <v>9.7934</v>
+        <v>-2.181</v>
       </c>
       <c r="X9" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.0308</v>
+        <v>2.2876</v>
       </c>
       <c r="Z9" t="n">
-        <v>-20.86</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.3605</v>
+        <v>2.0211</v>
       </c>
       <c r="AC9" t="n">
-        <v>-9.6134</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C10" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D10" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E10" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F10" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G10" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I10" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K10" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L10" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M10" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N10" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O10" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P10" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q10" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R10" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="T10" t="n">
-        <v>0.3194</v>
+        <v>-3.2577</v>
       </c>
       <c r="U10" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V10" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="W10" t="n">
-        <v>-2.181</v>
+        <v>-3.9839</v>
       </c>
       <c r="X10" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y10" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z10" t="n">
-        <v>-1.3297</v>
+        <v>2.591</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB10" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
       <c r="AC10" t="n">
-        <v>2.0947</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C11" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D11" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E11" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F11" t="n">
         <v>78.13</v>
       </c>
       <c r="G11" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I11" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J11" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K11" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L11" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M11" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N11" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O11" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P11" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q11" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R11" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S11" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="T11" t="n">
-        <v>-3.2577</v>
+        <v>1.1009</v>
       </c>
       <c r="U11" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="W11" t="n">
-        <v>-3.9839</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X11" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y11" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.591</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB11" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
       <c r="AC11" t="n">
-        <v>4.0935</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C12" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D12" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E12" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F12" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G12" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H12" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I12" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J12" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K12" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L12" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M12" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N12" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O12" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P12" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q12" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R12" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S12" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T12" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U12" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y12" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z12" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C13" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D13" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E13" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F13" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G13" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H13" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I13" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K13" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L13" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M13" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N13" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O13" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P13" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q13" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R13" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S13" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T13" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U13" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V13" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X13" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y13" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z13" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB13" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC13" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C14" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D14" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E14" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F14" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G14" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H14" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J14" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K14" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L14" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M14" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N14" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O14" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P14" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q14" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R14" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S14" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T14" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U14" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V14" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W14" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X14" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y14" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z14" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB14" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC14" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C15" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D15" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E15" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F15" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I15" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J15" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K15" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L15" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M15" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N15" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O15" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P15" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q15" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R15" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S15" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T15" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U15" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V15" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W15" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X15" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y15" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z15" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA15" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC15" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C16" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D16" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E16" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F16" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H16" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J16" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K16" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L16" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M16" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N16" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O16" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P16" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S16" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T16" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U16" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V16" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W16" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X16" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y16" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z16" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA16" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC16" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C17" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D17" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E17" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F17" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G17" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I17" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J17" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K17" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L17" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M17" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N17" t="n">
         <v>32.58</v>
       </c>
       <c r="O17" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P17" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q17" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R17" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S17" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T17" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V17" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W17" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X17" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y17" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z17" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB17" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC17" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C18" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D18" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E18" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F18" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G18" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H18" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I18" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J18" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K18" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L18" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M18" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N18" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O18" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P18" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q18" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R18" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S18" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T18" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U18" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V18" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W18" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X18" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y18" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z18" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA18" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB18" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC18" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C19" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D19" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E19" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F19" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G19" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H19" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I19" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J19" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K19" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L19" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M19" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N19" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O19" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P19" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q19" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R19" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S19" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T19" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U19" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W19" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X19" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y19" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z19" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC19" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C20" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D20" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E20" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F20" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H20" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I20" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J20" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K20" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L20" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M20" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N20" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O20" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P20" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q20" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R20" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S20" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T20" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V20" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W20" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X20" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y20" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z20" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA20" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C21" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D21" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E21" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F21" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G21" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I21" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J21" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K21" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L21" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M21" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N21" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O21" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P21" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q21" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R21" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S21" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T21" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U21" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V21" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W21" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X21" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y21" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z21" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB21" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC21" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C22" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D22" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E22" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F22" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G22" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K22" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L22" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M22" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N22" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O22" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P22" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q22" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R22" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S22" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T22" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U22" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V22" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W22" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X22" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y22" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z22" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA22" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB22" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC22" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-20 00:55
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1810 +568,1719 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>113.2557</v>
+        <v>131.9835</v>
       </c>
       <c r="C2" t="n">
-        <v>115.4043</v>
+        <v>143.9056</v>
       </c>
       <c r="D2" t="n">
-        <v>111.9366</v>
+        <v>129.5351</v>
       </c>
       <c r="E2" t="n">
-        <v>114.7448</v>
+        <v>141.837</v>
       </c>
       <c r="F2" t="n">
-        <v>70.9927</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>71.58159999999999</v>
+        <v>79.3366</v>
       </c>
       <c r="H2" t="n">
-        <v>70.2342</v>
+        <v>74.68559999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>71.2422</v>
+        <v>78.7577</v>
       </c>
       <c r="J2" t="n">
-        <v>45.1558</v>
+        <v>38.2718</v>
       </c>
       <c r="K2" t="n">
-        <v>45.7681</v>
+        <v>39.0224</v>
       </c>
       <c r="L2" t="n">
-        <v>44.1187</v>
+        <v>34.252</v>
       </c>
       <c r="M2" t="n">
-        <v>44.4348</v>
+        <v>34.894</v>
       </c>
       <c r="N2" t="n">
-        <v>38.1481</v>
+        <v>36.2155</v>
       </c>
       <c r="O2" t="n">
-        <v>38.5918</v>
+        <v>36.2254</v>
       </c>
       <c r="P2" t="n">
-        <v>37.7931</v>
+        <v>33.8294</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.9903</v>
+        <v>34.1154</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>116.9533</v>
+        <v>137.67</v>
       </c>
       <c r="C3" t="n">
-        <v>123.8188</v>
+        <v>152.64</v>
       </c>
       <c r="D3" t="n">
-        <v>116.6035</v>
+        <v>137.46</v>
       </c>
       <c r="E3" t="n">
-        <v>123.589</v>
+        <v>151.95</v>
       </c>
       <c r="F3" t="n">
-        <v>71.7812</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>72.6395</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>70.6733</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>72.49979999999999</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>43.5656</v>
+        <v>35.98</v>
       </c>
       <c r="K3" t="n">
-        <v>43.7138</v>
+        <v>36.01</v>
       </c>
       <c r="L3" t="n">
-        <v>40.9582</v>
+        <v>32.25</v>
       </c>
       <c r="M3" t="n">
-        <v>40.978</v>
+        <v>32.42</v>
       </c>
       <c r="N3" t="n">
-        <v>37.7241</v>
+        <v>34.1745</v>
       </c>
       <c r="O3" t="n">
-        <v>38.3256</v>
+        <v>34.1745</v>
       </c>
       <c r="P3" t="n">
-        <v>37.2706</v>
+        <v>33.1688</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.3396</v>
+        <v>33.297</v>
       </c>
       <c r="R3" t="n">
-        <v>7.7077</v>
+        <v>7.13</v>
       </c>
       <c r="U3" t="n">
-        <v>1.7652</v>
+        <v>2.4332</v>
       </c>
       <c r="X3" t="n">
-        <v>-7.7795</v>
+        <v>-7.09</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.7128</v>
+        <v>-2.3989</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>131.9835</v>
+        <v>149.89</v>
       </c>
       <c r="C4" t="n">
-        <v>143.9056</v>
+        <v>151</v>
       </c>
       <c r="D4" t="n">
-        <v>129.5351</v>
+        <v>139.58</v>
       </c>
       <c r="E4" t="n">
-        <v>141.837</v>
+        <v>146.25</v>
       </c>
       <c r="F4" t="n">
-        <v>74.68559999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G4" t="n">
-        <v>79.3366</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>74.68559999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I4" t="n">
-        <v>78.7577</v>
+        <v>78.66</v>
       </c>
       <c r="J4" t="n">
-        <v>38.2718</v>
+        <v>32.87</v>
       </c>
       <c r="K4" t="n">
-        <v>39.0224</v>
+        <v>35.06</v>
       </c>
       <c r="L4" t="n">
-        <v>34.252</v>
+        <v>32.63</v>
       </c>
       <c r="M4" t="n">
-        <v>34.894</v>
+        <v>33.66</v>
       </c>
       <c r="N4" t="n">
-        <v>36.2155</v>
+        <v>33.37</v>
       </c>
       <c r="O4" t="n">
-        <v>36.2254</v>
+        <v>34.54</v>
       </c>
       <c r="P4" t="n">
-        <v>33.8294</v>
+        <v>33.35</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.1154</v>
+        <v>34.14</v>
       </c>
       <c r="R4" t="n">
-        <v>14.7651</v>
+        <v>-3.7512</v>
       </c>
       <c r="U4" t="n">
-        <v>8.631600000000001</v>
+        <v>-2.4965</v>
       </c>
       <c r="X4" t="n">
-        <v>-14.847</v>
+        <v>3.8248</v>
       </c>
       <c r="AA4" t="n">
-        <v>-8.6348</v>
+        <v>2.5318</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>137.67</v>
+        <v>138.47</v>
       </c>
       <c r="C5" t="n">
-        <v>152.64</v>
+        <v>147.2</v>
       </c>
       <c r="D5" t="n">
-        <v>137.46</v>
+        <v>136.9</v>
       </c>
       <c r="E5" t="n">
-        <v>151.95</v>
+        <v>146.33</v>
       </c>
       <c r="F5" t="n">
-        <v>78.61799999999999</v>
+        <v>76.75</v>
       </c>
       <c r="G5" t="n">
-        <v>80.96339999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>78.61799999999999</v>
+        <v>76.55</v>
       </c>
       <c r="I5" t="n">
-        <v>80.67400000000001</v>
+        <v>78.58</v>
       </c>
       <c r="J5" t="n">
-        <v>35.98</v>
+        <v>35.45</v>
       </c>
       <c r="K5" t="n">
-        <v>36.01</v>
+        <v>35.85</v>
       </c>
       <c r="L5" t="n">
-        <v>32.25</v>
+        <v>33.43</v>
       </c>
       <c r="M5" t="n">
-        <v>32.42</v>
+        <v>33.63</v>
       </c>
       <c r="N5" t="n">
-        <v>34.1745</v>
+        <v>34.98</v>
       </c>
       <c r="O5" t="n">
-        <v>34.1745</v>
+        <v>35.06</v>
       </c>
       <c r="P5" t="n">
-        <v>33.1688</v>
+        <v>33.95</v>
       </c>
       <c r="Q5" t="n">
-        <v>33.297</v>
+        <v>34.18</v>
       </c>
       <c r="R5" t="n">
-        <v>7.13</v>
+        <v>0.0547</v>
       </c>
       <c r="S5" t="n">
-        <v>32.4243</v>
+        <v>3.1677</v>
       </c>
       <c r="U5" t="n">
-        <v>2.4332</v>
+        <v>-0.1017</v>
       </c>
       <c r="V5" t="n">
-        <v>13.2391</v>
+        <v>-0.2256</v>
       </c>
       <c r="X5" t="n">
-        <v>-7.09</v>
+        <v>-0.0891</v>
       </c>
       <c r="Y5" t="n">
-        <v>-27.0392</v>
+        <v>-3.6224</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.3989</v>
+        <v>0.1172</v>
       </c>
       <c r="AB5" t="n">
-        <v>-12.3539</v>
+        <v>0.1894</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>149.89</v>
+        <v>149.24</v>
       </c>
       <c r="C6" t="n">
-        <v>151</v>
+        <v>153.9</v>
       </c>
       <c r="D6" t="n">
-        <v>139.58</v>
+        <v>147.39</v>
       </c>
       <c r="E6" t="n">
-        <v>146.25</v>
+        <v>151.45</v>
       </c>
       <c r="F6" t="n">
-        <v>80.53</v>
+        <v>79.09</v>
       </c>
       <c r="G6" t="n">
-        <v>80.56999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H6" t="n">
-        <v>77.69</v>
+        <v>78.06</v>
       </c>
       <c r="I6" t="n">
-        <v>78.66</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>32.87</v>
+        <v>32.97</v>
       </c>
       <c r="K6" t="n">
-        <v>35.06</v>
+        <v>33.39</v>
       </c>
       <c r="L6" t="n">
-        <v>32.63</v>
+        <v>31.9</v>
       </c>
       <c r="M6" t="n">
-        <v>33.66</v>
+        <v>32.43</v>
       </c>
       <c r="N6" t="n">
-        <v>33.37</v>
+        <v>33.97</v>
       </c>
       <c r="O6" t="n">
-        <v>34.54</v>
+        <v>34.41</v>
       </c>
       <c r="P6" t="n">
-        <v>33.35</v>
+        <v>33.54</v>
       </c>
       <c r="Q6" t="n">
-        <v>34.14</v>
+        <v>33.75</v>
       </c>
       <c r="R6" t="n">
-        <v>-3.7512</v>
+        <v>3.4989</v>
       </c>
       <c r="S6" t="n">
-        <v>18.3358</v>
+        <v>-0.3291</v>
       </c>
       <c r="U6" t="n">
-        <v>-2.4965</v>
+        <v>1.298</v>
       </c>
       <c r="V6" t="n">
-        <v>8.4969</v>
+        <v>-1.3313</v>
       </c>
       <c r="X6" t="n">
-        <v>3.8248</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y6" t="n">
-        <v>-17.8584</v>
+        <v>0.0308</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.5318</v>
+        <v>-1.258</v>
       </c>
       <c r="AB6" t="n">
-        <v>-8.568899999999999</v>
+        <v>1.3605</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>138.47</v>
+        <v>148.14</v>
       </c>
       <c r="C7" t="n">
-        <v>147.2</v>
+        <v>149.99</v>
       </c>
       <c r="D7" t="n">
-        <v>136.9</v>
+        <v>135.21</v>
       </c>
       <c r="E7" t="n">
-        <v>146.33</v>
+        <v>142.29</v>
       </c>
       <c r="F7" t="n">
-        <v>76.75</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>79.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>76.55</v>
+        <v>75.47</v>
       </c>
       <c r="I7" t="n">
-        <v>78.58</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>35.45</v>
+        <v>33.17</v>
       </c>
       <c r="K7" t="n">
-        <v>35.85</v>
+        <v>35.95</v>
       </c>
       <c r="L7" t="n">
-        <v>33.43</v>
+        <v>32.77</v>
       </c>
       <c r="M7" t="n">
-        <v>33.63</v>
+        <v>34.43</v>
       </c>
       <c r="N7" t="n">
-        <v>34.98</v>
+        <v>34.31</v>
       </c>
       <c r="O7" t="n">
-        <v>35.06</v>
+        <v>35.53</v>
       </c>
       <c r="P7" t="n">
-        <v>33.95</v>
+        <v>34.17</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.18</v>
+        <v>34.83</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0547</v>
+        <v>-6.0482</v>
       </c>
       <c r="S7" t="n">
-        <v>3.1677</v>
+        <v>-2.7077</v>
       </c>
       <c r="T7" t="n">
-        <v>27.5265</v>
+        <v>0.3194</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.1017</v>
+        <v>-3.2161</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.2256</v>
+        <v>-2.0595</v>
       </c>
       <c r="W7" t="n">
-        <v>10.2998</v>
+        <v>-2.181</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.0891</v>
+        <v>6.1671</v>
       </c>
       <c r="Y7" t="n">
-        <v>-3.6224</v>
+        <v>2.2876</v>
       </c>
       <c r="Z7" t="n">
-        <v>-24.3161</v>
+        <v>-1.3297</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.1172</v>
+        <v>3.2</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.1894</v>
+        <v>2.0211</v>
       </c>
       <c r="AC7" t="n">
-        <v>-10.0297</v>
+        <v>2.0947</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>149.24</v>
+        <v>148.94</v>
       </c>
       <c r="C8" t="n">
-        <v>153.9</v>
+        <v>152.37</v>
       </c>
       <c r="D8" t="n">
-        <v>147.39</v>
+        <v>145.49</v>
       </c>
       <c r="E8" t="n">
-        <v>151.45</v>
+        <v>147</v>
       </c>
       <c r="F8" t="n">
-        <v>79.09</v>
+        <v>78.13</v>
       </c>
       <c r="G8" t="n">
-        <v>80.06</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>78.06</v>
+        <v>76.62</v>
       </c>
       <c r="I8" t="n">
-        <v>79.59999999999999</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>32.97</v>
+        <v>32.82</v>
       </c>
       <c r="K8" t="n">
-        <v>33.39</v>
+        <v>33.64</v>
       </c>
       <c r="L8" t="n">
-        <v>31.9</v>
+        <v>31.96</v>
       </c>
       <c r="M8" t="n">
-        <v>32.43</v>
+        <v>33.26</v>
       </c>
       <c r="N8" t="n">
-        <v>33.97</v>
+        <v>34.34</v>
       </c>
       <c r="O8" t="n">
-        <v>34.41</v>
+        <v>35.02</v>
       </c>
       <c r="P8" t="n">
-        <v>33.54</v>
+        <v>34.28</v>
       </c>
       <c r="Q8" t="n">
-        <v>33.75</v>
+        <v>34.66</v>
       </c>
       <c r="R8" t="n">
-        <v>3.4989</v>
+        <v>3.3101</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.3291</v>
+        <v>0.4579</v>
       </c>
       <c r="T8" t="n">
-        <v>22.5433</v>
+        <v>-3.2577</v>
       </c>
       <c r="U8" t="n">
-        <v>1.298</v>
+        <v>0.5452</v>
       </c>
       <c r="V8" t="n">
-        <v>-1.3313</v>
+        <v>-1.4253</v>
       </c>
       <c r="W8" t="n">
-        <v>9.7934</v>
+        <v>-3.9839</v>
       </c>
       <c r="X8" t="n">
-        <v>-3.5682</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.0308</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z8" t="n">
-        <v>-20.86</v>
+        <v>2.591</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.258</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.3605</v>
+        <v>1.4043</v>
       </c>
       <c r="AC8" t="n">
-        <v>-9.6134</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>148.14</v>
+        <v>147.95</v>
       </c>
       <c r="C9" t="n">
-        <v>149.99</v>
+        <v>150.77</v>
       </c>
       <c r="D9" t="n">
-        <v>135.21</v>
+        <v>144.41</v>
       </c>
       <c r="E9" t="n">
-        <v>142.29</v>
+        <v>147.86</v>
       </c>
       <c r="F9" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G9" t="n">
-        <v>78.59999999999999</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>75.47</v>
+        <v>77.94</v>
       </c>
       <c r="I9" t="n">
-        <v>77.04000000000001</v>
+        <v>78.03</v>
       </c>
       <c r="J9" t="n">
-        <v>33.17</v>
+        <v>33.07</v>
       </c>
       <c r="K9" t="n">
-        <v>35.95</v>
+        <v>33.86</v>
       </c>
       <c r="L9" t="n">
-        <v>32.77</v>
+        <v>32.42</v>
       </c>
       <c r="M9" t="n">
-        <v>34.43</v>
+        <v>33.08</v>
       </c>
       <c r="N9" t="n">
-        <v>34.31</v>
+        <v>34.36</v>
       </c>
       <c r="O9" t="n">
-        <v>35.53</v>
+        <v>34.44</v>
       </c>
       <c r="P9" t="n">
-        <v>34.17</v>
+        <v>33.66</v>
       </c>
       <c r="Q9" t="n">
-        <v>34.83</v>
+        <v>34.41</v>
       </c>
       <c r="R9" t="n">
-        <v>-6.0482</v>
+        <v>0.585</v>
       </c>
       <c r="S9" t="n">
-        <v>-2.7077</v>
+        <v>-2.3704</v>
       </c>
       <c r="T9" t="n">
-        <v>0.3194</v>
+        <v>1.1009</v>
       </c>
       <c r="U9" t="n">
-        <v>-3.2161</v>
+        <v>0.7359</v>
       </c>
       <c r="V9" t="n">
-        <v>-2.0595</v>
+        <v>-1.9724</v>
       </c>
       <c r="W9" t="n">
-        <v>-2.181</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X9" t="n">
-        <v>6.1671</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.2876</v>
+        <v>2.0043</v>
       </c>
       <c r="Z9" t="n">
-        <v>-1.3297</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA9" t="n">
-        <v>3.2</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB9" t="n">
-        <v>2.0211</v>
+        <v>1.9556</v>
       </c>
       <c r="AC9" t="n">
-        <v>2.0947</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>148.94</v>
+        <v>148.56</v>
       </c>
       <c r="C10" t="n">
-        <v>152.37</v>
+        <v>156.71</v>
       </c>
       <c r="D10" t="n">
-        <v>145.49</v>
+        <v>144.31</v>
       </c>
       <c r="E10" t="n">
-        <v>147</v>
+        <v>153.69</v>
       </c>
       <c r="F10" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G10" t="n">
-        <v>78.26000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H10" t="n">
-        <v>76.62</v>
+        <v>76.87</v>
       </c>
       <c r="I10" t="n">
-        <v>77.45999999999999</v>
+        <v>78.73</v>
       </c>
       <c r="J10" t="n">
-        <v>32.82</v>
+        <v>32.95</v>
       </c>
       <c r="K10" t="n">
-        <v>33.64</v>
+        <v>33.89</v>
       </c>
       <c r="L10" t="n">
-        <v>31.96</v>
+        <v>31.1</v>
       </c>
       <c r="M10" t="n">
-        <v>33.26</v>
+        <v>31.76</v>
       </c>
       <c r="N10" t="n">
-        <v>34.34</v>
+        <v>34.04</v>
       </c>
       <c r="O10" t="n">
-        <v>35.02</v>
+        <v>34.92</v>
       </c>
       <c r="P10" t="n">
-        <v>34.28</v>
+        <v>33.74</v>
       </c>
       <c r="Q10" t="n">
-        <v>34.66</v>
+        <v>34.11</v>
       </c>
       <c r="R10" t="n">
-        <v>3.3101</v>
+        <v>3.9429</v>
       </c>
       <c r="S10" t="n">
-        <v>0.4579</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T10" t="n">
-        <v>-3.2577</v>
+        <v>5.0297</v>
       </c>
       <c r="U10" t="n">
-        <v>0.5452</v>
+        <v>0.8971</v>
       </c>
       <c r="V10" t="n">
-        <v>-1.4253</v>
+        <v>2.1937</v>
       </c>
       <c r="W10" t="n">
-        <v>-3.9839</v>
+        <v>0.1909</v>
       </c>
       <c r="X10" t="n">
-        <v>-3.3982</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y10" t="n">
-        <v>-1.1002</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z10" t="n">
-        <v>2.591</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.4881</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.4043</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC10" t="n">
-        <v>4.0935</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>147.95</v>
+        <v>165.39</v>
       </c>
       <c r="C11" t="n">
-        <v>150.77</v>
+        <v>169.75</v>
       </c>
       <c r="D11" t="n">
-        <v>144.41</v>
+        <v>162.4</v>
       </c>
       <c r="E11" t="n">
-        <v>147.86</v>
+        <v>163.71</v>
       </c>
       <c r="F11" t="n">
-        <v>78.13</v>
+        <v>81.59</v>
       </c>
       <c r="G11" t="n">
-        <v>79.68000000000001</v>
+        <v>82.61</v>
       </c>
       <c r="H11" t="n">
-        <v>77.94</v>
+        <v>80.37</v>
       </c>
       <c r="I11" t="n">
-        <v>78.03</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>33.07</v>
+        <v>29.39</v>
       </c>
       <c r="K11" t="n">
-        <v>33.86</v>
+        <v>29.98</v>
       </c>
       <c r="L11" t="n">
-        <v>32.42</v>
+        <v>28.46</v>
       </c>
       <c r="M11" t="n">
-        <v>33.08</v>
+        <v>29.71</v>
       </c>
       <c r="N11" t="n">
-        <v>34.36</v>
+        <v>32.87</v>
       </c>
       <c r="O11" t="n">
-        <v>34.44</v>
+        <v>33.41</v>
       </c>
       <c r="P11" t="n">
-        <v>33.66</v>
+        <v>32.44</v>
       </c>
       <c r="Q11" t="n">
-        <v>34.41</v>
+        <v>33.12</v>
       </c>
       <c r="R11" t="n">
-        <v>0.585</v>
+        <v>6.5196</v>
       </c>
       <c r="S11" t="n">
-        <v>-2.3704</v>
+        <v>11.3673</v>
       </c>
       <c r="T11" t="n">
-        <v>1.1009</v>
+        <v>8.0951</v>
       </c>
       <c r="U11" t="n">
-        <v>0.7359</v>
+        <v>2.896</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.9724</v>
+        <v>4.583</v>
       </c>
       <c r="W11" t="n">
-        <v>-0.8008999999999999</v>
+        <v>1.7714</v>
       </c>
       <c r="X11" t="n">
-        <v>-0.5412</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.0043</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z11" t="n">
-        <v>-1.7231</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB11" t="n">
-        <v>1.9556</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.7909</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>148.56</v>
+        <v>161.66</v>
       </c>
       <c r="C12" t="n">
-        <v>156.71</v>
+        <v>164.38</v>
       </c>
       <c r="D12" t="n">
-        <v>144.31</v>
+        <v>158.08</v>
       </c>
       <c r="E12" t="n">
-        <v>153.69</v>
+        <v>164.27</v>
       </c>
       <c r="F12" t="n">
-        <v>78.88</v>
+        <v>80.95</v>
       </c>
       <c r="G12" t="n">
-        <v>79.53</v>
+        <v>83.38</v>
       </c>
       <c r="H12" t="n">
-        <v>76.87</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>78.73</v>
+        <v>83.12</v>
       </c>
       <c r="J12" t="n">
-        <v>32.95</v>
+        <v>30.09</v>
       </c>
       <c r="K12" t="n">
-        <v>33.89</v>
+        <v>30.75</v>
       </c>
       <c r="L12" t="n">
-        <v>31.1</v>
+        <v>29.62</v>
       </c>
       <c r="M12" t="n">
-        <v>31.76</v>
+        <v>29.62</v>
       </c>
       <c r="N12" t="n">
-        <v>34.04</v>
+        <v>33.17</v>
       </c>
       <c r="O12" t="n">
-        <v>34.92</v>
+        <v>33.2</v>
       </c>
       <c r="P12" t="n">
-        <v>33.74</v>
+        <v>32.16</v>
       </c>
       <c r="Q12" t="n">
-        <v>34.11</v>
+        <v>32.25</v>
       </c>
       <c r="R12" t="n">
-        <v>3.9429</v>
+        <v>0.3421</v>
       </c>
       <c r="S12" t="n">
-        <v>8.011799999999999</v>
+        <v>11.0983</v>
       </c>
       <c r="T12" t="n">
-        <v>5.0297</v>
+        <v>15.4473</v>
       </c>
       <c r="U12" t="n">
-        <v>0.8971</v>
+        <v>2.6046</v>
       </c>
       <c r="V12" t="n">
-        <v>2.1937</v>
+        <v>6.5231</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1909</v>
+        <v>7.892</v>
       </c>
       <c r="X12" t="n">
-        <v>-3.9903</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y12" t="n">
-        <v>-7.7549</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z12" t="n">
-        <v>-5.5605</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.8718</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB12" t="n">
-        <v>-2.0672</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC12" t="n">
-        <v>-0.2048</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>165.39</v>
+        <v>167.34</v>
       </c>
       <c r="C13" t="n">
-        <v>169.75</v>
+        <v>169.83</v>
       </c>
       <c r="D13" t="n">
-        <v>162.4</v>
+        <v>163.42</v>
       </c>
       <c r="E13" t="n">
-        <v>163.71</v>
+        <v>164.26</v>
       </c>
       <c r="F13" t="n">
-        <v>81.59</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>82.61</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>80.37</v>
+        <v>84.09</v>
       </c>
       <c r="I13" t="n">
-        <v>81.01000000000001</v>
+        <v>84.25</v>
       </c>
       <c r="J13" t="n">
-        <v>29.39</v>
+        <v>29.06</v>
       </c>
       <c r="K13" t="n">
-        <v>29.98</v>
+        <v>29.77</v>
       </c>
       <c r="L13" t="n">
-        <v>28.46</v>
+        <v>28.62</v>
       </c>
       <c r="M13" t="n">
-        <v>29.71</v>
+        <v>29.63</v>
       </c>
       <c r="N13" t="n">
-        <v>32.87</v>
+        <v>31.72</v>
       </c>
       <c r="O13" t="n">
-        <v>33.41</v>
+        <v>31.9</v>
       </c>
       <c r="P13" t="n">
-        <v>32.44</v>
+        <v>31.42</v>
       </c>
       <c r="Q13" t="n">
-        <v>33.12</v>
+        <v>31.83</v>
       </c>
       <c r="R13" t="n">
-        <v>6.5196</v>
+        <v>-0.0061</v>
       </c>
       <c r="S13" t="n">
-        <v>11.3673</v>
+        <v>6.8775</v>
       </c>
       <c r="T13" t="n">
-        <v>8.0951</v>
+        <v>11.7415</v>
       </c>
       <c r="U13" t="n">
-        <v>2.896</v>
+        <v>1.3595</v>
       </c>
       <c r="V13" t="n">
-        <v>4.583</v>
+        <v>7.0113</v>
       </c>
       <c r="W13" t="n">
-        <v>1.7714</v>
+        <v>8.7658</v>
       </c>
       <c r="X13" t="n">
-        <v>-6.4547</v>
+        <v>0.0338</v>
       </c>
       <c r="Y13" t="n">
-        <v>-10.6735</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z13" t="n">
-        <v>-8.3873</v>
+        <v>-10.914</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.9024</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB13" t="n">
-        <v>-4.4432</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC13" t="n">
-        <v>-1.8667</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>161.66</v>
+        <v>153.7</v>
       </c>
       <c r="C14" t="n">
-        <v>164.38</v>
+        <v>159.49</v>
       </c>
       <c r="D14" t="n">
-        <v>158.08</v>
+        <v>151.42</v>
       </c>
       <c r="E14" t="n">
-        <v>164.27</v>
+        <v>158.91</v>
       </c>
       <c r="F14" t="n">
-        <v>80.95</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>83.38</v>
+        <v>83.75</v>
       </c>
       <c r="H14" t="n">
-        <v>80.84999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>83.12</v>
+        <v>83.62</v>
       </c>
       <c r="J14" t="n">
-        <v>30.09</v>
+        <v>31.55</v>
       </c>
       <c r="K14" t="n">
-        <v>30.75</v>
+        <v>31.97</v>
       </c>
       <c r="L14" t="n">
-        <v>29.62</v>
+        <v>30.5</v>
       </c>
       <c r="M14" t="n">
-        <v>29.62</v>
+        <v>30.65</v>
       </c>
       <c r="N14" t="n">
-        <v>33.17</v>
+        <v>32.58</v>
       </c>
       <c r="O14" t="n">
-        <v>33.2</v>
+        <v>32.84</v>
       </c>
       <c r="P14" t="n">
-        <v>32.16</v>
+        <v>32.02</v>
       </c>
       <c r="Q14" t="n">
-        <v>32.25</v>
+        <v>32.07</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3421</v>
+        <v>-3.257</v>
       </c>
       <c r="S14" t="n">
-        <v>11.0983</v>
+        <v>-2.932</v>
       </c>
       <c r="T14" t="n">
-        <v>15.4473</v>
+        <v>7.4733</v>
       </c>
       <c r="U14" t="n">
-        <v>2.6046</v>
+        <v>-0.7478</v>
       </c>
       <c r="V14" t="n">
-        <v>6.5231</v>
+        <v>3.2218</v>
       </c>
       <c r="W14" t="n">
-        <v>7.892</v>
+        <v>7.1639</v>
       </c>
       <c r="X14" t="n">
-        <v>-0.3029</v>
+        <v>3.4425</v>
       </c>
       <c r="Y14" t="n">
-        <v>-10.4595</v>
+        <v>3.1639</v>
       </c>
       <c r="Z14" t="n">
-        <v>-13.9704</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.6268</v>
+        <v>0.754</v>
       </c>
       <c r="AB14" t="n">
-        <v>-6.2772</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC14" t="n">
-        <v>-7.4074</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>167.34</v>
+        <v>150.48</v>
       </c>
       <c r="C15" t="n">
-        <v>169.83</v>
+        <v>155.5</v>
       </c>
       <c r="D15" t="n">
-        <v>163.42</v>
+        <v>136.32</v>
       </c>
       <c r="E15" t="n">
-        <v>164.26</v>
+        <v>142.52</v>
       </c>
       <c r="F15" t="n">
-        <v>84.54000000000001</v>
+        <v>82.33</v>
       </c>
       <c r="G15" t="n">
-        <v>85.31999999999999</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>84.09</v>
+        <v>78.78</v>
       </c>
       <c r="I15" t="n">
-        <v>84.25</v>
+        <v>80.23</v>
       </c>
       <c r="J15" t="n">
-        <v>29.06</v>
+        <v>32.25</v>
       </c>
       <c r="K15" t="n">
-        <v>29.77</v>
+        <v>34.96</v>
       </c>
       <c r="L15" t="n">
-        <v>28.62</v>
+        <v>31.25</v>
       </c>
       <c r="M15" t="n">
-        <v>29.63</v>
+        <v>33.79</v>
       </c>
       <c r="N15" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O15" t="n">
-        <v>31.9</v>
+        <v>33.94</v>
       </c>
       <c r="P15" t="n">
-        <v>31.42</v>
+        <v>32.16</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.83</v>
+        <v>33.37</v>
       </c>
       <c r="R15" t="n">
-        <v>-0.0061</v>
+        <v>-10.314</v>
       </c>
       <c r="S15" t="n">
-        <v>6.8775</v>
+        <v>-13.2404</v>
       </c>
       <c r="T15" t="n">
-        <v>11.7415</v>
+        <v>-7.2679</v>
       </c>
       <c r="U15" t="n">
-        <v>1.3595</v>
+        <v>-4.0541</v>
       </c>
       <c r="V15" t="n">
-        <v>7.0113</v>
+        <v>-3.4769</v>
       </c>
       <c r="W15" t="n">
-        <v>8.7658</v>
+        <v>1.9052</v>
       </c>
       <c r="X15" t="n">
-        <v>0.0338</v>
+        <v>10.2447</v>
       </c>
       <c r="Y15" t="n">
-        <v>-6.7065</v>
+        <v>14.0783</v>
       </c>
       <c r="Z15" t="n">
-        <v>-10.914</v>
+        <v>6.3917</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.3023</v>
+        <v>4.0536</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.6843</v>
+        <v>3.4729</v>
       </c>
       <c r="AC15" t="n">
-        <v>-8.164999999999999</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>153.7</v>
+        <v>148.18</v>
       </c>
       <c r="C16" t="n">
-        <v>159.49</v>
+        <v>148.18</v>
       </c>
       <c r="D16" t="n">
-        <v>151.42</v>
+        <v>137.71</v>
       </c>
       <c r="E16" t="n">
-        <v>158.91</v>
+        <v>139.76</v>
       </c>
       <c r="F16" t="n">
-        <v>82.31999999999999</v>
+        <v>81.72</v>
       </c>
       <c r="G16" t="n">
-        <v>83.75</v>
+        <v>81.81</v>
       </c>
       <c r="H16" t="n">
-        <v>81.59999999999999</v>
+        <v>80.37</v>
       </c>
       <c r="I16" t="n">
-        <v>83.62</v>
+        <v>81.28</v>
       </c>
       <c r="J16" t="n">
-        <v>31.55</v>
+        <v>32.4</v>
       </c>
       <c r="K16" t="n">
-        <v>31.97</v>
+        <v>34.91</v>
       </c>
       <c r="L16" t="n">
-        <v>30.5</v>
+        <v>32.39</v>
       </c>
       <c r="M16" t="n">
-        <v>30.65</v>
+        <v>34.39</v>
       </c>
       <c r="N16" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O16" t="n">
-        <v>32.84</v>
+        <v>33.34</v>
       </c>
       <c r="P16" t="n">
-        <v>32.02</v>
+        <v>32.73</v>
       </c>
       <c r="Q16" t="n">
-        <v>32.07</v>
+        <v>32.95</v>
       </c>
       <c r="R16" t="n">
-        <v>-3.257</v>
+        <v>-1.9366</v>
       </c>
       <c r="S16" t="n">
-        <v>-2.932</v>
+        <v>-14.9154</v>
       </c>
       <c r="T16" t="n">
-        <v>7.4733</v>
+        <v>-14.6295</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.7478</v>
+        <v>1.3087</v>
       </c>
       <c r="V16" t="n">
-        <v>3.2218</v>
+        <v>-3.5252</v>
       </c>
       <c r="W16" t="n">
-        <v>7.1639</v>
+        <v>0.3333</v>
       </c>
       <c r="X16" t="n">
-        <v>3.4425</v>
+        <v>1.7757</v>
       </c>
       <c r="Y16" t="n">
-        <v>3.1639</v>
+        <v>16.0648</v>
       </c>
       <c r="Z16" t="n">
-        <v>-7.3458</v>
+        <v>15.7523</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.754</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB16" t="n">
-        <v>-3.1703</v>
+        <v>3.5187</v>
       </c>
       <c r="AC16" t="n">
-        <v>-6.8003</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>150.48</v>
+        <v>134.43</v>
       </c>
       <c r="C17" t="n">
-        <v>155.5</v>
+        <v>134.54</v>
       </c>
       <c r="D17" t="n">
-        <v>136.32</v>
+        <v>127.27</v>
       </c>
       <c r="E17" t="n">
-        <v>142.52</v>
+        <v>128.4</v>
       </c>
       <c r="F17" t="n">
-        <v>82.33</v>
+        <v>80.78</v>
       </c>
       <c r="G17" t="n">
-        <v>83.40000000000001</v>
+        <v>80.81</v>
       </c>
       <c r="H17" t="n">
-        <v>78.78</v>
+        <v>79.22</v>
       </c>
       <c r="I17" t="n">
-        <v>80.23</v>
+        <v>79.61</v>
       </c>
       <c r="J17" t="n">
-        <v>32.25</v>
+        <v>35.75</v>
       </c>
       <c r="K17" t="n">
-        <v>34.96</v>
+        <v>37.5</v>
       </c>
       <c r="L17" t="n">
-        <v>31.25</v>
+        <v>35.68</v>
       </c>
       <c r="M17" t="n">
-        <v>33.79</v>
+        <v>37.19</v>
       </c>
       <c r="N17" t="n">
-        <v>32.58</v>
+        <v>33.17</v>
       </c>
       <c r="O17" t="n">
-        <v>33.94</v>
+        <v>33.8</v>
       </c>
       <c r="P17" t="n">
-        <v>32.16</v>
+        <v>33.17</v>
       </c>
       <c r="Q17" t="n">
-        <v>33.37</v>
+        <v>33.63</v>
       </c>
       <c r="R17" t="n">
-        <v>-10.314</v>
+        <v>-8.1282</v>
       </c>
       <c r="S17" t="n">
-        <v>-13.2404</v>
+        <v>-19.1995</v>
       </c>
       <c r="T17" t="n">
-        <v>-7.2679</v>
+        <v>-21.836</v>
       </c>
       <c r="U17" t="n">
-        <v>-4.0541</v>
+        <v>-2.0546</v>
       </c>
       <c r="V17" t="n">
-        <v>-3.4769</v>
+        <v>-4.7955</v>
       </c>
       <c r="W17" t="n">
-        <v>1.9052</v>
+        <v>-4.2228</v>
       </c>
       <c r="X17" t="n">
-        <v>10.2447</v>
+        <v>8.1419</v>
       </c>
       <c r="Y17" t="n">
-        <v>14.0783</v>
+        <v>21.3377</v>
       </c>
       <c r="Z17" t="n">
-        <v>6.3917</v>
+        <v>25.5571</v>
       </c>
       <c r="AA17" t="n">
-        <v>4.0536</v>
+        <v>2.0637</v>
       </c>
       <c r="AB17" t="n">
-        <v>3.4729</v>
+        <v>4.8644</v>
       </c>
       <c r="AC17" t="n">
-        <v>-2.1695</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>148.18</v>
+        <v>118.42</v>
       </c>
       <c r="C18" t="n">
-        <v>148.18</v>
+        <v>127.92</v>
       </c>
       <c r="D18" t="n">
-        <v>137.71</v>
+        <v>115.84</v>
       </c>
       <c r="E18" t="n">
-        <v>139.76</v>
+        <v>127.57</v>
       </c>
       <c r="F18" t="n">
-        <v>81.72</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>81.81</v>
+        <v>79</v>
       </c>
       <c r="H18" t="n">
-        <v>80.37</v>
+        <v>77.28</v>
       </c>
       <c r="I18" t="n">
-        <v>81.28</v>
+        <v>78.81</v>
       </c>
       <c r="J18" t="n">
-        <v>32.4</v>
+        <v>40.15</v>
       </c>
       <c r="K18" t="n">
-        <v>34.91</v>
+        <v>40.9</v>
       </c>
       <c r="L18" t="n">
-        <v>32.39</v>
+        <v>37.36</v>
       </c>
       <c r="M18" t="n">
-        <v>34.39</v>
+        <v>37.42</v>
       </c>
       <c r="N18" t="n">
-        <v>32.78</v>
+        <v>34.54</v>
       </c>
       <c r="O18" t="n">
-        <v>33.34</v>
+        <v>34.63</v>
       </c>
       <c r="P18" t="n">
-        <v>32.73</v>
+        <v>33.89</v>
       </c>
       <c r="Q18" t="n">
-        <v>32.95</v>
+        <v>33.99</v>
       </c>
       <c r="R18" t="n">
-        <v>-1.9366</v>
+        <v>-0.6464</v>
       </c>
       <c r="S18" t="n">
-        <v>-14.9154</v>
+        <v>-10.4898</v>
       </c>
       <c r="T18" t="n">
-        <v>-14.6295</v>
+        <v>-22.3365</v>
       </c>
       <c r="U18" t="n">
-        <v>1.3087</v>
+        <v>-1.0049</v>
       </c>
       <c r="V18" t="n">
-        <v>-3.5252</v>
+        <v>-1.7699</v>
       </c>
       <c r="W18" t="n">
-        <v>0.3333</v>
+        <v>-6.457</v>
       </c>
       <c r="X18" t="n">
-        <v>1.7757</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y18" t="n">
-        <v>16.0648</v>
+        <v>10.7428</v>
       </c>
       <c r="Z18" t="n">
-        <v>15.7523</v>
+        <v>26.2909</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.2586</v>
+        <v>1.0705</v>
       </c>
       <c r="AB18" t="n">
-        <v>3.5187</v>
+        <v>1.858</v>
       </c>
       <c r="AC18" t="n">
-        <v>-0.5133</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>134.43</v>
+        <v>119.02</v>
       </c>
       <c r="C19" t="n">
-        <v>134.54</v>
+        <v>120.9</v>
       </c>
       <c r="D19" t="n">
-        <v>127.27</v>
+        <v>109</v>
       </c>
       <c r="E19" t="n">
-        <v>128.4</v>
+        <v>110.54</v>
       </c>
       <c r="F19" t="n">
-        <v>80.78</v>
+        <v>77</v>
       </c>
       <c r="G19" t="n">
-        <v>80.81</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>79.22</v>
+        <v>73.31</v>
       </c>
       <c r="I19" t="n">
-        <v>79.61</v>
+        <v>74.12</v>
       </c>
       <c r="J19" t="n">
-        <v>35.75</v>
+        <v>40.03</v>
       </c>
       <c r="K19" t="n">
-        <v>37.5</v>
+        <v>42.95</v>
       </c>
       <c r="L19" t="n">
-        <v>35.68</v>
+        <v>39.43</v>
       </c>
       <c r="M19" t="n">
-        <v>37.19</v>
+        <v>42.52</v>
       </c>
       <c r="N19" t="n">
-        <v>33.17</v>
+        <v>34.77</v>
       </c>
       <c r="O19" t="n">
-        <v>33.8</v>
+        <v>36.35</v>
       </c>
       <c r="P19" t="n">
-        <v>33.17</v>
+        <v>34.42</v>
       </c>
       <c r="Q19" t="n">
-        <v>33.63</v>
+        <v>36</v>
       </c>
       <c r="R19" t="n">
-        <v>-8.1282</v>
+        <v>-13.3495</v>
       </c>
       <c r="S19" t="n">
-        <v>-19.1995</v>
+        <v>-20.9073</v>
       </c>
       <c r="T19" t="n">
-        <v>-21.836</v>
+        <v>-30.4386</v>
       </c>
       <c r="U19" t="n">
-        <v>-2.0546</v>
+        <v>-5.951</v>
       </c>
       <c r="V19" t="n">
-        <v>-4.7955</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W19" t="n">
-        <v>-4.2228</v>
+        <v>-11.3609</v>
       </c>
       <c r="X19" t="n">
-        <v>8.1419</v>
+        <v>13.6291</v>
       </c>
       <c r="Y19" t="n">
-        <v>21.3377</v>
+        <v>23.6406</v>
       </c>
       <c r="Z19" t="n">
-        <v>25.5571</v>
+        <v>38.7276</v>
       </c>
       <c r="AA19" t="n">
-        <v>2.0637</v>
+        <v>5.9135</v>
       </c>
       <c r="AB19" t="n">
-        <v>4.8644</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC19" t="n">
-        <v>4.2791</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>118.42</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C20" t="n">
-        <v>127.92</v>
+        <v>108.8</v>
       </c>
       <c r="D20" t="n">
-        <v>115.84</v>
+        <v>95.23</v>
       </c>
       <c r="E20" t="n">
-        <v>127.57</v>
+        <v>107.35</v>
       </c>
       <c r="F20" t="n">
-        <v>77.51000000000001</v>
+        <v>70.95</v>
       </c>
       <c r="G20" t="n">
-        <v>79</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>77.28</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>78.81</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>40.15</v>
+        <v>47.19</v>
       </c>
       <c r="K20" t="n">
-        <v>40.9</v>
+        <v>48.37</v>
       </c>
       <c r="L20" t="n">
-        <v>37.36</v>
+        <v>43.11</v>
       </c>
       <c r="M20" t="n">
-        <v>37.42</v>
+        <v>43.64</v>
       </c>
       <c r="N20" t="n">
-        <v>34.54</v>
+        <v>37.57</v>
       </c>
       <c r="O20" t="n">
-        <v>34.63</v>
+        <v>38.02</v>
       </c>
       <c r="P20" t="n">
-        <v>33.89</v>
+        <v>35.94</v>
       </c>
       <c r="Q20" t="n">
-        <v>33.99</v>
+        <v>36.14</v>
       </c>
       <c r="R20" t="n">
-        <v>-0.6464</v>
+        <v>-2.8858</v>
       </c>
       <c r="S20" t="n">
-        <v>-10.4898</v>
+        <v>-16.3941</v>
       </c>
       <c r="T20" t="n">
-        <v>-22.3365</v>
+        <v>-24.6772</v>
       </c>
       <c r="U20" t="n">
-        <v>-1.0049</v>
+        <v>-0.4047</v>
       </c>
       <c r="V20" t="n">
-        <v>-1.7699</v>
+        <v>-7.273</v>
       </c>
       <c r="W20" t="n">
-        <v>-6.457</v>
+        <v>-7.9895</v>
       </c>
       <c r="X20" t="n">
-        <v>0.6183999999999999</v>
+        <v>2.6341</v>
       </c>
       <c r="Y20" t="n">
-        <v>10.7428</v>
+        <v>17.3434</v>
       </c>
       <c r="Z20" t="n">
-        <v>26.2909</v>
+        <v>29.1506</v>
       </c>
       <c r="AA20" t="n">
-        <v>1.0705</v>
+        <v>0.3889</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.858</v>
+        <v>7.4636</v>
       </c>
       <c r="AC20" t="n">
-        <v>6.7861</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>119.02</v>
+        <v>101.19</v>
       </c>
       <c r="C21" t="n">
-        <v>120.9</v>
+        <v>103.93</v>
       </c>
       <c r="D21" t="n">
-        <v>109</v>
+        <v>93.45</v>
       </c>
       <c r="E21" t="n">
-        <v>110.54</v>
+        <v>93.67</v>
       </c>
       <c r="F21" t="n">
-        <v>77</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>77.79000000000001</v>
+        <v>73.13</v>
       </c>
       <c r="H21" t="n">
-        <v>73.31</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>74.12</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>40.03</v>
+        <v>46.22</v>
       </c>
       <c r="K21" t="n">
-        <v>42.95</v>
+        <v>49.36</v>
       </c>
       <c r="L21" t="n">
-        <v>39.43</v>
+        <v>45.08</v>
       </c>
       <c r="M21" t="n">
-        <v>42.52</v>
+        <v>49.23</v>
       </c>
       <c r="N21" t="n">
-        <v>34.77</v>
+        <v>36.57</v>
       </c>
       <c r="O21" t="n">
-        <v>36.35</v>
+        <v>39.29</v>
       </c>
       <c r="P21" t="n">
-        <v>34.42</v>
+        <v>36.51</v>
       </c>
       <c r="Q21" t="n">
-        <v>36</v>
+        <v>38.9</v>
       </c>
       <c r="R21" t="n">
-        <v>-13.3495</v>
+        <v>-12.7434</v>
       </c>
       <c r="S21" t="n">
-        <v>-20.9073</v>
+        <v>-26.5736</v>
       </c>
       <c r="T21" t="n">
-        <v>-30.4386</v>
+        <v>-32.978</v>
       </c>
       <c r="U21" t="n">
-        <v>-5.951</v>
+        <v>-7.5996</v>
       </c>
       <c r="V21" t="n">
-        <v>-8.809100000000001</v>
+        <v>-13.4501</v>
       </c>
       <c r="W21" t="n">
-        <v>-11.3609</v>
+        <v>-16.0802</v>
       </c>
       <c r="X21" t="n">
-        <v>13.6291</v>
+        <v>12.8093</v>
       </c>
       <c r="Y21" t="n">
-        <v>23.6406</v>
+        <v>31.5607</v>
       </c>
       <c r="Z21" t="n">
-        <v>38.7276</v>
+        <v>43.1521</v>
       </c>
       <c r="AA21" t="n">
-        <v>5.9135</v>
+        <v>7.637</v>
       </c>
       <c r="AB21" t="n">
-        <v>9.256399999999999</v>
+        <v>14.4454</v>
       </c>
       <c r="AC21" t="n">
-        <v>12.2544</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>98.34999999999999</v>
-      </c>
-      <c r="C22" t="n">
-        <v>108.8</v>
-      </c>
-      <c r="D22" t="n">
-        <v>95.23</v>
-      </c>
-      <c r="E22" t="n">
-        <v>107.35</v>
-      </c>
-      <c r="F22" t="n">
-        <v>70.95</v>
-      </c>
-      <c r="G22" t="n">
-        <v>74.23999999999999</v>
-      </c>
-      <c r="H22" t="n">
-        <v>69.98999999999999</v>
-      </c>
-      <c r="I22" t="n">
-        <v>73.81999999999999</v>
-      </c>
-      <c r="J22" t="n">
-        <v>47.19</v>
-      </c>
-      <c r="K22" t="n">
-        <v>48.37</v>
-      </c>
-      <c r="L22" t="n">
-        <v>43.11</v>
-      </c>
-      <c r="M22" t="n">
-        <v>43.64</v>
-      </c>
-      <c r="N22" t="n">
-        <v>37.57</v>
-      </c>
-      <c r="O22" t="n">
-        <v>38.02</v>
-      </c>
-      <c r="P22" t="n">
-        <v>35.94</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>36.14</v>
-      </c>
-      <c r="R22" t="n">
-        <v>-2.8858</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-16.3941</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-24.6772</v>
-      </c>
-      <c r="U22" t="n">
-        <v>-0.4047</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-7.273</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-7.9895</v>
-      </c>
-      <c r="X22" t="n">
-        <v>2.6341</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>17.3434</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>29.1506</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>0.3889</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>7.4636</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>8.3009</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-21 00:23
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2281,6 +2281,97 @@
       <c r="A22" t="inlineStr">
         <is>
           <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>103.95</v>
+      </c>
+      <c r="C22" t="n">
+        <v>104.98</v>
+      </c>
+      <c r="D22" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="E22" t="n">
+        <v>98.65000000000001</v>
+      </c>
+      <c r="F22" t="n">
+        <v>71.01000000000001</v>
+      </c>
+      <c r="G22" t="n">
+        <v>72.44</v>
+      </c>
+      <c r="H22" t="n">
+        <v>70.13</v>
+      </c>
+      <c r="I22" t="n">
+        <v>70.64</v>
+      </c>
+      <c r="J22" t="n">
+        <v>43.86</v>
+      </c>
+      <c r="K22" t="n">
+        <v>47.07</v>
+      </c>
+      <c r="L22" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M22" t="n">
+        <v>46.63</v>
+      </c>
+      <c r="N22" t="n">
+        <v>37.33</v>
+      </c>
+      <c r="O22" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="P22" t="n">
+        <v>36.51</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>37.52</v>
+      </c>
+      <c r="R22" t="n">
+        <v>5.3165</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-10.7563</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-23.1698</v>
+      </c>
+      <c r="U22" t="n">
+        <v>3.5625</v>
+      </c>
+      <c r="V22" t="n">
+        <v>-4.6951</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-11.2674</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-5.2813</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>9.666</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>25.3832</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-3.5476</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>4.2222</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>11.5671</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-22 00:26
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1810 +568,1810 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>131.9835</v>
+        <v>137.67</v>
       </c>
       <c r="C2" t="n">
-        <v>143.9056</v>
+        <v>152.64</v>
       </c>
       <c r="D2" t="n">
-        <v>129.5351</v>
+        <v>137.46</v>
       </c>
       <c r="E2" t="n">
-        <v>141.837</v>
+        <v>151.95</v>
       </c>
       <c r="F2" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>79.3366</v>
+        <v>80.96339999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>74.68559999999999</v>
+        <v>78.61799999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>78.7577</v>
+        <v>80.67400000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>38.2718</v>
+        <v>35.98</v>
       </c>
       <c r="K2" t="n">
-        <v>39.0224</v>
+        <v>36.01</v>
       </c>
       <c r="L2" t="n">
-        <v>34.252</v>
+        <v>32.25</v>
       </c>
       <c r="M2" t="n">
-        <v>34.894</v>
+        <v>32.42</v>
       </c>
       <c r="N2" t="n">
-        <v>36.2155</v>
+        <v>34.1745</v>
       </c>
       <c r="O2" t="n">
-        <v>36.2254</v>
+        <v>34.1745</v>
       </c>
       <c r="P2" t="n">
-        <v>33.8294</v>
+        <v>33.1688</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.1154</v>
+        <v>33.297</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C3" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D3" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E3" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F3" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G3" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I3" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J3" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K3" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L3" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M3" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N3" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O3" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P3" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q3" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
       <c r="R3" t="n">
-        <v>7.13</v>
+        <v>-3.7512</v>
       </c>
       <c r="U3" t="n">
-        <v>2.4332</v>
+        <v>-2.4965</v>
       </c>
       <c r="X3" t="n">
-        <v>-7.09</v>
+        <v>3.8248</v>
       </c>
       <c r="AA3" t="n">
-        <v>-2.3989</v>
+        <v>2.5318</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C4" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D4" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E4" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F4" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G4" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I4" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J4" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K4" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L4" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M4" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N4" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O4" t="n">
         <v>35.06</v>
       </c>
-      <c r="L4" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M4" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N4" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O4" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P4" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R4" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="U4" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="X4" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="AA4" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C5" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D5" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E5" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F5" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G5" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H5" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I5" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K5" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L5" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M5" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N5" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O5" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P5" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q5" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="S5" t="n">
-        <v>3.1677</v>
+        <v>-0.3291</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.2256</v>
+        <v>-1.3313</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="Y5" t="n">
-        <v>-3.6224</v>
+        <v>0.0308</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.1894</v>
+        <v>1.3605</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C6" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D6" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E6" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F6" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I6" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K6" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L6" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M6" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N6" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O6" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P6" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q6" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R6" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.3291</v>
+        <v>-2.7077</v>
       </c>
       <c r="U6" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.3313</v>
+        <v>-2.0595</v>
       </c>
       <c r="X6" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.0308</v>
+        <v>2.2876</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.3605</v>
+        <v>2.0211</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C7" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D7" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E7" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F7" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G7" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I7" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K7" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L7" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M7" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N7" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O7" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P7" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R7" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S7" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="T7" t="n">
-        <v>0.3194</v>
+        <v>-3.2577</v>
       </c>
       <c r="U7" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V7" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="W7" t="n">
-        <v>-2.181</v>
+        <v>-3.9839</v>
       </c>
       <c r="X7" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y7" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="Z7" t="n">
-        <v>-1.3297</v>
+        <v>2.591</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB7" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.0947</v>
+        <v>4.0935</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C8" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D8" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E8" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F8" t="n">
         <v>78.13</v>
       </c>
       <c r="G8" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I8" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J8" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K8" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L8" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M8" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N8" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O8" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P8" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q8" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R8" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S8" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="T8" t="n">
-        <v>-3.2577</v>
+        <v>1.1009</v>
       </c>
       <c r="U8" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V8" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="W8" t="n">
-        <v>-3.9839</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X8" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y8" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.591</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
       <c r="AC8" t="n">
-        <v>4.0935</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C9" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D9" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E9" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F9" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G9" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H9" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I9" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J9" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K9" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L9" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M9" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N9" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O9" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P9" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q9" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R9" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S9" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T9" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U9" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V9" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z9" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C10" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D10" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E10" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F10" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G10" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H10" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I10" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K10" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L10" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M10" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N10" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O10" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P10" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q10" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R10" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S10" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T10" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U10" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V10" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X10" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y10" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z10" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC10" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C11" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D11" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E11" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F11" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G11" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H11" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J11" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K11" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L11" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M11" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N11" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O11" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P11" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q11" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R11" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S11" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T11" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U11" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V11" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W11" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X11" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y11" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z11" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA11" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB11" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC11" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C12" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D12" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E12" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F12" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I12" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J12" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K12" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L12" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M12" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N12" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O12" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P12" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q12" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S12" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T12" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U12" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V12" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W12" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y12" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z12" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB12" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC12" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C13" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D13" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E13" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F13" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H13" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J13" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K13" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L13" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M13" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N13" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O13" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P13" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q13" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R13" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S13" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T13" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U13" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V13" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W13" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X13" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y13" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z13" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB13" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC13" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C14" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D14" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E14" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F14" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G14" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I14" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J14" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K14" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L14" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M14" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N14" t="n">
         <v>32.58</v>
       </c>
       <c r="O14" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P14" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q14" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R14" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T14" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V14" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W14" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X14" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y14" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z14" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB14" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC14" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C15" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D15" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E15" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F15" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G15" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H15" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I15" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J15" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K15" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L15" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M15" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N15" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O15" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P15" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q15" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R15" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S15" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T15" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U15" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W15" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X15" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y15" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z15" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA15" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB15" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC15" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C16" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D16" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E16" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F16" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G16" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H16" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I16" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J16" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K16" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L16" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M16" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N16" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O16" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P16" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q16" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R16" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S16" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T16" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U16" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V16" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W16" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X16" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y16" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z16" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA16" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB16" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC16" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C17" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D17" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E17" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F17" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H17" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I17" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J17" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K17" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L17" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M17" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N17" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O17" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P17" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q17" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R17" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S17" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T17" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U17" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V17" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W17" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X17" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y17" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z17" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA17" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC17" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C18" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D18" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E18" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F18" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G18" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I18" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J18" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K18" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L18" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M18" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N18" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O18" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P18" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q18" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S18" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T18" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U18" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V18" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W18" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X18" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y18" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z18" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA18" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC18" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C19" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D19" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E19" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F19" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G19" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K19" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L19" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M19" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N19" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O19" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P19" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q19" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R19" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S19" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T19" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U19" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V19" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W19" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X19" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y19" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z19" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA19" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB19" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC19" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>98.34999999999999</v>
+        <v>101.19</v>
       </c>
       <c r="C20" t="n">
-        <v>108.8</v>
+        <v>103.93</v>
       </c>
       <c r="D20" t="n">
-        <v>95.23</v>
+        <v>93.45</v>
       </c>
       <c r="E20" t="n">
-        <v>107.35</v>
+        <v>93.67</v>
       </c>
       <c r="F20" t="n">
-        <v>70.95</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>74.23999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="H20" t="n">
-        <v>69.98999999999999</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>73.81999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>47.19</v>
+        <v>46.22</v>
       </c>
       <c r="K20" t="n">
-        <v>48.37</v>
+        <v>49.36</v>
       </c>
       <c r="L20" t="n">
-        <v>43.11</v>
+        <v>45.08</v>
       </c>
       <c r="M20" t="n">
-        <v>43.64</v>
+        <v>49.23</v>
       </c>
       <c r="N20" t="n">
-        <v>37.57</v>
+        <v>36.57</v>
       </c>
       <c r="O20" t="n">
-        <v>38.02</v>
+        <v>39.29</v>
       </c>
       <c r="P20" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q20" t="n">
-        <v>36.14</v>
+        <v>38.9</v>
       </c>
       <c r="R20" t="n">
-        <v>-2.8858</v>
+        <v>-12.7434</v>
       </c>
       <c r="S20" t="n">
-        <v>-16.3941</v>
+        <v>-26.5736</v>
       </c>
       <c r="T20" t="n">
-        <v>-24.6772</v>
+        <v>-32.978</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.4047</v>
+        <v>-7.5996</v>
       </c>
       <c r="V20" t="n">
-        <v>-7.273</v>
+        <v>-13.4501</v>
       </c>
       <c r="W20" t="n">
-        <v>-7.9895</v>
+        <v>-16.0802</v>
       </c>
       <c r="X20" t="n">
-        <v>2.6341</v>
+        <v>12.8093</v>
       </c>
       <c r="Y20" t="n">
-        <v>17.3434</v>
+        <v>31.5607</v>
       </c>
       <c r="Z20" t="n">
-        <v>29.1506</v>
+        <v>43.1521</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.3889</v>
+        <v>7.637</v>
       </c>
       <c r="AB20" t="n">
-        <v>7.4636</v>
+        <v>14.4454</v>
       </c>
       <c r="AC20" t="n">
-        <v>8.3009</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>101.19</v>
+        <v>103.95</v>
       </c>
       <c r="C21" t="n">
-        <v>103.93</v>
+        <v>104.98</v>
       </c>
       <c r="D21" t="n">
-        <v>93.45</v>
+        <v>97.8</v>
       </c>
       <c r="E21" t="n">
-        <v>93.67</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>73.01000000000001</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>73.13</v>
+        <v>72.44</v>
       </c>
       <c r="H21" t="n">
-        <v>67.43000000000001</v>
+        <v>70.13</v>
       </c>
       <c r="I21" t="n">
-        <v>68.20999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J21" t="n">
-        <v>46.22</v>
+        <v>43.86</v>
       </c>
       <c r="K21" t="n">
-        <v>49.36</v>
+        <v>47.07</v>
       </c>
       <c r="L21" t="n">
-        <v>45.08</v>
+        <v>43.32</v>
       </c>
       <c r="M21" t="n">
-        <v>49.23</v>
+        <v>46.63</v>
       </c>
       <c r="N21" t="n">
-        <v>36.57</v>
+        <v>37.33</v>
       </c>
       <c r="O21" t="n">
-        <v>39.29</v>
+        <v>37.82</v>
       </c>
       <c r="P21" t="n">
         <v>36.51</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.9</v>
+        <v>37.52</v>
       </c>
       <c r="R21" t="n">
-        <v>-12.7434</v>
+        <v>5.3165</v>
       </c>
       <c r="S21" t="n">
-        <v>-26.5736</v>
+        <v>-10.7563</v>
       </c>
       <c r="T21" t="n">
-        <v>-32.978</v>
+        <v>-23.1698</v>
       </c>
       <c r="U21" t="n">
-        <v>-7.5996</v>
+        <v>3.5625</v>
       </c>
       <c r="V21" t="n">
-        <v>-13.4501</v>
+        <v>-4.6951</v>
       </c>
       <c r="W21" t="n">
-        <v>-16.0802</v>
+        <v>-11.2674</v>
       </c>
       <c r="X21" t="n">
-        <v>12.8093</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y21" t="n">
-        <v>31.5607</v>
+        <v>9.666</v>
       </c>
       <c r="Z21" t="n">
-        <v>43.1521</v>
+        <v>25.3832</v>
       </c>
       <c r="AA21" t="n">
-        <v>7.637</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB21" t="n">
-        <v>14.4454</v>
+        <v>4.2222</v>
       </c>
       <c r="AC21" t="n">
-        <v>18.0577</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>103.95</v>
+        <v>94.52</v>
       </c>
       <c r="C22" t="n">
-        <v>104.98</v>
+        <v>102.62</v>
       </c>
       <c r="D22" t="n">
-        <v>97.8</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>98.65000000000001</v>
+        <v>97.55</v>
       </c>
       <c r="F22" t="n">
-        <v>71.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>72.44</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>70.13</v>
+        <v>68.28</v>
       </c>
       <c r="I22" t="n">
-        <v>70.64</v>
+        <v>70.41</v>
       </c>
       <c r="J22" t="n">
-        <v>43.86</v>
+        <v>48.64</v>
       </c>
       <c r="K22" t="n">
-        <v>47.07</v>
+        <v>50.12</v>
       </c>
       <c r="L22" t="n">
-        <v>43.32</v>
+        <v>44.76</v>
       </c>
       <c r="M22" t="n">
-        <v>46.63</v>
+        <v>47.13</v>
       </c>
       <c r="N22" t="n">
-        <v>37.33</v>
+        <v>38.03</v>
       </c>
       <c r="O22" t="n">
-        <v>37.82</v>
+        <v>38.79</v>
       </c>
       <c r="P22" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q22" t="n">
-        <v>37.52</v>
+        <v>37.68</v>
       </c>
       <c r="R22" t="n">
-        <v>5.3165</v>
+        <v>-1.1151</v>
       </c>
       <c r="S22" t="n">
-        <v>-10.7563</v>
+        <v>-9.129</v>
       </c>
       <c r="T22" t="n">
-        <v>-23.1698</v>
+        <v>-23.5322</v>
       </c>
       <c r="U22" t="n">
-        <v>3.5625</v>
+        <v>-0.3256</v>
       </c>
       <c r="V22" t="n">
-        <v>-4.6951</v>
+        <v>-4.6193</v>
       </c>
       <c r="W22" t="n">
-        <v>-11.2674</v>
+        <v>-10.6585</v>
       </c>
       <c r="X22" t="n">
-        <v>-5.2813</v>
+        <v>1.0723</v>
       </c>
       <c r="Y22" t="n">
-        <v>9.666</v>
+        <v>7.9973</v>
       </c>
       <c r="Z22" t="n">
-        <v>25.3832</v>
+        <v>25.9487</v>
       </c>
       <c r="AA22" t="n">
-        <v>-3.5476</v>
+        <v>0.4264</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.2222</v>
+        <v>4.2612</v>
       </c>
       <c r="AC22" t="n">
-        <v>11.5671</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-23 00:25
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1810 +568,1810 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>137.67</v>
+        <v>149.89</v>
       </c>
       <c r="C2" t="n">
-        <v>152.64</v>
+        <v>151</v>
       </c>
       <c r="D2" t="n">
-        <v>137.46</v>
+        <v>139.58</v>
       </c>
       <c r="E2" t="n">
-        <v>151.95</v>
+        <v>146.25</v>
       </c>
       <c r="F2" t="n">
-        <v>78.61799999999999</v>
+        <v>80.53</v>
       </c>
       <c r="G2" t="n">
-        <v>80.96339999999999</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>78.61799999999999</v>
+        <v>77.69</v>
       </c>
       <c r="I2" t="n">
-        <v>80.67400000000001</v>
+        <v>78.66</v>
       </c>
       <c r="J2" t="n">
-        <v>35.98</v>
+        <v>32.87</v>
       </c>
       <c r="K2" t="n">
-        <v>36.01</v>
+        <v>35.06</v>
       </c>
       <c r="L2" t="n">
-        <v>32.25</v>
+        <v>32.63</v>
       </c>
       <c r="M2" t="n">
-        <v>32.42</v>
+        <v>33.66</v>
       </c>
       <c r="N2" t="n">
-        <v>34.1745</v>
+        <v>33.37</v>
       </c>
       <c r="O2" t="n">
-        <v>34.1745</v>
+        <v>34.54</v>
       </c>
       <c r="P2" t="n">
-        <v>33.1688</v>
+        <v>33.35</v>
       </c>
       <c r="Q2" t="n">
-        <v>33.297</v>
+        <v>34.14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C3" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D3" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E3" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F3" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G3" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I3" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J3" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K3" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L3" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M3" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N3" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O3" t="n">
         <v>35.06</v>
       </c>
-      <c r="L3" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M3" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N3" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O3" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P3" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q3" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
       <c r="R3" t="n">
-        <v>-3.7512</v>
+        <v>0.0547</v>
       </c>
       <c r="U3" t="n">
-        <v>-2.4965</v>
+        <v>-0.1017</v>
       </c>
       <c r="X3" t="n">
-        <v>3.8248</v>
+        <v>-0.0891</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.5318</v>
+        <v>0.1172</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C4" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D4" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E4" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F4" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G4" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H4" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I4" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K4" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L4" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M4" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N4" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O4" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P4" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R4" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C5" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D5" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E5" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F5" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I5" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K5" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L5" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M5" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N5" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O5" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P5" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q5" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R5" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.3291</v>
+        <v>-2.7077</v>
       </c>
       <c r="U5" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="V5" t="n">
-        <v>-1.3313</v>
+        <v>-2.0595</v>
       </c>
       <c r="X5" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.0308</v>
+        <v>2.2876</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.3605</v>
+        <v>2.0211</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C6" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D6" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E6" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F6" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G6" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I6" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K6" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L6" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M6" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N6" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O6" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P6" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q6" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R6" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S6" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="U6" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V6" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="X6" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="AA6" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB6" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C7" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D7" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E7" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F7" t="n">
         <v>78.13</v>
       </c>
       <c r="G7" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I7" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J7" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K7" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L7" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M7" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N7" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O7" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P7" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R7" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S7" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="T7" t="n">
-        <v>-3.2577</v>
+        <v>1.1009</v>
       </c>
       <c r="U7" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V7" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.9839</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="X7" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y7" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="Z7" t="n">
-        <v>2.591</v>
+        <v>-1.7231</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
       <c r="AC7" t="n">
-        <v>4.0935</v>
+        <v>0.7909</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C8" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D8" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E8" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F8" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G8" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H8" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I8" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J8" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K8" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L8" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M8" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N8" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O8" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P8" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q8" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R8" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S8" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T8" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U8" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V8" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W8" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z8" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C9" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D9" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E9" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F9" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G9" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H9" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I9" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K9" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L9" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M9" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N9" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O9" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P9" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q9" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R9" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S9" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T9" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U9" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V9" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X9" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y9" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z9" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB9" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC9" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C10" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D10" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E10" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F10" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G10" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H10" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J10" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K10" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L10" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M10" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N10" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O10" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P10" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q10" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R10" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S10" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T10" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U10" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V10" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W10" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X10" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y10" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z10" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA10" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB10" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC10" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C11" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D11" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E11" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F11" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I11" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J11" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K11" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L11" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M11" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N11" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O11" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P11" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q11" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R11" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S11" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T11" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U11" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V11" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W11" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X11" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y11" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z11" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA11" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC11" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C12" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D12" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E12" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F12" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H12" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J12" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K12" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L12" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M12" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N12" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O12" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P12" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q12" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S12" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T12" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U12" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V12" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W12" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X12" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y12" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z12" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA12" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB12" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC12" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C13" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D13" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E13" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F13" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G13" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I13" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J13" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K13" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L13" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M13" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N13" t="n">
         <v>32.58</v>
       </c>
       <c r="O13" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P13" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q13" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R13" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S13" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T13" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V13" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W13" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X13" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y13" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z13" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB13" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC13" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C14" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D14" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E14" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F14" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G14" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H14" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I14" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J14" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K14" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L14" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M14" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N14" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O14" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P14" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q14" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R14" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S14" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T14" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U14" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W14" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X14" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y14" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z14" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA14" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC14" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C15" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D15" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E15" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F15" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G15" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H15" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I15" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J15" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K15" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L15" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M15" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N15" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O15" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P15" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q15" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R15" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S15" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T15" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U15" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W15" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X15" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y15" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z15" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB15" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC15" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C16" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D16" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E16" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F16" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H16" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I16" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J16" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K16" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L16" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M16" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N16" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O16" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P16" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q16" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R16" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S16" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T16" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U16" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V16" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W16" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X16" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y16" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z16" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA16" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C17" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D17" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E17" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F17" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G17" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I17" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J17" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K17" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L17" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M17" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N17" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O17" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P17" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q17" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S17" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T17" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V17" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W17" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X17" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y17" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z17" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC17" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C18" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D18" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E18" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F18" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G18" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K18" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L18" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M18" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N18" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O18" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P18" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q18" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R18" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S18" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T18" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U18" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V18" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W18" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X18" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y18" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z18" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA18" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB18" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC18" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>98.34999999999999</v>
+        <v>101.19</v>
       </c>
       <c r="C19" t="n">
-        <v>108.8</v>
+        <v>103.93</v>
       </c>
       <c r="D19" t="n">
-        <v>95.23</v>
+        <v>93.45</v>
       </c>
       <c r="E19" t="n">
-        <v>107.35</v>
+        <v>93.67</v>
       </c>
       <c r="F19" t="n">
-        <v>70.95</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>74.23999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="H19" t="n">
-        <v>69.98999999999999</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>73.81999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>47.19</v>
+        <v>46.22</v>
       </c>
       <c r="K19" t="n">
-        <v>48.37</v>
+        <v>49.36</v>
       </c>
       <c r="L19" t="n">
-        <v>43.11</v>
+        <v>45.08</v>
       </c>
       <c r="M19" t="n">
-        <v>43.64</v>
+        <v>49.23</v>
       </c>
       <c r="N19" t="n">
-        <v>37.57</v>
+        <v>36.57</v>
       </c>
       <c r="O19" t="n">
-        <v>38.02</v>
+        <v>39.29</v>
       </c>
       <c r="P19" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.14</v>
+        <v>38.9</v>
       </c>
       <c r="R19" t="n">
-        <v>-2.8858</v>
+        <v>-12.7434</v>
       </c>
       <c r="S19" t="n">
-        <v>-16.3941</v>
+        <v>-26.5736</v>
       </c>
       <c r="T19" t="n">
-        <v>-24.6772</v>
+        <v>-32.978</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.4047</v>
+        <v>-7.5996</v>
       </c>
       <c r="V19" t="n">
-        <v>-7.273</v>
+        <v>-13.4501</v>
       </c>
       <c r="W19" t="n">
-        <v>-7.9895</v>
+        <v>-16.0802</v>
       </c>
       <c r="X19" t="n">
-        <v>2.6341</v>
+        <v>12.8093</v>
       </c>
       <c r="Y19" t="n">
-        <v>17.3434</v>
+        <v>31.5607</v>
       </c>
       <c r="Z19" t="n">
-        <v>29.1506</v>
+        <v>43.1521</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.3889</v>
+        <v>7.637</v>
       </c>
       <c r="AB19" t="n">
-        <v>7.4636</v>
+        <v>14.4454</v>
       </c>
       <c r="AC19" t="n">
-        <v>8.3009</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>101.19</v>
+        <v>103.95</v>
       </c>
       <c r="C20" t="n">
-        <v>103.93</v>
+        <v>104.98</v>
       </c>
       <c r="D20" t="n">
-        <v>93.45</v>
+        <v>97.8</v>
       </c>
       <c r="E20" t="n">
-        <v>93.67</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>73.01000000000001</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>73.13</v>
+        <v>72.44</v>
       </c>
       <c r="H20" t="n">
-        <v>67.43000000000001</v>
+        <v>70.13</v>
       </c>
       <c r="I20" t="n">
-        <v>68.20999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J20" t="n">
-        <v>46.22</v>
+        <v>43.86</v>
       </c>
       <c r="K20" t="n">
-        <v>49.36</v>
+        <v>47.07</v>
       </c>
       <c r="L20" t="n">
-        <v>45.08</v>
+        <v>43.32</v>
       </c>
       <c r="M20" t="n">
-        <v>49.23</v>
+        <v>46.63</v>
       </c>
       <c r="N20" t="n">
-        <v>36.57</v>
+        <v>37.33</v>
       </c>
       <c r="O20" t="n">
-        <v>39.29</v>
+        <v>37.82</v>
       </c>
       <c r="P20" t="n">
         <v>36.51</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.9</v>
+        <v>37.52</v>
       </c>
       <c r="R20" t="n">
-        <v>-12.7434</v>
+        <v>5.3165</v>
       </c>
       <c r="S20" t="n">
-        <v>-26.5736</v>
+        <v>-10.7563</v>
       </c>
       <c r="T20" t="n">
-        <v>-32.978</v>
+        <v>-23.1698</v>
       </c>
       <c r="U20" t="n">
-        <v>-7.5996</v>
+        <v>3.5625</v>
       </c>
       <c r="V20" t="n">
-        <v>-13.4501</v>
+        <v>-4.6951</v>
       </c>
       <c r="W20" t="n">
-        <v>-16.0802</v>
+        <v>-11.2674</v>
       </c>
       <c r="X20" t="n">
-        <v>12.8093</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y20" t="n">
-        <v>31.5607</v>
+        <v>9.666</v>
       </c>
       <c r="Z20" t="n">
-        <v>43.1521</v>
+        <v>25.3832</v>
       </c>
       <c r="AA20" t="n">
-        <v>7.637</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB20" t="n">
-        <v>14.4454</v>
+        <v>4.2222</v>
       </c>
       <c r="AC20" t="n">
-        <v>18.0577</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>103.95</v>
+        <v>94.52</v>
       </c>
       <c r="C21" t="n">
-        <v>104.98</v>
+        <v>102.62</v>
       </c>
       <c r="D21" t="n">
-        <v>97.8</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>98.65000000000001</v>
+        <v>97.55</v>
       </c>
       <c r="F21" t="n">
-        <v>71.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>72.44</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>70.13</v>
+        <v>68.28</v>
       </c>
       <c r="I21" t="n">
-        <v>70.64</v>
+        <v>70.41</v>
       </c>
       <c r="J21" t="n">
-        <v>43.86</v>
+        <v>48.64</v>
       </c>
       <c r="K21" t="n">
-        <v>47.07</v>
+        <v>50.12</v>
       </c>
       <c r="L21" t="n">
-        <v>43.32</v>
+        <v>44.76</v>
       </c>
       <c r="M21" t="n">
-        <v>46.63</v>
+        <v>47.13</v>
       </c>
       <c r="N21" t="n">
-        <v>37.33</v>
+        <v>38.03</v>
       </c>
       <c r="O21" t="n">
-        <v>37.82</v>
+        <v>38.79</v>
       </c>
       <c r="P21" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.52</v>
+        <v>37.68</v>
       </c>
       <c r="R21" t="n">
-        <v>5.3165</v>
+        <v>-1.1151</v>
       </c>
       <c r="S21" t="n">
-        <v>-10.7563</v>
+        <v>-9.129</v>
       </c>
       <c r="T21" t="n">
-        <v>-23.1698</v>
+        <v>-23.5322</v>
       </c>
       <c r="U21" t="n">
-        <v>3.5625</v>
+        <v>-0.3256</v>
       </c>
       <c r="V21" t="n">
-        <v>-4.6951</v>
+        <v>-4.6193</v>
       </c>
       <c r="W21" t="n">
-        <v>-11.2674</v>
+        <v>-10.6585</v>
       </c>
       <c r="X21" t="n">
-        <v>-5.2813</v>
+        <v>1.0723</v>
       </c>
       <c r="Y21" t="n">
-        <v>9.666</v>
+        <v>7.9973</v>
       </c>
       <c r="Z21" t="n">
-        <v>25.3832</v>
+        <v>25.9487</v>
       </c>
       <c r="AA21" t="n">
-        <v>-3.5476</v>
+        <v>0.4264</v>
       </c>
       <c r="AB21" t="n">
-        <v>4.2222</v>
+        <v>4.2612</v>
       </c>
       <c r="AC21" t="n">
-        <v>11.5671</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>94.52</v>
+        <v>102.86</v>
       </c>
       <c r="C22" t="n">
-        <v>102.62</v>
+        <v>106.13</v>
       </c>
       <c r="D22" t="n">
-        <v>91.34999999999999</v>
+        <v>99.31</v>
       </c>
       <c r="E22" t="n">
-        <v>97.55</v>
+        <v>103.24</v>
       </c>
       <c r="F22" t="n">
-        <v>69.70999999999999</v>
+        <v>71.72</v>
       </c>
       <c r="G22" t="n">
-        <v>71.93000000000001</v>
+        <v>73.43000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>68.28</v>
+        <v>71.02</v>
       </c>
       <c r="I22" t="n">
-        <v>70.41</v>
+        <v>72.61</v>
       </c>
       <c r="J22" t="n">
-        <v>48.64</v>
+        <v>44.51</v>
       </c>
       <c r="K22" t="n">
-        <v>50.12</v>
+        <v>47.1</v>
       </c>
       <c r="L22" t="n">
-        <v>44.76</v>
+        <v>43.57</v>
       </c>
       <c r="M22" t="n">
-        <v>47.13</v>
+        <v>44.29</v>
       </c>
       <c r="N22" t="n">
-        <v>38.03</v>
+        <v>36.94</v>
       </c>
       <c r="O22" t="n">
-        <v>38.79</v>
+        <v>38.11</v>
       </c>
       <c r="P22" t="n">
-        <v>36.85</v>
+        <v>36.05</v>
       </c>
       <c r="Q22" t="n">
-        <v>37.68</v>
+        <v>36.48</v>
       </c>
       <c r="R22" t="n">
-        <v>-1.1151</v>
+        <v>5.8329</v>
       </c>
       <c r="S22" t="n">
-        <v>-9.129</v>
+        <v>10.2167</v>
       </c>
       <c r="T22" t="n">
-        <v>-23.5322</v>
+        <v>-6.6039</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.3256</v>
+        <v>3.1246</v>
       </c>
       <c r="V22" t="n">
-        <v>-4.6193</v>
+        <v>6.4507</v>
       </c>
       <c r="W22" t="n">
-        <v>-10.6585</v>
+        <v>-2.0372</v>
       </c>
       <c r="X22" t="n">
-        <v>1.0723</v>
+        <v>-6.0259</v>
       </c>
       <c r="Y22" t="n">
-        <v>7.9973</v>
+        <v>-10.0345</v>
       </c>
       <c r="Z22" t="n">
-        <v>25.9487</v>
+        <v>4.1627</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.4264</v>
+        <v>-3.1847</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.2612</v>
+        <v>-6.2211</v>
       </c>
       <c r="AC22" t="n">
-        <v>10.8561</v>
+        <v>1.3333</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-24 00:17
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1810 +568,1810 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149.89</v>
+        <v>138.47</v>
       </c>
       <c r="C2" t="n">
-        <v>151</v>
+        <v>147.2</v>
       </c>
       <c r="D2" t="n">
-        <v>139.58</v>
+        <v>136.9</v>
       </c>
       <c r="E2" t="n">
-        <v>146.25</v>
+        <v>146.33</v>
       </c>
       <c r="F2" t="n">
-        <v>80.53</v>
+        <v>76.75</v>
       </c>
       <c r="G2" t="n">
-        <v>80.56999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>77.69</v>
+        <v>76.55</v>
       </c>
       <c r="I2" t="n">
-        <v>78.66</v>
+        <v>78.58</v>
       </c>
       <c r="J2" t="n">
-        <v>32.87</v>
+        <v>35.45</v>
       </c>
       <c r="K2" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="L2" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="M2" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="N2" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O2" t="n">
         <v>35.06</v>
       </c>
-      <c r="L2" t="n">
-        <v>32.63</v>
-      </c>
-      <c r="M2" t="n">
-        <v>33.66</v>
-      </c>
-      <c r="N2" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="O2" t="n">
-        <v>34.54</v>
-      </c>
       <c r="P2" t="n">
-        <v>33.35</v>
+        <v>33.95</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.14</v>
+        <v>34.18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>138.47</v>
+        <v>149.24</v>
       </c>
       <c r="C3" t="n">
-        <v>147.2</v>
+        <v>153.9</v>
       </c>
       <c r="D3" t="n">
-        <v>136.9</v>
+        <v>147.39</v>
       </c>
       <c r="E3" t="n">
-        <v>146.33</v>
+        <v>151.45</v>
       </c>
       <c r="F3" t="n">
-        <v>76.75</v>
+        <v>79.09</v>
       </c>
       <c r="G3" t="n">
-        <v>79.09999999999999</v>
+        <v>80.06</v>
       </c>
       <c r="H3" t="n">
-        <v>76.55</v>
+        <v>78.06</v>
       </c>
       <c r="I3" t="n">
-        <v>78.58</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>35.45</v>
+        <v>32.97</v>
       </c>
       <c r="K3" t="n">
-        <v>35.85</v>
+        <v>33.39</v>
       </c>
       <c r="L3" t="n">
-        <v>33.43</v>
+        <v>31.9</v>
       </c>
       <c r="M3" t="n">
-        <v>33.63</v>
+        <v>32.43</v>
       </c>
       <c r="N3" t="n">
-        <v>34.98</v>
+        <v>33.97</v>
       </c>
       <c r="O3" t="n">
-        <v>35.06</v>
+        <v>34.41</v>
       </c>
       <c r="P3" t="n">
-        <v>33.95</v>
+        <v>33.54</v>
       </c>
       <c r="Q3" t="n">
-        <v>34.18</v>
+        <v>33.75</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0547</v>
+        <v>3.4989</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.1017</v>
+        <v>1.298</v>
       </c>
       <c r="X3" t="n">
-        <v>-0.0891</v>
+        <v>-3.5682</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.1172</v>
+        <v>-1.258</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>149.24</v>
+        <v>148.14</v>
       </c>
       <c r="C4" t="n">
-        <v>153.9</v>
+        <v>149.99</v>
       </c>
       <c r="D4" t="n">
-        <v>147.39</v>
+        <v>135.21</v>
       </c>
       <c r="E4" t="n">
-        <v>151.45</v>
+        <v>142.29</v>
       </c>
       <c r="F4" t="n">
-        <v>79.09</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>80.06</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>78.06</v>
+        <v>75.47</v>
       </c>
       <c r="I4" t="n">
-        <v>79.59999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>32.97</v>
+        <v>33.17</v>
       </c>
       <c r="K4" t="n">
-        <v>33.39</v>
+        <v>35.95</v>
       </c>
       <c r="L4" t="n">
-        <v>31.9</v>
+        <v>32.77</v>
       </c>
       <c r="M4" t="n">
-        <v>32.43</v>
+        <v>34.43</v>
       </c>
       <c r="N4" t="n">
-        <v>33.97</v>
+        <v>34.31</v>
       </c>
       <c r="O4" t="n">
-        <v>34.41</v>
+        <v>35.53</v>
       </c>
       <c r="P4" t="n">
-        <v>33.54</v>
+        <v>34.17</v>
       </c>
       <c r="Q4" t="n">
-        <v>33.75</v>
+        <v>34.83</v>
       </c>
       <c r="R4" t="n">
-        <v>3.4989</v>
+        <v>-6.0482</v>
       </c>
       <c r="U4" t="n">
-        <v>1.298</v>
+        <v>-3.2161</v>
       </c>
       <c r="X4" t="n">
-        <v>-3.5682</v>
+        <v>6.1671</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.258</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C5" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D5" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E5" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F5" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G5" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I5" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K5" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L5" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M5" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N5" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O5" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P5" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q5" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
       <c r="R5" t="n">
-        <v>-6.0482</v>
+        <v>3.3101</v>
       </c>
       <c r="S5" t="n">
-        <v>-2.7077</v>
+        <v>0.4579</v>
       </c>
       <c r="U5" t="n">
-        <v>-3.2161</v>
+        <v>0.5452</v>
       </c>
       <c r="V5" t="n">
-        <v>-2.0595</v>
+        <v>-1.4253</v>
       </c>
       <c r="X5" t="n">
-        <v>6.1671</v>
+        <v>-3.3982</v>
       </c>
       <c r="Y5" t="n">
-        <v>2.2876</v>
+        <v>-1.1002</v>
       </c>
       <c r="AA5" t="n">
-        <v>3.2</v>
+        <v>-0.4881</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.0211</v>
+        <v>1.4043</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C6" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D6" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E6" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F6" t="n">
         <v>78.13</v>
       </c>
       <c r="G6" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I6" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J6" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K6" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L6" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M6" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N6" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O6" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P6" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q6" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R6" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="S6" t="n">
-        <v>0.4579</v>
+        <v>-2.3704</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.4253</v>
+        <v>-1.9724</v>
       </c>
       <c r="X6" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="Y6" t="n">
-        <v>-1.1002</v>
+        <v>2.0043</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.4043</v>
+        <v>1.9556</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C7" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D7" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E7" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F7" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G7" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H7" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I7" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J7" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K7" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L7" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M7" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N7" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O7" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P7" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R7" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="S7" t="n">
-        <v>-2.3704</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="T7" t="n">
-        <v>1.1009</v>
+        <v>5.0297</v>
       </c>
       <c r="U7" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="V7" t="n">
-        <v>-1.9724</v>
+        <v>2.1937</v>
       </c>
       <c r="W7" t="n">
-        <v>-0.8008999999999999</v>
+        <v>0.1909</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y7" t="n">
-        <v>2.0043</v>
+        <v>-7.7549</v>
       </c>
       <c r="Z7" t="n">
-        <v>-1.7231</v>
+        <v>-5.5605</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.9556</v>
+        <v>-2.0672</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.7909</v>
+        <v>-0.2048</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C8" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D8" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E8" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F8" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G8" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H8" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I8" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K8" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L8" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M8" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N8" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O8" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P8" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q8" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R8" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S8" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="T8" t="n">
-        <v>5.0297</v>
+        <v>8.0951</v>
       </c>
       <c r="U8" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V8" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1909</v>
+        <v>1.7714</v>
       </c>
       <c r="X8" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y8" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="Z8" t="n">
-        <v>-5.5605</v>
+        <v>-8.3873</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
       <c r="AC8" t="n">
-        <v>-0.2048</v>
+        <v>-1.8667</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C9" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D9" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E9" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F9" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G9" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H9" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J9" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K9" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L9" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M9" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N9" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O9" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P9" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q9" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R9" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S9" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="T9" t="n">
-        <v>8.0951</v>
+        <v>15.4473</v>
       </c>
       <c r="U9" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V9" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="W9" t="n">
-        <v>1.7714</v>
+        <v>7.892</v>
       </c>
       <c r="X9" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y9" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z9" t="n">
-        <v>-8.3873</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB9" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC9" t="n">
-        <v>-1.8667</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C10" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D10" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E10" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F10" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I10" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J10" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K10" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L10" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M10" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N10" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O10" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P10" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q10" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S10" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T10" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U10" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V10" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W10" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X10" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y10" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z10" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA10" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC10" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C11" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D11" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E11" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F11" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H11" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J11" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K11" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L11" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M11" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N11" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O11" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P11" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q11" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R11" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S11" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T11" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U11" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V11" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W11" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X11" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y11" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z11" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC11" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C12" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D12" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E12" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F12" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G12" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I12" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J12" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K12" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L12" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M12" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N12" t="n">
         <v>32.58</v>
       </c>
       <c r="O12" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P12" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q12" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R12" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S12" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T12" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V12" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W12" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X12" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y12" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z12" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB12" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC12" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C13" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D13" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E13" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F13" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G13" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H13" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I13" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J13" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K13" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L13" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M13" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N13" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O13" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P13" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q13" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R13" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S13" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T13" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U13" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V13" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W13" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X13" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y13" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z13" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA13" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB13" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC13" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C14" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D14" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E14" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F14" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G14" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H14" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I14" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J14" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K14" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L14" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M14" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N14" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O14" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P14" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q14" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R14" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S14" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T14" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U14" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W14" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X14" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y14" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z14" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC14" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C15" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D15" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E15" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F15" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H15" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I15" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J15" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K15" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L15" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M15" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N15" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O15" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P15" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q15" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R15" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S15" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T15" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U15" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V15" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W15" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X15" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y15" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z15" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA15" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB15" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC15" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C16" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D16" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E16" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F16" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G16" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I16" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J16" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K16" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L16" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M16" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N16" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O16" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P16" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q16" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S16" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T16" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V16" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W16" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X16" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y16" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z16" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA16" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB16" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC16" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C17" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D17" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E17" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F17" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G17" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K17" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L17" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M17" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N17" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O17" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P17" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q17" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R17" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S17" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T17" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U17" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V17" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W17" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X17" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y17" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z17" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA17" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB17" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC17" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>98.34999999999999</v>
+        <v>101.19</v>
       </c>
       <c r="C18" t="n">
-        <v>108.8</v>
+        <v>103.93</v>
       </c>
       <c r="D18" t="n">
-        <v>95.23</v>
+        <v>93.45</v>
       </c>
       <c r="E18" t="n">
-        <v>107.35</v>
+        <v>93.67</v>
       </c>
       <c r="F18" t="n">
-        <v>70.95</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>74.23999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="H18" t="n">
-        <v>69.98999999999999</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>73.81999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>47.19</v>
+        <v>46.22</v>
       </c>
       <c r="K18" t="n">
-        <v>48.37</v>
+        <v>49.36</v>
       </c>
       <c r="L18" t="n">
-        <v>43.11</v>
+        <v>45.08</v>
       </c>
       <c r="M18" t="n">
-        <v>43.64</v>
+        <v>49.23</v>
       </c>
       <c r="N18" t="n">
-        <v>37.57</v>
+        <v>36.57</v>
       </c>
       <c r="O18" t="n">
-        <v>38.02</v>
+        <v>39.29</v>
       </c>
       <c r="P18" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q18" t="n">
-        <v>36.14</v>
+        <v>38.9</v>
       </c>
       <c r="R18" t="n">
-        <v>-2.8858</v>
+        <v>-12.7434</v>
       </c>
       <c r="S18" t="n">
-        <v>-16.3941</v>
+        <v>-26.5736</v>
       </c>
       <c r="T18" t="n">
-        <v>-24.6772</v>
+        <v>-32.978</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.4047</v>
+        <v>-7.5996</v>
       </c>
       <c r="V18" t="n">
-        <v>-7.273</v>
+        <v>-13.4501</v>
       </c>
       <c r="W18" t="n">
-        <v>-7.9895</v>
+        <v>-16.0802</v>
       </c>
       <c r="X18" t="n">
-        <v>2.6341</v>
+        <v>12.8093</v>
       </c>
       <c r="Y18" t="n">
-        <v>17.3434</v>
+        <v>31.5607</v>
       </c>
       <c r="Z18" t="n">
-        <v>29.1506</v>
+        <v>43.1521</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.3889</v>
+        <v>7.637</v>
       </c>
       <c r="AB18" t="n">
-        <v>7.4636</v>
+        <v>14.4454</v>
       </c>
       <c r="AC18" t="n">
-        <v>8.3009</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>101.19</v>
+        <v>103.95</v>
       </c>
       <c r="C19" t="n">
-        <v>103.93</v>
+        <v>104.98</v>
       </c>
       <c r="D19" t="n">
-        <v>93.45</v>
+        <v>97.8</v>
       </c>
       <c r="E19" t="n">
-        <v>93.67</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>73.01000000000001</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>73.13</v>
+        <v>72.44</v>
       </c>
       <c r="H19" t="n">
-        <v>67.43000000000001</v>
+        <v>70.13</v>
       </c>
       <c r="I19" t="n">
-        <v>68.20999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J19" t="n">
-        <v>46.22</v>
+        <v>43.86</v>
       </c>
       <c r="K19" t="n">
-        <v>49.36</v>
+        <v>47.07</v>
       </c>
       <c r="L19" t="n">
-        <v>45.08</v>
+        <v>43.32</v>
       </c>
       <c r="M19" t="n">
-        <v>49.23</v>
+        <v>46.63</v>
       </c>
       <c r="N19" t="n">
-        <v>36.57</v>
+        <v>37.33</v>
       </c>
       <c r="O19" t="n">
-        <v>39.29</v>
+        <v>37.82</v>
       </c>
       <c r="P19" t="n">
         <v>36.51</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.9</v>
+        <v>37.52</v>
       </c>
       <c r="R19" t="n">
-        <v>-12.7434</v>
+        <v>5.3165</v>
       </c>
       <c r="S19" t="n">
-        <v>-26.5736</v>
+        <v>-10.7563</v>
       </c>
       <c r="T19" t="n">
-        <v>-32.978</v>
+        <v>-23.1698</v>
       </c>
       <c r="U19" t="n">
-        <v>-7.5996</v>
+        <v>3.5625</v>
       </c>
       <c r="V19" t="n">
-        <v>-13.4501</v>
+        <v>-4.6951</v>
       </c>
       <c r="W19" t="n">
-        <v>-16.0802</v>
+        <v>-11.2674</v>
       </c>
       <c r="X19" t="n">
-        <v>12.8093</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y19" t="n">
-        <v>31.5607</v>
+        <v>9.666</v>
       </c>
       <c r="Z19" t="n">
-        <v>43.1521</v>
+        <v>25.3832</v>
       </c>
       <c r="AA19" t="n">
-        <v>7.637</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB19" t="n">
-        <v>14.4454</v>
+        <v>4.2222</v>
       </c>
       <c r="AC19" t="n">
-        <v>18.0577</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>103.95</v>
+        <v>94.52</v>
       </c>
       <c r="C20" t="n">
-        <v>104.98</v>
+        <v>102.62</v>
       </c>
       <c r="D20" t="n">
-        <v>97.8</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E20" t="n">
-        <v>98.65000000000001</v>
+        <v>97.55</v>
       </c>
       <c r="F20" t="n">
-        <v>71.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>72.44</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>70.13</v>
+        <v>68.28</v>
       </c>
       <c r="I20" t="n">
-        <v>70.64</v>
+        <v>70.41</v>
       </c>
       <c r="J20" t="n">
-        <v>43.86</v>
+        <v>48.64</v>
       </c>
       <c r="K20" t="n">
-        <v>47.07</v>
+        <v>50.12</v>
       </c>
       <c r="L20" t="n">
-        <v>43.32</v>
+        <v>44.76</v>
       </c>
       <c r="M20" t="n">
-        <v>46.63</v>
+        <v>47.13</v>
       </c>
       <c r="N20" t="n">
-        <v>37.33</v>
+        <v>38.03</v>
       </c>
       <c r="O20" t="n">
-        <v>37.82</v>
+        <v>38.79</v>
       </c>
       <c r="P20" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.52</v>
+        <v>37.68</v>
       </c>
       <c r="R20" t="n">
-        <v>5.3165</v>
+        <v>-1.1151</v>
       </c>
       <c r="S20" t="n">
-        <v>-10.7563</v>
+        <v>-9.129</v>
       </c>
       <c r="T20" t="n">
-        <v>-23.1698</v>
+        <v>-23.5322</v>
       </c>
       <c r="U20" t="n">
-        <v>3.5625</v>
+        <v>-0.3256</v>
       </c>
       <c r="V20" t="n">
-        <v>-4.6951</v>
+        <v>-4.6193</v>
       </c>
       <c r="W20" t="n">
-        <v>-11.2674</v>
+        <v>-10.6585</v>
       </c>
       <c r="X20" t="n">
-        <v>-5.2813</v>
+        <v>1.0723</v>
       </c>
       <c r="Y20" t="n">
-        <v>9.666</v>
+        <v>7.9973</v>
       </c>
       <c r="Z20" t="n">
-        <v>25.3832</v>
+        <v>25.9487</v>
       </c>
       <c r="AA20" t="n">
-        <v>-3.5476</v>
+        <v>0.4264</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.2222</v>
+        <v>4.2612</v>
       </c>
       <c r="AC20" t="n">
-        <v>11.5671</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>94.52</v>
+        <v>102.86</v>
       </c>
       <c r="C21" t="n">
-        <v>102.62</v>
+        <v>106.13</v>
       </c>
       <c r="D21" t="n">
-        <v>91.34999999999999</v>
+        <v>99.31</v>
       </c>
       <c r="E21" t="n">
-        <v>97.55</v>
+        <v>103.24</v>
       </c>
       <c r="F21" t="n">
-        <v>69.70999999999999</v>
+        <v>71.72</v>
       </c>
       <c r="G21" t="n">
-        <v>71.93000000000001</v>
+        <v>73.43000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>68.28</v>
+        <v>71.02</v>
       </c>
       <c r="I21" t="n">
-        <v>70.41</v>
+        <v>72.61</v>
       </c>
       <c r="J21" t="n">
-        <v>48.64</v>
+        <v>44.51</v>
       </c>
       <c r="K21" t="n">
-        <v>50.12</v>
+        <v>47.1</v>
       </c>
       <c r="L21" t="n">
-        <v>44.76</v>
+        <v>43.57</v>
       </c>
       <c r="M21" t="n">
-        <v>47.13</v>
+        <v>44.29</v>
       </c>
       <c r="N21" t="n">
-        <v>38.03</v>
+        <v>36.94</v>
       </c>
       <c r="O21" t="n">
-        <v>38.79</v>
+        <v>38.11</v>
       </c>
       <c r="P21" t="n">
-        <v>36.85</v>
+        <v>36.05</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.68</v>
+        <v>36.48</v>
       </c>
       <c r="R21" t="n">
-        <v>-1.1151</v>
+        <v>5.8329</v>
       </c>
       <c r="S21" t="n">
-        <v>-9.129</v>
+        <v>10.2167</v>
       </c>
       <c r="T21" t="n">
-        <v>-23.5322</v>
+        <v>-6.6039</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.3256</v>
+        <v>3.1246</v>
       </c>
       <c r="V21" t="n">
-        <v>-4.6193</v>
+        <v>6.4507</v>
       </c>
       <c r="W21" t="n">
-        <v>-10.6585</v>
+        <v>-2.0372</v>
       </c>
       <c r="X21" t="n">
-        <v>1.0723</v>
+        <v>-6.0259</v>
       </c>
       <c r="Y21" t="n">
-        <v>7.9973</v>
+        <v>-10.0345</v>
       </c>
       <c r="Z21" t="n">
-        <v>25.9487</v>
+        <v>4.1627</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.4264</v>
+        <v>-3.1847</v>
       </c>
       <c r="AB21" t="n">
-        <v>4.2612</v>
+        <v>-6.2211</v>
       </c>
       <c r="AC21" t="n">
-        <v>10.8561</v>
+        <v>1.3333</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>102.86</v>
+        <v>90.59</v>
       </c>
       <c r="C22" t="n">
-        <v>106.13</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="D22" t="n">
-        <v>99.31</v>
+        <v>80.22</v>
       </c>
       <c r="E22" t="n">
-        <v>103.24</v>
+        <v>82.11</v>
       </c>
       <c r="F22" t="n">
-        <v>71.72</v>
+        <v>69.14</v>
       </c>
       <c r="G22" t="n">
-        <v>73.43000000000001</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>71.02</v>
+        <v>65.61</v>
       </c>
       <c r="I22" t="n">
-        <v>72.61</v>
+        <v>66.42</v>
       </c>
       <c r="J22" t="n">
-        <v>44.51</v>
+        <v>49.82</v>
       </c>
       <c r="K22" t="n">
-        <v>47.1</v>
+        <v>54.31</v>
       </c>
       <c r="L22" t="n">
-        <v>43.57</v>
+        <v>48.62</v>
       </c>
       <c r="M22" t="n">
-        <v>44.29</v>
+        <v>53.45</v>
       </c>
       <c r="N22" t="n">
-        <v>36.94</v>
+        <v>38.23</v>
       </c>
       <c r="O22" t="n">
-        <v>38.11</v>
+        <v>40</v>
       </c>
       <c r="P22" t="n">
-        <v>36.05</v>
+        <v>37.96</v>
       </c>
       <c r="Q22" t="n">
-        <v>36.48</v>
+        <v>39.6</v>
       </c>
       <c r="R22" t="n">
-        <v>5.8329</v>
+        <v>-20.4669</v>
       </c>
       <c r="S22" t="n">
-        <v>10.2167</v>
+        <v>-16.7663</v>
       </c>
       <c r="T22" t="n">
-        <v>-6.6039</v>
+        <v>-23.5119</v>
       </c>
       <c r="U22" t="n">
-        <v>3.1246</v>
+        <v>-8.525</v>
       </c>
       <c r="V22" t="n">
-        <v>6.4507</v>
+        <v>-5.974</v>
       </c>
       <c r="W22" t="n">
-        <v>-2.0372</v>
+        <v>-10.0244</v>
       </c>
       <c r="X22" t="n">
-        <v>-6.0259</v>
+        <v>20.6819</v>
       </c>
       <c r="Y22" t="n">
-        <v>-10.0345</v>
+        <v>14.6258</v>
       </c>
       <c r="Z22" t="n">
-        <v>4.1627</v>
+        <v>22.4794</v>
       </c>
       <c r="AA22" t="n">
-        <v>-3.1847</v>
+        <v>8.5526</v>
       </c>
       <c r="AB22" t="n">
-        <v>-6.2211</v>
+        <v>5.5437</v>
       </c>
       <c r="AC22" t="n">
-        <v>1.3333</v>
+        <v>9.5739</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-27 01:11
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1810 +568,1719 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>138.47</v>
+        <v>148.14</v>
       </c>
       <c r="C2" t="n">
-        <v>147.2</v>
+        <v>149.99</v>
       </c>
       <c r="D2" t="n">
-        <v>136.9</v>
+        <v>135.21</v>
       </c>
       <c r="E2" t="n">
-        <v>146.33</v>
+        <v>142.29</v>
       </c>
       <c r="F2" t="n">
-        <v>76.75</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>79.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>76.55</v>
+        <v>75.47</v>
       </c>
       <c r="I2" t="n">
-        <v>78.58</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>35.45</v>
+        <v>33.17</v>
       </c>
       <c r="K2" t="n">
-        <v>35.85</v>
+        <v>35.95</v>
       </c>
       <c r="L2" t="n">
-        <v>33.43</v>
+        <v>32.77</v>
       </c>
       <c r="M2" t="n">
-        <v>33.63</v>
+        <v>34.43</v>
       </c>
       <c r="N2" t="n">
-        <v>34.98</v>
+        <v>34.31</v>
       </c>
       <c r="O2" t="n">
-        <v>35.06</v>
+        <v>35.53</v>
       </c>
       <c r="P2" t="n">
-        <v>33.95</v>
+        <v>34.17</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.18</v>
+        <v>34.83</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>149.24</v>
+        <v>148.94</v>
       </c>
       <c r="C3" t="n">
-        <v>153.9</v>
+        <v>152.37</v>
       </c>
       <c r="D3" t="n">
-        <v>147.39</v>
+        <v>145.49</v>
       </c>
       <c r="E3" t="n">
-        <v>151.45</v>
+        <v>147</v>
       </c>
       <c r="F3" t="n">
-        <v>79.09</v>
+        <v>78.13</v>
       </c>
       <c r="G3" t="n">
-        <v>80.06</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>78.06</v>
+        <v>76.62</v>
       </c>
       <c r="I3" t="n">
-        <v>79.59999999999999</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>32.97</v>
+        <v>32.82</v>
       </c>
       <c r="K3" t="n">
-        <v>33.39</v>
+        <v>33.64</v>
       </c>
       <c r="L3" t="n">
-        <v>31.9</v>
+        <v>31.96</v>
       </c>
       <c r="M3" t="n">
-        <v>32.43</v>
+        <v>33.26</v>
       </c>
       <c r="N3" t="n">
-        <v>33.97</v>
+        <v>34.34</v>
       </c>
       <c r="O3" t="n">
-        <v>34.41</v>
+        <v>35.02</v>
       </c>
       <c r="P3" t="n">
-        <v>33.54</v>
+        <v>34.28</v>
       </c>
       <c r="Q3" t="n">
-        <v>33.75</v>
+        <v>34.66</v>
       </c>
       <c r="R3" t="n">
-        <v>3.4989</v>
+        <v>3.3101</v>
       </c>
       <c r="U3" t="n">
-        <v>1.298</v>
+        <v>0.5452</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.5682</v>
+        <v>-3.3982</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.258</v>
+        <v>-0.4881</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>148.14</v>
+        <v>147.95</v>
       </c>
       <c r="C4" t="n">
-        <v>149.99</v>
+        <v>150.77</v>
       </c>
       <c r="D4" t="n">
-        <v>135.21</v>
+        <v>144.41</v>
       </c>
       <c r="E4" t="n">
-        <v>142.29</v>
+        <v>147.86</v>
       </c>
       <c r="F4" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G4" t="n">
-        <v>78.59999999999999</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>75.47</v>
+        <v>77.94</v>
       </c>
       <c r="I4" t="n">
-        <v>77.04000000000001</v>
+        <v>78.03</v>
       </c>
       <c r="J4" t="n">
-        <v>33.17</v>
+        <v>33.07</v>
       </c>
       <c r="K4" t="n">
-        <v>35.95</v>
+        <v>33.86</v>
       </c>
       <c r="L4" t="n">
-        <v>32.77</v>
+        <v>32.42</v>
       </c>
       <c r="M4" t="n">
-        <v>34.43</v>
+        <v>33.08</v>
       </c>
       <c r="N4" t="n">
-        <v>34.31</v>
+        <v>34.36</v>
       </c>
       <c r="O4" t="n">
-        <v>35.53</v>
+        <v>34.44</v>
       </c>
       <c r="P4" t="n">
-        <v>34.17</v>
+        <v>33.66</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.83</v>
+        <v>34.41</v>
       </c>
       <c r="R4" t="n">
-        <v>-6.0482</v>
+        <v>0.585</v>
       </c>
       <c r="U4" t="n">
-        <v>-3.2161</v>
+        <v>0.7359</v>
       </c>
       <c r="X4" t="n">
-        <v>6.1671</v>
+        <v>-0.5412</v>
       </c>
       <c r="AA4" t="n">
-        <v>3.2</v>
+        <v>-0.7213000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>148.94</v>
+        <v>148.56</v>
       </c>
       <c r="C5" t="n">
-        <v>152.37</v>
+        <v>156.71</v>
       </c>
       <c r="D5" t="n">
-        <v>145.49</v>
+        <v>144.31</v>
       </c>
       <c r="E5" t="n">
-        <v>147</v>
+        <v>153.69</v>
       </c>
       <c r="F5" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G5" t="n">
-        <v>78.26000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H5" t="n">
-        <v>76.62</v>
+        <v>76.87</v>
       </c>
       <c r="I5" t="n">
-        <v>77.45999999999999</v>
+        <v>78.73</v>
       </c>
       <c r="J5" t="n">
-        <v>32.82</v>
+        <v>32.95</v>
       </c>
       <c r="K5" t="n">
-        <v>33.64</v>
+        <v>33.89</v>
       </c>
       <c r="L5" t="n">
-        <v>31.96</v>
+        <v>31.1</v>
       </c>
       <c r="M5" t="n">
-        <v>33.26</v>
+        <v>31.76</v>
       </c>
       <c r="N5" t="n">
-        <v>34.34</v>
+        <v>34.04</v>
       </c>
       <c r="O5" t="n">
-        <v>35.02</v>
+        <v>34.92</v>
       </c>
       <c r="P5" t="n">
-        <v>34.28</v>
+        <v>33.74</v>
       </c>
       <c r="Q5" t="n">
-        <v>34.66</v>
+        <v>34.11</v>
       </c>
       <c r="R5" t="n">
-        <v>3.3101</v>
+        <v>3.9429</v>
       </c>
       <c r="S5" t="n">
-        <v>0.4579</v>
+        <v>8.011799999999999</v>
       </c>
       <c r="U5" t="n">
-        <v>0.5452</v>
+        <v>0.8971</v>
       </c>
       <c r="V5" t="n">
-        <v>-1.4253</v>
+        <v>2.1937</v>
       </c>
       <c r="X5" t="n">
-        <v>-3.3982</v>
+        <v>-3.9903</v>
       </c>
       <c r="Y5" t="n">
-        <v>-1.1002</v>
+        <v>-7.7549</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.4881</v>
+        <v>-0.8718</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.4043</v>
+        <v>-2.0672</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>147.95</v>
+        <v>165.39</v>
       </c>
       <c r="C6" t="n">
-        <v>150.77</v>
+        <v>169.75</v>
       </c>
       <c r="D6" t="n">
-        <v>144.41</v>
+        <v>162.4</v>
       </c>
       <c r="E6" t="n">
-        <v>147.86</v>
+        <v>163.71</v>
       </c>
       <c r="F6" t="n">
-        <v>78.13</v>
+        <v>81.59</v>
       </c>
       <c r="G6" t="n">
-        <v>79.68000000000001</v>
+        <v>82.61</v>
       </c>
       <c r="H6" t="n">
-        <v>77.94</v>
+        <v>80.37</v>
       </c>
       <c r="I6" t="n">
-        <v>78.03</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>33.07</v>
+        <v>29.39</v>
       </c>
       <c r="K6" t="n">
-        <v>33.86</v>
+        <v>29.98</v>
       </c>
       <c r="L6" t="n">
-        <v>32.42</v>
+        <v>28.46</v>
       </c>
       <c r="M6" t="n">
-        <v>33.08</v>
+        <v>29.71</v>
       </c>
       <c r="N6" t="n">
-        <v>34.36</v>
+        <v>32.87</v>
       </c>
       <c r="O6" t="n">
-        <v>34.44</v>
+        <v>33.41</v>
       </c>
       <c r="P6" t="n">
-        <v>33.66</v>
+        <v>32.44</v>
       </c>
       <c r="Q6" t="n">
-        <v>34.41</v>
+        <v>33.12</v>
       </c>
       <c r="R6" t="n">
-        <v>0.585</v>
+        <v>6.5196</v>
       </c>
       <c r="S6" t="n">
-        <v>-2.3704</v>
+        <v>11.3673</v>
       </c>
       <c r="U6" t="n">
-        <v>0.7359</v>
+        <v>2.896</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.9724</v>
+        <v>4.583</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.5412</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.0043</v>
+        <v>-10.6735</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.9556</v>
+        <v>-4.4432</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148.56</v>
+        <v>161.66</v>
       </c>
       <c r="C7" t="n">
-        <v>156.71</v>
+        <v>164.38</v>
       </c>
       <c r="D7" t="n">
-        <v>144.31</v>
+        <v>158.08</v>
       </c>
       <c r="E7" t="n">
-        <v>153.69</v>
+        <v>164.27</v>
       </c>
       <c r="F7" t="n">
-        <v>78.88</v>
+        <v>80.95</v>
       </c>
       <c r="G7" t="n">
-        <v>79.53</v>
+        <v>83.38</v>
       </c>
       <c r="H7" t="n">
-        <v>76.87</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>78.73</v>
+        <v>83.12</v>
       </c>
       <c r="J7" t="n">
-        <v>32.95</v>
+        <v>30.09</v>
       </c>
       <c r="K7" t="n">
-        <v>33.89</v>
+        <v>30.75</v>
       </c>
       <c r="L7" t="n">
-        <v>31.1</v>
+        <v>29.62</v>
       </c>
       <c r="M7" t="n">
-        <v>31.76</v>
+        <v>29.62</v>
       </c>
       <c r="N7" t="n">
-        <v>34.04</v>
+        <v>33.17</v>
       </c>
       <c r="O7" t="n">
-        <v>34.92</v>
+        <v>33.2</v>
       </c>
       <c r="P7" t="n">
-        <v>33.74</v>
+        <v>32.16</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.11</v>
+        <v>32.25</v>
       </c>
       <c r="R7" t="n">
-        <v>3.9429</v>
+        <v>0.3421</v>
       </c>
       <c r="S7" t="n">
-        <v>8.011799999999999</v>
+        <v>11.0983</v>
       </c>
       <c r="T7" t="n">
-        <v>5.0297</v>
+        <v>15.4473</v>
       </c>
       <c r="U7" t="n">
-        <v>0.8971</v>
+        <v>2.6046</v>
       </c>
       <c r="V7" t="n">
-        <v>2.1937</v>
+        <v>6.5231</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1909</v>
+        <v>7.892</v>
       </c>
       <c r="X7" t="n">
-        <v>-3.9903</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y7" t="n">
-        <v>-7.7549</v>
+        <v>-10.4595</v>
       </c>
       <c r="Z7" t="n">
-        <v>-5.5605</v>
+        <v>-13.9704</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.8718</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.0672</v>
+        <v>-6.2772</v>
       </c>
       <c r="AC7" t="n">
-        <v>-0.2048</v>
+        <v>-7.4074</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>165.39</v>
+        <v>167.34</v>
       </c>
       <c r="C8" t="n">
-        <v>169.75</v>
+        <v>169.83</v>
       </c>
       <c r="D8" t="n">
-        <v>162.4</v>
+        <v>163.42</v>
       </c>
       <c r="E8" t="n">
-        <v>163.71</v>
+        <v>164.26</v>
       </c>
       <c r="F8" t="n">
-        <v>81.59</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>82.61</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>80.37</v>
+        <v>84.09</v>
       </c>
       <c r="I8" t="n">
-        <v>81.01000000000001</v>
+        <v>84.25</v>
       </c>
       <c r="J8" t="n">
-        <v>29.39</v>
+        <v>29.06</v>
       </c>
       <c r="K8" t="n">
-        <v>29.98</v>
+        <v>29.77</v>
       </c>
       <c r="L8" t="n">
-        <v>28.46</v>
+        <v>28.62</v>
       </c>
       <c r="M8" t="n">
-        <v>29.71</v>
+        <v>29.63</v>
       </c>
       <c r="N8" t="n">
-        <v>32.87</v>
+        <v>31.72</v>
       </c>
       <c r="O8" t="n">
-        <v>33.41</v>
+        <v>31.9</v>
       </c>
       <c r="P8" t="n">
-        <v>32.44</v>
+        <v>31.42</v>
       </c>
       <c r="Q8" t="n">
-        <v>33.12</v>
+        <v>31.83</v>
       </c>
       <c r="R8" t="n">
-        <v>6.5196</v>
+        <v>-0.0061</v>
       </c>
       <c r="S8" t="n">
-        <v>11.3673</v>
+        <v>6.8775</v>
       </c>
       <c r="T8" t="n">
-        <v>8.0951</v>
+        <v>11.7415</v>
       </c>
       <c r="U8" t="n">
-        <v>2.896</v>
+        <v>1.3595</v>
       </c>
       <c r="V8" t="n">
-        <v>4.583</v>
+        <v>7.0113</v>
       </c>
       <c r="W8" t="n">
-        <v>1.7714</v>
+        <v>8.7658</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.4547</v>
+        <v>0.0338</v>
       </c>
       <c r="Y8" t="n">
-        <v>-10.6735</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z8" t="n">
-        <v>-8.3873</v>
+        <v>-10.914</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.9024</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB8" t="n">
-        <v>-4.4432</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC8" t="n">
-        <v>-1.8667</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>161.66</v>
+        <v>153.7</v>
       </c>
       <c r="C9" t="n">
-        <v>164.38</v>
+        <v>159.49</v>
       </c>
       <c r="D9" t="n">
-        <v>158.08</v>
+        <v>151.42</v>
       </c>
       <c r="E9" t="n">
-        <v>164.27</v>
+        <v>158.91</v>
       </c>
       <c r="F9" t="n">
-        <v>80.95</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>83.38</v>
+        <v>83.75</v>
       </c>
       <c r="H9" t="n">
-        <v>80.84999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>83.12</v>
+        <v>83.62</v>
       </c>
       <c r="J9" t="n">
-        <v>30.09</v>
+        <v>31.55</v>
       </c>
       <c r="K9" t="n">
-        <v>30.75</v>
+        <v>31.97</v>
       </c>
       <c r="L9" t="n">
-        <v>29.62</v>
+        <v>30.5</v>
       </c>
       <c r="M9" t="n">
-        <v>29.62</v>
+        <v>30.65</v>
       </c>
       <c r="N9" t="n">
-        <v>33.17</v>
+        <v>32.58</v>
       </c>
       <c r="O9" t="n">
-        <v>33.2</v>
+        <v>32.84</v>
       </c>
       <c r="P9" t="n">
-        <v>32.16</v>
+        <v>32.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>32.25</v>
+        <v>32.07</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3421</v>
+        <v>-3.257</v>
       </c>
       <c r="S9" t="n">
-        <v>11.0983</v>
+        <v>-2.932</v>
       </c>
       <c r="T9" t="n">
-        <v>15.4473</v>
+        <v>7.4733</v>
       </c>
       <c r="U9" t="n">
-        <v>2.6046</v>
+        <v>-0.7478</v>
       </c>
       <c r="V9" t="n">
-        <v>6.5231</v>
+        <v>3.2218</v>
       </c>
       <c r="W9" t="n">
-        <v>7.892</v>
+        <v>7.1639</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.3029</v>
+        <v>3.4425</v>
       </c>
       <c r="Y9" t="n">
-        <v>-10.4595</v>
+        <v>3.1639</v>
       </c>
       <c r="Z9" t="n">
-        <v>-13.9704</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.6268</v>
+        <v>0.754</v>
       </c>
       <c r="AB9" t="n">
-        <v>-6.2772</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC9" t="n">
-        <v>-7.4074</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>167.34</v>
+        <v>150.48</v>
       </c>
       <c r="C10" t="n">
-        <v>169.83</v>
+        <v>155.5</v>
       </c>
       <c r="D10" t="n">
-        <v>163.42</v>
+        <v>136.32</v>
       </c>
       <c r="E10" t="n">
-        <v>164.26</v>
+        <v>142.52</v>
       </c>
       <c r="F10" t="n">
-        <v>84.54000000000001</v>
+        <v>82.33</v>
       </c>
       <c r="G10" t="n">
-        <v>85.31999999999999</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>84.09</v>
+        <v>78.78</v>
       </c>
       <c r="I10" t="n">
-        <v>84.25</v>
+        <v>80.23</v>
       </c>
       <c r="J10" t="n">
-        <v>29.06</v>
+        <v>32.25</v>
       </c>
       <c r="K10" t="n">
-        <v>29.77</v>
+        <v>34.96</v>
       </c>
       <c r="L10" t="n">
-        <v>28.62</v>
+        <v>31.25</v>
       </c>
       <c r="M10" t="n">
-        <v>29.63</v>
+        <v>33.79</v>
       </c>
       <c r="N10" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O10" t="n">
-        <v>31.9</v>
+        <v>33.94</v>
       </c>
       <c r="P10" t="n">
-        <v>31.42</v>
+        <v>32.16</v>
       </c>
       <c r="Q10" t="n">
-        <v>31.83</v>
+        <v>33.37</v>
       </c>
       <c r="R10" t="n">
-        <v>-0.0061</v>
+        <v>-10.314</v>
       </c>
       <c r="S10" t="n">
-        <v>6.8775</v>
+        <v>-13.2404</v>
       </c>
       <c r="T10" t="n">
-        <v>11.7415</v>
+        <v>-7.2679</v>
       </c>
       <c r="U10" t="n">
-        <v>1.3595</v>
+        <v>-4.0541</v>
       </c>
       <c r="V10" t="n">
-        <v>7.0113</v>
+        <v>-3.4769</v>
       </c>
       <c r="W10" t="n">
-        <v>8.7658</v>
+        <v>1.9052</v>
       </c>
       <c r="X10" t="n">
-        <v>0.0338</v>
+        <v>10.2447</v>
       </c>
       <c r="Y10" t="n">
-        <v>-6.7065</v>
+        <v>14.0783</v>
       </c>
       <c r="Z10" t="n">
-        <v>-10.914</v>
+        <v>6.3917</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.3023</v>
+        <v>4.0536</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.6843</v>
+        <v>3.4729</v>
       </c>
       <c r="AC10" t="n">
-        <v>-8.164999999999999</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>153.7</v>
+        <v>148.18</v>
       </c>
       <c r="C11" t="n">
-        <v>159.49</v>
+        <v>148.18</v>
       </c>
       <c r="D11" t="n">
-        <v>151.42</v>
+        <v>137.71</v>
       </c>
       <c r="E11" t="n">
-        <v>158.91</v>
+        <v>139.76</v>
       </c>
       <c r="F11" t="n">
-        <v>82.31999999999999</v>
+        <v>81.72</v>
       </c>
       <c r="G11" t="n">
-        <v>83.75</v>
+        <v>81.81</v>
       </c>
       <c r="H11" t="n">
-        <v>81.59999999999999</v>
+        <v>80.37</v>
       </c>
       <c r="I11" t="n">
-        <v>83.62</v>
+        <v>81.28</v>
       </c>
       <c r="J11" t="n">
-        <v>31.55</v>
+        <v>32.4</v>
       </c>
       <c r="K11" t="n">
-        <v>31.97</v>
+        <v>34.91</v>
       </c>
       <c r="L11" t="n">
-        <v>30.5</v>
+        <v>32.39</v>
       </c>
       <c r="M11" t="n">
-        <v>30.65</v>
+        <v>34.39</v>
       </c>
       <c r="N11" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O11" t="n">
-        <v>32.84</v>
+        <v>33.34</v>
       </c>
       <c r="P11" t="n">
-        <v>32.02</v>
+        <v>32.73</v>
       </c>
       <c r="Q11" t="n">
-        <v>32.07</v>
+        <v>32.95</v>
       </c>
       <c r="R11" t="n">
-        <v>-3.257</v>
+        <v>-1.9366</v>
       </c>
       <c r="S11" t="n">
-        <v>-2.932</v>
+        <v>-14.9154</v>
       </c>
       <c r="T11" t="n">
-        <v>7.4733</v>
+        <v>-14.6295</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.7478</v>
+        <v>1.3087</v>
       </c>
       <c r="V11" t="n">
-        <v>3.2218</v>
+        <v>-3.5252</v>
       </c>
       <c r="W11" t="n">
-        <v>7.1639</v>
+        <v>0.3333</v>
       </c>
       <c r="X11" t="n">
-        <v>3.4425</v>
+        <v>1.7757</v>
       </c>
       <c r="Y11" t="n">
-        <v>3.1639</v>
+        <v>16.0648</v>
       </c>
       <c r="Z11" t="n">
-        <v>-7.3458</v>
+        <v>15.7523</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.754</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB11" t="n">
-        <v>-3.1703</v>
+        <v>3.5187</v>
       </c>
       <c r="AC11" t="n">
-        <v>-6.8003</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>150.48</v>
+        <v>134.43</v>
       </c>
       <c r="C12" t="n">
-        <v>155.5</v>
+        <v>134.54</v>
       </c>
       <c r="D12" t="n">
-        <v>136.32</v>
+        <v>127.27</v>
       </c>
       <c r="E12" t="n">
-        <v>142.52</v>
+        <v>128.4</v>
       </c>
       <c r="F12" t="n">
-        <v>82.33</v>
+        <v>80.78</v>
       </c>
       <c r="G12" t="n">
-        <v>83.40000000000001</v>
+        <v>80.81</v>
       </c>
       <c r="H12" t="n">
-        <v>78.78</v>
+        <v>79.22</v>
       </c>
       <c r="I12" t="n">
-        <v>80.23</v>
+        <v>79.61</v>
       </c>
       <c r="J12" t="n">
-        <v>32.25</v>
+        <v>35.75</v>
       </c>
       <c r="K12" t="n">
-        <v>34.96</v>
+        <v>37.5</v>
       </c>
       <c r="L12" t="n">
-        <v>31.25</v>
+        <v>35.68</v>
       </c>
       <c r="M12" t="n">
-        <v>33.79</v>
+        <v>37.19</v>
       </c>
       <c r="N12" t="n">
-        <v>32.58</v>
+        <v>33.17</v>
       </c>
       <c r="O12" t="n">
-        <v>33.94</v>
+        <v>33.8</v>
       </c>
       <c r="P12" t="n">
-        <v>32.16</v>
+        <v>33.17</v>
       </c>
       <c r="Q12" t="n">
-        <v>33.37</v>
+        <v>33.63</v>
       </c>
       <c r="R12" t="n">
-        <v>-10.314</v>
+        <v>-8.1282</v>
       </c>
       <c r="S12" t="n">
-        <v>-13.2404</v>
+        <v>-19.1995</v>
       </c>
       <c r="T12" t="n">
-        <v>-7.2679</v>
+        <v>-21.836</v>
       </c>
       <c r="U12" t="n">
-        <v>-4.0541</v>
+        <v>-2.0546</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.4769</v>
+        <v>-4.7955</v>
       </c>
       <c r="W12" t="n">
-        <v>1.9052</v>
+        <v>-4.2228</v>
       </c>
       <c r="X12" t="n">
-        <v>10.2447</v>
+        <v>8.1419</v>
       </c>
       <c r="Y12" t="n">
-        <v>14.0783</v>
+        <v>21.3377</v>
       </c>
       <c r="Z12" t="n">
-        <v>6.3917</v>
+        <v>25.5571</v>
       </c>
       <c r="AA12" t="n">
-        <v>4.0536</v>
+        <v>2.0637</v>
       </c>
       <c r="AB12" t="n">
-        <v>3.4729</v>
+        <v>4.8644</v>
       </c>
       <c r="AC12" t="n">
-        <v>-2.1695</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>148.18</v>
+        <v>118.42</v>
       </c>
       <c r="C13" t="n">
-        <v>148.18</v>
+        <v>127.92</v>
       </c>
       <c r="D13" t="n">
-        <v>137.71</v>
+        <v>115.84</v>
       </c>
       <c r="E13" t="n">
-        <v>139.76</v>
+        <v>127.57</v>
       </c>
       <c r="F13" t="n">
-        <v>81.72</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>81.81</v>
+        <v>79</v>
       </c>
       <c r="H13" t="n">
-        <v>80.37</v>
+        <v>77.28</v>
       </c>
       <c r="I13" t="n">
-        <v>81.28</v>
+        <v>78.81</v>
       </c>
       <c r="J13" t="n">
-        <v>32.4</v>
+        <v>40.15</v>
       </c>
       <c r="K13" t="n">
-        <v>34.91</v>
+        <v>40.9</v>
       </c>
       <c r="L13" t="n">
-        <v>32.39</v>
+        <v>37.36</v>
       </c>
       <c r="M13" t="n">
-        <v>34.39</v>
+        <v>37.42</v>
       </c>
       <c r="N13" t="n">
-        <v>32.78</v>
+        <v>34.54</v>
       </c>
       <c r="O13" t="n">
-        <v>33.34</v>
+        <v>34.63</v>
       </c>
       <c r="P13" t="n">
-        <v>32.73</v>
+        <v>33.89</v>
       </c>
       <c r="Q13" t="n">
-        <v>32.95</v>
+        <v>33.99</v>
       </c>
       <c r="R13" t="n">
-        <v>-1.9366</v>
+        <v>-0.6464</v>
       </c>
       <c r="S13" t="n">
-        <v>-14.9154</v>
+        <v>-10.4898</v>
       </c>
       <c r="T13" t="n">
-        <v>-14.6295</v>
+        <v>-22.3365</v>
       </c>
       <c r="U13" t="n">
-        <v>1.3087</v>
+        <v>-1.0049</v>
       </c>
       <c r="V13" t="n">
-        <v>-3.5252</v>
+        <v>-1.7699</v>
       </c>
       <c r="W13" t="n">
-        <v>0.3333</v>
+        <v>-6.457</v>
       </c>
       <c r="X13" t="n">
-        <v>1.7757</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y13" t="n">
-        <v>16.0648</v>
+        <v>10.7428</v>
       </c>
       <c r="Z13" t="n">
-        <v>15.7523</v>
+        <v>26.2909</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.2586</v>
+        <v>1.0705</v>
       </c>
       <c r="AB13" t="n">
-        <v>3.5187</v>
+        <v>1.858</v>
       </c>
       <c r="AC13" t="n">
-        <v>-0.5133</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>134.43</v>
+        <v>119.02</v>
       </c>
       <c r="C14" t="n">
-        <v>134.54</v>
+        <v>120.9</v>
       </c>
       <c r="D14" t="n">
-        <v>127.27</v>
+        <v>109</v>
       </c>
       <c r="E14" t="n">
-        <v>128.4</v>
+        <v>110.54</v>
       </c>
       <c r="F14" t="n">
-        <v>80.78</v>
+        <v>77</v>
       </c>
       <c r="G14" t="n">
-        <v>80.81</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>79.22</v>
+        <v>73.31</v>
       </c>
       <c r="I14" t="n">
-        <v>79.61</v>
+        <v>74.12</v>
       </c>
       <c r="J14" t="n">
-        <v>35.75</v>
+        <v>40.03</v>
       </c>
       <c r="K14" t="n">
-        <v>37.5</v>
+        <v>42.95</v>
       </c>
       <c r="L14" t="n">
-        <v>35.68</v>
+        <v>39.43</v>
       </c>
       <c r="M14" t="n">
-        <v>37.19</v>
+        <v>42.52</v>
       </c>
       <c r="N14" t="n">
-        <v>33.17</v>
+        <v>34.77</v>
       </c>
       <c r="O14" t="n">
-        <v>33.8</v>
+        <v>36.35</v>
       </c>
       <c r="P14" t="n">
-        <v>33.17</v>
+        <v>34.42</v>
       </c>
       <c r="Q14" t="n">
-        <v>33.63</v>
+        <v>36</v>
       </c>
       <c r="R14" t="n">
-        <v>-8.1282</v>
+        <v>-13.3495</v>
       </c>
       <c r="S14" t="n">
-        <v>-19.1995</v>
+        <v>-20.9073</v>
       </c>
       <c r="T14" t="n">
-        <v>-21.836</v>
+        <v>-30.4386</v>
       </c>
       <c r="U14" t="n">
-        <v>-2.0546</v>
+        <v>-5.951</v>
       </c>
       <c r="V14" t="n">
-        <v>-4.7955</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W14" t="n">
-        <v>-4.2228</v>
+        <v>-11.3609</v>
       </c>
       <c r="X14" t="n">
-        <v>8.1419</v>
+        <v>13.6291</v>
       </c>
       <c r="Y14" t="n">
-        <v>21.3377</v>
+        <v>23.6406</v>
       </c>
       <c r="Z14" t="n">
-        <v>25.5571</v>
+        <v>38.7276</v>
       </c>
       <c r="AA14" t="n">
-        <v>2.0637</v>
+        <v>5.9135</v>
       </c>
       <c r="AB14" t="n">
-        <v>4.8644</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC14" t="n">
-        <v>4.2791</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>118.42</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>127.92</v>
+        <v>108.8</v>
       </c>
       <c r="D15" t="n">
-        <v>115.84</v>
+        <v>95.23</v>
       </c>
       <c r="E15" t="n">
-        <v>127.57</v>
+        <v>107.35</v>
       </c>
       <c r="F15" t="n">
-        <v>77.51000000000001</v>
+        <v>70.95</v>
       </c>
       <c r="G15" t="n">
-        <v>79</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>77.28</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>78.81</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>40.15</v>
+        <v>47.19</v>
       </c>
       <c r="K15" t="n">
-        <v>40.9</v>
+        <v>48.37</v>
       </c>
       <c r="L15" t="n">
-        <v>37.36</v>
+        <v>43.11</v>
       </c>
       <c r="M15" t="n">
-        <v>37.42</v>
+        <v>43.64</v>
       </c>
       <c r="N15" t="n">
-        <v>34.54</v>
+        <v>37.57</v>
       </c>
       <c r="O15" t="n">
-        <v>34.63</v>
+        <v>38.02</v>
       </c>
       <c r="P15" t="n">
-        <v>33.89</v>
+        <v>35.94</v>
       </c>
       <c r="Q15" t="n">
-        <v>33.99</v>
+        <v>36.14</v>
       </c>
       <c r="R15" t="n">
-        <v>-0.6464</v>
+        <v>-2.8858</v>
       </c>
       <c r="S15" t="n">
-        <v>-10.4898</v>
+        <v>-16.3941</v>
       </c>
       <c r="T15" t="n">
-        <v>-22.3365</v>
+        <v>-24.6772</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.0049</v>
+        <v>-0.4047</v>
       </c>
       <c r="V15" t="n">
-        <v>-1.7699</v>
+        <v>-7.273</v>
       </c>
       <c r="W15" t="n">
-        <v>-6.457</v>
+        <v>-7.9895</v>
       </c>
       <c r="X15" t="n">
-        <v>0.6183999999999999</v>
+        <v>2.6341</v>
       </c>
       <c r="Y15" t="n">
-        <v>10.7428</v>
+        <v>17.3434</v>
       </c>
       <c r="Z15" t="n">
-        <v>26.2909</v>
+        <v>29.1506</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.0705</v>
+        <v>0.3889</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.858</v>
+        <v>7.4636</v>
       </c>
       <c r="AC15" t="n">
-        <v>6.7861</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>119.02</v>
+        <v>101.19</v>
       </c>
       <c r="C16" t="n">
-        <v>120.9</v>
+        <v>103.93</v>
       </c>
       <c r="D16" t="n">
-        <v>109</v>
+        <v>93.45</v>
       </c>
       <c r="E16" t="n">
-        <v>110.54</v>
+        <v>93.67</v>
       </c>
       <c r="F16" t="n">
-        <v>77</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>77.79000000000001</v>
+        <v>73.13</v>
       </c>
       <c r="H16" t="n">
-        <v>73.31</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>74.12</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>40.03</v>
+        <v>46.22</v>
       </c>
       <c r="K16" t="n">
-        <v>42.95</v>
+        <v>49.36</v>
       </c>
       <c r="L16" t="n">
-        <v>39.43</v>
+        <v>45.08</v>
       </c>
       <c r="M16" t="n">
-        <v>42.52</v>
+        <v>49.23</v>
       </c>
       <c r="N16" t="n">
-        <v>34.77</v>
+        <v>36.57</v>
       </c>
       <c r="O16" t="n">
-        <v>36.35</v>
+        <v>39.29</v>
       </c>
       <c r="P16" t="n">
-        <v>34.42</v>
+        <v>36.51</v>
       </c>
       <c r="Q16" t="n">
-        <v>36</v>
+        <v>38.9</v>
       </c>
       <c r="R16" t="n">
-        <v>-13.3495</v>
+        <v>-12.7434</v>
       </c>
       <c r="S16" t="n">
-        <v>-20.9073</v>
+        <v>-26.5736</v>
       </c>
       <c r="T16" t="n">
-        <v>-30.4386</v>
+        <v>-32.978</v>
       </c>
       <c r="U16" t="n">
-        <v>-5.951</v>
+        <v>-7.5996</v>
       </c>
       <c r="V16" t="n">
-        <v>-8.809100000000001</v>
+        <v>-13.4501</v>
       </c>
       <c r="W16" t="n">
-        <v>-11.3609</v>
+        <v>-16.0802</v>
       </c>
       <c r="X16" t="n">
-        <v>13.6291</v>
+        <v>12.8093</v>
       </c>
       <c r="Y16" t="n">
-        <v>23.6406</v>
+        <v>31.5607</v>
       </c>
       <c r="Z16" t="n">
-        <v>38.7276</v>
+        <v>43.1521</v>
       </c>
       <c r="AA16" t="n">
-        <v>5.9135</v>
+        <v>7.637</v>
       </c>
       <c r="AB16" t="n">
-        <v>9.256399999999999</v>
+        <v>14.4454</v>
       </c>
       <c r="AC16" t="n">
-        <v>12.2544</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>98.34999999999999</v>
+        <v>103.95</v>
       </c>
       <c r="C17" t="n">
-        <v>108.8</v>
+        <v>104.98</v>
       </c>
       <c r="D17" t="n">
-        <v>95.23</v>
+        <v>97.8</v>
       </c>
       <c r="E17" t="n">
-        <v>107.35</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>70.95</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>74.23999999999999</v>
+        <v>72.44</v>
       </c>
       <c r="H17" t="n">
-        <v>69.98999999999999</v>
+        <v>70.13</v>
       </c>
       <c r="I17" t="n">
-        <v>73.81999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J17" t="n">
-        <v>47.19</v>
+        <v>43.86</v>
       </c>
       <c r="K17" t="n">
-        <v>48.37</v>
+        <v>47.07</v>
       </c>
       <c r="L17" t="n">
-        <v>43.11</v>
+        <v>43.32</v>
       </c>
       <c r="M17" t="n">
-        <v>43.64</v>
+        <v>46.63</v>
       </c>
       <c r="N17" t="n">
-        <v>37.57</v>
+        <v>37.33</v>
       </c>
       <c r="O17" t="n">
-        <v>38.02</v>
+        <v>37.82</v>
       </c>
       <c r="P17" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.14</v>
+        <v>37.52</v>
       </c>
       <c r="R17" t="n">
-        <v>-2.8858</v>
+        <v>5.3165</v>
       </c>
       <c r="S17" t="n">
-        <v>-16.3941</v>
+        <v>-10.7563</v>
       </c>
       <c r="T17" t="n">
-        <v>-24.6772</v>
+        <v>-23.1698</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.4047</v>
+        <v>3.5625</v>
       </c>
       <c r="V17" t="n">
-        <v>-7.273</v>
+        <v>-4.6951</v>
       </c>
       <c r="W17" t="n">
-        <v>-7.9895</v>
+        <v>-11.2674</v>
       </c>
       <c r="X17" t="n">
-        <v>2.6341</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y17" t="n">
-        <v>17.3434</v>
+        <v>9.666</v>
       </c>
       <c r="Z17" t="n">
-        <v>29.1506</v>
+        <v>25.3832</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.3889</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB17" t="n">
-        <v>7.4636</v>
+        <v>4.2222</v>
       </c>
       <c r="AC17" t="n">
-        <v>8.3009</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>101.19</v>
+        <v>94.52</v>
       </c>
       <c r="C18" t="n">
-        <v>103.93</v>
+        <v>102.62</v>
       </c>
       <c r="D18" t="n">
-        <v>93.45</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>93.67</v>
+        <v>97.55</v>
       </c>
       <c r="F18" t="n">
-        <v>73.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>73.13</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>67.43000000000001</v>
+        <v>68.28</v>
       </c>
       <c r="I18" t="n">
-        <v>68.20999999999999</v>
+        <v>70.41</v>
       </c>
       <c r="J18" t="n">
-        <v>46.22</v>
+        <v>48.64</v>
       </c>
       <c r="K18" t="n">
-        <v>49.36</v>
+        <v>50.12</v>
       </c>
       <c r="L18" t="n">
-        <v>45.08</v>
+        <v>44.76</v>
       </c>
       <c r="M18" t="n">
-        <v>49.23</v>
+        <v>47.13</v>
       </c>
       <c r="N18" t="n">
-        <v>36.57</v>
+        <v>38.03</v>
       </c>
       <c r="O18" t="n">
-        <v>39.29</v>
+        <v>38.79</v>
       </c>
       <c r="P18" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.9</v>
+        <v>37.68</v>
       </c>
       <c r="R18" t="n">
-        <v>-12.7434</v>
+        <v>-1.1151</v>
       </c>
       <c r="S18" t="n">
-        <v>-26.5736</v>
+        <v>-9.129</v>
       </c>
       <c r="T18" t="n">
-        <v>-32.978</v>
+        <v>-23.5322</v>
       </c>
       <c r="U18" t="n">
-        <v>-7.5996</v>
+        <v>-0.3256</v>
       </c>
       <c r="V18" t="n">
-        <v>-13.4501</v>
+        <v>-4.6193</v>
       </c>
       <c r="W18" t="n">
-        <v>-16.0802</v>
+        <v>-10.6585</v>
       </c>
       <c r="X18" t="n">
-        <v>12.8093</v>
+        <v>1.0723</v>
       </c>
       <c r="Y18" t="n">
-        <v>31.5607</v>
+        <v>7.9973</v>
       </c>
       <c r="Z18" t="n">
-        <v>43.1521</v>
+        <v>25.9487</v>
       </c>
       <c r="AA18" t="n">
-        <v>7.637</v>
+        <v>0.4264</v>
       </c>
       <c r="AB18" t="n">
-        <v>14.4454</v>
+        <v>4.2612</v>
       </c>
       <c r="AC18" t="n">
-        <v>18.0577</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>103.95</v>
+        <v>102.86</v>
       </c>
       <c r="C19" t="n">
-        <v>104.98</v>
+        <v>106.13</v>
       </c>
       <c r="D19" t="n">
-        <v>97.8</v>
+        <v>99.31</v>
       </c>
       <c r="E19" t="n">
-        <v>98.65000000000001</v>
+        <v>103.24</v>
       </c>
       <c r="F19" t="n">
-        <v>71.01000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="G19" t="n">
-        <v>72.44</v>
+        <v>73.43000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>70.13</v>
+        <v>71.02</v>
       </c>
       <c r="I19" t="n">
-        <v>70.64</v>
+        <v>72.61</v>
       </c>
       <c r="J19" t="n">
-        <v>43.86</v>
+        <v>44.51</v>
       </c>
       <c r="K19" t="n">
-        <v>47.07</v>
+        <v>47.1</v>
       </c>
       <c r="L19" t="n">
-        <v>43.32</v>
+        <v>43.57</v>
       </c>
       <c r="M19" t="n">
-        <v>46.63</v>
+        <v>44.29</v>
       </c>
       <c r="N19" t="n">
-        <v>37.33</v>
+        <v>36.94</v>
       </c>
       <c r="O19" t="n">
-        <v>37.82</v>
+        <v>38.11</v>
       </c>
       <c r="P19" t="n">
-        <v>36.51</v>
+        <v>36.05</v>
       </c>
       <c r="Q19" t="n">
-        <v>37.52</v>
+        <v>36.48</v>
       </c>
       <c r="R19" t="n">
-        <v>5.3165</v>
+        <v>5.8329</v>
       </c>
       <c r="S19" t="n">
-        <v>-10.7563</v>
+        <v>10.2167</v>
       </c>
       <c r="T19" t="n">
-        <v>-23.1698</v>
+        <v>-6.6039</v>
       </c>
       <c r="U19" t="n">
-        <v>3.5625</v>
+        <v>3.1246</v>
       </c>
       <c r="V19" t="n">
-        <v>-4.6951</v>
+        <v>6.4507</v>
       </c>
       <c r="W19" t="n">
-        <v>-11.2674</v>
+        <v>-2.0372</v>
       </c>
       <c r="X19" t="n">
-        <v>-5.2813</v>
+        <v>-6.0259</v>
       </c>
       <c r="Y19" t="n">
-        <v>9.666</v>
+        <v>-10.0345</v>
       </c>
       <c r="Z19" t="n">
-        <v>25.3832</v>
+        <v>4.1627</v>
       </c>
       <c r="AA19" t="n">
-        <v>-3.5476</v>
+        <v>-3.1847</v>
       </c>
       <c r="AB19" t="n">
-        <v>4.2222</v>
+        <v>-6.2211</v>
       </c>
       <c r="AC19" t="n">
-        <v>11.5671</v>
+        <v>1.3333</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>94.52</v>
+        <v>90.59</v>
       </c>
       <c r="C20" t="n">
-        <v>102.62</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>91.34999999999999</v>
+        <v>80.22</v>
       </c>
       <c r="E20" t="n">
-        <v>97.55</v>
+        <v>82.11</v>
       </c>
       <c r="F20" t="n">
-        <v>69.70999999999999</v>
+        <v>69.14</v>
       </c>
       <c r="G20" t="n">
-        <v>71.93000000000001</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>68.28</v>
+        <v>65.61</v>
       </c>
       <c r="I20" t="n">
-        <v>70.41</v>
+        <v>66.42</v>
       </c>
       <c r="J20" t="n">
-        <v>48.64</v>
+        <v>49.82</v>
       </c>
       <c r="K20" t="n">
-        <v>50.12</v>
+        <v>54.31</v>
       </c>
       <c r="L20" t="n">
-        <v>44.76</v>
+        <v>48.62</v>
       </c>
       <c r="M20" t="n">
-        <v>47.13</v>
+        <v>53.45</v>
       </c>
       <c r="N20" t="n">
-        <v>38.03</v>
+        <v>38.23</v>
       </c>
       <c r="O20" t="n">
-        <v>38.79</v>
+        <v>40</v>
       </c>
       <c r="P20" t="n">
-        <v>36.85</v>
+        <v>37.96</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.68</v>
+        <v>39.6</v>
       </c>
       <c r="R20" t="n">
-        <v>-1.1151</v>
+        <v>-20.4669</v>
       </c>
       <c r="S20" t="n">
-        <v>-9.129</v>
+        <v>-16.7663</v>
       </c>
       <c r="T20" t="n">
-        <v>-23.5322</v>
+        <v>-23.5119</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.3256</v>
+        <v>-8.525</v>
       </c>
       <c r="V20" t="n">
-        <v>-4.6193</v>
+        <v>-5.974</v>
       </c>
       <c r="W20" t="n">
-        <v>-10.6585</v>
+        <v>-10.0244</v>
       </c>
       <c r="X20" t="n">
-        <v>1.0723</v>
+        <v>20.6819</v>
       </c>
       <c r="Y20" t="n">
-        <v>7.9973</v>
+        <v>14.6258</v>
       </c>
       <c r="Z20" t="n">
-        <v>25.9487</v>
+        <v>22.4794</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.4264</v>
+        <v>8.5526</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.2612</v>
+        <v>5.5437</v>
       </c>
       <c r="AC20" t="n">
-        <v>10.8561</v>
+        <v>9.5739</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>102.86</v>
+        <v>81.64</v>
       </c>
       <c r="C21" t="n">
-        <v>106.13</v>
+        <v>87.61</v>
       </c>
       <c r="D21" t="n">
-        <v>99.31</v>
+        <v>80.83</v>
       </c>
       <c r="E21" t="n">
-        <v>103.24</v>
+        <v>83.56</v>
       </c>
       <c r="F21" t="n">
-        <v>71.72</v>
+        <v>65.66</v>
       </c>
       <c r="G21" t="n">
-        <v>73.43000000000001</v>
+        <v>67.67</v>
       </c>
       <c r="H21" t="n">
-        <v>71.02</v>
+        <v>65.37</v>
       </c>
       <c r="I21" t="n">
-        <v>72.61</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>44.51</v>
+        <v>53.77</v>
       </c>
       <c r="K21" t="n">
-        <v>47.1</v>
+        <v>54.38</v>
       </c>
       <c r="L21" t="n">
-        <v>43.57</v>
+        <v>50.27</v>
       </c>
       <c r="M21" t="n">
-        <v>44.29</v>
+        <v>52.46</v>
       </c>
       <c r="N21" t="n">
-        <v>36.94</v>
+        <v>40.07</v>
       </c>
       <c r="O21" t="n">
-        <v>38.11</v>
+        <v>40.23</v>
       </c>
       <c r="P21" t="n">
-        <v>36.05</v>
+        <v>38.86</v>
       </c>
       <c r="Q21" t="n">
-        <v>36.48</v>
+        <v>39.68</v>
       </c>
       <c r="R21" t="n">
-        <v>5.8329</v>
+        <v>1.7659</v>
       </c>
       <c r="S21" t="n">
-        <v>10.2167</v>
+        <v>-14.3414</v>
       </c>
       <c r="T21" t="n">
-        <v>-6.6039</v>
+        <v>-10.7932</v>
       </c>
       <c r="U21" t="n">
-        <v>3.1246</v>
+        <v>-0.1957</v>
       </c>
       <c r="V21" t="n">
-        <v>6.4507</v>
+        <v>-5.8514</v>
       </c>
       <c r="W21" t="n">
-        <v>-2.0372</v>
+        <v>-2.8148</v>
       </c>
       <c r="X21" t="n">
-        <v>-6.0259</v>
+        <v>-1.8522</v>
       </c>
       <c r="Y21" t="n">
-        <v>-10.0345</v>
+        <v>11.3091</v>
       </c>
       <c r="Z21" t="n">
-        <v>4.1627</v>
+        <v>6.561</v>
       </c>
       <c r="AA21" t="n">
-        <v>-3.1847</v>
+        <v>0.202</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.2211</v>
+        <v>5.3079</v>
       </c>
       <c r="AC21" t="n">
-        <v>1.3333</v>
+        <v>2.0051</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>90.59</v>
-      </c>
-      <c r="C22" t="n">
-        <v>93.40000000000001</v>
-      </c>
-      <c r="D22" t="n">
-        <v>80.22</v>
-      </c>
-      <c r="E22" t="n">
-        <v>82.11</v>
-      </c>
-      <c r="F22" t="n">
-        <v>69.14</v>
-      </c>
-      <c r="G22" t="n">
-        <v>69.65000000000001</v>
-      </c>
-      <c r="H22" t="n">
-        <v>65.61</v>
-      </c>
-      <c r="I22" t="n">
-        <v>66.42</v>
-      </c>
-      <c r="J22" t="n">
-        <v>49.82</v>
-      </c>
-      <c r="K22" t="n">
-        <v>54.31</v>
-      </c>
-      <c r="L22" t="n">
-        <v>48.62</v>
-      </c>
-      <c r="M22" t="n">
-        <v>53.45</v>
-      </c>
-      <c r="N22" t="n">
-        <v>38.23</v>
-      </c>
-      <c r="O22" t="n">
-        <v>40</v>
-      </c>
-      <c r="P22" t="n">
-        <v>37.96</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="R22" t="n">
-        <v>-20.4669</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-16.7663</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-23.5119</v>
-      </c>
-      <c r="U22" t="n">
-        <v>-8.525</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-5.974</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-10.0244</v>
-      </c>
-      <c r="X22" t="n">
-        <v>20.6819</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>14.6258</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>22.4794</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>8.5526</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>5.5437</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>9.5739</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2328,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-28 00:59
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2281,6 +2281,97 @@
       <c r="A22" t="inlineStr">
         <is>
           <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>85.88</v>
+      </c>
+      <c r="C22" t="n">
+        <v>93.15000000000001</v>
+      </c>
+      <c r="D22" t="n">
+        <v>84.22</v>
+      </c>
+      <c r="E22" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>67.02</v>
+      </c>
+      <c r="G22" t="n">
+        <v>69.33</v>
+      </c>
+      <c r="H22" t="n">
+        <v>66.61</v>
+      </c>
+      <c r="I22" t="n">
+        <v>68.43000000000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>51.03</v>
+      </c>
+      <c r="K22" t="n">
+        <v>52.09</v>
+      </c>
+      <c r="L22" t="n">
+        <v>46.47</v>
+      </c>
+      <c r="M22" t="n">
+        <v>47.98</v>
+      </c>
+      <c r="N22" t="n">
+        <v>39.23</v>
+      </c>
+      <c r="O22" t="n">
+        <v>39.51</v>
+      </c>
+      <c r="P22" t="n">
+        <v>37.86</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="R22" t="n">
+        <v>8.305400000000001</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-12.3402</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-8.2615</v>
+      </c>
+      <c r="U22" t="n">
+        <v>3.2282</v>
+      </c>
+      <c r="V22" t="n">
+        <v>-5.7568</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-3.1285</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-8.5398</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>8.3315</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>2.8951</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-3.2762</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>5.2083</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>2.2921</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2419,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-29 01:35
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1811 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>148.14</v>
+        <v>148.94</v>
       </c>
       <c r="C2" t="n">
-        <v>149.99</v>
+        <v>152.37</v>
       </c>
       <c r="D2" t="n">
-        <v>135.21</v>
+        <v>145.49</v>
       </c>
       <c r="E2" t="n">
-        <v>142.29</v>
+        <v>147</v>
       </c>
       <c r="F2" t="n">
-        <v>78.29000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="G2" t="n">
-        <v>78.59999999999999</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>75.47</v>
+        <v>76.62</v>
       </c>
       <c r="I2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="K2" t="n">
-        <v>35.95</v>
+        <v>33.64</v>
       </c>
       <c r="L2" t="n">
-        <v>32.77</v>
+        <v>31.96</v>
       </c>
       <c r="M2" t="n">
-        <v>34.43</v>
+        <v>33.26</v>
       </c>
       <c r="N2" t="n">
-        <v>34.31</v>
+        <v>34.34</v>
       </c>
       <c r="O2" t="n">
-        <v>35.53</v>
+        <v>35.02</v>
       </c>
       <c r="P2" t="n">
-        <v>34.17</v>
+        <v>34.28</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.83</v>
+        <v>34.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C3" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D3" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E3" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F3" t="n">
         <v>78.13</v>
       </c>
       <c r="G3" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I3" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J3" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K3" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L3" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M3" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N3" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O3" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P3" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q3" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
       <c r="R3" t="n">
-        <v>3.3101</v>
+        <v>0.585</v>
       </c>
       <c r="U3" t="n">
-        <v>0.5452</v>
+        <v>0.7359</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.3982</v>
+        <v>-0.5412</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.4881</v>
+        <v>-0.7213000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C4" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D4" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E4" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F4" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G4" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H4" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I4" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J4" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K4" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L4" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M4" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N4" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O4" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P4" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R4" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="U4" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C5" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D5" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E5" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F5" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G5" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H5" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I5" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K5" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L5" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M5" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N5" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O5" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P5" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q5" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R5" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="S5" t="n">
-        <v>8.011799999999999</v>
+        <v>11.3673</v>
       </c>
       <c r="U5" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="V5" t="n">
-        <v>2.1937</v>
+        <v>4.583</v>
       </c>
       <c r="X5" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="Y5" t="n">
-        <v>-7.7549</v>
+        <v>-10.6735</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
       <c r="AB5" t="n">
-        <v>-2.0672</v>
+        <v>-4.4432</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C6" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D6" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E6" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F6" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G6" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H6" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J6" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K6" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L6" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M6" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N6" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O6" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P6" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q6" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R6" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S6" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="U6" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V6" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="X6" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y6" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="AA6" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB6" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C7" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D7" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E7" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F7" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I7" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J7" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K7" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L7" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M7" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N7" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O7" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P7" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q7" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R7" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S7" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="T7" t="n">
-        <v>15.4473</v>
+        <v>11.7415</v>
       </c>
       <c r="U7" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V7" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="W7" t="n">
-        <v>7.892</v>
+        <v>8.7658</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y7" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="Z7" t="n">
-        <v>-13.9704</v>
+        <v>-10.914</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB7" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
       <c r="AC7" t="n">
-        <v>-7.4074</v>
+        <v>-8.164999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C8" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D8" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E8" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F8" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H8" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J8" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K8" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L8" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M8" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N8" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O8" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P8" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q8" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R8" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S8" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T8" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U8" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V8" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W8" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X8" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y8" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z8" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC8" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C9" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D9" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E9" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F9" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G9" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I9" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J9" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K9" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L9" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M9" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N9" t="n">
         <v>32.58</v>
       </c>
       <c r="O9" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P9" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q9" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R9" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S9" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T9" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V9" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W9" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X9" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y9" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z9" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC9" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C10" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D10" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E10" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F10" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G10" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H10" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I10" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J10" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K10" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L10" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M10" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N10" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O10" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P10" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q10" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R10" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S10" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T10" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U10" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V10" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W10" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X10" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y10" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z10" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA10" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB10" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC10" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C11" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D11" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E11" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F11" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G11" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H11" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I11" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J11" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K11" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L11" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M11" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N11" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O11" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P11" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q11" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R11" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S11" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T11" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U11" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V11" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W11" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X11" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y11" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z11" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC11" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C12" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D12" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E12" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F12" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H12" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I12" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J12" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K12" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L12" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M12" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N12" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O12" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P12" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q12" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R12" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S12" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T12" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U12" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V12" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W12" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X12" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y12" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z12" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA12" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB12" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC12" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C13" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D13" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E13" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F13" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G13" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I13" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J13" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K13" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L13" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M13" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N13" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O13" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P13" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q13" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R13" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S13" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T13" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W13" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X13" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y13" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z13" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC13" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C14" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D14" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E14" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F14" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G14" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K14" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L14" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M14" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N14" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O14" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P14" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q14" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R14" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S14" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T14" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U14" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V14" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W14" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X14" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y14" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z14" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA14" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB14" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC14" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>98.34999999999999</v>
+        <v>101.19</v>
       </c>
       <c r="C15" t="n">
-        <v>108.8</v>
+        <v>103.93</v>
       </c>
       <c r="D15" t="n">
-        <v>95.23</v>
+        <v>93.45</v>
       </c>
       <c r="E15" t="n">
-        <v>107.35</v>
+        <v>93.67</v>
       </c>
       <c r="F15" t="n">
-        <v>70.95</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>74.23999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="H15" t="n">
-        <v>69.98999999999999</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>73.81999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>47.19</v>
+        <v>46.22</v>
       </c>
       <c r="K15" t="n">
-        <v>48.37</v>
+        <v>49.36</v>
       </c>
       <c r="L15" t="n">
-        <v>43.11</v>
+        <v>45.08</v>
       </c>
       <c r="M15" t="n">
-        <v>43.64</v>
+        <v>49.23</v>
       </c>
       <c r="N15" t="n">
-        <v>37.57</v>
+        <v>36.57</v>
       </c>
       <c r="O15" t="n">
-        <v>38.02</v>
+        <v>39.29</v>
       </c>
       <c r="P15" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q15" t="n">
-        <v>36.14</v>
+        <v>38.9</v>
       </c>
       <c r="R15" t="n">
-        <v>-2.8858</v>
+        <v>-12.7434</v>
       </c>
       <c r="S15" t="n">
-        <v>-16.3941</v>
+        <v>-26.5736</v>
       </c>
       <c r="T15" t="n">
-        <v>-24.6772</v>
+        <v>-32.978</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.4047</v>
+        <v>-7.5996</v>
       </c>
       <c r="V15" t="n">
-        <v>-7.273</v>
+        <v>-13.4501</v>
       </c>
       <c r="W15" t="n">
-        <v>-7.9895</v>
+        <v>-16.0802</v>
       </c>
       <c r="X15" t="n">
-        <v>2.6341</v>
+        <v>12.8093</v>
       </c>
       <c r="Y15" t="n">
-        <v>17.3434</v>
+        <v>31.5607</v>
       </c>
       <c r="Z15" t="n">
-        <v>29.1506</v>
+        <v>43.1521</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.3889</v>
+        <v>7.637</v>
       </c>
       <c r="AB15" t="n">
-        <v>7.4636</v>
+        <v>14.4454</v>
       </c>
       <c r="AC15" t="n">
-        <v>8.3009</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>101.19</v>
+        <v>103.95</v>
       </c>
       <c r="C16" t="n">
-        <v>103.93</v>
+        <v>104.98</v>
       </c>
       <c r="D16" t="n">
-        <v>93.45</v>
+        <v>97.8</v>
       </c>
       <c r="E16" t="n">
-        <v>93.67</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>73.01000000000001</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>73.13</v>
+        <v>72.44</v>
       </c>
       <c r="H16" t="n">
-        <v>67.43000000000001</v>
+        <v>70.13</v>
       </c>
       <c r="I16" t="n">
-        <v>68.20999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J16" t="n">
-        <v>46.22</v>
+        <v>43.86</v>
       </c>
       <c r="K16" t="n">
-        <v>49.36</v>
+        <v>47.07</v>
       </c>
       <c r="L16" t="n">
-        <v>45.08</v>
+        <v>43.32</v>
       </c>
       <c r="M16" t="n">
-        <v>49.23</v>
+        <v>46.63</v>
       </c>
       <c r="N16" t="n">
-        <v>36.57</v>
+        <v>37.33</v>
       </c>
       <c r="O16" t="n">
-        <v>39.29</v>
+        <v>37.82</v>
       </c>
       <c r="P16" t="n">
         <v>36.51</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.9</v>
+        <v>37.52</v>
       </c>
       <c r="R16" t="n">
-        <v>-12.7434</v>
+        <v>5.3165</v>
       </c>
       <c r="S16" t="n">
-        <v>-26.5736</v>
+        <v>-10.7563</v>
       </c>
       <c r="T16" t="n">
-        <v>-32.978</v>
+        <v>-23.1698</v>
       </c>
       <c r="U16" t="n">
-        <v>-7.5996</v>
+        <v>3.5625</v>
       </c>
       <c r="V16" t="n">
-        <v>-13.4501</v>
+        <v>-4.6951</v>
       </c>
       <c r="W16" t="n">
-        <v>-16.0802</v>
+        <v>-11.2674</v>
       </c>
       <c r="X16" t="n">
-        <v>12.8093</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y16" t="n">
-        <v>31.5607</v>
+        <v>9.666</v>
       </c>
       <c r="Z16" t="n">
-        <v>43.1521</v>
+        <v>25.3832</v>
       </c>
       <c r="AA16" t="n">
-        <v>7.637</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB16" t="n">
-        <v>14.4454</v>
+        <v>4.2222</v>
       </c>
       <c r="AC16" t="n">
-        <v>18.0577</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>103.95</v>
+        <v>94.52</v>
       </c>
       <c r="C17" t="n">
-        <v>104.98</v>
+        <v>102.62</v>
       </c>
       <c r="D17" t="n">
-        <v>97.8</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>98.65000000000001</v>
+        <v>97.55</v>
       </c>
       <c r="F17" t="n">
-        <v>71.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>72.44</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>70.13</v>
+        <v>68.28</v>
       </c>
       <c r="I17" t="n">
-        <v>70.64</v>
+        <v>70.41</v>
       </c>
       <c r="J17" t="n">
-        <v>43.86</v>
+        <v>48.64</v>
       </c>
       <c r="K17" t="n">
-        <v>47.07</v>
+        <v>50.12</v>
       </c>
       <c r="L17" t="n">
-        <v>43.32</v>
+        <v>44.76</v>
       </c>
       <c r="M17" t="n">
-        <v>46.63</v>
+        <v>47.13</v>
       </c>
       <c r="N17" t="n">
-        <v>37.33</v>
+        <v>38.03</v>
       </c>
       <c r="O17" t="n">
-        <v>37.82</v>
+        <v>38.79</v>
       </c>
       <c r="P17" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.52</v>
+        <v>37.68</v>
       </c>
       <c r="R17" t="n">
-        <v>5.3165</v>
+        <v>-1.1151</v>
       </c>
       <c r="S17" t="n">
-        <v>-10.7563</v>
+        <v>-9.129</v>
       </c>
       <c r="T17" t="n">
-        <v>-23.1698</v>
+        <v>-23.5322</v>
       </c>
       <c r="U17" t="n">
-        <v>3.5625</v>
+        <v>-0.3256</v>
       </c>
       <c r="V17" t="n">
-        <v>-4.6951</v>
+        <v>-4.6193</v>
       </c>
       <c r="W17" t="n">
-        <v>-11.2674</v>
+        <v>-10.6585</v>
       </c>
       <c r="X17" t="n">
-        <v>-5.2813</v>
+        <v>1.0723</v>
       </c>
       <c r="Y17" t="n">
-        <v>9.666</v>
+        <v>7.9973</v>
       </c>
       <c r="Z17" t="n">
-        <v>25.3832</v>
+        <v>25.9487</v>
       </c>
       <c r="AA17" t="n">
-        <v>-3.5476</v>
+        <v>0.4264</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.2222</v>
+        <v>4.2612</v>
       </c>
       <c r="AC17" t="n">
-        <v>11.5671</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>94.52</v>
+        <v>102.86</v>
       </c>
       <c r="C18" t="n">
-        <v>102.62</v>
+        <v>106.13</v>
       </c>
       <c r="D18" t="n">
-        <v>91.34999999999999</v>
+        <v>99.31</v>
       </c>
       <c r="E18" t="n">
-        <v>97.55</v>
+        <v>103.24</v>
       </c>
       <c r="F18" t="n">
-        <v>69.70999999999999</v>
+        <v>71.72</v>
       </c>
       <c r="G18" t="n">
-        <v>71.93000000000001</v>
+        <v>73.43000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>68.28</v>
+        <v>71.02</v>
       </c>
       <c r="I18" t="n">
-        <v>70.41</v>
+        <v>72.61</v>
       </c>
       <c r="J18" t="n">
-        <v>48.64</v>
+        <v>44.51</v>
       </c>
       <c r="K18" t="n">
-        <v>50.12</v>
+        <v>47.1</v>
       </c>
       <c r="L18" t="n">
-        <v>44.76</v>
+        <v>43.57</v>
       </c>
       <c r="M18" t="n">
-        <v>47.13</v>
+        <v>44.29</v>
       </c>
       <c r="N18" t="n">
-        <v>38.03</v>
+        <v>36.94</v>
       </c>
       <c r="O18" t="n">
-        <v>38.79</v>
+        <v>38.11</v>
       </c>
       <c r="P18" t="n">
-        <v>36.85</v>
+        <v>36.05</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.68</v>
+        <v>36.48</v>
       </c>
       <c r="R18" t="n">
-        <v>-1.1151</v>
+        <v>5.8329</v>
       </c>
       <c r="S18" t="n">
-        <v>-9.129</v>
+        <v>10.2167</v>
       </c>
       <c r="T18" t="n">
-        <v>-23.5322</v>
+        <v>-6.6039</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.3256</v>
+        <v>3.1246</v>
       </c>
       <c r="V18" t="n">
-        <v>-4.6193</v>
+        <v>6.4507</v>
       </c>
       <c r="W18" t="n">
-        <v>-10.6585</v>
+        <v>-2.0372</v>
       </c>
       <c r="X18" t="n">
-        <v>1.0723</v>
+        <v>-6.0259</v>
       </c>
       <c r="Y18" t="n">
-        <v>7.9973</v>
+        <v>-10.0345</v>
       </c>
       <c r="Z18" t="n">
-        <v>25.9487</v>
+        <v>4.1627</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.4264</v>
+        <v>-3.1847</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.2612</v>
+        <v>-6.2211</v>
       </c>
       <c r="AC18" t="n">
-        <v>10.8561</v>
+        <v>1.3333</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>102.86</v>
+        <v>90.59</v>
       </c>
       <c r="C19" t="n">
-        <v>106.13</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>99.31</v>
+        <v>80.22</v>
       </c>
       <c r="E19" t="n">
-        <v>103.24</v>
+        <v>82.11</v>
       </c>
       <c r="F19" t="n">
-        <v>71.72</v>
+        <v>69.14</v>
       </c>
       <c r="G19" t="n">
-        <v>73.43000000000001</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>71.02</v>
+        <v>65.61</v>
       </c>
       <c r="I19" t="n">
-        <v>72.61</v>
+        <v>66.42</v>
       </c>
       <c r="J19" t="n">
-        <v>44.51</v>
+        <v>49.82</v>
       </c>
       <c r="K19" t="n">
-        <v>47.1</v>
+        <v>54.31</v>
       </c>
       <c r="L19" t="n">
-        <v>43.57</v>
+        <v>48.62</v>
       </c>
       <c r="M19" t="n">
-        <v>44.29</v>
+        <v>53.45</v>
       </c>
       <c r="N19" t="n">
-        <v>36.94</v>
+        <v>38.23</v>
       </c>
       <c r="O19" t="n">
-        <v>38.11</v>
+        <v>40</v>
       </c>
       <c r="P19" t="n">
-        <v>36.05</v>
+        <v>37.96</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.48</v>
+        <v>39.6</v>
       </c>
       <c r="R19" t="n">
-        <v>5.8329</v>
+        <v>-20.4669</v>
       </c>
       <c r="S19" t="n">
-        <v>10.2167</v>
+        <v>-16.7663</v>
       </c>
       <c r="T19" t="n">
-        <v>-6.6039</v>
+        <v>-23.5119</v>
       </c>
       <c r="U19" t="n">
-        <v>3.1246</v>
+        <v>-8.525</v>
       </c>
       <c r="V19" t="n">
-        <v>6.4507</v>
+        <v>-5.974</v>
       </c>
       <c r="W19" t="n">
-        <v>-2.0372</v>
+        <v>-10.0244</v>
       </c>
       <c r="X19" t="n">
-        <v>-6.0259</v>
+        <v>20.6819</v>
       </c>
       <c r="Y19" t="n">
-        <v>-10.0345</v>
+        <v>14.6258</v>
       </c>
       <c r="Z19" t="n">
-        <v>4.1627</v>
+        <v>22.4794</v>
       </c>
       <c r="AA19" t="n">
-        <v>-3.1847</v>
+        <v>8.5526</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.2211</v>
+        <v>5.5437</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.3333</v>
+        <v>9.5739</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>90.59</v>
+        <v>81.64</v>
       </c>
       <c r="C20" t="n">
-        <v>93.40000000000001</v>
+        <v>87.61</v>
       </c>
       <c r="D20" t="n">
-        <v>80.22</v>
+        <v>80.83</v>
       </c>
       <c r="E20" t="n">
-        <v>82.11</v>
+        <v>83.56</v>
       </c>
       <c r="F20" t="n">
-        <v>69.14</v>
+        <v>65.66</v>
       </c>
       <c r="G20" t="n">
-        <v>69.65000000000001</v>
+        <v>67.67</v>
       </c>
       <c r="H20" t="n">
-        <v>65.61</v>
+        <v>65.37</v>
       </c>
       <c r="I20" t="n">
-        <v>66.42</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>49.82</v>
+        <v>53.77</v>
       </c>
       <c r="K20" t="n">
-        <v>54.31</v>
+        <v>54.38</v>
       </c>
       <c r="L20" t="n">
-        <v>48.62</v>
+        <v>50.27</v>
       </c>
       <c r="M20" t="n">
-        <v>53.45</v>
+        <v>52.46</v>
       </c>
       <c r="N20" t="n">
-        <v>38.23</v>
+        <v>40.07</v>
       </c>
       <c r="O20" t="n">
-        <v>40</v>
+        <v>40.23</v>
       </c>
       <c r="P20" t="n">
-        <v>37.96</v>
+        <v>38.86</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.6</v>
+        <v>39.68</v>
       </c>
       <c r="R20" t="n">
-        <v>-20.4669</v>
+        <v>1.7659</v>
       </c>
       <c r="S20" t="n">
-        <v>-16.7663</v>
+        <v>-14.3414</v>
       </c>
       <c r="T20" t="n">
-        <v>-23.5119</v>
+        <v>-10.7932</v>
       </c>
       <c r="U20" t="n">
-        <v>-8.525</v>
+        <v>-0.1957</v>
       </c>
       <c r="V20" t="n">
-        <v>-5.974</v>
+        <v>-5.8514</v>
       </c>
       <c r="W20" t="n">
-        <v>-10.0244</v>
+        <v>-2.8148</v>
       </c>
       <c r="X20" t="n">
-        <v>20.6819</v>
+        <v>-1.8522</v>
       </c>
       <c r="Y20" t="n">
-        <v>14.6258</v>
+        <v>11.3091</v>
       </c>
       <c r="Z20" t="n">
-        <v>22.4794</v>
+        <v>6.561</v>
       </c>
       <c r="AA20" t="n">
-        <v>8.5526</v>
+        <v>0.202</v>
       </c>
       <c r="AB20" t="n">
-        <v>5.5437</v>
+        <v>5.3079</v>
       </c>
       <c r="AC20" t="n">
-        <v>9.5739</v>
+        <v>2.0051</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>81.64</v>
+        <v>85.88</v>
       </c>
       <c r="C21" t="n">
-        <v>87.61</v>
+        <v>93.15000000000001</v>
       </c>
       <c r="D21" t="n">
-        <v>80.83</v>
+        <v>84.22</v>
       </c>
       <c r="E21" t="n">
-        <v>83.56</v>
+        <v>90.5</v>
       </c>
       <c r="F21" t="n">
-        <v>65.66</v>
+        <v>67.02</v>
       </c>
       <c r="G21" t="n">
-        <v>67.67</v>
+        <v>69.33</v>
       </c>
       <c r="H21" t="n">
-        <v>65.37</v>
+        <v>66.61</v>
       </c>
       <c r="I21" t="n">
-        <v>66.29000000000001</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>53.77</v>
+        <v>51.03</v>
       </c>
       <c r="K21" t="n">
-        <v>54.38</v>
+        <v>52.09</v>
       </c>
       <c r="L21" t="n">
-        <v>50.27</v>
+        <v>46.47</v>
       </c>
       <c r="M21" t="n">
-        <v>52.46</v>
+        <v>47.98</v>
       </c>
       <c r="N21" t="n">
-        <v>40.07</v>
+        <v>39.23</v>
       </c>
       <c r="O21" t="n">
-        <v>40.23</v>
+        <v>39.51</v>
       </c>
       <c r="P21" t="n">
-        <v>38.86</v>
+        <v>37.86</v>
       </c>
       <c r="Q21" t="n">
-        <v>39.68</v>
+        <v>38.38</v>
       </c>
       <c r="R21" t="n">
-        <v>1.7659</v>
+        <v>8.305400000000001</v>
       </c>
       <c r="S21" t="n">
-        <v>-14.3414</v>
+        <v>-12.3402</v>
       </c>
       <c r="T21" t="n">
-        <v>-10.7932</v>
+        <v>-8.2615</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.1957</v>
+        <v>3.2282</v>
       </c>
       <c r="V21" t="n">
-        <v>-5.8514</v>
+        <v>-5.7568</v>
       </c>
       <c r="W21" t="n">
-        <v>-2.8148</v>
+        <v>-3.1285</v>
       </c>
       <c r="X21" t="n">
-        <v>-1.8522</v>
+        <v>-8.5398</v>
       </c>
       <c r="Y21" t="n">
-        <v>11.3091</v>
+        <v>8.3315</v>
       </c>
       <c r="Z21" t="n">
-        <v>6.561</v>
+        <v>2.8951</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.202</v>
+        <v>-3.2762</v>
       </c>
       <c r="AB21" t="n">
-        <v>5.3079</v>
+        <v>5.2083</v>
       </c>
       <c r="AC21" t="n">
-        <v>2.0051</v>
+        <v>2.2921</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>85.88</v>
+        <v>95.04000000000001</v>
       </c>
       <c r="C22" t="n">
-        <v>93.15000000000001</v>
+        <v>102.2</v>
       </c>
       <c r="D22" t="n">
-        <v>84.22</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>90.5</v>
+        <v>101.08</v>
       </c>
       <c r="F22" t="n">
-        <v>67.02</v>
+        <v>69.3</v>
       </c>
       <c r="G22" t="n">
-        <v>69.33</v>
+        <v>71.53</v>
       </c>
       <c r="H22" t="n">
-        <v>66.61</v>
+        <v>68.86</v>
       </c>
       <c r="I22" t="n">
-        <v>68.43000000000001</v>
+        <v>71.04000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>51.03</v>
+        <v>45.8</v>
       </c>
       <c r="K22" t="n">
-        <v>52.09</v>
+        <v>46.21</v>
       </c>
       <c r="L22" t="n">
-        <v>46.47</v>
+        <v>41.9</v>
       </c>
       <c r="M22" t="n">
-        <v>47.98</v>
+        <v>42.5</v>
       </c>
       <c r="N22" t="n">
-        <v>39.23</v>
+        <v>37.93</v>
       </c>
       <c r="O22" t="n">
-        <v>39.51</v>
+        <v>38.17</v>
       </c>
       <c r="P22" t="n">
-        <v>37.86</v>
+        <v>36.67</v>
       </c>
       <c r="Q22" t="n">
-        <v>38.38</v>
+        <v>36.93</v>
       </c>
       <c r="R22" t="n">
-        <v>8.305400000000001</v>
+        <v>11.6906</v>
       </c>
       <c r="S22" t="n">
-        <v>-12.3402</v>
+        <v>23.1032</v>
       </c>
       <c r="T22" t="n">
-        <v>-8.2615</v>
+        <v>3.6187</v>
       </c>
       <c r="U22" t="n">
-        <v>3.2282</v>
+        <v>3.8141</v>
       </c>
       <c r="V22" t="n">
-        <v>-5.7568</v>
+        <v>6.9557</v>
       </c>
       <c r="W22" t="n">
-        <v>-3.1285</v>
+        <v>0.8948</v>
       </c>
       <c r="X22" t="n">
-        <v>-8.5398</v>
+        <v>-11.4214</v>
       </c>
       <c r="Y22" t="n">
-        <v>8.3315</v>
+        <v>-20.4864</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.8951</v>
+        <v>-9.8239</v>
       </c>
       <c r="AA22" t="n">
-        <v>-3.2762</v>
+        <v>-3.778</v>
       </c>
       <c r="AB22" t="n">
-        <v>5.2083</v>
+        <v>-6.7424</v>
       </c>
       <c r="AC22" t="n">
-        <v>2.2921</v>
+        <v>-1.9904</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
-        </is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>103.97</v>
+      </c>
+      <c r="C23" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>101.32</v>
+      </c>
+      <c r="E23" t="n">
+        <v>107.35</v>
+      </c>
+      <c r="F23" t="n">
+        <v>71.91</v>
+      </c>
+      <c r="G23" t="n">
+        <v>72.53</v>
+      </c>
+      <c r="H23" t="n">
+        <v>70.76000000000001</v>
+      </c>
+      <c r="I23" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="J23" t="n">
+        <v>41.33</v>
+      </c>
+      <c r="K23" t="n">
+        <v>42.41</v>
+      </c>
+      <c r="L23" t="n">
+        <v>39.33</v>
+      </c>
+      <c r="M23" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="N23" t="n">
+        <v>36.51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>37.09</v>
+      </c>
+      <c r="P23" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>36.28</v>
+      </c>
+      <c r="R23" t="n">
+        <v>6.203</v>
+      </c>
+      <c r="S23" t="n">
+        <v>28.4706</v>
+      </c>
+      <c r="T23" t="n">
+        <v>3.981</v>
+      </c>
+      <c r="U23" t="n">
+        <v>1.8581</v>
+      </c>
+      <c r="V23" t="n">
+        <v>9.156700000000001</v>
+      </c>
+      <c r="W23" t="n">
+        <v>-0.3443</v>
+      </c>
+      <c r="X23" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>-24.1708</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>-10.1829</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>-1.7601</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>-8.5685</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>-0.5482</v>
       </c>
     </row>
   </sheetData>
@@ -2419,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-30 01:35
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>148.94</v>
+        <v>147.95</v>
       </c>
       <c r="C2" t="n">
-        <v>152.37</v>
+        <v>150.77</v>
       </c>
       <c r="D2" t="n">
-        <v>145.49</v>
+        <v>144.41</v>
       </c>
       <c r="E2" t="n">
-        <v>147</v>
+        <v>147.86</v>
       </c>
       <c r="F2" t="n">
         <v>78.13</v>
       </c>
       <c r="G2" t="n">
-        <v>78.26000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>76.62</v>
+        <v>77.94</v>
       </c>
       <c r="I2" t="n">
-        <v>77.45999999999999</v>
+        <v>78.03</v>
       </c>
       <c r="J2" t="n">
-        <v>32.82</v>
+        <v>33.07</v>
       </c>
       <c r="K2" t="n">
-        <v>33.64</v>
+        <v>33.86</v>
       </c>
       <c r="L2" t="n">
-        <v>31.96</v>
+        <v>32.42</v>
       </c>
       <c r="M2" t="n">
-        <v>33.26</v>
+        <v>33.08</v>
       </c>
       <c r="N2" t="n">
-        <v>34.34</v>
+        <v>34.36</v>
       </c>
       <c r="O2" t="n">
-        <v>35.02</v>
+        <v>34.44</v>
       </c>
       <c r="P2" t="n">
-        <v>34.28</v>
+        <v>33.66</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.66</v>
+        <v>34.41</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C3" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D3" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E3" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F3" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G3" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H3" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I3" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J3" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K3" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L3" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M3" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N3" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O3" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P3" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q3" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
       <c r="R3" t="n">
-        <v>0.585</v>
+        <v>3.9429</v>
       </c>
       <c r="U3" t="n">
-        <v>0.7359</v>
+        <v>0.8971</v>
       </c>
       <c r="X3" t="n">
-        <v>-0.5412</v>
+        <v>-3.9903</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.7213000000000001</v>
+        <v>-0.8718</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C4" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D4" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E4" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F4" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G4" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H4" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I4" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K4" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L4" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M4" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N4" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O4" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P4" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R4" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="U4" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="X4" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C5" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D5" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E5" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F5" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G5" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H5" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J5" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K5" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L5" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M5" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N5" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O5" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P5" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q5" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R5" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="S5" t="n">
-        <v>11.3673</v>
+        <v>11.0983</v>
       </c>
       <c r="U5" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="V5" t="n">
-        <v>4.583</v>
+        <v>6.5231</v>
       </c>
       <c r="X5" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="Y5" t="n">
-        <v>-10.6735</v>
+        <v>-10.4595</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
       <c r="AB5" t="n">
-        <v>-4.4432</v>
+        <v>-6.2772</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C6" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D6" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E6" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F6" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I6" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J6" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K6" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L6" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M6" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N6" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O6" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P6" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q6" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R6" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S6" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="U6" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V6" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y6" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="AA6" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C7" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D7" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E7" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F7" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H7" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J7" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K7" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L7" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M7" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N7" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O7" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P7" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q7" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R7" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S7" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="T7" t="n">
-        <v>11.7415</v>
+        <v>7.4733</v>
       </c>
       <c r="U7" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V7" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="W7" t="n">
-        <v>8.7658</v>
+        <v>7.1639</v>
       </c>
       <c r="X7" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y7" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="Z7" t="n">
-        <v>-10.914</v>
+        <v>-7.3458</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB7" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
       <c r="AC7" t="n">
-        <v>-8.164999999999999</v>
+        <v>-6.8003</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C8" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D8" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E8" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F8" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G8" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I8" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J8" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K8" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L8" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M8" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N8" t="n">
         <v>32.58</v>
       </c>
       <c r="O8" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P8" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q8" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R8" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S8" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T8" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V8" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W8" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X8" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y8" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z8" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB8" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC8" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C9" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D9" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E9" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F9" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G9" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H9" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I9" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J9" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K9" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L9" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M9" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N9" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O9" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P9" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q9" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R9" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S9" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T9" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U9" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V9" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W9" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X9" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y9" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z9" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA9" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC9" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C10" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D10" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E10" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F10" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G10" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H10" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I10" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J10" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K10" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L10" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M10" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N10" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O10" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P10" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q10" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R10" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S10" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T10" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U10" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V10" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W10" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X10" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y10" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z10" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB10" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC10" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C11" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D11" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E11" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F11" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H11" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I11" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J11" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K11" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L11" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M11" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N11" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O11" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P11" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q11" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R11" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S11" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T11" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U11" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V11" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X11" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y11" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z11" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA11" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB11" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC11" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C12" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D12" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E12" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F12" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G12" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I12" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J12" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K12" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L12" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M12" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N12" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O12" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P12" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q12" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S12" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T12" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W12" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X12" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y12" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z12" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC12" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C13" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D13" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E13" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F13" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G13" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K13" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L13" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M13" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N13" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O13" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P13" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q13" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R13" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S13" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T13" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U13" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V13" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W13" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X13" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y13" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z13" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA13" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB13" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC13" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>98.34999999999999</v>
+        <v>101.19</v>
       </c>
       <c r="C14" t="n">
-        <v>108.8</v>
+        <v>103.93</v>
       </c>
       <c r="D14" t="n">
-        <v>95.23</v>
+        <v>93.45</v>
       </c>
       <c r="E14" t="n">
-        <v>107.35</v>
+        <v>93.67</v>
       </c>
       <c r="F14" t="n">
-        <v>70.95</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>74.23999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="H14" t="n">
-        <v>69.98999999999999</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>73.81999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>47.19</v>
+        <v>46.22</v>
       </c>
       <c r="K14" t="n">
-        <v>48.37</v>
+        <v>49.36</v>
       </c>
       <c r="L14" t="n">
-        <v>43.11</v>
+        <v>45.08</v>
       </c>
       <c r="M14" t="n">
-        <v>43.64</v>
+        <v>49.23</v>
       </c>
       <c r="N14" t="n">
-        <v>37.57</v>
+        <v>36.57</v>
       </c>
       <c r="O14" t="n">
-        <v>38.02</v>
+        <v>39.29</v>
       </c>
       <c r="P14" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q14" t="n">
-        <v>36.14</v>
+        <v>38.9</v>
       </c>
       <c r="R14" t="n">
-        <v>-2.8858</v>
+        <v>-12.7434</v>
       </c>
       <c r="S14" t="n">
-        <v>-16.3941</v>
+        <v>-26.5736</v>
       </c>
       <c r="T14" t="n">
-        <v>-24.6772</v>
+        <v>-32.978</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.4047</v>
+        <v>-7.5996</v>
       </c>
       <c r="V14" t="n">
-        <v>-7.273</v>
+        <v>-13.4501</v>
       </c>
       <c r="W14" t="n">
-        <v>-7.9895</v>
+        <v>-16.0802</v>
       </c>
       <c r="X14" t="n">
-        <v>2.6341</v>
+        <v>12.8093</v>
       </c>
       <c r="Y14" t="n">
-        <v>17.3434</v>
+        <v>31.5607</v>
       </c>
       <c r="Z14" t="n">
-        <v>29.1506</v>
+        <v>43.1521</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.3889</v>
+        <v>7.637</v>
       </c>
       <c r="AB14" t="n">
-        <v>7.4636</v>
+        <v>14.4454</v>
       </c>
       <c r="AC14" t="n">
-        <v>8.3009</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>101.19</v>
+        <v>103.95</v>
       </c>
       <c r="C15" t="n">
-        <v>103.93</v>
+        <v>104.98</v>
       </c>
       <c r="D15" t="n">
-        <v>93.45</v>
+        <v>97.8</v>
       </c>
       <c r="E15" t="n">
-        <v>93.67</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>73.01000000000001</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>73.13</v>
+        <v>72.44</v>
       </c>
       <c r="H15" t="n">
-        <v>67.43000000000001</v>
+        <v>70.13</v>
       </c>
       <c r="I15" t="n">
-        <v>68.20999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J15" t="n">
-        <v>46.22</v>
+        <v>43.86</v>
       </c>
       <c r="K15" t="n">
-        <v>49.36</v>
+        <v>47.07</v>
       </c>
       <c r="L15" t="n">
-        <v>45.08</v>
+        <v>43.32</v>
       </c>
       <c r="M15" t="n">
-        <v>49.23</v>
+        <v>46.63</v>
       </c>
       <c r="N15" t="n">
-        <v>36.57</v>
+        <v>37.33</v>
       </c>
       <c r="O15" t="n">
-        <v>39.29</v>
+        <v>37.82</v>
       </c>
       <c r="P15" t="n">
         <v>36.51</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.9</v>
+        <v>37.52</v>
       </c>
       <c r="R15" t="n">
-        <v>-12.7434</v>
+        <v>5.3165</v>
       </c>
       <c r="S15" t="n">
-        <v>-26.5736</v>
+        <v>-10.7563</v>
       </c>
       <c r="T15" t="n">
-        <v>-32.978</v>
+        <v>-23.1698</v>
       </c>
       <c r="U15" t="n">
-        <v>-7.5996</v>
+        <v>3.5625</v>
       </c>
       <c r="V15" t="n">
-        <v>-13.4501</v>
+        <v>-4.6951</v>
       </c>
       <c r="W15" t="n">
-        <v>-16.0802</v>
+        <v>-11.2674</v>
       </c>
       <c r="X15" t="n">
-        <v>12.8093</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y15" t="n">
-        <v>31.5607</v>
+        <v>9.666</v>
       </c>
       <c r="Z15" t="n">
-        <v>43.1521</v>
+        <v>25.3832</v>
       </c>
       <c r="AA15" t="n">
-        <v>7.637</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB15" t="n">
-        <v>14.4454</v>
+        <v>4.2222</v>
       </c>
       <c r="AC15" t="n">
-        <v>18.0577</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>103.95</v>
+        <v>94.52</v>
       </c>
       <c r="C16" t="n">
-        <v>104.98</v>
+        <v>102.62</v>
       </c>
       <c r="D16" t="n">
-        <v>97.8</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>98.65000000000001</v>
+        <v>97.55</v>
       </c>
       <c r="F16" t="n">
-        <v>71.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>72.44</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>70.13</v>
+        <v>68.28</v>
       </c>
       <c r="I16" t="n">
-        <v>70.64</v>
+        <v>70.41</v>
       </c>
       <c r="J16" t="n">
-        <v>43.86</v>
+        <v>48.64</v>
       </c>
       <c r="K16" t="n">
-        <v>47.07</v>
+        <v>50.12</v>
       </c>
       <c r="L16" t="n">
-        <v>43.32</v>
+        <v>44.76</v>
       </c>
       <c r="M16" t="n">
-        <v>46.63</v>
+        <v>47.13</v>
       </c>
       <c r="N16" t="n">
-        <v>37.33</v>
+        <v>38.03</v>
       </c>
       <c r="O16" t="n">
-        <v>37.82</v>
+        <v>38.79</v>
       </c>
       <c r="P16" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.52</v>
+        <v>37.68</v>
       </c>
       <c r="R16" t="n">
-        <v>5.3165</v>
+        <v>-1.1151</v>
       </c>
       <c r="S16" t="n">
-        <v>-10.7563</v>
+        <v>-9.129</v>
       </c>
       <c r="T16" t="n">
-        <v>-23.1698</v>
+        <v>-23.5322</v>
       </c>
       <c r="U16" t="n">
-        <v>3.5625</v>
+        <v>-0.3256</v>
       </c>
       <c r="V16" t="n">
-        <v>-4.6951</v>
+        <v>-4.6193</v>
       </c>
       <c r="W16" t="n">
-        <v>-11.2674</v>
+        <v>-10.6585</v>
       </c>
       <c r="X16" t="n">
-        <v>-5.2813</v>
+        <v>1.0723</v>
       </c>
       <c r="Y16" t="n">
-        <v>9.666</v>
+        <v>7.9973</v>
       </c>
       <c r="Z16" t="n">
-        <v>25.3832</v>
+        <v>25.9487</v>
       </c>
       <c r="AA16" t="n">
-        <v>-3.5476</v>
+        <v>0.4264</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.2222</v>
+        <v>4.2612</v>
       </c>
       <c r="AC16" t="n">
-        <v>11.5671</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>94.52</v>
+        <v>102.86</v>
       </c>
       <c r="C17" t="n">
-        <v>102.62</v>
+        <v>106.13</v>
       </c>
       <c r="D17" t="n">
-        <v>91.34999999999999</v>
+        <v>99.31</v>
       </c>
       <c r="E17" t="n">
-        <v>97.55</v>
+        <v>103.24</v>
       </c>
       <c r="F17" t="n">
-        <v>69.70999999999999</v>
+        <v>71.72</v>
       </c>
       <c r="G17" t="n">
-        <v>71.93000000000001</v>
+        <v>73.43000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>68.28</v>
+        <v>71.02</v>
       </c>
       <c r="I17" t="n">
-        <v>70.41</v>
+        <v>72.61</v>
       </c>
       <c r="J17" t="n">
-        <v>48.64</v>
+        <v>44.51</v>
       </c>
       <c r="K17" t="n">
-        <v>50.12</v>
+        <v>47.1</v>
       </c>
       <c r="L17" t="n">
-        <v>44.76</v>
+        <v>43.57</v>
       </c>
       <c r="M17" t="n">
-        <v>47.13</v>
+        <v>44.29</v>
       </c>
       <c r="N17" t="n">
-        <v>38.03</v>
+        <v>36.94</v>
       </c>
       <c r="O17" t="n">
-        <v>38.79</v>
+        <v>38.11</v>
       </c>
       <c r="P17" t="n">
-        <v>36.85</v>
+        <v>36.05</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.68</v>
+        <v>36.48</v>
       </c>
       <c r="R17" t="n">
-        <v>-1.1151</v>
+        <v>5.8329</v>
       </c>
       <c r="S17" t="n">
-        <v>-9.129</v>
+        <v>10.2167</v>
       </c>
       <c r="T17" t="n">
-        <v>-23.5322</v>
+        <v>-6.6039</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.3256</v>
+        <v>3.1246</v>
       </c>
       <c r="V17" t="n">
-        <v>-4.6193</v>
+        <v>6.4507</v>
       </c>
       <c r="W17" t="n">
-        <v>-10.6585</v>
+        <v>-2.0372</v>
       </c>
       <c r="X17" t="n">
-        <v>1.0723</v>
+        <v>-6.0259</v>
       </c>
       <c r="Y17" t="n">
-        <v>7.9973</v>
+        <v>-10.0345</v>
       </c>
       <c r="Z17" t="n">
-        <v>25.9487</v>
+        <v>4.1627</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.4264</v>
+        <v>-3.1847</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.2612</v>
+        <v>-6.2211</v>
       </c>
       <c r="AC17" t="n">
-        <v>10.8561</v>
+        <v>1.3333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>102.86</v>
+        <v>90.59</v>
       </c>
       <c r="C18" t="n">
-        <v>106.13</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>99.31</v>
+        <v>80.22</v>
       </c>
       <c r="E18" t="n">
-        <v>103.24</v>
+        <v>82.11</v>
       </c>
       <c r="F18" t="n">
-        <v>71.72</v>
+        <v>69.14</v>
       </c>
       <c r="G18" t="n">
-        <v>73.43000000000001</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>71.02</v>
+        <v>65.61</v>
       </c>
       <c r="I18" t="n">
-        <v>72.61</v>
+        <v>66.42</v>
       </c>
       <c r="J18" t="n">
-        <v>44.51</v>
+        <v>49.82</v>
       </c>
       <c r="K18" t="n">
-        <v>47.1</v>
+        <v>54.31</v>
       </c>
       <c r="L18" t="n">
-        <v>43.57</v>
+        <v>48.62</v>
       </c>
       <c r="M18" t="n">
-        <v>44.29</v>
+        <v>53.45</v>
       </c>
       <c r="N18" t="n">
-        <v>36.94</v>
+        <v>38.23</v>
       </c>
       <c r="O18" t="n">
-        <v>38.11</v>
+        <v>40</v>
       </c>
       <c r="P18" t="n">
-        <v>36.05</v>
+        <v>37.96</v>
       </c>
       <c r="Q18" t="n">
-        <v>36.48</v>
+        <v>39.6</v>
       </c>
       <c r="R18" t="n">
-        <v>5.8329</v>
+        <v>-20.4669</v>
       </c>
       <c r="S18" t="n">
-        <v>10.2167</v>
+        <v>-16.7663</v>
       </c>
       <c r="T18" t="n">
-        <v>-6.6039</v>
+        <v>-23.5119</v>
       </c>
       <c r="U18" t="n">
-        <v>3.1246</v>
+        <v>-8.525</v>
       </c>
       <c r="V18" t="n">
-        <v>6.4507</v>
+        <v>-5.974</v>
       </c>
       <c r="W18" t="n">
-        <v>-2.0372</v>
+        <v>-10.0244</v>
       </c>
       <c r="X18" t="n">
-        <v>-6.0259</v>
+        <v>20.6819</v>
       </c>
       <c r="Y18" t="n">
-        <v>-10.0345</v>
+        <v>14.6258</v>
       </c>
       <c r="Z18" t="n">
-        <v>4.1627</v>
+        <v>22.4794</v>
       </c>
       <c r="AA18" t="n">
-        <v>-3.1847</v>
+        <v>8.5526</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.2211</v>
+        <v>5.5437</v>
       </c>
       <c r="AC18" t="n">
-        <v>1.3333</v>
+        <v>9.5739</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>90.59</v>
+        <v>81.64</v>
       </c>
       <c r="C19" t="n">
-        <v>93.40000000000001</v>
+        <v>87.61</v>
       </c>
       <c r="D19" t="n">
-        <v>80.22</v>
+        <v>80.83</v>
       </c>
       <c r="E19" t="n">
-        <v>82.11</v>
+        <v>83.56</v>
       </c>
       <c r="F19" t="n">
-        <v>69.14</v>
+        <v>65.66</v>
       </c>
       <c r="G19" t="n">
-        <v>69.65000000000001</v>
+        <v>67.67</v>
       </c>
       <c r="H19" t="n">
-        <v>65.61</v>
+        <v>65.37</v>
       </c>
       <c r="I19" t="n">
-        <v>66.42</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>49.82</v>
+        <v>53.77</v>
       </c>
       <c r="K19" t="n">
-        <v>54.31</v>
+        <v>54.38</v>
       </c>
       <c r="L19" t="n">
-        <v>48.62</v>
+        <v>50.27</v>
       </c>
       <c r="M19" t="n">
-        <v>53.45</v>
+        <v>52.46</v>
       </c>
       <c r="N19" t="n">
-        <v>38.23</v>
+        <v>40.07</v>
       </c>
       <c r="O19" t="n">
-        <v>40</v>
+        <v>40.23</v>
       </c>
       <c r="P19" t="n">
-        <v>37.96</v>
+        <v>38.86</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.6</v>
+        <v>39.68</v>
       </c>
       <c r="R19" t="n">
-        <v>-20.4669</v>
+        <v>1.7659</v>
       </c>
       <c r="S19" t="n">
-        <v>-16.7663</v>
+        <v>-14.3414</v>
       </c>
       <c r="T19" t="n">
-        <v>-23.5119</v>
+        <v>-10.7932</v>
       </c>
       <c r="U19" t="n">
-        <v>-8.525</v>
+        <v>-0.1957</v>
       </c>
       <c r="V19" t="n">
-        <v>-5.974</v>
+        <v>-5.8514</v>
       </c>
       <c r="W19" t="n">
-        <v>-10.0244</v>
+        <v>-2.8148</v>
       </c>
       <c r="X19" t="n">
-        <v>20.6819</v>
+        <v>-1.8522</v>
       </c>
       <c r="Y19" t="n">
-        <v>14.6258</v>
+        <v>11.3091</v>
       </c>
       <c r="Z19" t="n">
-        <v>22.4794</v>
+        <v>6.561</v>
       </c>
       <c r="AA19" t="n">
-        <v>8.5526</v>
+        <v>0.202</v>
       </c>
       <c r="AB19" t="n">
-        <v>5.5437</v>
+        <v>5.3079</v>
       </c>
       <c r="AC19" t="n">
-        <v>9.5739</v>
+        <v>2.0051</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>81.64</v>
+        <v>85.88</v>
       </c>
       <c r="C20" t="n">
-        <v>87.61</v>
+        <v>93.15000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>80.83</v>
+        <v>84.22</v>
       </c>
       <c r="E20" t="n">
-        <v>83.56</v>
+        <v>90.5</v>
       </c>
       <c r="F20" t="n">
-        <v>65.66</v>
+        <v>67.02</v>
       </c>
       <c r="G20" t="n">
-        <v>67.67</v>
+        <v>69.33</v>
       </c>
       <c r="H20" t="n">
-        <v>65.37</v>
+        <v>66.61</v>
       </c>
       <c r="I20" t="n">
-        <v>66.29000000000001</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>53.77</v>
+        <v>51.03</v>
       </c>
       <c r="K20" t="n">
-        <v>54.38</v>
+        <v>52.09</v>
       </c>
       <c r="L20" t="n">
-        <v>50.27</v>
+        <v>46.47</v>
       </c>
       <c r="M20" t="n">
-        <v>52.46</v>
+        <v>47.98</v>
       </c>
       <c r="N20" t="n">
-        <v>40.07</v>
+        <v>39.23</v>
       </c>
       <c r="O20" t="n">
-        <v>40.23</v>
+        <v>39.51</v>
       </c>
       <c r="P20" t="n">
-        <v>38.86</v>
+        <v>37.86</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.68</v>
+        <v>38.38</v>
       </c>
       <c r="R20" t="n">
-        <v>1.7659</v>
+        <v>8.305400000000001</v>
       </c>
       <c r="S20" t="n">
-        <v>-14.3414</v>
+        <v>-12.3402</v>
       </c>
       <c r="T20" t="n">
-        <v>-10.7932</v>
+        <v>-8.2615</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.1957</v>
+        <v>3.2282</v>
       </c>
       <c r="V20" t="n">
-        <v>-5.8514</v>
+        <v>-5.7568</v>
       </c>
       <c r="W20" t="n">
-        <v>-2.8148</v>
+        <v>-3.1285</v>
       </c>
       <c r="X20" t="n">
-        <v>-1.8522</v>
+        <v>-8.5398</v>
       </c>
       <c r="Y20" t="n">
-        <v>11.3091</v>
+        <v>8.3315</v>
       </c>
       <c r="Z20" t="n">
-        <v>6.561</v>
+        <v>2.8951</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.202</v>
+        <v>-3.2762</v>
       </c>
       <c r="AB20" t="n">
-        <v>5.3079</v>
+        <v>5.2083</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.0051</v>
+        <v>2.2921</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>85.88</v>
+        <v>95.04000000000001</v>
       </c>
       <c r="C21" t="n">
-        <v>93.15000000000001</v>
+        <v>102.2</v>
       </c>
       <c r="D21" t="n">
-        <v>84.22</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>90.5</v>
+        <v>101.08</v>
       </c>
       <c r="F21" t="n">
-        <v>67.02</v>
+        <v>69.3</v>
       </c>
       <c r="G21" t="n">
-        <v>69.33</v>
+        <v>71.53</v>
       </c>
       <c r="H21" t="n">
-        <v>66.61</v>
+        <v>68.86</v>
       </c>
       <c r="I21" t="n">
-        <v>68.43000000000001</v>
+        <v>71.04000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>51.03</v>
+        <v>45.8</v>
       </c>
       <c r="K21" t="n">
-        <v>52.09</v>
+        <v>46.21</v>
       </c>
       <c r="L21" t="n">
-        <v>46.47</v>
+        <v>41.9</v>
       </c>
       <c r="M21" t="n">
-        <v>47.98</v>
+        <v>42.5</v>
       </c>
       <c r="N21" t="n">
-        <v>39.23</v>
+        <v>37.93</v>
       </c>
       <c r="O21" t="n">
-        <v>39.51</v>
+        <v>38.17</v>
       </c>
       <c r="P21" t="n">
-        <v>37.86</v>
+        <v>36.67</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.38</v>
+        <v>36.93</v>
       </c>
       <c r="R21" t="n">
-        <v>8.305400000000001</v>
+        <v>11.6906</v>
       </c>
       <c r="S21" t="n">
-        <v>-12.3402</v>
+        <v>23.1032</v>
       </c>
       <c r="T21" t="n">
-        <v>-8.2615</v>
+        <v>3.6187</v>
       </c>
       <c r="U21" t="n">
-        <v>3.2282</v>
+        <v>3.8141</v>
       </c>
       <c r="V21" t="n">
-        <v>-5.7568</v>
+        <v>6.9557</v>
       </c>
       <c r="W21" t="n">
-        <v>-3.1285</v>
+        <v>0.8948</v>
       </c>
       <c r="X21" t="n">
-        <v>-8.5398</v>
+        <v>-11.4214</v>
       </c>
       <c r="Y21" t="n">
-        <v>8.3315</v>
+        <v>-20.4864</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.8951</v>
+        <v>-9.8239</v>
       </c>
       <c r="AA21" t="n">
-        <v>-3.2762</v>
+        <v>-3.778</v>
       </c>
       <c r="AB21" t="n">
-        <v>5.2083</v>
+        <v>-6.7424</v>
       </c>
       <c r="AC21" t="n">
-        <v>2.2921</v>
+        <v>-1.9904</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>95.04000000000001</v>
+        <v>103.97</v>
       </c>
       <c r="C22" t="n">
-        <v>102.2</v>
+        <v>108.6</v>
       </c>
       <c r="D22" t="n">
-        <v>94.09999999999999</v>
+        <v>101.32</v>
       </c>
       <c r="E22" t="n">
-        <v>101.08</v>
+        <v>107.35</v>
       </c>
       <c r="F22" t="n">
-        <v>69.3</v>
+        <v>71.91</v>
       </c>
       <c r="G22" t="n">
-        <v>71.53</v>
+        <v>72.53</v>
       </c>
       <c r="H22" t="n">
-        <v>68.86</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>71.04000000000001</v>
+        <v>72.36</v>
       </c>
       <c r="J22" t="n">
-        <v>45.8</v>
+        <v>41.33</v>
       </c>
       <c r="K22" t="n">
-        <v>46.21</v>
+        <v>42.41</v>
       </c>
       <c r="L22" t="n">
-        <v>41.9</v>
+        <v>39.33</v>
       </c>
       <c r="M22" t="n">
-        <v>42.5</v>
+        <v>39.78</v>
       </c>
       <c r="N22" t="n">
-        <v>37.93</v>
+        <v>36.51</v>
       </c>
       <c r="O22" t="n">
-        <v>38.17</v>
+        <v>37.09</v>
       </c>
       <c r="P22" t="n">
-        <v>36.67</v>
+        <v>36.2</v>
       </c>
       <c r="Q22" t="n">
-        <v>36.93</v>
+        <v>36.28</v>
       </c>
       <c r="R22" t="n">
-        <v>11.6906</v>
+        <v>6.203</v>
       </c>
       <c r="S22" t="n">
-        <v>23.1032</v>
+        <v>28.4706</v>
       </c>
       <c r="T22" t="n">
-        <v>3.6187</v>
+        <v>3.981</v>
       </c>
       <c r="U22" t="n">
-        <v>3.8141</v>
+        <v>1.8581</v>
       </c>
       <c r="V22" t="n">
-        <v>6.9557</v>
+        <v>9.156700000000001</v>
       </c>
       <c r="W22" t="n">
-        <v>0.8948</v>
+        <v>-0.3443</v>
       </c>
       <c r="X22" t="n">
-        <v>-11.4214</v>
+        <v>-6.4</v>
       </c>
       <c r="Y22" t="n">
-        <v>-20.4864</v>
+        <v>-24.1708</v>
       </c>
       <c r="Z22" t="n">
-        <v>-9.8239</v>
+        <v>-10.1829</v>
       </c>
       <c r="AA22" t="n">
-        <v>-3.778</v>
+        <v>-1.7601</v>
       </c>
       <c r="AB22" t="n">
-        <v>-6.7424</v>
+        <v>-8.5685</v>
       </c>
       <c r="AC22" t="n">
-        <v>-1.9904</v>
+        <v>-0.5482</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>103.97</v>
+        <v>101.36</v>
       </c>
       <c r="C23" t="n">
-        <v>108.6</v>
+        <v>105.44</v>
       </c>
       <c r="D23" t="n">
-        <v>101.32</v>
+        <v>97.95</v>
       </c>
       <c r="E23" t="n">
-        <v>107.35</v>
+        <v>102.39</v>
       </c>
       <c r="F23" t="n">
-        <v>71.91</v>
+        <v>69.61</v>
       </c>
       <c r="G23" t="n">
-        <v>72.53</v>
+        <v>70.06</v>
       </c>
       <c r="H23" t="n">
-        <v>70.76000000000001</v>
+        <v>68.13</v>
       </c>
       <c r="I23" t="n">
-        <v>72.36</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>41.33</v>
+        <v>42.08</v>
       </c>
       <c r="K23" t="n">
-        <v>42.41</v>
+        <v>43.36</v>
       </c>
       <c r="L23" t="n">
-        <v>39.33</v>
+        <v>40.58</v>
       </c>
       <c r="M23" t="n">
-        <v>39.78</v>
+        <v>41.68</v>
       </c>
       <c r="N23" t="n">
-        <v>36.51</v>
+        <v>37.65</v>
       </c>
       <c r="O23" t="n">
-        <v>37.09</v>
+        <v>38.4</v>
       </c>
       <c r="P23" t="n">
-        <v>36.2</v>
+        <v>37.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>36.28</v>
+        <v>37.83</v>
       </c>
       <c r="R23" t="n">
-        <v>6.203</v>
+        <v>-4.6204</v>
       </c>
       <c r="S23" t="n">
-        <v>28.4706</v>
+        <v>13.1381</v>
       </c>
       <c r="T23" t="n">
-        <v>3.981</v>
+        <v>24.6986</v>
       </c>
       <c r="U23" t="n">
-        <v>1.8581</v>
+        <v>-4.2841</v>
       </c>
       <c r="V23" t="n">
-        <v>9.156700000000001</v>
+        <v>1.2129</v>
       </c>
       <c r="W23" t="n">
-        <v>-0.3443</v>
+        <v>4.2758</v>
       </c>
       <c r="X23" t="n">
-        <v>-6.4</v>
+        <v>4.7763</v>
       </c>
       <c r="Y23" t="n">
-        <v>-24.1708</v>
+        <v>-13.1305</v>
       </c>
       <c r="Z23" t="n">
-        <v>-10.1829</v>
+        <v>-22.0206</v>
       </c>
       <c r="AA23" t="n">
-        <v>-1.7601</v>
+        <v>4.2723</v>
       </c>
       <c r="AB23" t="n">
-        <v>-8.5685</v>
+        <v>-1.433</v>
       </c>
       <c r="AC23" t="n">
-        <v>-0.5482</v>
+        <v>-4.4697</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-10-31 01:26
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>147.95</v>
+        <v>148.56</v>
       </c>
       <c r="C2" t="n">
-        <v>150.77</v>
+        <v>156.71</v>
       </c>
       <c r="D2" t="n">
-        <v>144.41</v>
+        <v>144.31</v>
       </c>
       <c r="E2" t="n">
-        <v>147.86</v>
+        <v>153.69</v>
       </c>
       <c r="F2" t="n">
-        <v>78.13</v>
+        <v>78.88</v>
       </c>
       <c r="G2" t="n">
-        <v>79.68000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="H2" t="n">
-        <v>77.94</v>
+        <v>76.87</v>
       </c>
       <c r="I2" t="n">
-        <v>78.03</v>
+        <v>78.73</v>
       </c>
       <c r="J2" t="n">
-        <v>33.07</v>
+        <v>32.95</v>
       </c>
       <c r="K2" t="n">
-        <v>33.86</v>
+        <v>33.89</v>
       </c>
       <c r="L2" t="n">
-        <v>32.42</v>
+        <v>31.1</v>
       </c>
       <c r="M2" t="n">
-        <v>33.08</v>
+        <v>31.76</v>
       </c>
       <c r="N2" t="n">
-        <v>34.36</v>
+        <v>34.04</v>
       </c>
       <c r="O2" t="n">
-        <v>34.44</v>
+        <v>34.92</v>
       </c>
       <c r="P2" t="n">
-        <v>33.66</v>
+        <v>33.74</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.41</v>
+        <v>34.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>148.56</v>
+        <v>165.39</v>
       </c>
       <c r="C3" t="n">
-        <v>156.71</v>
+        <v>169.75</v>
       </c>
       <c r="D3" t="n">
-        <v>144.31</v>
+        <v>162.4</v>
       </c>
       <c r="E3" t="n">
-        <v>153.69</v>
+        <v>163.71</v>
       </c>
       <c r="F3" t="n">
-        <v>78.88</v>
+        <v>81.59</v>
       </c>
       <c r="G3" t="n">
-        <v>79.53</v>
+        <v>82.61</v>
       </c>
       <c r="H3" t="n">
-        <v>76.87</v>
+        <v>80.37</v>
       </c>
       <c r="I3" t="n">
-        <v>78.73</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>32.95</v>
+        <v>29.39</v>
       </c>
       <c r="K3" t="n">
-        <v>33.89</v>
+        <v>29.98</v>
       </c>
       <c r="L3" t="n">
-        <v>31.1</v>
+        <v>28.46</v>
       </c>
       <c r="M3" t="n">
-        <v>31.76</v>
+        <v>29.71</v>
       </c>
       <c r="N3" t="n">
-        <v>34.04</v>
+        <v>32.87</v>
       </c>
       <c r="O3" t="n">
-        <v>34.92</v>
+        <v>33.41</v>
       </c>
       <c r="P3" t="n">
-        <v>33.74</v>
+        <v>32.44</v>
       </c>
       <c r="Q3" t="n">
-        <v>34.11</v>
+        <v>33.12</v>
       </c>
       <c r="R3" t="n">
-        <v>3.9429</v>
+        <v>6.5196</v>
       </c>
       <c r="U3" t="n">
-        <v>0.8971</v>
+        <v>2.896</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.9903</v>
+        <v>-6.4547</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.8718</v>
+        <v>-2.9024</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>165.39</v>
+        <v>161.66</v>
       </c>
       <c r="C4" t="n">
-        <v>169.75</v>
+        <v>164.38</v>
       </c>
       <c r="D4" t="n">
-        <v>162.4</v>
+        <v>158.08</v>
       </c>
       <c r="E4" t="n">
-        <v>163.71</v>
+        <v>164.27</v>
       </c>
       <c r="F4" t="n">
-        <v>81.59</v>
+        <v>80.95</v>
       </c>
       <c r="G4" t="n">
-        <v>82.61</v>
+        <v>83.38</v>
       </c>
       <c r="H4" t="n">
-        <v>80.37</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>81.01000000000001</v>
+        <v>83.12</v>
       </c>
       <c r="J4" t="n">
-        <v>29.39</v>
+        <v>30.09</v>
       </c>
       <c r="K4" t="n">
-        <v>29.98</v>
+        <v>30.75</v>
       </c>
       <c r="L4" t="n">
-        <v>28.46</v>
+        <v>29.62</v>
       </c>
       <c r="M4" t="n">
-        <v>29.71</v>
+        <v>29.62</v>
       </c>
       <c r="N4" t="n">
-        <v>32.87</v>
+        <v>33.17</v>
       </c>
       <c r="O4" t="n">
-        <v>33.41</v>
+        <v>33.2</v>
       </c>
       <c r="P4" t="n">
-        <v>32.44</v>
+        <v>32.16</v>
       </c>
       <c r="Q4" t="n">
-        <v>33.12</v>
+        <v>32.25</v>
       </c>
       <c r="R4" t="n">
-        <v>6.5196</v>
+        <v>0.3421</v>
       </c>
       <c r="U4" t="n">
-        <v>2.896</v>
+        <v>2.6046</v>
       </c>
       <c r="X4" t="n">
-        <v>-6.4547</v>
+        <v>-0.3029</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.9024</v>
+        <v>-2.6268</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>161.66</v>
+        <v>167.34</v>
       </c>
       <c r="C5" t="n">
-        <v>164.38</v>
+        <v>169.83</v>
       </c>
       <c r="D5" t="n">
-        <v>158.08</v>
+        <v>163.42</v>
       </c>
       <c r="E5" t="n">
-        <v>164.27</v>
+        <v>164.26</v>
       </c>
       <c r="F5" t="n">
-        <v>80.95</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>83.38</v>
+        <v>85.31999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>80.84999999999999</v>
+        <v>84.09</v>
       </c>
       <c r="I5" t="n">
-        <v>83.12</v>
+        <v>84.25</v>
       </c>
       <c r="J5" t="n">
-        <v>30.09</v>
+        <v>29.06</v>
       </c>
       <c r="K5" t="n">
-        <v>30.75</v>
+        <v>29.77</v>
       </c>
       <c r="L5" t="n">
-        <v>29.62</v>
+        <v>28.62</v>
       </c>
       <c r="M5" t="n">
-        <v>29.62</v>
+        <v>29.63</v>
       </c>
       <c r="N5" t="n">
-        <v>33.17</v>
+        <v>31.72</v>
       </c>
       <c r="O5" t="n">
-        <v>33.2</v>
+        <v>31.9</v>
       </c>
       <c r="P5" t="n">
-        <v>32.16</v>
+        <v>31.42</v>
       </c>
       <c r="Q5" t="n">
-        <v>32.25</v>
+        <v>31.83</v>
       </c>
       <c r="R5" t="n">
-        <v>0.3421</v>
+        <v>-0.0061</v>
       </c>
       <c r="S5" t="n">
-        <v>11.0983</v>
+        <v>6.8775</v>
       </c>
       <c r="U5" t="n">
-        <v>2.6046</v>
+        <v>1.3595</v>
       </c>
       <c r="V5" t="n">
-        <v>6.5231</v>
+        <v>7.0113</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.3029</v>
+        <v>0.0338</v>
       </c>
       <c r="Y5" t="n">
-        <v>-10.4595</v>
+        <v>-6.7065</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.6268</v>
+        <v>-1.3023</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.2772</v>
+        <v>-6.6843</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>167.34</v>
+        <v>153.7</v>
       </c>
       <c r="C6" t="n">
-        <v>169.83</v>
+        <v>159.49</v>
       </c>
       <c r="D6" t="n">
-        <v>163.42</v>
+        <v>151.42</v>
       </c>
       <c r="E6" t="n">
-        <v>164.26</v>
+        <v>158.91</v>
       </c>
       <c r="F6" t="n">
-        <v>84.54000000000001</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>85.31999999999999</v>
+        <v>83.75</v>
       </c>
       <c r="H6" t="n">
-        <v>84.09</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>84.25</v>
+        <v>83.62</v>
       </c>
       <c r="J6" t="n">
-        <v>29.06</v>
+        <v>31.55</v>
       </c>
       <c r="K6" t="n">
-        <v>29.77</v>
+        <v>31.97</v>
       </c>
       <c r="L6" t="n">
-        <v>28.62</v>
+        <v>30.5</v>
       </c>
       <c r="M6" t="n">
-        <v>29.63</v>
+        <v>30.65</v>
       </c>
       <c r="N6" t="n">
-        <v>31.72</v>
+        <v>32.58</v>
       </c>
       <c r="O6" t="n">
-        <v>31.9</v>
+        <v>32.84</v>
       </c>
       <c r="P6" t="n">
-        <v>31.42</v>
+        <v>32.02</v>
       </c>
       <c r="Q6" t="n">
-        <v>31.83</v>
+        <v>32.07</v>
       </c>
       <c r="R6" t="n">
-        <v>-0.0061</v>
+        <v>-3.257</v>
       </c>
       <c r="S6" t="n">
-        <v>6.8775</v>
+        <v>-2.932</v>
       </c>
       <c r="U6" t="n">
-        <v>1.3595</v>
+        <v>-0.7478</v>
       </c>
       <c r="V6" t="n">
-        <v>7.0113</v>
+        <v>3.2218</v>
       </c>
       <c r="X6" t="n">
-        <v>0.0338</v>
+        <v>3.4425</v>
       </c>
       <c r="Y6" t="n">
-        <v>-6.7065</v>
+        <v>3.1639</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.3023</v>
+        <v>0.754</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.6843</v>
+        <v>-3.1703</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>153.7</v>
+        <v>150.48</v>
       </c>
       <c r="C7" t="n">
-        <v>159.49</v>
+        <v>155.5</v>
       </c>
       <c r="D7" t="n">
-        <v>151.42</v>
+        <v>136.32</v>
       </c>
       <c r="E7" t="n">
-        <v>158.91</v>
+        <v>142.52</v>
       </c>
       <c r="F7" t="n">
-        <v>82.31999999999999</v>
+        <v>82.33</v>
       </c>
       <c r="G7" t="n">
-        <v>83.75</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>81.59999999999999</v>
+        <v>78.78</v>
       </c>
       <c r="I7" t="n">
-        <v>83.62</v>
+        <v>80.23</v>
       </c>
       <c r="J7" t="n">
-        <v>31.55</v>
+        <v>32.25</v>
       </c>
       <c r="K7" t="n">
-        <v>31.97</v>
+        <v>34.96</v>
       </c>
       <c r="L7" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="M7" t="n">
-        <v>30.65</v>
+        <v>33.79</v>
       </c>
       <c r="N7" t="n">
         <v>32.58</v>
       </c>
       <c r="O7" t="n">
-        <v>32.84</v>
+        <v>33.94</v>
       </c>
       <c r="P7" t="n">
-        <v>32.02</v>
+        <v>32.16</v>
       </c>
       <c r="Q7" t="n">
-        <v>32.07</v>
+        <v>33.37</v>
       </c>
       <c r="R7" t="n">
-        <v>-3.257</v>
+        <v>-10.314</v>
       </c>
       <c r="S7" t="n">
-        <v>-2.932</v>
+        <v>-13.2404</v>
       </c>
       <c r="T7" t="n">
-        <v>7.4733</v>
+        <v>-7.2679</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.7478</v>
+        <v>-4.0541</v>
       </c>
       <c r="V7" t="n">
-        <v>3.2218</v>
+        <v>-3.4769</v>
       </c>
       <c r="W7" t="n">
-        <v>7.1639</v>
+        <v>1.9052</v>
       </c>
       <c r="X7" t="n">
-        <v>3.4425</v>
+        <v>10.2447</v>
       </c>
       <c r="Y7" t="n">
-        <v>3.1639</v>
+        <v>14.0783</v>
       </c>
       <c r="Z7" t="n">
-        <v>-7.3458</v>
+        <v>6.3917</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.754</v>
+        <v>4.0536</v>
       </c>
       <c r="AB7" t="n">
-        <v>-3.1703</v>
+        <v>3.4729</v>
       </c>
       <c r="AC7" t="n">
-        <v>-6.8003</v>
+        <v>-2.1695</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>150.48</v>
+        <v>148.18</v>
       </c>
       <c r="C8" t="n">
-        <v>155.5</v>
+        <v>148.18</v>
       </c>
       <c r="D8" t="n">
-        <v>136.32</v>
+        <v>137.71</v>
       </c>
       <c r="E8" t="n">
-        <v>142.52</v>
+        <v>139.76</v>
       </c>
       <c r="F8" t="n">
-        <v>82.33</v>
+        <v>81.72</v>
       </c>
       <c r="G8" t="n">
-        <v>83.40000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="H8" t="n">
-        <v>78.78</v>
+        <v>80.37</v>
       </c>
       <c r="I8" t="n">
-        <v>80.23</v>
+        <v>81.28</v>
       </c>
       <c r="J8" t="n">
-        <v>32.25</v>
+        <v>32.4</v>
       </c>
       <c r="K8" t="n">
-        <v>34.96</v>
+        <v>34.91</v>
       </c>
       <c r="L8" t="n">
-        <v>31.25</v>
+        <v>32.39</v>
       </c>
       <c r="M8" t="n">
-        <v>33.79</v>
+        <v>34.39</v>
       </c>
       <c r="N8" t="n">
-        <v>32.58</v>
+        <v>32.78</v>
       </c>
       <c r="O8" t="n">
-        <v>33.94</v>
+        <v>33.34</v>
       </c>
       <c r="P8" t="n">
-        <v>32.16</v>
+        <v>32.73</v>
       </c>
       <c r="Q8" t="n">
-        <v>33.37</v>
+        <v>32.95</v>
       </c>
       <c r="R8" t="n">
-        <v>-10.314</v>
+        <v>-1.9366</v>
       </c>
       <c r="S8" t="n">
-        <v>-13.2404</v>
+        <v>-14.9154</v>
       </c>
       <c r="T8" t="n">
-        <v>-7.2679</v>
+        <v>-14.6295</v>
       </c>
       <c r="U8" t="n">
-        <v>-4.0541</v>
+        <v>1.3087</v>
       </c>
       <c r="V8" t="n">
-        <v>-3.4769</v>
+        <v>-3.5252</v>
       </c>
       <c r="W8" t="n">
-        <v>1.9052</v>
+        <v>0.3333</v>
       </c>
       <c r="X8" t="n">
-        <v>10.2447</v>
+        <v>1.7757</v>
       </c>
       <c r="Y8" t="n">
-        <v>14.0783</v>
+        <v>16.0648</v>
       </c>
       <c r="Z8" t="n">
-        <v>6.3917</v>
+        <v>15.7523</v>
       </c>
       <c r="AA8" t="n">
-        <v>4.0536</v>
+        <v>-1.2586</v>
       </c>
       <c r="AB8" t="n">
-        <v>3.4729</v>
+        <v>3.5187</v>
       </c>
       <c r="AC8" t="n">
-        <v>-2.1695</v>
+        <v>-0.5133</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>148.18</v>
+        <v>134.43</v>
       </c>
       <c r="C9" t="n">
-        <v>148.18</v>
+        <v>134.54</v>
       </c>
       <c r="D9" t="n">
-        <v>137.71</v>
+        <v>127.27</v>
       </c>
       <c r="E9" t="n">
-        <v>139.76</v>
+        <v>128.4</v>
       </c>
       <c r="F9" t="n">
-        <v>81.72</v>
+        <v>80.78</v>
       </c>
       <c r="G9" t="n">
-        <v>81.81</v>
+        <v>80.81</v>
       </c>
       <c r="H9" t="n">
-        <v>80.37</v>
+        <v>79.22</v>
       </c>
       <c r="I9" t="n">
-        <v>81.28</v>
+        <v>79.61</v>
       </c>
       <c r="J9" t="n">
-        <v>32.4</v>
+        <v>35.75</v>
       </c>
       <c r="K9" t="n">
-        <v>34.91</v>
+        <v>37.5</v>
       </c>
       <c r="L9" t="n">
-        <v>32.39</v>
+        <v>35.68</v>
       </c>
       <c r="M9" t="n">
-        <v>34.39</v>
+        <v>37.19</v>
       </c>
       <c r="N9" t="n">
-        <v>32.78</v>
+        <v>33.17</v>
       </c>
       <c r="O9" t="n">
-        <v>33.34</v>
+        <v>33.8</v>
       </c>
       <c r="P9" t="n">
-        <v>32.73</v>
+        <v>33.17</v>
       </c>
       <c r="Q9" t="n">
-        <v>32.95</v>
+        <v>33.63</v>
       </c>
       <c r="R9" t="n">
-        <v>-1.9366</v>
+        <v>-8.1282</v>
       </c>
       <c r="S9" t="n">
-        <v>-14.9154</v>
+        <v>-19.1995</v>
       </c>
       <c r="T9" t="n">
-        <v>-14.6295</v>
+        <v>-21.836</v>
       </c>
       <c r="U9" t="n">
-        <v>1.3087</v>
+        <v>-2.0546</v>
       </c>
       <c r="V9" t="n">
-        <v>-3.5252</v>
+        <v>-4.7955</v>
       </c>
       <c r="W9" t="n">
-        <v>0.3333</v>
+        <v>-4.2228</v>
       </c>
       <c r="X9" t="n">
-        <v>1.7757</v>
+        <v>8.1419</v>
       </c>
       <c r="Y9" t="n">
-        <v>16.0648</v>
+        <v>21.3377</v>
       </c>
       <c r="Z9" t="n">
-        <v>15.7523</v>
+        <v>25.5571</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.2586</v>
+        <v>2.0637</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.5187</v>
+        <v>4.8644</v>
       </c>
       <c r="AC9" t="n">
-        <v>-0.5133</v>
+        <v>4.2791</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>134.43</v>
+        <v>118.42</v>
       </c>
       <c r="C10" t="n">
-        <v>134.54</v>
+        <v>127.92</v>
       </c>
       <c r="D10" t="n">
-        <v>127.27</v>
+        <v>115.84</v>
       </c>
       <c r="E10" t="n">
-        <v>128.4</v>
+        <v>127.57</v>
       </c>
       <c r="F10" t="n">
-        <v>80.78</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>80.81</v>
+        <v>79</v>
       </c>
       <c r="H10" t="n">
-        <v>79.22</v>
+        <v>77.28</v>
       </c>
       <c r="I10" t="n">
-        <v>79.61</v>
+        <v>78.81</v>
       </c>
       <c r="J10" t="n">
-        <v>35.75</v>
+        <v>40.15</v>
       </c>
       <c r="K10" t="n">
-        <v>37.5</v>
+        <v>40.9</v>
       </c>
       <c r="L10" t="n">
-        <v>35.68</v>
+        <v>37.36</v>
       </c>
       <c r="M10" t="n">
-        <v>37.19</v>
+        <v>37.42</v>
       </c>
       <c r="N10" t="n">
-        <v>33.17</v>
+        <v>34.54</v>
       </c>
       <c r="O10" t="n">
-        <v>33.8</v>
+        <v>34.63</v>
       </c>
       <c r="P10" t="n">
-        <v>33.17</v>
+        <v>33.89</v>
       </c>
       <c r="Q10" t="n">
-        <v>33.63</v>
+        <v>33.99</v>
       </c>
       <c r="R10" t="n">
-        <v>-8.1282</v>
+        <v>-0.6464</v>
       </c>
       <c r="S10" t="n">
-        <v>-19.1995</v>
+        <v>-10.4898</v>
       </c>
       <c r="T10" t="n">
-        <v>-21.836</v>
+        <v>-22.3365</v>
       </c>
       <c r="U10" t="n">
-        <v>-2.0546</v>
+        <v>-1.0049</v>
       </c>
       <c r="V10" t="n">
-        <v>-4.7955</v>
+        <v>-1.7699</v>
       </c>
       <c r="W10" t="n">
-        <v>-4.2228</v>
+        <v>-6.457</v>
       </c>
       <c r="X10" t="n">
-        <v>8.1419</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="Y10" t="n">
-        <v>21.3377</v>
+        <v>10.7428</v>
       </c>
       <c r="Z10" t="n">
-        <v>25.5571</v>
+        <v>26.2909</v>
       </c>
       <c r="AA10" t="n">
-        <v>2.0637</v>
+        <v>1.0705</v>
       </c>
       <c r="AB10" t="n">
-        <v>4.8644</v>
+        <v>1.858</v>
       </c>
       <c r="AC10" t="n">
-        <v>4.2791</v>
+        <v>6.7861</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>118.42</v>
+        <v>119.02</v>
       </c>
       <c r="C11" t="n">
-        <v>127.92</v>
+        <v>120.9</v>
       </c>
       <c r="D11" t="n">
-        <v>115.84</v>
+        <v>109</v>
       </c>
       <c r="E11" t="n">
-        <v>127.57</v>
+        <v>110.54</v>
       </c>
       <c r="F11" t="n">
-        <v>77.51000000000001</v>
+        <v>77</v>
       </c>
       <c r="G11" t="n">
-        <v>79</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>77.28</v>
+        <v>73.31</v>
       </c>
       <c r="I11" t="n">
-        <v>78.81</v>
+        <v>74.12</v>
       </c>
       <c r="J11" t="n">
-        <v>40.15</v>
+        <v>40.03</v>
       </c>
       <c r="K11" t="n">
-        <v>40.9</v>
+        <v>42.95</v>
       </c>
       <c r="L11" t="n">
-        <v>37.36</v>
+        <v>39.43</v>
       </c>
       <c r="M11" t="n">
-        <v>37.42</v>
+        <v>42.52</v>
       </c>
       <c r="N11" t="n">
-        <v>34.54</v>
+        <v>34.77</v>
       </c>
       <c r="O11" t="n">
-        <v>34.63</v>
+        <v>36.35</v>
       </c>
       <c r="P11" t="n">
-        <v>33.89</v>
+        <v>34.42</v>
       </c>
       <c r="Q11" t="n">
-        <v>33.99</v>
+        <v>36</v>
       </c>
       <c r="R11" t="n">
-        <v>-0.6464</v>
+        <v>-13.3495</v>
       </c>
       <c r="S11" t="n">
-        <v>-10.4898</v>
+        <v>-20.9073</v>
       </c>
       <c r="T11" t="n">
-        <v>-22.3365</v>
+        <v>-30.4386</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.0049</v>
+        <v>-5.951</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.7699</v>
+        <v>-8.809100000000001</v>
       </c>
       <c r="W11" t="n">
-        <v>-6.457</v>
+        <v>-11.3609</v>
       </c>
       <c r="X11" t="n">
-        <v>0.6183999999999999</v>
+        <v>13.6291</v>
       </c>
       <c r="Y11" t="n">
-        <v>10.7428</v>
+        <v>23.6406</v>
       </c>
       <c r="Z11" t="n">
-        <v>26.2909</v>
+        <v>38.7276</v>
       </c>
       <c r="AA11" t="n">
-        <v>1.0705</v>
+        <v>5.9135</v>
       </c>
       <c r="AB11" t="n">
-        <v>1.858</v>
+        <v>9.256399999999999</v>
       </c>
       <c r="AC11" t="n">
-        <v>6.7861</v>
+        <v>12.2544</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>119.02</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>120.9</v>
+        <v>108.8</v>
       </c>
       <c r="D12" t="n">
-        <v>109</v>
+        <v>95.23</v>
       </c>
       <c r="E12" t="n">
-        <v>110.54</v>
+        <v>107.35</v>
       </c>
       <c r="F12" t="n">
-        <v>77</v>
+        <v>70.95</v>
       </c>
       <c r="G12" t="n">
-        <v>77.79000000000001</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>73.31</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>74.12</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>40.03</v>
+        <v>47.19</v>
       </c>
       <c r="K12" t="n">
-        <v>42.95</v>
+        <v>48.37</v>
       </c>
       <c r="L12" t="n">
-        <v>39.43</v>
+        <v>43.11</v>
       </c>
       <c r="M12" t="n">
-        <v>42.52</v>
+        <v>43.64</v>
       </c>
       <c r="N12" t="n">
-        <v>34.77</v>
+        <v>37.57</v>
       </c>
       <c r="O12" t="n">
-        <v>36.35</v>
+        <v>38.02</v>
       </c>
       <c r="P12" t="n">
-        <v>34.42</v>
+        <v>35.94</v>
       </c>
       <c r="Q12" t="n">
-        <v>36</v>
+        <v>36.14</v>
       </c>
       <c r="R12" t="n">
-        <v>-13.3495</v>
+        <v>-2.8858</v>
       </c>
       <c r="S12" t="n">
-        <v>-20.9073</v>
+        <v>-16.3941</v>
       </c>
       <c r="T12" t="n">
-        <v>-30.4386</v>
+        <v>-24.6772</v>
       </c>
       <c r="U12" t="n">
-        <v>-5.951</v>
+        <v>-0.4047</v>
       </c>
       <c r="V12" t="n">
-        <v>-8.809100000000001</v>
+        <v>-7.273</v>
       </c>
       <c r="W12" t="n">
-        <v>-11.3609</v>
+        <v>-7.9895</v>
       </c>
       <c r="X12" t="n">
-        <v>13.6291</v>
+        <v>2.6341</v>
       </c>
       <c r="Y12" t="n">
-        <v>23.6406</v>
+        <v>17.3434</v>
       </c>
       <c r="Z12" t="n">
-        <v>38.7276</v>
+        <v>29.1506</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.9135</v>
+        <v>0.3889</v>
       </c>
       <c r="AB12" t="n">
-        <v>9.256399999999999</v>
+        <v>7.4636</v>
       </c>
       <c r="AC12" t="n">
-        <v>12.2544</v>
+        <v>8.3009</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>98.34999999999999</v>
+        <v>101.19</v>
       </c>
       <c r="C13" t="n">
-        <v>108.8</v>
+        <v>103.93</v>
       </c>
       <c r="D13" t="n">
-        <v>95.23</v>
+        <v>93.45</v>
       </c>
       <c r="E13" t="n">
-        <v>107.35</v>
+        <v>93.67</v>
       </c>
       <c r="F13" t="n">
-        <v>70.95</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>74.23999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="H13" t="n">
-        <v>69.98999999999999</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>73.81999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>47.19</v>
+        <v>46.22</v>
       </c>
       <c r="K13" t="n">
-        <v>48.37</v>
+        <v>49.36</v>
       </c>
       <c r="L13" t="n">
-        <v>43.11</v>
+        <v>45.08</v>
       </c>
       <c r="M13" t="n">
-        <v>43.64</v>
+        <v>49.23</v>
       </c>
       <c r="N13" t="n">
-        <v>37.57</v>
+        <v>36.57</v>
       </c>
       <c r="O13" t="n">
-        <v>38.02</v>
+        <v>39.29</v>
       </c>
       <c r="P13" t="n">
-        <v>35.94</v>
+        <v>36.51</v>
       </c>
       <c r="Q13" t="n">
-        <v>36.14</v>
+        <v>38.9</v>
       </c>
       <c r="R13" t="n">
-        <v>-2.8858</v>
+        <v>-12.7434</v>
       </c>
       <c r="S13" t="n">
-        <v>-16.3941</v>
+        <v>-26.5736</v>
       </c>
       <c r="T13" t="n">
-        <v>-24.6772</v>
+        <v>-32.978</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.4047</v>
+        <v>-7.5996</v>
       </c>
       <c r="V13" t="n">
-        <v>-7.273</v>
+        <v>-13.4501</v>
       </c>
       <c r="W13" t="n">
-        <v>-7.9895</v>
+        <v>-16.0802</v>
       </c>
       <c r="X13" t="n">
-        <v>2.6341</v>
+        <v>12.8093</v>
       </c>
       <c r="Y13" t="n">
-        <v>17.3434</v>
+        <v>31.5607</v>
       </c>
       <c r="Z13" t="n">
-        <v>29.1506</v>
+        <v>43.1521</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.3889</v>
+        <v>7.637</v>
       </c>
       <c r="AB13" t="n">
-        <v>7.4636</v>
+        <v>14.4454</v>
       </c>
       <c r="AC13" t="n">
-        <v>8.3009</v>
+        <v>18.0577</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>101.19</v>
+        <v>103.95</v>
       </c>
       <c r="C14" t="n">
-        <v>103.93</v>
+        <v>104.98</v>
       </c>
       <c r="D14" t="n">
-        <v>93.45</v>
+        <v>97.8</v>
       </c>
       <c r="E14" t="n">
-        <v>93.67</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>73.01000000000001</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>73.13</v>
+        <v>72.44</v>
       </c>
       <c r="H14" t="n">
-        <v>67.43000000000001</v>
+        <v>70.13</v>
       </c>
       <c r="I14" t="n">
-        <v>68.20999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="J14" t="n">
-        <v>46.22</v>
+        <v>43.86</v>
       </c>
       <c r="K14" t="n">
-        <v>49.36</v>
+        <v>47.07</v>
       </c>
       <c r="L14" t="n">
-        <v>45.08</v>
+        <v>43.32</v>
       </c>
       <c r="M14" t="n">
-        <v>49.23</v>
+        <v>46.63</v>
       </c>
       <c r="N14" t="n">
-        <v>36.57</v>
+        <v>37.33</v>
       </c>
       <c r="O14" t="n">
-        <v>39.29</v>
+        <v>37.82</v>
       </c>
       <c r="P14" t="n">
         <v>36.51</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.9</v>
+        <v>37.52</v>
       </c>
       <c r="R14" t="n">
-        <v>-12.7434</v>
+        <v>5.3165</v>
       </c>
       <c r="S14" t="n">
-        <v>-26.5736</v>
+        <v>-10.7563</v>
       </c>
       <c r="T14" t="n">
-        <v>-32.978</v>
+        <v>-23.1698</v>
       </c>
       <c r="U14" t="n">
-        <v>-7.5996</v>
+        <v>3.5625</v>
       </c>
       <c r="V14" t="n">
-        <v>-13.4501</v>
+        <v>-4.6951</v>
       </c>
       <c r="W14" t="n">
-        <v>-16.0802</v>
+        <v>-11.2674</v>
       </c>
       <c r="X14" t="n">
-        <v>12.8093</v>
+        <v>-5.2813</v>
       </c>
       <c r="Y14" t="n">
-        <v>31.5607</v>
+        <v>9.666</v>
       </c>
       <c r="Z14" t="n">
-        <v>43.1521</v>
+        <v>25.3832</v>
       </c>
       <c r="AA14" t="n">
-        <v>7.637</v>
+        <v>-3.5476</v>
       </c>
       <c r="AB14" t="n">
-        <v>14.4454</v>
+        <v>4.2222</v>
       </c>
       <c r="AC14" t="n">
-        <v>18.0577</v>
+        <v>11.5671</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>103.95</v>
+        <v>94.52</v>
       </c>
       <c r="C15" t="n">
-        <v>104.98</v>
+        <v>102.62</v>
       </c>
       <c r="D15" t="n">
-        <v>97.8</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>98.65000000000001</v>
+        <v>97.55</v>
       </c>
       <c r="F15" t="n">
-        <v>71.01000000000001</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>72.44</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>70.13</v>
+        <v>68.28</v>
       </c>
       <c r="I15" t="n">
-        <v>70.64</v>
+        <v>70.41</v>
       </c>
       <c r="J15" t="n">
-        <v>43.86</v>
+        <v>48.64</v>
       </c>
       <c r="K15" t="n">
-        <v>47.07</v>
+        <v>50.12</v>
       </c>
       <c r="L15" t="n">
-        <v>43.32</v>
+        <v>44.76</v>
       </c>
       <c r="M15" t="n">
-        <v>46.63</v>
+        <v>47.13</v>
       </c>
       <c r="N15" t="n">
-        <v>37.33</v>
+        <v>38.03</v>
       </c>
       <c r="O15" t="n">
-        <v>37.82</v>
+        <v>38.79</v>
       </c>
       <c r="P15" t="n">
-        <v>36.51</v>
+        <v>36.85</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.52</v>
+        <v>37.68</v>
       </c>
       <c r="R15" t="n">
-        <v>5.3165</v>
+        <v>-1.1151</v>
       </c>
       <c r="S15" t="n">
-        <v>-10.7563</v>
+        <v>-9.129</v>
       </c>
       <c r="T15" t="n">
-        <v>-23.1698</v>
+        <v>-23.5322</v>
       </c>
       <c r="U15" t="n">
-        <v>3.5625</v>
+        <v>-0.3256</v>
       </c>
       <c r="V15" t="n">
-        <v>-4.6951</v>
+        <v>-4.6193</v>
       </c>
       <c r="W15" t="n">
-        <v>-11.2674</v>
+        <v>-10.6585</v>
       </c>
       <c r="X15" t="n">
-        <v>-5.2813</v>
+        <v>1.0723</v>
       </c>
       <c r="Y15" t="n">
-        <v>9.666</v>
+        <v>7.9973</v>
       </c>
       <c r="Z15" t="n">
-        <v>25.3832</v>
+        <v>25.9487</v>
       </c>
       <c r="AA15" t="n">
-        <v>-3.5476</v>
+        <v>0.4264</v>
       </c>
       <c r="AB15" t="n">
-        <v>4.2222</v>
+        <v>4.2612</v>
       </c>
       <c r="AC15" t="n">
-        <v>11.5671</v>
+        <v>10.8561</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>94.52</v>
+        <v>102.86</v>
       </c>
       <c r="C16" t="n">
-        <v>102.62</v>
+        <v>106.13</v>
       </c>
       <c r="D16" t="n">
-        <v>91.34999999999999</v>
+        <v>99.31</v>
       </c>
       <c r="E16" t="n">
-        <v>97.55</v>
+        <v>103.24</v>
       </c>
       <c r="F16" t="n">
-        <v>69.70999999999999</v>
+        <v>71.72</v>
       </c>
       <c r="G16" t="n">
-        <v>71.93000000000001</v>
+        <v>73.43000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>68.28</v>
+        <v>71.02</v>
       </c>
       <c r="I16" t="n">
-        <v>70.41</v>
+        <v>72.61</v>
       </c>
       <c r="J16" t="n">
-        <v>48.64</v>
+        <v>44.51</v>
       </c>
       <c r="K16" t="n">
-        <v>50.12</v>
+        <v>47.1</v>
       </c>
       <c r="L16" t="n">
-        <v>44.76</v>
+        <v>43.57</v>
       </c>
       <c r="M16" t="n">
-        <v>47.13</v>
+        <v>44.29</v>
       </c>
       <c r="N16" t="n">
-        <v>38.03</v>
+        <v>36.94</v>
       </c>
       <c r="O16" t="n">
-        <v>38.79</v>
+        <v>38.11</v>
       </c>
       <c r="P16" t="n">
-        <v>36.85</v>
+        <v>36.05</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.68</v>
+        <v>36.48</v>
       </c>
       <c r="R16" t="n">
-        <v>-1.1151</v>
+        <v>5.8329</v>
       </c>
       <c r="S16" t="n">
-        <v>-9.129</v>
+        <v>10.2167</v>
       </c>
       <c r="T16" t="n">
-        <v>-23.5322</v>
+        <v>-6.6039</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.3256</v>
+        <v>3.1246</v>
       </c>
       <c r="V16" t="n">
-        <v>-4.6193</v>
+        <v>6.4507</v>
       </c>
       <c r="W16" t="n">
-        <v>-10.6585</v>
+        <v>-2.0372</v>
       </c>
       <c r="X16" t="n">
-        <v>1.0723</v>
+        <v>-6.0259</v>
       </c>
       <c r="Y16" t="n">
-        <v>7.9973</v>
+        <v>-10.0345</v>
       </c>
       <c r="Z16" t="n">
-        <v>25.9487</v>
+        <v>4.1627</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.4264</v>
+        <v>-3.1847</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.2612</v>
+        <v>-6.2211</v>
       </c>
       <c r="AC16" t="n">
-        <v>10.8561</v>
+        <v>1.3333</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>102.86</v>
+        <v>90.59</v>
       </c>
       <c r="C17" t="n">
-        <v>106.13</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>99.31</v>
+        <v>80.22</v>
       </c>
       <c r="E17" t="n">
-        <v>103.24</v>
+        <v>82.11</v>
       </c>
       <c r="F17" t="n">
-        <v>71.72</v>
+        <v>69.14</v>
       </c>
       <c r="G17" t="n">
-        <v>73.43000000000001</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>71.02</v>
+        <v>65.61</v>
       </c>
       <c r="I17" t="n">
-        <v>72.61</v>
+        <v>66.42</v>
       </c>
       <c r="J17" t="n">
-        <v>44.51</v>
+        <v>49.82</v>
       </c>
       <c r="K17" t="n">
-        <v>47.1</v>
+        <v>54.31</v>
       </c>
       <c r="L17" t="n">
-        <v>43.57</v>
+        <v>48.62</v>
       </c>
       <c r="M17" t="n">
-        <v>44.29</v>
+        <v>53.45</v>
       </c>
       <c r="N17" t="n">
-        <v>36.94</v>
+        <v>38.23</v>
       </c>
       <c r="O17" t="n">
-        <v>38.11</v>
+        <v>40</v>
       </c>
       <c r="P17" t="n">
-        <v>36.05</v>
+        <v>37.96</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.48</v>
+        <v>39.6</v>
       </c>
       <c r="R17" t="n">
-        <v>5.8329</v>
+        <v>-20.4669</v>
       </c>
       <c r="S17" t="n">
-        <v>10.2167</v>
+        <v>-16.7663</v>
       </c>
       <c r="T17" t="n">
-        <v>-6.6039</v>
+        <v>-23.5119</v>
       </c>
       <c r="U17" t="n">
-        <v>3.1246</v>
+        <v>-8.525</v>
       </c>
       <c r="V17" t="n">
-        <v>6.4507</v>
+        <v>-5.974</v>
       </c>
       <c r="W17" t="n">
-        <v>-2.0372</v>
+        <v>-10.0244</v>
       </c>
       <c r="X17" t="n">
-        <v>-6.0259</v>
+        <v>20.6819</v>
       </c>
       <c r="Y17" t="n">
-        <v>-10.0345</v>
+        <v>14.6258</v>
       </c>
       <c r="Z17" t="n">
-        <v>4.1627</v>
+        <v>22.4794</v>
       </c>
       <c r="AA17" t="n">
-        <v>-3.1847</v>
+        <v>8.5526</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.2211</v>
+        <v>5.5437</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.3333</v>
+        <v>9.5739</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>90.59</v>
+        <v>81.64</v>
       </c>
       <c r="C18" t="n">
-        <v>93.40000000000001</v>
+        <v>87.61</v>
       </c>
       <c r="D18" t="n">
-        <v>80.22</v>
+        <v>80.83</v>
       </c>
       <c r="E18" t="n">
-        <v>82.11</v>
+        <v>83.56</v>
       </c>
       <c r="F18" t="n">
-        <v>69.14</v>
+        <v>65.66</v>
       </c>
       <c r="G18" t="n">
-        <v>69.65000000000001</v>
+        <v>67.67</v>
       </c>
       <c r="H18" t="n">
-        <v>65.61</v>
+        <v>65.37</v>
       </c>
       <c r="I18" t="n">
-        <v>66.42</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>49.82</v>
+        <v>53.77</v>
       </c>
       <c r="K18" t="n">
-        <v>54.31</v>
+        <v>54.38</v>
       </c>
       <c r="L18" t="n">
-        <v>48.62</v>
+        <v>50.27</v>
       </c>
       <c r="M18" t="n">
-        <v>53.45</v>
+        <v>52.46</v>
       </c>
       <c r="N18" t="n">
-        <v>38.23</v>
+        <v>40.07</v>
       </c>
       <c r="O18" t="n">
-        <v>40</v>
+        <v>40.23</v>
       </c>
       <c r="P18" t="n">
-        <v>37.96</v>
+        <v>38.86</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.6</v>
+        <v>39.68</v>
       </c>
       <c r="R18" t="n">
-        <v>-20.4669</v>
+        <v>1.7659</v>
       </c>
       <c r="S18" t="n">
-        <v>-16.7663</v>
+        <v>-14.3414</v>
       </c>
       <c r="T18" t="n">
-        <v>-23.5119</v>
+        <v>-10.7932</v>
       </c>
       <c r="U18" t="n">
-        <v>-8.525</v>
+        <v>-0.1957</v>
       </c>
       <c r="V18" t="n">
-        <v>-5.974</v>
+        <v>-5.8514</v>
       </c>
       <c r="W18" t="n">
-        <v>-10.0244</v>
+        <v>-2.8148</v>
       </c>
       <c r="X18" t="n">
-        <v>20.6819</v>
+        <v>-1.8522</v>
       </c>
       <c r="Y18" t="n">
-        <v>14.6258</v>
+        <v>11.3091</v>
       </c>
       <c r="Z18" t="n">
-        <v>22.4794</v>
+        <v>6.561</v>
       </c>
       <c r="AA18" t="n">
-        <v>8.5526</v>
+        <v>0.202</v>
       </c>
       <c r="AB18" t="n">
-        <v>5.5437</v>
+        <v>5.3079</v>
       </c>
       <c r="AC18" t="n">
-        <v>9.5739</v>
+        <v>2.0051</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>81.64</v>
+        <v>85.88</v>
       </c>
       <c r="C19" t="n">
-        <v>87.61</v>
+        <v>93.15000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>80.83</v>
+        <v>84.22</v>
       </c>
       <c r="E19" t="n">
-        <v>83.56</v>
+        <v>90.5</v>
       </c>
       <c r="F19" t="n">
-        <v>65.66</v>
+        <v>67.02</v>
       </c>
       <c r="G19" t="n">
-        <v>67.67</v>
+        <v>69.33</v>
       </c>
       <c r="H19" t="n">
-        <v>65.37</v>
+        <v>66.61</v>
       </c>
       <c r="I19" t="n">
-        <v>66.29000000000001</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>53.77</v>
+        <v>51.03</v>
       </c>
       <c r="K19" t="n">
-        <v>54.38</v>
+        <v>52.09</v>
       </c>
       <c r="L19" t="n">
-        <v>50.27</v>
+        <v>46.47</v>
       </c>
       <c r="M19" t="n">
-        <v>52.46</v>
+        <v>47.98</v>
       </c>
       <c r="N19" t="n">
-        <v>40.07</v>
+        <v>39.23</v>
       </c>
       <c r="O19" t="n">
-        <v>40.23</v>
+        <v>39.51</v>
       </c>
       <c r="P19" t="n">
-        <v>38.86</v>
+        <v>37.86</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.68</v>
+        <v>38.38</v>
       </c>
       <c r="R19" t="n">
-        <v>1.7659</v>
+        <v>8.305400000000001</v>
       </c>
       <c r="S19" t="n">
-        <v>-14.3414</v>
+        <v>-12.3402</v>
       </c>
       <c r="T19" t="n">
-        <v>-10.7932</v>
+        <v>-8.2615</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.1957</v>
+        <v>3.2282</v>
       </c>
       <c r="V19" t="n">
-        <v>-5.8514</v>
+        <v>-5.7568</v>
       </c>
       <c r="W19" t="n">
-        <v>-2.8148</v>
+        <v>-3.1285</v>
       </c>
       <c r="X19" t="n">
-        <v>-1.8522</v>
+        <v>-8.5398</v>
       </c>
       <c r="Y19" t="n">
-        <v>11.3091</v>
+        <v>8.3315</v>
       </c>
       <c r="Z19" t="n">
-        <v>6.561</v>
+        <v>2.8951</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.202</v>
+        <v>-3.2762</v>
       </c>
       <c r="AB19" t="n">
-        <v>5.3079</v>
+        <v>5.2083</v>
       </c>
       <c r="AC19" t="n">
-        <v>2.0051</v>
+        <v>2.2921</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>85.88</v>
+        <v>95.04000000000001</v>
       </c>
       <c r="C20" t="n">
-        <v>93.15000000000001</v>
+        <v>102.2</v>
       </c>
       <c r="D20" t="n">
-        <v>84.22</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E20" t="n">
-        <v>90.5</v>
+        <v>101.08</v>
       </c>
       <c r="F20" t="n">
-        <v>67.02</v>
+        <v>69.3</v>
       </c>
       <c r="G20" t="n">
-        <v>69.33</v>
+        <v>71.53</v>
       </c>
       <c r="H20" t="n">
-        <v>66.61</v>
+        <v>68.86</v>
       </c>
       <c r="I20" t="n">
-        <v>68.43000000000001</v>
+        <v>71.04000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>51.03</v>
+        <v>45.8</v>
       </c>
       <c r="K20" t="n">
-        <v>52.09</v>
+        <v>46.21</v>
       </c>
       <c r="L20" t="n">
-        <v>46.47</v>
+        <v>41.9</v>
       </c>
       <c r="M20" t="n">
-        <v>47.98</v>
+        <v>42.5</v>
       </c>
       <c r="N20" t="n">
-        <v>39.23</v>
+        <v>37.93</v>
       </c>
       <c r="O20" t="n">
-        <v>39.51</v>
+        <v>38.17</v>
       </c>
       <c r="P20" t="n">
-        <v>37.86</v>
+        <v>36.67</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.38</v>
+        <v>36.93</v>
       </c>
       <c r="R20" t="n">
-        <v>8.305400000000001</v>
+        <v>11.6906</v>
       </c>
       <c r="S20" t="n">
-        <v>-12.3402</v>
+        <v>23.1032</v>
       </c>
       <c r="T20" t="n">
-        <v>-8.2615</v>
+        <v>3.6187</v>
       </c>
       <c r="U20" t="n">
-        <v>3.2282</v>
+        <v>3.8141</v>
       </c>
       <c r="V20" t="n">
-        <v>-5.7568</v>
+        <v>6.9557</v>
       </c>
       <c r="W20" t="n">
-        <v>-3.1285</v>
+        <v>0.8948</v>
       </c>
       <c r="X20" t="n">
-        <v>-8.5398</v>
+        <v>-11.4214</v>
       </c>
       <c r="Y20" t="n">
-        <v>8.3315</v>
+        <v>-20.4864</v>
       </c>
       <c r="Z20" t="n">
-        <v>2.8951</v>
+        <v>-9.8239</v>
       </c>
       <c r="AA20" t="n">
-        <v>-3.2762</v>
+        <v>-3.778</v>
       </c>
       <c r="AB20" t="n">
-        <v>5.2083</v>
+        <v>-6.7424</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.2921</v>
+        <v>-1.9904</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>95.04000000000001</v>
+        <v>103.97</v>
       </c>
       <c r="C21" t="n">
-        <v>102.2</v>
+        <v>108.6</v>
       </c>
       <c r="D21" t="n">
-        <v>94.09999999999999</v>
+        <v>101.32</v>
       </c>
       <c r="E21" t="n">
-        <v>101.08</v>
+        <v>107.35</v>
       </c>
       <c r="F21" t="n">
-        <v>69.3</v>
+        <v>71.91</v>
       </c>
       <c r="G21" t="n">
-        <v>71.53</v>
+        <v>72.53</v>
       </c>
       <c r="H21" t="n">
-        <v>68.86</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>71.04000000000001</v>
+        <v>72.36</v>
       </c>
       <c r="J21" t="n">
-        <v>45.8</v>
+        <v>41.33</v>
       </c>
       <c r="K21" t="n">
-        <v>46.21</v>
+        <v>42.41</v>
       </c>
       <c r="L21" t="n">
-        <v>41.9</v>
+        <v>39.33</v>
       </c>
       <c r="M21" t="n">
-        <v>42.5</v>
+        <v>39.78</v>
       </c>
       <c r="N21" t="n">
-        <v>37.93</v>
+        <v>36.51</v>
       </c>
       <c r="O21" t="n">
-        <v>38.17</v>
+        <v>37.09</v>
       </c>
       <c r="P21" t="n">
-        <v>36.67</v>
+        <v>36.2</v>
       </c>
       <c r="Q21" t="n">
-        <v>36.93</v>
+        <v>36.28</v>
       </c>
       <c r="R21" t="n">
-        <v>11.6906</v>
+        <v>6.203</v>
       </c>
       <c r="S21" t="n">
-        <v>23.1032</v>
+        <v>28.4706</v>
       </c>
       <c r="T21" t="n">
-        <v>3.6187</v>
+        <v>3.981</v>
       </c>
       <c r="U21" t="n">
-        <v>3.8141</v>
+        <v>1.8581</v>
       </c>
       <c r="V21" t="n">
-        <v>6.9557</v>
+        <v>9.156700000000001</v>
       </c>
       <c r="W21" t="n">
-        <v>0.8948</v>
+        <v>-0.3443</v>
       </c>
       <c r="X21" t="n">
-        <v>-11.4214</v>
+        <v>-6.4</v>
       </c>
       <c r="Y21" t="n">
-        <v>-20.4864</v>
+        <v>-24.1708</v>
       </c>
       <c r="Z21" t="n">
-        <v>-9.8239</v>
+        <v>-10.1829</v>
       </c>
       <c r="AA21" t="n">
-        <v>-3.778</v>
+        <v>-1.7601</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.7424</v>
+        <v>-8.5685</v>
       </c>
       <c r="AC21" t="n">
-        <v>-1.9904</v>
+        <v>-0.5482</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>103.97</v>
+        <v>101.36</v>
       </c>
       <c r="C22" t="n">
-        <v>108.6</v>
+        <v>105.44</v>
       </c>
       <c r="D22" t="n">
-        <v>101.32</v>
+        <v>97.95</v>
       </c>
       <c r="E22" t="n">
-        <v>107.35</v>
+        <v>102.39</v>
       </c>
       <c r="F22" t="n">
-        <v>71.91</v>
+        <v>69.61</v>
       </c>
       <c r="G22" t="n">
-        <v>72.53</v>
+        <v>70.06</v>
       </c>
       <c r="H22" t="n">
-        <v>70.76000000000001</v>
+        <v>68.13</v>
       </c>
       <c r="I22" t="n">
-        <v>72.36</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>41.33</v>
+        <v>42.08</v>
       </c>
       <c r="K22" t="n">
-        <v>42.41</v>
+        <v>43.36</v>
       </c>
       <c r="L22" t="n">
-        <v>39.33</v>
+        <v>40.58</v>
       </c>
       <c r="M22" t="n">
-        <v>39.78</v>
+        <v>41.68</v>
       </c>
       <c r="N22" t="n">
-        <v>36.51</v>
+        <v>37.65</v>
       </c>
       <c r="O22" t="n">
-        <v>37.09</v>
+        <v>38.4</v>
       </c>
       <c r="P22" t="n">
-        <v>36.2</v>
+        <v>37.42</v>
       </c>
       <c r="Q22" t="n">
-        <v>36.28</v>
+        <v>37.83</v>
       </c>
       <c r="R22" t="n">
-        <v>6.203</v>
+        <v>-4.6204</v>
       </c>
       <c r="S22" t="n">
-        <v>28.4706</v>
+        <v>13.1381</v>
       </c>
       <c r="T22" t="n">
-        <v>3.981</v>
+        <v>24.6986</v>
       </c>
       <c r="U22" t="n">
-        <v>1.8581</v>
+        <v>-4.2841</v>
       </c>
       <c r="V22" t="n">
-        <v>9.156700000000001</v>
+        <v>1.2129</v>
       </c>
       <c r="W22" t="n">
-        <v>-0.3443</v>
+        <v>4.2758</v>
       </c>
       <c r="X22" t="n">
-        <v>-6.4</v>
+        <v>4.7763</v>
       </c>
       <c r="Y22" t="n">
-        <v>-24.1708</v>
+        <v>-13.1305</v>
       </c>
       <c r="Z22" t="n">
-        <v>-10.1829</v>
+        <v>-22.0206</v>
       </c>
       <c r="AA22" t="n">
-        <v>-1.7601</v>
+        <v>4.2723</v>
       </c>
       <c r="AB22" t="n">
-        <v>-8.5685</v>
+        <v>-1.433</v>
       </c>
       <c r="AC22" t="n">
-        <v>-0.5482</v>
+        <v>-4.4697</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>101.36</v>
+        <v>81.79000000000001</v>
       </c>
       <c r="C23" t="n">
-        <v>105.44</v>
+        <v>84.19</v>
       </c>
       <c r="D23" t="n">
-        <v>97.95</v>
+        <v>70.23</v>
       </c>
       <c r="E23" t="n">
-        <v>102.39</v>
+        <v>77.05</v>
       </c>
       <c r="F23" t="n">
-        <v>69.61</v>
+        <v>63.93</v>
       </c>
       <c r="G23" t="n">
-        <v>70.06</v>
+        <v>64.33</v>
       </c>
       <c r="H23" t="n">
-        <v>68.13</v>
+        <v>59.95</v>
       </c>
       <c r="I23" t="n">
-        <v>69.26000000000001</v>
+        <v>62.01</v>
       </c>
       <c r="J23" t="n">
-        <v>42.08</v>
+        <v>50.12</v>
       </c>
       <c r="K23" t="n">
-        <v>43.36</v>
+        <v>54.85</v>
       </c>
       <c r="L23" t="n">
-        <v>40.58</v>
+        <v>49.14</v>
       </c>
       <c r="M23" t="n">
-        <v>41.68</v>
+        <v>52.08</v>
       </c>
       <c r="N23" t="n">
-        <v>37.65</v>
+        <v>40.78</v>
       </c>
       <c r="O23" t="n">
-        <v>38.4</v>
+        <v>42.96</v>
       </c>
       <c r="P23" t="n">
-        <v>37.42</v>
+        <v>40.55</v>
       </c>
       <c r="Q23" t="n">
-        <v>37.83</v>
+        <v>41.83</v>
       </c>
       <c r="R23" t="n">
-        <v>-4.6204</v>
+        <v>-24.7485</v>
       </c>
       <c r="S23" t="n">
-        <v>13.1381</v>
+        <v>-23.7732</v>
       </c>
       <c r="T23" t="n">
-        <v>24.6986</v>
+        <v>-7.7908</v>
       </c>
       <c r="U23" t="n">
-        <v>-4.2841</v>
+        <v>-10.4678</v>
       </c>
       <c r="V23" t="n">
-        <v>1.2129</v>
+        <v>-12.7111</v>
       </c>
       <c r="W23" t="n">
-        <v>4.2758</v>
+        <v>-6.4565</v>
       </c>
       <c r="X23" t="n">
-        <v>4.7763</v>
+        <v>24.952</v>
       </c>
       <c r="Y23" t="n">
-        <v>-13.1305</v>
+        <v>22.5412</v>
       </c>
       <c r="Z23" t="n">
-        <v>-22.0206</v>
+        <v>-0.7244</v>
       </c>
       <c r="AA23" t="n">
-        <v>4.2723</v>
+        <v>10.5736</v>
       </c>
       <c r="AB23" t="n">
-        <v>-1.433</v>
+        <v>13.2683</v>
       </c>
       <c r="AC23" t="n">
-        <v>-4.4697</v>
+        <v>5.4183</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>

</xml_diff>